<commit_message>
Atualização automática: mta (10/07/2026 17:31)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -20,16 +20,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -48,21 +45,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -433,112 +421,112 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>linha</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>projeto_coordenador</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>projeto_atividade</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>situacao_consolidada</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>aprovado</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>acao</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>tramite</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>data_pedido</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>digito</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>rodada</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>preenchimento_tgco</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>observacao_coordenador</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>impactos_nao_atendimento</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>atividade</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>tarefa</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>valor</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>executora</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>nd</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>pacote</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>para_contrato</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>para_motores</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>mes_previsto</t>
         </is>
@@ -578,7 +566,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H2" s="2" t="n">
+      <c r="H2" s="1" t="n">
         <v>46076</v>
       </c>
       <c r="I2" t="inlineStr">
@@ -628,7 +616,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V2" s="2" t="n">
+      <c r="V2" s="1" t="n">
         <v>46079</v>
       </c>
     </row>
@@ -666,7 +654,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H3" s="2" t="n">
+      <c r="H3" s="1" t="n">
         <v>46076</v>
       </c>
       <c r="I3" t="inlineStr">
@@ -716,7 +704,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V3" s="2" t="n">
+      <c r="V3" s="1" t="n">
         <v>46079</v>
       </c>
     </row>
@@ -754,7 +742,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H4" s="2" t="n">
+      <c r="H4" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="I4" t="inlineStr">
@@ -808,7 +796,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V4" s="2" t="n">
+      <c r="V4" s="1" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -846,7 +834,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H5" s="2" t="n">
+      <c r="H5" s="1" t="n">
         <v>46119</v>
       </c>
       <c r="I5" t="inlineStr">
@@ -896,7 +884,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V5" s="2" t="n">
+      <c r="V5" s="1" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -934,7 +922,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H6" s="2" t="n">
+      <c r="H6" s="1" t="n">
         <v>46175</v>
       </c>
       <c r="I6" t="inlineStr">
@@ -984,7 +972,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V6" s="2" t="n">
+      <c r="V6" s="1" t="n">
         <v>46229</v>
       </c>
     </row>
@@ -1062,7 +1050,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V7" s="2" t="n">
+      <c r="V7" s="1" t="n">
         <v>46260</v>
       </c>
     </row>
@@ -1100,7 +1088,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H8" s="2" t="n">
+      <c r="H8" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="I8" t="inlineStr">
@@ -1150,7 +1138,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V8" s="2" t="n">
+      <c r="V8" s="1" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -1188,7 +1176,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H9" s="2" t="n">
+      <c r="H9" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="I9" t="inlineStr">
@@ -1238,7 +1226,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V9" s="2" t="n">
+      <c r="V9" s="1" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -1276,7 +1264,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H10" s="2" t="n">
+      <c r="H10" s="1" t="n">
         <v>46204</v>
       </c>
       <c r="I10" t="inlineStr">
@@ -1326,7 +1314,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V10" s="2" t="n">
+      <c r="V10" s="1" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -1364,7 +1352,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H11" s="2" t="n">
+      <c r="H11" s="1" t="n">
         <v>46191</v>
       </c>
       <c r="I11" t="inlineStr">
@@ -1414,7 +1402,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V11" s="2" t="n">
+      <c r="V11" s="1" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -1452,7 +1440,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H12" s="2" t="n">
+      <c r="H12" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="I12" t="inlineStr">
@@ -1502,7 +1490,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V12" s="2" t="n">
+      <c r="V12" s="1" t="n">
         <v>46229</v>
       </c>
     </row>
@@ -1540,7 +1528,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H13" s="2" t="n">
+      <c r="H13" s="1" t="n">
         <v>46176</v>
       </c>
       <c r="I13" t="inlineStr">
@@ -1594,7 +1582,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V13" s="2" t="n">
+      <c r="V13" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -1676,7 +1664,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V14" s="2" t="n">
+      <c r="V14" s="1" t="n">
         <v>46321</v>
       </c>
     </row>
@@ -1750,7 +1738,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V15" s="2" t="n">
+      <c r="V15" s="1" t="n">
         <v>46107</v>
       </c>
     </row>
@@ -1824,7 +1812,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V16" s="2" t="n">
+      <c r="V16" s="1" t="n">
         <v>46107</v>
       </c>
     </row>
@@ -1898,7 +1886,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V17" s="2" t="n">
+      <c r="V17" s="1" t="n">
         <v>46107</v>
       </c>
     </row>
@@ -1972,7 +1960,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V18" s="2" t="n">
+      <c r="V18" s="1" t="n">
         <v>46107</v>
       </c>
     </row>
@@ -2046,7 +2034,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V19" s="2" t="n">
+      <c r="V19" s="1" t="n">
         <v>46107</v>
       </c>
     </row>
@@ -2120,7 +2108,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V20" s="2" t="n">
+      <c r="V20" s="1" t="n">
         <v>46107</v>
       </c>
     </row>
@@ -2202,7 +2190,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V21" s="2" t="n">
+      <c r="V21" s="1" t="n">
         <v>46381</v>
       </c>
     </row>
@@ -2284,7 +2272,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V22" s="2" t="n">
+      <c r="V22" s="1" t="n">
         <v>46381</v>
       </c>
     </row>
@@ -2322,7 +2310,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H23" s="2" t="n">
+      <c r="H23" s="1" t="n">
         <v>46098</v>
       </c>
       <c r="I23" t="inlineStr">
@@ -2376,7 +2364,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V23" s="2" t="n">
+      <c r="V23" s="1" t="n">
         <v>46107</v>
       </c>
     </row>
@@ -2414,7 +2402,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H24" s="2" t="n">
+      <c r="H24" s="1" t="n">
         <v>46119</v>
       </c>
       <c r="I24" t="inlineStr">
@@ -2468,7 +2456,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V24" s="2" t="n">
+      <c r="V24" s="1" t="n">
         <v>46138</v>
       </c>
     </row>
@@ -2506,7 +2494,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H25" s="2" t="n">
+      <c r="H25" s="1" t="n">
         <v>46191</v>
       </c>
       <c r="I25" t="inlineStr">
@@ -2560,7 +2548,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V25" s="2" t="n">
+      <c r="V25" s="1" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -2646,7 +2634,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V26" s="2" t="n">
+      <c r="V26" s="1" t="n">
         <v>46229</v>
       </c>
     </row>
@@ -2732,7 +2720,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V27" s="2" t="n">
+      <c r="V27" s="1" t="n">
         <v>46260</v>
       </c>
     </row>
@@ -2818,7 +2806,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V28" s="2" t="n">
+      <c r="V28" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -2896,7 +2884,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V29" s="2" t="n">
+      <c r="V29" s="1" t="n">
         <v>46321</v>
       </c>
     </row>
@@ -2974,7 +2962,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V30" s="2" t="n">
+      <c r="V30" s="1" t="n">
         <v>46352</v>
       </c>
     </row>
@@ -3052,7 +3040,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V31" s="2" t="n">
+      <c r="V31" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -3090,7 +3078,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H32" s="2" t="n">
+      <c r="H32" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="I32" t="inlineStr">
@@ -3144,7 +3132,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V32" s="2" t="n">
+      <c r="V32" s="1" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -3182,7 +3170,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H33" s="2" t="n">
+      <c r="H33" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="I33" t="inlineStr">
@@ -3236,7 +3224,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V33" s="2" t="n">
+      <c r="V33" s="1" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -3274,7 +3262,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H34" s="2" t="n">
+      <c r="H34" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="I34" t="inlineStr">
@@ -3328,7 +3316,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V34" s="2" t="n">
+      <c r="V34" s="1" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -3410,7 +3398,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V35" s="2" t="n">
+      <c r="V35" s="1" t="n">
         <v>46381</v>
       </c>
     </row>
@@ -3492,7 +3480,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V36" s="2" t="n">
+      <c r="V36" s="1" t="n">
         <v>46381</v>
       </c>
     </row>
@@ -3530,7 +3518,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H37" s="2" t="n">
+      <c r="H37" s="1" t="n">
         <v>46121</v>
       </c>
       <c r="I37" t="inlineStr">
@@ -3580,7 +3568,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V37" s="2" t="n">
+      <c r="V37" s="1" t="n">
         <v>46107</v>
       </c>
     </row>
@@ -3618,7 +3606,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H38" s="2" t="n">
+      <c r="H38" s="1" t="n">
         <v>46076</v>
       </c>
       <c r="I38" t="inlineStr">
@@ -3668,7 +3656,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V38" s="2" t="n">
+      <c r="V38" s="1" t="n">
         <v>46079</v>
       </c>
     </row>
@@ -3706,7 +3694,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H39" s="2" t="n">
+      <c r="H39" s="1" t="n">
         <v>46191</v>
       </c>
       <c r="I39" t="inlineStr">
@@ -3756,7 +3744,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V39" s="2" t="n">
+      <c r="V39" s="1" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -3834,7 +3822,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V40" s="2" t="n">
+      <c r="V40" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -3912,7 +3900,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V41" s="2" t="n">
+      <c r="V41" s="1" t="n">
         <v>46260</v>
       </c>
     </row>
@@ -3990,7 +3978,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V42" s="2" t="n">
+      <c r="V42" s="1" t="n">
         <v>46321</v>
       </c>
     </row>
@@ -4028,7 +4016,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H43" s="2" t="n">
+      <c r="H43" s="1" t="n">
         <v>46121</v>
       </c>
       <c r="I43" t="inlineStr">
@@ -4078,7 +4066,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V43" s="2" t="n">
+      <c r="V43" s="1" t="n">
         <v>46168</v>
       </c>
     </row>
@@ -4156,7 +4144,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V44" s="2" t="n">
+      <c r="V44" s="1" t="n">
         <v>46260</v>
       </c>
     </row>
@@ -4232,7 +4220,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V45" s="2" t="n">
+      <c r="V45" s="1" t="n">
         <v>46260</v>
       </c>
     </row>
@@ -4314,7 +4302,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V46" s="2" t="n">
+      <c r="V46" s="1" t="n">
         <v>46229</v>
       </c>
     </row>
@@ -4392,7 +4380,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V47" s="2" t="n">
+      <c r="V47" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -4470,7 +4458,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V48" s="2" t="n">
+      <c r="V48" s="1" t="n">
         <v>46321</v>
       </c>
     </row>
@@ -4548,7 +4536,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V49" s="2" t="n">
+      <c r="V49" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -4586,7 +4574,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H50" s="2" t="n">
+      <c r="H50" s="1" t="n">
         <v>46079</v>
       </c>
       <c r="I50" t="inlineStr">
@@ -4640,7 +4628,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V50" s="2" t="n">
+      <c r="V50" s="1" t="n">
         <v>46107</v>
       </c>
     </row>
@@ -4718,7 +4706,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V51" s="2" t="n">
+      <c r="V51" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -4796,7 +4784,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V52" s="2" t="n">
+      <c r="V52" s="1" t="n">
         <v>46352</v>
       </c>
     </row>
@@ -4870,7 +4858,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V53" s="2" t="n">
+      <c r="V53" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -4948,7 +4936,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V54" s="2" t="n">
+      <c r="V54" s="1" t="n">
         <v>46352</v>
       </c>
     </row>
@@ -5022,7 +5010,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V55" s="2" t="n">
+      <c r="V55" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -5100,7 +5088,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V56" s="2" t="n">
+      <c r="V56" s="1" t="n">
         <v>46352</v>
       </c>
     </row>
@@ -5174,7 +5162,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V57" s="2" t="n">
+      <c r="V57" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -5252,7 +5240,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V58" s="2" t="n">
+      <c r="V58" s="1" t="n">
         <v>46229</v>
       </c>
     </row>
@@ -5330,7 +5318,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V59" s="2" t="n">
+      <c r="V59" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -5408,7 +5396,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V60" s="2" t="n">
+      <c r="V60" s="1" t="n">
         <v>46229</v>
       </c>
     </row>
@@ -5482,7 +5470,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V61" s="2" t="n">
+      <c r="V61" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -5560,7 +5548,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V62" s="2" t="n">
+      <c r="V62" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -5642,7 +5630,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V63" s="2" t="n">
+      <c r="V63" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -5720,7 +5708,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V64" s="2" t="n">
+      <c r="V64" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -5798,7 +5786,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V65" s="2" t="n">
+      <c r="V65" s="1" t="n">
         <v>46321</v>
       </c>
     </row>
@@ -5872,7 +5860,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V66" s="2" t="n">
+      <c r="V66" s="1" t="n">
         <v>46168</v>
       </c>
     </row>
@@ -5950,7 +5938,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V67" s="2" t="n">
+      <c r="V67" s="1" t="n">
         <v>46321</v>
       </c>
     </row>
@@ -6024,7 +6012,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V68" s="2" t="n">
+      <c r="V68" s="1" t="n">
         <v>46260</v>
       </c>
     </row>
@@ -6102,7 +6090,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V69" s="2" t="n">
+      <c r="V69" s="1" t="n">
         <v>46260</v>
       </c>
     </row>
@@ -6180,7 +6168,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V70" s="2" t="n">
+      <c r="V70" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -6258,7 +6246,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V71" s="2" t="n">
+      <c r="V71" s="1" t="n">
         <v>46260</v>
       </c>
     </row>
@@ -6336,7 +6324,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V72" s="2" t="n">
+      <c r="V72" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -6414,7 +6402,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V73" s="2" t="n">
+      <c r="V73" s="1" t="n">
         <v>46321</v>
       </c>
     </row>
@@ -6492,7 +6480,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V74" s="2" t="n">
+      <c r="V74" s="1" t="n">
         <v>46049</v>
       </c>
     </row>
@@ -6718,7 +6706,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V77" s="2" t="n">
+      <c r="V77" s="1" t="n">
         <v>46168</v>
       </c>
     </row>
@@ -6792,7 +6780,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V78" s="2" t="n">
+      <c r="V78" s="1" t="n">
         <v>46382</v>
       </c>
     </row>
@@ -6866,7 +6854,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V79" s="2" t="n">
+      <c r="V79" s="1" t="n">
         <v>46382</v>
       </c>
     </row>
@@ -6944,7 +6932,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V80" s="2" t="n">
+      <c r="V80" s="1" t="n">
         <v>46382</v>
       </c>
     </row>
@@ -7018,7 +7006,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V81" s="2" t="n">
+      <c r="V81" s="1" t="n">
         <v>46321</v>
       </c>
     </row>
@@ -7092,7 +7080,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V82" s="2" t="n">
+      <c r="V82" s="1" t="n">
         <v>46382</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (10/07/2026 16:01)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -20,13 +20,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +40,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +48,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -421,112 +433,112 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>linha</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>projeto_coordenador</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>projeto_atividade</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>situacao_consolidada</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>aprovado</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>acao</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>tramite</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>data_pedido</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>digito</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>rodada</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>preenchimento_tgco</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>observacao_coordenador</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>impactos_nao_atendimento</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>atividade</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>tarefa</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>valor</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>executora</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>nd</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>pacote</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>para_contrato</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>para_motores</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>mes_previsto</t>
         </is>
@@ -566,7 +578,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H2" s="1" t="n">
+      <c r="H2" s="2" t="n">
         <v>46076</v>
       </c>
       <c r="I2" t="inlineStr">
@@ -616,7 +628,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V2" s="1" t="n">
+      <c r="V2" s="2" t="n">
         <v>46079</v>
       </c>
     </row>
@@ -654,7 +666,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H3" s="1" t="n">
+      <c r="H3" s="2" t="n">
         <v>46076</v>
       </c>
       <c r="I3" t="inlineStr">
@@ -704,7 +716,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V3" s="1" t="n">
+      <c r="V3" s="2" t="n">
         <v>46079</v>
       </c>
     </row>
@@ -742,7 +754,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H4" s="1" t="n">
+      <c r="H4" s="2" t="n">
         <v>46199</v>
       </c>
       <c r="I4" t="inlineStr">
@@ -796,7 +808,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V4" s="1" t="n">
+      <c r="V4" s="2" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -834,7 +846,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H5" s="1" t="n">
+      <c r="H5" s="2" t="n">
         <v>46119</v>
       </c>
       <c r="I5" t="inlineStr">
@@ -884,7 +896,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V5" s="1" t="n">
+      <c r="V5" s="2" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -922,7 +934,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H6" s="1" t="n">
+      <c r="H6" s="2" t="n">
         <v>46175</v>
       </c>
       <c r="I6" t="inlineStr">
@@ -972,7 +984,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V6" s="1" t="n">
+      <c r="V6" s="2" t="n">
         <v>46229</v>
       </c>
     </row>
@@ -1050,7 +1062,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V7" s="1" t="n">
+      <c r="V7" s="2" t="n">
         <v>46260</v>
       </c>
     </row>
@@ -1088,7 +1100,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H8" s="1" t="n">
+      <c r="H8" s="2" t="n">
         <v>46199</v>
       </c>
       <c r="I8" t="inlineStr">
@@ -1138,7 +1150,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V8" s="1" t="n">
+      <c r="V8" s="2" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -1176,7 +1188,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H9" s="1" t="n">
+      <c r="H9" s="2" t="n">
         <v>46199</v>
       </c>
       <c r="I9" t="inlineStr">
@@ -1226,7 +1238,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V9" s="1" t="n">
+      <c r="V9" s="2" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -1264,7 +1276,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H10" s="1" t="n">
+      <c r="H10" s="2" t="n">
         <v>46204</v>
       </c>
       <c r="I10" t="inlineStr">
@@ -1314,7 +1326,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V10" s="1" t="n">
+      <c r="V10" s="2" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -1352,7 +1364,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H11" s="1" t="n">
+      <c r="H11" s="2" t="n">
         <v>46191</v>
       </c>
       <c r="I11" t="inlineStr">
@@ -1402,7 +1414,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V11" s="1" t="n">
+      <c r="V11" s="2" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -1440,7 +1452,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H12" s="1" t="n">
+      <c r="H12" s="2" t="n">
         <v>46210</v>
       </c>
       <c r="I12" t="inlineStr">
@@ -1490,7 +1502,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V12" s="1" t="n">
+      <c r="V12" s="2" t="n">
         <v>46229</v>
       </c>
     </row>
@@ -1528,7 +1540,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H13" s="1" t="n">
+      <c r="H13" s="2" t="n">
         <v>46176</v>
       </c>
       <c r="I13" t="inlineStr">
@@ -1582,7 +1594,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V13" s="1" t="n">
+      <c r="V13" s="2" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -1664,7 +1676,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V14" s="1" t="n">
+      <c r="V14" s="2" t="n">
         <v>46321</v>
       </c>
     </row>
@@ -1738,7 +1750,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V15" s="1" t="n">
+      <c r="V15" s="2" t="n">
         <v>46107</v>
       </c>
     </row>
@@ -1812,7 +1824,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V16" s="1" t="n">
+      <c r="V16" s="2" t="n">
         <v>46107</v>
       </c>
     </row>
@@ -1886,7 +1898,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V17" s="1" t="n">
+      <c r="V17" s="2" t="n">
         <v>46107</v>
       </c>
     </row>
@@ -1960,7 +1972,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V18" s="1" t="n">
+      <c r="V18" s="2" t="n">
         <v>46107</v>
       </c>
     </row>
@@ -2034,7 +2046,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V19" s="1" t="n">
+      <c r="V19" s="2" t="n">
         <v>46107</v>
       </c>
     </row>
@@ -2108,7 +2120,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V20" s="1" t="n">
+      <c r="V20" s="2" t="n">
         <v>46107</v>
       </c>
     </row>
@@ -2190,7 +2202,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V21" s="1" t="n">
+      <c r="V21" s="2" t="n">
         <v>46381</v>
       </c>
     </row>
@@ -2272,7 +2284,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V22" s="1" t="n">
+      <c r="V22" s="2" t="n">
         <v>46381</v>
       </c>
     </row>
@@ -2310,7 +2322,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H23" s="1" t="n">
+      <c r="H23" s="2" t="n">
         <v>46098</v>
       </c>
       <c r="I23" t="inlineStr">
@@ -2364,7 +2376,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V23" s="1" t="n">
+      <c r="V23" s="2" t="n">
         <v>46107</v>
       </c>
     </row>
@@ -2402,7 +2414,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H24" s="1" t="n">
+      <c r="H24" s="2" t="n">
         <v>46119</v>
       </c>
       <c r="I24" t="inlineStr">
@@ -2456,7 +2468,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V24" s="1" t="n">
+      <c r="V24" s="2" t="n">
         <v>46138</v>
       </c>
     </row>
@@ -2494,7 +2506,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H25" s="1" t="n">
+      <c r="H25" s="2" t="n">
         <v>46191</v>
       </c>
       <c r="I25" t="inlineStr">
@@ -2548,7 +2560,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V25" s="1" t="n">
+      <c r="V25" s="2" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -2634,7 +2646,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V26" s="1" t="n">
+      <c r="V26" s="2" t="n">
         <v>46229</v>
       </c>
     </row>
@@ -2720,7 +2732,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V27" s="1" t="n">
+      <c r="V27" s="2" t="n">
         <v>46260</v>
       </c>
     </row>
@@ -2806,7 +2818,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V28" s="1" t="n">
+      <c r="V28" s="2" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -2884,7 +2896,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V29" s="1" t="n">
+      <c r="V29" s="2" t="n">
         <v>46321</v>
       </c>
     </row>
@@ -2962,7 +2974,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V30" s="1" t="n">
+      <c r="V30" s="2" t="n">
         <v>46352</v>
       </c>
     </row>
@@ -3040,7 +3052,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V31" s="1" t="n">
+      <c r="V31" s="2" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -3078,7 +3090,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H32" s="1" t="n">
+      <c r="H32" s="2" t="n">
         <v>46199</v>
       </c>
       <c r="I32" t="inlineStr">
@@ -3132,7 +3144,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V32" s="1" t="n">
+      <c r="V32" s="2" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -3170,7 +3182,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H33" s="1" t="n">
+      <c r="H33" s="2" t="n">
         <v>46199</v>
       </c>
       <c r="I33" t="inlineStr">
@@ -3224,7 +3236,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V33" s="1" t="n">
+      <c r="V33" s="2" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -3262,7 +3274,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H34" s="1" t="n">
+      <c r="H34" s="2" t="n">
         <v>46199</v>
       </c>
       <c r="I34" t="inlineStr">
@@ -3316,7 +3328,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V34" s="1" t="n">
+      <c r="V34" s="2" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -3398,7 +3410,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V35" s="1" t="n">
+      <c r="V35" s="2" t="n">
         <v>46381</v>
       </c>
     </row>
@@ -3480,7 +3492,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V36" s="1" t="n">
+      <c r="V36" s="2" t="n">
         <v>46381</v>
       </c>
     </row>
@@ -3518,7 +3530,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H37" s="1" t="n">
+      <c r="H37" s="2" t="n">
         <v>46121</v>
       </c>
       <c r="I37" t="inlineStr">
@@ -3568,7 +3580,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V37" s="1" t="n">
+      <c r="V37" s="2" t="n">
         <v>46107</v>
       </c>
     </row>
@@ -3606,7 +3618,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H38" s="1" t="n">
+      <c r="H38" s="2" t="n">
         <v>46076</v>
       </c>
       <c r="I38" t="inlineStr">
@@ -3656,7 +3668,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V38" s="1" t="n">
+      <c r="V38" s="2" t="n">
         <v>46079</v>
       </c>
     </row>
@@ -3694,7 +3706,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H39" s="1" t="n">
+      <c r="H39" s="2" t="n">
         <v>46191</v>
       </c>
       <c r="I39" t="inlineStr">
@@ -3744,7 +3756,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V39" s="1" t="n">
+      <c r="V39" s="2" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -3822,7 +3834,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V40" s="1" t="n">
+      <c r="V40" s="2" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -3900,7 +3912,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V41" s="1" t="n">
+      <c r="V41" s="2" t="n">
         <v>46260</v>
       </c>
     </row>
@@ -3978,7 +3990,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V42" s="1" t="n">
+      <c r="V42" s="2" t="n">
         <v>46321</v>
       </c>
     </row>
@@ -4016,7 +4028,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H43" s="1" t="n">
+      <c r="H43" s="2" t="n">
         <v>46121</v>
       </c>
       <c r="I43" t="inlineStr">
@@ -4066,7 +4078,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V43" s="1" t="n">
+      <c r="V43" s="2" t="n">
         <v>46168</v>
       </c>
     </row>
@@ -4144,7 +4156,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V44" s="1" t="n">
+      <c r="V44" s="2" t="n">
         <v>46260</v>
       </c>
     </row>
@@ -4220,7 +4232,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V45" s="1" t="n">
+      <c r="V45" s="2" t="n">
         <v>46260</v>
       </c>
     </row>
@@ -4302,7 +4314,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V46" s="1" t="n">
+      <c r="V46" s="2" t="n">
         <v>46229</v>
       </c>
     </row>
@@ -4380,7 +4392,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V47" s="1" t="n">
+      <c r="V47" s="2" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -4458,7 +4470,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V48" s="1" t="n">
+      <c r="V48" s="2" t="n">
         <v>46321</v>
       </c>
     </row>
@@ -4536,7 +4548,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V49" s="1" t="n">
+      <c r="V49" s="2" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -4574,7 +4586,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H50" s="1" t="n">
+      <c r="H50" s="2" t="n">
         <v>46079</v>
       </c>
       <c r="I50" t="inlineStr">
@@ -4628,7 +4640,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V50" s="1" t="n">
+      <c r="V50" s="2" t="n">
         <v>46107</v>
       </c>
     </row>
@@ -4706,7 +4718,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V51" s="1" t="n">
+      <c r="V51" s="2" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -4784,7 +4796,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V52" s="1" t="n">
+      <c r="V52" s="2" t="n">
         <v>46352</v>
       </c>
     </row>
@@ -4858,7 +4870,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V53" s="1" t="n">
+      <c r="V53" s="2" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -4936,7 +4948,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V54" s="1" t="n">
+      <c r="V54" s="2" t="n">
         <v>46352</v>
       </c>
     </row>
@@ -5010,7 +5022,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V55" s="1" t="n">
+      <c r="V55" s="2" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -5088,7 +5100,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V56" s="1" t="n">
+      <c r="V56" s="2" t="n">
         <v>46352</v>
       </c>
     </row>
@@ -5162,7 +5174,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V57" s="1" t="n">
+      <c r="V57" s="2" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -5240,7 +5252,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V58" s="1" t="n">
+      <c r="V58" s="2" t="n">
         <v>46229</v>
       </c>
     </row>
@@ -5318,7 +5330,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V59" s="1" t="n">
+      <c r="V59" s="2" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -5396,7 +5408,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V60" s="1" t="n">
+      <c r="V60" s="2" t="n">
         <v>46229</v>
       </c>
     </row>
@@ -5470,7 +5482,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V61" s="1" t="n">
+      <c r="V61" s="2" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -5548,7 +5560,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V62" s="1" t="n">
+      <c r="V62" s="2" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -5630,7 +5642,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V63" s="1" t="n">
+      <c r="V63" s="2" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -5708,7 +5720,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V64" s="1" t="n">
+      <c r="V64" s="2" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -5786,7 +5798,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V65" s="1" t="n">
+      <c r="V65" s="2" t="n">
         <v>46321</v>
       </c>
     </row>
@@ -5860,7 +5872,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V66" s="1" t="n">
+      <c r="V66" s="2" t="n">
         <v>46168</v>
       </c>
     </row>
@@ -5938,7 +5950,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V67" s="1" t="n">
+      <c r="V67" s="2" t="n">
         <v>46321</v>
       </c>
     </row>
@@ -6012,7 +6024,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V68" s="1" t="n">
+      <c r="V68" s="2" t="n">
         <v>46260</v>
       </c>
     </row>
@@ -6090,7 +6102,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V69" s="1" t="n">
+      <c r="V69" s="2" t="n">
         <v>46260</v>
       </c>
     </row>
@@ -6168,7 +6180,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V70" s="1" t="n">
+      <c r="V70" s="2" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -6246,7 +6258,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V71" s="1" t="n">
+      <c r="V71" s="2" t="n">
         <v>46260</v>
       </c>
     </row>
@@ -6324,7 +6336,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V72" s="1" t="n">
+      <c r="V72" s="2" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -6402,7 +6414,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V73" s="1" t="n">
+      <c r="V73" s="2" t="n">
         <v>46321</v>
       </c>
     </row>
@@ -6480,7 +6492,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V74" s="1" t="n">
+      <c r="V74" s="2" t="n">
         <v>46049</v>
       </c>
     </row>
@@ -6706,7 +6718,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V77" s="1" t="n">
+      <c r="V77" s="2" t="n">
         <v>46168</v>
       </c>
     </row>
@@ -6780,7 +6792,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V78" s="1" t="n">
+      <c r="V78" s="2" t="n">
         <v>46382</v>
       </c>
     </row>
@@ -6854,7 +6866,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V79" s="1" t="n">
+      <c r="V79" s="2" t="n">
         <v>46382</v>
       </c>
     </row>
@@ -6932,7 +6944,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V80" s="1" t="n">
+      <c r="V80" s="2" t="n">
         <v>46382</v>
       </c>
     </row>
@@ -7006,7 +7018,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V81" s="1" t="n">
+      <c r="V81" s="2" t="n">
         <v>46321</v>
       </c>
     </row>
@@ -7080,7 +7092,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V82" s="1" t="n">
+      <c r="V82" s="2" t="n">
         <v>46382</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (10/07/2026 22:39)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -20,16 +20,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -48,21 +45,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -433,112 +421,112 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>linha</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>projeto_coordenador</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>projeto_atividade</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>situacao_consolidada</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>aprovado</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>acao</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>tramite</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>data_pedido</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>digito</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>rodada</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>preenchimento_tgco</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>observacao_coordenador</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>impactos_nao_atendimento</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>atividade</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>tarefa</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>valor</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>executora</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>nd</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>pacote</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>para_contrato</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>para_motores</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>mes_previsto</t>
         </is>
@@ -578,7 +566,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H2" s="2" t="n">
+      <c r="H2" s="1" t="n">
         <v>46076</v>
       </c>
       <c r="I2" t="inlineStr">
@@ -628,7 +616,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V2" s="2" t="n">
+      <c r="V2" s="1" t="n">
         <v>46079</v>
       </c>
     </row>
@@ -666,7 +654,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H3" s="2" t="n">
+      <c r="H3" s="1" t="n">
         <v>46076</v>
       </c>
       <c r="I3" t="inlineStr">
@@ -716,7 +704,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V3" s="2" t="n">
+      <c r="V3" s="1" t="n">
         <v>46079</v>
       </c>
     </row>
@@ -754,7 +742,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H4" s="2" t="n">
+      <c r="H4" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="I4" t="inlineStr">
@@ -808,7 +796,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V4" s="2" t="n">
+      <c r="V4" s="1" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -846,7 +834,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H5" s="2" t="n">
+      <c r="H5" s="1" t="n">
         <v>46119</v>
       </c>
       <c r="I5" t="inlineStr">
@@ -896,7 +884,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V5" s="2" t="n">
+      <c r="V5" s="1" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -934,7 +922,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H6" s="2" t="n">
+      <c r="H6" s="1" t="n">
         <v>46175</v>
       </c>
       <c r="I6" t="inlineStr">
@@ -984,7 +972,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V6" s="2" t="n">
+      <c r="V6" s="1" t="n">
         <v>46229</v>
       </c>
     </row>
@@ -1062,7 +1050,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V7" s="2" t="n">
+      <c r="V7" s="1" t="n">
         <v>46260</v>
       </c>
     </row>
@@ -1100,7 +1088,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H8" s="2" t="n">
+      <c r="H8" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="I8" t="inlineStr">
@@ -1150,7 +1138,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V8" s="2" t="n">
+      <c r="V8" s="1" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -1188,7 +1176,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H9" s="2" t="n">
+      <c r="H9" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="I9" t="inlineStr">
@@ -1238,7 +1226,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V9" s="2" t="n">
+      <c r="V9" s="1" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -1276,7 +1264,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H10" s="2" t="n">
+      <c r="H10" s="1" t="n">
         <v>46204</v>
       </c>
       <c r="I10" t="inlineStr">
@@ -1326,7 +1314,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V10" s="2" t="n">
+      <c r="V10" s="1" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -1364,7 +1352,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H11" s="2" t="n">
+      <c r="H11" s="1" t="n">
         <v>46191</v>
       </c>
       <c r="I11" t="inlineStr">
@@ -1414,7 +1402,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V11" s="2" t="n">
+      <c r="V11" s="1" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -1452,7 +1440,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H12" s="2" t="n">
+      <c r="H12" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="I12" t="inlineStr">
@@ -1502,7 +1490,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V12" s="2" t="n">
+      <c r="V12" s="1" t="n">
         <v>46229</v>
       </c>
     </row>
@@ -1540,7 +1528,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H13" s="2" t="n">
+      <c r="H13" s="1" t="n">
         <v>46176</v>
       </c>
       <c r="I13" t="inlineStr">
@@ -1594,7 +1582,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V13" s="2" t="n">
+      <c r="V13" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -1676,7 +1664,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V14" s="2" t="n">
+      <c r="V14" s="1" t="n">
         <v>46321</v>
       </c>
     </row>
@@ -1750,7 +1738,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V15" s="2" t="n">
+      <c r="V15" s="1" t="n">
         <v>46107</v>
       </c>
     </row>
@@ -1824,7 +1812,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V16" s="2" t="n">
+      <c r="V16" s="1" t="n">
         <v>46107</v>
       </c>
     </row>
@@ -1898,7 +1886,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V17" s="2" t="n">
+      <c r="V17" s="1" t="n">
         <v>46107</v>
       </c>
     </row>
@@ -1972,7 +1960,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V18" s="2" t="n">
+      <c r="V18" s="1" t="n">
         <v>46107</v>
       </c>
     </row>
@@ -2046,7 +2034,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V19" s="2" t="n">
+      <c r="V19" s="1" t="n">
         <v>46107</v>
       </c>
     </row>
@@ -2120,7 +2108,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V20" s="2" t="n">
+      <c r="V20" s="1" t="n">
         <v>46107</v>
       </c>
     </row>
@@ -2202,7 +2190,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V21" s="2" t="n">
+      <c r="V21" s="1" t="n">
         <v>46381</v>
       </c>
     </row>
@@ -2284,7 +2272,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V22" s="2" t="n">
+      <c r="V22" s="1" t="n">
         <v>46381</v>
       </c>
     </row>
@@ -2322,7 +2310,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H23" s="2" t="n">
+      <c r="H23" s="1" t="n">
         <v>46098</v>
       </c>
       <c r="I23" t="inlineStr">
@@ -2376,7 +2364,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V23" s="2" t="n">
+      <c r="V23" s="1" t="n">
         <v>46107</v>
       </c>
     </row>
@@ -2414,7 +2402,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H24" s="2" t="n">
+      <c r="H24" s="1" t="n">
         <v>46119</v>
       </c>
       <c r="I24" t="inlineStr">
@@ -2468,7 +2456,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V24" s="2" t="n">
+      <c r="V24" s="1" t="n">
         <v>46138</v>
       </c>
     </row>
@@ -2506,7 +2494,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H25" s="2" t="n">
+      <c r="H25" s="1" t="n">
         <v>46191</v>
       </c>
       <c r="I25" t="inlineStr">
@@ -2560,7 +2548,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V25" s="2" t="n">
+      <c r="V25" s="1" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -2646,7 +2634,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V26" s="2" t="n">
+      <c r="V26" s="1" t="n">
         <v>46229</v>
       </c>
     </row>
@@ -2732,7 +2720,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V27" s="2" t="n">
+      <c r="V27" s="1" t="n">
         <v>46260</v>
       </c>
     </row>
@@ -2818,7 +2806,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V28" s="2" t="n">
+      <c r="V28" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -2896,7 +2884,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V29" s="2" t="n">
+      <c r="V29" s="1" t="n">
         <v>46321</v>
       </c>
     </row>
@@ -2974,7 +2962,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V30" s="2" t="n">
+      <c r="V30" s="1" t="n">
         <v>46352</v>
       </c>
     </row>
@@ -3052,7 +3040,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V31" s="2" t="n">
+      <c r="V31" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -3090,7 +3078,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H32" s="2" t="n">
+      <c r="H32" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="I32" t="inlineStr">
@@ -3144,7 +3132,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V32" s="2" t="n">
+      <c r="V32" s="1" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -3182,7 +3170,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H33" s="2" t="n">
+      <c r="H33" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="I33" t="inlineStr">
@@ -3236,7 +3224,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V33" s="2" t="n">
+      <c r="V33" s="1" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -3274,7 +3262,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H34" s="2" t="n">
+      <c r="H34" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="I34" t="inlineStr">
@@ -3328,7 +3316,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V34" s="2" t="n">
+      <c r="V34" s="1" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -3410,7 +3398,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V35" s="2" t="n">
+      <c r="V35" s="1" t="n">
         <v>46381</v>
       </c>
     </row>
@@ -3492,7 +3480,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V36" s="2" t="n">
+      <c r="V36" s="1" t="n">
         <v>46381</v>
       </c>
     </row>
@@ -3530,7 +3518,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H37" s="2" t="n">
+      <c r="H37" s="1" t="n">
         <v>46121</v>
       </c>
       <c r="I37" t="inlineStr">
@@ -3580,7 +3568,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V37" s="2" t="n">
+      <c r="V37" s="1" t="n">
         <v>46107</v>
       </c>
     </row>
@@ -3618,7 +3606,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H38" s="2" t="n">
+      <c r="H38" s="1" t="n">
         <v>46076</v>
       </c>
       <c r="I38" t="inlineStr">
@@ -3668,7 +3656,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V38" s="2" t="n">
+      <c r="V38" s="1" t="n">
         <v>46079</v>
       </c>
     </row>
@@ -3706,7 +3694,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H39" s="2" t="n">
+      <c r="H39" s="1" t="n">
         <v>46191</v>
       </c>
       <c r="I39" t="inlineStr">
@@ -3756,7 +3744,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V39" s="2" t="n">
+      <c r="V39" s="1" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -3834,7 +3822,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V40" s="2" t="n">
+      <c r="V40" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -3912,7 +3900,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V41" s="2" t="n">
+      <c r="V41" s="1" t="n">
         <v>46260</v>
       </c>
     </row>
@@ -3990,7 +3978,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V42" s="2" t="n">
+      <c r="V42" s="1" t="n">
         <v>46321</v>
       </c>
     </row>
@@ -4028,7 +4016,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H43" s="2" t="n">
+      <c r="H43" s="1" t="n">
         <v>46121</v>
       </c>
       <c r="I43" t="inlineStr">
@@ -4078,7 +4066,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V43" s="2" t="n">
+      <c r="V43" s="1" t="n">
         <v>46168</v>
       </c>
     </row>
@@ -4156,7 +4144,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V44" s="2" t="n">
+      <c r="V44" s="1" t="n">
         <v>46260</v>
       </c>
     </row>
@@ -4232,7 +4220,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V45" s="2" t="n">
+      <c r="V45" s="1" t="n">
         <v>46260</v>
       </c>
     </row>
@@ -4314,7 +4302,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V46" s="2" t="n">
+      <c r="V46" s="1" t="n">
         <v>46229</v>
       </c>
     </row>
@@ -4392,7 +4380,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V47" s="2" t="n">
+      <c r="V47" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -4470,7 +4458,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V48" s="2" t="n">
+      <c r="V48" s="1" t="n">
         <v>46321</v>
       </c>
     </row>
@@ -4548,7 +4536,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V49" s="2" t="n">
+      <c r="V49" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -4586,7 +4574,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H50" s="2" t="n">
+      <c r="H50" s="1" t="n">
         <v>46079</v>
       </c>
       <c r="I50" t="inlineStr">
@@ -4640,7 +4628,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V50" s="2" t="n">
+      <c r="V50" s="1" t="n">
         <v>46107</v>
       </c>
     </row>
@@ -4718,7 +4706,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V51" s="2" t="n">
+      <c r="V51" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -4796,7 +4784,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V52" s="2" t="n">
+      <c r="V52" s="1" t="n">
         <v>46352</v>
       </c>
     </row>
@@ -4870,7 +4858,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V53" s="2" t="n">
+      <c r="V53" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -4948,7 +4936,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V54" s="2" t="n">
+      <c r="V54" s="1" t="n">
         <v>46352</v>
       </c>
     </row>
@@ -5022,7 +5010,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V55" s="2" t="n">
+      <c r="V55" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -5100,7 +5088,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V56" s="2" t="n">
+      <c r="V56" s="1" t="n">
         <v>46352</v>
       </c>
     </row>
@@ -5174,7 +5162,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V57" s="2" t="n">
+      <c r="V57" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -5252,7 +5240,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V58" s="2" t="n">
+      <c r="V58" s="1" t="n">
         <v>46229</v>
       </c>
     </row>
@@ -5330,7 +5318,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V59" s="2" t="n">
+      <c r="V59" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -5408,7 +5396,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V60" s="2" t="n">
+      <c r="V60" s="1" t="n">
         <v>46229</v>
       </c>
     </row>
@@ -5482,7 +5470,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V61" s="2" t="n">
+      <c r="V61" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -5560,7 +5548,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V62" s="2" t="n">
+      <c r="V62" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -5642,7 +5630,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V63" s="2" t="n">
+      <c r="V63" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -5720,7 +5708,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V64" s="2" t="n">
+      <c r="V64" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -5798,7 +5786,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V65" s="2" t="n">
+      <c r="V65" s="1" t="n">
         <v>46321</v>
       </c>
     </row>
@@ -5872,7 +5860,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V66" s="2" t="n">
+      <c r="V66" s="1" t="n">
         <v>46168</v>
       </c>
     </row>
@@ -5950,7 +5938,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V67" s="2" t="n">
+      <c r="V67" s="1" t="n">
         <v>46321</v>
       </c>
     </row>
@@ -6024,7 +6012,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V68" s="2" t="n">
+      <c r="V68" s="1" t="n">
         <v>46260</v>
       </c>
     </row>
@@ -6102,7 +6090,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V69" s="2" t="n">
+      <c r="V69" s="1" t="n">
         <v>46260</v>
       </c>
     </row>
@@ -6180,7 +6168,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V70" s="2" t="n">
+      <c r="V70" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -6258,7 +6246,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V71" s="2" t="n">
+      <c r="V71" s="1" t="n">
         <v>46260</v>
       </c>
     </row>
@@ -6336,7 +6324,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V72" s="2" t="n">
+      <c r="V72" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -6414,7 +6402,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V73" s="2" t="n">
+      <c r="V73" s="1" t="n">
         <v>46321</v>
       </c>
     </row>
@@ -6492,7 +6480,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V74" s="2" t="n">
+      <c r="V74" s="1" t="n">
         <v>46049</v>
       </c>
     </row>
@@ -6718,7 +6706,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V77" s="2" t="n">
+      <c r="V77" s="1" t="n">
         <v>46168</v>
       </c>
     </row>
@@ -6792,7 +6780,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V78" s="2" t="n">
+      <c r="V78" s="1" t="n">
         <v>46382</v>
       </c>
     </row>
@@ -6866,7 +6854,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V79" s="2" t="n">
+      <c r="V79" s="1" t="n">
         <v>46382</v>
       </c>
     </row>
@@ -6944,7 +6932,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V80" s="2" t="n">
+      <c r="V80" s="1" t="n">
         <v>46382</v>
       </c>
     </row>
@@ -7018,7 +7006,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V81" s="2" t="n">
+      <c r="V81" s="1" t="n">
         <v>46321</v>
       </c>
     </row>
@@ -7092,7 +7080,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V82" s="2" t="n">
+      <c r="V82" s="1" t="n">
         <v>46382</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (10/07/2026 20:01)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -20,13 +20,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +40,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +48,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -421,112 +433,112 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>linha</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>projeto_coordenador</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>projeto_atividade</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>situacao_consolidada</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>aprovado</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>acao</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>tramite</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>data_pedido</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>digito</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>rodada</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>preenchimento_tgco</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>observacao_coordenador</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>impactos_nao_atendimento</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>atividade</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>tarefa</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>valor</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>executora</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>nd</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>pacote</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>para_contrato</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>para_motores</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>mes_previsto</t>
         </is>
@@ -566,7 +578,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H2" s="1" t="n">
+      <c r="H2" s="2" t="n">
         <v>46076</v>
       </c>
       <c r="I2" t="inlineStr">
@@ -616,7 +628,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V2" s="1" t="n">
+      <c r="V2" s="2" t="n">
         <v>46079</v>
       </c>
     </row>
@@ -654,7 +666,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H3" s="1" t="n">
+      <c r="H3" s="2" t="n">
         <v>46076</v>
       </c>
       <c r="I3" t="inlineStr">
@@ -704,7 +716,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V3" s="1" t="n">
+      <c r="V3" s="2" t="n">
         <v>46079</v>
       </c>
     </row>
@@ -742,7 +754,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H4" s="1" t="n">
+      <c r="H4" s="2" t="n">
         <v>46199</v>
       </c>
       <c r="I4" t="inlineStr">
@@ -796,7 +808,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V4" s="1" t="n">
+      <c r="V4" s="2" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -834,7 +846,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H5" s="1" t="n">
+      <c r="H5" s="2" t="n">
         <v>46119</v>
       </c>
       <c r="I5" t="inlineStr">
@@ -884,7 +896,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V5" s="1" t="n">
+      <c r="V5" s="2" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -922,7 +934,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H6" s="1" t="n">
+      <c r="H6" s="2" t="n">
         <v>46175</v>
       </c>
       <c r="I6" t="inlineStr">
@@ -972,7 +984,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V6" s="1" t="n">
+      <c r="V6" s="2" t="n">
         <v>46229</v>
       </c>
     </row>
@@ -1050,7 +1062,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V7" s="1" t="n">
+      <c r="V7" s="2" t="n">
         <v>46260</v>
       </c>
     </row>
@@ -1088,7 +1100,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H8" s="1" t="n">
+      <c r="H8" s="2" t="n">
         <v>46199</v>
       </c>
       <c r="I8" t="inlineStr">
@@ -1138,7 +1150,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V8" s="1" t="n">
+      <c r="V8" s="2" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -1176,7 +1188,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H9" s="1" t="n">
+      <c r="H9" s="2" t="n">
         <v>46199</v>
       </c>
       <c r="I9" t="inlineStr">
@@ -1226,7 +1238,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V9" s="1" t="n">
+      <c r="V9" s="2" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -1264,7 +1276,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H10" s="1" t="n">
+      <c r="H10" s="2" t="n">
         <v>46204</v>
       </c>
       <c r="I10" t="inlineStr">
@@ -1314,7 +1326,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V10" s="1" t="n">
+      <c r="V10" s="2" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -1352,7 +1364,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H11" s="1" t="n">
+      <c r="H11" s="2" t="n">
         <v>46191</v>
       </c>
       <c r="I11" t="inlineStr">
@@ -1402,7 +1414,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V11" s="1" t="n">
+      <c r="V11" s="2" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -1440,7 +1452,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H12" s="1" t="n">
+      <c r="H12" s="2" t="n">
         <v>46210</v>
       </c>
       <c r="I12" t="inlineStr">
@@ -1490,7 +1502,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V12" s="1" t="n">
+      <c r="V12" s="2" t="n">
         <v>46229</v>
       </c>
     </row>
@@ -1528,7 +1540,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H13" s="1" t="n">
+      <c r="H13" s="2" t="n">
         <v>46176</v>
       </c>
       <c r="I13" t="inlineStr">
@@ -1582,7 +1594,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V13" s="1" t="n">
+      <c r="V13" s="2" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -1664,7 +1676,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V14" s="1" t="n">
+      <c r="V14" s="2" t="n">
         <v>46321</v>
       </c>
     </row>
@@ -1738,7 +1750,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V15" s="1" t="n">
+      <c r="V15" s="2" t="n">
         <v>46107</v>
       </c>
     </row>
@@ -1812,7 +1824,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V16" s="1" t="n">
+      <c r="V16" s="2" t="n">
         <v>46107</v>
       </c>
     </row>
@@ -1886,7 +1898,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V17" s="1" t="n">
+      <c r="V17" s="2" t="n">
         <v>46107</v>
       </c>
     </row>
@@ -1960,7 +1972,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V18" s="1" t="n">
+      <c r="V18" s="2" t="n">
         <v>46107</v>
       </c>
     </row>
@@ -2034,7 +2046,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V19" s="1" t="n">
+      <c r="V19" s="2" t="n">
         <v>46107</v>
       </c>
     </row>
@@ -2108,7 +2120,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V20" s="1" t="n">
+      <c r="V20" s="2" t="n">
         <v>46107</v>
       </c>
     </row>
@@ -2190,7 +2202,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V21" s="1" t="n">
+      <c r="V21" s="2" t="n">
         <v>46381</v>
       </c>
     </row>
@@ -2272,7 +2284,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V22" s="1" t="n">
+      <c r="V22" s="2" t="n">
         <v>46381</v>
       </c>
     </row>
@@ -2310,7 +2322,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H23" s="1" t="n">
+      <c r="H23" s="2" t="n">
         <v>46098</v>
       </c>
       <c r="I23" t="inlineStr">
@@ -2364,7 +2376,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V23" s="1" t="n">
+      <c r="V23" s="2" t="n">
         <v>46107</v>
       </c>
     </row>
@@ -2402,7 +2414,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H24" s="1" t="n">
+      <c r="H24" s="2" t="n">
         <v>46119</v>
       </c>
       <c r="I24" t="inlineStr">
@@ -2456,7 +2468,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V24" s="1" t="n">
+      <c r="V24" s="2" t="n">
         <v>46138</v>
       </c>
     </row>
@@ -2494,7 +2506,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H25" s="1" t="n">
+      <c r="H25" s="2" t="n">
         <v>46191</v>
       </c>
       <c r="I25" t="inlineStr">
@@ -2548,7 +2560,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V25" s="1" t="n">
+      <c r="V25" s="2" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -2634,7 +2646,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V26" s="1" t="n">
+      <c r="V26" s="2" t="n">
         <v>46229</v>
       </c>
     </row>
@@ -2720,7 +2732,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V27" s="1" t="n">
+      <c r="V27" s="2" t="n">
         <v>46260</v>
       </c>
     </row>
@@ -2806,7 +2818,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V28" s="1" t="n">
+      <c r="V28" s="2" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -2884,7 +2896,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V29" s="1" t="n">
+      <c r="V29" s="2" t="n">
         <v>46321</v>
       </c>
     </row>
@@ -2962,7 +2974,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V30" s="1" t="n">
+      <c r="V30" s="2" t="n">
         <v>46352</v>
       </c>
     </row>
@@ -3040,7 +3052,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V31" s="1" t="n">
+      <c r="V31" s="2" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -3078,7 +3090,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H32" s="1" t="n">
+      <c r="H32" s="2" t="n">
         <v>46199</v>
       </c>
       <c r="I32" t="inlineStr">
@@ -3132,7 +3144,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V32" s="1" t="n">
+      <c r="V32" s="2" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -3170,7 +3182,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H33" s="1" t="n">
+      <c r="H33" s="2" t="n">
         <v>46199</v>
       </c>
       <c r="I33" t="inlineStr">
@@ -3224,7 +3236,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V33" s="1" t="n">
+      <c r="V33" s="2" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -3262,7 +3274,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H34" s="1" t="n">
+      <c r="H34" s="2" t="n">
         <v>46199</v>
       </c>
       <c r="I34" t="inlineStr">
@@ -3316,7 +3328,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V34" s="1" t="n">
+      <c r="V34" s="2" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -3398,7 +3410,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V35" s="1" t="n">
+      <c r="V35" s="2" t="n">
         <v>46381</v>
       </c>
     </row>
@@ -3480,7 +3492,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V36" s="1" t="n">
+      <c r="V36" s="2" t="n">
         <v>46381</v>
       </c>
     </row>
@@ -3518,7 +3530,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H37" s="1" t="n">
+      <c r="H37" s="2" t="n">
         <v>46121</v>
       </c>
       <c r="I37" t="inlineStr">
@@ -3568,7 +3580,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V37" s="1" t="n">
+      <c r="V37" s="2" t="n">
         <v>46107</v>
       </c>
     </row>
@@ -3606,7 +3618,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H38" s="1" t="n">
+      <c r="H38" s="2" t="n">
         <v>46076</v>
       </c>
       <c r="I38" t="inlineStr">
@@ -3656,7 +3668,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V38" s="1" t="n">
+      <c r="V38" s="2" t="n">
         <v>46079</v>
       </c>
     </row>
@@ -3694,7 +3706,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H39" s="1" t="n">
+      <c r="H39" s="2" t="n">
         <v>46191</v>
       </c>
       <c r="I39" t="inlineStr">
@@ -3744,7 +3756,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V39" s="1" t="n">
+      <c r="V39" s="2" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -3822,7 +3834,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V40" s="1" t="n">
+      <c r="V40" s="2" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -3900,7 +3912,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V41" s="1" t="n">
+      <c r="V41" s="2" t="n">
         <v>46260</v>
       </c>
     </row>
@@ -3978,7 +3990,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V42" s="1" t="n">
+      <c r="V42" s="2" t="n">
         <v>46321</v>
       </c>
     </row>
@@ -4016,7 +4028,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H43" s="1" t="n">
+      <c r="H43" s="2" t="n">
         <v>46121</v>
       </c>
       <c r="I43" t="inlineStr">
@@ -4066,7 +4078,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V43" s="1" t="n">
+      <c r="V43" s="2" t="n">
         <v>46168</v>
       </c>
     </row>
@@ -4144,7 +4156,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V44" s="1" t="n">
+      <c r="V44" s="2" t="n">
         <v>46260</v>
       </c>
     </row>
@@ -4220,7 +4232,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V45" s="1" t="n">
+      <c r="V45" s="2" t="n">
         <v>46260</v>
       </c>
     </row>
@@ -4302,7 +4314,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V46" s="1" t="n">
+      <c r="V46" s="2" t="n">
         <v>46229</v>
       </c>
     </row>
@@ -4380,7 +4392,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V47" s="1" t="n">
+      <c r="V47" s="2" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -4458,7 +4470,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V48" s="1" t="n">
+      <c r="V48" s="2" t="n">
         <v>46321</v>
       </c>
     </row>
@@ -4536,7 +4548,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V49" s="1" t="n">
+      <c r="V49" s="2" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -4574,7 +4586,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H50" s="1" t="n">
+      <c r="H50" s="2" t="n">
         <v>46079</v>
       </c>
       <c r="I50" t="inlineStr">
@@ -4628,7 +4640,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V50" s="1" t="n">
+      <c r="V50" s="2" t="n">
         <v>46107</v>
       </c>
     </row>
@@ -4706,7 +4718,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V51" s="1" t="n">
+      <c r="V51" s="2" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -4784,7 +4796,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V52" s="1" t="n">
+      <c r="V52" s="2" t="n">
         <v>46352</v>
       </c>
     </row>
@@ -4858,7 +4870,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V53" s="1" t="n">
+      <c r="V53" s="2" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -4936,7 +4948,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V54" s="1" t="n">
+      <c r="V54" s="2" t="n">
         <v>46352</v>
       </c>
     </row>
@@ -5010,7 +5022,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V55" s="1" t="n">
+      <c r="V55" s="2" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -5088,7 +5100,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V56" s="1" t="n">
+      <c r="V56" s="2" t="n">
         <v>46352</v>
       </c>
     </row>
@@ -5162,7 +5174,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V57" s="1" t="n">
+      <c r="V57" s="2" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -5240,7 +5252,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V58" s="1" t="n">
+      <c r="V58" s="2" t="n">
         <v>46229</v>
       </c>
     </row>
@@ -5318,7 +5330,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V59" s="1" t="n">
+      <c r="V59" s="2" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -5396,7 +5408,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V60" s="1" t="n">
+      <c r="V60" s="2" t="n">
         <v>46229</v>
       </c>
     </row>
@@ -5470,7 +5482,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V61" s="1" t="n">
+      <c r="V61" s="2" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -5548,7 +5560,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V62" s="1" t="n">
+      <c r="V62" s="2" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -5630,7 +5642,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V63" s="1" t="n">
+      <c r="V63" s="2" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -5708,7 +5720,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V64" s="1" t="n">
+      <c r="V64" s="2" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -5786,7 +5798,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V65" s="1" t="n">
+      <c r="V65" s="2" t="n">
         <v>46321</v>
       </c>
     </row>
@@ -5860,7 +5872,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V66" s="1" t="n">
+      <c r="V66" s="2" t="n">
         <v>46168</v>
       </c>
     </row>
@@ -5938,7 +5950,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V67" s="1" t="n">
+      <c r="V67" s="2" t="n">
         <v>46321</v>
       </c>
     </row>
@@ -6012,7 +6024,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V68" s="1" t="n">
+      <c r="V68" s="2" t="n">
         <v>46260</v>
       </c>
     </row>
@@ -6090,7 +6102,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V69" s="1" t="n">
+      <c r="V69" s="2" t="n">
         <v>46260</v>
       </c>
     </row>
@@ -6168,7 +6180,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V70" s="1" t="n">
+      <c r="V70" s="2" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -6246,7 +6258,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V71" s="1" t="n">
+      <c r="V71" s="2" t="n">
         <v>46260</v>
       </c>
     </row>
@@ -6324,7 +6336,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V72" s="1" t="n">
+      <c r="V72" s="2" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -6402,7 +6414,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V73" s="1" t="n">
+      <c r="V73" s="2" t="n">
         <v>46321</v>
       </c>
     </row>
@@ -6480,7 +6492,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V74" s="1" t="n">
+      <c r="V74" s="2" t="n">
         <v>46049</v>
       </c>
     </row>
@@ -6706,7 +6718,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V77" s="1" t="n">
+      <c r="V77" s="2" t="n">
         <v>46168</v>
       </c>
     </row>
@@ -6780,7 +6792,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V78" s="1" t="n">
+      <c r="V78" s="2" t="n">
         <v>46382</v>
       </c>
     </row>
@@ -6854,7 +6866,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V79" s="1" t="n">
+      <c r="V79" s="2" t="n">
         <v>46382</v>
       </c>
     </row>
@@ -6932,7 +6944,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V80" s="1" t="n">
+      <c r="V80" s="2" t="n">
         <v>46382</v>
       </c>
     </row>
@@ -7006,7 +7018,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V81" s="1" t="n">
+      <c r="V81" s="2" t="n">
         <v>46321</v>
       </c>
     </row>
@@ -7080,7 +7092,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V82" s="1" t="n">
+      <c r="V82" s="2" t="n">
         <v>46382</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (11/07/2026 07:20)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -20,16 +20,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -48,21 +45,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -433,112 +421,112 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>linha</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>projeto_coordenador</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>projeto_atividade</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>situacao_consolidada</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>aprovado</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>acao</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>tramite</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>data_pedido</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>digito</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>rodada</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>preenchimento_tgco</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>observacao_coordenador</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>impactos_nao_atendimento</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>atividade</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>tarefa</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>valor</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>executora</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>nd</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>pacote</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>para_contrato</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>para_motores</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>mes_previsto</t>
         </is>
@@ -578,7 +566,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H2" s="2" t="n">
+      <c r="H2" s="1" t="n">
         <v>46076</v>
       </c>
       <c r="I2" t="inlineStr">
@@ -628,7 +616,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V2" s="2" t="n">
+      <c r="V2" s="1" t="n">
         <v>46079</v>
       </c>
     </row>
@@ -666,7 +654,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H3" s="2" t="n">
+      <c r="H3" s="1" t="n">
         <v>46076</v>
       </c>
       <c r="I3" t="inlineStr">
@@ -716,7 +704,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V3" s="2" t="n">
+      <c r="V3" s="1" t="n">
         <v>46079</v>
       </c>
     </row>
@@ -754,7 +742,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H4" s="2" t="n">
+      <c r="H4" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="I4" t="inlineStr">
@@ -808,7 +796,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V4" s="2" t="n">
+      <c r="V4" s="1" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -846,7 +834,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H5" s="2" t="n">
+      <c r="H5" s="1" t="n">
         <v>46119</v>
       </c>
       <c r="I5" t="inlineStr">
@@ -896,7 +884,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V5" s="2" t="n">
+      <c r="V5" s="1" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -934,7 +922,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H6" s="2" t="n">
+      <c r="H6" s="1" t="n">
         <v>46175</v>
       </c>
       <c r="I6" t="inlineStr">
@@ -984,7 +972,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V6" s="2" t="n">
+      <c r="V6" s="1" t="n">
         <v>46229</v>
       </c>
     </row>
@@ -1062,7 +1050,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V7" s="2" t="n">
+      <c r="V7" s="1" t="n">
         <v>46260</v>
       </c>
     </row>
@@ -1100,7 +1088,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H8" s="2" t="n">
+      <c r="H8" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="I8" t="inlineStr">
@@ -1150,7 +1138,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V8" s="2" t="n">
+      <c r="V8" s="1" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -1188,7 +1176,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H9" s="2" t="n">
+      <c r="H9" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="I9" t="inlineStr">
@@ -1238,7 +1226,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V9" s="2" t="n">
+      <c r="V9" s="1" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -1276,7 +1264,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H10" s="2" t="n">
+      <c r="H10" s="1" t="n">
         <v>46204</v>
       </c>
       <c r="I10" t="inlineStr">
@@ -1326,7 +1314,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V10" s="2" t="n">
+      <c r="V10" s="1" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -1364,7 +1352,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H11" s="2" t="n">
+      <c r="H11" s="1" t="n">
         <v>46191</v>
       </c>
       <c r="I11" t="inlineStr">
@@ -1414,7 +1402,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V11" s="2" t="n">
+      <c r="V11" s="1" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -1452,7 +1440,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H12" s="2" t="n">
+      <c r="H12" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="I12" t="inlineStr">
@@ -1502,7 +1490,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V12" s="2" t="n">
+      <c r="V12" s="1" t="n">
         <v>46229</v>
       </c>
     </row>
@@ -1540,7 +1528,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H13" s="2" t="n">
+      <c r="H13" s="1" t="n">
         <v>46176</v>
       </c>
       <c r="I13" t="inlineStr">
@@ -1594,7 +1582,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V13" s="2" t="n">
+      <c r="V13" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -1676,7 +1664,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V14" s="2" t="n">
+      <c r="V14" s="1" t="n">
         <v>46321</v>
       </c>
     </row>
@@ -1750,7 +1738,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V15" s="2" t="n">
+      <c r="V15" s="1" t="n">
         <v>46107</v>
       </c>
     </row>
@@ -1824,7 +1812,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V16" s="2" t="n">
+      <c r="V16" s="1" t="n">
         <v>46107</v>
       </c>
     </row>
@@ -1898,7 +1886,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V17" s="2" t="n">
+      <c r="V17" s="1" t="n">
         <v>46107</v>
       </c>
     </row>
@@ -1972,7 +1960,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V18" s="2" t="n">
+      <c r="V18" s="1" t="n">
         <v>46107</v>
       </c>
     </row>
@@ -2046,7 +2034,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V19" s="2" t="n">
+      <c r="V19" s="1" t="n">
         <v>46107</v>
       </c>
     </row>
@@ -2120,7 +2108,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V20" s="2" t="n">
+      <c r="V20" s="1" t="n">
         <v>46107</v>
       </c>
     </row>
@@ -2202,7 +2190,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V21" s="2" t="n">
+      <c r="V21" s="1" t="n">
         <v>46381</v>
       </c>
     </row>
@@ -2284,7 +2272,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V22" s="2" t="n">
+      <c r="V22" s="1" t="n">
         <v>46381</v>
       </c>
     </row>
@@ -2322,7 +2310,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H23" s="2" t="n">
+      <c r="H23" s="1" t="n">
         <v>46098</v>
       </c>
       <c r="I23" t="inlineStr">
@@ -2376,7 +2364,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V23" s="2" t="n">
+      <c r="V23" s="1" t="n">
         <v>46107</v>
       </c>
     </row>
@@ -2414,7 +2402,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H24" s="2" t="n">
+      <c r="H24" s="1" t="n">
         <v>46119</v>
       </c>
       <c r="I24" t="inlineStr">
@@ -2468,7 +2456,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V24" s="2" t="n">
+      <c r="V24" s="1" t="n">
         <v>46138</v>
       </c>
     </row>
@@ -2506,7 +2494,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H25" s="2" t="n">
+      <c r="H25" s="1" t="n">
         <v>46191</v>
       </c>
       <c r="I25" t="inlineStr">
@@ -2560,7 +2548,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V25" s="2" t="n">
+      <c r="V25" s="1" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -2646,7 +2634,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V26" s="2" t="n">
+      <c r="V26" s="1" t="n">
         <v>46229</v>
       </c>
     </row>
@@ -2732,7 +2720,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V27" s="2" t="n">
+      <c r="V27" s="1" t="n">
         <v>46260</v>
       </c>
     </row>
@@ -2818,7 +2806,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V28" s="2" t="n">
+      <c r="V28" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -2896,7 +2884,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V29" s="2" t="n">
+      <c r="V29" s="1" t="n">
         <v>46321</v>
       </c>
     </row>
@@ -2974,7 +2962,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V30" s="2" t="n">
+      <c r="V30" s="1" t="n">
         <v>46352</v>
       </c>
     </row>
@@ -3052,7 +3040,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V31" s="2" t="n">
+      <c r="V31" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -3090,7 +3078,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H32" s="2" t="n">
+      <c r="H32" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="I32" t="inlineStr">
@@ -3144,7 +3132,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V32" s="2" t="n">
+      <c r="V32" s="1" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -3182,7 +3170,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H33" s="2" t="n">
+      <c r="H33" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="I33" t="inlineStr">
@@ -3236,7 +3224,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V33" s="2" t="n">
+      <c r="V33" s="1" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -3274,7 +3262,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H34" s="2" t="n">
+      <c r="H34" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="I34" t="inlineStr">
@@ -3328,7 +3316,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V34" s="2" t="n">
+      <c r="V34" s="1" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -3410,7 +3398,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V35" s="2" t="n">
+      <c r="V35" s="1" t="n">
         <v>46381</v>
       </c>
     </row>
@@ -3492,7 +3480,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V36" s="2" t="n">
+      <c r="V36" s="1" t="n">
         <v>46381</v>
       </c>
     </row>
@@ -3530,7 +3518,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H37" s="2" t="n">
+      <c r="H37" s="1" t="n">
         <v>46121</v>
       </c>
       <c r="I37" t="inlineStr">
@@ -3580,7 +3568,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V37" s="2" t="n">
+      <c r="V37" s="1" t="n">
         <v>46107</v>
       </c>
     </row>
@@ -3618,7 +3606,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H38" s="2" t="n">
+      <c r="H38" s="1" t="n">
         <v>46076</v>
       </c>
       <c r="I38" t="inlineStr">
@@ -3668,7 +3656,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V38" s="2" t="n">
+      <c r="V38" s="1" t="n">
         <v>46079</v>
       </c>
     </row>
@@ -3706,7 +3694,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H39" s="2" t="n">
+      <c r="H39" s="1" t="n">
         <v>46191</v>
       </c>
       <c r="I39" t="inlineStr">
@@ -3756,7 +3744,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V39" s="2" t="n">
+      <c r="V39" s="1" t="n">
         <v>46199</v>
       </c>
     </row>
@@ -3834,7 +3822,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V40" s="2" t="n">
+      <c r="V40" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -3912,7 +3900,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V41" s="2" t="n">
+      <c r="V41" s="1" t="n">
         <v>46260</v>
       </c>
     </row>
@@ -3990,7 +3978,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V42" s="2" t="n">
+      <c r="V42" s="1" t="n">
         <v>46321</v>
       </c>
     </row>
@@ -4028,7 +4016,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H43" s="2" t="n">
+      <c r="H43" s="1" t="n">
         <v>46121</v>
       </c>
       <c r="I43" t="inlineStr">
@@ -4078,7 +4066,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V43" s="2" t="n">
+      <c r="V43" s="1" t="n">
         <v>46168</v>
       </c>
     </row>
@@ -4156,7 +4144,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V44" s="2" t="n">
+      <c r="V44" s="1" t="n">
         <v>46260</v>
       </c>
     </row>
@@ -4232,7 +4220,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V45" s="2" t="n">
+      <c r="V45" s="1" t="n">
         <v>46260</v>
       </c>
     </row>
@@ -4314,7 +4302,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V46" s="2" t="n">
+      <c r="V46" s="1" t="n">
         <v>46229</v>
       </c>
     </row>
@@ -4392,7 +4380,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V47" s="2" t="n">
+      <c r="V47" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -4470,7 +4458,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V48" s="2" t="n">
+      <c r="V48" s="1" t="n">
         <v>46321</v>
       </c>
     </row>
@@ -4548,7 +4536,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V49" s="2" t="n">
+      <c r="V49" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -4586,7 +4574,7 @@
           <t>ATENDIDO</t>
         </is>
       </c>
-      <c r="H50" s="2" t="n">
+      <c r="H50" s="1" t="n">
         <v>46079</v>
       </c>
       <c r="I50" t="inlineStr">
@@ -4640,7 +4628,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V50" s="2" t="n">
+      <c r="V50" s="1" t="n">
         <v>46107</v>
       </c>
     </row>
@@ -4718,7 +4706,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V51" s="2" t="n">
+      <c r="V51" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -4796,7 +4784,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V52" s="2" t="n">
+      <c r="V52" s="1" t="n">
         <v>46352</v>
       </c>
     </row>
@@ -4870,7 +4858,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V53" s="2" t="n">
+      <c r="V53" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -4948,7 +4936,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V54" s="2" t="n">
+      <c r="V54" s="1" t="n">
         <v>46352</v>
       </c>
     </row>
@@ -5022,7 +5010,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V55" s="2" t="n">
+      <c r="V55" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -5100,7 +5088,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V56" s="2" t="n">
+      <c r="V56" s="1" t="n">
         <v>46352</v>
       </c>
     </row>
@@ -5174,7 +5162,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V57" s="2" t="n">
+      <c r="V57" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -5252,7 +5240,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V58" s="2" t="n">
+      <c r="V58" s="1" t="n">
         <v>46229</v>
       </c>
     </row>
@@ -5330,7 +5318,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V59" s="2" t="n">
+      <c r="V59" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -5408,7 +5396,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V60" s="2" t="n">
+      <c r="V60" s="1" t="n">
         <v>46229</v>
       </c>
     </row>
@@ -5482,7 +5470,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V61" s="2" t="n">
+      <c r="V61" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -5560,7 +5548,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V62" s="2" t="n">
+      <c r="V62" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -5642,7 +5630,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V63" s="2" t="n">
+      <c r="V63" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -5720,7 +5708,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V64" s="2" t="n">
+      <c r="V64" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -5798,7 +5786,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V65" s="2" t="n">
+      <c r="V65" s="1" t="n">
         <v>46321</v>
       </c>
     </row>
@@ -5872,7 +5860,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V66" s="2" t="n">
+      <c r="V66" s="1" t="n">
         <v>46168</v>
       </c>
     </row>
@@ -5950,7 +5938,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V67" s="2" t="n">
+      <c r="V67" s="1" t="n">
         <v>46321</v>
       </c>
     </row>
@@ -6024,7 +6012,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V68" s="2" t="n">
+      <c r="V68" s="1" t="n">
         <v>46260</v>
       </c>
     </row>
@@ -6102,7 +6090,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V69" s="2" t="n">
+      <c r="V69" s="1" t="n">
         <v>46260</v>
       </c>
     </row>
@@ -6180,7 +6168,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V70" s="2" t="n">
+      <c r="V70" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -6258,7 +6246,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V71" s="2" t="n">
+      <c r="V71" s="1" t="n">
         <v>46260</v>
       </c>
     </row>
@@ -6336,7 +6324,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V72" s="2" t="n">
+      <c r="V72" s="1" t="n">
         <v>46291</v>
       </c>
     </row>
@@ -6414,7 +6402,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V73" s="2" t="n">
+      <c r="V73" s="1" t="n">
         <v>46321</v>
       </c>
     </row>
@@ -6492,7 +6480,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V74" s="2" t="n">
+      <c r="V74" s="1" t="n">
         <v>46049</v>
       </c>
     </row>
@@ -6718,7 +6706,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V77" s="2" t="n">
+      <c r="V77" s="1" t="n">
         <v>46168</v>
       </c>
     </row>
@@ -6792,7 +6780,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V78" s="2" t="n">
+      <c r="V78" s="1" t="n">
         <v>46382</v>
       </c>
     </row>
@@ -6866,7 +6854,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V79" s="2" t="n">
+      <c r="V79" s="1" t="n">
         <v>46382</v>
       </c>
     </row>
@@ -6944,7 +6932,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="V80" s="2" t="n">
+      <c r="V80" s="1" t="n">
         <v>46382</v>
       </c>
     </row>
@@ -7018,7 +7006,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V81" s="2" t="n">
+      <c r="V81" s="1" t="n">
         <v>46321</v>
       </c>
     </row>
@@ -7092,7 +7080,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="V82" s="2" t="n">
+      <c r="V82" s="1" t="n">
         <v>46382</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (14/07/2026 16:04)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -992,7 +992,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Aprovado, aguardando atendimento</t>
+          <t>Em trâmite</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1005,8 +1005,14 @@
           <t>2048</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>EM TRÂMITE</t>
+        </is>
+      </c>
+      <c r="H7" s="1" t="n">
+        <v>46213</v>
+      </c>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
@@ -2568,7 +2574,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Aprovado, aguardando atendimento</t>
+          <t>Em trâmite</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2581,8 +2587,14 @@
           <t>2048</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>EM TRÂMITE</t>
+        </is>
+      </c>
+      <c r="H26" s="1" t="n">
+        <v>46213</v>
+      </c>
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr">
         <is>
@@ -4086,7 +4098,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Aprovado, aguardando atendimento</t>
+          <t>Em trâmite</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -4099,8 +4111,14 @@
           <t>2048</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr"/>
-      <c r="H44" t="inlineStr"/>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>EM TRÂMITE</t>
+        </is>
+      </c>
+      <c r="H44" s="1" t="n">
+        <v>46213</v>
+      </c>
       <c r="I44" t="inlineStr"/>
       <c r="J44" t="inlineStr"/>
       <c r="K44" t="inlineStr"/>

</xml_diff>

<commit_message>
Atualização automática: mta (22/07/2026 16:09)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -527,16 +527,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -552,7 +544,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -560,30 +552,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -883,70 +857,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -996,7 +970,7 @@
       <c r="U2" t="s">
         <v>167</v>
       </c>
-      <c r="V2" s="2">
+      <c r="V2" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1043,7 +1017,7 @@
       <c r="U3" t="s">
         <v>28</v>
       </c>
-      <c r="V3" s="2">
+      <c r="V3" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1090,7 +1064,7 @@
       <c r="U4" t="s">
         <v>28</v>
       </c>
-      <c r="V4" s="2">
+      <c r="V4" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -1137,7 +1111,7 @@
       <c r="U5" t="s">
         <v>28</v>
       </c>
-      <c r="V5" s="2">
+      <c r="V5" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -1187,7 +1161,7 @@
       <c r="U6" t="s">
         <v>28</v>
       </c>
-      <c r="V6" s="2">
+      <c r="V6" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1213,7 +1187,7 @@
       <c r="G7" t="s">
         <v>40</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1243,7 +1217,7 @@
       <c r="U7" t="s">
         <v>28</v>
       </c>
-      <c r="V7" s="2">
+      <c r="V7" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -1290,7 +1264,7 @@
       <c r="U8" t="s">
         <v>28</v>
       </c>
-      <c r="V8" s="2">
+      <c r="V8" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1337,7 +1311,7 @@
       <c r="U9" t="s">
         <v>28</v>
       </c>
-      <c r="V9" s="2">
+      <c r="V9" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1384,7 +1358,7 @@
       <c r="U10" t="s">
         <v>28</v>
       </c>
-      <c r="V10" s="2">
+      <c r="V10" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1431,7 +1405,7 @@
       <c r="U11" t="s">
         <v>28</v>
       </c>
-      <c r="V11" s="2">
+      <c r="V11" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1457,7 +1431,7 @@
       <c r="G12" t="s">
         <v>40</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46079</v>
       </c>
       <c r="I12" t="s">
@@ -1490,7 +1464,7 @@
       <c r="U12" t="s">
         <v>167</v>
       </c>
-      <c r="V12" s="2">
+      <c r="V12" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -1537,7 +1511,7 @@
       <c r="U13" t="s">
         <v>167</v>
       </c>
-      <c r="V13" s="2">
+      <c r="V13" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1584,7 +1558,7 @@
       <c r="U14" t="s">
         <v>167</v>
       </c>
-      <c r="V14" s="2">
+      <c r="V14" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1631,7 +1605,7 @@
       <c r="U15" t="s">
         <v>167</v>
       </c>
-      <c r="V15" s="2">
+      <c r="V15" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1678,7 +1652,7 @@
       <c r="U16" t="s">
         <v>167</v>
       </c>
-      <c r="V16" s="2">
+      <c r="V16" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1704,7 +1678,7 @@
       <c r="G17" t="s">
         <v>40</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46098</v>
       </c>
       <c r="I17" t="s">
@@ -1737,7 +1711,7 @@
       <c r="U17" t="s">
         <v>167</v>
       </c>
-      <c r="V17" s="2">
+      <c r="V17" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -1763,7 +1737,7 @@
       <c r="G18" t="s">
         <v>40</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46076</v>
       </c>
       <c r="I18" t="s">
@@ -1793,7 +1767,7 @@
       <c r="U18" t="s">
         <v>28</v>
       </c>
-      <c r="V18" s="2">
+      <c r="V18" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1819,7 +1793,7 @@
       <c r="G19" t="s">
         <v>40</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1849,7 +1823,7 @@
       <c r="U19" t="s">
         <v>28</v>
       </c>
-      <c r="V19" s="2">
+      <c r="V19" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1896,7 +1870,7 @@
       <c r="U20" t="s">
         <v>28</v>
       </c>
-      <c r="V20" s="2">
+      <c r="V20" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1943,7 +1917,7 @@
       <c r="U21" t="s">
         <v>28</v>
       </c>
-      <c r="V21" s="2">
+      <c r="V21" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1990,7 +1964,7 @@
       <c r="U22" t="s">
         <v>28</v>
       </c>
-      <c r="V22" s="2">
+      <c r="V22" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2037,7 +2011,7 @@
       <c r="U23" t="s">
         <v>28</v>
       </c>
-      <c r="V23" s="2">
+      <c r="V23" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2063,7 +2037,7 @@
       <c r="G24" t="s">
         <v>40</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>46119</v>
       </c>
       <c r="I24" t="s">
@@ -2096,7 +2070,7 @@
       <c r="U24" t="s">
         <v>167</v>
       </c>
-      <c r="V24" s="2">
+      <c r="V24" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2122,7 +2096,7 @@
       <c r="G25" t="s">
         <v>40</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>46121</v>
       </c>
       <c r="I25" t="s">
@@ -2152,7 +2126,7 @@
       <c r="U25" t="s">
         <v>28</v>
       </c>
-      <c r="V25" s="2">
+      <c r="V25" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -2178,7 +2152,7 @@
       <c r="G26" t="s">
         <v>40</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>46076</v>
       </c>
       <c r="I26" t="s">
@@ -2208,7 +2182,7 @@
       <c r="U26" t="s">
         <v>28</v>
       </c>
-      <c r="V26" s="2">
+      <c r="V26" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -2255,7 +2229,7 @@
       <c r="U27" t="s">
         <v>167</v>
       </c>
-      <c r="V27" s="2">
+      <c r="V27" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2281,7 +2255,7 @@
       <c r="G28" t="s">
         <v>40</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>46199</v>
       </c>
       <c r="I28" t="s">
@@ -2314,7 +2288,7 @@
       <c r="U28" t="s">
         <v>167</v>
       </c>
-      <c r="V28" s="2">
+      <c r="V28" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2340,7 +2314,7 @@
       <c r="G29" t="s">
         <v>40</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2373,7 +2347,7 @@
       <c r="U29" t="s">
         <v>167</v>
       </c>
-      <c r="V29" s="2">
+      <c r="V29" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2399,7 +2373,7 @@
       <c r="G30" t="s">
         <v>40</v>
       </c>
-      <c r="H30" s="2">
+      <c r="H30" s="1">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2432,7 +2406,7 @@
       <c r="U30" t="s">
         <v>167</v>
       </c>
-      <c r="V30" s="2">
+      <c r="V30" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2458,7 +2432,7 @@
       <c r="G31" t="s">
         <v>40</v>
       </c>
-      <c r="H31" s="2">
+      <c r="H31" s="1">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2491,7 +2465,7 @@
       <c r="U31" t="s">
         <v>167</v>
       </c>
-      <c r="V31" s="2">
+      <c r="V31" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2538,7 +2512,7 @@
       <c r="U32" t="s">
         <v>167</v>
       </c>
-      <c r="V32" s="2">
+      <c r="V32" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2564,7 +2538,7 @@
       <c r="G33" t="s">
         <v>40</v>
       </c>
-      <c r="H33" s="2">
+      <c r="H33" s="1">
         <v>46191</v>
       </c>
       <c r="I33" t="s">
@@ -2597,7 +2571,7 @@
       <c r="U33" t="s">
         <v>167</v>
       </c>
-      <c r="V33" s="2">
+      <c r="V33" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2623,7 +2597,7 @@
       <c r="G34" t="s">
         <v>40</v>
       </c>
-      <c r="H34" s="2">
+      <c r="H34" s="1">
         <v>46119</v>
       </c>
       <c r="I34" t="s">
@@ -2653,7 +2627,7 @@
       <c r="U34" t="s">
         <v>167</v>
       </c>
-      <c r="V34" s="2">
+      <c r="V34" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2679,7 +2653,7 @@
       <c r="G35" t="s">
         <v>41</v>
       </c>
-      <c r="H35" s="2">
+      <c r="H35" s="1">
         <v>46213</v>
       </c>
       <c r="N35" t="s">
@@ -2706,7 +2680,7 @@
       <c r="U35" t="s">
         <v>28</v>
       </c>
-      <c r="V35" s="2">
+      <c r="V35" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -2732,7 +2706,7 @@
       <c r="G36" t="s">
         <v>40</v>
       </c>
-      <c r="H36" s="2">
+      <c r="H36" s="1">
         <v>46175</v>
       </c>
       <c r="I36" t="s">
@@ -2762,7 +2736,7 @@
       <c r="U36" t="s">
         <v>28</v>
       </c>
-      <c r="V36" s="2">
+      <c r="V36" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -2788,7 +2762,7 @@
       <c r="G37" t="s">
         <v>41</v>
       </c>
-      <c r="H37" s="2">
+      <c r="H37" s="1">
         <v>46213</v>
       </c>
       <c r="N37" t="s">
@@ -2815,7 +2789,7 @@
       <c r="U37" t="s">
         <v>28</v>
       </c>
-      <c r="V37" s="2">
+      <c r="V37" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -2841,7 +2815,7 @@
       <c r="G38" t="s">
         <v>40</v>
       </c>
-      <c r="H38" s="2">
+      <c r="H38" s="1">
         <v>46199</v>
       </c>
       <c r="I38" t="s">
@@ -2871,7 +2845,7 @@
       <c r="U38" t="s">
         <v>28</v>
       </c>
-      <c r="V38" s="2">
+      <c r="V38" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2897,7 +2871,7 @@
       <c r="G39" t="s">
         <v>40</v>
       </c>
-      <c r="H39" s="2">
+      <c r="H39" s="1">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -2927,7 +2901,7 @@
       <c r="U39" t="s">
         <v>28</v>
       </c>
-      <c r="V39" s="2">
+      <c r="V39" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2953,7 +2927,7 @@
       <c r="G40" t="s">
         <v>40</v>
       </c>
-      <c r="H40" s="2">
+      <c r="H40" s="1">
         <v>46204</v>
       </c>
       <c r="I40" t="s">
@@ -2983,7 +2957,7 @@
       <c r="U40" t="s">
         <v>28</v>
       </c>
-      <c r="V40" s="2">
+      <c r="V40" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3027,7 +3001,7 @@
       <c r="U41" t="s">
         <v>28</v>
       </c>
-      <c r="V41" s="2">
+      <c r="V41" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3053,7 +3027,7 @@
       <c r="G42" t="s">
         <v>40</v>
       </c>
-      <c r="H42" s="2">
+      <c r="H42" s="1">
         <v>46191</v>
       </c>
       <c r="I42" t="s">
@@ -3083,7 +3057,7 @@
       <c r="U42" t="s">
         <v>28</v>
       </c>
-      <c r="V42" s="2">
+      <c r="V42" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3109,7 +3083,7 @@
       <c r="G43" t="s">
         <v>40</v>
       </c>
-      <c r="H43" s="2">
+      <c r="H43" s="1">
         <v>46191</v>
       </c>
       <c r="I43" t="s">
@@ -3139,7 +3113,7 @@
       <c r="U43" t="s">
         <v>28</v>
       </c>
-      <c r="V43" s="2">
+      <c r="V43" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3165,7 +3139,7 @@
       <c r="G44" t="s">
         <v>41</v>
       </c>
-      <c r="H44" s="2">
+      <c r="H44" s="1">
         <v>46213</v>
       </c>
       <c r="J44" t="s">
@@ -3198,7 +3172,7 @@
       <c r="U44" t="s">
         <v>167</v>
       </c>
-      <c r="V44" s="2">
+      <c r="V44" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3224,7 +3198,7 @@
       <c r="G45" t="s">
         <v>40</v>
       </c>
-      <c r="H45" s="2">
+      <c r="H45" s="1">
         <v>46210</v>
       </c>
       <c r="I45" t="s">
@@ -3254,7 +3228,7 @@
       <c r="U45" t="s">
         <v>167</v>
       </c>
-      <c r="V45" s="2">
+      <c r="V45" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3301,7 +3275,7 @@
       <c r="U46" t="s">
         <v>28</v>
       </c>
-      <c r="V46" s="2">
+      <c r="V46" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3348,7 +3322,7 @@
       <c r="U47" t="s">
         <v>167</v>
       </c>
-      <c r="V47" s="2">
+      <c r="V47" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3374,7 +3348,7 @@
       <c r="G48" t="s">
         <v>40</v>
       </c>
-      <c r="H48" s="2">
+      <c r="H48" s="1">
         <v>46176</v>
       </c>
       <c r="I48" t="s">
@@ -3407,7 +3381,7 @@
       <c r="U48" t="s">
         <v>167</v>
       </c>
-      <c r="V48" s="2">
+      <c r="V48" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3460,7 +3434,7 @@
       <c r="U49" t="s">
         <v>167</v>
       </c>
-      <c r="V49" s="2">
+      <c r="V49" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3513,7 +3487,7 @@
       <c r="U50" t="s">
         <v>167</v>
       </c>
-      <c r="V50" s="2">
+      <c r="V50" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3560,7 +3534,7 @@
       <c r="U51" t="s">
         <v>167</v>
       </c>
-      <c r="V51" s="2">
+      <c r="V51" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3607,7 +3581,7 @@
       <c r="U52" t="s">
         <v>167</v>
       </c>
-      <c r="V52" s="2">
+      <c r="V52" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -3654,7 +3628,7 @@
       <c r="U53" t="s">
         <v>167</v>
       </c>
-      <c r="V53" s="2">
+      <c r="V53" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3704,7 +3678,7 @@
       <c r="U54" t="s">
         <v>167</v>
       </c>
-      <c r="V54" s="2">
+      <c r="V54" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3751,7 +3725,7 @@
       <c r="U55" t="s">
         <v>167</v>
       </c>
-      <c r="V55" s="2">
+      <c r="V55" s="1">
         <v>46049</v>
       </c>
     </row>
@@ -3883,7 +3857,7 @@
       <c r="U58" t="s">
         <v>167</v>
       </c>
-      <c r="V58" s="2">
+      <c r="V58" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -3927,7 +3901,7 @@
       <c r="U59" t="s">
         <v>167</v>
       </c>
-      <c r="V59" s="2">
+      <c r="V59" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -3971,7 +3945,7 @@
       <c r="U60" t="s">
         <v>167</v>
       </c>
-      <c r="V60" s="2">
+      <c r="V60" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4015,7 +3989,7 @@
       <c r="U61" t="s">
         <v>167</v>
       </c>
-      <c r="V61" s="2">
+      <c r="V61" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4059,7 +4033,7 @@
       <c r="U62" t="s">
         <v>167</v>
       </c>
-      <c r="V62" s="2">
+      <c r="V62" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4103,7 +4077,7 @@
       <c r="U63" t="s">
         <v>167</v>
       </c>
-      <c r="V63" s="2">
+      <c r="V63" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4147,7 +4121,7 @@
       <c r="U64" t="s">
         <v>28</v>
       </c>
-      <c r="V64" s="2">
+      <c r="V64" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4194,7 +4168,7 @@
       <c r="U65" t="s">
         <v>28</v>
       </c>
-      <c r="V65" s="2">
+      <c r="V65" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4241,7 +4215,7 @@
       <c r="U66" t="s">
         <v>167</v>
       </c>
-      <c r="V66" s="2">
+      <c r="V66" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -4285,7 +4259,7 @@
       <c r="U67" t="s">
         <v>28</v>
       </c>
-      <c r="V67" s="2">
+      <c r="V67" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -4329,7 +4303,7 @@
       <c r="U68" t="s">
         <v>167</v>
       </c>
-      <c r="V68" s="2">
+      <c r="V68" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4373,7 +4347,7 @@
       <c r="U69" t="s">
         <v>167</v>
       </c>
-      <c r="V69" s="2">
+      <c r="V69" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4417,7 +4391,7 @@
       <c r="U70" t="s">
         <v>167</v>
       </c>
-      <c r="V70" s="2">
+      <c r="V70" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4461,7 +4435,7 @@
       <c r="U71" t="s">
         <v>167</v>
       </c>
-      <c r="V71" s="2">
+      <c r="V71" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4505,7 +4479,7 @@
       <c r="U72" t="s">
         <v>167</v>
       </c>
-      <c r="V72" s="2">
+      <c r="V72" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4552,7 +4526,7 @@
       <c r="U73" t="s">
         <v>28</v>
       </c>
-      <c r="V73" s="2">
+      <c r="V73" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -4602,7 +4576,7 @@
       <c r="U74" t="s">
         <v>167</v>
       </c>
-      <c r="V74" s="2">
+      <c r="V74" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4652,7 +4626,7 @@
       <c r="U75" t="s">
         <v>167</v>
       </c>
-      <c r="V75" s="2">
+      <c r="V75" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4702,7 +4676,7 @@
       <c r="U76" t="s">
         <v>28</v>
       </c>
-      <c r="V76" s="2">
+      <c r="V76" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4752,7 +4726,7 @@
       <c r="U77" t="s">
         <v>28</v>
       </c>
-      <c r="V77" s="2">
+      <c r="V77" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4796,7 +4770,7 @@
       <c r="U78" t="s">
         <v>28</v>
       </c>
-      <c r="V78" s="2">
+      <c r="V78" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -4840,7 +4814,7 @@
       <c r="U79" t="s">
         <v>28</v>
       </c>
-      <c r="V79" s="2">
+      <c r="V79" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -4887,7 +4861,7 @@
       <c r="U80" t="s">
         <v>167</v>
       </c>
-      <c r="V80" s="2">
+      <c r="V80" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -4931,7 +4905,7 @@
       <c r="U81" t="s">
         <v>28</v>
       </c>
-      <c r="V81" s="2">
+      <c r="V81" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -4975,7 +4949,7 @@
       <c r="U82" t="s">
         <v>28</v>
       </c>
-      <c r="V82" s="2">
+      <c r="V82" s="1">
         <v>46382</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (23/07/2026 11:41)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -527,8 +527,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -544,7 +552,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -552,12 +560,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -857,70 +883,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -970,7 +996,7 @@
       <c r="U2" t="s">
         <v>167</v>
       </c>
-      <c r="V2" s="1">
+      <c r="V2" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -1017,7 +1043,7 @@
       <c r="U3" t="s">
         <v>28</v>
       </c>
-      <c r="V3" s="1">
+      <c r="V3" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1064,7 +1090,7 @@
       <c r="U4" t="s">
         <v>28</v>
       </c>
-      <c r="V4" s="1">
+      <c r="V4" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -1111,7 +1137,7 @@
       <c r="U5" t="s">
         <v>28</v>
       </c>
-      <c r="V5" s="1">
+      <c r="V5" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -1161,7 +1187,7 @@
       <c r="U6" t="s">
         <v>28</v>
       </c>
-      <c r="V6" s="1">
+      <c r="V6" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1187,7 +1213,7 @@
       <c r="G7" t="s">
         <v>40</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1217,7 +1243,7 @@
       <c r="U7" t="s">
         <v>28</v>
       </c>
-      <c r="V7" s="1">
+      <c r="V7" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -1264,7 +1290,7 @@
       <c r="U8" t="s">
         <v>28</v>
       </c>
-      <c r="V8" s="1">
+      <c r="V8" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1311,7 +1337,7 @@
       <c r="U9" t="s">
         <v>28</v>
       </c>
-      <c r="V9" s="1">
+      <c r="V9" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1358,7 +1384,7 @@
       <c r="U10" t="s">
         <v>28</v>
       </c>
-      <c r="V10" s="1">
+      <c r="V10" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1405,7 +1431,7 @@
       <c r="U11" t="s">
         <v>28</v>
       </c>
-      <c r="V11" s="1">
+      <c r="V11" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1431,7 +1457,7 @@
       <c r="G12" t="s">
         <v>40</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46079</v>
       </c>
       <c r="I12" t="s">
@@ -1464,7 +1490,7 @@
       <c r="U12" t="s">
         <v>167</v>
       </c>
-      <c r="V12" s="1">
+      <c r="V12" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -1511,7 +1537,7 @@
       <c r="U13" t="s">
         <v>167</v>
       </c>
-      <c r="V13" s="1">
+      <c r="V13" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1558,7 +1584,7 @@
       <c r="U14" t="s">
         <v>167</v>
       </c>
-      <c r="V14" s="1">
+      <c r="V14" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1605,7 +1631,7 @@
       <c r="U15" t="s">
         <v>167</v>
       </c>
-      <c r="V15" s="1">
+      <c r="V15" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1652,7 +1678,7 @@
       <c r="U16" t="s">
         <v>167</v>
       </c>
-      <c r="V16" s="1">
+      <c r="V16" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -1678,7 +1704,7 @@
       <c r="G17" t="s">
         <v>40</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46098</v>
       </c>
       <c r="I17" t="s">
@@ -1711,7 +1737,7 @@
       <c r="U17" t="s">
         <v>167</v>
       </c>
-      <c r="V17" s="1">
+      <c r="V17" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -1737,7 +1763,7 @@
       <c r="G18" t="s">
         <v>40</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46076</v>
       </c>
       <c r="I18" t="s">
@@ -1767,7 +1793,7 @@
       <c r="U18" t="s">
         <v>28</v>
       </c>
-      <c r="V18" s="1">
+      <c r="V18" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1793,7 +1819,7 @@
       <c r="G19" t="s">
         <v>40</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1823,7 +1849,7 @@
       <c r="U19" t="s">
         <v>28</v>
       </c>
-      <c r="V19" s="1">
+      <c r="V19" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1870,7 +1896,7 @@
       <c r="U20" t="s">
         <v>28</v>
       </c>
-      <c r="V20" s="1">
+      <c r="V20" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1917,7 +1943,7 @@
       <c r="U21" t="s">
         <v>28</v>
       </c>
-      <c r="V21" s="1">
+      <c r="V21" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1964,7 +1990,7 @@
       <c r="U22" t="s">
         <v>28</v>
       </c>
-      <c r="V22" s="1">
+      <c r="V22" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2011,7 +2037,7 @@
       <c r="U23" t="s">
         <v>28</v>
       </c>
-      <c r="V23" s="1">
+      <c r="V23" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2037,7 +2063,7 @@
       <c r="G24" t="s">
         <v>40</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>46119</v>
       </c>
       <c r="I24" t="s">
@@ -2070,7 +2096,7 @@
       <c r="U24" t="s">
         <v>167</v>
       </c>
-      <c r="V24" s="1">
+      <c r="V24" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2096,7 +2122,7 @@
       <c r="G25" t="s">
         <v>40</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>46121</v>
       </c>
       <c r="I25" t="s">
@@ -2126,7 +2152,7 @@
       <c r="U25" t="s">
         <v>28</v>
       </c>
-      <c r="V25" s="1">
+      <c r="V25" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -2152,7 +2178,7 @@
       <c r="G26" t="s">
         <v>40</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>46076</v>
       </c>
       <c r="I26" t="s">
@@ -2182,7 +2208,7 @@
       <c r="U26" t="s">
         <v>28</v>
       </c>
-      <c r="V26" s="1">
+      <c r="V26" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -2229,7 +2255,7 @@
       <c r="U27" t="s">
         <v>167</v>
       </c>
-      <c r="V27" s="1">
+      <c r="V27" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -2255,7 +2281,7 @@
       <c r="G28" t="s">
         <v>40</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>46199</v>
       </c>
       <c r="I28" t="s">
@@ -2288,7 +2314,7 @@
       <c r="U28" t="s">
         <v>167</v>
       </c>
-      <c r="V28" s="1">
+      <c r="V28" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2314,7 +2340,7 @@
       <c r="G29" t="s">
         <v>40</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2347,7 +2373,7 @@
       <c r="U29" t="s">
         <v>167</v>
       </c>
-      <c r="V29" s="1">
+      <c r="V29" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2373,7 +2399,7 @@
       <c r="G30" t="s">
         <v>40</v>
       </c>
-      <c r="H30" s="1">
+      <c r="H30" s="2">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2406,7 +2432,7 @@
       <c r="U30" t="s">
         <v>167</v>
       </c>
-      <c r="V30" s="1">
+      <c r="V30" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2432,7 +2458,7 @@
       <c r="G31" t="s">
         <v>40</v>
       </c>
-      <c r="H31" s="1">
+      <c r="H31" s="2">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2465,7 +2491,7 @@
       <c r="U31" t="s">
         <v>167</v>
       </c>
-      <c r="V31" s="1">
+      <c r="V31" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2512,7 +2538,7 @@
       <c r="U32" t="s">
         <v>167</v>
       </c>
-      <c r="V32" s="1">
+      <c r="V32" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -2538,7 +2564,7 @@
       <c r="G33" t="s">
         <v>40</v>
       </c>
-      <c r="H33" s="1">
+      <c r="H33" s="2">
         <v>46191</v>
       </c>
       <c r="I33" t="s">
@@ -2571,7 +2597,7 @@
       <c r="U33" t="s">
         <v>167</v>
       </c>
-      <c r="V33" s="1">
+      <c r="V33" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2597,7 +2623,7 @@
       <c r="G34" t="s">
         <v>40</v>
       </c>
-      <c r="H34" s="1">
+      <c r="H34" s="2">
         <v>46119</v>
       </c>
       <c r="I34" t="s">
@@ -2627,7 +2653,7 @@
       <c r="U34" t="s">
         <v>167</v>
       </c>
-      <c r="V34" s="1">
+      <c r="V34" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2653,7 +2679,7 @@
       <c r="G35" t="s">
         <v>41</v>
       </c>
-      <c r="H35" s="1">
+      <c r="H35" s="2">
         <v>46213</v>
       </c>
       <c r="N35" t="s">
@@ -2680,7 +2706,7 @@
       <c r="U35" t="s">
         <v>28</v>
       </c>
-      <c r="V35" s="1">
+      <c r="V35" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -2706,7 +2732,7 @@
       <c r="G36" t="s">
         <v>40</v>
       </c>
-      <c r="H36" s="1">
+      <c r="H36" s="2">
         <v>46175</v>
       </c>
       <c r="I36" t="s">
@@ -2736,7 +2762,7 @@
       <c r="U36" t="s">
         <v>28</v>
       </c>
-      <c r="V36" s="1">
+      <c r="V36" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -2762,7 +2788,7 @@
       <c r="G37" t="s">
         <v>41</v>
       </c>
-      <c r="H37" s="1">
+      <c r="H37" s="2">
         <v>46213</v>
       </c>
       <c r="N37" t="s">
@@ -2789,7 +2815,7 @@
       <c r="U37" t="s">
         <v>28</v>
       </c>
-      <c r="V37" s="1">
+      <c r="V37" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -2815,7 +2841,7 @@
       <c r="G38" t="s">
         <v>40</v>
       </c>
-      <c r="H38" s="1">
+      <c r="H38" s="2">
         <v>46199</v>
       </c>
       <c r="I38" t="s">
@@ -2845,7 +2871,7 @@
       <c r="U38" t="s">
         <v>28</v>
       </c>
-      <c r="V38" s="1">
+      <c r="V38" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2871,7 +2897,7 @@
       <c r="G39" t="s">
         <v>40</v>
       </c>
-      <c r="H39" s="1">
+      <c r="H39" s="2">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -2901,7 +2927,7 @@
       <c r="U39" t="s">
         <v>28</v>
       </c>
-      <c r="V39" s="1">
+      <c r="V39" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2927,7 +2953,7 @@
       <c r="G40" t="s">
         <v>40</v>
       </c>
-      <c r="H40" s="1">
+      <c r="H40" s="2">
         <v>46204</v>
       </c>
       <c r="I40" t="s">
@@ -2957,7 +2983,7 @@
       <c r="U40" t="s">
         <v>28</v>
       </c>
-      <c r="V40" s="1">
+      <c r="V40" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3001,7 +3027,7 @@
       <c r="U41" t="s">
         <v>28</v>
       </c>
-      <c r="V41" s="1">
+      <c r="V41" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3027,7 +3053,7 @@
       <c r="G42" t="s">
         <v>40</v>
       </c>
-      <c r="H42" s="1">
+      <c r="H42" s="2">
         <v>46191</v>
       </c>
       <c r="I42" t="s">
@@ -3057,7 +3083,7 @@
       <c r="U42" t="s">
         <v>28</v>
       </c>
-      <c r="V42" s="1">
+      <c r="V42" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3083,7 +3109,7 @@
       <c r="G43" t="s">
         <v>40</v>
       </c>
-      <c r="H43" s="1">
+      <c r="H43" s="2">
         <v>46191</v>
       </c>
       <c r="I43" t="s">
@@ -3113,7 +3139,7 @@
       <c r="U43" t="s">
         <v>28</v>
       </c>
-      <c r="V43" s="1">
+      <c r="V43" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3139,7 +3165,7 @@
       <c r="G44" t="s">
         <v>41</v>
       </c>
-      <c r="H44" s="1">
+      <c r="H44" s="2">
         <v>46213</v>
       </c>
       <c r="J44" t="s">
@@ -3172,7 +3198,7 @@
       <c r="U44" t="s">
         <v>167</v>
       </c>
-      <c r="V44" s="1">
+      <c r="V44" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3198,7 +3224,7 @@
       <c r="G45" t="s">
         <v>40</v>
       </c>
-      <c r="H45" s="1">
+      <c r="H45" s="2">
         <v>46210</v>
       </c>
       <c r="I45" t="s">
@@ -3228,7 +3254,7 @@
       <c r="U45" t="s">
         <v>167</v>
       </c>
-      <c r="V45" s="1">
+      <c r="V45" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3275,7 +3301,7 @@
       <c r="U46" t="s">
         <v>28</v>
       </c>
-      <c r="V46" s="1">
+      <c r="V46" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3322,7 +3348,7 @@
       <c r="U47" t="s">
         <v>167</v>
       </c>
-      <c r="V47" s="1">
+      <c r="V47" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3348,7 +3374,7 @@
       <c r="G48" t="s">
         <v>40</v>
       </c>
-      <c r="H48" s="1">
+      <c r="H48" s="2">
         <v>46176</v>
       </c>
       <c r="I48" t="s">
@@ -3381,7 +3407,7 @@
       <c r="U48" t="s">
         <v>167</v>
       </c>
-      <c r="V48" s="1">
+      <c r="V48" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3434,7 +3460,7 @@
       <c r="U49" t="s">
         <v>167</v>
       </c>
-      <c r="V49" s="1">
+      <c r="V49" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3487,7 +3513,7 @@
       <c r="U50" t="s">
         <v>167</v>
       </c>
-      <c r="V50" s="1">
+      <c r="V50" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3534,7 +3560,7 @@
       <c r="U51" t="s">
         <v>167</v>
       </c>
-      <c r="V51" s="1">
+      <c r="V51" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3581,7 +3607,7 @@
       <c r="U52" t="s">
         <v>167</v>
       </c>
-      <c r="V52" s="1">
+      <c r="V52" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -3628,7 +3654,7 @@
       <c r="U53" t="s">
         <v>167</v>
       </c>
-      <c r="V53" s="1">
+      <c r="V53" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3678,7 +3704,7 @@
       <c r="U54" t="s">
         <v>167</v>
       </c>
-      <c r="V54" s="1">
+      <c r="V54" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3725,7 +3751,7 @@
       <c r="U55" t="s">
         <v>167</v>
       </c>
-      <c r="V55" s="1">
+      <c r="V55" s="2">
         <v>46049</v>
       </c>
     </row>
@@ -3857,7 +3883,7 @@
       <c r="U58" t="s">
         <v>167</v>
       </c>
-      <c r="V58" s="1">
+      <c r="V58" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -3901,7 +3927,7 @@
       <c r="U59" t="s">
         <v>167</v>
       </c>
-      <c r="V59" s="1">
+      <c r="V59" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -3945,7 +3971,7 @@
       <c r="U60" t="s">
         <v>167</v>
       </c>
-      <c r="V60" s="1">
+      <c r="V60" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -3989,7 +4015,7 @@
       <c r="U61" t="s">
         <v>167</v>
       </c>
-      <c r="V61" s="1">
+      <c r="V61" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4033,7 +4059,7 @@
       <c r="U62" t="s">
         <v>167</v>
       </c>
-      <c r="V62" s="1">
+      <c r="V62" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4077,7 +4103,7 @@
       <c r="U63" t="s">
         <v>167</v>
       </c>
-      <c r="V63" s="1">
+      <c r="V63" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4121,7 +4147,7 @@
       <c r="U64" t="s">
         <v>28</v>
       </c>
-      <c r="V64" s="1">
+      <c r="V64" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4168,7 +4194,7 @@
       <c r="U65" t="s">
         <v>28</v>
       </c>
-      <c r="V65" s="1">
+      <c r="V65" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4215,7 +4241,7 @@
       <c r="U66" t="s">
         <v>167</v>
       </c>
-      <c r="V66" s="1">
+      <c r="V66" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -4259,7 +4285,7 @@
       <c r="U67" t="s">
         <v>28</v>
       </c>
-      <c r="V67" s="1">
+      <c r="V67" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -4303,7 +4329,7 @@
       <c r="U68" t="s">
         <v>167</v>
       </c>
-      <c r="V68" s="1">
+      <c r="V68" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4347,7 +4373,7 @@
       <c r="U69" t="s">
         <v>167</v>
       </c>
-      <c r="V69" s="1">
+      <c r="V69" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4391,7 +4417,7 @@
       <c r="U70" t="s">
         <v>167</v>
       </c>
-      <c r="V70" s="1">
+      <c r="V70" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4435,7 +4461,7 @@
       <c r="U71" t="s">
         <v>167</v>
       </c>
-      <c r="V71" s="1">
+      <c r="V71" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4479,7 +4505,7 @@
       <c r="U72" t="s">
         <v>167</v>
       </c>
-      <c r="V72" s="1">
+      <c r="V72" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4526,7 +4552,7 @@
       <c r="U73" t="s">
         <v>28</v>
       </c>
-      <c r="V73" s="1">
+      <c r="V73" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -4576,7 +4602,7 @@
       <c r="U74" t="s">
         <v>167</v>
       </c>
-      <c r="V74" s="1">
+      <c r="V74" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4626,7 +4652,7 @@
       <c r="U75" t="s">
         <v>167</v>
       </c>
-      <c r="V75" s="1">
+      <c r="V75" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4676,7 +4702,7 @@
       <c r="U76" t="s">
         <v>28</v>
       </c>
-      <c r="V76" s="1">
+      <c r="V76" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4726,7 +4752,7 @@
       <c r="U77" t="s">
         <v>28</v>
       </c>
-      <c r="V77" s="1">
+      <c r="V77" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4770,7 +4796,7 @@
       <c r="U78" t="s">
         <v>28</v>
       </c>
-      <c r="V78" s="1">
+      <c r="V78" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -4814,7 +4840,7 @@
       <c r="U79" t="s">
         <v>28</v>
       </c>
-      <c r="V79" s="1">
+      <c r="V79" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -4861,7 +4887,7 @@
       <c r="U80" t="s">
         <v>167</v>
       </c>
-      <c r="V80" s="1">
+      <c r="V80" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -4905,7 +4931,7 @@
       <c r="U81" t="s">
         <v>28</v>
       </c>
-      <c r="V81" s="1">
+      <c r="V81" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -4949,7 +4975,7 @@
       <c r="U82" t="s">
         <v>28</v>
       </c>
-      <c r="V82" s="1">
+      <c r="V82" s="2">
         <v>46382</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (23/07/2026 16:17)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -527,16 +527,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -552,7 +544,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -560,30 +552,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -883,70 +857,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -996,7 +970,7 @@
       <c r="U2" t="s">
         <v>167</v>
       </c>
-      <c r="V2" s="2">
+      <c r="V2" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1043,7 +1017,7 @@
       <c r="U3" t="s">
         <v>28</v>
       </c>
-      <c r="V3" s="2">
+      <c r="V3" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1090,7 +1064,7 @@
       <c r="U4" t="s">
         <v>28</v>
       </c>
-      <c r="V4" s="2">
+      <c r="V4" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -1137,7 +1111,7 @@
       <c r="U5" t="s">
         <v>28</v>
       </c>
-      <c r="V5" s="2">
+      <c r="V5" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -1187,7 +1161,7 @@
       <c r="U6" t="s">
         <v>28</v>
       </c>
-      <c r="V6" s="2">
+      <c r="V6" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1213,7 +1187,7 @@
       <c r="G7" t="s">
         <v>40</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1243,7 +1217,7 @@
       <c r="U7" t="s">
         <v>28</v>
       </c>
-      <c r="V7" s="2">
+      <c r="V7" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -1290,7 +1264,7 @@
       <c r="U8" t="s">
         <v>28</v>
       </c>
-      <c r="V8" s="2">
+      <c r="V8" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1337,7 +1311,7 @@
       <c r="U9" t="s">
         <v>28</v>
       </c>
-      <c r="V9" s="2">
+      <c r="V9" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1384,7 +1358,7 @@
       <c r="U10" t="s">
         <v>28</v>
       </c>
-      <c r="V10" s="2">
+      <c r="V10" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1431,7 +1405,7 @@
       <c r="U11" t="s">
         <v>28</v>
       </c>
-      <c r="V11" s="2">
+      <c r="V11" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1457,7 +1431,7 @@
       <c r="G12" t="s">
         <v>40</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46079</v>
       </c>
       <c r="I12" t="s">
@@ -1490,7 +1464,7 @@
       <c r="U12" t="s">
         <v>167</v>
       </c>
-      <c r="V12" s="2">
+      <c r="V12" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -1537,7 +1511,7 @@
       <c r="U13" t="s">
         <v>167</v>
       </c>
-      <c r="V13" s="2">
+      <c r="V13" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1584,7 +1558,7 @@
       <c r="U14" t="s">
         <v>167</v>
       </c>
-      <c r="V14" s="2">
+      <c r="V14" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1631,7 +1605,7 @@
       <c r="U15" t="s">
         <v>167</v>
       </c>
-      <c r="V15" s="2">
+      <c r="V15" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1678,7 +1652,7 @@
       <c r="U16" t="s">
         <v>167</v>
       </c>
-      <c r="V16" s="2">
+      <c r="V16" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1704,7 +1678,7 @@
       <c r="G17" t="s">
         <v>40</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46098</v>
       </c>
       <c r="I17" t="s">
@@ -1737,7 +1711,7 @@
       <c r="U17" t="s">
         <v>167</v>
       </c>
-      <c r="V17" s="2">
+      <c r="V17" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -1763,7 +1737,7 @@
       <c r="G18" t="s">
         <v>40</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46076</v>
       </c>
       <c r="I18" t="s">
@@ -1793,7 +1767,7 @@
       <c r="U18" t="s">
         <v>28</v>
       </c>
-      <c r="V18" s="2">
+      <c r="V18" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1819,7 +1793,7 @@
       <c r="G19" t="s">
         <v>40</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1849,7 +1823,7 @@
       <c r="U19" t="s">
         <v>28</v>
       </c>
-      <c r="V19" s="2">
+      <c r="V19" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1896,7 +1870,7 @@
       <c r="U20" t="s">
         <v>28</v>
       </c>
-      <c r="V20" s="2">
+      <c r="V20" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1943,7 +1917,7 @@
       <c r="U21" t="s">
         <v>28</v>
       </c>
-      <c r="V21" s="2">
+      <c r="V21" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1990,7 +1964,7 @@
       <c r="U22" t="s">
         <v>28</v>
       </c>
-      <c r="V22" s="2">
+      <c r="V22" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2037,7 +2011,7 @@
       <c r="U23" t="s">
         <v>28</v>
       </c>
-      <c r="V23" s="2">
+      <c r="V23" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2063,7 +2037,7 @@
       <c r="G24" t="s">
         <v>40</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>46119</v>
       </c>
       <c r="I24" t="s">
@@ -2096,7 +2070,7 @@
       <c r="U24" t="s">
         <v>167</v>
       </c>
-      <c r="V24" s="2">
+      <c r="V24" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2122,7 +2096,7 @@
       <c r="G25" t="s">
         <v>40</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>46121</v>
       </c>
       <c r="I25" t="s">
@@ -2152,7 +2126,7 @@
       <c r="U25" t="s">
         <v>28</v>
       </c>
-      <c r="V25" s="2">
+      <c r="V25" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -2178,7 +2152,7 @@
       <c r="G26" t="s">
         <v>40</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>46076</v>
       </c>
       <c r="I26" t="s">
@@ -2208,7 +2182,7 @@
       <c r="U26" t="s">
         <v>28</v>
       </c>
-      <c r="V26" s="2">
+      <c r="V26" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -2255,7 +2229,7 @@
       <c r="U27" t="s">
         <v>167</v>
       </c>
-      <c r="V27" s="2">
+      <c r="V27" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2281,7 +2255,7 @@
       <c r="G28" t="s">
         <v>40</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>46199</v>
       </c>
       <c r="I28" t="s">
@@ -2314,7 +2288,7 @@
       <c r="U28" t="s">
         <v>167</v>
       </c>
-      <c r="V28" s="2">
+      <c r="V28" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2340,7 +2314,7 @@
       <c r="G29" t="s">
         <v>40</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2373,7 +2347,7 @@
       <c r="U29" t="s">
         <v>167</v>
       </c>
-      <c r="V29" s="2">
+      <c r="V29" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2399,7 +2373,7 @@
       <c r="G30" t="s">
         <v>40</v>
       </c>
-      <c r="H30" s="2">
+      <c r="H30" s="1">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2432,7 +2406,7 @@
       <c r="U30" t="s">
         <v>167</v>
       </c>
-      <c r="V30" s="2">
+      <c r="V30" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2458,7 +2432,7 @@
       <c r="G31" t="s">
         <v>40</v>
       </c>
-      <c r="H31" s="2">
+      <c r="H31" s="1">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2491,7 +2465,7 @@
       <c r="U31" t="s">
         <v>167</v>
       </c>
-      <c r="V31" s="2">
+      <c r="V31" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2538,7 +2512,7 @@
       <c r="U32" t="s">
         <v>167</v>
       </c>
-      <c r="V32" s="2">
+      <c r="V32" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2564,7 +2538,7 @@
       <c r="G33" t="s">
         <v>40</v>
       </c>
-      <c r="H33" s="2">
+      <c r="H33" s="1">
         <v>46191</v>
       </c>
       <c r="I33" t="s">
@@ -2597,7 +2571,7 @@
       <c r="U33" t="s">
         <v>167</v>
       </c>
-      <c r="V33" s="2">
+      <c r="V33" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2623,7 +2597,7 @@
       <c r="G34" t="s">
         <v>40</v>
       </c>
-      <c r="H34" s="2">
+      <c r="H34" s="1">
         <v>46119</v>
       </c>
       <c r="I34" t="s">
@@ -2653,7 +2627,7 @@
       <c r="U34" t="s">
         <v>167</v>
       </c>
-      <c r="V34" s="2">
+      <c r="V34" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2679,7 +2653,7 @@
       <c r="G35" t="s">
         <v>41</v>
       </c>
-      <c r="H35" s="2">
+      <c r="H35" s="1">
         <v>46213</v>
       </c>
       <c r="N35" t="s">
@@ -2706,7 +2680,7 @@
       <c r="U35" t="s">
         <v>28</v>
       </c>
-      <c r="V35" s="2">
+      <c r="V35" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -2732,7 +2706,7 @@
       <c r="G36" t="s">
         <v>40</v>
       </c>
-      <c r="H36" s="2">
+      <c r="H36" s="1">
         <v>46175</v>
       </c>
       <c r="I36" t="s">
@@ -2762,7 +2736,7 @@
       <c r="U36" t="s">
         <v>28</v>
       </c>
-      <c r="V36" s="2">
+      <c r="V36" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -2788,7 +2762,7 @@
       <c r="G37" t="s">
         <v>41</v>
       </c>
-      <c r="H37" s="2">
+      <c r="H37" s="1">
         <v>46213</v>
       </c>
       <c r="N37" t="s">
@@ -2815,7 +2789,7 @@
       <c r="U37" t="s">
         <v>28</v>
       </c>
-      <c r="V37" s="2">
+      <c r="V37" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -2841,7 +2815,7 @@
       <c r="G38" t="s">
         <v>40</v>
       </c>
-      <c r="H38" s="2">
+      <c r="H38" s="1">
         <v>46199</v>
       </c>
       <c r="I38" t="s">
@@ -2871,7 +2845,7 @@
       <c r="U38" t="s">
         <v>28</v>
       </c>
-      <c r="V38" s="2">
+      <c r="V38" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2897,7 +2871,7 @@
       <c r="G39" t="s">
         <v>40</v>
       </c>
-      <c r="H39" s="2">
+      <c r="H39" s="1">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -2927,7 +2901,7 @@
       <c r="U39" t="s">
         <v>28</v>
       </c>
-      <c r="V39" s="2">
+      <c r="V39" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2953,7 +2927,7 @@
       <c r="G40" t="s">
         <v>40</v>
       </c>
-      <c r="H40" s="2">
+      <c r="H40" s="1">
         <v>46204</v>
       </c>
       <c r="I40" t="s">
@@ -2983,7 +2957,7 @@
       <c r="U40" t="s">
         <v>28</v>
       </c>
-      <c r="V40" s="2">
+      <c r="V40" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3027,7 +3001,7 @@
       <c r="U41" t="s">
         <v>28</v>
       </c>
-      <c r="V41" s="2">
+      <c r="V41" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3053,7 +3027,7 @@
       <c r="G42" t="s">
         <v>40</v>
       </c>
-      <c r="H42" s="2">
+      <c r="H42" s="1">
         <v>46191</v>
       </c>
       <c r="I42" t="s">
@@ -3083,7 +3057,7 @@
       <c r="U42" t="s">
         <v>28</v>
       </c>
-      <c r="V42" s="2">
+      <c r="V42" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3109,7 +3083,7 @@
       <c r="G43" t="s">
         <v>40</v>
       </c>
-      <c r="H43" s="2">
+      <c r="H43" s="1">
         <v>46191</v>
       </c>
       <c r="I43" t="s">
@@ -3139,7 +3113,7 @@
       <c r="U43" t="s">
         <v>28</v>
       </c>
-      <c r="V43" s="2">
+      <c r="V43" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3165,7 +3139,7 @@
       <c r="G44" t="s">
         <v>41</v>
       </c>
-      <c r="H44" s="2">
+      <c r="H44" s="1">
         <v>46213</v>
       </c>
       <c r="J44" t="s">
@@ -3198,7 +3172,7 @@
       <c r="U44" t="s">
         <v>167</v>
       </c>
-      <c r="V44" s="2">
+      <c r="V44" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3224,7 +3198,7 @@
       <c r="G45" t="s">
         <v>40</v>
       </c>
-      <c r="H45" s="2">
+      <c r="H45" s="1">
         <v>46210</v>
       </c>
       <c r="I45" t="s">
@@ -3254,7 +3228,7 @@
       <c r="U45" t="s">
         <v>167</v>
       </c>
-      <c r="V45" s="2">
+      <c r="V45" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3301,7 +3275,7 @@
       <c r="U46" t="s">
         <v>28</v>
       </c>
-      <c r="V46" s="2">
+      <c r="V46" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3348,7 +3322,7 @@
       <c r="U47" t="s">
         <v>167</v>
       </c>
-      <c r="V47" s="2">
+      <c r="V47" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3374,7 +3348,7 @@
       <c r="G48" t="s">
         <v>40</v>
       </c>
-      <c r="H48" s="2">
+      <c r="H48" s="1">
         <v>46176</v>
       </c>
       <c r="I48" t="s">
@@ -3407,7 +3381,7 @@
       <c r="U48" t="s">
         <v>167</v>
       </c>
-      <c r="V48" s="2">
+      <c r="V48" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3460,7 +3434,7 @@
       <c r="U49" t="s">
         <v>167</v>
       </c>
-      <c r="V49" s="2">
+      <c r="V49" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3513,7 +3487,7 @@
       <c r="U50" t="s">
         <v>167</v>
       </c>
-      <c r="V50" s="2">
+      <c r="V50" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3560,7 +3534,7 @@
       <c r="U51" t="s">
         <v>167</v>
       </c>
-      <c r="V51" s="2">
+      <c r="V51" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3607,7 +3581,7 @@
       <c r="U52" t="s">
         <v>167</v>
       </c>
-      <c r="V52" s="2">
+      <c r="V52" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -3654,7 +3628,7 @@
       <c r="U53" t="s">
         <v>167</v>
       </c>
-      <c r="V53" s="2">
+      <c r="V53" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3704,7 +3678,7 @@
       <c r="U54" t="s">
         <v>167</v>
       </c>
-      <c r="V54" s="2">
+      <c r="V54" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3751,7 +3725,7 @@
       <c r="U55" t="s">
         <v>167</v>
       </c>
-      <c r="V55" s="2">
+      <c r="V55" s="1">
         <v>46049</v>
       </c>
     </row>
@@ -3883,7 +3857,7 @@
       <c r="U58" t="s">
         <v>167</v>
       </c>
-      <c r="V58" s="2">
+      <c r="V58" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -3927,7 +3901,7 @@
       <c r="U59" t="s">
         <v>167</v>
       </c>
-      <c r="V59" s="2">
+      <c r="V59" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -3971,7 +3945,7 @@
       <c r="U60" t="s">
         <v>167</v>
       </c>
-      <c r="V60" s="2">
+      <c r="V60" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4015,7 +3989,7 @@
       <c r="U61" t="s">
         <v>167</v>
       </c>
-      <c r="V61" s="2">
+      <c r="V61" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4059,7 +4033,7 @@
       <c r="U62" t="s">
         <v>167</v>
       </c>
-      <c r="V62" s="2">
+      <c r="V62" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4103,7 +4077,7 @@
       <c r="U63" t="s">
         <v>167</v>
       </c>
-      <c r="V63" s="2">
+      <c r="V63" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4147,7 +4121,7 @@
       <c r="U64" t="s">
         <v>28</v>
       </c>
-      <c r="V64" s="2">
+      <c r="V64" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4194,7 +4168,7 @@
       <c r="U65" t="s">
         <v>28</v>
       </c>
-      <c r="V65" s="2">
+      <c r="V65" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4241,7 +4215,7 @@
       <c r="U66" t="s">
         <v>167</v>
       </c>
-      <c r="V66" s="2">
+      <c r="V66" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -4285,7 +4259,7 @@
       <c r="U67" t="s">
         <v>28</v>
       </c>
-      <c r="V67" s="2">
+      <c r="V67" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -4329,7 +4303,7 @@
       <c r="U68" t="s">
         <v>167</v>
       </c>
-      <c r="V68" s="2">
+      <c r="V68" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4373,7 +4347,7 @@
       <c r="U69" t="s">
         <v>167</v>
       </c>
-      <c r="V69" s="2">
+      <c r="V69" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4417,7 +4391,7 @@
       <c r="U70" t="s">
         <v>167</v>
       </c>
-      <c r="V70" s="2">
+      <c r="V70" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4461,7 +4435,7 @@
       <c r="U71" t="s">
         <v>167</v>
       </c>
-      <c r="V71" s="2">
+      <c r="V71" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4505,7 +4479,7 @@
       <c r="U72" t="s">
         <v>167</v>
       </c>
-      <c r="V72" s="2">
+      <c r="V72" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4552,7 +4526,7 @@
       <c r="U73" t="s">
         <v>28</v>
       </c>
-      <c r="V73" s="2">
+      <c r="V73" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -4602,7 +4576,7 @@
       <c r="U74" t="s">
         <v>167</v>
       </c>
-      <c r="V74" s="2">
+      <c r="V74" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4652,7 +4626,7 @@
       <c r="U75" t="s">
         <v>167</v>
       </c>
-      <c r="V75" s="2">
+      <c r="V75" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4702,7 +4676,7 @@
       <c r="U76" t="s">
         <v>28</v>
       </c>
-      <c r="V76" s="2">
+      <c r="V76" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4752,7 +4726,7 @@
       <c r="U77" t="s">
         <v>28</v>
       </c>
-      <c r="V77" s="2">
+      <c r="V77" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4796,7 +4770,7 @@
       <c r="U78" t="s">
         <v>28</v>
       </c>
-      <c r="V78" s="2">
+      <c r="V78" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -4840,7 +4814,7 @@
       <c r="U79" t="s">
         <v>28</v>
       </c>
-      <c r="V79" s="2">
+      <c r="V79" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -4887,7 +4861,7 @@
       <c r="U80" t="s">
         <v>167</v>
       </c>
-      <c r="V80" s="2">
+      <c r="V80" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -4931,7 +4905,7 @@
       <c r="U81" t="s">
         <v>28</v>
       </c>
-      <c r="V81" s="2">
+      <c r="V81" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -4975,7 +4949,7 @@
       <c r="U82" t="s">
         <v>28</v>
       </c>
-      <c r="V82" s="2">
+      <c r="V82" s="1">
         <v>46382</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (23/07/2026 20:41)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -193,6 +193,9 @@
     <t>1</t>
   </si>
   <si>
+    <t>email do dia 09/07</t>
+  </si>
+  <si>
     <t>email do dia 19/03</t>
   </si>
   <si>
@@ -202,9 +205,6 @@
     <t>email do dia 25/05</t>
   </si>
   <si>
-    <t>email do dia 09/07</t>
-  </si>
-  <si>
     <t>email do dia 24/04</t>
   </si>
   <si>
@@ -337,6 +337,12 @@
     <t>Reparo de PTVR 2 EA (1/2)</t>
   </si>
   <si>
+    <t>Hora de Voo 06/10 - 1000 HV</t>
+  </si>
+  <si>
+    <t>Material reparo PT6A-114A (4/4)</t>
+  </si>
+  <si>
     <t>Hora de Voo 04/10 - 1000 HV</t>
   </si>
   <si>
@@ -373,7 +379,7 @@
     <t>Material HSI PT6A-114A (4/4)</t>
   </si>
   <si>
-    <t>Hora de Voo 06/10 - 1000 HV</t>
+    <t>Hora de Voo 07/10 - 1000 HV</t>
   </si>
   <si>
     <t>Material reparo PT6A-114A (2/4)</t>
@@ -382,18 +388,15 @@
     <t>Requisições Consumíveis 2/8</t>
   </si>
   <si>
-    <t>Hora de Voo 07/10 - 1000 HV</t>
+    <t>Hora de Voo 09/10 - 1000 HV</t>
+  </si>
+  <si>
+    <t>Hora de Voo 10/10 - 760 HV</t>
   </si>
   <si>
     <t>Hora de Voo 08/10 - 1000 HV</t>
   </si>
   <si>
-    <t>Hora de Voo 09/10 - 1000 HV</t>
-  </si>
-  <si>
-    <t>Hora de Voo 10/10 - 760 HV</t>
-  </si>
-  <si>
     <t>Modernização 1/4</t>
   </si>
   <si>
@@ -469,9 +472,6 @@
     <t>Hora de Voo 10/10 - 310 HV</t>
   </si>
   <si>
-    <t>Material reparo PT6A-114A (4/4)</t>
-  </si>
-  <si>
     <t>CABW</t>
   </si>
   <si>
@@ -496,13 +496,13 @@
     <t>A</t>
   </si>
   <si>
+    <t>B</t>
+  </si>
+  <si>
     <t>C</t>
   </si>
   <si>
     <t>D</t>
-  </si>
-  <si>
-    <t>B</t>
   </si>
   <si>
     <t>REQUISIÇÃO</t>
@@ -2017,7 +2017,7 @@
     </row>
     <row r="24" spans="1:22">
       <c r="A24">
-        <v>13760</v>
+        <v>16560</v>
       </c>
       <c r="B24" t="s">
         <v>22</v>
@@ -2026,26 +2026,26 @@
         <v>22</v>
       </c>
       <c r="D24" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E24" t="s">
         <v>28</v>
       </c>
       <c r="F24" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G24" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H24" s="1">
-        <v>46119</v>
-      </c>
-      <c r="I24" t="s">
-        <v>48</v>
+        <v>46213</v>
       </c>
       <c r="J24" t="s">
         <v>59</v>
       </c>
+      <c r="K24" t="s">
+        <v>64</v>
+      </c>
       <c r="N24" t="s">
         <v>73</v>
       </c>
@@ -2053,7 +2053,7 @@
         <v>107</v>
       </c>
       <c r="P24">
-        <v>1704503</v>
+        <v>173846.38</v>
       </c>
       <c r="Q24" t="s">
         <v>154</v>
@@ -2071,12 +2071,12 @@
         <v>167</v>
       </c>
       <c r="V24" s="1">
-        <v>46138</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="25" spans="1:22">
       <c r="A25">
-        <v>14160</v>
+        <v>63960</v>
       </c>
       <c r="B25" t="s">
         <v>22</v>
@@ -2085,40 +2085,28 @@
         <v>22</v>
       </c>
       <c r="D25" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E25" t="s">
-        <v>28</v>
-      </c>
-      <c r="F25" t="s">
-        <v>30</v>
-      </c>
-      <c r="G25" t="s">
-        <v>40</v>
-      </c>
-      <c r="H25" s="1">
-        <v>46121</v>
-      </c>
-      <c r="I25" t="s">
-        <v>49</v>
+        <v>29</v>
       </c>
       <c r="N25" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="O25" t="s">
         <v>108</v>
       </c>
       <c r="P25">
-        <v>3799000</v>
+        <v>1000000</v>
       </c>
       <c r="Q25" t="s">
         <v>154</v>
       </c>
       <c r="R25" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="S25" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="T25" t="s">
         <v>164</v>
@@ -2127,12 +2115,12 @@
         <v>28</v>
       </c>
       <c r="V25" s="1">
-        <v>46168</v>
+        <v>46321</v>
       </c>
     </row>
     <row r="26" spans="1:22">
       <c r="A26">
-        <v>14161</v>
+        <v>13760</v>
       </c>
       <c r="B26" t="s">
         <v>22</v>
@@ -2147,48 +2135,51 @@
         <v>28</v>
       </c>
       <c r="F26" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G26" t="s">
         <v>40</v>
       </c>
       <c r="H26" s="1">
-        <v>46076</v>
+        <v>46119</v>
       </c>
       <c r="I26" t="s">
-        <v>50</v>
+        <v>48</v>
+      </c>
+      <c r="J26" t="s">
+        <v>60</v>
       </c>
       <c r="N26" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="O26" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="P26">
-        <v>1000</v>
+        <v>1704503</v>
       </c>
       <c r="Q26" t="s">
         <v>154</v>
       </c>
       <c r="R26" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="S26" t="s">
         <v>159</v>
       </c>
       <c r="T26" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="U26" t="s">
-        <v>28</v>
+        <v>167</v>
       </c>
       <c r="V26" s="1">
-        <v>46079</v>
+        <v>46138</v>
       </c>
     </row>
     <row r="27" spans="1:22">
       <c r="A27">
-        <v>14180</v>
+        <v>14160</v>
       </c>
       <c r="B27" t="s">
         <v>22</v>
@@ -2197,7 +2188,7 @@
         <v>22</v>
       </c>
       <c r="D27" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E27" t="s">
         <v>28</v>
@@ -2205,37 +2196,46 @@
       <c r="F27" t="s">
         <v>30</v>
       </c>
+      <c r="G27" t="s">
+        <v>40</v>
+      </c>
+      <c r="H27" s="1">
+        <v>46121</v>
+      </c>
+      <c r="I27" t="s">
+        <v>49</v>
+      </c>
       <c r="N27" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="O27" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="P27">
-        <v>100000</v>
+        <v>3799000</v>
       </c>
       <c r="Q27" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="R27" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="S27" t="s">
         <v>159</v>
       </c>
       <c r="T27" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="U27" t="s">
-        <v>167</v>
+        <v>28</v>
       </c>
       <c r="V27" s="1">
-        <v>46291</v>
+        <v>46168</v>
       </c>
     </row>
     <row r="28" spans="1:22">
       <c r="A28">
-        <v>15380</v>
+        <v>14161</v>
       </c>
       <c r="B28" t="s">
         <v>22</v>
@@ -2250,34 +2250,31 @@
         <v>28</v>
       </c>
       <c r="F28" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="G28" t="s">
         <v>40</v>
       </c>
       <c r="H28" s="1">
-        <v>46199</v>
+        <v>46076</v>
       </c>
       <c r="I28" t="s">
-        <v>51</v>
-      </c>
-      <c r="J28" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="N28" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="O28" t="s">
         <v>110</v>
       </c>
       <c r="P28">
-        <v>150000</v>
+        <v>1000</v>
       </c>
       <c r="Q28" t="s">
         <v>154</v>
       </c>
       <c r="R28" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="S28" t="s">
         <v>159</v>
@@ -2286,15 +2283,15 @@
         <v>164</v>
       </c>
       <c r="U28" t="s">
-        <v>167</v>
+        <v>28</v>
       </c>
       <c r="V28" s="1">
-        <v>46199</v>
+        <v>46079</v>
       </c>
     </row>
     <row r="29" spans="1:22">
       <c r="A29">
-        <v>15400</v>
+        <v>14180</v>
       </c>
       <c r="B29" t="s">
         <v>22</v>
@@ -2303,57 +2300,45 @@
         <v>22</v>
       </c>
       <c r="D29" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E29" t="s">
         <v>28</v>
       </c>
       <c r="F29" t="s">
-        <v>32</v>
-      </c>
-      <c r="G29" t="s">
-        <v>40</v>
-      </c>
-      <c r="H29" s="1">
-        <v>46199</v>
-      </c>
-      <c r="I29" t="s">
-        <v>51</v>
-      </c>
-      <c r="J29" t="s">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="N29" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O29" t="s">
         <v>111</v>
       </c>
       <c r="P29">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="Q29" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="R29" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="S29" t="s">
         <v>159</v>
       </c>
       <c r="T29" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="U29" t="s">
         <v>167</v>
       </c>
       <c r="V29" s="1">
-        <v>46199</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="30" spans="1:22">
       <c r="A30">
-        <v>15420</v>
+        <v>15380</v>
       </c>
       <c r="B30" t="s">
         <v>22</v>
@@ -2368,7 +2353,7 @@
         <v>28</v>
       </c>
       <c r="F30" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G30" t="s">
         <v>40</v>
@@ -2377,10 +2362,10 @@
         <v>46199</v>
       </c>
       <c r="I30" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="J30" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="N30" t="s">
         <v>73</v>
@@ -2389,7 +2374,7 @@
         <v>112</v>
       </c>
       <c r="P30">
-        <v>18462.36</v>
+        <v>150000</v>
       </c>
       <c r="Q30" t="s">
         <v>154</v>
@@ -2412,7 +2397,7 @@
     </row>
     <row r="31" spans="1:22">
       <c r="A31">
-        <v>15421</v>
+        <v>15400</v>
       </c>
       <c r="B31" t="s">
         <v>22</v>
@@ -2439,16 +2424,16 @@
         <v>51</v>
       </c>
       <c r="J31" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="N31" t="s">
         <v>73</v>
       </c>
       <c r="O31" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="P31">
-        <v>324166.14</v>
+        <v>150000</v>
       </c>
       <c r="Q31" t="s">
         <v>154</v>
@@ -2471,7 +2456,7 @@
     </row>
     <row r="32" spans="1:22">
       <c r="A32">
-        <v>15440</v>
+        <v>15420</v>
       </c>
       <c r="B32" t="s">
         <v>22</v>
@@ -2480,22 +2465,34 @@
         <v>22</v>
       </c>
       <c r="D32" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E32" t="s">
         <v>28</v>
       </c>
       <c r="F32" t="s">
-        <v>30</v>
+        <v>33</v>
+      </c>
+      <c r="G32" t="s">
+        <v>40</v>
+      </c>
+      <c r="H32" s="1">
+        <v>46199</v>
+      </c>
+      <c r="I32" t="s">
+        <v>52</v>
+      </c>
+      <c r="J32" t="s">
+        <v>61</v>
       </c>
       <c r="N32" t="s">
         <v>73</v>
       </c>
       <c r="O32" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="P32">
-        <v>30000</v>
+        <v>18462.36</v>
       </c>
       <c r="Q32" t="s">
         <v>154</v>
@@ -2513,12 +2510,12 @@
         <v>167</v>
       </c>
       <c r="V32" s="1">
-        <v>46291</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="33" spans="1:22">
       <c r="A33">
-        <v>15680</v>
+        <v>15421</v>
       </c>
       <c r="B33" t="s">
         <v>22</v>
@@ -2533,16 +2530,16 @@
         <v>28</v>
       </c>
       <c r="F33" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="G33" t="s">
         <v>40</v>
       </c>
       <c r="H33" s="1">
-        <v>46191</v>
+        <v>46199</v>
       </c>
       <c r="I33" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="J33" t="s">
         <v>61</v>
@@ -2554,7 +2551,7 @@
         <v>114</v>
       </c>
       <c r="P33">
-        <v>1496713.48</v>
+        <v>324166.14</v>
       </c>
       <c r="Q33" t="s">
         <v>154</v>
@@ -2566,7 +2563,7 @@
         <v>159</v>
       </c>
       <c r="T33" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="U33" t="s">
         <v>167</v>
@@ -2577,7 +2574,7 @@
     </row>
     <row r="34" spans="1:22">
       <c r="A34">
-        <v>15681</v>
+        <v>15440</v>
       </c>
       <c r="B34" t="s">
         <v>22</v>
@@ -2586,31 +2583,22 @@
         <v>22</v>
       </c>
       <c r="D34" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E34" t="s">
         <v>28</v>
       </c>
       <c r="F34" t="s">
-        <v>31</v>
-      </c>
-      <c r="G34" t="s">
-        <v>40</v>
-      </c>
-      <c r="H34" s="1">
-        <v>46119</v>
-      </c>
-      <c r="I34" t="s">
-        <v>48</v>
+        <v>30</v>
       </c>
       <c r="N34" t="s">
         <v>73</v>
       </c>
       <c r="O34" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="P34">
-        <v>207789.52</v>
+        <v>30000</v>
       </c>
       <c r="Q34" t="s">
         <v>154</v>
@@ -2622,18 +2610,18 @@
         <v>159</v>
       </c>
       <c r="T34" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="U34" t="s">
         <v>167</v>
       </c>
       <c r="V34" s="1">
-        <v>46199</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="35" spans="1:22">
       <c r="A35">
-        <v>15960</v>
+        <v>15680</v>
       </c>
       <c r="B35" t="s">
         <v>22</v>
@@ -2642,7 +2630,7 @@
         <v>22</v>
       </c>
       <c r="D35" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E35" t="s">
         <v>28</v>
@@ -2651,42 +2639,48 @@
         <v>30</v>
       </c>
       <c r="G35" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H35" s="1">
-        <v>46213</v>
+        <v>46191</v>
+      </c>
+      <c r="I35" t="s">
+        <v>53</v>
+      </c>
+      <c r="J35" t="s">
+        <v>62</v>
       </c>
       <c r="N35" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="O35" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="P35">
-        <v>962290.8</v>
+        <v>1496713.48</v>
       </c>
       <c r="Q35" t="s">
         <v>154</v>
       </c>
       <c r="R35" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="S35" t="s">
         <v>159</v>
       </c>
       <c r="T35" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="U35" t="s">
-        <v>28</v>
+        <v>167</v>
       </c>
       <c r="V35" s="1">
-        <v>46260</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="36" spans="1:22">
       <c r="A36">
-        <v>15961</v>
+        <v>15681</v>
       </c>
       <c r="B36" t="s">
         <v>22</v>
@@ -2701,25 +2695,25 @@
         <v>28</v>
       </c>
       <c r="F36" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="G36" t="s">
         <v>40</v>
       </c>
       <c r="H36" s="1">
-        <v>46175</v>
+        <v>46119</v>
       </c>
       <c r="I36" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="N36" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="O36" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="P36">
-        <v>800000</v>
+        <v>207789.52</v>
       </c>
       <c r="Q36" t="s">
         <v>154</v>
@@ -2731,18 +2725,18 @@
         <v>159</v>
       </c>
       <c r="T36" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="U36" t="s">
-        <v>28</v>
+        <v>167</v>
       </c>
       <c r="V36" s="1">
-        <v>46229</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="37" spans="1:22">
       <c r="A37">
-        <v>15962</v>
+        <v>15960</v>
       </c>
       <c r="B37" t="s">
         <v>22</v>
@@ -2769,10 +2763,10 @@
         <v>76</v>
       </c>
       <c r="O37" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="P37">
-        <v>1530656.62</v>
+        <v>962290.8</v>
       </c>
       <c r="Q37" t="s">
         <v>154</v>
@@ -2795,7 +2789,7 @@
     </row>
     <row r="38" spans="1:22">
       <c r="A38">
-        <v>15963</v>
+        <v>15961</v>
       </c>
       <c r="B38" t="s">
         <v>22</v>
@@ -2810,31 +2804,31 @@
         <v>28</v>
       </c>
       <c r="F38" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G38" t="s">
         <v>40</v>
       </c>
       <c r="H38" s="1">
-        <v>46199</v>
+        <v>46175</v>
       </c>
       <c r="I38" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="N38" t="s">
         <v>76</v>
       </c>
       <c r="O38" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="P38">
-        <v>72958.08</v>
+        <v>800000</v>
       </c>
       <c r="Q38" t="s">
         <v>154</v>
       </c>
       <c r="R38" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="S38" t="s">
         <v>159</v>
@@ -2846,12 +2840,12 @@
         <v>28</v>
       </c>
       <c r="V38" s="1">
-        <v>46199</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="39" spans="1:22">
       <c r="A39">
-        <v>15964</v>
+        <v>15962</v>
       </c>
       <c r="B39" t="s">
         <v>22</v>
@@ -2860,31 +2854,28 @@
         <v>22</v>
       </c>
       <c r="D39" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E39" t="s">
         <v>28</v>
       </c>
       <c r="F39" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="G39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H39" s="1">
-        <v>46199</v>
-      </c>
-      <c r="I39" t="s">
-        <v>55</v>
+        <v>46213</v>
       </c>
       <c r="N39" t="s">
         <v>76</v>
       </c>
       <c r="O39" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="P39">
-        <v>8916</v>
+        <v>1530656.62</v>
       </c>
       <c r="Q39" t="s">
         <v>154</v>
@@ -2902,12 +2893,12 @@
         <v>28</v>
       </c>
       <c r="V39" s="1">
-        <v>46199</v>
+        <v>46260</v>
       </c>
     </row>
     <row r="40" spans="1:22">
       <c r="A40">
-        <v>15965</v>
+        <v>15963</v>
       </c>
       <c r="B40" t="s">
         <v>22</v>
@@ -2922,13 +2913,13 @@
         <v>28</v>
       </c>
       <c r="F40" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="G40" t="s">
         <v>40</v>
       </c>
       <c r="H40" s="1">
-        <v>46204</v>
+        <v>46199</v>
       </c>
       <c r="I40" t="s">
         <v>55</v>
@@ -2937,10 +2928,10 @@
         <v>76</v>
       </c>
       <c r="O40" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="P40">
-        <v>425178.5</v>
+        <v>72958.08</v>
       </c>
       <c r="Q40" t="s">
         <v>154</v>
@@ -2963,7 +2954,7 @@
     </row>
     <row r="41" spans="1:22">
       <c r="A41">
-        <v>15980</v>
+        <v>15964</v>
       </c>
       <c r="B41" t="s">
         <v>22</v>
@@ -2972,19 +2963,31 @@
         <v>22</v>
       </c>
       <c r="D41" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E41" t="s">
-        <v>29</v>
+        <v>28</v>
+      </c>
+      <c r="F41" t="s">
+        <v>36</v>
       </c>
       <c r="G41" t="s">
-        <v>42</v>
+        <v>40</v>
+      </c>
+      <c r="H41" s="1">
+        <v>46199</v>
+      </c>
+      <c r="I41" t="s">
+        <v>55</v>
       </c>
       <c r="N41" t="s">
         <v>76</v>
       </c>
       <c r="O41" t="s">
-        <v>116</v>
+        <v>117</v>
+      </c>
+      <c r="P41">
+        <v>8916</v>
       </c>
       <c r="Q41" t="s">
         <v>154</v>
@@ -2993,7 +2996,7 @@
         <v>156</v>
       </c>
       <c r="S41" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="T41" t="s">
         <v>164</v>
@@ -3002,12 +3005,12 @@
         <v>28</v>
       </c>
       <c r="V41" s="1">
-        <v>46260</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="42" spans="1:22">
       <c r="A42">
-        <v>16000</v>
+        <v>15965</v>
       </c>
       <c r="B42" t="s">
         <v>22</v>
@@ -3022,25 +3025,25 @@
         <v>28</v>
       </c>
       <c r="F42" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="G42" t="s">
         <v>40</v>
       </c>
       <c r="H42" s="1">
-        <v>46191</v>
+        <v>46204</v>
       </c>
       <c r="I42" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="N42" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="O42" t="s">
         <v>117</v>
       </c>
       <c r="P42">
-        <v>400000</v>
+        <v>425178.5</v>
       </c>
       <c r="Q42" t="s">
         <v>154</v>
@@ -3063,7 +3066,7 @@
     </row>
     <row r="43" spans="1:22">
       <c r="A43">
-        <v>16001</v>
+        <v>15980</v>
       </c>
       <c r="B43" t="s">
         <v>22</v>
@@ -3072,32 +3075,20 @@
         <v>22</v>
       </c>
       <c r="D43" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E43" t="s">
-        <v>28</v>
-      </c>
-      <c r="F43" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G43" t="s">
-        <v>40</v>
-      </c>
-      <c r="H43" s="1">
-        <v>46191</v>
-      </c>
-      <c r="I43" t="s">
-        <v>56</v>
+        <v>42</v>
       </c>
       <c r="N43" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="O43" t="s">
         <v>118</v>
       </c>
-      <c r="P43">
-        <v>400000</v>
-      </c>
       <c r="Q43" t="s">
         <v>154</v>
       </c>
@@ -3105,7 +3096,7 @@
         <v>156</v>
       </c>
       <c r="S43" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="T43" t="s">
         <v>164</v>
@@ -3114,12 +3105,12 @@
         <v>28</v>
       </c>
       <c r="V43" s="1">
-        <v>46199</v>
+        <v>46260</v>
       </c>
     </row>
     <row r="44" spans="1:22">
       <c r="A44">
-        <v>16560</v>
+        <v>16000</v>
       </c>
       <c r="B44" t="s">
         <v>22</v>
@@ -3128,7 +3119,7 @@
         <v>22</v>
       </c>
       <c r="D44" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E44" t="s">
         <v>28</v>
@@ -3137,48 +3128,45 @@
         <v>30</v>
       </c>
       <c r="G44" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H44" s="1">
-        <v>46213</v>
-      </c>
-      <c r="J44" t="s">
-        <v>62</v>
-      </c>
-      <c r="K44" t="s">
-        <v>64</v>
+        <v>46191</v>
+      </c>
+      <c r="I44" t="s">
+        <v>56</v>
       </c>
       <c r="N44" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="O44" t="s">
         <v>119</v>
       </c>
       <c r="P44">
-        <v>173846.38</v>
+        <v>400000</v>
       </c>
       <c r="Q44" t="s">
         <v>154</v>
       </c>
       <c r="R44" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="S44" t="s">
         <v>159</v>
       </c>
       <c r="T44" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="U44" t="s">
-        <v>167</v>
+        <v>28</v>
       </c>
       <c r="V44" s="1">
-        <v>46229</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="45" spans="1:22">
       <c r="A45">
-        <v>16561</v>
+        <v>16001</v>
       </c>
       <c r="B45" t="s">
         <v>22</v>
@@ -3193,48 +3181,48 @@
         <v>28</v>
       </c>
       <c r="F45" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="G45" t="s">
         <v>40</v>
       </c>
       <c r="H45" s="1">
-        <v>46210</v>
+        <v>46191</v>
       </c>
       <c r="I45" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="N45" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="O45" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="P45">
-        <v>1530656.62</v>
+        <v>400000</v>
       </c>
       <c r="Q45" t="s">
         <v>154</v>
       </c>
       <c r="R45" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="S45" t="s">
         <v>159</v>
       </c>
       <c r="T45" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="U45" t="s">
-        <v>167</v>
+        <v>28</v>
       </c>
       <c r="V45" s="1">
-        <v>46229</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="46" spans="1:22">
       <c r="A46">
-        <v>16700</v>
+        <v>17760</v>
       </c>
       <c r="B46" t="s">
         <v>22</v>
@@ -3251,29 +3239,35 @@
       <c r="F46" t="s">
         <v>30</v>
       </c>
+      <c r="J46" t="s">
+        <v>59</v>
+      </c>
+      <c r="K46" t="s">
+        <v>65</v>
+      </c>
       <c r="N46" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="O46" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="P46">
-        <v>1000000</v>
+        <v>1704503</v>
       </c>
       <c r="Q46" t="s">
         <v>154</v>
       </c>
       <c r="R46" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="S46" t="s">
         <v>159</v>
       </c>
       <c r="T46" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="U46" t="s">
-        <v>28</v>
+        <v>167</v>
       </c>
       <c r="V46" s="1">
         <v>46260</v>
@@ -3281,7 +3275,7 @@
     </row>
     <row r="47" spans="1:22">
       <c r="A47">
-        <v>17200</v>
+        <v>16561</v>
       </c>
       <c r="B47" t="s">
         <v>22</v>
@@ -3290,45 +3284,54 @@
         <v>22</v>
       </c>
       <c r="D47" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E47" t="s">
         <v>28</v>
       </c>
       <c r="F47" t="s">
-        <v>30</v>
+        <v>33</v>
+      </c>
+      <c r="G47" t="s">
+        <v>40</v>
+      </c>
+      <c r="H47" s="1">
+        <v>46210</v>
+      </c>
+      <c r="I47" t="s">
+        <v>52</v>
       </c>
       <c r="N47" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="O47" t="s">
-        <v>121</v>
+        <v>107</v>
       </c>
       <c r="P47">
-        <v>958040</v>
+        <v>1530656.62</v>
       </c>
       <c r="Q47" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="R47" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="S47" t="s">
         <v>159</v>
       </c>
       <c r="T47" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="U47" t="s">
         <v>167</v>
       </c>
       <c r="V47" s="1">
-        <v>46291</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="48" spans="1:22">
       <c r="A48">
-        <v>17201</v>
+        <v>16700</v>
       </c>
       <c r="B48" t="s">
         <v>22</v>
@@ -3337,7 +3340,7 @@
         <v>22</v>
       </c>
       <c r="D48" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E48" t="s">
         <v>28</v>
@@ -3345,49 +3348,37 @@
       <c r="F48" t="s">
         <v>30</v>
       </c>
-      <c r="G48" t="s">
-        <v>40</v>
-      </c>
-      <c r="H48" s="1">
-        <v>46176</v>
-      </c>
-      <c r="I48" t="s">
-        <v>57</v>
-      </c>
-      <c r="J48" t="s">
-        <v>63</v>
-      </c>
       <c r="N48" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="O48" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="P48">
-        <v>41730.64</v>
+        <v>1000000</v>
       </c>
       <c r="Q48" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="R48" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="S48" t="s">
         <v>159</v>
       </c>
       <c r="T48" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="U48" t="s">
-        <v>167</v>
+        <v>28</v>
       </c>
       <c r="V48" s="1">
-        <v>46291</v>
+        <v>46260</v>
       </c>
     </row>
     <row r="49" spans="1:22">
       <c r="A49">
-        <v>17760</v>
+        <v>17200</v>
       </c>
       <c r="B49" t="s">
         <v>22</v>
@@ -3404,43 +3395,37 @@
       <c r="F49" t="s">
         <v>30</v>
       </c>
-      <c r="J49" t="s">
-        <v>62</v>
-      </c>
-      <c r="K49" t="s">
-        <v>65</v>
-      </c>
       <c r="N49" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="O49" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="P49">
-        <v>1704503</v>
+        <v>958040</v>
       </c>
       <c r="Q49" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="R49" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="S49" t="s">
         <v>159</v>
       </c>
       <c r="T49" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="U49" t="s">
         <v>167</v>
       </c>
       <c r="V49" s="1">
-        <v>46260</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="50" spans="1:22">
       <c r="A50">
-        <v>17761</v>
+        <v>17201</v>
       </c>
       <c r="B50" t="s">
         <v>22</v>
@@ -3449,7 +3434,7 @@
         <v>22</v>
       </c>
       <c r="D50" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E50" t="s">
         <v>28</v>
@@ -3457,32 +3442,38 @@
       <c r="F50" t="s">
         <v>30</v>
       </c>
+      <c r="G50" t="s">
+        <v>40</v>
+      </c>
+      <c r="H50" s="1">
+        <v>46176</v>
+      </c>
+      <c r="I50" t="s">
+        <v>57</v>
+      </c>
       <c r="J50" t="s">
-        <v>62</v>
-      </c>
-      <c r="K50" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="N50" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="O50" t="s">
         <v>123</v>
       </c>
       <c r="P50">
-        <v>1704503</v>
+        <v>41730.64</v>
       </c>
       <c r="Q50" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="R50" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="S50" t="s">
         <v>159</v>
       </c>
       <c r="T50" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="U50" t="s">
         <v>167</v>
@@ -3587,10 +3578,10 @@
     </row>
     <row r="53" spans="1:22">
       <c r="A53">
-        <v>19240</v>
+        <v>17761</v>
       </c>
       <c r="B53" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C53" t="s">
         <v>22</v>
@@ -3602,16 +3593,22 @@
         <v>28</v>
       </c>
       <c r="F53" t="s">
-        <v>38</v>
+        <v>30</v>
+      </c>
+      <c r="J53" t="s">
+        <v>59</v>
+      </c>
+      <c r="K53" t="s">
+        <v>66</v>
       </c>
       <c r="N53" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="O53" t="s">
         <v>126</v>
       </c>
       <c r="P53">
-        <v>500000</v>
+        <v>1704503</v>
       </c>
       <c r="Q53" t="s">
         <v>154</v>
@@ -3620,21 +3617,21 @@
         <v>155</v>
       </c>
       <c r="S53" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="T53" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="U53" t="s">
         <v>167</v>
       </c>
       <c r="V53" s="1">
-        <v>46321</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="54" spans="1:22">
       <c r="A54">
-        <v>19241</v>
+        <v>19240</v>
       </c>
       <c r="B54" t="s">
         <v>23</v>
@@ -3643,25 +3640,22 @@
         <v>22</v>
       </c>
       <c r="D54" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="E54" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F54" t="s">
         <v>38</v>
       </c>
-      <c r="G54" t="s">
-        <v>43</v>
-      </c>
       <c r="N54" t="s">
         <v>77</v>
       </c>
       <c r="O54" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="P54">
-        <v>5000000</v>
+        <v>500000</v>
       </c>
       <c r="Q54" t="s">
         <v>154</v>
@@ -3670,7 +3664,7 @@
         <v>155</v>
       </c>
       <c r="S54" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T54" t="s">
         <v>166</v>
@@ -3684,7 +3678,7 @@
     </row>
     <row r="55" spans="1:22">
       <c r="A55">
-        <v>19260</v>
+        <v>19241</v>
       </c>
       <c r="B55" t="s">
         <v>23</v>
@@ -3693,14 +3687,17 @@
         <v>22</v>
       </c>
       <c r="D55" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E55" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F55" t="s">
         <v>38</v>
       </c>
+      <c r="G55" t="s">
+        <v>43</v>
+      </c>
       <c r="N55" t="s">
         <v>77</v>
       </c>
@@ -3708,7 +3705,7 @@
         <v>127</v>
       </c>
       <c r="P55">
-        <v>4000000</v>
+        <v>5000000</v>
       </c>
       <c r="Q55" t="s">
         <v>154</v>
@@ -3717,7 +3714,7 @@
         <v>155</v>
       </c>
       <c r="S55" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T55" t="s">
         <v>166</v>
@@ -3726,12 +3723,12 @@
         <v>167</v>
       </c>
       <c r="V55" s="1">
-        <v>46049</v>
+        <v>46321</v>
       </c>
     </row>
     <row r="56" spans="1:22">
       <c r="A56">
-        <v>19600</v>
+        <v>19260</v>
       </c>
       <c r="B56" t="s">
         <v>23</v>
@@ -3740,10 +3737,10 @@
         <v>22</v>
       </c>
       <c r="D56" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="E56" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F56" t="s">
         <v>38</v>
@@ -3755,7 +3752,7 @@
         <v>128</v>
       </c>
       <c r="P56">
-        <v>5500000</v>
+        <v>4000000</v>
       </c>
       <c r="Q56" t="s">
         <v>154</v>
@@ -3764,7 +3761,7 @@
         <v>155</v>
       </c>
       <c r="S56" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T56" t="s">
         <v>166</v>
@@ -3772,10 +3769,13 @@
       <c r="U56" t="s">
         <v>167</v>
       </c>
+      <c r="V56" s="1">
+        <v>46049</v>
+      </c>
     </row>
     <row r="57" spans="1:22">
       <c r="A57">
-        <v>19620</v>
+        <v>19600</v>
       </c>
       <c r="B57" t="s">
         <v>23</v>
@@ -3808,7 +3808,7 @@
         <v>155</v>
       </c>
       <c r="S57" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T57" t="s">
         <v>166</v>
@@ -3819,10 +3819,10 @@
     </row>
     <row r="58" spans="1:22">
       <c r="A58">
-        <v>23080</v>
+        <v>19620</v>
       </c>
       <c r="B58" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C58" t="s">
         <v>22</v>
@@ -3833,37 +3833,37 @@
       <c r="E58" t="s">
         <v>29</v>
       </c>
+      <c r="F58" t="s">
+        <v>38</v>
+      </c>
       <c r="N58" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="O58" t="s">
         <v>130</v>
       </c>
       <c r="P58">
-        <v>4064.54</v>
+        <v>5500000</v>
       </c>
       <c r="Q58" t="s">
         <v>154</v>
       </c>
       <c r="R58" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="S58" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="T58" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="U58" t="s">
         <v>167</v>
       </c>
-      <c r="V58" s="1">
-        <v>46107</v>
-      </c>
     </row>
     <row r="59" spans="1:22">
       <c r="A59">
-        <v>23100</v>
+        <v>23080</v>
       </c>
       <c r="B59" t="s">
         <v>22</v>
@@ -3878,22 +3878,22 @@
         <v>29</v>
       </c>
       <c r="N59" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O59" t="s">
         <v>131</v>
       </c>
       <c r="P59">
-        <v>4227.84</v>
+        <v>4064.54</v>
       </c>
       <c r="Q59" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="R59" t="s">
         <v>158</v>
       </c>
       <c r="S59" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="T59" t="s">
         <v>163</v>
@@ -3907,7 +3907,7 @@
     </row>
     <row r="60" spans="1:22">
       <c r="A60">
-        <v>23120</v>
+        <v>23100</v>
       </c>
       <c r="B60" t="s">
         <v>22</v>
@@ -3922,13 +3922,13 @@
         <v>29</v>
       </c>
       <c r="N60" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="O60" t="s">
         <v>132</v>
       </c>
       <c r="P60">
-        <v>9389.959999999999</v>
+        <v>4227.84</v>
       </c>
       <c r="Q60" t="s">
         <v>152</v>
@@ -3937,7 +3937,7 @@
         <v>158</v>
       </c>
       <c r="S60" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="T60" t="s">
         <v>163</v>
@@ -3951,7 +3951,7 @@
     </row>
     <row r="61" spans="1:22">
       <c r="A61">
-        <v>23140</v>
+        <v>23120</v>
       </c>
       <c r="B61" t="s">
         <v>22</v>
@@ -3966,22 +3966,22 @@
         <v>29</v>
       </c>
       <c r="N61" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O61" t="s">
         <v>133</v>
       </c>
       <c r="P61">
-        <v>1163.64</v>
+        <v>9389.959999999999</v>
       </c>
       <c r="Q61" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="R61" t="s">
         <v>158</v>
       </c>
       <c r="S61" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="T61" t="s">
         <v>163</v>
@@ -3995,7 +3995,7 @@
     </row>
     <row r="62" spans="1:22">
       <c r="A62">
-        <v>23160</v>
+        <v>23140</v>
       </c>
       <c r="B62" t="s">
         <v>22</v>
@@ -4010,22 +4010,22 @@
         <v>29</v>
       </c>
       <c r="N62" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O62" t="s">
         <v>134</v>
       </c>
       <c r="P62">
-        <v>7204.82</v>
+        <v>1163.64</v>
       </c>
       <c r="Q62" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="R62" t="s">
         <v>158</v>
       </c>
       <c r="S62" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="T62" t="s">
         <v>163</v>
@@ -4039,7 +4039,7 @@
     </row>
     <row r="63" spans="1:22">
       <c r="A63">
-        <v>23180</v>
+        <v>23160</v>
       </c>
       <c r="B63" t="s">
         <v>22</v>
@@ -4054,13 +4054,13 @@
         <v>29</v>
       </c>
       <c r="N63" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="O63" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="P63">
-        <v>3662.66</v>
+        <v>7204.82</v>
       </c>
       <c r="Q63" t="s">
         <v>152</v>
@@ -4069,7 +4069,7 @@
         <v>158</v>
       </c>
       <c r="S63" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="T63" t="s">
         <v>163</v>
@@ -4083,7 +4083,7 @@
     </row>
     <row r="64" spans="1:22">
       <c r="A64">
-        <v>23640</v>
+        <v>23180</v>
       </c>
       <c r="B64" t="s">
         <v>22</v>
@@ -4098,36 +4098,36 @@
         <v>29</v>
       </c>
       <c r="N64" t="s">
-        <v>69</v>
+        <v>83</v>
       </c>
       <c r="O64" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="P64">
-        <v>120000</v>
+        <v>3662.66</v>
       </c>
       <c r="Q64" t="s">
         <v>152</v>
       </c>
       <c r="R64" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="S64" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="T64" t="s">
         <v>163</v>
       </c>
       <c r="U64" t="s">
-        <v>28</v>
+        <v>167</v>
       </c>
       <c r="V64" s="1">
-        <v>46168</v>
+        <v>46107</v>
       </c>
     </row>
     <row r="65" spans="1:22">
       <c r="A65">
-        <v>23740</v>
+        <v>23640</v>
       </c>
       <c r="B65" t="s">
         <v>22</v>
@@ -4136,31 +4136,28 @@
         <v>22</v>
       </c>
       <c r="D65" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E65" t="s">
-        <v>28</v>
-      </c>
-      <c r="F65" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N65" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="O65" t="s">
         <v>136</v>
       </c>
       <c r="P65">
-        <v>400000</v>
+        <v>120000</v>
       </c>
       <c r="Q65" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="R65" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="S65" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="T65" t="s">
         <v>163</v>
@@ -4169,12 +4166,12 @@
         <v>28</v>
       </c>
       <c r="V65" s="1">
-        <v>46291</v>
+        <v>46168</v>
       </c>
     </row>
     <row r="66" spans="1:22">
       <c r="A66">
-        <v>24180</v>
+        <v>23740</v>
       </c>
       <c r="B66" t="s">
         <v>22</v>
@@ -4192,13 +4189,13 @@
         <v>30</v>
       </c>
       <c r="N66" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="O66" t="s">
         <v>137</v>
       </c>
       <c r="P66">
-        <v>100000</v>
+        <v>400000</v>
       </c>
       <c r="Q66" t="s">
         <v>153</v>
@@ -4213,15 +4210,15 @@
         <v>163</v>
       </c>
       <c r="U66" t="s">
-        <v>167</v>
+        <v>28</v>
       </c>
       <c r="V66" s="1">
-        <v>46229</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="67" spans="1:22">
       <c r="A67">
-        <v>24380</v>
+        <v>24180</v>
       </c>
       <c r="B67" t="s">
         <v>22</v>
@@ -4230,42 +4227,45 @@
         <v>22</v>
       </c>
       <c r="D67" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="E67" t="s">
-        <v>29</v>
+        <v>28</v>
+      </c>
+      <c r="F67" t="s">
+        <v>30</v>
       </c>
       <c r="N67" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="O67" t="s">
         <v>138</v>
       </c>
       <c r="P67">
-        <v>80000</v>
+        <v>100000</v>
       </c>
       <c r="Q67" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="R67" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="S67" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="T67" t="s">
         <v>163</v>
       </c>
       <c r="U67" t="s">
-        <v>28</v>
+        <v>167</v>
       </c>
       <c r="V67" s="1">
-        <v>46260</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="68" spans="1:22">
       <c r="A68">
-        <v>24660</v>
+        <v>24380</v>
       </c>
       <c r="B68" t="s">
         <v>22</v>
@@ -4280,36 +4280,36 @@
         <v>29</v>
       </c>
       <c r="N68" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="O68" t="s">
         <v>139</v>
       </c>
       <c r="P68">
-        <v>835000</v>
+        <v>80000</v>
       </c>
       <c r="Q68" t="s">
         <v>152</v>
       </c>
       <c r="R68" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="S68" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="T68" t="s">
         <v>163</v>
       </c>
       <c r="U68" t="s">
-        <v>167</v>
+        <v>28</v>
       </c>
       <c r="V68" s="1">
-        <v>46291</v>
+        <v>46260</v>
       </c>
     </row>
     <row r="69" spans="1:22">
       <c r="A69">
-        <v>24661</v>
+        <v>24660</v>
       </c>
       <c r="B69" t="s">
         <v>22</v>
@@ -4327,10 +4327,10 @@
         <v>68</v>
       </c>
       <c r="O69" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="P69">
-        <v>165000</v>
+        <v>835000</v>
       </c>
       <c r="Q69" t="s">
         <v>152</v>
@@ -4339,7 +4339,7 @@
         <v>156</v>
       </c>
       <c r="S69" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="T69" t="s">
         <v>163</v>
@@ -4348,12 +4348,12 @@
         <v>167</v>
       </c>
       <c r="V69" s="1">
-        <v>46168</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="70" spans="1:22">
       <c r="A70">
-        <v>24680</v>
+        <v>24661</v>
       </c>
       <c r="B70" t="s">
         <v>22</v>
@@ -4374,7 +4374,7 @@
         <v>140</v>
       </c>
       <c r="P70">
-        <v>1000000</v>
+        <v>165000</v>
       </c>
       <c r="Q70" t="s">
         <v>152</v>
@@ -4383,7 +4383,7 @@
         <v>156</v>
       </c>
       <c r="S70" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="T70" t="s">
         <v>163</v>
@@ -4392,12 +4392,12 @@
         <v>167</v>
       </c>
       <c r="V70" s="1">
-        <v>46291</v>
+        <v>46168</v>
       </c>
     </row>
     <row r="71" spans="1:22">
       <c r="A71">
-        <v>24700</v>
+        <v>24680</v>
       </c>
       <c r="B71" t="s">
         <v>22</v>
@@ -4427,7 +4427,7 @@
         <v>156</v>
       </c>
       <c r="S71" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="T71" t="s">
         <v>163</v>
@@ -4441,7 +4441,7 @@
     </row>
     <row r="72" spans="1:22">
       <c r="A72">
-        <v>24720</v>
+        <v>24700</v>
       </c>
       <c r="B72" t="s">
         <v>22</v>
@@ -4456,22 +4456,22 @@
         <v>29</v>
       </c>
       <c r="N72" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="O72" t="s">
         <v>142</v>
       </c>
       <c r="P72">
-        <v>100000</v>
+        <v>1000000</v>
       </c>
       <c r="Q72" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="R72" t="s">
         <v>156</v>
       </c>
       <c r="S72" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="T72" t="s">
         <v>163</v>
@@ -4485,7 +4485,7 @@
     </row>
     <row r="73" spans="1:22">
       <c r="A73">
-        <v>25180</v>
+        <v>24720</v>
       </c>
       <c r="B73" t="s">
         <v>22</v>
@@ -4494,45 +4494,42 @@
         <v>22</v>
       </c>
       <c r="D73" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E73" t="s">
-        <v>28</v>
-      </c>
-      <c r="F73" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N73" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="O73" t="s">
         <v>143</v>
       </c>
       <c r="P73">
-        <v>1000000</v>
+        <v>100000</v>
       </c>
       <c r="Q73" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="R73" t="s">
         <v>156</v>
       </c>
       <c r="S73" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="T73" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="U73" t="s">
-        <v>28</v>
+        <v>167</v>
       </c>
       <c r="V73" s="1">
-        <v>46321</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="74" spans="1:22">
       <c r="A74">
-        <v>25900</v>
+        <v>25180</v>
       </c>
       <c r="B74" t="s">
         <v>22</v>
@@ -4541,48 +4538,45 @@
         <v>22</v>
       </c>
       <c r="D74" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E74" t="s">
         <v>28</v>
       </c>
       <c r="F74" t="s">
-        <v>39</v>
-      </c>
-      <c r="G74" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="N74" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="O74" t="s">
         <v>144</v>
       </c>
       <c r="P74">
-        <v>1704503</v>
+        <v>1000000</v>
       </c>
       <c r="Q74" t="s">
         <v>154</v>
       </c>
       <c r="R74" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="S74" t="s">
-        <v>39</v>
+        <v>159</v>
       </c>
       <c r="T74" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="U74" t="s">
-        <v>167</v>
+        <v>28</v>
       </c>
       <c r="V74" s="1">
-        <v>46381</v>
+        <v>46321</v>
       </c>
     </row>
     <row r="75" spans="1:22">
       <c r="A75">
-        <v>25920</v>
+        <v>25900</v>
       </c>
       <c r="B75" t="s">
         <v>22</v>
@@ -4609,7 +4603,7 @@
         <v>145</v>
       </c>
       <c r="P75">
-        <v>1638125.5</v>
+        <v>1704503</v>
       </c>
       <c r="Q75" t="s">
         <v>154</v>
@@ -4632,7 +4626,7 @@
     </row>
     <row r="76" spans="1:22">
       <c r="A76">
-        <v>25940</v>
+        <v>25920</v>
       </c>
       <c r="B76" t="s">
         <v>22</v>
@@ -4653,13 +4647,13 @@
         <v>40</v>
       </c>
       <c r="N76" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="O76" t="s">
         <v>146</v>
       </c>
       <c r="P76">
-        <v>3800000</v>
+        <v>1638125.5</v>
       </c>
       <c r="Q76" t="s">
         <v>154</v>
@@ -4671,10 +4665,10 @@
         <v>39</v>
       </c>
       <c r="T76" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="U76" t="s">
-        <v>28</v>
+        <v>167</v>
       </c>
       <c r="V76" s="1">
         <v>46381</v>
@@ -4682,7 +4676,7 @@
     </row>
     <row r="77" spans="1:22">
       <c r="A77">
-        <v>25960</v>
+        <v>25940</v>
       </c>
       <c r="B77" t="s">
         <v>22</v>
@@ -4732,7 +4726,7 @@
     </row>
     <row r="78" spans="1:22">
       <c r="A78">
-        <v>63120</v>
+        <v>25960</v>
       </c>
       <c r="B78" t="s">
         <v>22</v>
@@ -4741,13 +4735,19 @@
         <v>22</v>
       </c>
       <c r="D78" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E78" t="s">
-        <v>29</v>
+        <v>28</v>
+      </c>
+      <c r="F78" t="s">
+        <v>39</v>
+      </c>
+      <c r="G78" t="s">
+        <v>40</v>
       </c>
       <c r="N78" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="O78" t="s">
         <v>148</v>
@@ -4762,7 +4762,7 @@
         <v>155</v>
       </c>
       <c r="S78" t="s">
-        <v>160</v>
+        <v>39</v>
       </c>
       <c r="T78" t="s">
         <v>164</v>
@@ -4771,12 +4771,12 @@
         <v>28</v>
       </c>
       <c r="V78" s="1">
-        <v>46382</v>
+        <v>46381</v>
       </c>
     </row>
     <row r="79" spans="1:22">
       <c r="A79">
-        <v>63140</v>
+        <v>63120</v>
       </c>
       <c r="B79" t="s">
         <v>22</v>
@@ -4785,28 +4785,28 @@
         <v>22</v>
       </c>
       <c r="D79" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E79" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N79" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="O79" t="s">
         <v>149</v>
       </c>
       <c r="P79">
-        <v>4394700</v>
+        <v>3800000</v>
       </c>
       <c r="Q79" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="R79" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="S79" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="T79" t="s">
         <v>164</v>
@@ -4820,7 +4820,7 @@
     </row>
     <row r="80" spans="1:22">
       <c r="A80">
-        <v>63940</v>
+        <v>63140</v>
       </c>
       <c r="B80" t="s">
         <v>22</v>
@@ -4834,32 +4834,29 @@
       <c r="E80" t="s">
         <v>28</v>
       </c>
-      <c r="F80" t="s">
-        <v>30</v>
-      </c>
       <c r="N80" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="O80" t="s">
         <v>150</v>
       </c>
       <c r="P80">
-        <v>528395.9300000001</v>
+        <v>4394700</v>
       </c>
       <c r="Q80" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="R80" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="S80" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="T80" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="U80" t="s">
-        <v>167</v>
+        <v>28</v>
       </c>
       <c r="V80" s="1">
         <v>46382</v>
@@ -4867,7 +4864,7 @@
     </row>
     <row r="81" spans="1:22">
       <c r="A81">
-        <v>63960</v>
+        <v>63940</v>
       </c>
       <c r="B81" t="s">
         <v>22</v>
@@ -4876,37 +4873,40 @@
         <v>22</v>
       </c>
       <c r="D81" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="E81" t="s">
-        <v>29</v>
+        <v>28</v>
+      </c>
+      <c r="F81" t="s">
+        <v>30</v>
       </c>
       <c r="N81" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="O81" t="s">
         <v>151</v>
       </c>
       <c r="P81">
-        <v>1000000</v>
+        <v>528395.9300000001</v>
       </c>
       <c r="Q81" t="s">
         <v>154</v>
       </c>
       <c r="R81" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="S81" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="T81" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="U81" t="s">
-        <v>28</v>
+        <v>167</v>
       </c>
       <c r="V81" s="1">
-        <v>46321</v>
+        <v>46382</v>
       </c>
     </row>
     <row r="82" spans="1:22">
@@ -4929,7 +4929,7 @@
         <v>84</v>
       </c>
       <c r="O82" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="P82">
         <v>4394700</v>
@@ -4941,7 +4941,7 @@
         <v>156</v>
       </c>
       <c r="S82" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="T82" t="s">
         <v>164</v>

</xml_diff>

<commit_message>
Atualização automática: mta (24/07/2026 17:53)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1046" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1048" uniqueCount="168">
   <si>
     <t>linha</t>
   </si>
@@ -94,12 +94,12 @@
     <t>Atendido</t>
   </si>
   <si>
-    <t>Em trâmite</t>
-  </si>
-  <si>
     <t>Não aprovado</t>
   </si>
   <si>
+    <t>Sem informação</t>
+  </si>
+  <si>
     <t>SIM</t>
   </si>
   <si>
@@ -139,15 +139,15 @@
     <t>ATENDIDO</t>
   </si>
   <si>
-    <t>EM TRÂMITE</t>
-  </si>
-  <si>
     <t>CANCELADO</t>
   </si>
   <si>
     <t>BLOQUEIO</t>
   </si>
   <si>
+    <t>PROCESSADO</t>
+  </si>
+  <si>
     <t>C26216</t>
   </si>
   <si>
@@ -160,6 +160,9 @@
     <t>C26113</t>
   </si>
   <si>
+    <t>C26312</t>
+  </si>
+  <si>
     <t>C26193</t>
   </si>
   <si>
@@ -175,7 +178,7 @@
     <t>C26326</t>
   </si>
   <si>
-    <t>C26312</t>
+    <t>C26360</t>
   </si>
   <si>
     <t>C26285</t>
@@ -206,9 +209,6 @@
   </si>
   <si>
     <t>email do dia 24/04</t>
-  </si>
-  <si>
-    <t>Atender</t>
   </si>
   <si>
     <t>Atender AGO</t>
@@ -1438,7 +1438,7 @@
         <v>45</v>
       </c>
       <c r="J12" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="N12" t="s">
         <v>68</v>
@@ -1685,7 +1685,7 @@
         <v>46</v>
       </c>
       <c r="J17" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="N17" t="s">
         <v>73</v>
@@ -2026,7 +2026,7 @@
         <v>22</v>
       </c>
       <c r="D24" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E24" t="s">
         <v>28</v>
@@ -2035,16 +2035,16 @@
         <v>30</v>
       </c>
       <c r="G24" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H24" s="1">
         <v>46213</v>
       </c>
+      <c r="I24" t="s">
+        <v>48</v>
+      </c>
       <c r="J24" t="s">
-        <v>59</v>
-      </c>
-      <c r="K24" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="N24" t="s">
         <v>73</v>
@@ -2085,7 +2085,7 @@
         <v>22</v>
       </c>
       <c r="D25" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E25" t="s">
         <v>29</v>
@@ -2144,10 +2144,10 @@
         <v>46119</v>
       </c>
       <c r="I26" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="J26" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="N26" t="s">
         <v>73</v>
@@ -2203,7 +2203,7 @@
         <v>46121</v>
       </c>
       <c r="I27" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="N27" t="s">
         <v>76</v>
@@ -2259,7 +2259,7 @@
         <v>46076</v>
       </c>
       <c r="I28" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="N28" t="s">
         <v>76</v>
@@ -2362,10 +2362,10 @@
         <v>46199</v>
       </c>
       <c r="I30" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="J30" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="N30" t="s">
         <v>73</v>
@@ -2421,10 +2421,10 @@
         <v>46199</v>
       </c>
       <c r="I31" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="J31" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="N31" t="s">
         <v>73</v>
@@ -2480,10 +2480,10 @@
         <v>46199</v>
       </c>
       <c r="I32" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J32" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="N32" t="s">
         <v>73</v>
@@ -2539,10 +2539,10 @@
         <v>46199</v>
       </c>
       <c r="I33" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="J33" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="N33" t="s">
         <v>73</v>
@@ -2645,10 +2645,10 @@
         <v>46191</v>
       </c>
       <c r="I35" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="J35" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="N35" t="s">
         <v>73</v>
@@ -2704,7 +2704,7 @@
         <v>46119</v>
       </c>
       <c r="I36" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="N36" t="s">
         <v>73</v>
@@ -2745,7 +2745,7 @@
         <v>22</v>
       </c>
       <c r="D37" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E37" t="s">
         <v>28</v>
@@ -2754,10 +2754,13 @@
         <v>30</v>
       </c>
       <c r="G37" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H37" s="1">
         <v>46213</v>
+      </c>
+      <c r="I37" t="s">
+        <v>54</v>
       </c>
       <c r="N37" t="s">
         <v>76</v>
@@ -2813,7 +2816,7 @@
         <v>46175</v>
       </c>
       <c r="I38" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="N38" t="s">
         <v>76</v>
@@ -2854,7 +2857,7 @@
         <v>22</v>
       </c>
       <c r="D39" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E39" t="s">
         <v>28</v>
@@ -2863,10 +2866,13 @@
         <v>30</v>
       </c>
       <c r="G39" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H39" s="1">
         <v>46213</v>
+      </c>
+      <c r="I39" t="s">
+        <v>54</v>
       </c>
       <c r="N39" t="s">
         <v>76</v>
@@ -2922,7 +2928,7 @@
         <v>46199</v>
       </c>
       <c r="I40" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="N40" t="s">
         <v>76</v>
@@ -2978,7 +2984,7 @@
         <v>46199</v>
       </c>
       <c r="I41" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="N41" t="s">
         <v>76</v>
@@ -3034,7 +3040,7 @@
         <v>46204</v>
       </c>
       <c r="I42" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="N42" t="s">
         <v>76</v>
@@ -3075,13 +3081,13 @@
         <v>22</v>
       </c>
       <c r="D43" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E43" t="s">
         <v>29</v>
       </c>
       <c r="G43" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="N43" t="s">
         <v>76</v>
@@ -3134,7 +3140,7 @@
         <v>46191</v>
       </c>
       <c r="I44" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="N44" t="s">
         <v>74</v>
@@ -3190,7 +3196,7 @@
         <v>46191</v>
       </c>
       <c r="I45" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="N45" t="s">
         <v>74</v>
@@ -3240,7 +3246,7 @@
         <v>30</v>
       </c>
       <c r="J46" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="K46" t="s">
         <v>65</v>
@@ -3299,7 +3305,7 @@
         <v>46210</v>
       </c>
       <c r="I47" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="N47" t="s">
         <v>73</v>
@@ -3449,10 +3455,10 @@
         <v>46176</v>
       </c>
       <c r="I50" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="J50" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="N50" t="s">
         <v>68</v>
@@ -3596,7 +3602,7 @@
         <v>30</v>
       </c>
       <c r="J53" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="K53" t="s">
         <v>66</v>
@@ -3687,7 +3693,7 @@
         <v>22</v>
       </c>
       <c r="D55" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E55" t="s">
         <v>29</v>
@@ -3696,7 +3702,7 @@
         <v>38</v>
       </c>
       <c r="G55" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="N55" t="s">
         <v>77</v>
@@ -3784,7 +3790,7 @@
         <v>22</v>
       </c>
       <c r="D57" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E57" t="s">
         <v>29</v>
@@ -3828,7 +3834,7 @@
         <v>22</v>
       </c>
       <c r="D58" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E58" t="s">
         <v>29</v>
@@ -3872,7 +3878,7 @@
         <v>22</v>
       </c>
       <c r="D59" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E59" t="s">
         <v>29</v>
@@ -3916,7 +3922,7 @@
         <v>22</v>
       </c>
       <c r="D60" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E60" t="s">
         <v>29</v>
@@ -3960,7 +3966,7 @@
         <v>22</v>
       </c>
       <c r="D61" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E61" t="s">
         <v>29</v>
@@ -4004,7 +4010,7 @@
         <v>22</v>
       </c>
       <c r="D62" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E62" t="s">
         <v>29</v>
@@ -4048,7 +4054,7 @@
         <v>22</v>
       </c>
       <c r="D63" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E63" t="s">
         <v>29</v>
@@ -4092,7 +4098,7 @@
         <v>22</v>
       </c>
       <c r="D64" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E64" t="s">
         <v>29</v>
@@ -4136,7 +4142,7 @@
         <v>22</v>
       </c>
       <c r="D65" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E65" t="s">
         <v>29</v>
@@ -4274,7 +4280,7 @@
         <v>22</v>
       </c>
       <c r="D68" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E68" t="s">
         <v>29</v>
@@ -4318,7 +4324,7 @@
         <v>22</v>
       </c>
       <c r="D69" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E69" t="s">
         <v>29</v>
@@ -4362,7 +4368,7 @@
         <v>22</v>
       </c>
       <c r="D70" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E70" t="s">
         <v>29</v>
@@ -4406,7 +4412,7 @@
         <v>22</v>
       </c>
       <c r="D71" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E71" t="s">
         <v>29</v>
@@ -4450,7 +4456,7 @@
         <v>22</v>
       </c>
       <c r="D72" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E72" t="s">
         <v>29</v>
@@ -4494,7 +4500,7 @@
         <v>22</v>
       </c>
       <c r="D73" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E73" t="s">
         <v>29</v>
@@ -4585,7 +4591,7 @@
         <v>22</v>
       </c>
       <c r="D75" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E75" t="s">
         <v>28</v>
@@ -4594,7 +4600,7 @@
         <v>39</v>
       </c>
       <c r="G75" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="N75" t="s">
         <v>73</v>
@@ -4635,7 +4641,7 @@
         <v>22</v>
       </c>
       <c r="D76" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E76" t="s">
         <v>28</v>
@@ -4644,7 +4650,7 @@
         <v>39</v>
       </c>
       <c r="G76" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="N76" t="s">
         <v>73</v>
@@ -4685,7 +4691,7 @@
         <v>22</v>
       </c>
       <c r="D77" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E77" t="s">
         <v>28</v>
@@ -4694,7 +4700,7 @@
         <v>39</v>
       </c>
       <c r="G77" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="N77" t="s">
         <v>71</v>
@@ -4735,7 +4741,7 @@
         <v>22</v>
       </c>
       <c r="D78" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E78" t="s">
         <v>28</v>
@@ -4744,7 +4750,7 @@
         <v>39</v>
       </c>
       <c r="G78" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="N78" t="s">
         <v>71</v>
@@ -4785,7 +4791,7 @@
         <v>22</v>
       </c>
       <c r="D79" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E79" t="s">
         <v>29</v>

</xml_diff>

<commit_message>
Atualização automática: mta (27/07/2026 14:22)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1048" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1061" uniqueCount="171">
   <si>
     <t>linha</t>
   </si>
@@ -97,6 +97,9 @@
     <t>Não aprovado</t>
   </si>
   <si>
+    <t>Em trâmite</t>
+  </si>
+  <si>
     <t>Sem informação</t>
   </si>
   <si>
@@ -130,6 +133,9 @@
     <t>DESTQ32</t>
   </si>
   <si>
+    <t>20XV</t>
+  </si>
+  <si>
     <t>20IH</t>
   </si>
   <si>
@@ -142,6 +148,9 @@
     <t>CANCELADO</t>
   </si>
   <si>
+    <t>EM TRÂMITE</t>
+  </si>
+  <si>
     <t>BLOQUEIO</t>
   </si>
   <si>
@@ -160,24 +169,24 @@
     <t>C26113</t>
   </si>
   <si>
+    <t>C26193</t>
+  </si>
+  <si>
+    <t>C26162</t>
+  </si>
+  <si>
+    <t>C26112</t>
+  </si>
+  <si>
+    <t>C26324</t>
+  </si>
+  <si>
+    <t>C26326</t>
+  </si>
+  <si>
     <t>C26312</t>
   </si>
   <si>
-    <t>C26193</t>
-  </si>
-  <si>
-    <t>C26162</t>
-  </si>
-  <si>
-    <t>C26112</t>
-  </si>
-  <si>
-    <t>C26324</t>
-  </si>
-  <si>
-    <t>C26326</t>
-  </si>
-  <si>
     <t>C26360</t>
   </si>
   <si>
@@ -196,18 +205,18 @@
     <t>1</t>
   </si>
   <si>
+    <t>email do dia 19/03</t>
+  </si>
+  <si>
+    <t>email do dia 19/06</t>
+  </si>
+  <si>
+    <t>email do dia 25/05</t>
+  </si>
+  <si>
     <t>email do dia 09/07</t>
   </si>
   <si>
-    <t>email do dia 19/03</t>
-  </si>
-  <si>
-    <t>email do dia 19/06</t>
-  </si>
-  <si>
-    <t>email do dia 25/05</t>
-  </si>
-  <si>
     <t>email do dia 24/04</t>
   </si>
   <si>
@@ -250,24 +259,24 @@
     <t>CNT XXX/CELOG-PAMALS/2026 - Modernização - C-98</t>
   </si>
   <si>
+    <t>2025-BABR-24</t>
+  </si>
+  <si>
+    <t>2025-BABV-07</t>
+  </si>
+  <si>
+    <t>2025-BABR-13</t>
+  </si>
+  <si>
     <t>2025-BABR-11</t>
   </si>
   <si>
-    <t>2025-BABR-13</t>
-  </si>
-  <si>
-    <t>2025-BABR-24</t>
+    <t>2025-BABV-11</t>
   </si>
   <si>
     <t>2025-BABV-02</t>
   </si>
   <si>
-    <t>2025-BABV-07</t>
-  </si>
-  <si>
-    <t>2025-BABV-11</t>
-  </si>
-  <si>
     <t>CNT XXX/CABW-PAMASP/2026 - XX- Exchange</t>
   </si>
   <si>
@@ -337,141 +346,141 @@
     <t>Reparo de PTVR 2 EA (1/2)</t>
   </si>
   <si>
+    <t>Hora de Voo 04/10 - 1000 HV</t>
+  </si>
+  <si>
+    <t>Revisão Geral PT6A-114A (4/6)</t>
+  </si>
+  <si>
+    <t>Requisições Consumíveis 2/4</t>
+  </si>
+  <si>
+    <t>Módulo Extra - Sob demanda 1/3</t>
+  </si>
+  <si>
+    <t>Módulo Extra - Sob demanda 2/3</t>
+  </si>
+  <si>
+    <t>Módulo Extra - Sob demanda 3/3</t>
+  </si>
+  <si>
+    <t>Módulo Extra - Aquisição e publicações</t>
+  </si>
+  <si>
+    <t>Hora de Voo 05/10 - 1000 HV</t>
+  </si>
+  <si>
+    <t>Revisão Geral PT6A-114A (5/6)</t>
+  </si>
+  <si>
+    <t>Revisão Geral PT6A-114A (6/6)</t>
+  </si>
+  <si>
+    <t>Material HSI PT6A-114A (3/4)</t>
+  </si>
+  <si>
+    <t>Material HSI PT6A-114A (4/4)</t>
+  </si>
+  <si>
     <t>Hora de Voo 06/10 - 1000 HV</t>
   </si>
   <si>
+    <t>Material reparo PT6A-114A (2/4)</t>
+  </si>
+  <si>
+    <t>Requisições Consumíveis 2/8</t>
+  </si>
+  <si>
+    <t>Hora de Voo 07/10 - 1000 HV</t>
+  </si>
+  <si>
+    <t>Hora de Voo 08/10 - 1000 HV</t>
+  </si>
+  <si>
+    <t>Hora de Voo 09/10 - 1000 HV</t>
+  </si>
+  <si>
+    <t>Hora de Voo 10/10 - 760 HV</t>
+  </si>
+  <si>
+    <t>Modernização 1/4</t>
+  </si>
+  <si>
+    <t>Modernização 2/4</t>
+  </si>
+  <si>
+    <t>Modernização 3/4</t>
+  </si>
+  <si>
+    <t>Modernização 4/4</t>
+  </si>
+  <si>
+    <t>PN PS47699-3-4 - PITOT TEST, ADAPTOR</t>
+  </si>
+  <si>
+    <t>PN PS4769 - PITOT STATIC TEST ADAPTOR</t>
+  </si>
+  <si>
+    <t>PN T2680003-10 - TEMPLATE/SCALE ASSEMBLY</t>
+  </si>
+  <si>
+    <t>PN 543-250 - RELÓGIO COMPARADOR</t>
+  </si>
+  <si>
+    <t>PN DBE4-0040 - GARFO DE REBOQUE COM TRATOR ANV C-98</t>
+  </si>
+  <si>
+    <t>Reparo de CTVR 2 EA (2/2)</t>
+  </si>
+  <si>
+    <t>Material reparo acessórios PT6A-114A (3/3)</t>
+  </si>
+  <si>
+    <t>Requisições Consumíveis 3/4</t>
+  </si>
+  <si>
+    <t>Reparo de PTVR 2 EA (2/2)</t>
+  </si>
+  <si>
+    <t>Requisições Consumíveis 4/8</t>
+  </si>
+  <si>
+    <t>Requisições Consumíveis 6/8</t>
+  </si>
+  <si>
+    <t>Requisições Consumíveis 8/8</t>
+  </si>
+  <si>
+    <t>Requisições Consumíveis 4/4</t>
+  </si>
+  <si>
+    <t>Material reparo PT6A-114A (3/4)</t>
+  </si>
+  <si>
+    <t>Hora de Voo 01/10 - 1000 HV</t>
+  </si>
+  <si>
+    <t>Hora de Voo 02/10 - 1000 HV</t>
+  </si>
+  <si>
+    <t>Revisão Geral PT6A-114A (1/6)</t>
+  </si>
+  <si>
+    <t>Revisão Geral PT6A-114A (2/6)</t>
+  </si>
+  <si>
+    <t>Revisão Geral PT6A-114A</t>
+  </si>
+  <si>
+    <t>Exchange PT6A-114A</t>
+  </si>
+  <si>
+    <t>Hora de Voo 10/10 - 310 HV</t>
+  </si>
+  <si>
     <t>Material reparo PT6A-114A (4/4)</t>
   </si>
   <si>
-    <t>Hora de Voo 04/10 - 1000 HV</t>
-  </si>
-  <si>
-    <t>Revisão Geral PT6A-114A (4/6)</t>
-  </si>
-  <si>
-    <t>Requisições Consumíveis 2/4</t>
-  </si>
-  <si>
-    <t>Módulo Extra - Sob demanda 1/3</t>
-  </si>
-  <si>
-    <t>Módulo Extra - Sob demanda 2/3</t>
-  </si>
-  <si>
-    <t>Módulo Extra - Sob demanda 3/3</t>
-  </si>
-  <si>
-    <t>Módulo Extra - Aquisição e publicações</t>
-  </si>
-  <si>
-    <t>Hora de Voo 05/10 - 1000 HV</t>
-  </si>
-  <si>
-    <t>Revisão Geral PT6A-114A (5/6)</t>
-  </si>
-  <si>
-    <t>Revisão Geral PT6A-114A (6/6)</t>
-  </si>
-  <si>
-    <t>Material HSI PT6A-114A (3/4)</t>
-  </si>
-  <si>
-    <t>Material HSI PT6A-114A (4/4)</t>
-  </si>
-  <si>
-    <t>Hora de Voo 07/10 - 1000 HV</t>
-  </si>
-  <si>
-    <t>Material reparo PT6A-114A (2/4)</t>
-  </si>
-  <si>
-    <t>Requisições Consumíveis 2/8</t>
-  </si>
-  <si>
-    <t>Hora de Voo 09/10 - 1000 HV</t>
-  </si>
-  <si>
-    <t>Hora de Voo 10/10 - 760 HV</t>
-  </si>
-  <si>
-    <t>Hora de Voo 08/10 - 1000 HV</t>
-  </si>
-  <si>
-    <t>Modernização 1/4</t>
-  </si>
-  <si>
-    <t>Modernização 2/4</t>
-  </si>
-  <si>
-    <t>Modernização 3/4</t>
-  </si>
-  <si>
-    <t>Modernização 4/4</t>
-  </si>
-  <si>
-    <t>PN 543-250 - RELÓGIO COMPARADOR</t>
-  </si>
-  <si>
-    <t>PN T2680003-10 - TEMPLATE/SCALE ASSEMBLY</t>
-  </si>
-  <si>
-    <t>PN PS47699-3-4 - PITOT TEST, ADAPTOR</t>
-  </si>
-  <si>
-    <t>PN DBE4-0040 - GARFO DE REBOQUE COM TRATOR ANV C-98</t>
-  </si>
-  <si>
-    <t>PN PS4769 - PITOT STATIC TEST ADAPTOR</t>
-  </si>
-  <si>
-    <t>Reparo de CTVR 2 EA (2/2)</t>
-  </si>
-  <si>
-    <t>Material reparo acessórios PT6A-114A (3/3)</t>
-  </si>
-  <si>
-    <t>Requisições Consumíveis 3/4</t>
-  </si>
-  <si>
-    <t>Reparo de PTVR 2 EA (2/2)</t>
-  </si>
-  <si>
-    <t>Requisições Consumíveis 4/8</t>
-  </si>
-  <si>
-    <t>Requisições Consumíveis 6/8</t>
-  </si>
-  <si>
-    <t>Requisições Consumíveis 8/8</t>
-  </si>
-  <si>
-    <t>Requisições Consumíveis 4/4</t>
-  </si>
-  <si>
-    <t>Material reparo PT6A-114A (3/4)</t>
-  </si>
-  <si>
-    <t>Hora de Voo 01/10 - 1000 HV</t>
-  </si>
-  <si>
-    <t>Hora de Voo 02/10 - 1000 HV</t>
-  </si>
-  <si>
-    <t>Revisão Geral PT6A-114A (1/6)</t>
-  </si>
-  <si>
-    <t>Revisão Geral PT6A-114A (2/6)</t>
-  </si>
-  <si>
-    <t>Revisão Geral PT6A-114A</t>
-  </si>
-  <si>
-    <t>Exchange PT6A-114A</t>
-  </si>
-  <si>
-    <t>Hora de Voo 10/10 - 310 HV</t>
-  </si>
-  <si>
     <t>CABW</t>
   </si>
   <si>
@@ -496,13 +505,13 @@
     <t>A</t>
   </si>
   <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
     <t>B</t>
-  </si>
-  <si>
-    <t>C</t>
-  </si>
-  <si>
-    <t>D</t>
   </si>
   <si>
     <t>REQUISIÇÃO</t>
@@ -853,7 +862,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V82"/>
+  <dimension ref="A1:V83"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
@@ -938,37 +947,37 @@
         <v>24</v>
       </c>
       <c r="E2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="L2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="N2" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="O2" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="P2">
         <v>135000</v>
       </c>
       <c r="Q2" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="R2" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="S2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T2" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="U2" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="V2" s="1">
         <v>46229</v>
@@ -988,34 +997,34 @@
         <v>24</v>
       </c>
       <c r="E3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N3" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="O3" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="P3">
         <v>400000</v>
       </c>
       <c r="Q3" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="R3" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="S3" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T3" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="U3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V3" s="1">
         <v>46291</v>
@@ -1035,34 +1044,34 @@
         <v>24</v>
       </c>
       <c r="E4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N4" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="O4" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="P4">
         <v>430000</v>
       </c>
       <c r="Q4" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="R4" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="S4" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T4" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="U4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V4" s="1">
         <v>46260</v>
@@ -1082,34 +1091,34 @@
         <v>24</v>
       </c>
       <c r="E5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N5" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="O5" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="P5">
         <v>425000</v>
       </c>
       <c r="Q5" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="R5" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="S5" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T5" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="U5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V5" s="1">
         <v>46260</v>
@@ -1129,37 +1138,37 @@
         <v>24</v>
       </c>
       <c r="E6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="L6" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="N6" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="O6" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="P6">
         <v>563000</v>
       </c>
       <c r="Q6" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="R6" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="S6" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T6" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="U6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V6" s="1">
         <v>46291</v>
@@ -1179,43 +1188,43 @@
         <v>25</v>
       </c>
       <c r="E7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G7" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H7" s="1">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="N7" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="O7" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="P7">
         <v>3799999.6</v>
       </c>
       <c r="Q7" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="R7" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="S7" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T7" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="U7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V7" s="1">
         <v>46107</v>
@@ -1235,34 +1244,34 @@
         <v>24</v>
       </c>
       <c r="E8" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N8" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="O8" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="P8">
         <v>430000</v>
       </c>
       <c r="Q8" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="R8" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="S8" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T8" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="U8" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V8" s="1">
         <v>46291</v>
@@ -1282,34 +1291,34 @@
         <v>24</v>
       </c>
       <c r="E9" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F9" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N9" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="O9" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="P9">
         <v>60000</v>
       </c>
       <c r="Q9" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="R9" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="S9" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T9" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="U9" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V9" s="1">
         <v>46291</v>
@@ -1329,34 +1338,34 @@
         <v>24</v>
       </c>
       <c r="E10" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F10" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N10" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="O10" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="P10">
         <v>200000</v>
       </c>
       <c r="Q10" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="R10" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="S10" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T10" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="U10" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V10" s="1">
         <v>46291</v>
@@ -1376,34 +1385,34 @@
         <v>24</v>
       </c>
       <c r="E11" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F11" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N11" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="O11" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="P11">
         <v>320000</v>
       </c>
       <c r="Q11" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="R11" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="S11" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T11" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="U11" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V11" s="1">
         <v>46291</v>
@@ -1423,46 +1432,46 @@
         <v>25</v>
       </c>
       <c r="E12" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F12" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G12" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H12" s="1">
         <v>46079</v>
       </c>
       <c r="I12" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="J12" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="N12" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="O12" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="P12">
         <v>1187433.02</v>
       </c>
       <c r="Q12" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="R12" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="S12" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T12" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="U12" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="V12" s="1">
         <v>46107</v>
@@ -1482,34 +1491,34 @@
         <v>24</v>
       </c>
       <c r="E13" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F13" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N13" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="O13" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="P13">
         <v>1000000</v>
       </c>
       <c r="Q13" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="R13" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="S13" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T13" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="U13" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="V13" s="1">
         <v>46352</v>
@@ -1529,34 +1538,34 @@
         <v>24</v>
       </c>
       <c r="E14" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F14" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N14" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="O14" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="P14">
         <v>1000000</v>
       </c>
       <c r="Q14" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="R14" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="S14" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T14" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="U14" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="V14" s="1">
         <v>46352</v>
@@ -1576,34 +1585,34 @@
         <v>24</v>
       </c>
       <c r="E15" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F15" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N15" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="O15" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="P15">
         <v>1000000</v>
       </c>
       <c r="Q15" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="R15" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="S15" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T15" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="U15" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="V15" s="1">
         <v>46352</v>
@@ -1623,34 +1632,34 @@
         <v>24</v>
       </c>
       <c r="E16" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F16" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N16" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="O16" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="P16">
         <v>100000</v>
       </c>
       <c r="Q16" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="R16" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="S16" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T16" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="U16" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="V16" s="1">
         <v>46229</v>
@@ -1670,46 +1679,46 @@
         <v>25</v>
       </c>
       <c r="E17" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F17" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G17" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H17" s="1">
         <v>46098</v>
       </c>
       <c r="I17" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="J17" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="N17" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="O17" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="P17">
         <v>1770880.5</v>
       </c>
       <c r="Q17" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="R17" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="S17" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T17" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="U17" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="V17" s="1">
         <v>46107</v>
@@ -1729,43 +1738,43 @@
         <v>25</v>
       </c>
       <c r="E18" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F18" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G18" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H18" s="1">
         <v>46076</v>
       </c>
       <c r="I18" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="N18" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="O18" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="P18">
         <v>350000</v>
       </c>
       <c r="Q18" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="R18" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="S18" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T18" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="U18" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V18" s="1">
         <v>46079</v>
@@ -1785,43 +1794,43 @@
         <v>25</v>
       </c>
       <c r="E19" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F19" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G19" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H19" s="1">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="N19" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="O19" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="P19">
         <v>350000</v>
       </c>
       <c r="Q19" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="R19" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="S19" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T19" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="U19" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V19" s="1">
         <v>46079</v>
@@ -1841,34 +1850,34 @@
         <v>24</v>
       </c>
       <c r="E20" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F20" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N20" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="O20" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="P20">
         <v>1000000</v>
       </c>
       <c r="Q20" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="R20" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="S20" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T20" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="U20" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V20" s="1">
         <v>46291</v>
@@ -1888,34 +1897,34 @@
         <v>24</v>
       </c>
       <c r="E21" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F21" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N21" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="O21" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="P21">
         <v>400000</v>
       </c>
       <c r="Q21" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="R21" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="S21" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T21" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="U21" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V21" s="1">
         <v>46321</v>
@@ -1935,34 +1944,34 @@
         <v>24</v>
       </c>
       <c r="E22" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F22" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N22" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="O22" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="P22">
         <v>120000</v>
       </c>
       <c r="Q22" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="R22" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="S22" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T22" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="U22" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V22" s="1">
         <v>46321</v>
@@ -1982,34 +1991,34 @@
         <v>24</v>
       </c>
       <c r="E23" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F23" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N23" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="O23" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="P23">
         <v>80000</v>
       </c>
       <c r="Q23" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="R23" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="S23" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T23" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="U23" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V23" s="1">
         <v>46321</v>
@@ -2017,7 +2026,7 @@
     </row>
     <row r="24" spans="1:22">
       <c r="A24">
-        <v>16560</v>
+        <v>13760</v>
       </c>
       <c r="B24" t="s">
         <v>22</v>
@@ -2029,54 +2038,54 @@
         <v>25</v>
       </c>
       <c r="E24" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F24" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="G24" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H24" s="1">
-        <v>46213</v>
+        <v>46119</v>
       </c>
       <c r="I24" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="J24" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="N24" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="O24" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="P24">
-        <v>173846.38</v>
+        <v>1704503</v>
       </c>
       <c r="Q24" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="R24" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="S24" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T24" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="U24" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="V24" s="1">
-        <v>46229</v>
+        <v>46138</v>
       </c>
     </row>
     <row r="25" spans="1:22">
       <c r="A25">
-        <v>63960</v>
+        <v>14160</v>
       </c>
       <c r="B25" t="s">
         <v>22</v>
@@ -2085,42 +2094,54 @@
         <v>22</v>
       </c>
       <c r="D25" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E25" t="s">
         <v>29</v>
       </c>
+      <c r="F25" t="s">
+        <v>31</v>
+      </c>
+      <c r="G25" t="s">
+        <v>42</v>
+      </c>
+      <c r="H25" s="1">
+        <v>46121</v>
+      </c>
+      <c r="I25" t="s">
+        <v>52</v>
+      </c>
       <c r="N25" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="O25" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="P25">
-        <v>1000000</v>
+        <v>3799000</v>
       </c>
       <c r="Q25" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="R25" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="S25" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="T25" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="U25" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V25" s="1">
-        <v>46321</v>
+        <v>46168</v>
       </c>
     </row>
     <row r="26" spans="1:22">
       <c r="A26">
-        <v>13760</v>
+        <v>14161</v>
       </c>
       <c r="B26" t="s">
         <v>22</v>
@@ -2132,54 +2153,51 @@
         <v>25</v>
       </c>
       <c r="E26" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F26" t="s">
         <v>31</v>
       </c>
       <c r="G26" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H26" s="1">
-        <v>46119</v>
+        <v>46076</v>
       </c>
       <c r="I26" t="s">
-        <v>49</v>
-      </c>
-      <c r="J26" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="N26" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="O26" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="P26">
-        <v>1704503</v>
+        <v>1000</v>
       </c>
       <c r="Q26" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="R26" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="S26" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T26" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="U26" t="s">
-        <v>167</v>
+        <v>29</v>
       </c>
       <c r="V26" s="1">
-        <v>46138</v>
+        <v>46079</v>
       </c>
     </row>
     <row r="27" spans="1:22">
       <c r="A27">
-        <v>14160</v>
+        <v>14180</v>
       </c>
       <c r="B27" t="s">
         <v>22</v>
@@ -2188,54 +2206,45 @@
         <v>22</v>
       </c>
       <c r="D27" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E27" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F27" t="s">
-        <v>30</v>
-      </c>
-      <c r="G27" t="s">
-        <v>40</v>
-      </c>
-      <c r="H27" s="1">
-        <v>46121</v>
-      </c>
-      <c r="I27" t="s">
-        <v>50</v>
+        <v>31</v>
       </c>
       <c r="N27" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="O27" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="P27">
-        <v>3799000</v>
+        <v>100000</v>
       </c>
       <c r="Q27" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="R27" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="S27" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T27" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="U27" t="s">
-        <v>28</v>
+        <v>170</v>
       </c>
       <c r="V27" s="1">
-        <v>46168</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="28" spans="1:22">
       <c r="A28">
-        <v>14161</v>
+        <v>15380</v>
       </c>
       <c r="B28" t="s">
         <v>22</v>
@@ -2247,51 +2256,54 @@
         <v>25</v>
       </c>
       <c r="E28" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F28" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="G28" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H28" s="1">
-        <v>46076</v>
+        <v>46199</v>
       </c>
       <c r="I28" t="s">
-        <v>51</v>
+        <v>54</v>
+      </c>
+      <c r="J28" t="s">
+        <v>64</v>
       </c>
       <c r="N28" t="s">
         <v>76</v>
       </c>
       <c r="O28" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="P28">
-        <v>1000</v>
+        <v>150000</v>
       </c>
       <c r="Q28" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="R28" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="S28" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T28" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="U28" t="s">
-        <v>28</v>
+        <v>170</v>
       </c>
       <c r="V28" s="1">
-        <v>46079</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="29" spans="1:22">
       <c r="A29">
-        <v>14180</v>
+        <v>15400</v>
       </c>
       <c r="B29" t="s">
         <v>22</v>
@@ -2300,45 +2312,57 @@
         <v>22</v>
       </c>
       <c r="D29" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E29" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F29" t="s">
-        <v>30</v>
+        <v>33</v>
+      </c>
+      <c r="G29" t="s">
+        <v>42</v>
+      </c>
+      <c r="H29" s="1">
+        <v>46199</v>
+      </c>
+      <c r="I29" t="s">
+        <v>54</v>
+      </c>
+      <c r="J29" t="s">
+        <v>64</v>
       </c>
       <c r="N29" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="O29" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="P29">
-        <v>100000</v>
+        <v>150000</v>
       </c>
       <c r="Q29" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="R29" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="S29" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T29" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="U29" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="V29" s="1">
-        <v>46291</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="30" spans="1:22">
       <c r="A30">
-        <v>15380</v>
+        <v>15420</v>
       </c>
       <c r="B30" t="s">
         <v>22</v>
@@ -2350,46 +2374,46 @@
         <v>25</v>
       </c>
       <c r="E30" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F30" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G30" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H30" s="1">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="J30" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="N30" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="O30" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="P30">
-        <v>150000</v>
+        <v>18462.36</v>
       </c>
       <c r="Q30" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="R30" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="S30" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T30" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="U30" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="V30" s="1">
         <v>46199</v>
@@ -2397,7 +2421,7 @@
     </row>
     <row r="31" spans="1:22">
       <c r="A31">
-        <v>15400</v>
+        <v>15421</v>
       </c>
       <c r="B31" t="s">
         <v>22</v>
@@ -2409,46 +2433,46 @@
         <v>25</v>
       </c>
       <c r="E31" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F31" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G31" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H31" s="1">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="J31" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="N31" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="O31" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="P31">
-        <v>150000</v>
+        <v>324166.14</v>
       </c>
       <c r="Q31" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="R31" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="S31" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T31" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="U31" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="V31" s="1">
         <v>46199</v>
@@ -2456,7 +2480,7 @@
     </row>
     <row r="32" spans="1:22">
       <c r="A32">
-        <v>15420</v>
+        <v>15440</v>
       </c>
       <c r="B32" t="s">
         <v>22</v>
@@ -2465,57 +2489,45 @@
         <v>22</v>
       </c>
       <c r="D32" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E32" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F32" t="s">
-        <v>33</v>
-      </c>
-      <c r="G32" t="s">
-        <v>40</v>
-      </c>
-      <c r="H32" s="1">
-        <v>46199</v>
-      </c>
-      <c r="I32" t="s">
-        <v>53</v>
-      </c>
-      <c r="J32" t="s">
-        <v>62</v>
+        <v>31</v>
       </c>
       <c r="N32" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="O32" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="P32">
-        <v>18462.36</v>
+        <v>30000</v>
       </c>
       <c r="Q32" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="R32" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="S32" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T32" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="U32" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="V32" s="1">
-        <v>46199</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="33" spans="1:22">
       <c r="A33">
-        <v>15421</v>
+        <v>15680</v>
       </c>
       <c r="B33" t="s">
         <v>22</v>
@@ -2527,46 +2539,46 @@
         <v>25</v>
       </c>
       <c r="E33" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F33" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G33" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H33" s="1">
-        <v>46199</v>
+        <v>46191</v>
       </c>
       <c r="I33" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="J33" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="N33" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="O33" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="P33">
-        <v>324166.14</v>
+        <v>1496713.48</v>
       </c>
       <c r="Q33" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="R33" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="S33" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T33" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="U33" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="V33" s="1">
         <v>46199</v>
@@ -2574,7 +2586,7 @@
     </row>
     <row r="34" spans="1:22">
       <c r="A34">
-        <v>15440</v>
+        <v>15681</v>
       </c>
       <c r="B34" t="s">
         <v>22</v>
@@ -2583,45 +2595,54 @@
         <v>22</v>
       </c>
       <c r="D34" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E34" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F34" t="s">
-        <v>30</v>
+        <v>32</v>
+      </c>
+      <c r="G34" t="s">
+        <v>42</v>
+      </c>
+      <c r="H34" s="1">
+        <v>46119</v>
+      </c>
+      <c r="I34" t="s">
+        <v>51</v>
       </c>
       <c r="N34" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="O34" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="P34">
-        <v>30000</v>
+        <v>207789.52</v>
       </c>
       <c r="Q34" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="R34" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="S34" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T34" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="U34" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="V34" s="1">
-        <v>46291</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="35" spans="1:22">
       <c r="A35">
-        <v>15680</v>
+        <v>15960</v>
       </c>
       <c r="B35" t="s">
         <v>22</v>
@@ -2633,54 +2654,51 @@
         <v>25</v>
       </c>
       <c r="E35" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F35" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G35" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H35" s="1">
-        <v>46191</v>
+        <v>46213</v>
       </c>
       <c r="I35" t="s">
-        <v>48</v>
-      </c>
-      <c r="J35" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="N35" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="O35" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="P35">
-        <v>1496713.48</v>
+        <v>962290.8</v>
       </c>
       <c r="Q35" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="R35" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="S35" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T35" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="U35" t="s">
-        <v>167</v>
+        <v>29</v>
       </c>
       <c r="V35" s="1">
-        <v>46199</v>
+        <v>46260</v>
       </c>
     </row>
     <row r="36" spans="1:22">
       <c r="A36">
-        <v>15681</v>
+        <v>15961</v>
       </c>
       <c r="B36" t="s">
         <v>22</v>
@@ -2692,51 +2710,51 @@
         <v>25</v>
       </c>
       <c r="E36" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F36" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="G36" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H36" s="1">
-        <v>46119</v>
+        <v>46175</v>
       </c>
       <c r="I36" t="s">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="N36" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="O36" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="P36">
-        <v>207789.52</v>
+        <v>800000</v>
       </c>
       <c r="Q36" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="R36" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="S36" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T36" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="U36" t="s">
-        <v>167</v>
+        <v>29</v>
       </c>
       <c r="V36" s="1">
-        <v>46199</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="37" spans="1:22">
       <c r="A37">
-        <v>15960</v>
+        <v>15962</v>
       </c>
       <c r="B37" t="s">
         <v>22</v>
@@ -2748,43 +2766,43 @@
         <v>25</v>
       </c>
       <c r="E37" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F37" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G37" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H37" s="1">
         <v>46213</v>
       </c>
       <c r="I37" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="N37" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="O37" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="P37">
-        <v>962290.8</v>
+        <v>1530656.62</v>
       </c>
       <c r="Q37" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="R37" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="S37" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T37" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="U37" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V37" s="1">
         <v>46260</v>
@@ -2792,7 +2810,7 @@
     </row>
     <row r="38" spans="1:22">
       <c r="A38">
-        <v>15961</v>
+        <v>15963</v>
       </c>
       <c r="B38" t="s">
         <v>22</v>
@@ -2804,51 +2822,51 @@
         <v>25</v>
       </c>
       <c r="E38" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F38" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G38" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H38" s="1">
-        <v>46175</v>
+        <v>46199</v>
       </c>
       <c r="I38" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="N38" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="O38" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="P38">
-        <v>800000</v>
+        <v>72958.08</v>
       </c>
       <c r="Q38" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="R38" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="S38" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T38" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="U38" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V38" s="1">
-        <v>46229</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="39" spans="1:22">
       <c r="A39">
-        <v>15962</v>
+        <v>15964</v>
       </c>
       <c r="B39" t="s">
         <v>22</v>
@@ -2860,51 +2878,51 @@
         <v>25</v>
       </c>
       <c r="E39" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F39" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="G39" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H39" s="1">
-        <v>46213</v>
+        <v>46199</v>
       </c>
       <c r="I39" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="N39" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="O39" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="P39">
-        <v>1530656.62</v>
+        <v>8916</v>
       </c>
       <c r="Q39" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="R39" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="S39" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T39" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="U39" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V39" s="1">
-        <v>46260</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="40" spans="1:22">
       <c r="A40">
-        <v>15963</v>
+        <v>15965</v>
       </c>
       <c r="B40" t="s">
         <v>22</v>
@@ -2916,43 +2934,43 @@
         <v>25</v>
       </c>
       <c r="E40" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F40" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="G40" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H40" s="1">
-        <v>46199</v>
+        <v>46204</v>
       </c>
       <c r="I40" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="N40" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="O40" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="P40">
-        <v>72958.08</v>
+        <v>425178.5</v>
       </c>
       <c r="Q40" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="R40" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="S40" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T40" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="U40" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V40" s="1">
         <v>46199</v>
@@ -2960,7 +2978,7 @@
     </row>
     <row r="41" spans="1:22">
       <c r="A41">
-        <v>15964</v>
+        <v>15980</v>
       </c>
       <c r="B41" t="s">
         <v>22</v>
@@ -2969,54 +2987,42 @@
         <v>22</v>
       </c>
       <c r="D41" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E41" t="s">
-        <v>28</v>
-      </c>
-      <c r="F41" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="G41" t="s">
-        <v>40</v>
-      </c>
-      <c r="H41" s="1">
-        <v>46199</v>
-      </c>
-      <c r="I41" t="s">
-        <v>56</v>
+        <v>43</v>
       </c>
       <c r="N41" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="O41" t="s">
-        <v>117</v>
-      </c>
-      <c r="P41">
-        <v>8916</v>
+        <v>119</v>
       </c>
       <c r="Q41" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="R41" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="S41" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="T41" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="U41" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V41" s="1">
-        <v>46199</v>
+        <v>46260</v>
       </c>
     </row>
     <row r="42" spans="1:22">
       <c r="A42">
-        <v>15965</v>
+        <v>16000</v>
       </c>
       <c r="B42" t="s">
         <v>22</v>
@@ -3028,43 +3034,43 @@
         <v>25</v>
       </c>
       <c r="E42" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F42" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="G42" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H42" s="1">
-        <v>46204</v>
+        <v>46191</v>
       </c>
       <c r="I42" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="N42" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O42" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="P42">
-        <v>425178.5</v>
+        <v>400000</v>
       </c>
       <c r="Q42" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="R42" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="S42" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T42" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="U42" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V42" s="1">
         <v>46199</v>
@@ -3072,7 +3078,7 @@
     </row>
     <row r="43" spans="1:22">
       <c r="A43">
-        <v>15980</v>
+        <v>16001</v>
       </c>
       <c r="B43" t="s">
         <v>22</v>
@@ -3081,42 +3087,54 @@
         <v>22</v>
       </c>
       <c r="D43" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E43" t="s">
         <v>29</v>
       </c>
+      <c r="F43" t="s">
+        <v>31</v>
+      </c>
       <c r="G43" t="s">
-        <v>41</v>
+        <v>42</v>
+      </c>
+      <c r="H43" s="1">
+        <v>46191</v>
+      </c>
+      <c r="I43" t="s">
+        <v>60</v>
       </c>
       <c r="N43" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O43" t="s">
-        <v>118</v>
+        <v>121</v>
+      </c>
+      <c r="P43">
+        <v>400000</v>
       </c>
       <c r="Q43" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="R43" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="S43" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T43" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="U43" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V43" s="1">
-        <v>46260</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="44" spans="1:22">
       <c r="A44">
-        <v>16000</v>
+        <v>16560</v>
       </c>
       <c r="B44" t="s">
         <v>22</v>
@@ -3128,51 +3146,54 @@
         <v>25</v>
       </c>
       <c r="E44" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F44" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G44" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H44" s="1">
-        <v>46191</v>
+        <v>46213</v>
       </c>
       <c r="I44" t="s">
-        <v>57</v>
+        <v>56</v>
+      </c>
+      <c r="J44" t="s">
+        <v>66</v>
       </c>
       <c r="N44" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="O44" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="P44">
-        <v>400000</v>
+        <v>173846.38</v>
       </c>
       <c r="Q44" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="R44" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="S44" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T44" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="U44" t="s">
-        <v>28</v>
+        <v>170</v>
       </c>
       <c r="V44" s="1">
-        <v>46199</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="45" spans="1:22">
       <c r="A45">
-        <v>16001</v>
+        <v>16561</v>
       </c>
       <c r="B45" t="s">
         <v>22</v>
@@ -3184,51 +3205,51 @@
         <v>25</v>
       </c>
       <c r="E45" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F45" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="G45" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H45" s="1">
-        <v>46191</v>
+        <v>46210</v>
       </c>
       <c r="I45" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="N45" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="O45" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="P45">
-        <v>400000</v>
+        <v>1530656.62</v>
       </c>
       <c r="Q45" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="R45" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="S45" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T45" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="U45" t="s">
-        <v>28</v>
+        <v>170</v>
       </c>
       <c r="V45" s="1">
-        <v>46199</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="46" spans="1:22">
       <c r="A46">
-        <v>17760</v>
+        <v>16700</v>
       </c>
       <c r="B46" t="s">
         <v>22</v>
@@ -3240,40 +3261,34 @@
         <v>24</v>
       </c>
       <c r="E46" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F46" t="s">
-        <v>30</v>
-      </c>
-      <c r="J46" t="s">
-        <v>60</v>
-      </c>
-      <c r="K46" t="s">
-        <v>65</v>
+        <v>31</v>
       </c>
       <c r="N46" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="O46" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="P46">
-        <v>1704503</v>
+        <v>1000000</v>
       </c>
       <c r="Q46" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="R46" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="S46" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T46" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="U46" t="s">
-        <v>167</v>
+        <v>29</v>
       </c>
       <c r="V46" s="1">
         <v>46260</v>
@@ -3281,7 +3296,7 @@
     </row>
     <row r="47" spans="1:22">
       <c r="A47">
-        <v>16561</v>
+        <v>17200</v>
       </c>
       <c r="B47" t="s">
         <v>22</v>
@@ -3290,54 +3305,45 @@
         <v>22</v>
       </c>
       <c r="D47" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E47" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F47" t="s">
-        <v>33</v>
-      </c>
-      <c r="G47" t="s">
-        <v>40</v>
-      </c>
-      <c r="H47" s="1">
-        <v>46210</v>
-      </c>
-      <c r="I47" t="s">
-        <v>53</v>
+        <v>31</v>
       </c>
       <c r="N47" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="O47" t="s">
-        <v>107</v>
+        <v>124</v>
       </c>
       <c r="P47">
-        <v>1530656.62</v>
+        <v>958040</v>
       </c>
       <c r="Q47" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="R47" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="S47" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T47" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="U47" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="V47" s="1">
-        <v>46229</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="48" spans="1:22">
       <c r="A48">
-        <v>16700</v>
+        <v>17201</v>
       </c>
       <c r="B48" t="s">
         <v>22</v>
@@ -3346,45 +3352,57 @@
         <v>22</v>
       </c>
       <c r="D48" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E48" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F48" t="s">
-        <v>30</v>
+        <v>31</v>
+      </c>
+      <c r="G48" t="s">
+        <v>42</v>
+      </c>
+      <c r="H48" s="1">
+        <v>46176</v>
+      </c>
+      <c r="I48" t="s">
+        <v>61</v>
+      </c>
+      <c r="J48" t="s">
+        <v>67</v>
       </c>
       <c r="N48" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="O48" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="P48">
-        <v>1000000</v>
+        <v>41730.64</v>
       </c>
       <c r="Q48" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="R48" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="S48" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T48" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="U48" t="s">
-        <v>28</v>
+        <v>170</v>
       </c>
       <c r="V48" s="1">
-        <v>46260</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="49" spans="1:22">
       <c r="A49">
-        <v>17200</v>
+        <v>17760</v>
       </c>
       <c r="B49" t="s">
         <v>22</v>
@@ -3396,42 +3414,48 @@
         <v>24</v>
       </c>
       <c r="E49" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F49" t="s">
-        <v>30</v>
+        <v>31</v>
+      </c>
+      <c r="J49" t="s">
+        <v>66</v>
+      </c>
+      <c r="K49" t="s">
+        <v>68</v>
       </c>
       <c r="N49" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="O49" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="P49">
-        <v>958040</v>
+        <v>1468159.32</v>
       </c>
       <c r="Q49" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="R49" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="S49" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T49" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="U49" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="V49" s="1">
-        <v>46291</v>
+        <v>46260</v>
       </c>
     </row>
     <row r="50" spans="1:22">
       <c r="A50">
-        <v>17201</v>
+        <v>17761</v>
       </c>
       <c r="B50" t="s">
         <v>22</v>
@@ -3440,49 +3464,43 @@
         <v>22</v>
       </c>
       <c r="D50" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E50" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F50" t="s">
-        <v>30</v>
-      </c>
-      <c r="G50" t="s">
-        <v>40</v>
-      </c>
-      <c r="H50" s="1">
-        <v>46176</v>
-      </c>
-      <c r="I50" t="s">
-        <v>58</v>
+        <v>31</v>
       </c>
       <c r="J50" t="s">
-        <v>64</v>
+        <v>66</v>
+      </c>
+      <c r="K50" t="s">
+        <v>69</v>
       </c>
       <c r="N50" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="O50" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="P50">
-        <v>41730.64</v>
+        <v>1704503</v>
       </c>
       <c r="Q50" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="R50" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="S50" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T50" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="U50" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="V50" s="1">
         <v>46291</v>
@@ -3502,34 +3520,34 @@
         <v>24</v>
       </c>
       <c r="E51" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F51" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N51" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="O51" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="P51">
         <v>1704503</v>
       </c>
       <c r="Q51" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="R51" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="S51" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T51" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="U51" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="V51" s="1">
         <v>46321</v>
@@ -3537,7 +3555,7 @@
     </row>
     <row r="52" spans="1:22">
       <c r="A52">
-        <v>18140</v>
+        <v>17763</v>
       </c>
       <c r="B52" t="s">
         <v>22</v>
@@ -3546,45 +3564,51 @@
         <v>22</v>
       </c>
       <c r="D52" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E52" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F52" t="s">
-        <v>30</v>
+        <v>39</v>
+      </c>
+      <c r="G52" t="s">
+        <v>44</v>
+      </c>
+      <c r="H52" s="1">
+        <v>46227</v>
       </c>
       <c r="N52" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="O52" t="s">
         <v>125</v>
       </c>
       <c r="P52">
-        <v>1295422.28</v>
+        <v>236343.68</v>
       </c>
       <c r="Q52" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="R52" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="S52" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T52" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="U52" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="V52" s="1">
-        <v>46352</v>
+        <v>46260</v>
       </c>
     </row>
     <row r="53" spans="1:22">
       <c r="A53">
-        <v>17761</v>
+        <v>18140</v>
       </c>
       <c r="B53" t="s">
         <v>22</v>
@@ -3596,43 +3620,37 @@
         <v>24</v>
       </c>
       <c r="E53" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F53" t="s">
-        <v>30</v>
-      </c>
-      <c r="J53" t="s">
-        <v>60</v>
-      </c>
-      <c r="K53" t="s">
-        <v>66</v>
+        <v>31</v>
       </c>
       <c r="N53" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="O53" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="P53">
-        <v>1704503</v>
+        <v>1295422.28</v>
       </c>
       <c r="Q53" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="R53" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="S53" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T53" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="U53" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="V53" s="1">
-        <v>46291</v>
+        <v>46352</v>
       </c>
     </row>
     <row r="54" spans="1:22">
@@ -3649,34 +3667,34 @@
         <v>24</v>
       </c>
       <c r="E54" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F54" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="N54" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="O54" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="P54">
         <v>500000</v>
       </c>
       <c r="Q54" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="R54" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="S54" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="T54" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="U54" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="V54" s="1">
         <v>46321</v>
@@ -3696,37 +3714,37 @@
         <v>26</v>
       </c>
       <c r="E55" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F55" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G55" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="N55" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="O55" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="P55">
         <v>5000000</v>
       </c>
       <c r="Q55" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="R55" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="S55" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="T55" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="U55" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="V55" s="1">
         <v>46321</v>
@@ -3746,34 +3764,34 @@
         <v>24</v>
       </c>
       <c r="E56" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F56" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="N56" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="O56" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="P56">
         <v>4000000</v>
       </c>
       <c r="Q56" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="R56" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="S56" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="T56" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="U56" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="V56" s="1">
         <v>46049</v>
@@ -3793,34 +3811,34 @@
         <v>26</v>
       </c>
       <c r="E57" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F57" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="N57" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="O57" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="P57">
         <v>5500000</v>
       </c>
       <c r="Q57" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="R57" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="S57" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="T57" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="U57" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
     </row>
     <row r="58" spans="1:22">
@@ -3837,39 +3855,39 @@
         <v>26</v>
       </c>
       <c r="E58" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F58" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="N58" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="O58" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="P58">
         <v>5500000</v>
       </c>
       <c r="Q58" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="R58" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="S58" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="T58" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="U58" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
     </row>
     <row r="59" spans="1:22">
       <c r="A59">
-        <v>23080</v>
+        <v>23120</v>
       </c>
       <c r="B59" t="s">
         <v>22</v>
@@ -3881,31 +3899,31 @@
         <v>26</v>
       </c>
       <c r="E59" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N59" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="O59" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="P59">
-        <v>4064.54</v>
+        <v>9389.959999999999</v>
       </c>
       <c r="Q59" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="R59" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="S59" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="T59" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="U59" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="V59" s="1">
         <v>46107</v>
@@ -3913,7 +3931,7 @@
     </row>
     <row r="60" spans="1:22">
       <c r="A60">
-        <v>23100</v>
+        <v>23160</v>
       </c>
       <c r="B60" t="s">
         <v>22</v>
@@ -3925,31 +3943,31 @@
         <v>26</v>
       </c>
       <c r="E60" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N60" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="O60" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="P60">
-        <v>4227.84</v>
+        <v>7204.82</v>
       </c>
       <c r="Q60" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="R60" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="S60" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="T60" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="U60" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="V60" s="1">
         <v>46107</v>
@@ -3957,7 +3975,7 @@
     </row>
     <row r="61" spans="1:22">
       <c r="A61">
-        <v>23120</v>
+        <v>23100</v>
       </c>
       <c r="B61" t="s">
         <v>22</v>
@@ -3969,31 +3987,31 @@
         <v>26</v>
       </c>
       <c r="E61" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N61" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="O61" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="P61">
-        <v>9389.959999999999</v>
+        <v>4227.84</v>
       </c>
       <c r="Q61" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="R61" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="S61" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="T61" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="U61" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="V61" s="1">
         <v>46107</v>
@@ -4001,7 +4019,7 @@
     </row>
     <row r="62" spans="1:22">
       <c r="A62">
-        <v>23140</v>
+        <v>23080</v>
       </c>
       <c r="B62" t="s">
         <v>22</v>
@@ -4013,31 +4031,31 @@
         <v>26</v>
       </c>
       <c r="E62" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N62" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="O62" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="P62">
-        <v>1163.64</v>
+        <v>4064.54</v>
       </c>
       <c r="Q62" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="R62" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="S62" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="T62" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="U62" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="V62" s="1">
         <v>46107</v>
@@ -4045,7 +4063,7 @@
     </row>
     <row r="63" spans="1:22">
       <c r="A63">
-        <v>23160</v>
+        <v>23180</v>
       </c>
       <c r="B63" t="s">
         <v>22</v>
@@ -4057,31 +4075,31 @@
         <v>26</v>
       </c>
       <c r="E63" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N63" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="O63" t="s">
         <v>135</v>
       </c>
       <c r="P63">
-        <v>7204.82</v>
+        <v>3662.66</v>
       </c>
       <c r="Q63" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="R63" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="S63" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="T63" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="U63" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="V63" s="1">
         <v>46107</v>
@@ -4089,7 +4107,7 @@
     </row>
     <row r="64" spans="1:22">
       <c r="A64">
-        <v>23180</v>
+        <v>23140</v>
       </c>
       <c r="B64" t="s">
         <v>22</v>
@@ -4101,31 +4119,31 @@
         <v>26</v>
       </c>
       <c r="E64" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N64" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="O64" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="P64">
-        <v>3662.66</v>
+        <v>1163.64</v>
       </c>
       <c r="Q64" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="R64" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="S64" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="T64" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="U64" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="V64" s="1">
         <v>46107</v>
@@ -4145,31 +4163,31 @@
         <v>26</v>
       </c>
       <c r="E65" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N65" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="O65" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="P65">
         <v>120000</v>
       </c>
       <c r="Q65" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="R65" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="S65" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="T65" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="U65" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V65" s="1">
         <v>46168</v>
@@ -4189,34 +4207,34 @@
         <v>24</v>
       </c>
       <c r="E66" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F66" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N66" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="O66" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="P66">
         <v>400000</v>
       </c>
       <c r="Q66" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="R66" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="S66" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T66" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="U66" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V66" s="1">
         <v>46291</v>
@@ -4236,34 +4254,34 @@
         <v>24</v>
       </c>
       <c r="E67" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F67" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N67" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="O67" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="P67">
         <v>100000</v>
       </c>
       <c r="Q67" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="R67" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="S67" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T67" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="U67" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="V67" s="1">
         <v>46229</v>
@@ -4283,31 +4301,31 @@
         <v>26</v>
       </c>
       <c r="E68" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N68" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="O68" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="P68">
         <v>80000</v>
       </c>
       <c r="Q68" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="R68" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="S68" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="T68" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="U68" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V68" s="1">
         <v>46260</v>
@@ -4327,31 +4345,31 @@
         <v>26</v>
       </c>
       <c r="E69" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N69" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="O69" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="P69">
         <v>835000</v>
       </c>
       <c r="Q69" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="R69" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="S69" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="T69" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="U69" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="V69" s="1">
         <v>46291</v>
@@ -4371,31 +4389,31 @@
         <v>26</v>
       </c>
       <c r="E70" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N70" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="O70" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="P70">
         <v>165000</v>
       </c>
       <c r="Q70" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="R70" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="S70" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="T70" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="U70" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="V70" s="1">
         <v>46168</v>
@@ -4415,31 +4433,31 @@
         <v>26</v>
       </c>
       <c r="E71" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N71" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="O71" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="P71">
         <v>1000000</v>
       </c>
       <c r="Q71" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="R71" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="S71" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="T71" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="U71" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="V71" s="1">
         <v>46291</v>
@@ -4459,31 +4477,31 @@
         <v>26</v>
       </c>
       <c r="E72" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N72" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="O72" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="P72">
         <v>1000000</v>
       </c>
       <c r="Q72" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="R72" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="S72" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="T72" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="U72" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="V72" s="1">
         <v>46291</v>
@@ -4503,31 +4521,31 @@
         <v>26</v>
       </c>
       <c r="E73" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N73" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="O73" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="P73">
         <v>100000</v>
       </c>
       <c r="Q73" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="R73" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="S73" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="T73" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="U73" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="V73" s="1">
         <v>46291</v>
@@ -4547,34 +4565,34 @@
         <v>24</v>
       </c>
       <c r="E74" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F74" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N74" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="O74" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="P74">
         <v>1000000</v>
       </c>
       <c r="Q74" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="R74" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="S74" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T74" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="U74" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V74" s="1">
         <v>46321</v>
@@ -4591,40 +4609,40 @@
         <v>22</v>
       </c>
       <c r="D75" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E75" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F75" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="G75" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="N75" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="O75" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="P75">
         <v>1704503</v>
       </c>
       <c r="Q75" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="R75" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="S75" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="T75" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="U75" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="V75" s="1">
         <v>46381</v>
@@ -4641,40 +4659,40 @@
         <v>22</v>
       </c>
       <c r="D76" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E76" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F76" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="G76" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="N76" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="O76" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="P76">
         <v>1638125.5</v>
       </c>
       <c r="Q76" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="R76" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="S76" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="T76" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="U76" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="V76" s="1">
         <v>46381</v>
@@ -4691,40 +4709,40 @@
         <v>22</v>
       </c>
       <c r="D77" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E77" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F77" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="G77" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="N77" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="O77" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="P77">
         <v>3800000</v>
       </c>
       <c r="Q77" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="R77" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="S77" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="T77" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="U77" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V77" s="1">
         <v>46381</v>
@@ -4741,40 +4759,40 @@
         <v>22</v>
       </c>
       <c r="D78" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E78" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F78" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="G78" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="N78" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="O78" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="P78">
         <v>3800000</v>
       </c>
       <c r="Q78" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="R78" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="S78" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="T78" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="U78" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V78" s="1">
         <v>46381</v>
@@ -4794,31 +4812,31 @@
         <v>26</v>
       </c>
       <c r="E79" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N79" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="O79" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="P79">
         <v>3800000</v>
       </c>
       <c r="Q79" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="R79" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="S79" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="T79" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="U79" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V79" s="1">
         <v>46382</v>
@@ -4838,31 +4856,31 @@
         <v>24</v>
       </c>
       <c r="E80" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N80" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="O80" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="P80">
         <v>4394700</v>
       </c>
       <c r="Q80" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="R80" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="S80" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="T80" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="U80" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V80" s="1">
         <v>46382</v>
@@ -4882,34 +4900,34 @@
         <v>24</v>
       </c>
       <c r="E81" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F81" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N81" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="O81" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="P81">
         <v>528395.9300000001</v>
       </c>
       <c r="Q81" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="R81" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="S81" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T81" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="U81" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="V81" s="1">
         <v>46382</v>
@@ -4917,45 +4935,89 @@
     </row>
     <row r="82" spans="1:22">
       <c r="A82">
+        <v>63960</v>
+      </c>
+      <c r="B82" t="s">
+        <v>22</v>
+      </c>
+      <c r="C82" t="s">
+        <v>22</v>
+      </c>
+      <c r="D82" t="s">
+        <v>26</v>
+      </c>
+      <c r="E82" t="s">
+        <v>30</v>
+      </c>
+      <c r="N82" t="s">
+        <v>78</v>
+      </c>
+      <c r="O82" t="s">
+        <v>154</v>
+      </c>
+      <c r="P82">
+        <v>1000000</v>
+      </c>
+      <c r="Q82" t="s">
+        <v>157</v>
+      </c>
+      <c r="R82" t="s">
+        <v>159</v>
+      </c>
+      <c r="S82" t="s">
+        <v>165</v>
+      </c>
+      <c r="T82" t="s">
+        <v>167</v>
+      </c>
+      <c r="U82" t="s">
+        <v>29</v>
+      </c>
+      <c r="V82" s="1">
+        <v>46321</v>
+      </c>
+    </row>
+    <row r="83" spans="1:22">
+      <c r="A83">
         <v>64340</v>
       </c>
-      <c r="B82" t="s">
-        <v>22</v>
-      </c>
-      <c r="C82" t="s">
-        <v>22</v>
-      </c>
-      <c r="D82" t="s">
+      <c r="B83" t="s">
+        <v>22</v>
+      </c>
+      <c r="C83" t="s">
+        <v>22</v>
+      </c>
+      <c r="D83" t="s">
         <v>24</v>
       </c>
-      <c r="E82" t="s">
-        <v>28</v>
-      </c>
-      <c r="N82" t="s">
-        <v>84</v>
-      </c>
-      <c r="O82" t="s">
-        <v>150</v>
-      </c>
-      <c r="P82">
+      <c r="E83" t="s">
+        <v>29</v>
+      </c>
+      <c r="N83" t="s">
+        <v>87</v>
+      </c>
+      <c r="O83" t="s">
+        <v>152</v>
+      </c>
+      <c r="P83">
         <v>4394700</v>
       </c>
-      <c r="Q82" t="s">
-        <v>152</v>
-      </c>
-      <c r="R82" t="s">
-        <v>156</v>
-      </c>
-      <c r="S82" t="s">
-        <v>161</v>
-      </c>
-      <c r="T82" t="s">
-        <v>164</v>
-      </c>
-      <c r="U82" t="s">
-        <v>28</v>
-      </c>
-      <c r="V82" s="1">
+      <c r="Q83" t="s">
+        <v>155</v>
+      </c>
+      <c r="R83" t="s">
+        <v>159</v>
+      </c>
+      <c r="S83" t="s">
+        <v>163</v>
+      </c>
+      <c r="T83" t="s">
+        <v>167</v>
+      </c>
+      <c r="U83" t="s">
+        <v>29</v>
+      </c>
+      <c r="V83" s="1">
         <v>46382</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (28/07/2026 17:50)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1061" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1062" uniqueCount="170">
   <si>
     <t>linha</t>
   </si>
@@ -97,9 +97,6 @@
     <t>Não aprovado</t>
   </si>
   <si>
-    <t>Em trâmite</t>
-  </si>
-  <si>
     <t>Sem informação</t>
   </si>
   <si>
@@ -148,9 +145,6 @@
     <t>CANCELADO</t>
   </si>
   <si>
-    <t>EM TRÂMITE</t>
-  </si>
-  <si>
     <t>BLOQUEIO</t>
   </si>
   <si>
@@ -200,6 +194,9 @@
   </si>
   <si>
     <t>C26116</t>
+  </si>
+  <si>
+    <t>C26363</t>
   </si>
   <si>
     <t>1</t>
@@ -947,37 +944,37 @@
         <v>24</v>
       </c>
       <c r="E2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="L2" t="s">
+        <v>69</v>
+      </c>
+      <c r="N2" t="s">
         <v>70</v>
       </c>
-      <c r="N2" t="s">
-        <v>71</v>
-      </c>
       <c r="O2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="P2">
         <v>135000</v>
       </c>
       <c r="Q2" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="R2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="S2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="U2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="V2" s="1">
         <v>46229</v>
@@ -997,34 +994,34 @@
         <v>24</v>
       </c>
       <c r="E3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="O3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="P3">
         <v>400000</v>
       </c>
       <c r="Q3" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="R3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="S3" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T3" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="U3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V3" s="1">
         <v>46291</v>
@@ -1044,34 +1041,34 @@
         <v>24</v>
       </c>
       <c r="E4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="O4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="P4">
         <v>430000</v>
       </c>
       <c r="Q4" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="R4" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="S4" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="U4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V4" s="1">
         <v>46260</v>
@@ -1091,34 +1088,34 @@
         <v>24</v>
       </c>
       <c r="E5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="O5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="P5">
         <v>425000</v>
       </c>
       <c r="Q5" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="R5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="S5" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T5" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="U5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V5" s="1">
         <v>46260</v>
@@ -1138,37 +1135,37 @@
         <v>24</v>
       </c>
       <c r="E6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="L6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="N6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="P6">
         <v>563000</v>
       </c>
       <c r="Q6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="R6" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="S6" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T6" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="U6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V6" s="1">
         <v>46291</v>
@@ -1188,43 +1185,43 @@
         <v>25</v>
       </c>
       <c r="E7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H7" s="1">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="N7" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="O7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="P7">
         <v>3799999.6</v>
       </c>
       <c r="Q7" t="s">
+        <v>156</v>
+      </c>
+      <c r="R7" t="s">
         <v>157</v>
       </c>
-      <c r="R7" t="s">
-        <v>158</v>
-      </c>
       <c r="S7" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T7" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="U7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V7" s="1">
         <v>46107</v>
@@ -1244,34 +1241,34 @@
         <v>24</v>
       </c>
       <c r="E8" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="O8" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="P8">
         <v>430000</v>
       </c>
       <c r="Q8" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="R8" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="S8" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="U8" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V8" s="1">
         <v>46291</v>
@@ -1291,34 +1288,34 @@
         <v>24</v>
       </c>
       <c r="E9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="O9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="P9">
         <v>60000</v>
       </c>
       <c r="Q9" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="R9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="S9" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T9" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="U9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V9" s="1">
         <v>46291</v>
@@ -1338,34 +1335,34 @@
         <v>24</v>
       </c>
       <c r="E10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O10" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="P10">
         <v>200000</v>
       </c>
       <c r="Q10" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="R10" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="S10" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T10" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="U10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V10" s="1">
         <v>46291</v>
@@ -1385,34 +1382,34 @@
         <v>24</v>
       </c>
       <c r="E11" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O11" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="P11">
         <v>320000</v>
       </c>
       <c r="Q11" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="R11" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="S11" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T11" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="U11" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V11" s="1">
         <v>46291</v>
@@ -1432,46 +1429,46 @@
         <v>25</v>
       </c>
       <c r="E12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F12" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G12" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H12" s="1">
         <v>46079</v>
       </c>
       <c r="I12" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="J12" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="N12" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="O12" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="P12">
         <v>1187433.02</v>
       </c>
       <c r="Q12" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="R12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="S12" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T12" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="U12" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="V12" s="1">
         <v>46107</v>
@@ -1491,34 +1488,34 @@
         <v>24</v>
       </c>
       <c r="E13" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F13" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N13" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="O13" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="P13">
         <v>1000000</v>
       </c>
       <c r="Q13" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="R13" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="S13" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T13" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="U13" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="V13" s="1">
         <v>46352</v>
@@ -1538,34 +1535,34 @@
         <v>24</v>
       </c>
       <c r="E14" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F14" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="O14" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="P14">
         <v>1000000</v>
       </c>
       <c r="Q14" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="R14" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="S14" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T14" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="U14" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="V14" s="1">
         <v>46352</v>
@@ -1585,34 +1582,34 @@
         <v>24</v>
       </c>
       <c r="E15" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F15" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="O15" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="P15">
         <v>1000000</v>
       </c>
       <c r="Q15" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="R15" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="S15" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T15" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="U15" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="V15" s="1">
         <v>46352</v>
@@ -1632,34 +1629,34 @@
         <v>24</v>
       </c>
       <c r="E16" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F16" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N16" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O16" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="P16">
         <v>100000</v>
       </c>
       <c r="Q16" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="R16" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="S16" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T16" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="U16" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="V16" s="1">
         <v>46229</v>
@@ -1679,46 +1676,46 @@
         <v>25</v>
       </c>
       <c r="E17" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F17" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G17" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H17" s="1">
         <v>46098</v>
       </c>
       <c r="I17" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="J17" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="N17" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="O17" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="P17">
         <v>1770880.5</v>
       </c>
       <c r="Q17" t="s">
+        <v>156</v>
+      </c>
+      <c r="R17" t="s">
         <v>157</v>
       </c>
-      <c r="R17" t="s">
-        <v>158</v>
-      </c>
       <c r="S17" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T17" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="U17" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="V17" s="1">
         <v>46107</v>
@@ -1738,43 +1735,43 @@
         <v>25</v>
       </c>
       <c r="E18" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F18" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G18" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H18" s="1">
         <v>46076</v>
       </c>
       <c r="I18" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="N18" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="O18" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="P18">
         <v>350000</v>
       </c>
       <c r="Q18" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="R18" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="S18" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T18" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="U18" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V18" s="1">
         <v>46079</v>
@@ -1794,43 +1791,43 @@
         <v>25</v>
       </c>
       <c r="E19" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F19" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G19" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H19" s="1">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="N19" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="O19" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="P19">
         <v>350000</v>
       </c>
       <c r="Q19" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="R19" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="S19" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T19" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="U19" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V19" s="1">
         <v>46079</v>
@@ -1850,34 +1847,34 @@
         <v>24</v>
       </c>
       <c r="E20" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F20" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N20" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="O20" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="P20">
         <v>1000000</v>
       </c>
       <c r="Q20" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="R20" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="S20" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T20" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="U20" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V20" s="1">
         <v>46291</v>
@@ -1897,34 +1894,34 @@
         <v>24</v>
       </c>
       <c r="E21" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F21" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N21" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="O21" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="P21">
         <v>400000</v>
       </c>
       <c r="Q21" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="R21" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="S21" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T21" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="U21" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V21" s="1">
         <v>46321</v>
@@ -1944,34 +1941,34 @@
         <v>24</v>
       </c>
       <c r="E22" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F22" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N22" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="O22" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="P22">
         <v>120000</v>
       </c>
       <c r="Q22" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="R22" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="S22" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T22" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="U22" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V22" s="1">
         <v>46321</v>
@@ -1991,34 +1988,34 @@
         <v>24</v>
       </c>
       <c r="E23" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F23" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N23" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="O23" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="P23">
         <v>80000</v>
       </c>
       <c r="Q23" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="R23" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="S23" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T23" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="U23" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V23" s="1">
         <v>46321</v>
@@ -2038,46 +2035,46 @@
         <v>25</v>
       </c>
       <c r="E24" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F24" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G24" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H24" s="1">
         <v>46119</v>
       </c>
       <c r="I24" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="J24" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="N24" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="O24" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="P24">
         <v>1704503</v>
       </c>
       <c r="Q24" t="s">
+        <v>156</v>
+      </c>
+      <c r="R24" t="s">
         <v>157</v>
       </c>
-      <c r="R24" t="s">
-        <v>158</v>
-      </c>
       <c r="S24" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T24" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="U24" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="V24" s="1">
         <v>46138</v>
@@ -2097,43 +2094,43 @@
         <v>25</v>
       </c>
       <c r="E25" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F25" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G25" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H25" s="1">
         <v>46121</v>
       </c>
       <c r="I25" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="N25" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O25" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="P25">
         <v>3799000</v>
       </c>
       <c r="Q25" t="s">
+        <v>156</v>
+      </c>
+      <c r="R25" t="s">
         <v>157</v>
       </c>
-      <c r="R25" t="s">
-        <v>158</v>
-      </c>
       <c r="S25" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T25" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="U25" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V25" s="1">
         <v>46168</v>
@@ -2153,43 +2150,43 @@
         <v>25</v>
       </c>
       <c r="E26" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F26" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G26" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H26" s="1">
         <v>46076</v>
       </c>
       <c r="I26" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="N26" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O26" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="P26">
         <v>1000</v>
       </c>
       <c r="Q26" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="R26" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="S26" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T26" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="U26" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V26" s="1">
         <v>46079</v>
@@ -2209,34 +2206,34 @@
         <v>24</v>
       </c>
       <c r="E27" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F27" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N27" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O27" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="P27">
         <v>100000</v>
       </c>
       <c r="Q27" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="R27" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="S27" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T27" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="U27" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="V27" s="1">
         <v>46291</v>
@@ -2256,46 +2253,46 @@
         <v>25</v>
       </c>
       <c r="E28" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F28" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G28" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H28" s="1">
         <v>46199</v>
       </c>
       <c r="I28" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="J28" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="N28" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="O28" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="P28">
         <v>150000</v>
       </c>
       <c r="Q28" t="s">
+        <v>156</v>
+      </c>
+      <c r="R28" t="s">
         <v>157</v>
       </c>
-      <c r="R28" t="s">
-        <v>158</v>
-      </c>
       <c r="S28" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T28" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="U28" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="V28" s="1">
         <v>46199</v>
@@ -2315,46 +2312,46 @@
         <v>25</v>
       </c>
       <c r="E29" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F29" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G29" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H29" s="1">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="J29" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="N29" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="O29" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="P29">
         <v>150000</v>
       </c>
       <c r="Q29" t="s">
+        <v>156</v>
+      </c>
+      <c r="R29" t="s">
         <v>157</v>
       </c>
-      <c r="R29" t="s">
-        <v>158</v>
-      </c>
       <c r="S29" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T29" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="U29" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="V29" s="1">
         <v>46199</v>
@@ -2374,46 +2371,46 @@
         <v>25</v>
       </c>
       <c r="E30" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F30" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G30" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H30" s="1">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="J30" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="N30" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="O30" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="P30">
         <v>18462.36</v>
       </c>
       <c r="Q30" t="s">
+        <v>156</v>
+      </c>
+      <c r="R30" t="s">
         <v>157</v>
       </c>
-      <c r="R30" t="s">
-        <v>158</v>
-      </c>
       <c r="S30" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T30" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="U30" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="V30" s="1">
         <v>46199</v>
@@ -2433,46 +2430,46 @@
         <v>25</v>
       </c>
       <c r="E31" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F31" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G31" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H31" s="1">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="J31" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="N31" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="O31" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="P31">
         <v>324166.14</v>
       </c>
       <c r="Q31" t="s">
+        <v>156</v>
+      </c>
+      <c r="R31" t="s">
         <v>157</v>
       </c>
-      <c r="R31" t="s">
-        <v>158</v>
-      </c>
       <c r="S31" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T31" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="U31" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="V31" s="1">
         <v>46199</v>
@@ -2492,34 +2489,34 @@
         <v>24</v>
       </c>
       <c r="E32" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F32" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N32" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="O32" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="P32">
         <v>30000</v>
       </c>
       <c r="Q32" t="s">
+        <v>156</v>
+      </c>
+      <c r="R32" t="s">
         <v>157</v>
       </c>
-      <c r="R32" t="s">
-        <v>158</v>
-      </c>
       <c r="S32" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T32" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="U32" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="V32" s="1">
         <v>46291</v>
@@ -2539,46 +2536,46 @@
         <v>25</v>
       </c>
       <c r="E33" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F33" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G33" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H33" s="1">
         <v>46191</v>
       </c>
       <c r="I33" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="J33" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="N33" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="O33" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="P33">
         <v>1496713.48</v>
       </c>
       <c r="Q33" t="s">
+        <v>156</v>
+      </c>
+      <c r="R33" t="s">
         <v>157</v>
       </c>
-      <c r="R33" t="s">
-        <v>158</v>
-      </c>
       <c r="S33" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T33" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="U33" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="V33" s="1">
         <v>46199</v>
@@ -2598,43 +2595,43 @@
         <v>25</v>
       </c>
       <c r="E34" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F34" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G34" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H34" s="1">
         <v>46119</v>
       </c>
       <c r="I34" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="N34" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="O34" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="P34">
         <v>207789.52</v>
       </c>
       <c r="Q34" t="s">
+        <v>156</v>
+      </c>
+      <c r="R34" t="s">
         <v>157</v>
       </c>
-      <c r="R34" t="s">
-        <v>158</v>
-      </c>
       <c r="S34" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T34" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="U34" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="V34" s="1">
         <v>46199</v>
@@ -2654,43 +2651,43 @@
         <v>25</v>
       </c>
       <c r="E35" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F35" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G35" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H35" s="1">
         <v>46213</v>
       </c>
       <c r="I35" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="N35" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O35" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="P35">
         <v>962290.8</v>
       </c>
       <c r="Q35" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="R35" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="S35" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T35" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="U35" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V35" s="1">
         <v>46260</v>
@@ -2710,43 +2707,43 @@
         <v>25</v>
       </c>
       <c r="E36" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F36" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G36" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H36" s="1">
         <v>46175</v>
       </c>
       <c r="I36" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="N36" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O36" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="P36">
         <v>800000</v>
       </c>
       <c r="Q36" t="s">
+        <v>156</v>
+      </c>
+      <c r="R36" t="s">
         <v>157</v>
       </c>
-      <c r="R36" t="s">
-        <v>158</v>
-      </c>
       <c r="S36" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T36" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="U36" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V36" s="1">
         <v>46229</v>
@@ -2766,43 +2763,43 @@
         <v>25</v>
       </c>
       <c r="E37" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F37" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G37" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H37" s="1">
         <v>46213</v>
       </c>
       <c r="I37" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="N37" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O37" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="P37">
         <v>1530656.62</v>
       </c>
       <c r="Q37" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="R37" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="S37" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T37" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="U37" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V37" s="1">
         <v>46260</v>
@@ -2822,43 +2819,43 @@
         <v>25</v>
       </c>
       <c r="E38" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F38" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G38" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H38" s="1">
         <v>46199</v>
       </c>
       <c r="I38" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="N38" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O38" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="P38">
         <v>72958.08</v>
       </c>
       <c r="Q38" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="R38" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="S38" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T38" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="U38" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V38" s="1">
         <v>46199</v>
@@ -2878,43 +2875,43 @@
         <v>25</v>
       </c>
       <c r="E39" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F39" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G39" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H39" s="1">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="N39" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O39" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="P39">
         <v>8916</v>
       </c>
       <c r="Q39" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="R39" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="S39" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T39" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="U39" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V39" s="1">
         <v>46199</v>
@@ -2934,43 +2931,43 @@
         <v>25</v>
       </c>
       <c r="E40" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F40" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G40" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H40" s="1">
         <v>46204</v>
       </c>
       <c r="I40" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="N40" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O40" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="P40">
         <v>425178.5</v>
       </c>
       <c r="Q40" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="R40" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="S40" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T40" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="U40" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V40" s="1">
         <v>46199</v>
@@ -2990,31 +2987,31 @@
         <v>26</v>
       </c>
       <c r="E41" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G41" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="N41" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O41" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="Q41" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="R41" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="S41" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="T41" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="U41" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V41" s="1">
         <v>46260</v>
@@ -3034,43 +3031,43 @@
         <v>25</v>
       </c>
       <c r="E42" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F42" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G42" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H42" s="1">
         <v>46191</v>
       </c>
       <c r="I42" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="N42" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="O42" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="P42">
         <v>400000</v>
       </c>
       <c r="Q42" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="R42" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="S42" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T42" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="U42" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V42" s="1">
         <v>46199</v>
@@ -3090,43 +3087,43 @@
         <v>25</v>
       </c>
       <c r="E43" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F43" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G43" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H43" s="1">
         <v>46191</v>
       </c>
       <c r="I43" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="N43" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="O43" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="P43">
         <v>400000</v>
       </c>
       <c r="Q43" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="R43" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="S43" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T43" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="U43" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V43" s="1">
         <v>46199</v>
@@ -3146,46 +3143,46 @@
         <v>25</v>
       </c>
       <c r="E44" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F44" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G44" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H44" s="1">
         <v>46213</v>
       </c>
       <c r="I44" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="J44" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="N44" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="O44" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="P44">
         <v>173846.38</v>
       </c>
       <c r="Q44" t="s">
+        <v>156</v>
+      </c>
+      <c r="R44" t="s">
         <v>157</v>
       </c>
-      <c r="R44" t="s">
-        <v>158</v>
-      </c>
       <c r="S44" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T44" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="U44" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="V44" s="1">
         <v>46229</v>
@@ -3205,43 +3202,43 @@
         <v>25</v>
       </c>
       <c r="E45" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F45" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G45" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H45" s="1">
         <v>46210</v>
       </c>
       <c r="I45" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="N45" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="O45" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="P45">
         <v>1530656.62</v>
       </c>
       <c r="Q45" t="s">
+        <v>156</v>
+      </c>
+      <c r="R45" t="s">
         <v>157</v>
       </c>
-      <c r="R45" t="s">
-        <v>158</v>
-      </c>
       <c r="S45" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T45" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="U45" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="V45" s="1">
         <v>46229</v>
@@ -3261,34 +3258,34 @@
         <v>24</v>
       </c>
       <c r="E46" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F46" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N46" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="O46" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="P46">
         <v>1000000</v>
       </c>
       <c r="Q46" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="R46" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="S46" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T46" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="U46" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V46" s="1">
         <v>46260</v>
@@ -3308,34 +3305,34 @@
         <v>24</v>
       </c>
       <c r="E47" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F47" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N47" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="O47" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="P47">
         <v>958040</v>
       </c>
       <c r="Q47" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="R47" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="S47" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T47" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="U47" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="V47" s="1">
         <v>46291</v>
@@ -3355,46 +3352,46 @@
         <v>25</v>
       </c>
       <c r="E48" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F48" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G48" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H48" s="1">
         <v>46176</v>
       </c>
       <c r="I48" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="J48" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="N48" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="O48" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="P48">
         <v>41730.64</v>
       </c>
       <c r="Q48" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="R48" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="S48" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T48" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="U48" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="V48" s="1">
         <v>46291</v>
@@ -3414,40 +3411,40 @@
         <v>24</v>
       </c>
       <c r="E49" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F49" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="J49" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="K49" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="N49" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="O49" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="P49">
         <v>1468159.32</v>
       </c>
       <c r="Q49" t="s">
+        <v>156</v>
+      </c>
+      <c r="R49" t="s">
         <v>157</v>
       </c>
-      <c r="R49" t="s">
-        <v>158</v>
-      </c>
       <c r="S49" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T49" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="U49" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="V49" s="1">
         <v>46260</v>
@@ -3467,40 +3464,40 @@
         <v>24</v>
       </c>
       <c r="E50" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F50" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="J50" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="K50" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="N50" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="O50" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="P50">
         <v>1704503</v>
       </c>
       <c r="Q50" t="s">
+        <v>156</v>
+      </c>
+      <c r="R50" t="s">
         <v>157</v>
       </c>
-      <c r="R50" t="s">
-        <v>158</v>
-      </c>
       <c r="S50" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T50" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="U50" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="V50" s="1">
         <v>46291</v>
@@ -3520,34 +3517,34 @@
         <v>24</v>
       </c>
       <c r="E51" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F51" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N51" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="O51" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="P51">
         <v>1704503</v>
       </c>
       <c r="Q51" t="s">
+        <v>156</v>
+      </c>
+      <c r="R51" t="s">
         <v>157</v>
       </c>
-      <c r="R51" t="s">
-        <v>158</v>
-      </c>
       <c r="S51" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T51" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="U51" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="V51" s="1">
         <v>46321</v>
@@ -3564,43 +3561,46 @@
         <v>22</v>
       </c>
       <c r="D52" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E52" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F52" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G52" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="H52" s="1">
         <v>46227</v>
       </c>
+      <c r="I52" t="s">
+        <v>60</v>
+      </c>
       <c r="N52" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="O52" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="P52">
         <v>236343.68</v>
       </c>
       <c r="Q52" t="s">
+        <v>156</v>
+      </c>
+      <c r="R52" t="s">
         <v>157</v>
       </c>
-      <c r="R52" t="s">
-        <v>158</v>
-      </c>
       <c r="S52" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T52" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="U52" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="V52" s="1">
         <v>46260</v>
@@ -3620,34 +3620,34 @@
         <v>24</v>
       </c>
       <c r="E53" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F53" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N53" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="O53" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="P53">
         <v>1295422.28</v>
       </c>
       <c r="Q53" t="s">
+        <v>156</v>
+      </c>
+      <c r="R53" t="s">
         <v>157</v>
       </c>
-      <c r="R53" t="s">
-        <v>158</v>
-      </c>
       <c r="S53" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T53" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="U53" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="V53" s="1">
         <v>46352</v>
@@ -3667,34 +3667,34 @@
         <v>24</v>
       </c>
       <c r="E54" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F54" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="N54" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="O54" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="P54">
         <v>500000</v>
       </c>
       <c r="Q54" t="s">
+        <v>156</v>
+      </c>
+      <c r="R54" t="s">
         <v>157</v>
       </c>
-      <c r="R54" t="s">
-        <v>158</v>
-      </c>
       <c r="S54" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="T54" t="s">
+        <v>168</v>
+      </c>
+      <c r="U54" t="s">
         <v>169</v>
-      </c>
-      <c r="U54" t="s">
-        <v>170</v>
       </c>
       <c r="V54" s="1">
         <v>46321</v>
@@ -3714,37 +3714,37 @@
         <v>26</v>
       </c>
       <c r="E55" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F55" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G55" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="N55" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="O55" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="P55">
         <v>5000000</v>
       </c>
       <c r="Q55" t="s">
+        <v>156</v>
+      </c>
+      <c r="R55" t="s">
         <v>157</v>
       </c>
-      <c r="R55" t="s">
-        <v>158</v>
-      </c>
       <c r="S55" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="T55" t="s">
+        <v>168</v>
+      </c>
+      <c r="U55" t="s">
         <v>169</v>
-      </c>
-      <c r="U55" t="s">
-        <v>170</v>
       </c>
       <c r="V55" s="1">
         <v>46321</v>
@@ -3764,34 +3764,34 @@
         <v>24</v>
       </c>
       <c r="E56" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F56" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="N56" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="O56" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="P56">
         <v>4000000</v>
       </c>
       <c r="Q56" t="s">
+        <v>156</v>
+      </c>
+      <c r="R56" t="s">
         <v>157</v>
       </c>
-      <c r="R56" t="s">
-        <v>158</v>
-      </c>
       <c r="S56" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="T56" t="s">
+        <v>168</v>
+      </c>
+      <c r="U56" t="s">
         <v>169</v>
-      </c>
-      <c r="U56" t="s">
-        <v>170</v>
       </c>
       <c r="V56" s="1">
         <v>46049</v>
@@ -3811,34 +3811,34 @@
         <v>26</v>
       </c>
       <c r="E57" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F57" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="N57" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="O57" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="P57">
         <v>5500000</v>
       </c>
       <c r="Q57" t="s">
+        <v>156</v>
+      </c>
+      <c r="R57" t="s">
         <v>157</v>
       </c>
-      <c r="R57" t="s">
-        <v>158</v>
-      </c>
       <c r="S57" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="T57" t="s">
+        <v>168</v>
+      </c>
+      <c r="U57" t="s">
         <v>169</v>
-      </c>
-      <c r="U57" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="58" spans="1:22">
@@ -3855,34 +3855,34 @@
         <v>26</v>
       </c>
       <c r="E58" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F58" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="N58" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="O58" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="P58">
         <v>5500000</v>
       </c>
       <c r="Q58" t="s">
+        <v>156</v>
+      </c>
+      <c r="R58" t="s">
         <v>157</v>
       </c>
-      <c r="R58" t="s">
-        <v>158</v>
-      </c>
       <c r="S58" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="T58" t="s">
+        <v>168</v>
+      </c>
+      <c r="U58" t="s">
         <v>169</v>
-      </c>
-      <c r="U58" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="59" spans="1:22">
@@ -3899,31 +3899,31 @@
         <v>26</v>
       </c>
       <c r="E59" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N59" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O59" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="P59">
         <v>9389.959999999999</v>
       </c>
       <c r="Q59" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="R59" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="S59" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="T59" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="U59" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="V59" s="1">
         <v>46107</v>
@@ -3943,31 +3943,31 @@
         <v>26</v>
       </c>
       <c r="E60" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N60" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O60" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="P60">
         <v>7204.82</v>
       </c>
       <c r="Q60" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="R60" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="S60" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="T60" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="U60" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="V60" s="1">
         <v>46107</v>
@@ -3987,31 +3987,31 @@
         <v>26</v>
       </c>
       <c r="E61" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N61" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="O61" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="P61">
         <v>4227.84</v>
       </c>
       <c r="Q61" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="R61" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="S61" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="T61" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="U61" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="V61" s="1">
         <v>46107</v>
@@ -4031,31 +4031,31 @@
         <v>26</v>
       </c>
       <c r="E62" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N62" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O62" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="P62">
         <v>4064.54</v>
       </c>
       <c r="Q62" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="R62" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="S62" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="T62" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="U62" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="V62" s="1">
         <v>46107</v>
@@ -4075,31 +4075,31 @@
         <v>26</v>
       </c>
       <c r="E63" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N63" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="O63" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="P63">
         <v>3662.66</v>
       </c>
       <c r="Q63" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="R63" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="S63" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="T63" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="U63" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="V63" s="1">
         <v>46107</v>
@@ -4119,31 +4119,31 @@
         <v>26</v>
       </c>
       <c r="E64" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N64" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="O64" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="P64">
         <v>1163.64</v>
       </c>
       <c r="Q64" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="R64" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="S64" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="T64" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="U64" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="V64" s="1">
         <v>46107</v>
@@ -4163,31 +4163,31 @@
         <v>26</v>
       </c>
       <c r="E65" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N65" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="O65" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="P65">
         <v>120000</v>
       </c>
       <c r="Q65" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="R65" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="S65" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="T65" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="U65" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V65" s="1">
         <v>46168</v>
@@ -4207,34 +4207,34 @@
         <v>24</v>
       </c>
       <c r="E66" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F66" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N66" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="O66" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="P66">
         <v>400000</v>
       </c>
       <c r="Q66" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="R66" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="S66" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T66" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="U66" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V66" s="1">
         <v>46291</v>
@@ -4254,34 +4254,34 @@
         <v>24</v>
       </c>
       <c r="E67" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F67" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N67" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O67" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="P67">
         <v>100000</v>
       </c>
       <c r="Q67" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="R67" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="S67" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T67" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="U67" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="V67" s="1">
         <v>46229</v>
@@ -4301,31 +4301,31 @@
         <v>26</v>
       </c>
       <c r="E68" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N68" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="O68" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P68">
         <v>80000</v>
       </c>
       <c r="Q68" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="R68" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="S68" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="T68" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="U68" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V68" s="1">
         <v>46260</v>
@@ -4345,31 +4345,31 @@
         <v>26</v>
       </c>
       <c r="E69" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N69" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="O69" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="P69">
         <v>835000</v>
       </c>
       <c r="Q69" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="R69" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="S69" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="T69" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="U69" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="V69" s="1">
         <v>46291</v>
@@ -4389,31 +4389,31 @@
         <v>26</v>
       </c>
       <c r="E70" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N70" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="O70" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="P70">
         <v>165000</v>
       </c>
       <c r="Q70" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="R70" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="S70" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="T70" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="U70" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="V70" s="1">
         <v>46168</v>
@@ -4433,31 +4433,31 @@
         <v>26</v>
       </c>
       <c r="E71" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N71" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="O71" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="P71">
         <v>1000000</v>
       </c>
       <c r="Q71" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="R71" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="S71" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="T71" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="U71" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="V71" s="1">
         <v>46291</v>
@@ -4477,31 +4477,31 @@
         <v>26</v>
       </c>
       <c r="E72" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N72" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="O72" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="P72">
         <v>1000000</v>
       </c>
       <c r="Q72" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="R72" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="S72" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="T72" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="U72" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="V72" s="1">
         <v>46291</v>
@@ -4521,31 +4521,31 @@
         <v>26</v>
       </c>
       <c r="E73" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N73" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O73" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="P73">
         <v>100000</v>
       </c>
       <c r="Q73" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="R73" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="S73" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="T73" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="U73" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="V73" s="1">
         <v>46291</v>
@@ -4565,34 +4565,34 @@
         <v>24</v>
       </c>
       <c r="E74" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F74" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N74" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="O74" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="P74">
         <v>1000000</v>
       </c>
       <c r="Q74" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="R74" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="S74" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T74" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="U74" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V74" s="1">
         <v>46321</v>
@@ -4609,40 +4609,40 @@
         <v>22</v>
       </c>
       <c r="D75" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E75" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F75" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G75" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="N75" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="O75" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="P75">
         <v>1704503</v>
       </c>
       <c r="Q75" t="s">
+        <v>156</v>
+      </c>
+      <c r="R75" t="s">
         <v>157</v>
       </c>
-      <c r="R75" t="s">
-        <v>158</v>
-      </c>
       <c r="S75" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="T75" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="U75" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="V75" s="1">
         <v>46381</v>
@@ -4659,40 +4659,40 @@
         <v>22</v>
       </c>
       <c r="D76" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E76" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F76" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G76" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="N76" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="O76" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="P76">
         <v>1638125.5</v>
       </c>
       <c r="Q76" t="s">
+        <v>156</v>
+      </c>
+      <c r="R76" t="s">
         <v>157</v>
       </c>
-      <c r="R76" t="s">
-        <v>158</v>
-      </c>
       <c r="S76" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="T76" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="U76" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="V76" s="1">
         <v>46381</v>
@@ -4709,40 +4709,40 @@
         <v>22</v>
       </c>
       <c r="D77" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E77" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F77" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G77" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="N77" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="O77" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="P77">
         <v>3800000</v>
       </c>
       <c r="Q77" t="s">
+        <v>156</v>
+      </c>
+      <c r="R77" t="s">
         <v>157</v>
       </c>
-      <c r="R77" t="s">
-        <v>158</v>
-      </c>
       <c r="S77" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="T77" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="U77" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V77" s="1">
         <v>46381</v>
@@ -4759,40 +4759,40 @@
         <v>22</v>
       </c>
       <c r="D78" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E78" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F78" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G78" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="N78" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="O78" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="P78">
         <v>3800000</v>
       </c>
       <c r="Q78" t="s">
+        <v>156</v>
+      </c>
+      <c r="R78" t="s">
         <v>157</v>
       </c>
-      <c r="R78" t="s">
-        <v>158</v>
-      </c>
       <c r="S78" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="T78" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="U78" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V78" s="1">
         <v>46381</v>
@@ -4812,31 +4812,31 @@
         <v>26</v>
       </c>
       <c r="E79" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N79" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O79" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="P79">
         <v>3800000</v>
       </c>
       <c r="Q79" t="s">
+        <v>156</v>
+      </c>
+      <c r="R79" t="s">
         <v>157</v>
       </c>
-      <c r="R79" t="s">
-        <v>158</v>
-      </c>
       <c r="S79" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="T79" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="U79" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V79" s="1">
         <v>46382</v>
@@ -4856,31 +4856,31 @@
         <v>24</v>
       </c>
       <c r="E80" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N80" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O80" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="P80">
         <v>4394700</v>
       </c>
       <c r="Q80" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="R80" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="S80" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="T80" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="U80" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V80" s="1">
         <v>46382</v>
@@ -4900,34 +4900,34 @@
         <v>24</v>
       </c>
       <c r="E81" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F81" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N81" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="O81" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="P81">
         <v>528395.9300000001</v>
       </c>
       <c r="Q81" t="s">
+        <v>156</v>
+      </c>
+      <c r="R81" t="s">
         <v>157</v>
       </c>
-      <c r="R81" t="s">
-        <v>158</v>
-      </c>
       <c r="S81" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T81" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="U81" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="V81" s="1">
         <v>46382</v>
@@ -4947,31 +4947,31 @@
         <v>26</v>
       </c>
       <c r="E82" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N82" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="O82" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="P82">
         <v>1000000</v>
       </c>
       <c r="Q82" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="R82" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="S82" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="T82" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="U82" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V82" s="1">
         <v>46321</v>
@@ -4991,31 +4991,31 @@
         <v>24</v>
       </c>
       <c r="E83" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N83" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O83" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="P83">
         <v>4394700</v>
       </c>
       <c r="Q83" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="R83" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="S83" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="T83" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="U83" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V83" s="1">
         <v>46382</v>

</xml_diff>

<commit_message>
Atualização automática: mta (04/08/2026 14:16)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1062" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1065" uniqueCount="170">
   <si>
     <t>linha</t>
   </si>
@@ -1224,7 +1224,7 @@
         <v>28</v>
       </c>
       <c r="V7" s="1">
-        <v>46107</v>
+        <v>46138</v>
       </c>
     </row>
     <row r="8" spans="1:22">
@@ -1471,7 +1471,7 @@
         <v>169</v>
       </c>
       <c r="V12" s="1">
-        <v>46107</v>
+        <v>46079</v>
       </c>
     </row>
     <row r="13" spans="1:22">
@@ -2133,7 +2133,7 @@
         <v>28</v>
       </c>
       <c r="V25" s="1">
-        <v>46168</v>
+        <v>46138</v>
       </c>
     </row>
     <row r="26" spans="1:22">
@@ -2634,7 +2634,7 @@
         <v>169</v>
       </c>
       <c r="V34" s="1">
-        <v>46199</v>
+        <v>46138</v>
       </c>
     </row>
     <row r="35" spans="1:22">
@@ -2690,7 +2690,7 @@
         <v>28</v>
       </c>
       <c r="V35" s="1">
-        <v>46260</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="36" spans="1:22">
@@ -2746,7 +2746,7 @@
         <v>28</v>
       </c>
       <c r="V36" s="1">
-        <v>46229</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="37" spans="1:22">
@@ -2802,7 +2802,7 @@
         <v>28</v>
       </c>
       <c r="V37" s="1">
-        <v>46260</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="38" spans="1:22">
@@ -2970,7 +2970,7 @@
         <v>28</v>
       </c>
       <c r="V40" s="1">
-        <v>46199</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="41" spans="1:22">
@@ -3394,7 +3394,7 @@
         <v>169</v>
       </c>
       <c r="V48" s="1">
-        <v>46291</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="49" spans="1:22">
@@ -3603,7 +3603,7 @@
         <v>169</v>
       </c>
       <c r="V52" s="1">
-        <v>46260</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="53" spans="1:22">
@@ -3761,7 +3761,7 @@
         <v>22</v>
       </c>
       <c r="D56" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E56" t="s">
         <v>28</v>
@@ -3769,14 +3769,14 @@
       <c r="F56" t="s">
         <v>39</v>
       </c>
+      <c r="G56" t="s">
+        <v>42</v>
+      </c>
       <c r="N56" t="s">
         <v>79</v>
       </c>
       <c r="O56" t="s">
         <v>129</v>
-      </c>
-      <c r="P56">
-        <v>4000000</v>
       </c>
       <c r="Q56" t="s">
         <v>156</v>
@@ -3816,14 +3816,14 @@
       <c r="F57" t="s">
         <v>39</v>
       </c>
+      <c r="G57" t="s">
+        <v>42</v>
+      </c>
       <c r="N57" t="s">
         <v>79</v>
       </c>
       <c r="O57" t="s">
         <v>130</v>
-      </c>
-      <c r="P57">
-        <v>5500000</v>
       </c>
       <c r="Q57" t="s">
         <v>156</v>
@@ -3860,14 +3860,14 @@
       <c r="F58" t="s">
         <v>39</v>
       </c>
+      <c r="G58" t="s">
+        <v>42</v>
+      </c>
       <c r="N58" t="s">
         <v>79</v>
       </c>
       <c r="O58" t="s">
         <v>131</v>
-      </c>
-      <c r="P58">
-        <v>5500000</v>
       </c>
       <c r="Q58" t="s">
         <v>156</v>

</xml_diff>

<commit_message>
Atualização automática: mta (06/08/2026 12:23)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1065" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1067" uniqueCount="171">
   <si>
     <t>linha</t>
   </si>
@@ -221,6 +221,9 @@
   </si>
   <si>
     <t>Atender SET</t>
+  </si>
+  <si>
+    <t>Atender OUT</t>
   </si>
   <si>
     <t>LIVRE</t>
@@ -950,31 +953,31 @@
         <v>30</v>
       </c>
       <c r="L2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="N2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="O2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="P2">
         <v>135000</v>
       </c>
       <c r="Q2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="R2" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="S2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T2" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="U2" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="V2" s="1">
         <v>46229</v>
@@ -1000,25 +1003,25 @@
         <v>30</v>
       </c>
       <c r="N3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="O3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="P3">
         <v>400000</v>
       </c>
       <c r="Q3" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="R3" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="S3" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T3" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="U3" t="s">
         <v>28</v>
@@ -1047,25 +1050,25 @@
         <v>30</v>
       </c>
       <c r="N4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="O4" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="P4">
         <v>430000</v>
       </c>
       <c r="Q4" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="R4" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="S4" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T4" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="U4" t="s">
         <v>28</v>
@@ -1094,25 +1097,25 @@
         <v>30</v>
       </c>
       <c r="N5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="O5" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="P5">
         <v>425000</v>
       </c>
       <c r="Q5" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="R5" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="S5" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T5" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="U5" t="s">
         <v>28</v>
@@ -1141,28 +1144,28 @@
         <v>30</v>
       </c>
       <c r="L6" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="N6" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="O6" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="P6">
         <v>563000</v>
       </c>
       <c r="Q6" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="R6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="S6" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="U6" t="s">
         <v>28</v>
@@ -1200,25 +1203,25 @@
         <v>45</v>
       </c>
       <c r="N7" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="O7" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="P7">
         <v>3799999.6</v>
       </c>
       <c r="Q7" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="R7" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="S7" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T7" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="U7" t="s">
         <v>28</v>
@@ -1247,25 +1250,25 @@
         <v>30</v>
       </c>
       <c r="N8" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="O8" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="P8">
         <v>430000</v>
       </c>
       <c r="Q8" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="R8" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="S8" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T8" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="U8" t="s">
         <v>28</v>
@@ -1294,25 +1297,25 @@
         <v>30</v>
       </c>
       <c r="N9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="O9" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="P9">
         <v>60000</v>
       </c>
       <c r="Q9" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="R9" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="S9" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T9" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="U9" t="s">
         <v>28</v>
@@ -1341,25 +1344,25 @@
         <v>30</v>
       </c>
       <c r="N10" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="O10" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="P10">
         <v>200000</v>
       </c>
       <c r="Q10" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="R10" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="S10" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T10" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="U10" t="s">
         <v>28</v>
@@ -1388,25 +1391,25 @@
         <v>30</v>
       </c>
       <c r="N11" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="O11" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="P11">
         <v>320000</v>
       </c>
       <c r="Q11" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="R11" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="S11" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T11" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="U11" t="s">
         <v>28</v>
@@ -1447,28 +1450,28 @@
         <v>61</v>
       </c>
       <c r="N12" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="O12" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="P12">
         <v>1187433.02</v>
       </c>
       <c r="Q12" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="R12" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="S12" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T12" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="U12" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="V12" s="1">
         <v>46079</v>
@@ -1494,28 +1497,28 @@
         <v>30</v>
       </c>
       <c r="N13" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="O13" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="P13">
         <v>1000000</v>
       </c>
       <c r="Q13" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="R13" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="S13" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T13" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="U13" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="V13" s="1">
         <v>46352</v>
@@ -1541,28 +1544,28 @@
         <v>30</v>
       </c>
       <c r="N14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="O14" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="P14">
         <v>1000000</v>
       </c>
       <c r="Q14" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="R14" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="S14" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T14" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="U14" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="V14" s="1">
         <v>46352</v>
@@ -1588,28 +1591,28 @@
         <v>30</v>
       </c>
       <c r="N15" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="O15" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="P15">
         <v>1000000</v>
       </c>
       <c r="Q15" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="R15" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="S15" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T15" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="U15" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="V15" s="1">
         <v>46352</v>
@@ -1635,28 +1638,28 @@
         <v>30</v>
       </c>
       <c r="N16" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="O16" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="P16">
         <v>100000</v>
       </c>
       <c r="Q16" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="R16" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="S16" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T16" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="U16" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="V16" s="1">
         <v>46229</v>
@@ -1694,28 +1697,28 @@
         <v>61</v>
       </c>
       <c r="N17" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="O17" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="P17">
         <v>1770880.5</v>
       </c>
       <c r="Q17" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="R17" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="S17" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T17" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="U17" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="V17" s="1">
         <v>46107</v>
@@ -1750,25 +1753,25 @@
         <v>48</v>
       </c>
       <c r="N18" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O18" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="P18">
         <v>350000</v>
       </c>
       <c r="Q18" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="R18" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="S18" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T18" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="U18" t="s">
         <v>28</v>
@@ -1806,25 +1809,25 @@
         <v>48</v>
       </c>
       <c r="N19" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O19" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="P19">
         <v>350000</v>
       </c>
       <c r="Q19" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="R19" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="S19" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T19" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="U19" t="s">
         <v>28</v>
@@ -1853,25 +1856,25 @@
         <v>30</v>
       </c>
       <c r="N20" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="O20" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="P20">
         <v>1000000</v>
       </c>
       <c r="Q20" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="R20" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="S20" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T20" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="U20" t="s">
         <v>28</v>
@@ -1900,25 +1903,25 @@
         <v>30</v>
       </c>
       <c r="N21" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="O21" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="P21">
         <v>400000</v>
       </c>
       <c r="Q21" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="R21" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="S21" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T21" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="U21" t="s">
         <v>28</v>
@@ -1947,25 +1950,25 @@
         <v>30</v>
       </c>
       <c r="N22" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="O22" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="P22">
         <v>120000</v>
       </c>
       <c r="Q22" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="R22" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="S22" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T22" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="U22" t="s">
         <v>28</v>
@@ -1994,25 +1997,25 @@
         <v>30</v>
       </c>
       <c r="N23" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="O23" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="P23">
         <v>80000</v>
       </c>
       <c r="Q23" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="R23" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="S23" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T23" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="U23" t="s">
         <v>28</v>
@@ -2053,28 +2056,28 @@
         <v>62</v>
       </c>
       <c r="N24" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="O24" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="P24">
         <v>1704503</v>
       </c>
       <c r="Q24" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="R24" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="S24" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T24" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="U24" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="V24" s="1">
         <v>46138</v>
@@ -2109,25 +2112,25 @@
         <v>50</v>
       </c>
       <c r="N25" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="O25" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="P25">
         <v>3799000</v>
       </c>
       <c r="Q25" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="R25" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="S25" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T25" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="U25" t="s">
         <v>28</v>
@@ -2165,25 +2168,25 @@
         <v>51</v>
       </c>
       <c r="N26" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="O26" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="P26">
         <v>1000</v>
       </c>
       <c r="Q26" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="R26" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="S26" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T26" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="U26" t="s">
         <v>28</v>
@@ -2212,28 +2215,28 @@
         <v>30</v>
       </c>
       <c r="N27" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="O27" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="P27">
         <v>100000</v>
       </c>
       <c r="Q27" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="R27" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="S27" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T27" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="U27" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="V27" s="1">
         <v>46291</v>
@@ -2271,28 +2274,28 @@
         <v>63</v>
       </c>
       <c r="N28" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="O28" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="P28">
         <v>150000</v>
       </c>
       <c r="Q28" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="R28" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="S28" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T28" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="U28" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="V28" s="1">
         <v>46199</v>
@@ -2330,28 +2333,28 @@
         <v>63</v>
       </c>
       <c r="N29" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="O29" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="P29">
         <v>150000</v>
       </c>
       <c r="Q29" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="R29" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="S29" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T29" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="U29" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="V29" s="1">
         <v>46199</v>
@@ -2389,28 +2392,28 @@
         <v>63</v>
       </c>
       <c r="N30" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="O30" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="P30">
         <v>18462.36</v>
       </c>
       <c r="Q30" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="R30" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="S30" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T30" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="U30" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="V30" s="1">
         <v>46199</v>
@@ -2448,28 +2451,28 @@
         <v>63</v>
       </c>
       <c r="N31" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="O31" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="P31">
         <v>324166.14</v>
       </c>
       <c r="Q31" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="R31" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="S31" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T31" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="U31" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="V31" s="1">
         <v>46199</v>
@@ -2495,28 +2498,28 @@
         <v>30</v>
       </c>
       <c r="N32" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="O32" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="P32">
         <v>30000</v>
       </c>
       <c r="Q32" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="R32" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="S32" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T32" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="U32" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="V32" s="1">
         <v>46291</v>
@@ -2554,28 +2557,28 @@
         <v>64</v>
       </c>
       <c r="N33" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="O33" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="P33">
         <v>1496713.48</v>
       </c>
       <c r="Q33" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="R33" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="S33" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T33" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="U33" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="V33" s="1">
         <v>46199</v>
@@ -2610,28 +2613,28 @@
         <v>49</v>
       </c>
       <c r="N34" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="O34" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="P34">
         <v>207789.52</v>
       </c>
       <c r="Q34" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="R34" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="S34" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T34" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="U34" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="V34" s="1">
         <v>46138</v>
@@ -2666,25 +2669,25 @@
         <v>55</v>
       </c>
       <c r="N35" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="O35" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="P35">
         <v>962290.8</v>
       </c>
       <c r="Q35" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="R35" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="S35" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T35" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="U35" t="s">
         <v>28</v>
@@ -2722,25 +2725,25 @@
         <v>56</v>
       </c>
       <c r="N36" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="O36" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="P36">
         <v>800000</v>
       </c>
       <c r="Q36" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="R36" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="S36" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T36" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="U36" t="s">
         <v>28</v>
@@ -2778,25 +2781,25 @@
         <v>55</v>
       </c>
       <c r="N37" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="O37" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="P37">
         <v>1530656.62</v>
       </c>
       <c r="Q37" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="R37" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="S37" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T37" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="U37" t="s">
         <v>28</v>
@@ -2834,25 +2837,25 @@
         <v>57</v>
       </c>
       <c r="N38" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="O38" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="P38">
         <v>72958.08</v>
       </c>
       <c r="Q38" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="R38" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="S38" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T38" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="U38" t="s">
         <v>28</v>
@@ -2890,25 +2893,25 @@
         <v>57</v>
       </c>
       <c r="N39" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="O39" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="P39">
         <v>8916</v>
       </c>
       <c r="Q39" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="R39" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="S39" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T39" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="U39" t="s">
         <v>28</v>
@@ -2946,25 +2949,25 @@
         <v>57</v>
       </c>
       <c r="N40" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="O40" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="P40">
         <v>425178.5</v>
       </c>
       <c r="Q40" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="R40" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="S40" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T40" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="U40" t="s">
         <v>28</v>
@@ -2993,22 +2996,22 @@
         <v>42</v>
       </c>
       <c r="N41" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="O41" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="Q41" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="R41" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="S41" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="T41" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="U41" t="s">
         <v>28</v>
@@ -3046,25 +3049,25 @@
         <v>58</v>
       </c>
       <c r="N42" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O42" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="P42">
         <v>400000</v>
       </c>
       <c r="Q42" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="R42" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="S42" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T42" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="U42" t="s">
         <v>28</v>
@@ -3102,25 +3105,25 @@
         <v>58</v>
       </c>
       <c r="N43" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O43" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="P43">
         <v>400000</v>
       </c>
       <c r="Q43" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="R43" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="S43" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T43" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="U43" t="s">
         <v>28</v>
@@ -3161,28 +3164,28 @@
         <v>65</v>
       </c>
       <c r="N44" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="O44" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="P44">
         <v>173846.38</v>
       </c>
       <c r="Q44" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="R44" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="S44" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T44" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="U44" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="V44" s="1">
         <v>46229</v>
@@ -3217,28 +3220,28 @@
         <v>53</v>
       </c>
       <c r="N45" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="O45" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="P45">
         <v>1530656.62</v>
       </c>
       <c r="Q45" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="R45" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="S45" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T45" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="U45" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="V45" s="1">
         <v>46229</v>
@@ -3264,25 +3267,25 @@
         <v>30</v>
       </c>
       <c r="N46" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="O46" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="P46">
         <v>1000000</v>
       </c>
       <c r="Q46" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="R46" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="S46" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T46" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="U46" t="s">
         <v>28</v>
@@ -3311,28 +3314,28 @@
         <v>30</v>
       </c>
       <c r="N47" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="O47" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="P47">
         <v>958040</v>
       </c>
       <c r="Q47" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="R47" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="S47" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T47" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="U47" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="V47" s="1">
         <v>46291</v>
@@ -3370,28 +3373,28 @@
         <v>66</v>
       </c>
       <c r="N48" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="O48" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="P48">
         <v>41730.64</v>
       </c>
       <c r="Q48" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="R48" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="S48" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T48" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="U48" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="V48" s="1">
         <v>46199</v>
@@ -3423,28 +3426,28 @@
         <v>67</v>
       </c>
       <c r="N49" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="O49" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="P49">
         <v>1468159.32</v>
       </c>
       <c r="Q49" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="R49" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="S49" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T49" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="U49" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="V49" s="1">
         <v>46260</v>
@@ -3476,28 +3479,28 @@
         <v>68</v>
       </c>
       <c r="N50" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="O50" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="P50">
         <v>1704503</v>
       </c>
       <c r="Q50" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="R50" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="S50" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T50" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="U50" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="V50" s="1">
         <v>46291</v>
@@ -3522,29 +3525,32 @@
       <c r="F51" t="s">
         <v>30</v>
       </c>
+      <c r="K51" t="s">
+        <v>69</v>
+      </c>
       <c r="N51" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="O51" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="P51">
         <v>1704503</v>
       </c>
       <c r="Q51" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="R51" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="S51" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T51" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="U51" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="V51" s="1">
         <v>46321</v>
@@ -3579,28 +3585,28 @@
         <v>60</v>
       </c>
       <c r="N52" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="O52" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="P52">
         <v>236343.68</v>
       </c>
       <c r="Q52" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="R52" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="S52" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T52" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="U52" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="V52" s="1">
         <v>46229</v>
@@ -3626,28 +3632,28 @@
         <v>30</v>
       </c>
       <c r="N53" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="O53" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="P53">
         <v>1295422.28</v>
       </c>
       <c r="Q53" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="R53" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="S53" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T53" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="U53" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="V53" s="1">
         <v>46352</v>
@@ -3672,29 +3678,32 @@
       <c r="F54" t="s">
         <v>39</v>
       </c>
+      <c r="K54" t="s">
+        <v>69</v>
+      </c>
       <c r="N54" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O54" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="P54">
         <v>500000</v>
       </c>
       <c r="Q54" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="R54" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="S54" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="T54" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="U54" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="V54" s="1">
         <v>46321</v>
@@ -3723,28 +3732,28 @@
         <v>43</v>
       </c>
       <c r="N55" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O55" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="P55">
         <v>5000000</v>
       </c>
       <c r="Q55" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="R55" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="S55" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="T55" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="U55" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="V55" s="1">
         <v>46321</v>
@@ -3773,25 +3782,25 @@
         <v>42</v>
       </c>
       <c r="N56" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O56" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="Q56" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="R56" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="S56" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="T56" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="U56" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="V56" s="1">
         <v>46049</v>
@@ -3820,25 +3829,25 @@
         <v>42</v>
       </c>
       <c r="N57" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O57" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="Q57" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="R57" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="S57" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="T57" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="U57" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="58" spans="1:22">
@@ -3864,25 +3873,25 @@
         <v>42</v>
       </c>
       <c r="N58" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O58" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="Q58" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="R58" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="S58" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="T58" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="U58" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="59" spans="1:22">
@@ -3902,28 +3911,28 @@
         <v>29</v>
       </c>
       <c r="N59" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="O59" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="P59">
         <v>9389.959999999999</v>
       </c>
       <c r="Q59" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="R59" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="S59" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="T59" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="U59" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="V59" s="1">
         <v>46107</v>
@@ -3946,28 +3955,28 @@
         <v>29</v>
       </c>
       <c r="N60" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="O60" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="P60">
         <v>7204.82</v>
       </c>
       <c r="Q60" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="R60" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="S60" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="T60" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="U60" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="V60" s="1">
         <v>46107</v>
@@ -3990,28 +3999,28 @@
         <v>29</v>
       </c>
       <c r="N61" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="O61" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="P61">
         <v>4227.84</v>
       </c>
       <c r="Q61" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="R61" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="S61" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="T61" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="U61" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="V61" s="1">
         <v>46107</v>
@@ -4034,28 +4043,28 @@
         <v>29</v>
       </c>
       <c r="N62" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="O62" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="P62">
         <v>4064.54</v>
       </c>
       <c r="Q62" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="R62" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="S62" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="T62" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="U62" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="V62" s="1">
         <v>46107</v>
@@ -4078,28 +4087,28 @@
         <v>29</v>
       </c>
       <c r="N63" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="O63" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="P63">
         <v>3662.66</v>
       </c>
       <c r="Q63" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="R63" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="S63" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="T63" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="U63" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="V63" s="1">
         <v>46107</v>
@@ -4122,28 +4131,28 @@
         <v>29</v>
       </c>
       <c r="N64" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="O64" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="P64">
         <v>1163.64</v>
       </c>
       <c r="Q64" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="R64" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="S64" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="T64" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="U64" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="V64" s="1">
         <v>46107</v>
@@ -4166,25 +4175,25 @@
         <v>29</v>
       </c>
       <c r="N65" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="O65" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="P65">
         <v>120000</v>
       </c>
       <c r="Q65" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="R65" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="S65" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="T65" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="U65" t="s">
         <v>28</v>
@@ -4213,25 +4222,25 @@
         <v>30</v>
       </c>
       <c r="N66" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="O66" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="P66">
         <v>400000</v>
       </c>
       <c r="Q66" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="R66" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="S66" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T66" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="U66" t="s">
         <v>28</v>
@@ -4260,28 +4269,28 @@
         <v>30</v>
       </c>
       <c r="N67" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="O67" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="P67">
         <v>100000</v>
       </c>
       <c r="Q67" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="R67" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="S67" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T67" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="U67" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="V67" s="1">
         <v>46229</v>
@@ -4304,25 +4313,25 @@
         <v>29</v>
       </c>
       <c r="N68" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="O68" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="P68">
         <v>80000</v>
       </c>
       <c r="Q68" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="R68" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="S68" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="T68" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="U68" t="s">
         <v>28</v>
@@ -4348,28 +4357,28 @@
         <v>29</v>
       </c>
       <c r="N69" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="O69" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="P69">
         <v>835000</v>
       </c>
       <c r="Q69" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="R69" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="S69" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="T69" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="U69" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="V69" s="1">
         <v>46291</v>
@@ -4392,28 +4401,28 @@
         <v>29</v>
       </c>
       <c r="N70" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="O70" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="P70">
         <v>165000</v>
       </c>
       <c r="Q70" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="R70" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="S70" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="T70" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="U70" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="V70" s="1">
         <v>46168</v>
@@ -4436,28 +4445,28 @@
         <v>29</v>
       </c>
       <c r="N71" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="O71" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="P71">
         <v>1000000</v>
       </c>
       <c r="Q71" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="R71" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="S71" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="T71" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="U71" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="V71" s="1">
         <v>46291</v>
@@ -4480,28 +4489,28 @@
         <v>29</v>
       </c>
       <c r="N72" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="O72" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="P72">
         <v>1000000</v>
       </c>
       <c r="Q72" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="R72" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="S72" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="T72" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="U72" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="V72" s="1">
         <v>46291</v>
@@ -4524,28 +4533,28 @@
         <v>29</v>
       </c>
       <c r="N73" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="O73" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="P73">
         <v>100000</v>
       </c>
       <c r="Q73" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="R73" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="S73" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="T73" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="U73" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="V73" s="1">
         <v>46291</v>
@@ -4571,25 +4580,25 @@
         <v>30</v>
       </c>
       <c r="N74" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="O74" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="P74">
         <v>1000000</v>
       </c>
       <c r="Q74" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="R74" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="S74" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T74" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="U74" t="s">
         <v>28</v>
@@ -4621,28 +4630,28 @@
         <v>44</v>
       </c>
       <c r="N75" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="O75" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="P75">
         <v>1704503</v>
       </c>
       <c r="Q75" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="R75" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="S75" t="s">
         <v>40</v>
       </c>
       <c r="T75" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="U75" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="V75" s="1">
         <v>46381</v>
@@ -4671,28 +4680,28 @@
         <v>44</v>
       </c>
       <c r="N76" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="O76" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="P76">
         <v>1638125.5</v>
       </c>
       <c r="Q76" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="R76" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="S76" t="s">
         <v>40</v>
       </c>
       <c r="T76" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="U76" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="V76" s="1">
         <v>46381</v>
@@ -4721,25 +4730,25 @@
         <v>44</v>
       </c>
       <c r="N77" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="O77" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="P77">
         <v>3800000</v>
       </c>
       <c r="Q77" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="R77" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="S77" t="s">
         <v>40</v>
       </c>
       <c r="T77" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="U77" t="s">
         <v>28</v>
@@ -4771,25 +4780,25 @@
         <v>44</v>
       </c>
       <c r="N78" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="O78" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="P78">
         <v>3800000</v>
       </c>
       <c r="Q78" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="R78" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="S78" t="s">
         <v>40</v>
       </c>
       <c r="T78" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="U78" t="s">
         <v>28</v>
@@ -4815,25 +4824,25 @@
         <v>29</v>
       </c>
       <c r="N79" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="O79" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="P79">
         <v>3800000</v>
       </c>
       <c r="Q79" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="R79" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="S79" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="T79" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="U79" t="s">
         <v>28</v>
@@ -4859,25 +4868,25 @@
         <v>28</v>
       </c>
       <c r="N80" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="O80" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="P80">
         <v>4394700</v>
       </c>
       <c r="Q80" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="R80" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="S80" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="T80" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="U80" t="s">
         <v>28</v>
@@ -4906,28 +4915,28 @@
         <v>30</v>
       </c>
       <c r="N81" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="O81" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="P81">
         <v>528395.9300000001</v>
       </c>
       <c r="Q81" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="R81" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="S81" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="T81" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="U81" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="V81" s="1">
         <v>46382</v>
@@ -4950,25 +4959,25 @@
         <v>29</v>
       </c>
       <c r="N82" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="O82" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="P82">
         <v>1000000</v>
       </c>
       <c r="Q82" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="R82" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="S82" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="T82" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="U82" t="s">
         <v>28</v>
@@ -4994,25 +5003,25 @@
         <v>28</v>
       </c>
       <c r="N83" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="O83" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="P83">
         <v>4394700</v>
       </c>
       <c r="Q83" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="R83" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="S83" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="T83" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="U83" t="s">
         <v>28</v>

</xml_diff>

<commit_message>
Atualização automática: mta (10/08/2026 13:05)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1067" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1064" uniqueCount="171">
   <si>
     <t>linha</t>
   </si>
@@ -1074,7 +1074,7 @@
         <v>28</v>
       </c>
       <c r="V4" s="1">
-        <v>46260</v>
+        <v>46321</v>
       </c>
     </row>
     <row r="5" spans="1:22">
@@ -1121,7 +1121,7 @@
         <v>28</v>
       </c>
       <c r="V5" s="1">
-        <v>46260</v>
+        <v>46321</v>
       </c>
     </row>
     <row r="6" spans="1:22">
@@ -1880,7 +1880,7 @@
         <v>28</v>
       </c>
       <c r="V20" s="1">
-        <v>46291</v>
+        <v>46321</v>
       </c>
     </row>
     <row r="21" spans="1:22">
@@ -3291,7 +3291,7 @@
         <v>28</v>
       </c>
       <c r="V46" s="1">
-        <v>46260</v>
+        <v>46321</v>
       </c>
     </row>
     <row r="47" spans="1:22">
@@ -3770,13 +3770,10 @@
         <v>22</v>
       </c>
       <c r="D56" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E56" t="s">
-        <v>28</v>
-      </c>
-      <c r="F56" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="G56" t="s">
         <v>42</v>
@@ -3822,9 +3819,6 @@
       <c r="E57" t="s">
         <v>29</v>
       </c>
-      <c r="F57" t="s">
-        <v>39</v>
-      </c>
       <c r="G57" t="s">
         <v>42</v>
       </c>
@@ -3865,9 +3859,6 @@
       </c>
       <c r="E58" t="s">
         <v>29</v>
-      </c>
-      <c r="F58" t="s">
-        <v>39</v>
       </c>
       <c r="G58" t="s">
         <v>42</v>

</xml_diff>

<commit_message>
Atualização automática: mta (10/08/2026 14:56)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1064" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1102" uniqueCount="174">
   <si>
     <t>linha</t>
   </si>
@@ -88,6 +88,9 @@
     <t>MOD C-98</t>
   </si>
   <si>
+    <t>T-27</t>
+  </si>
+  <si>
     <t>Aprovado, aguardando atendimento</t>
   </si>
   <si>
@@ -280,6 +283,12 @@
     <t>CNT XXX/CABW-PAMASP/2026 - XX- Exchange</t>
   </si>
   <si>
+    <t>Exchange PT6A-114A</t>
+  </si>
+  <si>
+    <t>CNT 018/CELOG-PAMASP/2026 - SERVIÇO - TOFI</t>
+  </si>
+  <si>
     <t>Atualização de GPS</t>
   </si>
   <si>
@@ -472,13 +481,13 @@
     <t>Revisão Geral PT6A-114A</t>
   </si>
   <si>
-    <t>Exchange PT6A-114A</t>
-  </si>
-  <si>
     <t>Hora de Voo 10/10 - 310 HV</t>
   </si>
   <si>
     <t>Material reparo PT6A-114A (4/4)</t>
+  </si>
+  <si>
+    <t>Reparo de estatores dos geradores DO C95/T/27 - TOEG</t>
   </si>
   <si>
     <t>CABW</t>
@@ -862,7 +871,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V83"/>
+  <dimension ref="A1:V86"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
@@ -944,40 +953,40 @@
         <v>22</v>
       </c>
       <c r="D2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="L2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="N2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="O2" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="P2">
         <v>135000</v>
       </c>
       <c r="Q2" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="R2" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="S2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T2" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="U2" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="V2" s="1">
         <v>46229</v>
@@ -994,37 +1003,37 @@
         <v>22</v>
       </c>
       <c r="D3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="O3" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="P3">
         <v>400000</v>
       </c>
       <c r="Q3" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="R3" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="S3" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T3" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="U3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V3" s="1">
         <v>46291</v>
@@ -1041,37 +1050,37 @@
         <v>22</v>
       </c>
       <c r="D4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N4" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="O4" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="P4">
         <v>430000</v>
       </c>
       <c r="Q4" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="R4" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="S4" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T4" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="U4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V4" s="1">
         <v>46321</v>
@@ -1088,37 +1097,37 @@
         <v>22</v>
       </c>
       <c r="D5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="O5" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="P5">
         <v>425000</v>
       </c>
       <c r="Q5" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="R5" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="S5" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T5" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="U5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V5" s="1">
         <v>46321</v>
@@ -1135,40 +1144,40 @@
         <v>22</v>
       </c>
       <c r="D6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="L6" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="N6" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="O6" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="P6">
         <v>563000</v>
       </c>
       <c r="Q6" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="R6" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="S6" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T6" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="U6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V6" s="1">
         <v>46291</v>
@@ -1185,46 +1194,46 @@
         <v>22</v>
       </c>
       <c r="D7" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G7" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H7" s="1">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="N7" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="O7" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="P7">
         <v>3799999.6</v>
       </c>
       <c r="Q7" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="R7" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="S7" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T7" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="U7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V7" s="1">
         <v>46138</v>
@@ -1241,37 +1250,37 @@
         <v>22</v>
       </c>
       <c r="D8" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E8" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N8" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="O8" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="P8">
         <v>430000</v>
       </c>
       <c r="Q8" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="R8" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="S8" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T8" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="U8" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V8" s="1">
         <v>46291</v>
@@ -1288,37 +1297,37 @@
         <v>22</v>
       </c>
       <c r="D9" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E9" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F9" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="O9" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="P9">
         <v>60000</v>
       </c>
       <c r="Q9" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="R9" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="S9" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T9" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="U9" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V9" s="1">
         <v>46291</v>
@@ -1335,37 +1344,37 @@
         <v>22</v>
       </c>
       <c r="D10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E10" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F10" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N10" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="O10" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="P10">
         <v>200000</v>
       </c>
       <c r="Q10" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="R10" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="S10" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T10" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="U10" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V10" s="1">
         <v>46291</v>
@@ -1382,37 +1391,37 @@
         <v>22</v>
       </c>
       <c r="D11" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E11" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F11" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N11" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="O11" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="P11">
         <v>320000</v>
       </c>
       <c r="Q11" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="R11" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="S11" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T11" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="U11" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V11" s="1">
         <v>46291</v>
@@ -1429,49 +1438,49 @@
         <v>22</v>
       </c>
       <c r="D12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E12" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F12" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G12" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H12" s="1">
         <v>46079</v>
       </c>
       <c r="I12" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J12" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="N12" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="O12" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="P12">
         <v>1187433.02</v>
       </c>
       <c r="Q12" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="R12" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="S12" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T12" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="U12" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="V12" s="1">
         <v>46079</v>
@@ -1488,37 +1497,37 @@
         <v>22</v>
       </c>
       <c r="D13" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E13" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F13" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N13" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="O13" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="P13">
         <v>1000000</v>
       </c>
       <c r="Q13" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="R13" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="S13" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T13" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="U13" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="V13" s="1">
         <v>46352</v>
@@ -1535,37 +1544,37 @@
         <v>22</v>
       </c>
       <c r="D14" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E14" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F14" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N14" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="O14" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="P14">
         <v>1000000</v>
       </c>
       <c r="Q14" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="R14" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="S14" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T14" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="U14" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="V14" s="1">
         <v>46352</v>
@@ -1582,37 +1591,37 @@
         <v>22</v>
       </c>
       <c r="D15" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E15" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F15" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N15" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="O15" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="P15">
         <v>1000000</v>
       </c>
       <c r="Q15" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="R15" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="S15" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T15" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="U15" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="V15" s="1">
         <v>46352</v>
@@ -1629,37 +1638,37 @@
         <v>22</v>
       </c>
       <c r="D16" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E16" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F16" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N16" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="O16" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="P16">
         <v>100000</v>
       </c>
       <c r="Q16" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="R16" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="S16" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T16" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="U16" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="V16" s="1">
         <v>46229</v>
@@ -1676,49 +1685,49 @@
         <v>22</v>
       </c>
       <c r="D17" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E17" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F17" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G17" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H17" s="1">
         <v>46098</v>
       </c>
       <c r="I17" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J17" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="N17" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O17" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="P17">
         <v>1770880.5</v>
       </c>
       <c r="Q17" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="R17" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="S17" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T17" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="U17" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="V17" s="1">
         <v>46107</v>
@@ -1735,46 +1744,46 @@
         <v>22</v>
       </c>
       <c r="D18" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E18" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F18" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G18" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H18" s="1">
         <v>46076</v>
       </c>
       <c r="I18" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="N18" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="O18" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="P18">
         <v>350000</v>
       </c>
       <c r="Q18" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="R18" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="S18" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T18" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="U18" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V18" s="1">
         <v>46079</v>
@@ -1791,46 +1800,46 @@
         <v>22</v>
       </c>
       <c r="D19" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E19" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F19" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G19" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H19" s="1">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="N19" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="O19" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="P19">
         <v>350000</v>
       </c>
       <c r="Q19" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="R19" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="S19" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T19" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="U19" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V19" s="1">
         <v>46079</v>
@@ -1847,37 +1856,37 @@
         <v>22</v>
       </c>
       <c r="D20" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E20" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F20" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N20" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="O20" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="P20">
         <v>1000000</v>
       </c>
       <c r="Q20" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="R20" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="S20" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T20" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="U20" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V20" s="1">
         <v>46321</v>
@@ -1894,37 +1903,37 @@
         <v>22</v>
       </c>
       <c r="D21" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E21" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F21" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N21" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="O21" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="P21">
         <v>400000</v>
       </c>
       <c r="Q21" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="R21" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="S21" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T21" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="U21" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V21" s="1">
         <v>46321</v>
@@ -1941,37 +1950,37 @@
         <v>22</v>
       </c>
       <c r="D22" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E22" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F22" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N22" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="O22" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="P22">
         <v>120000</v>
       </c>
       <c r="Q22" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="R22" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="S22" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T22" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="U22" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V22" s="1">
         <v>46321</v>
@@ -1988,37 +1997,37 @@
         <v>22</v>
       </c>
       <c r="D23" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E23" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F23" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N23" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="O23" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="P23">
         <v>80000</v>
       </c>
       <c r="Q23" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="R23" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="S23" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T23" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="U23" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V23" s="1">
         <v>46321</v>
@@ -2035,49 +2044,49 @@
         <v>22</v>
       </c>
       <c r="D24" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E24" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F24" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G24" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H24" s="1">
         <v>46119</v>
       </c>
       <c r="I24" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J24" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="N24" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O24" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="P24">
         <v>1704503</v>
       </c>
       <c r="Q24" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="R24" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="S24" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T24" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="U24" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="V24" s="1">
         <v>46138</v>
@@ -2094,46 +2103,46 @@
         <v>22</v>
       </c>
       <c r="D25" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E25" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F25" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G25" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H25" s="1">
         <v>46121</v>
       </c>
       <c r="I25" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="N25" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O25" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="P25">
         <v>3799000</v>
       </c>
       <c r="Q25" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="R25" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="S25" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T25" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="U25" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V25" s="1">
         <v>46138</v>
@@ -2150,46 +2159,46 @@
         <v>22</v>
       </c>
       <c r="D26" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E26" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F26" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G26" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H26" s="1">
         <v>46076</v>
       </c>
       <c r="I26" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="N26" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O26" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="P26">
         <v>1000</v>
       </c>
       <c r="Q26" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="R26" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="S26" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T26" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="U26" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V26" s="1">
         <v>46079</v>
@@ -2206,37 +2215,37 @@
         <v>22</v>
       </c>
       <c r="D27" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E27" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F27" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N27" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="O27" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="P27">
         <v>100000</v>
       </c>
       <c r="Q27" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="R27" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="S27" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T27" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="U27" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="V27" s="1">
         <v>46291</v>
@@ -2253,49 +2262,49 @@
         <v>22</v>
       </c>
       <c r="D28" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E28" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F28" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G28" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H28" s="1">
         <v>46199</v>
       </c>
       <c r="I28" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J28" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="N28" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O28" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="P28">
         <v>150000</v>
       </c>
       <c r="Q28" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="R28" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="S28" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T28" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="U28" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="V28" s="1">
         <v>46199</v>
@@ -2312,49 +2321,49 @@
         <v>22</v>
       </c>
       <c r="D29" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E29" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F29" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G29" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H29" s="1">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J29" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="N29" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O29" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="P29">
         <v>150000</v>
       </c>
       <c r="Q29" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="R29" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="S29" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T29" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="U29" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="V29" s="1">
         <v>46199</v>
@@ -2371,49 +2380,49 @@
         <v>22</v>
       </c>
       <c r="D30" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E30" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F30" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G30" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H30" s="1">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="J30" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="N30" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O30" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="P30">
         <v>18462.36</v>
       </c>
       <c r="Q30" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="R30" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="S30" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T30" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="U30" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="V30" s="1">
         <v>46199</v>
@@ -2430,49 +2439,49 @@
         <v>22</v>
       </c>
       <c r="D31" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E31" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F31" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G31" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H31" s="1">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J31" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="N31" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O31" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="P31">
         <v>324166.14</v>
       </c>
       <c r="Q31" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="R31" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="S31" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T31" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="U31" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="V31" s="1">
         <v>46199</v>
@@ -2489,37 +2498,37 @@
         <v>22</v>
       </c>
       <c r="D32" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E32" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F32" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N32" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O32" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="P32">
         <v>30000</v>
       </c>
       <c r="Q32" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="R32" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="S32" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T32" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="U32" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="V32" s="1">
         <v>46291</v>
@@ -2536,49 +2545,49 @@
         <v>22</v>
       </c>
       <c r="D33" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E33" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F33" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G33" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H33" s="1">
         <v>46191</v>
       </c>
       <c r="I33" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J33" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="N33" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O33" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="P33">
         <v>1496713.48</v>
       </c>
       <c r="Q33" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="R33" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="S33" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T33" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="U33" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="V33" s="1">
         <v>46199</v>
@@ -2595,46 +2604,46 @@
         <v>22</v>
       </c>
       <c r="D34" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E34" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F34" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G34" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H34" s="1">
         <v>46119</v>
       </c>
       <c r="I34" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="N34" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O34" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="P34">
         <v>207789.52</v>
       </c>
       <c r="Q34" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="R34" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="S34" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T34" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="U34" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="V34" s="1">
         <v>46138</v>
@@ -2651,46 +2660,46 @@
         <v>22</v>
       </c>
       <c r="D35" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E35" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F35" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G35" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H35" s="1">
         <v>46213</v>
       </c>
       <c r="I35" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="N35" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O35" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="P35">
         <v>962290.8</v>
       </c>
       <c r="Q35" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="R35" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="S35" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T35" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="U35" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V35" s="1">
         <v>46229</v>
@@ -2707,46 +2716,46 @@
         <v>22</v>
       </c>
       <c r="D36" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E36" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F36" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G36" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H36" s="1">
         <v>46175</v>
       </c>
       <c r="I36" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="N36" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O36" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="P36">
         <v>800000</v>
       </c>
       <c r="Q36" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="R36" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="S36" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T36" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="U36" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V36" s="1">
         <v>46199</v>
@@ -2763,46 +2772,46 @@
         <v>22</v>
       </c>
       <c r="D37" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E37" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F37" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G37" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H37" s="1">
         <v>46213</v>
       </c>
       <c r="I37" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="N37" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O37" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="P37">
         <v>1530656.62</v>
       </c>
       <c r="Q37" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="R37" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="S37" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T37" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="U37" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V37" s="1">
         <v>46229</v>
@@ -2819,46 +2828,46 @@
         <v>22</v>
       </c>
       <c r="D38" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E38" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F38" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G38" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H38" s="1">
         <v>46199</v>
       </c>
       <c r="I38" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="N38" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O38" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="P38">
         <v>72958.08</v>
       </c>
       <c r="Q38" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="R38" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="S38" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T38" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="U38" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V38" s="1">
         <v>46199</v>
@@ -2875,46 +2884,46 @@
         <v>22</v>
       </c>
       <c r="D39" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E39" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F39" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G39" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H39" s="1">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="N39" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O39" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="P39">
         <v>8916</v>
       </c>
       <c r="Q39" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="R39" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="S39" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T39" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="U39" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V39" s="1">
         <v>46199</v>
@@ -2931,46 +2940,46 @@
         <v>22</v>
       </c>
       <c r="D40" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E40" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F40" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G40" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H40" s="1">
         <v>46204</v>
       </c>
       <c r="I40" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="N40" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O40" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="P40">
         <v>425178.5</v>
       </c>
       <c r="Q40" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="R40" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="S40" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T40" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="U40" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V40" s="1">
         <v>46229</v>
@@ -2987,34 +2996,34 @@
         <v>22</v>
       </c>
       <c r="D41" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E41" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G41" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="N41" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O41" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="Q41" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="R41" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="S41" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="T41" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="U41" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V41" s="1">
         <v>46260</v>
@@ -3031,46 +3040,46 @@
         <v>22</v>
       </c>
       <c r="D42" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E42" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F42" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G42" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H42" s="1">
         <v>46191</v>
       </c>
       <c r="I42" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="N42" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="O42" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="P42">
         <v>400000</v>
       </c>
       <c r="Q42" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="R42" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="S42" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T42" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="U42" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V42" s="1">
         <v>46199</v>
@@ -3087,46 +3096,46 @@
         <v>22</v>
       </c>
       <c r="D43" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E43" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F43" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G43" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H43" s="1">
         <v>46191</v>
       </c>
       <c r="I43" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="N43" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="O43" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="P43">
         <v>400000</v>
       </c>
       <c r="Q43" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="R43" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="S43" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T43" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="U43" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V43" s="1">
         <v>46199</v>
@@ -3143,49 +3152,49 @@
         <v>22</v>
       </c>
       <c r="D44" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E44" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F44" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G44" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H44" s="1">
         <v>46213</v>
       </c>
       <c r="I44" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J44" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="N44" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O44" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="P44">
         <v>173846.38</v>
       </c>
       <c r="Q44" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="R44" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="S44" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T44" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="U44" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="V44" s="1">
         <v>46229</v>
@@ -3202,46 +3211,46 @@
         <v>22</v>
       </c>
       <c r="D45" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E45" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F45" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G45" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H45" s="1">
         <v>46210</v>
       </c>
       <c r="I45" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="N45" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O45" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="P45">
         <v>1530656.62</v>
       </c>
       <c r="Q45" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="R45" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="S45" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T45" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="U45" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="V45" s="1">
         <v>46229</v>
@@ -3258,37 +3267,37 @@
         <v>22</v>
       </c>
       <c r="D46" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E46" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F46" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N46" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="O46" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="P46">
         <v>1000000</v>
       </c>
       <c r="Q46" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="R46" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="S46" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T46" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="U46" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V46" s="1">
         <v>46321</v>
@@ -3305,37 +3314,37 @@
         <v>22</v>
       </c>
       <c r="D47" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E47" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F47" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N47" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="O47" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="P47">
         <v>958040</v>
       </c>
       <c r="Q47" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="R47" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="S47" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T47" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="U47" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="V47" s="1">
         <v>46291</v>
@@ -3352,49 +3361,49 @@
         <v>22</v>
       </c>
       <c r="D48" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E48" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F48" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G48" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H48" s="1">
         <v>46176</v>
       </c>
       <c r="I48" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="J48" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="N48" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="O48" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="P48">
         <v>41730.64</v>
       </c>
       <c r="Q48" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="R48" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="S48" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T48" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="U48" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="V48" s="1">
         <v>46199</v>
@@ -3411,43 +3420,43 @@
         <v>22</v>
       </c>
       <c r="D49" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E49" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F49" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="J49" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="K49" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="N49" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O49" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="P49">
         <v>1468159.32</v>
       </c>
       <c r="Q49" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="R49" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="S49" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T49" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="U49" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="V49" s="1">
         <v>46260</v>
@@ -3464,43 +3473,43 @@
         <v>22</v>
       </c>
       <c r="D50" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E50" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F50" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="J50" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="K50" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="N50" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O50" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="P50">
         <v>1704503</v>
       </c>
       <c r="Q50" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="R50" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="S50" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T50" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="U50" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="V50" s="1">
         <v>46291</v>
@@ -3517,40 +3526,40 @@
         <v>22</v>
       </c>
       <c r="D51" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E51" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F51" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="K51" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="N51" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O51" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="P51">
         <v>1704503</v>
       </c>
       <c r="Q51" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="R51" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="S51" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T51" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="U51" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="V51" s="1">
         <v>46321</v>
@@ -3567,46 +3576,46 @@
         <v>22</v>
       </c>
       <c r="D52" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E52" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F52" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G52" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H52" s="1">
         <v>46227</v>
       </c>
       <c r="I52" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="N52" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O52" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="P52">
         <v>236343.68</v>
       </c>
       <c r="Q52" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="R52" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="S52" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T52" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="U52" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="V52" s="1">
         <v>46229</v>
@@ -3623,37 +3632,37 @@
         <v>22</v>
       </c>
       <c r="D53" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E53" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F53" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N53" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O53" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="P53">
         <v>1295422.28</v>
       </c>
       <c r="Q53" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="R53" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="S53" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T53" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="U53" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="V53" s="1">
         <v>46352</v>
@@ -3670,40 +3679,40 @@
         <v>22</v>
       </c>
       <c r="D54" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E54" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F54" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="K54" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="N54" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="O54" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="P54">
         <v>500000</v>
       </c>
       <c r="Q54" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="R54" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="S54" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="T54" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="U54" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="V54" s="1">
         <v>46321</v>
@@ -3720,40 +3729,40 @@
         <v>22</v>
       </c>
       <c r="D55" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E55" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F55" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G55" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="N55" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="O55" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="P55">
         <v>5000000</v>
       </c>
       <c r="Q55" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="R55" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="S55" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="T55" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="U55" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="V55" s="1">
         <v>46321</v>
@@ -3770,34 +3779,34 @@
         <v>22</v>
       </c>
       <c r="D56" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E56" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G56" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="N56" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="O56" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="Q56" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="R56" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="S56" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="T56" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="U56" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="V56" s="1">
         <v>46049</v>
@@ -3814,34 +3823,34 @@
         <v>22</v>
       </c>
       <c r="D57" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E57" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G57" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="N57" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="O57" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="Q57" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="R57" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="S57" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="T57" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="U57" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
     </row>
     <row r="58" spans="1:22">
@@ -3855,34 +3864,34 @@
         <v>22</v>
       </c>
       <c r="D58" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E58" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G58" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="N58" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="O58" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="Q58" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="R58" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="S58" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="T58" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="U58" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
     </row>
     <row r="59" spans="1:22">
@@ -3896,34 +3905,34 @@
         <v>22</v>
       </c>
       <c r="D59" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E59" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N59" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="O59" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="P59">
         <v>9389.959999999999</v>
       </c>
       <c r="Q59" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="R59" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="S59" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="T59" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="U59" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="V59" s="1">
         <v>46107</v>
@@ -3940,34 +3949,34 @@
         <v>22</v>
       </c>
       <c r="D60" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E60" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N60" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="O60" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="P60">
         <v>7204.82</v>
       </c>
       <c r="Q60" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="R60" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="S60" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="T60" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="U60" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="V60" s="1">
         <v>46107</v>
@@ -3984,34 +3993,34 @@
         <v>22</v>
       </c>
       <c r="D61" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E61" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N61" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="O61" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="P61">
         <v>4227.84</v>
       </c>
       <c r="Q61" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="R61" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="S61" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="T61" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="U61" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="V61" s="1">
         <v>46107</v>
@@ -4028,34 +4037,34 @@
         <v>22</v>
       </c>
       <c r="D62" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E62" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N62" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="O62" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="P62">
         <v>4064.54</v>
       </c>
       <c r="Q62" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="R62" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="S62" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="T62" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="U62" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="V62" s="1">
         <v>46107</v>
@@ -4072,34 +4081,34 @@
         <v>22</v>
       </c>
       <c r="D63" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E63" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N63" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="O63" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="P63">
         <v>3662.66</v>
       </c>
       <c r="Q63" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="R63" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="S63" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="T63" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="U63" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="V63" s="1">
         <v>46107</v>
@@ -4116,34 +4125,34 @@
         <v>22</v>
       </c>
       <c r="D64" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E64" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N64" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="O64" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="P64">
         <v>1163.64</v>
       </c>
       <c r="Q64" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="R64" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="S64" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="T64" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="U64" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="V64" s="1">
         <v>46107</v>
@@ -4160,34 +4169,34 @@
         <v>22</v>
       </c>
       <c r="D65" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E65" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N65" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="O65" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="P65">
         <v>120000</v>
       </c>
       <c r="Q65" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="R65" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="S65" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="T65" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="U65" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V65" s="1">
         <v>46168</v>
@@ -4204,37 +4213,37 @@
         <v>22</v>
       </c>
       <c r="D66" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E66" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F66" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N66" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="O66" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="P66">
         <v>400000</v>
       </c>
       <c r="Q66" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="R66" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="S66" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T66" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="U66" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V66" s="1">
         <v>46291</v>
@@ -4251,37 +4260,37 @@
         <v>22</v>
       </c>
       <c r="D67" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E67" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F67" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N67" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="O67" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="P67">
         <v>100000</v>
       </c>
       <c r="Q67" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="R67" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="S67" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T67" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="U67" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="V67" s="1">
         <v>46229</v>
@@ -4298,34 +4307,34 @@
         <v>22</v>
       </c>
       <c r="D68" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E68" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N68" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="O68" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="P68">
         <v>80000</v>
       </c>
       <c r="Q68" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="R68" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="S68" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="T68" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="U68" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V68" s="1">
         <v>46260</v>
@@ -4342,34 +4351,34 @@
         <v>22</v>
       </c>
       <c r="D69" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E69" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N69" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="O69" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="P69">
         <v>835000</v>
       </c>
       <c r="Q69" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="R69" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="S69" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="T69" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="U69" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="V69" s="1">
         <v>46291</v>
@@ -4386,34 +4395,34 @@
         <v>22</v>
       </c>
       <c r="D70" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E70" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N70" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="O70" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="P70">
         <v>165000</v>
       </c>
       <c r="Q70" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="R70" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="S70" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="T70" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="U70" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="V70" s="1">
         <v>46168</v>
@@ -4430,34 +4439,34 @@
         <v>22</v>
       </c>
       <c r="D71" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E71" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N71" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="O71" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="P71">
         <v>1000000</v>
       </c>
       <c r="Q71" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="R71" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="S71" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="T71" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="U71" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="V71" s="1">
         <v>46291</v>
@@ -4474,34 +4483,34 @@
         <v>22</v>
       </c>
       <c r="D72" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E72" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N72" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="O72" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="P72">
         <v>1000000</v>
       </c>
       <c r="Q72" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="R72" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="S72" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="T72" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="U72" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="V72" s="1">
         <v>46291</v>
@@ -4518,34 +4527,34 @@
         <v>22</v>
       </c>
       <c r="D73" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E73" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N73" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="O73" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="P73">
         <v>100000</v>
       </c>
       <c r="Q73" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="R73" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="S73" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="T73" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="U73" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="V73" s="1">
         <v>46291</v>
@@ -4562,37 +4571,37 @@
         <v>22</v>
       </c>
       <c r="D74" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E74" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F74" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N74" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="O74" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="P74">
         <v>1000000</v>
       </c>
       <c r="Q74" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="R74" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="S74" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T74" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="U74" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V74" s="1">
         <v>46321</v>
@@ -4609,40 +4618,40 @@
         <v>22</v>
       </c>
       <c r="D75" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E75" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F75" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G75" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="N75" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O75" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="P75">
         <v>1704503</v>
       </c>
       <c r="Q75" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="R75" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="S75" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="T75" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="U75" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="V75" s="1">
         <v>46381</v>
@@ -4659,40 +4668,40 @@
         <v>22</v>
       </c>
       <c r="D76" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E76" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F76" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G76" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="N76" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O76" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="P76">
         <v>1638125.5</v>
       </c>
       <c r="Q76" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="R76" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="S76" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="T76" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="U76" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="V76" s="1">
         <v>46381</v>
@@ -4709,40 +4718,40 @@
         <v>22</v>
       </c>
       <c r="D77" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E77" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F77" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G77" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="N77" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="O77" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="P77">
         <v>3800000</v>
       </c>
       <c r="Q77" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="R77" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="S77" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="T77" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="U77" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V77" s="1">
         <v>46381</v>
@@ -4759,40 +4768,40 @@
         <v>22</v>
       </c>
       <c r="D78" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E78" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F78" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G78" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="N78" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="O78" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="P78">
         <v>3800000</v>
       </c>
       <c r="Q78" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="R78" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="S78" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="T78" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="U78" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V78" s="1">
         <v>46381</v>
@@ -4809,34 +4818,34 @@
         <v>22</v>
       </c>
       <c r="D79" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E79" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N79" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O79" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="P79">
         <v>3800000</v>
       </c>
       <c r="Q79" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="R79" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="S79" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="T79" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="U79" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V79" s="1">
         <v>46382</v>
@@ -4853,34 +4862,34 @@
         <v>22</v>
       </c>
       <c r="D80" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E80" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N80" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="O80" t="s">
-        <v>152</v>
+        <v>89</v>
       </c>
       <c r="P80">
         <v>4394700</v>
       </c>
       <c r="Q80" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="R80" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="S80" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="T80" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="U80" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V80" s="1">
         <v>46382</v>
@@ -4897,37 +4906,37 @@
         <v>22</v>
       </c>
       <c r="D81" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E81" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F81" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N81" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O81" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="P81">
         <v>528395.9300000001</v>
       </c>
       <c r="Q81" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="R81" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="S81" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="T81" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="U81" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="V81" s="1">
         <v>46382</v>
@@ -4944,34 +4953,34 @@
         <v>22</v>
       </c>
       <c r="D82" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E82" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N82" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="O82" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="P82">
         <v>1000000</v>
       </c>
       <c r="Q82" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="R82" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="S82" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="T82" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="U82" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V82" s="1">
         <v>46321</v>
@@ -4988,37 +4997,178 @@
         <v>22</v>
       </c>
       <c r="D83" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E83" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N83" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="O83" t="s">
-        <v>152</v>
+        <v>89</v>
       </c>
       <c r="P83">
         <v>4394700</v>
       </c>
       <c r="Q83" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="R83" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="S83" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="T83" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="U83" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V83" s="1">
         <v>46382</v>
+      </c>
+    </row>
+    <row r="84" spans="1:22">
+      <c r="A84">
+        <v>64760</v>
+      </c>
+      <c r="B84" t="s">
+        <v>22</v>
+      </c>
+      <c r="C84" t="s">
+        <v>22</v>
+      </c>
+      <c r="D84" t="s">
+        <v>28</v>
+      </c>
+      <c r="E84" t="s">
+        <v>29</v>
+      </c>
+      <c r="F84" t="s">
+        <v>41</v>
+      </c>
+      <c r="G84" t="s">
+        <v>45</v>
+      </c>
+      <c r="N84" t="s">
+        <v>89</v>
+      </c>
+      <c r="O84" t="s">
+        <v>89</v>
+      </c>
+      <c r="P84">
+        <v>3306000</v>
+      </c>
+      <c r="Q84" t="s">
+        <v>158</v>
+      </c>
+      <c r="R84" t="s">
+        <v>162</v>
+      </c>
+      <c r="S84" t="s">
+        <v>41</v>
+      </c>
+      <c r="T84" t="s">
+        <v>170</v>
+      </c>
+      <c r="U84" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="85" spans="1:22">
+      <c r="A85">
+        <v>64780</v>
+      </c>
+      <c r="B85" t="s">
+        <v>22</v>
+      </c>
+      <c r="C85" t="s">
+        <v>22</v>
+      </c>
+      <c r="D85" t="s">
+        <v>28</v>
+      </c>
+      <c r="E85" t="s">
+        <v>29</v>
+      </c>
+      <c r="F85" t="s">
+        <v>41</v>
+      </c>
+      <c r="G85" t="s">
+        <v>45</v>
+      </c>
+      <c r="N85" t="s">
+        <v>89</v>
+      </c>
+      <c r="O85" t="s">
+        <v>89</v>
+      </c>
+      <c r="P85">
+        <v>3306000</v>
+      </c>
+      <c r="Q85" t="s">
+        <v>158</v>
+      </c>
+      <c r="R85" t="s">
+        <v>162</v>
+      </c>
+      <c r="S85" t="s">
+        <v>41</v>
+      </c>
+      <c r="T85" t="s">
+        <v>170</v>
+      </c>
+      <c r="U85" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="86" spans="1:22">
+      <c r="A86">
+        <v>64800</v>
+      </c>
+      <c r="B86" t="s">
+        <v>22</v>
+      </c>
+      <c r="C86" t="s">
+        <v>24</v>
+      </c>
+      <c r="D86" t="s">
+        <v>25</v>
+      </c>
+      <c r="E86" t="s">
+        <v>29</v>
+      </c>
+      <c r="F86" t="s">
+        <v>31</v>
+      </c>
+      <c r="N86" t="s">
+        <v>90</v>
+      </c>
+      <c r="O86" t="s">
+        <v>157</v>
+      </c>
+      <c r="P86">
+        <v>212577</v>
+      </c>
+      <c r="Q86" t="s">
+        <v>160</v>
+      </c>
+      <c r="R86" t="s">
+        <v>161</v>
+      </c>
+      <c r="S86" t="s">
+        <v>165</v>
+      </c>
+      <c r="T86" t="s">
+        <v>172</v>
+      </c>
+      <c r="U86" t="s">
+        <v>30</v>
+      </c>
+      <c r="V86" s="1">
+        <v>46260</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: mta (11/08/2026 11:23)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1102" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1102" uniqueCount="175">
   <si>
     <t>linha</t>
   </si>
@@ -188,6 +188,9 @@
   </si>
   <si>
     <t>C26285</t>
+  </si>
+  <si>
+    <t>C26393</t>
   </si>
   <si>
     <t>C26332</t>
@@ -962,31 +965,31 @@
         <v>31</v>
       </c>
       <c r="L2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="N2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="O2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="P2">
         <v>135000</v>
       </c>
       <c r="Q2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S2" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T2" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U2" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V2" s="1">
         <v>46229</v>
@@ -1012,25 +1015,25 @@
         <v>31</v>
       </c>
       <c r="N3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="O3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="P3">
         <v>400000</v>
       </c>
       <c r="Q3" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="R3" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S3" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T3" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U3" t="s">
         <v>29</v>
@@ -1059,25 +1062,25 @@
         <v>31</v>
       </c>
       <c r="N4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="O4" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="P4">
         <v>430000</v>
       </c>
       <c r="Q4" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R4" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S4" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T4" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U4" t="s">
         <v>29</v>
@@ -1106,25 +1109,25 @@
         <v>31</v>
       </c>
       <c r="N5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="O5" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="P5">
         <v>425000</v>
       </c>
       <c r="Q5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R5" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S5" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T5" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U5" t="s">
         <v>29</v>
@@ -1153,28 +1156,28 @@
         <v>31</v>
       </c>
       <c r="L6" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="N6" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="O6" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="P6">
         <v>563000</v>
       </c>
       <c r="Q6" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R6" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T6" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U6" t="s">
         <v>29</v>
@@ -1212,25 +1215,25 @@
         <v>46</v>
       </c>
       <c r="N7" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="O7" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="P7">
         <v>3799999.6</v>
       </c>
       <c r="Q7" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R7" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S7" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T7" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U7" t="s">
         <v>29</v>
@@ -1259,25 +1262,25 @@
         <v>31</v>
       </c>
       <c r="N8" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="O8" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="P8">
         <v>430000</v>
       </c>
       <c r="Q8" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R8" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S8" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T8" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U8" t="s">
         <v>29</v>
@@ -1306,25 +1309,25 @@
         <v>31</v>
       </c>
       <c r="N9" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="O9" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="P9">
         <v>60000</v>
       </c>
       <c r="Q9" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R9" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S9" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T9" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U9" t="s">
         <v>29</v>
@@ -1353,25 +1356,25 @@
         <v>31</v>
       </c>
       <c r="N10" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="O10" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="P10">
         <v>200000</v>
       </c>
       <c r="Q10" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R10" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S10" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T10" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U10" t="s">
         <v>29</v>
@@ -1400,25 +1403,25 @@
         <v>31</v>
       </c>
       <c r="N11" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="O11" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="P11">
         <v>320000</v>
       </c>
       <c r="Q11" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R11" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S11" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T11" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U11" t="s">
         <v>29</v>
@@ -1456,31 +1459,31 @@
         <v>47</v>
       </c>
       <c r="J12" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="N12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="O12" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="P12">
         <v>1187433.02</v>
       </c>
       <c r="Q12" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R12" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S12" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T12" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U12" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V12" s="1">
         <v>46079</v>
@@ -1506,28 +1509,28 @@
         <v>31</v>
       </c>
       <c r="N13" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="O13" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="P13">
         <v>1000000</v>
       </c>
       <c r="Q13" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R13" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S13" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T13" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U13" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V13" s="1">
         <v>46352</v>
@@ -1553,28 +1556,28 @@
         <v>31</v>
       </c>
       <c r="N14" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="O14" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="P14">
         <v>1000000</v>
       </c>
       <c r="Q14" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R14" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S14" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T14" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U14" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V14" s="1">
         <v>46352</v>
@@ -1600,28 +1603,28 @@
         <v>31</v>
       </c>
       <c r="N15" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="O15" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="P15">
         <v>1000000</v>
       </c>
       <c r="Q15" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R15" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S15" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T15" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U15" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V15" s="1">
         <v>46352</v>
@@ -1647,28 +1650,28 @@
         <v>31</v>
       </c>
       <c r="N16" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O16" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="P16">
         <v>100000</v>
       </c>
       <c r="Q16" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="R16" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S16" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T16" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U16" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V16" s="1">
         <v>46229</v>
@@ -1703,31 +1706,31 @@
         <v>48</v>
       </c>
       <c r="J17" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="N17" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="O17" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="P17">
         <v>1770880.5</v>
       </c>
       <c r="Q17" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R17" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S17" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T17" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U17" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V17" s="1">
         <v>46107</v>
@@ -1762,25 +1765,25 @@
         <v>49</v>
       </c>
       <c r="N18" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="O18" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="P18">
         <v>350000</v>
       </c>
       <c r="Q18" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R18" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S18" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T18" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U18" t="s">
         <v>29</v>
@@ -1818,25 +1821,25 @@
         <v>49</v>
       </c>
       <c r="N19" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="O19" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="P19">
         <v>350000</v>
       </c>
       <c r="Q19" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R19" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S19" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T19" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U19" t="s">
         <v>29</v>
@@ -1865,25 +1868,25 @@
         <v>31</v>
       </c>
       <c r="N20" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O20" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="P20">
         <v>1000000</v>
       </c>
       <c r="Q20" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R20" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S20" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T20" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U20" t="s">
         <v>29</v>
@@ -1912,25 +1915,25 @@
         <v>31</v>
       </c>
       <c r="N21" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="O21" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="P21">
         <v>400000</v>
       </c>
       <c r="Q21" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="R21" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S21" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T21" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U21" t="s">
         <v>29</v>
@@ -1959,25 +1962,25 @@
         <v>31</v>
       </c>
       <c r="N22" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="O22" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="P22">
         <v>120000</v>
       </c>
       <c r="Q22" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R22" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S22" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T22" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U22" t="s">
         <v>29</v>
@@ -2006,25 +2009,25 @@
         <v>31</v>
       </c>
       <c r="N23" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="O23" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="P23">
         <v>80000</v>
       </c>
       <c r="Q23" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R23" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S23" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T23" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U23" t="s">
         <v>29</v>
@@ -2062,31 +2065,31 @@
         <v>50</v>
       </c>
       <c r="J24" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="N24" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="O24" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="P24">
         <v>1704503</v>
       </c>
       <c r="Q24" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R24" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S24" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T24" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U24" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V24" s="1">
         <v>46138</v>
@@ -2121,25 +2124,25 @@
         <v>51</v>
       </c>
       <c r="N25" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="O25" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="P25">
         <v>3799000</v>
       </c>
       <c r="Q25" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R25" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S25" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T25" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U25" t="s">
         <v>29</v>
@@ -2177,25 +2180,25 @@
         <v>52</v>
       </c>
       <c r="N26" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="O26" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="P26">
         <v>1000</v>
       </c>
       <c r="Q26" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R26" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S26" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T26" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U26" t="s">
         <v>29</v>
@@ -2224,28 +2227,28 @@
         <v>31</v>
       </c>
       <c r="N27" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O27" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="P27">
         <v>100000</v>
       </c>
       <c r="Q27" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="R27" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S27" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T27" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U27" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V27" s="1">
         <v>46291</v>
@@ -2280,31 +2283,31 @@
         <v>53</v>
       </c>
       <c r="J28" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="N28" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="O28" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="P28">
         <v>150000</v>
       </c>
       <c r="Q28" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R28" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S28" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T28" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U28" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V28" s="1">
         <v>46199</v>
@@ -2339,31 +2342,31 @@
         <v>53</v>
       </c>
       <c r="J29" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="N29" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="O29" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="P29">
         <v>150000</v>
       </c>
       <c r="Q29" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R29" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S29" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T29" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U29" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V29" s="1">
         <v>46199</v>
@@ -2398,31 +2401,31 @@
         <v>54</v>
       </c>
       <c r="J30" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="N30" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="O30" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="P30">
         <v>18462.36</v>
       </c>
       <c r="Q30" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R30" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S30" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T30" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U30" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V30" s="1">
         <v>46199</v>
@@ -2457,31 +2460,31 @@
         <v>53</v>
       </c>
       <c r="J31" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="N31" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="O31" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="P31">
         <v>324166.14</v>
       </c>
       <c r="Q31" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R31" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S31" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T31" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U31" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V31" s="1">
         <v>46199</v>
@@ -2507,28 +2510,28 @@
         <v>31</v>
       </c>
       <c r="N32" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="O32" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="P32">
         <v>30000</v>
       </c>
       <c r="Q32" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R32" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S32" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T32" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U32" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V32" s="1">
         <v>46291</v>
@@ -2563,31 +2566,31 @@
         <v>55</v>
       </c>
       <c r="J33" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="N33" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="O33" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="P33">
         <v>1496713.48</v>
       </c>
       <c r="Q33" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R33" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S33" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T33" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U33" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V33" s="1">
         <v>46199</v>
@@ -2622,28 +2625,28 @@
         <v>50</v>
       </c>
       <c r="N34" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="O34" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="P34">
         <v>207789.52</v>
       </c>
       <c r="Q34" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R34" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S34" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T34" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U34" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V34" s="1">
         <v>46138</v>
@@ -2678,25 +2681,25 @@
         <v>56</v>
       </c>
       <c r="N35" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="O35" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="P35">
         <v>962290.8</v>
       </c>
       <c r="Q35" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R35" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S35" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T35" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U35" t="s">
         <v>29</v>
@@ -2734,25 +2737,25 @@
         <v>57</v>
       </c>
       <c r="N36" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="O36" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="P36">
-        <v>800000</v>
+        <v>798776.97</v>
       </c>
       <c r="Q36" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R36" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S36" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T36" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U36" t="s">
         <v>29</v>
@@ -2778,43 +2781,43 @@
         <v>29</v>
       </c>
       <c r="F37" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="G37" t="s">
         <v>42</v>
       </c>
       <c r="H37" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="I37" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="N37" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="O37" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="P37">
-        <v>1530656.62</v>
+        <v>1223.03</v>
       </c>
       <c r="Q37" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R37" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S37" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T37" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U37" t="s">
         <v>29</v>
       </c>
       <c r="V37" s="1">
-        <v>46229</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="38" spans="1:22">
@@ -2843,28 +2846,28 @@
         <v>46199</v>
       </c>
       <c r="I38" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="N38" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="O38" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="P38">
         <v>72958.08</v>
       </c>
       <c r="Q38" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R38" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S38" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T38" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U38" t="s">
         <v>29</v>
@@ -2899,28 +2902,28 @@
         <v>46199</v>
       </c>
       <c r="I39" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="N39" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="O39" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="P39">
         <v>8916</v>
       </c>
       <c r="Q39" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R39" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S39" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T39" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U39" t="s">
         <v>29</v>
@@ -2955,28 +2958,28 @@
         <v>46204</v>
       </c>
       <c r="I40" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="N40" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="O40" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="P40">
         <v>425178.5</v>
       </c>
       <c r="Q40" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R40" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S40" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T40" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U40" t="s">
         <v>29</v>
@@ -3005,22 +3008,22 @@
         <v>43</v>
       </c>
       <c r="N41" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="O41" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="Q41" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R41" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S41" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="T41" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U41" t="s">
         <v>29</v>
@@ -3055,28 +3058,28 @@
         <v>46191</v>
       </c>
       <c r="I42" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="N42" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="O42" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="P42">
         <v>400000</v>
       </c>
       <c r="Q42" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R42" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S42" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T42" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U42" t="s">
         <v>29</v>
@@ -3111,28 +3114,28 @@
         <v>46191</v>
       </c>
       <c r="I43" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="N43" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="O43" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="P43">
         <v>400000</v>
       </c>
       <c r="Q43" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R43" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S43" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T43" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U43" t="s">
         <v>29</v>
@@ -3170,31 +3173,31 @@
         <v>55</v>
       </c>
       <c r="J44" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="N44" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="O44" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="P44">
         <v>173846.38</v>
       </c>
       <c r="Q44" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R44" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S44" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T44" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U44" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V44" s="1">
         <v>46229</v>
@@ -3229,28 +3232,28 @@
         <v>54</v>
       </c>
       <c r="N45" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="O45" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="P45">
         <v>1530656.62</v>
       </c>
       <c r="Q45" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R45" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S45" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T45" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U45" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V45" s="1">
         <v>46229</v>
@@ -3276,25 +3279,25 @@
         <v>31</v>
       </c>
       <c r="N46" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O46" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="P46">
         <v>1000000</v>
       </c>
       <c r="Q46" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R46" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S46" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T46" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U46" t="s">
         <v>29</v>
@@ -3323,28 +3326,28 @@
         <v>31</v>
       </c>
       <c r="N47" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="O47" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="P47">
         <v>958040</v>
       </c>
       <c r="Q47" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R47" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S47" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T47" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U47" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V47" s="1">
         <v>46291</v>
@@ -3376,34 +3379,34 @@
         <v>46176</v>
       </c>
       <c r="I48" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="J48" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="N48" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="O48" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="P48">
         <v>41730.64</v>
       </c>
       <c r="Q48" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R48" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="S48" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T48" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U48" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V48" s="1">
         <v>46199</v>
@@ -3429,34 +3432,34 @@
         <v>31</v>
       </c>
       <c r="J49" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="K49" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="N49" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="O49" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="P49">
         <v>1468159.32</v>
       </c>
       <c r="Q49" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R49" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S49" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T49" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U49" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V49" s="1">
         <v>46260</v>
@@ -3482,34 +3485,34 @@
         <v>31</v>
       </c>
       <c r="J50" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="K50" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="N50" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="O50" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="P50">
         <v>1704503</v>
       </c>
       <c r="Q50" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R50" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S50" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T50" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U50" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V50" s="1">
         <v>46291</v>
@@ -3535,31 +3538,31 @@
         <v>31</v>
       </c>
       <c r="K51" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="N51" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="O51" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="P51">
         <v>1704503</v>
       </c>
       <c r="Q51" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R51" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S51" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T51" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U51" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V51" s="1">
         <v>46321</v>
@@ -3591,31 +3594,31 @@
         <v>46227</v>
       </c>
       <c r="I52" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="N52" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="O52" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="P52">
         <v>236343.68</v>
       </c>
       <c r="Q52" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R52" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S52" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T52" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U52" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V52" s="1">
         <v>46229</v>
@@ -3641,28 +3644,28 @@
         <v>31</v>
       </c>
       <c r="N53" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="O53" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="P53">
         <v>1295422.28</v>
       </c>
       <c r="Q53" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R53" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S53" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T53" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U53" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V53" s="1">
         <v>46352</v>
@@ -3688,31 +3691,31 @@
         <v>40</v>
       </c>
       <c r="K54" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="N54" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="O54" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="P54">
         <v>500000</v>
       </c>
       <c r="Q54" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R54" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S54" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="T54" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="U54" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V54" s="1">
         <v>46321</v>
@@ -3741,28 +3744,28 @@
         <v>44</v>
       </c>
       <c r="N55" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="O55" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="P55">
         <v>5000000</v>
       </c>
       <c r="Q55" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R55" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S55" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="T55" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="U55" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V55" s="1">
         <v>46321</v>
@@ -3788,25 +3791,25 @@
         <v>43</v>
       </c>
       <c r="N56" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="O56" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="Q56" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R56" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S56" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="T56" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="U56" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V56" s="1">
         <v>46049</v>
@@ -3832,25 +3835,25 @@
         <v>43</v>
       </c>
       <c r="N57" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="O57" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="Q57" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R57" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S57" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="T57" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="U57" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="58" spans="1:22">
@@ -3873,25 +3876,25 @@
         <v>43</v>
       </c>
       <c r="N58" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="O58" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="Q58" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R58" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S58" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="T58" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="U58" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="59" spans="1:22">
@@ -3911,28 +3914,28 @@
         <v>30</v>
       </c>
       <c r="N59" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="O59" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="P59">
         <v>9389.959999999999</v>
       </c>
       <c r="Q59" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R59" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="S59" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="T59" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U59" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V59" s="1">
         <v>46107</v>
@@ -3955,28 +3958,28 @@
         <v>30</v>
       </c>
       <c r="N60" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="O60" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="P60">
         <v>7204.82</v>
       </c>
       <c r="Q60" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R60" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="S60" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="T60" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U60" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V60" s="1">
         <v>46107</v>
@@ -3999,28 +4002,28 @@
         <v>30</v>
       </c>
       <c r="N61" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="O61" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="P61">
         <v>4227.84</v>
       </c>
       <c r="Q61" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R61" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="S61" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="T61" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U61" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V61" s="1">
         <v>46107</v>
@@ -4043,28 +4046,28 @@
         <v>30</v>
       </c>
       <c r="N62" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="O62" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="P62">
         <v>4064.54</v>
       </c>
       <c r="Q62" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R62" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="S62" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="T62" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U62" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V62" s="1">
         <v>46107</v>
@@ -4087,28 +4090,28 @@
         <v>30</v>
       </c>
       <c r="N63" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="O63" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="P63">
         <v>3662.66</v>
       </c>
       <c r="Q63" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R63" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="S63" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="T63" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U63" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V63" s="1">
         <v>46107</v>
@@ -4131,28 +4134,28 @@
         <v>30</v>
       </c>
       <c r="N64" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="O64" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="P64">
         <v>1163.64</v>
       </c>
       <c r="Q64" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="R64" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="S64" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="T64" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U64" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V64" s="1">
         <v>46107</v>
@@ -4175,25 +4178,25 @@
         <v>30</v>
       </c>
       <c r="N65" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="O65" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="P65">
         <v>120000</v>
       </c>
       <c r="Q65" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R65" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S65" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="T65" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U65" t="s">
         <v>29</v>
@@ -4222,25 +4225,25 @@
         <v>31</v>
       </c>
       <c r="N66" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="O66" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="P66">
         <v>400000</v>
       </c>
       <c r="Q66" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="R66" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S66" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T66" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U66" t="s">
         <v>29</v>
@@ -4269,28 +4272,28 @@
         <v>31</v>
       </c>
       <c r="N67" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O67" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="P67">
         <v>100000</v>
       </c>
       <c r="Q67" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="R67" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S67" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T67" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U67" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V67" s="1">
         <v>46229</v>
@@ -4313,25 +4316,25 @@
         <v>30</v>
       </c>
       <c r="N68" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="O68" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="P68">
         <v>80000</v>
       </c>
       <c r="Q68" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R68" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S68" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="T68" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U68" t="s">
         <v>29</v>
@@ -4357,28 +4360,28 @@
         <v>30</v>
       </c>
       <c r="N69" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="O69" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="P69">
         <v>835000</v>
       </c>
       <c r="Q69" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R69" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S69" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="T69" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U69" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V69" s="1">
         <v>46291</v>
@@ -4401,28 +4404,28 @@
         <v>30</v>
       </c>
       <c r="N70" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="O70" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="P70">
         <v>165000</v>
       </c>
       <c r="Q70" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R70" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S70" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="T70" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U70" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V70" s="1">
         <v>46168</v>
@@ -4445,28 +4448,28 @@
         <v>30</v>
       </c>
       <c r="N71" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="O71" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="P71">
         <v>1000000</v>
       </c>
       <c r="Q71" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R71" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S71" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="T71" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U71" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V71" s="1">
         <v>46291</v>
@@ -4489,28 +4492,28 @@
         <v>30</v>
       </c>
       <c r="N72" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="O72" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="P72">
         <v>1000000</v>
       </c>
       <c r="Q72" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R72" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S72" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="T72" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U72" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V72" s="1">
         <v>46291</v>
@@ -4533,28 +4536,28 @@
         <v>30</v>
       </c>
       <c r="N73" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O73" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="P73">
         <v>100000</v>
       </c>
       <c r="Q73" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="R73" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S73" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="T73" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U73" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V73" s="1">
         <v>46291</v>
@@ -4580,25 +4583,25 @@
         <v>31</v>
       </c>
       <c r="N74" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O74" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="P74">
         <v>1000000</v>
       </c>
       <c r="Q74" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R74" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S74" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T74" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U74" t="s">
         <v>29</v>
@@ -4630,28 +4633,28 @@
         <v>45</v>
       </c>
       <c r="N75" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="O75" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="P75">
         <v>1704503</v>
       </c>
       <c r="Q75" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R75" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S75" t="s">
         <v>41</v>
       </c>
       <c r="T75" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U75" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V75" s="1">
         <v>46381</v>
@@ -4680,28 +4683,28 @@
         <v>45</v>
       </c>
       <c r="N76" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="O76" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="P76">
         <v>1638125.5</v>
       </c>
       <c r="Q76" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R76" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S76" t="s">
         <v>41</v>
       </c>
       <c r="T76" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U76" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V76" s="1">
         <v>46381</v>
@@ -4730,25 +4733,25 @@
         <v>45</v>
       </c>
       <c r="N77" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="O77" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="P77">
         <v>3800000</v>
       </c>
       <c r="Q77" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R77" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S77" t="s">
         <v>41</v>
       </c>
       <c r="T77" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U77" t="s">
         <v>29</v>
@@ -4780,25 +4783,25 @@
         <v>45</v>
       </c>
       <c r="N78" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="O78" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="P78">
         <v>3800000</v>
       </c>
       <c r="Q78" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R78" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S78" t="s">
         <v>41</v>
       </c>
       <c r="T78" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U78" t="s">
         <v>29</v>
@@ -4824,25 +4827,25 @@
         <v>30</v>
       </c>
       <c r="N79" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="O79" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="P79">
         <v>3800000</v>
       </c>
       <c r="Q79" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R79" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S79" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="T79" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U79" t="s">
         <v>29</v>
@@ -4868,25 +4871,25 @@
         <v>29</v>
       </c>
       <c r="N80" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="O80" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="P80">
         <v>4394700</v>
       </c>
       <c r="Q80" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R80" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S80" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="T80" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U80" t="s">
         <v>29</v>
@@ -4915,28 +4918,28 @@
         <v>31</v>
       </c>
       <c r="N81" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="O81" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="P81">
         <v>528395.9300000001</v>
       </c>
       <c r="Q81" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R81" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S81" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T81" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U81" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V81" s="1">
         <v>46382</v>
@@ -4959,25 +4962,25 @@
         <v>30</v>
       </c>
       <c r="N82" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O82" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="P82">
         <v>1000000</v>
       </c>
       <c r="Q82" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R82" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S82" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="T82" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U82" t="s">
         <v>29</v>
@@ -5003,25 +5006,25 @@
         <v>29</v>
       </c>
       <c r="N83" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="O83" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="P83">
         <v>4394700</v>
       </c>
       <c r="Q83" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R83" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S83" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="T83" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U83" t="s">
         <v>29</v>
@@ -5053,25 +5056,25 @@
         <v>45</v>
       </c>
       <c r="N84" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="O84" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="P84">
         <v>3306000</v>
       </c>
       <c r="Q84" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R84" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S84" t="s">
         <v>41</v>
       </c>
       <c r="T84" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U84" t="s">
         <v>29</v>
@@ -5100,25 +5103,25 @@
         <v>45</v>
       </c>
       <c r="N85" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="O85" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="P85">
         <v>3306000</v>
       </c>
       <c r="Q85" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R85" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S85" t="s">
         <v>41</v>
       </c>
       <c r="T85" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U85" t="s">
         <v>29</v>
@@ -5144,25 +5147,25 @@
         <v>31</v>
       </c>
       <c r="N86" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="O86" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="P86">
         <v>212577</v>
       </c>
       <c r="Q86" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R86" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S86" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T86" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="U86" t="s">
         <v>30</v>

</xml_diff>

<commit_message>
Atualização automática: mta (12/08/2026 08:55)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1102" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1102" uniqueCount="174">
   <si>
     <t>linha</t>
   </si>
@@ -188,9 +188,6 @@
   </si>
   <si>
     <t>C26285</t>
-  </si>
-  <si>
-    <t>C26393</t>
   </si>
   <si>
     <t>C26332</t>
@@ -965,31 +962,31 @@
         <v>31</v>
       </c>
       <c r="L2" t="s">
+        <v>71</v>
+      </c>
+      <c r="N2" t="s">
         <v>72</v>
       </c>
-      <c r="N2" t="s">
-        <v>73</v>
-      </c>
       <c r="O2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="P2">
         <v>135000</v>
       </c>
       <c r="Q2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="R2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="S2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U2" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V2" s="1">
         <v>46229</v>
@@ -1015,25 +1012,25 @@
         <v>31</v>
       </c>
       <c r="N3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="P3">
         <v>400000</v>
       </c>
       <c r="Q3" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="R3" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="S3" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U3" t="s">
         <v>29</v>
@@ -1062,25 +1059,25 @@
         <v>31</v>
       </c>
       <c r="N4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="O4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="P4">
         <v>430000</v>
       </c>
       <c r="Q4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="R4" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="S4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T4" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U4" t="s">
         <v>29</v>
@@ -1109,25 +1106,25 @@
         <v>31</v>
       </c>
       <c r="N5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="O5" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="P5">
         <v>425000</v>
       </c>
       <c r="Q5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="R5" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="S5" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T5" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U5" t="s">
         <v>29</v>
@@ -1156,28 +1153,28 @@
         <v>31</v>
       </c>
       <c r="L6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="N6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O6" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="P6">
         <v>563000</v>
       </c>
       <c r="Q6" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="R6" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="S6" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T6" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U6" t="s">
         <v>29</v>
@@ -1215,25 +1212,25 @@
         <v>46</v>
       </c>
       <c r="N7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="O7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="P7">
         <v>3799999.6</v>
       </c>
       <c r="Q7" t="s">
+        <v>160</v>
+      </c>
+      <c r="R7" t="s">
         <v>161</v>
       </c>
-      <c r="R7" t="s">
-        <v>162</v>
-      </c>
       <c r="S7" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T7" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U7" t="s">
         <v>29</v>
@@ -1262,25 +1259,25 @@
         <v>31</v>
       </c>
       <c r="N8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="O8" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="P8">
         <v>430000</v>
       </c>
       <c r="Q8" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="R8" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="S8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T8" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U8" t="s">
         <v>29</v>
@@ -1309,25 +1306,25 @@
         <v>31</v>
       </c>
       <c r="N9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="O9" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="P9">
         <v>60000</v>
       </c>
       <c r="Q9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="R9" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="S9" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T9" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U9" t="s">
         <v>29</v>
@@ -1356,25 +1353,25 @@
         <v>31</v>
       </c>
       <c r="N10" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O10" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="P10">
         <v>200000</v>
       </c>
       <c r="Q10" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="R10" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="S10" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T10" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U10" t="s">
         <v>29</v>
@@ -1403,25 +1400,25 @@
         <v>31</v>
       </c>
       <c r="N11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="P11">
         <v>320000</v>
       </c>
       <c r="Q11" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="R11" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="S11" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T11" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U11" t="s">
         <v>29</v>
@@ -1459,31 +1456,31 @@
         <v>47</v>
       </c>
       <c r="J12" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="N12" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O12" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="P12">
         <v>1187433.02</v>
       </c>
       <c r="Q12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="R12" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="S12" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T12" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U12" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V12" s="1">
         <v>46079</v>
@@ -1509,28 +1506,28 @@
         <v>31</v>
       </c>
       <c r="N13" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O13" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="P13">
         <v>1000000</v>
       </c>
       <c r="Q13" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="R13" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="S13" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T13" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U13" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V13" s="1">
         <v>46352</v>
@@ -1556,28 +1553,28 @@
         <v>31</v>
       </c>
       <c r="N14" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O14" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="P14">
         <v>1000000</v>
       </c>
       <c r="Q14" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="R14" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="S14" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T14" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U14" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V14" s="1">
         <v>46352</v>
@@ -1603,28 +1600,28 @@
         <v>31</v>
       </c>
       <c r="N15" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O15" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="P15">
         <v>1000000</v>
       </c>
       <c r="Q15" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="R15" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="S15" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T15" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U15" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V15" s="1">
         <v>46352</v>
@@ -1650,28 +1647,28 @@
         <v>31</v>
       </c>
       <c r="N16" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="O16" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="P16">
         <v>100000</v>
       </c>
       <c r="Q16" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="R16" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="S16" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T16" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U16" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V16" s="1">
         <v>46229</v>
@@ -1706,31 +1703,31 @@
         <v>48</v>
       </c>
       <c r="J17" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="N17" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="O17" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="P17">
         <v>1770880.5</v>
       </c>
       <c r="Q17" t="s">
+        <v>160</v>
+      </c>
+      <c r="R17" t="s">
         <v>161</v>
       </c>
-      <c r="R17" t="s">
-        <v>162</v>
-      </c>
       <c r="S17" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T17" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="U17" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V17" s="1">
         <v>46107</v>
@@ -1765,25 +1762,25 @@
         <v>49</v>
       </c>
       <c r="N18" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O18" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="P18">
         <v>350000</v>
       </c>
       <c r="Q18" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="R18" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="S18" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T18" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U18" t="s">
         <v>29</v>
@@ -1821,25 +1818,25 @@
         <v>49</v>
       </c>
       <c r="N19" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O19" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="P19">
         <v>350000</v>
       </c>
       <c r="Q19" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="R19" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="S19" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T19" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U19" t="s">
         <v>29</v>
@@ -1868,25 +1865,25 @@
         <v>31</v>
       </c>
       <c r="N20" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="O20" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="P20">
         <v>1000000</v>
       </c>
       <c r="Q20" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="R20" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="S20" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T20" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U20" t="s">
         <v>29</v>
@@ -1915,25 +1912,25 @@
         <v>31</v>
       </c>
       <c r="N21" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O21" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="P21">
         <v>400000</v>
       </c>
       <c r="Q21" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="R21" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="S21" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T21" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U21" t="s">
         <v>29</v>
@@ -1962,25 +1959,25 @@
         <v>31</v>
       </c>
       <c r="N22" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="O22" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="P22">
         <v>120000</v>
       </c>
       <c r="Q22" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="R22" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="S22" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T22" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U22" t="s">
         <v>29</v>
@@ -2009,25 +2006,25 @@
         <v>31</v>
       </c>
       <c r="N23" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="O23" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="P23">
         <v>80000</v>
       </c>
       <c r="Q23" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="R23" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="S23" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T23" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U23" t="s">
         <v>29</v>
@@ -2065,31 +2062,31 @@
         <v>50</v>
       </c>
       <c r="J24" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="N24" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="O24" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="P24">
         <v>1704503</v>
       </c>
       <c r="Q24" t="s">
+        <v>160</v>
+      </c>
+      <c r="R24" t="s">
         <v>161</v>
       </c>
-      <c r="R24" t="s">
-        <v>162</v>
-      </c>
       <c r="S24" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T24" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="U24" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V24" s="1">
         <v>46138</v>
@@ -2124,25 +2121,25 @@
         <v>51</v>
       </c>
       <c r="N25" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O25" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="P25">
         <v>3799000</v>
       </c>
       <c r="Q25" t="s">
+        <v>160</v>
+      </c>
+      <c r="R25" t="s">
         <v>161</v>
       </c>
-      <c r="R25" t="s">
-        <v>162</v>
-      </c>
       <c r="S25" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T25" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U25" t="s">
         <v>29</v>
@@ -2180,25 +2177,25 @@
         <v>52</v>
       </c>
       <c r="N26" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O26" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="P26">
         <v>1000</v>
       </c>
       <c r="Q26" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="R26" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="S26" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T26" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U26" t="s">
         <v>29</v>
@@ -2227,28 +2224,28 @@
         <v>31</v>
       </c>
       <c r="N27" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="O27" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="P27">
         <v>100000</v>
       </c>
       <c r="Q27" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="R27" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="S27" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T27" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U27" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V27" s="1">
         <v>46291</v>
@@ -2283,31 +2280,31 @@
         <v>53</v>
       </c>
       <c r="J28" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="N28" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="O28" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="P28">
         <v>150000</v>
       </c>
       <c r="Q28" t="s">
+        <v>160</v>
+      </c>
+      <c r="R28" t="s">
         <v>161</v>
       </c>
-      <c r="R28" t="s">
-        <v>162</v>
-      </c>
       <c r="S28" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T28" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U28" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V28" s="1">
         <v>46199</v>
@@ -2342,31 +2339,31 @@
         <v>53</v>
       </c>
       <c r="J29" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="N29" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="O29" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="P29">
         <v>150000</v>
       </c>
       <c r="Q29" t="s">
+        <v>160</v>
+      </c>
+      <c r="R29" t="s">
         <v>161</v>
       </c>
-      <c r="R29" t="s">
-        <v>162</v>
-      </c>
       <c r="S29" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T29" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U29" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V29" s="1">
         <v>46199</v>
@@ -2401,31 +2398,31 @@
         <v>54</v>
       </c>
       <c r="J30" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="N30" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="O30" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="P30">
         <v>18462.36</v>
       </c>
       <c r="Q30" t="s">
+        <v>160</v>
+      </c>
+      <c r="R30" t="s">
         <v>161</v>
       </c>
-      <c r="R30" t="s">
-        <v>162</v>
-      </c>
       <c r="S30" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T30" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U30" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V30" s="1">
         <v>46199</v>
@@ -2460,31 +2457,31 @@
         <v>53</v>
       </c>
       <c r="J31" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="N31" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="O31" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="P31">
         <v>324166.14</v>
       </c>
       <c r="Q31" t="s">
+        <v>160</v>
+      </c>
+      <c r="R31" t="s">
         <v>161</v>
       </c>
-      <c r="R31" t="s">
-        <v>162</v>
-      </c>
       <c r="S31" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T31" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U31" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V31" s="1">
         <v>46199</v>
@@ -2510,28 +2507,28 @@
         <v>31</v>
       </c>
       <c r="N32" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="O32" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="P32">
         <v>30000</v>
       </c>
       <c r="Q32" t="s">
+        <v>160</v>
+      </c>
+      <c r="R32" t="s">
         <v>161</v>
       </c>
-      <c r="R32" t="s">
-        <v>162</v>
-      </c>
       <c r="S32" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T32" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U32" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V32" s="1">
         <v>46291</v>
@@ -2566,31 +2563,31 @@
         <v>55</v>
       </c>
       <c r="J33" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="N33" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="O33" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="P33">
         <v>1496713.48</v>
       </c>
       <c r="Q33" t="s">
+        <v>160</v>
+      </c>
+      <c r="R33" t="s">
         <v>161</v>
       </c>
-      <c r="R33" t="s">
-        <v>162</v>
-      </c>
       <c r="S33" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T33" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="U33" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V33" s="1">
         <v>46199</v>
@@ -2625,28 +2622,28 @@
         <v>50</v>
       </c>
       <c r="N34" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="O34" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="P34">
         <v>207789.52</v>
       </c>
       <c r="Q34" t="s">
+        <v>160</v>
+      </c>
+      <c r="R34" t="s">
         <v>161</v>
       </c>
-      <c r="R34" t="s">
-        <v>162</v>
-      </c>
       <c r="S34" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T34" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="U34" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V34" s="1">
         <v>46138</v>
@@ -2681,25 +2678,25 @@
         <v>56</v>
       </c>
       <c r="N35" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O35" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="P35">
         <v>962290.8</v>
       </c>
       <c r="Q35" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="R35" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="S35" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T35" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U35" t="s">
         <v>29</v>
@@ -2737,25 +2734,25 @@
         <v>57</v>
       </c>
       <c r="N36" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O36" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="P36">
         <v>798776.97</v>
       </c>
       <c r="Q36" t="s">
+        <v>160</v>
+      </c>
+      <c r="R36" t="s">
         <v>161</v>
       </c>
-      <c r="R36" t="s">
-        <v>162</v>
-      </c>
       <c r="S36" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T36" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U36" t="s">
         <v>29</v>
@@ -2781,43 +2778,43 @@
         <v>29</v>
       </c>
       <c r="F37" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="G37" t="s">
         <v>42</v>
       </c>
       <c r="H37" s="1">
-        <v>46244</v>
+        <v>46213</v>
       </c>
       <c r="I37" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="N37" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O37" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="P37">
-        <v>1223.03</v>
+        <v>1530656.62</v>
       </c>
       <c r="Q37" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="R37" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="S37" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T37" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U37" t="s">
         <v>29</v>
       </c>
       <c r="V37" s="1">
-        <v>46199</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="38" spans="1:22">
@@ -2846,28 +2843,28 @@
         <v>46199</v>
       </c>
       <c r="I38" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="N38" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O38" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="P38">
         <v>72958.08</v>
       </c>
       <c r="Q38" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="R38" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="S38" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T38" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U38" t="s">
         <v>29</v>
@@ -2902,28 +2899,28 @@
         <v>46199</v>
       </c>
       <c r="I39" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="N39" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O39" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="P39">
         <v>8916</v>
       </c>
       <c r="Q39" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="R39" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="S39" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T39" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U39" t="s">
         <v>29</v>
@@ -2958,28 +2955,28 @@
         <v>46204</v>
       </c>
       <c r="I40" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="N40" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O40" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="P40">
         <v>425178.5</v>
       </c>
       <c r="Q40" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="R40" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="S40" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T40" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U40" t="s">
         <v>29</v>
@@ -3008,22 +3005,22 @@
         <v>43</v>
       </c>
       <c r="N41" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O41" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="Q41" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="R41" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="S41" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="T41" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U41" t="s">
         <v>29</v>
@@ -3058,28 +3055,28 @@
         <v>46191</v>
       </c>
       <c r="I42" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="N42" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O42" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="P42">
         <v>400000</v>
       </c>
       <c r="Q42" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="R42" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="S42" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T42" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U42" t="s">
         <v>29</v>
@@ -3114,28 +3111,28 @@
         <v>46191</v>
       </c>
       <c r="I43" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="N43" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O43" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="P43">
         <v>400000</v>
       </c>
       <c r="Q43" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="R43" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="S43" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T43" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U43" t="s">
         <v>29</v>
@@ -3173,31 +3170,31 @@
         <v>55</v>
       </c>
       <c r="J44" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="N44" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="O44" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="P44">
         <v>173846.38</v>
       </c>
       <c r="Q44" t="s">
+        <v>160</v>
+      </c>
+      <c r="R44" t="s">
         <v>161</v>
       </c>
-      <c r="R44" t="s">
-        <v>162</v>
-      </c>
       <c r="S44" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T44" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="U44" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V44" s="1">
         <v>46229</v>
@@ -3232,28 +3229,28 @@
         <v>54</v>
       </c>
       <c r="N45" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="O45" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="P45">
         <v>1530656.62</v>
       </c>
       <c r="Q45" t="s">
+        <v>160</v>
+      </c>
+      <c r="R45" t="s">
         <v>161</v>
       </c>
-      <c r="R45" t="s">
-        <v>162</v>
-      </c>
       <c r="S45" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T45" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="U45" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V45" s="1">
         <v>46229</v>
@@ -3279,25 +3276,25 @@
         <v>31</v>
       </c>
       <c r="N46" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="O46" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="P46">
         <v>1000000</v>
       </c>
       <c r="Q46" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="R46" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="S46" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T46" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U46" t="s">
         <v>29</v>
@@ -3326,28 +3323,28 @@
         <v>31</v>
       </c>
       <c r="N47" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O47" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="P47">
         <v>958040</v>
       </c>
       <c r="Q47" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="R47" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="S47" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T47" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U47" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V47" s="1">
         <v>46291</v>
@@ -3379,34 +3376,34 @@
         <v>46176</v>
       </c>
       <c r="I48" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J48" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="N48" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O48" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="P48">
         <v>41730.64</v>
       </c>
       <c r="Q48" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="R48" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="S48" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T48" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U48" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V48" s="1">
         <v>46199</v>
@@ -3432,34 +3429,34 @@
         <v>31</v>
       </c>
       <c r="J49" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="K49" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="N49" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="O49" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="P49">
         <v>1468159.32</v>
       </c>
       <c r="Q49" t="s">
+        <v>160</v>
+      </c>
+      <c r="R49" t="s">
         <v>161</v>
       </c>
-      <c r="R49" t="s">
-        <v>162</v>
-      </c>
       <c r="S49" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T49" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="U49" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V49" s="1">
         <v>46260</v>
@@ -3485,34 +3482,34 @@
         <v>31</v>
       </c>
       <c r="J50" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="K50" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="N50" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="O50" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="P50">
         <v>1704503</v>
       </c>
       <c r="Q50" t="s">
+        <v>160</v>
+      </c>
+      <c r="R50" t="s">
         <v>161</v>
       </c>
-      <c r="R50" t="s">
-        <v>162</v>
-      </c>
       <c r="S50" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T50" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="U50" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V50" s="1">
         <v>46291</v>
@@ -3538,31 +3535,31 @@
         <v>31</v>
       </c>
       <c r="K51" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="N51" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="O51" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="P51">
         <v>1704503</v>
       </c>
       <c r="Q51" t="s">
+        <v>160</v>
+      </c>
+      <c r="R51" t="s">
         <v>161</v>
       </c>
-      <c r="R51" t="s">
-        <v>162</v>
-      </c>
       <c r="S51" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T51" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="U51" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V51" s="1">
         <v>46321</v>
@@ -3594,31 +3591,31 @@
         <v>46227</v>
       </c>
       <c r="I52" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="N52" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="O52" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="P52">
         <v>236343.68</v>
       </c>
       <c r="Q52" t="s">
+        <v>160</v>
+      </c>
+      <c r="R52" t="s">
         <v>161</v>
       </c>
-      <c r="R52" t="s">
-        <v>162</v>
-      </c>
       <c r="S52" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T52" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="U52" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V52" s="1">
         <v>46229</v>
@@ -3644,28 +3641,28 @@
         <v>31</v>
       </c>
       <c r="N53" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="O53" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="P53">
         <v>1295422.28</v>
       </c>
       <c r="Q53" t="s">
+        <v>160</v>
+      </c>
+      <c r="R53" t="s">
         <v>161</v>
       </c>
-      <c r="R53" t="s">
-        <v>162</v>
-      </c>
       <c r="S53" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T53" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="U53" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V53" s="1">
         <v>46352</v>
@@ -3691,31 +3688,31 @@
         <v>40</v>
       </c>
       <c r="K54" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="N54" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O54" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="P54">
         <v>500000</v>
       </c>
       <c r="Q54" t="s">
+        <v>160</v>
+      </c>
+      <c r="R54" t="s">
         <v>161</v>
       </c>
-      <c r="R54" t="s">
-        <v>162</v>
-      </c>
       <c r="S54" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="T54" t="s">
+        <v>172</v>
+      </c>
+      <c r="U54" t="s">
         <v>173</v>
-      </c>
-      <c r="U54" t="s">
-        <v>174</v>
       </c>
       <c r="V54" s="1">
         <v>46321</v>
@@ -3744,28 +3741,28 @@
         <v>44</v>
       </c>
       <c r="N55" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O55" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="P55">
         <v>5000000</v>
       </c>
       <c r="Q55" t="s">
+        <v>160</v>
+      </c>
+      <c r="R55" t="s">
         <v>161</v>
       </c>
-      <c r="R55" t="s">
-        <v>162</v>
-      </c>
       <c r="S55" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="T55" t="s">
+        <v>172</v>
+      </c>
+      <c r="U55" t="s">
         <v>173</v>
-      </c>
-      <c r="U55" t="s">
-        <v>174</v>
       </c>
       <c r="V55" s="1">
         <v>46321</v>
@@ -3791,25 +3788,25 @@
         <v>43</v>
       </c>
       <c r="N56" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O56" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Q56" t="s">
+        <v>160</v>
+      </c>
+      <c r="R56" t="s">
         <v>161</v>
       </c>
-      <c r="R56" t="s">
-        <v>162</v>
-      </c>
       <c r="S56" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="T56" t="s">
+        <v>172</v>
+      </c>
+      <c r="U56" t="s">
         <v>173</v>
-      </c>
-      <c r="U56" t="s">
-        <v>174</v>
       </c>
       <c r="V56" s="1">
         <v>46049</v>
@@ -3835,25 +3832,25 @@
         <v>43</v>
       </c>
       <c r="N57" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O57" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="Q57" t="s">
+        <v>160</v>
+      </c>
+      <c r="R57" t="s">
         <v>161</v>
       </c>
-      <c r="R57" t="s">
-        <v>162</v>
-      </c>
       <c r="S57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="T57" t="s">
+        <v>172</v>
+      </c>
+      <c r="U57" t="s">
         <v>173</v>
-      </c>
-      <c r="U57" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="58" spans="1:22">
@@ -3876,25 +3873,25 @@
         <v>43</v>
       </c>
       <c r="N58" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O58" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="Q58" t="s">
+        <v>160</v>
+      </c>
+      <c r="R58" t="s">
         <v>161</v>
       </c>
-      <c r="R58" t="s">
-        <v>162</v>
-      </c>
       <c r="S58" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="T58" t="s">
+        <v>172</v>
+      </c>
+      <c r="U58" t="s">
         <v>173</v>
-      </c>
-      <c r="U58" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="59" spans="1:22">
@@ -3914,28 +3911,28 @@
         <v>30</v>
       </c>
       <c r="N59" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="O59" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="P59">
         <v>9389.959999999999</v>
       </c>
       <c r="Q59" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="R59" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="S59" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="T59" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U59" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V59" s="1">
         <v>46107</v>
@@ -3958,28 +3955,28 @@
         <v>30</v>
       </c>
       <c r="N60" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O60" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="P60">
         <v>7204.82</v>
       </c>
       <c r="Q60" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="R60" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="S60" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="T60" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U60" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V60" s="1">
         <v>46107</v>
@@ -4002,28 +3999,28 @@
         <v>30</v>
       </c>
       <c r="N61" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="O61" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="P61">
         <v>4227.84</v>
       </c>
       <c r="Q61" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="R61" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="S61" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="T61" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U61" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V61" s="1">
         <v>46107</v>
@@ -4046,28 +4043,28 @@
         <v>30</v>
       </c>
       <c r="N62" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="O62" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="P62">
         <v>4064.54</v>
       </c>
       <c r="Q62" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="R62" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="S62" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="T62" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U62" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V62" s="1">
         <v>46107</v>
@@ -4090,28 +4087,28 @@
         <v>30</v>
       </c>
       <c r="N63" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O63" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="P63">
         <v>3662.66</v>
       </c>
       <c r="Q63" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="R63" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="S63" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="T63" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U63" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V63" s="1">
         <v>46107</v>
@@ -4134,28 +4131,28 @@
         <v>30</v>
       </c>
       <c r="N64" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="O64" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P64">
         <v>1163.64</v>
       </c>
       <c r="Q64" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="R64" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="S64" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="T64" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U64" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V64" s="1">
         <v>46107</v>
@@ -4178,25 +4175,25 @@
         <v>30</v>
       </c>
       <c r="N65" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="O65" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="P65">
         <v>120000</v>
       </c>
       <c r="Q65" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="R65" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="S65" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="T65" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U65" t="s">
         <v>29</v>
@@ -4225,25 +4222,25 @@
         <v>31</v>
       </c>
       <c r="N66" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O66" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="P66">
         <v>400000</v>
       </c>
       <c r="Q66" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="R66" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="S66" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T66" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U66" t="s">
         <v>29</v>
@@ -4272,28 +4269,28 @@
         <v>31</v>
       </c>
       <c r="N67" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="O67" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="P67">
         <v>100000</v>
       </c>
       <c r="Q67" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="R67" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="S67" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T67" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U67" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V67" s="1">
         <v>46229</v>
@@ -4316,25 +4313,25 @@
         <v>30</v>
       </c>
       <c r="N68" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="O68" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="P68">
         <v>80000</v>
       </c>
       <c r="Q68" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="R68" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="S68" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="T68" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U68" t="s">
         <v>29</v>
@@ -4360,28 +4357,28 @@
         <v>30</v>
       </c>
       <c r="N69" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O69" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="P69">
         <v>835000</v>
       </c>
       <c r="Q69" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="R69" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="S69" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="T69" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U69" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V69" s="1">
         <v>46291</v>
@@ -4404,28 +4401,28 @@
         <v>30</v>
       </c>
       <c r="N70" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O70" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="P70">
         <v>165000</v>
       </c>
       <c r="Q70" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="R70" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="S70" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="T70" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U70" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V70" s="1">
         <v>46168</v>
@@ -4448,28 +4445,28 @@
         <v>30</v>
       </c>
       <c r="N71" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O71" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="P71">
         <v>1000000</v>
       </c>
       <c r="Q71" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="R71" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="S71" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="T71" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U71" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V71" s="1">
         <v>46291</v>
@@ -4492,28 +4489,28 @@
         <v>30</v>
       </c>
       <c r="N72" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O72" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="P72">
         <v>1000000</v>
       </c>
       <c r="Q72" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="R72" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="S72" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="T72" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U72" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V72" s="1">
         <v>46291</v>
@@ -4536,28 +4533,28 @@
         <v>30</v>
       </c>
       <c r="N73" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="O73" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="P73">
         <v>100000</v>
       </c>
       <c r="Q73" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="R73" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="S73" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="T73" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U73" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V73" s="1">
         <v>46291</v>
@@ -4583,25 +4580,25 @@
         <v>31</v>
       </c>
       <c r="N74" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="O74" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="P74">
         <v>1000000</v>
       </c>
       <c r="Q74" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="R74" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="S74" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T74" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U74" t="s">
         <v>29</v>
@@ -4633,28 +4630,28 @@
         <v>45</v>
       </c>
       <c r="N75" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="O75" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="P75">
         <v>1704503</v>
       </c>
       <c r="Q75" t="s">
+        <v>160</v>
+      </c>
+      <c r="R75" t="s">
         <v>161</v>
-      </c>
-      <c r="R75" t="s">
-        <v>162</v>
       </c>
       <c r="S75" t="s">
         <v>41</v>
       </c>
       <c r="T75" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="U75" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V75" s="1">
         <v>46381</v>
@@ -4683,28 +4680,28 @@
         <v>45</v>
       </c>
       <c r="N76" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="O76" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="P76">
         <v>1638125.5</v>
       </c>
       <c r="Q76" t="s">
+        <v>160</v>
+      </c>
+      <c r="R76" t="s">
         <v>161</v>
-      </c>
-      <c r="R76" t="s">
-        <v>162</v>
       </c>
       <c r="S76" t="s">
         <v>41</v>
       </c>
       <c r="T76" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="U76" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V76" s="1">
         <v>46381</v>
@@ -4733,25 +4730,25 @@
         <v>45</v>
       </c>
       <c r="N77" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="O77" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="P77">
         <v>3800000</v>
       </c>
       <c r="Q77" t="s">
+        <v>160</v>
+      </c>
+      <c r="R77" t="s">
         <v>161</v>
-      </c>
-      <c r="R77" t="s">
-        <v>162</v>
       </c>
       <c r="S77" t="s">
         <v>41</v>
       </c>
       <c r="T77" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U77" t="s">
         <v>29</v>
@@ -4783,25 +4780,25 @@
         <v>45</v>
       </c>
       <c r="N78" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="O78" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="P78">
         <v>3800000</v>
       </c>
       <c r="Q78" t="s">
+        <v>160</v>
+      </c>
+      <c r="R78" t="s">
         <v>161</v>
-      </c>
-      <c r="R78" t="s">
-        <v>162</v>
       </c>
       <c r="S78" t="s">
         <v>41</v>
       </c>
       <c r="T78" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U78" t="s">
         <v>29</v>
@@ -4827,25 +4824,25 @@
         <v>30</v>
       </c>
       <c r="N79" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O79" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="P79">
         <v>3800000</v>
       </c>
       <c r="Q79" t="s">
+        <v>160</v>
+      </c>
+      <c r="R79" t="s">
         <v>161</v>
       </c>
-      <c r="R79" t="s">
-        <v>162</v>
-      </c>
       <c r="S79" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="T79" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U79" t="s">
         <v>29</v>
@@ -4871,25 +4868,25 @@
         <v>29</v>
       </c>
       <c r="N80" t="s">
+        <v>88</v>
+      </c>
+      <c r="O80" t="s">
         <v>89</v>
-      </c>
-      <c r="O80" t="s">
-        <v>90</v>
       </c>
       <c r="P80">
         <v>4394700</v>
       </c>
       <c r="Q80" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="R80" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="S80" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="T80" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U80" t="s">
         <v>29</v>
@@ -4918,28 +4915,28 @@
         <v>31</v>
       </c>
       <c r="N81" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="O81" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="P81">
         <v>528395.9300000001</v>
       </c>
       <c r="Q81" t="s">
+        <v>160</v>
+      </c>
+      <c r="R81" t="s">
         <v>161</v>
       </c>
-      <c r="R81" t="s">
-        <v>162</v>
-      </c>
       <c r="S81" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T81" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="U81" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V81" s="1">
         <v>46382</v>
@@ -4962,25 +4959,25 @@
         <v>30</v>
       </c>
       <c r="N82" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="O82" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="P82">
         <v>1000000</v>
       </c>
       <c r="Q82" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="R82" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="S82" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="T82" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U82" t="s">
         <v>29</v>
@@ -5006,25 +5003,25 @@
         <v>29</v>
       </c>
       <c r="N83" t="s">
+        <v>88</v>
+      </c>
+      <c r="O83" t="s">
         <v>89</v>
-      </c>
-      <c r="O83" t="s">
-        <v>90</v>
       </c>
       <c r="P83">
         <v>4394700</v>
       </c>
       <c r="Q83" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="R83" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="S83" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="T83" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U83" t="s">
         <v>29</v>
@@ -5056,25 +5053,25 @@
         <v>45</v>
       </c>
       <c r="N84" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="O84" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="P84">
         <v>3306000</v>
       </c>
       <c r="Q84" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="R84" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="S84" t="s">
         <v>41</v>
       </c>
       <c r="T84" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U84" t="s">
         <v>29</v>
@@ -5103,25 +5100,25 @@
         <v>45</v>
       </c>
       <c r="N85" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="O85" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="P85">
         <v>3306000</v>
       </c>
       <c r="Q85" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="R85" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="S85" t="s">
         <v>41</v>
       </c>
       <c r="T85" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U85" t="s">
         <v>29</v>
@@ -5147,25 +5144,25 @@
         <v>31</v>
       </c>
       <c r="N86" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="O86" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="P86">
         <v>212577</v>
       </c>
       <c r="Q86" t="s">
+        <v>160</v>
+      </c>
+      <c r="R86" t="s">
         <v>161</v>
       </c>
-      <c r="R86" t="s">
-        <v>162</v>
-      </c>
       <c r="S86" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T86" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="U86" t="s">
         <v>30</v>

</xml_diff>

<commit_message>
Atualização automática: mta (17/08/2026 08:34)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -970,9 +970,6 @@
       <c r="O2" t="s">
         <v>91</v>
       </c>
-      <c r="P2">
-        <v>135000</v>
-      </c>
       <c r="Q2" t="s">
         <v>158</v>
       </c>
@@ -1017,9 +1014,6 @@
       <c r="O3" t="s">
         <v>92</v>
       </c>
-      <c r="P3">
-        <v>400000</v>
-      </c>
       <c r="Q3" t="s">
         <v>159</v>
       </c>
@@ -1064,9 +1058,6 @@
       <c r="O4" t="s">
         <v>93</v>
       </c>
-      <c r="P4">
-        <v>430000</v>
-      </c>
       <c r="Q4" t="s">
         <v>158</v>
       </c>
@@ -1111,9 +1102,6 @@
       <c r="O5" t="s">
         <v>94</v>
       </c>
-      <c r="P5">
-        <v>425000</v>
-      </c>
       <c r="Q5" t="s">
         <v>158</v>
       </c>
@@ -1161,9 +1149,6 @@
       <c r="O6" t="s">
         <v>95</v>
       </c>
-      <c r="P6">
-        <v>563000</v>
-      </c>
       <c r="Q6" t="s">
         <v>158</v>
       </c>
@@ -1217,9 +1202,6 @@
       <c r="O7" t="s">
         <v>96</v>
       </c>
-      <c r="P7">
-        <v>3799999.6</v>
-      </c>
       <c r="Q7" t="s">
         <v>160</v>
       </c>
@@ -1264,9 +1246,6 @@
       <c r="O8" t="s">
         <v>97</v>
       </c>
-      <c r="P8">
-        <v>430000</v>
-      </c>
       <c r="Q8" t="s">
         <v>158</v>
       </c>
@@ -1311,9 +1290,6 @@
       <c r="O9" t="s">
         <v>98</v>
       </c>
-      <c r="P9">
-        <v>60000</v>
-      </c>
       <c r="Q9" t="s">
         <v>158</v>
       </c>
@@ -1358,9 +1334,6 @@
       <c r="O10" t="s">
         <v>99</v>
       </c>
-      <c r="P10">
-        <v>200000</v>
-      </c>
       <c r="Q10" t="s">
         <v>158</v>
       </c>
@@ -1405,9 +1378,6 @@
       <c r="O11" t="s">
         <v>100</v>
       </c>
-      <c r="P11">
-        <v>320000</v>
-      </c>
       <c r="Q11" t="s">
         <v>158</v>
       </c>
@@ -1464,9 +1434,6 @@
       <c r="O12" t="s">
         <v>101</v>
       </c>
-      <c r="P12">
-        <v>1187433.02</v>
-      </c>
       <c r="Q12" t="s">
         <v>158</v>
       </c>
@@ -1511,9 +1478,6 @@
       <c r="O13" t="s">
         <v>102</v>
       </c>
-      <c r="P13">
-        <v>1000000</v>
-      </c>
       <c r="Q13" t="s">
         <v>158</v>
       </c>
@@ -1558,9 +1522,6 @@
       <c r="O14" t="s">
         <v>103</v>
       </c>
-      <c r="P14">
-        <v>1000000</v>
-      </c>
       <c r="Q14" t="s">
         <v>158</v>
       </c>
@@ -1605,9 +1566,6 @@
       <c r="O15" t="s">
         <v>104</v>
       </c>
-      <c r="P15">
-        <v>1000000</v>
-      </c>
       <c r="Q15" t="s">
         <v>158</v>
       </c>
@@ -1652,9 +1610,6 @@
       <c r="O16" t="s">
         <v>105</v>
       </c>
-      <c r="P16">
-        <v>100000</v>
-      </c>
       <c r="Q16" t="s">
         <v>159</v>
       </c>
@@ -1711,9 +1666,6 @@
       <c r="O17" t="s">
         <v>106</v>
       </c>
-      <c r="P17">
-        <v>1770880.5</v>
-      </c>
       <c r="Q17" t="s">
         <v>160</v>
       </c>
@@ -1767,9 +1719,6 @@
       <c r="O18" t="s">
         <v>107</v>
       </c>
-      <c r="P18">
-        <v>350000</v>
-      </c>
       <c r="Q18" t="s">
         <v>160</v>
       </c>
@@ -1823,9 +1772,6 @@
       <c r="O19" t="s">
         <v>108</v>
       </c>
-      <c r="P19">
-        <v>350000</v>
-      </c>
       <c r="Q19" t="s">
         <v>160</v>
       </c>
@@ -1870,9 +1816,6 @@
       <c r="O20" t="s">
         <v>109</v>
       </c>
-      <c r="P20">
-        <v>1000000</v>
-      </c>
       <c r="Q20" t="s">
         <v>160</v>
       </c>
@@ -1917,9 +1860,6 @@
       <c r="O21" t="s">
         <v>110</v>
       </c>
-      <c r="P21">
-        <v>400000</v>
-      </c>
       <c r="Q21" t="s">
         <v>159</v>
       </c>
@@ -1964,9 +1904,6 @@
       <c r="O22" t="s">
         <v>111</v>
       </c>
-      <c r="P22">
-        <v>120000</v>
-      </c>
       <c r="Q22" t="s">
         <v>158</v>
       </c>
@@ -2011,9 +1948,6 @@
       <c r="O23" t="s">
         <v>112</v>
       </c>
-      <c r="P23">
-        <v>80000</v>
-      </c>
       <c r="Q23" t="s">
         <v>158</v>
       </c>
@@ -2070,9 +2004,6 @@
       <c r="O24" t="s">
         <v>113</v>
       </c>
-      <c r="P24">
-        <v>1704503</v>
-      </c>
       <c r="Q24" t="s">
         <v>160</v>
       </c>
@@ -2126,9 +2057,6 @@
       <c r="O25" t="s">
         <v>114</v>
       </c>
-      <c r="P25">
-        <v>3799000</v>
-      </c>
       <c r="Q25" t="s">
         <v>160</v>
       </c>
@@ -2182,9 +2110,6 @@
       <c r="O26" t="s">
         <v>114</v>
       </c>
-      <c r="P26">
-        <v>1000</v>
-      </c>
       <c r="Q26" t="s">
         <v>160</v>
       </c>
@@ -2229,9 +2154,6 @@
       <c r="O27" t="s">
         <v>115</v>
       </c>
-      <c r="P27">
-        <v>100000</v>
-      </c>
       <c r="Q27" t="s">
         <v>159</v>
       </c>
@@ -2288,9 +2210,6 @@
       <c r="O28" t="s">
         <v>116</v>
       </c>
-      <c r="P28">
-        <v>150000</v>
-      </c>
       <c r="Q28" t="s">
         <v>160</v>
       </c>
@@ -2347,9 +2266,6 @@
       <c r="O29" t="s">
         <v>117</v>
       </c>
-      <c r="P29">
-        <v>150000</v>
-      </c>
       <c r="Q29" t="s">
         <v>160</v>
       </c>
@@ -2406,9 +2322,6 @@
       <c r="O30" t="s">
         <v>118</v>
       </c>
-      <c r="P30">
-        <v>18462.36</v>
-      </c>
       <c r="Q30" t="s">
         <v>160</v>
       </c>
@@ -2465,9 +2378,6 @@
       <c r="O31" t="s">
         <v>118</v>
       </c>
-      <c r="P31">
-        <v>324166.14</v>
-      </c>
       <c r="Q31" t="s">
         <v>160</v>
       </c>
@@ -2512,9 +2422,6 @@
       <c r="O32" t="s">
         <v>119</v>
       </c>
-      <c r="P32">
-        <v>30000</v>
-      </c>
       <c r="Q32" t="s">
         <v>160</v>
       </c>
@@ -2571,9 +2478,6 @@
       <c r="O33" t="s">
         <v>120</v>
       </c>
-      <c r="P33">
-        <v>1496713.48</v>
-      </c>
       <c r="Q33" t="s">
         <v>160</v>
       </c>
@@ -2627,9 +2531,6 @@
       <c r="O34" t="s">
         <v>120</v>
       </c>
-      <c r="P34">
-        <v>207789.52</v>
-      </c>
       <c r="Q34" t="s">
         <v>160</v>
       </c>
@@ -2683,9 +2584,6 @@
       <c r="O35" t="s">
         <v>121</v>
       </c>
-      <c r="P35">
-        <v>962290.8</v>
-      </c>
       <c r="Q35" t="s">
         <v>160</v>
       </c>
@@ -2739,9 +2637,6 @@
       <c r="O36" t="s">
         <v>121</v>
       </c>
-      <c r="P36">
-        <v>798776.97</v>
-      </c>
       <c r="Q36" t="s">
         <v>160</v>
       </c>
@@ -2795,9 +2690,6 @@
       <c r="O37" t="s">
         <v>121</v>
       </c>
-      <c r="P37">
-        <v>1530656.62</v>
-      </c>
       <c r="Q37" t="s">
         <v>160</v>
       </c>
@@ -2851,9 +2743,6 @@
       <c r="O38" t="s">
         <v>121</v>
       </c>
-      <c r="P38">
-        <v>72958.08</v>
-      </c>
       <c r="Q38" t="s">
         <v>160</v>
       </c>
@@ -2907,9 +2796,6 @@
       <c r="O39" t="s">
         <v>121</v>
       </c>
-      <c r="P39">
-        <v>8916</v>
-      </c>
       <c r="Q39" t="s">
         <v>160</v>
       </c>
@@ -2963,9 +2849,6 @@
       <c r="O40" t="s">
         <v>121</v>
       </c>
-      <c r="P40">
-        <v>425178.5</v>
-      </c>
       <c r="Q40" t="s">
         <v>160</v>
       </c>
@@ -3063,9 +2946,6 @@
       <c r="O42" t="s">
         <v>123</v>
       </c>
-      <c r="P42">
-        <v>400000</v>
-      </c>
       <c r="Q42" t="s">
         <v>160</v>
       </c>
@@ -3119,9 +2999,6 @@
       <c r="O43" t="s">
         <v>124</v>
       </c>
-      <c r="P43">
-        <v>400000</v>
-      </c>
       <c r="Q43" t="s">
         <v>160</v>
       </c>
@@ -3178,9 +3055,6 @@
       <c r="O44" t="s">
         <v>125</v>
       </c>
-      <c r="P44">
-        <v>173846.38</v>
-      </c>
       <c r="Q44" t="s">
         <v>160</v>
       </c>
@@ -3234,9 +3108,6 @@
       <c r="O45" t="s">
         <v>125</v>
       </c>
-      <c r="P45">
-        <v>1530656.62</v>
-      </c>
       <c r="Q45" t="s">
         <v>160</v>
       </c>
@@ -3281,9 +3152,6 @@
       <c r="O46" t="s">
         <v>126</v>
       </c>
-      <c r="P46">
-        <v>1000000</v>
-      </c>
       <c r="Q46" t="s">
         <v>160</v>
       </c>
@@ -3328,9 +3196,6 @@
       <c r="O47" t="s">
         <v>127</v>
       </c>
-      <c r="P47">
-        <v>958040</v>
-      </c>
       <c r="Q47" t="s">
         <v>158</v>
       </c>
@@ -3387,9 +3252,6 @@
       <c r="O48" t="s">
         <v>127</v>
       </c>
-      <c r="P48">
-        <v>41730.64</v>
-      </c>
       <c r="Q48" t="s">
         <v>158</v>
       </c>
@@ -3440,9 +3302,6 @@
       <c r="O49" t="s">
         <v>128</v>
       </c>
-      <c r="P49">
-        <v>1468159.32</v>
-      </c>
       <c r="Q49" t="s">
         <v>160</v>
       </c>
@@ -3493,9 +3352,6 @@
       <c r="O50" t="s">
         <v>129</v>
       </c>
-      <c r="P50">
-        <v>1704503</v>
-      </c>
       <c r="Q50" t="s">
         <v>160</v>
       </c>
@@ -3543,9 +3399,6 @@
       <c r="O51" t="s">
         <v>130</v>
       </c>
-      <c r="P51">
-        <v>1704503</v>
-      </c>
       <c r="Q51" t="s">
         <v>160</v>
       </c>
@@ -3599,9 +3452,6 @@
       <c r="O52" t="s">
         <v>128</v>
       </c>
-      <c r="P52">
-        <v>236343.68</v>
-      </c>
       <c r="Q52" t="s">
         <v>160</v>
       </c>
@@ -3646,9 +3496,6 @@
       <c r="O53" t="s">
         <v>131</v>
       </c>
-      <c r="P53">
-        <v>1295422.28</v>
-      </c>
       <c r="Q53" t="s">
         <v>160</v>
       </c>
@@ -3696,9 +3543,6 @@
       <c r="O54" t="s">
         <v>132</v>
       </c>
-      <c r="P54">
-        <v>500000</v>
-      </c>
       <c r="Q54" t="s">
         <v>160</v>
       </c>
@@ -3746,9 +3590,6 @@
       <c r="O55" t="s">
         <v>132</v>
       </c>
-      <c r="P55">
-        <v>5000000</v>
-      </c>
       <c r="Q55" t="s">
         <v>160</v>
       </c>
@@ -3916,9 +3757,6 @@
       <c r="O59" t="s">
         <v>136</v>
       </c>
-      <c r="P59">
-        <v>9389.959999999999</v>
-      </c>
       <c r="Q59" t="s">
         <v>158</v>
       </c>
@@ -3960,9 +3798,6 @@
       <c r="O60" t="s">
         <v>137</v>
       </c>
-      <c r="P60">
-        <v>7204.82</v>
-      </c>
       <c r="Q60" t="s">
         <v>158</v>
       </c>
@@ -4004,9 +3839,6 @@
       <c r="O61" t="s">
         <v>138</v>
       </c>
-      <c r="P61">
-        <v>4227.84</v>
-      </c>
       <c r="Q61" t="s">
         <v>158</v>
       </c>
@@ -4048,9 +3880,6 @@
       <c r="O62" t="s">
         <v>139</v>
       </c>
-      <c r="P62">
-        <v>4064.54</v>
-      </c>
       <c r="Q62" t="s">
         <v>160</v>
       </c>
@@ -4092,9 +3921,6 @@
       <c r="O63" t="s">
         <v>138</v>
       </c>
-      <c r="P63">
-        <v>3662.66</v>
-      </c>
       <c r="Q63" t="s">
         <v>158</v>
       </c>
@@ -4136,9 +3962,6 @@
       <c r="O64" t="s">
         <v>140</v>
       </c>
-      <c r="P64">
-        <v>1163.64</v>
-      </c>
       <c r="Q64" t="s">
         <v>159</v>
       </c>
@@ -4180,9 +4003,6 @@
       <c r="O65" t="s">
         <v>141</v>
       </c>
-      <c r="P65">
-        <v>120000</v>
-      </c>
       <c r="Q65" t="s">
         <v>158</v>
       </c>
@@ -4227,9 +4047,6 @@
       <c r="O66" t="s">
         <v>142</v>
       </c>
-      <c r="P66">
-        <v>400000</v>
-      </c>
       <c r="Q66" t="s">
         <v>159</v>
       </c>
@@ -4274,9 +4091,6 @@
       <c r="O67" t="s">
         <v>143</v>
       </c>
-      <c r="P67">
-        <v>100000</v>
-      </c>
       <c r="Q67" t="s">
         <v>159</v>
       </c>
@@ -4318,9 +4132,6 @@
       <c r="O68" t="s">
         <v>144</v>
       </c>
-      <c r="P68">
-        <v>80000</v>
-      </c>
       <c r="Q68" t="s">
         <v>158</v>
       </c>
@@ -4362,9 +4173,6 @@
       <c r="O69" t="s">
         <v>145</v>
       </c>
-      <c r="P69">
-        <v>835000</v>
-      </c>
       <c r="Q69" t="s">
         <v>158</v>
       </c>
@@ -4406,9 +4214,6 @@
       <c r="O70" t="s">
         <v>145</v>
       </c>
-      <c r="P70">
-        <v>165000</v>
-      </c>
       <c r="Q70" t="s">
         <v>158</v>
       </c>
@@ -4450,9 +4255,6 @@
       <c r="O71" t="s">
         <v>146</v>
       </c>
-      <c r="P71">
-        <v>1000000</v>
-      </c>
       <c r="Q71" t="s">
         <v>158</v>
       </c>
@@ -4494,9 +4296,6 @@
       <c r="O72" t="s">
         <v>147</v>
       </c>
-      <c r="P72">
-        <v>1000000</v>
-      </c>
       <c r="Q72" t="s">
         <v>158</v>
       </c>
@@ -4538,9 +4337,6 @@
       <c r="O73" t="s">
         <v>148</v>
       </c>
-      <c r="P73">
-        <v>100000</v>
-      </c>
       <c r="Q73" t="s">
         <v>159</v>
       </c>
@@ -4585,9 +4381,6 @@
       <c r="O74" t="s">
         <v>149</v>
       </c>
-      <c r="P74">
-        <v>1000000</v>
-      </c>
       <c r="Q74" t="s">
         <v>160</v>
       </c>
@@ -4635,9 +4428,6 @@
       <c r="O75" t="s">
         <v>150</v>
       </c>
-      <c r="P75">
-        <v>1704503</v>
-      </c>
       <c r="Q75" t="s">
         <v>160</v>
       </c>
@@ -4685,9 +4475,6 @@
       <c r="O76" t="s">
         <v>151</v>
       </c>
-      <c r="P76">
-        <v>1638125.5</v>
-      </c>
       <c r="Q76" t="s">
         <v>160</v>
       </c>
@@ -4735,9 +4522,6 @@
       <c r="O77" t="s">
         <v>152</v>
       </c>
-      <c r="P77">
-        <v>3800000</v>
-      </c>
       <c r="Q77" t="s">
         <v>160</v>
       </c>
@@ -4785,9 +4569,6 @@
       <c r="O78" t="s">
         <v>153</v>
       </c>
-      <c r="P78">
-        <v>3800000</v>
-      </c>
       <c r="Q78" t="s">
         <v>160</v>
       </c>
@@ -4829,9 +4610,6 @@
       <c r="O79" t="s">
         <v>154</v>
       </c>
-      <c r="P79">
-        <v>3800000</v>
-      </c>
       <c r="Q79" t="s">
         <v>160</v>
       </c>
@@ -4873,9 +4651,6 @@
       <c r="O80" t="s">
         <v>89</v>
       </c>
-      <c r="P80">
-        <v>4394700</v>
-      </c>
       <c r="Q80" t="s">
         <v>158</v>
       </c>
@@ -4920,9 +4695,6 @@
       <c r="O81" t="s">
         <v>155</v>
       </c>
-      <c r="P81">
-        <v>528395.9300000001</v>
-      </c>
       <c r="Q81" t="s">
         <v>160</v>
       </c>
@@ -4964,9 +4736,6 @@
       <c r="O82" t="s">
         <v>156</v>
       </c>
-      <c r="P82">
-        <v>1000000</v>
-      </c>
       <c r="Q82" t="s">
         <v>160</v>
       </c>
@@ -5008,9 +4777,6 @@
       <c r="O83" t="s">
         <v>89</v>
       </c>
-      <c r="P83">
-        <v>4394700</v>
-      </c>
       <c r="Q83" t="s">
         <v>158</v>
       </c>
@@ -5058,9 +4824,6 @@
       <c r="O84" t="s">
         <v>89</v>
       </c>
-      <c r="P84">
-        <v>3306000</v>
-      </c>
       <c r="Q84" t="s">
         <v>158</v>
       </c>
@@ -5105,9 +4868,6 @@
       <c r="O85" t="s">
         <v>89</v>
       </c>
-      <c r="P85">
-        <v>3306000</v>
-      </c>
       <c r="Q85" t="s">
         <v>158</v>
       </c>
@@ -5148,9 +4908,6 @@
       </c>
       <c r="O86" t="s">
         <v>157</v>
-      </c>
-      <c r="P86">
-        <v>212577</v>
       </c>
       <c r="Q86" t="s">
         <v>160</v>

</xml_diff>

<commit_message>
Atualização automática: mta (17/08/2026 10:45)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1102" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1116" uniqueCount="175">
   <si>
     <t>linha</t>
   </si>
@@ -191,6 +191,9 @@
   </si>
   <si>
     <t>C26332</t>
+  </si>
+  <si>
+    <t>C26393</t>
   </si>
   <si>
     <t>C26310</t>
@@ -871,7 +874,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V86"/>
+  <dimension ref="A1:V87"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
@@ -962,28 +965,31 @@
         <v>31</v>
       </c>
       <c r="L2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="N2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="O2" t="s">
-        <v>91</v>
+        <v>92</v>
+      </c>
+      <c r="P2">
+        <v>135000</v>
       </c>
       <c r="Q2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S2" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T2" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U2" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V2" s="1">
         <v>46229</v>
@@ -1009,22 +1015,25 @@
         <v>31</v>
       </c>
       <c r="N3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="O3" t="s">
-        <v>92</v>
+        <v>93</v>
+      </c>
+      <c r="P3">
+        <v>400000</v>
       </c>
       <c r="Q3" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="R3" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S3" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T3" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U3" t="s">
         <v>29</v>
@@ -1053,22 +1062,25 @@
         <v>31</v>
       </c>
       <c r="N4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="O4" t="s">
-        <v>93</v>
+        <v>94</v>
+      </c>
+      <c r="P4">
+        <v>430000</v>
       </c>
       <c r="Q4" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R4" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S4" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T4" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U4" t="s">
         <v>29</v>
@@ -1097,22 +1109,25 @@
         <v>31</v>
       </c>
       <c r="N5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="O5" t="s">
-        <v>94</v>
+        <v>95</v>
+      </c>
+      <c r="P5">
+        <v>425000</v>
       </c>
       <c r="Q5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R5" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S5" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T5" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U5" t="s">
         <v>29</v>
@@ -1141,25 +1156,28 @@
         <v>31</v>
       </c>
       <c r="L6" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="N6" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="O6" t="s">
-        <v>95</v>
+        <v>96</v>
+      </c>
+      <c r="P6">
+        <v>563000</v>
       </c>
       <c r="Q6" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R6" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T6" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U6" t="s">
         <v>29</v>
@@ -1197,22 +1215,25 @@
         <v>46</v>
       </c>
       <c r="N7" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="O7" t="s">
-        <v>96</v>
+        <v>97</v>
+      </c>
+      <c r="P7">
+        <v>3799999.6</v>
       </c>
       <c r="Q7" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R7" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S7" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T7" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U7" t="s">
         <v>29</v>
@@ -1241,22 +1262,25 @@
         <v>31</v>
       </c>
       <c r="N8" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="O8" t="s">
-        <v>97</v>
+        <v>98</v>
+      </c>
+      <c r="P8">
+        <v>430000</v>
       </c>
       <c r="Q8" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R8" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S8" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T8" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U8" t="s">
         <v>29</v>
@@ -1285,22 +1309,25 @@
         <v>31</v>
       </c>
       <c r="N9" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="O9" t="s">
-        <v>98</v>
+        <v>99</v>
+      </c>
+      <c r="P9">
+        <v>60000</v>
       </c>
       <c r="Q9" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R9" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S9" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T9" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U9" t="s">
         <v>29</v>
@@ -1329,22 +1356,25 @@
         <v>31</v>
       </c>
       <c r="N10" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="O10" t="s">
-        <v>99</v>
+        <v>100</v>
+      </c>
+      <c r="P10">
+        <v>200000</v>
       </c>
       <c r="Q10" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R10" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S10" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T10" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U10" t="s">
         <v>29</v>
@@ -1373,22 +1403,25 @@
         <v>31</v>
       </c>
       <c r="N11" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="O11" t="s">
-        <v>100</v>
+        <v>101</v>
+      </c>
+      <c r="P11">
+        <v>320000</v>
       </c>
       <c r="Q11" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R11" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S11" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T11" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U11" t="s">
         <v>29</v>
@@ -1426,28 +1459,31 @@
         <v>47</v>
       </c>
       <c r="J12" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="N12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="O12" t="s">
-        <v>101</v>
+        <v>102</v>
+      </c>
+      <c r="P12">
+        <v>1187433.02</v>
       </c>
       <c r="Q12" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R12" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S12" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T12" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U12" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V12" s="1">
         <v>46079</v>
@@ -1473,25 +1509,28 @@
         <v>31</v>
       </c>
       <c r="N13" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="O13" t="s">
-        <v>102</v>
+        <v>103</v>
+      </c>
+      <c r="P13">
+        <v>1000000</v>
       </c>
       <c r="Q13" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R13" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S13" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T13" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U13" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V13" s="1">
         <v>46352</v>
@@ -1517,25 +1556,28 @@
         <v>31</v>
       </c>
       <c r="N14" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="O14" t="s">
-        <v>103</v>
+        <v>104</v>
+      </c>
+      <c r="P14">
+        <v>1000000</v>
       </c>
       <c r="Q14" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R14" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S14" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T14" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U14" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V14" s="1">
         <v>46352</v>
@@ -1561,25 +1603,28 @@
         <v>31</v>
       </c>
       <c r="N15" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="O15" t="s">
-        <v>104</v>
+        <v>105</v>
+      </c>
+      <c r="P15">
+        <v>1000000</v>
       </c>
       <c r="Q15" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R15" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S15" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T15" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U15" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V15" s="1">
         <v>46352</v>
@@ -1605,25 +1650,28 @@
         <v>31</v>
       </c>
       <c r="N16" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O16" t="s">
-        <v>105</v>
+        <v>106</v>
+      </c>
+      <c r="P16">
+        <v>100000</v>
       </c>
       <c r="Q16" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="R16" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S16" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T16" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U16" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V16" s="1">
         <v>46229</v>
@@ -1658,28 +1706,31 @@
         <v>48</v>
       </c>
       <c r="J17" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="N17" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="O17" t="s">
-        <v>106</v>
+        <v>107</v>
+      </c>
+      <c r="P17">
+        <v>1770880.5</v>
       </c>
       <c r="Q17" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R17" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S17" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T17" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U17" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V17" s="1">
         <v>46107</v>
@@ -1714,22 +1765,25 @@
         <v>49</v>
       </c>
       <c r="N18" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="O18" t="s">
-        <v>107</v>
+        <v>108</v>
+      </c>
+      <c r="P18">
+        <v>350000</v>
       </c>
       <c r="Q18" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R18" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S18" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T18" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U18" t="s">
         <v>29</v>
@@ -1767,22 +1821,25 @@
         <v>49</v>
       </c>
       <c r="N19" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="O19" t="s">
-        <v>108</v>
+        <v>109</v>
+      </c>
+      <c r="P19">
+        <v>350000</v>
       </c>
       <c r="Q19" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R19" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S19" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T19" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U19" t="s">
         <v>29</v>
@@ -1811,22 +1868,25 @@
         <v>31</v>
       </c>
       <c r="N20" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O20" t="s">
-        <v>109</v>
+        <v>110</v>
+      </c>
+      <c r="P20">
+        <v>1000000</v>
       </c>
       <c r="Q20" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R20" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S20" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T20" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U20" t="s">
         <v>29</v>
@@ -1855,22 +1915,25 @@
         <v>31</v>
       </c>
       <c r="N21" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="O21" t="s">
-        <v>110</v>
+        <v>111</v>
+      </c>
+      <c r="P21">
+        <v>400000</v>
       </c>
       <c r="Q21" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="R21" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S21" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T21" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U21" t="s">
         <v>29</v>
@@ -1899,22 +1962,25 @@
         <v>31</v>
       </c>
       <c r="N22" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="O22" t="s">
-        <v>111</v>
+        <v>112</v>
+      </c>
+      <c r="P22">
+        <v>120000</v>
       </c>
       <c r="Q22" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R22" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S22" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T22" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U22" t="s">
         <v>29</v>
@@ -1943,22 +2009,25 @@
         <v>31</v>
       </c>
       <c r="N23" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="O23" t="s">
-        <v>112</v>
+        <v>113</v>
+      </c>
+      <c r="P23">
+        <v>80000</v>
       </c>
       <c r="Q23" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R23" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S23" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T23" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U23" t="s">
         <v>29</v>
@@ -1996,28 +2065,31 @@
         <v>50</v>
       </c>
       <c r="J24" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="N24" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="O24" t="s">
-        <v>113</v>
+        <v>114</v>
+      </c>
+      <c r="P24">
+        <v>1704503</v>
       </c>
       <c r="Q24" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R24" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S24" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T24" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U24" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V24" s="1">
         <v>46138</v>
@@ -2052,22 +2124,25 @@
         <v>51</v>
       </c>
       <c r="N25" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="O25" t="s">
-        <v>114</v>
+        <v>115</v>
+      </c>
+      <c r="P25">
+        <v>3799000</v>
       </c>
       <c r="Q25" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R25" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S25" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T25" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U25" t="s">
         <v>29</v>
@@ -2105,22 +2180,25 @@
         <v>52</v>
       </c>
       <c r="N26" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="O26" t="s">
-        <v>114</v>
+        <v>115</v>
+      </c>
+      <c r="P26">
+        <v>1000</v>
       </c>
       <c r="Q26" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R26" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S26" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T26" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U26" t="s">
         <v>29</v>
@@ -2149,25 +2227,28 @@
         <v>31</v>
       </c>
       <c r="N27" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O27" t="s">
-        <v>115</v>
+        <v>116</v>
+      </c>
+      <c r="P27">
+        <v>100000</v>
       </c>
       <c r="Q27" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="R27" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S27" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T27" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U27" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V27" s="1">
         <v>46291</v>
@@ -2202,28 +2283,31 @@
         <v>53</v>
       </c>
       <c r="J28" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="N28" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="O28" t="s">
-        <v>116</v>
+        <v>117</v>
+      </c>
+      <c r="P28">
+        <v>150000</v>
       </c>
       <c r="Q28" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R28" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S28" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T28" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U28" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V28" s="1">
         <v>46199</v>
@@ -2258,28 +2342,31 @@
         <v>53</v>
       </c>
       <c r="J29" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="N29" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="O29" t="s">
-        <v>117</v>
+        <v>118</v>
+      </c>
+      <c r="P29">
+        <v>150000</v>
       </c>
       <c r="Q29" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R29" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S29" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T29" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U29" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V29" s="1">
         <v>46199</v>
@@ -2314,28 +2401,31 @@
         <v>54</v>
       </c>
       <c r="J30" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="N30" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="O30" t="s">
-        <v>118</v>
+        <v>119</v>
+      </c>
+      <c r="P30">
+        <v>18462.36</v>
       </c>
       <c r="Q30" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R30" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S30" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T30" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U30" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V30" s="1">
         <v>46199</v>
@@ -2370,28 +2460,31 @@
         <v>53</v>
       </c>
       <c r="J31" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="N31" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="O31" t="s">
-        <v>118</v>
+        <v>119</v>
+      </c>
+      <c r="P31">
+        <v>324166.14</v>
       </c>
       <c r="Q31" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R31" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S31" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T31" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U31" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V31" s="1">
         <v>46199</v>
@@ -2417,25 +2510,28 @@
         <v>31</v>
       </c>
       <c r="N32" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="O32" t="s">
-        <v>119</v>
+        <v>120</v>
+      </c>
+      <c r="P32">
+        <v>30000</v>
       </c>
       <c r="Q32" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R32" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S32" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T32" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U32" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V32" s="1">
         <v>46291</v>
@@ -2470,28 +2566,31 @@
         <v>55</v>
       </c>
       <c r="J33" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="N33" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="O33" t="s">
-        <v>120</v>
+        <v>121</v>
+      </c>
+      <c r="P33">
+        <v>1496713.48</v>
       </c>
       <c r="Q33" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R33" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S33" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T33" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U33" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V33" s="1">
         <v>46199</v>
@@ -2526,25 +2625,28 @@
         <v>50</v>
       </c>
       <c r="N34" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="O34" t="s">
-        <v>120</v>
+        <v>121</v>
+      </c>
+      <c r="P34">
+        <v>207789.52</v>
       </c>
       <c r="Q34" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R34" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S34" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T34" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U34" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V34" s="1">
         <v>46138</v>
@@ -2579,22 +2681,25 @@
         <v>56</v>
       </c>
       <c r="N35" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="O35" t="s">
-        <v>121</v>
+        <v>122</v>
+      </c>
+      <c r="P35">
+        <v>962290.8</v>
       </c>
       <c r="Q35" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R35" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S35" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T35" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U35" t="s">
         <v>29</v>
@@ -2632,22 +2737,25 @@
         <v>57</v>
       </c>
       <c r="N36" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="O36" t="s">
-        <v>121</v>
+        <v>122</v>
+      </c>
+      <c r="P36">
+        <v>798776.97</v>
       </c>
       <c r="Q36" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R36" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S36" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T36" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U36" t="s">
         <v>29</v>
@@ -2685,22 +2793,25 @@
         <v>56</v>
       </c>
       <c r="N37" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="O37" t="s">
-        <v>121</v>
+        <v>122</v>
+      </c>
+      <c r="P37">
+        <v>1530656.62</v>
       </c>
       <c r="Q37" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R37" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S37" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T37" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U37" t="s">
         <v>29</v>
@@ -2738,22 +2849,25 @@
         <v>58</v>
       </c>
       <c r="N38" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="O38" t="s">
-        <v>121</v>
+        <v>122</v>
+      </c>
+      <c r="P38">
+        <v>72958.08</v>
       </c>
       <c r="Q38" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R38" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S38" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T38" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U38" t="s">
         <v>29</v>
@@ -2791,22 +2905,25 @@
         <v>58</v>
       </c>
       <c r="N39" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="O39" t="s">
-        <v>121</v>
+        <v>122</v>
+      </c>
+      <c r="P39">
+        <v>8916</v>
       </c>
       <c r="Q39" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R39" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S39" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T39" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U39" t="s">
         <v>29</v>
@@ -2844,22 +2961,25 @@
         <v>58</v>
       </c>
       <c r="N40" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="O40" t="s">
-        <v>121</v>
+        <v>122</v>
+      </c>
+      <c r="P40">
+        <v>425178.5</v>
       </c>
       <c r="Q40" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R40" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S40" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T40" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U40" t="s">
         <v>29</v>
@@ -2870,7 +2990,7 @@
     </row>
     <row r="41" spans="1:22">
       <c r="A41">
-        <v>15980</v>
+        <v>15966</v>
       </c>
       <c r="B41" t="s">
         <v>22</v>
@@ -2879,42 +2999,54 @@
         <v>22</v>
       </c>
       <c r="D41" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E41" t="s">
-        <v>30</v>
+        <v>29</v>
+      </c>
+      <c r="F41" t="s">
+        <v>35</v>
       </c>
       <c r="G41" t="s">
-        <v>43</v>
+        <v>42</v>
+      </c>
+      <c r="H41" s="1">
+        <v>46244</v>
+      </c>
+      <c r="I41" t="s">
+        <v>59</v>
       </c>
       <c r="N41" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="O41" t="s">
         <v>122</v>
       </c>
+      <c r="P41">
+        <v>1223.03</v>
+      </c>
       <c r="Q41" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R41" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S41" t="s">
         <v>166</v>
       </c>
       <c r="T41" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U41" t="s">
         <v>29</v>
       </c>
       <c r="V41" s="1">
-        <v>46260</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="42" spans="1:22">
       <c r="A42">
-        <v>16000</v>
+        <v>15980</v>
       </c>
       <c r="B42" t="s">
         <v>22</v>
@@ -2923,51 +3055,42 @@
         <v>22</v>
       </c>
       <c r="D42" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E42" t="s">
-        <v>29</v>
-      </c>
-      <c r="F42" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G42" t="s">
-        <v>42</v>
-      </c>
-      <c r="H42" s="1">
-        <v>46191</v>
-      </c>
-      <c r="I42" t="s">
-        <v>59</v>
+        <v>43</v>
       </c>
       <c r="N42" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="O42" t="s">
         <v>123</v>
       </c>
       <c r="Q42" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R42" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S42" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T42" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U42" t="s">
         <v>29</v>
       </c>
       <c r="V42" s="1">
-        <v>46199</v>
+        <v>46260</v>
       </c>
     </row>
     <row r="43" spans="1:22">
       <c r="A43">
-        <v>16001</v>
+        <v>16000</v>
       </c>
       <c r="B43" t="s">
         <v>22</v>
@@ -2991,25 +3114,28 @@
         <v>46191</v>
       </c>
       <c r="I43" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="N43" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="O43" t="s">
         <v>124</v>
       </c>
+      <c r="P43">
+        <v>400000</v>
+      </c>
       <c r="Q43" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R43" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S43" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T43" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U43" t="s">
         <v>29</v>
@@ -3020,7 +3146,7 @@
     </row>
     <row r="44" spans="1:22">
       <c r="A44">
-        <v>16560</v>
+        <v>16001</v>
       </c>
       <c r="B44" t="s">
         <v>22</v>
@@ -3041,42 +3167,42 @@
         <v>42</v>
       </c>
       <c r="H44" s="1">
-        <v>46213</v>
+        <v>46191</v>
       </c>
       <c r="I44" t="s">
-        <v>55</v>
-      </c>
-      <c r="J44" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="N44" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="O44" t="s">
         <v>125</v>
       </c>
+      <c r="P44">
+        <v>400000</v>
+      </c>
       <c r="Q44" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R44" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="S44" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T44" t="s">
         <v>171</v>
       </c>
       <c r="U44" t="s">
-        <v>173</v>
+        <v>29</v>
       </c>
       <c r="V44" s="1">
-        <v>46229</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="45" spans="1:22">
       <c r="A45">
-        <v>16561</v>
+        <v>16560</v>
       </c>
       <c r="B45" t="s">
         <v>22</v>
@@ -3091,37 +3217,43 @@
         <v>29</v>
       </c>
       <c r="F45" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="G45" t="s">
         <v>42</v>
       </c>
       <c r="H45" s="1">
-        <v>46210</v>
+        <v>46213</v>
       </c>
       <c r="I45" t="s">
-        <v>54</v>
+        <v>55</v>
+      </c>
+      <c r="J45" t="s">
+        <v>67</v>
       </c>
       <c r="N45" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="O45" t="s">
-        <v>125</v>
+        <v>126</v>
+      </c>
+      <c r="P45">
+        <v>173846.38</v>
       </c>
       <c r="Q45" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R45" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S45" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T45" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U45" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V45" s="1">
         <v>46229</v>
@@ -3129,7 +3261,7 @@
     </row>
     <row r="46" spans="1:22">
       <c r="A46">
-        <v>16700</v>
+        <v>16561</v>
       </c>
       <c r="B46" t="s">
         <v>22</v>
@@ -3138,42 +3270,54 @@
         <v>22</v>
       </c>
       <c r="D46" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E46" t="s">
         <v>29</v>
       </c>
       <c r="F46" t="s">
-        <v>31</v>
+        <v>34</v>
+      </c>
+      <c r="G46" t="s">
+        <v>42</v>
+      </c>
+      <c r="H46" s="1">
+        <v>46210</v>
+      </c>
+      <c r="I46" t="s">
+        <v>54</v>
       </c>
       <c r="N46" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O46" t="s">
         <v>126</v>
       </c>
+      <c r="P46">
+        <v>1530656.62</v>
+      </c>
       <c r="Q46" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R46" t="s">
         <v>162</v>
       </c>
       <c r="S46" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T46" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="U46" t="s">
-        <v>29</v>
+        <v>174</v>
       </c>
       <c r="V46" s="1">
-        <v>46321</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="47" spans="1:22">
       <c r="A47">
-        <v>17200</v>
+        <v>16700</v>
       </c>
       <c r="B47" t="s">
         <v>22</v>
@@ -3191,33 +3335,36 @@
         <v>31</v>
       </c>
       <c r="N47" t="s">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="O47" t="s">
         <v>127</v>
       </c>
+      <c r="P47">
+        <v>1000000</v>
+      </c>
       <c r="Q47" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="R47" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S47" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T47" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="U47" t="s">
-        <v>173</v>
+        <v>29</v>
       </c>
       <c r="V47" s="1">
-        <v>46291</v>
+        <v>46321</v>
       </c>
     </row>
     <row r="48" spans="1:22">
       <c r="A48">
-        <v>17201</v>
+        <v>17200</v>
       </c>
       <c r="B48" t="s">
         <v>22</v>
@@ -3226,7 +3373,7 @@
         <v>22</v>
       </c>
       <c r="D48" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E48" t="s">
         <v>29</v>
@@ -3234,46 +3381,37 @@
       <c r="F48" t="s">
         <v>31</v>
       </c>
-      <c r="G48" t="s">
-        <v>42</v>
-      </c>
-      <c r="H48" s="1">
-        <v>46176</v>
-      </c>
-      <c r="I48" t="s">
-        <v>60</v>
-      </c>
-      <c r="J48" t="s">
-        <v>67</v>
-      </c>
       <c r="N48" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="O48" t="s">
-        <v>127</v>
+        <v>128</v>
+      </c>
+      <c r="P48">
+        <v>958040</v>
       </c>
       <c r="Q48" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R48" t="s">
         <v>163</v>
       </c>
       <c r="S48" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T48" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U48" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V48" s="1">
-        <v>46199</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="49" spans="1:22">
       <c r="A49">
-        <v>17760</v>
+        <v>17201</v>
       </c>
       <c r="B49" t="s">
         <v>22</v>
@@ -3282,7 +3420,7 @@
         <v>22</v>
       </c>
       <c r="D49" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E49" t="s">
         <v>29</v>
@@ -3290,40 +3428,49 @@
       <c r="F49" t="s">
         <v>31</v>
       </c>
+      <c r="G49" t="s">
+        <v>42</v>
+      </c>
+      <c r="H49" s="1">
+        <v>46176</v>
+      </c>
+      <c r="I49" t="s">
+        <v>61</v>
+      </c>
       <c r="J49" t="s">
-        <v>66</v>
-      </c>
-      <c r="K49" t="s">
         <v>68</v>
       </c>
       <c r="N49" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="O49" t="s">
         <v>128</v>
       </c>
+      <c r="P49">
+        <v>41730.64</v>
+      </c>
       <c r="Q49" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="R49" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="S49" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T49" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U49" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V49" s="1">
-        <v>46260</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="50" spans="1:22">
       <c r="A50">
-        <v>17761</v>
+        <v>17760</v>
       </c>
       <c r="B50" t="s">
         <v>22</v>
@@ -3341,39 +3488,42 @@
         <v>31</v>
       </c>
       <c r="J50" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="K50" t="s">
         <v>69</v>
       </c>
       <c r="N50" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="O50" t="s">
         <v>129</v>
       </c>
+      <c r="P50">
+        <v>1468159.32</v>
+      </c>
       <c r="Q50" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R50" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S50" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T50" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U50" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V50" s="1">
-        <v>46291</v>
+        <v>46260</v>
       </c>
     </row>
     <row r="51" spans="1:22">
       <c r="A51">
-        <v>17762</v>
+        <v>17761</v>
       </c>
       <c r="B51" t="s">
         <v>22</v>
@@ -3390,37 +3540,43 @@
       <c r="F51" t="s">
         <v>31</v>
       </c>
+      <c r="J51" t="s">
+        <v>67</v>
+      </c>
       <c r="K51" t="s">
         <v>70</v>
       </c>
       <c r="N51" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="O51" t="s">
         <v>130</v>
       </c>
+      <c r="P51">
+        <v>1704503</v>
+      </c>
       <c r="Q51" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R51" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S51" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T51" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U51" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V51" s="1">
-        <v>46321</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="52" spans="1:22">
       <c r="A52">
-        <v>17763</v>
+        <v>17762</v>
       </c>
       <c r="B52" t="s">
         <v>22</v>
@@ -3429,51 +3585,48 @@
         <v>22</v>
       </c>
       <c r="D52" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E52" t="s">
         <v>29</v>
       </c>
       <c r="F52" t="s">
-        <v>39</v>
-      </c>
-      <c r="G52" t="s">
-        <v>42</v>
-      </c>
-      <c r="H52" s="1">
-        <v>46227</v>
-      </c>
-      <c r="I52" t="s">
-        <v>61</v>
+        <v>31</v>
+      </c>
+      <c r="K52" t="s">
+        <v>71</v>
       </c>
       <c r="N52" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="O52" t="s">
-        <v>128</v>
+        <v>131</v>
+      </c>
+      <c r="P52">
+        <v>1704503</v>
       </c>
       <c r="Q52" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R52" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S52" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T52" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U52" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V52" s="1">
-        <v>46229</v>
+        <v>46321</v>
       </c>
     </row>
     <row r="53" spans="1:22">
       <c r="A53">
-        <v>18140</v>
+        <v>17763</v>
       </c>
       <c r="B53" t="s">
         <v>22</v>
@@ -3482,45 +3635,57 @@
         <v>22</v>
       </c>
       <c r="D53" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E53" t="s">
         <v>29</v>
       </c>
       <c r="F53" t="s">
-        <v>31</v>
+        <v>39</v>
+      </c>
+      <c r="G53" t="s">
+        <v>42</v>
+      </c>
+      <c r="H53" s="1">
+        <v>46227</v>
+      </c>
+      <c r="I53" t="s">
+        <v>62</v>
       </c>
       <c r="N53" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="O53" t="s">
-        <v>131</v>
+        <v>129</v>
+      </c>
+      <c r="P53">
+        <v>236343.68</v>
       </c>
       <c r="Q53" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R53" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S53" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T53" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U53" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V53" s="1">
-        <v>46352</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="54" spans="1:22">
       <c r="A54">
-        <v>19240</v>
+        <v>18140</v>
       </c>
       <c r="B54" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C54" t="s">
         <v>22</v>
@@ -3532,39 +3697,39 @@
         <v>29</v>
       </c>
       <c r="F54" t="s">
-        <v>40</v>
-      </c>
-      <c r="K54" t="s">
-        <v>70</v>
+        <v>31</v>
       </c>
       <c r="N54" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="O54" t="s">
         <v>132</v>
       </c>
+      <c r="P54">
+        <v>1295422.28</v>
+      </c>
       <c r="Q54" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R54" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S54" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="T54" t="s">
         <v>172</v>
       </c>
       <c r="U54" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V54" s="1">
-        <v>46321</v>
+        <v>46352</v>
       </c>
     </row>
     <row r="55" spans="1:22">
       <c r="A55">
-        <v>19241</v>
+        <v>19240</v>
       </c>
       <c r="B55" t="s">
         <v>23</v>
@@ -3573,37 +3738,40 @@
         <v>22</v>
       </c>
       <c r="D55" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E55" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F55" t="s">
         <v>40</v>
       </c>
-      <c r="G55" t="s">
-        <v>44</v>
+      <c r="K55" t="s">
+        <v>71</v>
       </c>
       <c r="N55" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="O55" t="s">
-        <v>132</v>
+        <v>133</v>
+      </c>
+      <c r="P55">
+        <v>500000</v>
       </c>
       <c r="Q55" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R55" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S55" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="T55" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="U55" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V55" s="1">
         <v>46321</v>
@@ -3611,7 +3779,7 @@
     </row>
     <row r="56" spans="1:22">
       <c r="A56">
-        <v>19260</v>
+        <v>19241</v>
       </c>
       <c r="B56" t="s">
         <v>23</v>
@@ -3625,37 +3793,43 @@
       <c r="E56" t="s">
         <v>30</v>
       </c>
+      <c r="F56" t="s">
+        <v>40</v>
+      </c>
       <c r="G56" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="N56" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="O56" t="s">
         <v>133</v>
       </c>
+      <c r="P56">
+        <v>5000000</v>
+      </c>
       <c r="Q56" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R56" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S56" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="T56" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="U56" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V56" s="1">
-        <v>46049</v>
+        <v>46321</v>
       </c>
     </row>
     <row r="57" spans="1:22">
       <c r="A57">
-        <v>19600</v>
+        <v>19260</v>
       </c>
       <c r="B57" t="s">
         <v>23</v>
@@ -3673,30 +3847,33 @@
         <v>43</v>
       </c>
       <c r="N57" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="O57" t="s">
         <v>134</v>
       </c>
       <c r="Q57" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R57" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S57" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="T57" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="U57" t="s">
-        <v>173</v>
+        <v>174</v>
+      </c>
+      <c r="V57" s="1">
+        <v>46049</v>
       </c>
     </row>
     <row r="58" spans="1:22">
       <c r="A58">
-        <v>19620</v>
+        <v>19600</v>
       </c>
       <c r="B58" t="s">
         <v>23</v>
@@ -3714,33 +3891,33 @@
         <v>43</v>
       </c>
       <c r="N58" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="O58" t="s">
         <v>135</v>
       </c>
       <c r="Q58" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R58" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S58" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="T58" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="U58" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="59" spans="1:22">
       <c r="A59">
-        <v>23120</v>
+        <v>19620</v>
       </c>
       <c r="B59" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C59" t="s">
         <v>22</v>
@@ -3751,6 +3928,9 @@
       <c r="E59" t="s">
         <v>30</v>
       </c>
+      <c r="G59" t="s">
+        <v>43</v>
+      </c>
       <c r="N59" t="s">
         <v>82</v>
       </c>
@@ -3758,27 +3938,24 @@
         <v>136</v>
       </c>
       <c r="Q59" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="R59" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="S59" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="T59" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="U59" t="s">
-        <v>173</v>
-      </c>
-      <c r="V59" s="1">
-        <v>46107</v>
+        <v>174</v>
       </c>
     </row>
     <row r="60" spans="1:22">
       <c r="A60">
-        <v>23160</v>
+        <v>23120</v>
       </c>
       <c r="B60" t="s">
         <v>22</v>
@@ -3798,20 +3975,23 @@
       <c r="O60" t="s">
         <v>137</v>
       </c>
+      <c r="P60">
+        <v>9389.959999999999</v>
+      </c>
       <c r="Q60" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R60" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="S60" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="T60" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U60" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V60" s="1">
         <v>46107</v>
@@ -3819,7 +3999,7 @@
     </row>
     <row r="61" spans="1:22">
       <c r="A61">
-        <v>23100</v>
+        <v>23160</v>
       </c>
       <c r="B61" t="s">
         <v>22</v>
@@ -3839,20 +4019,23 @@
       <c r="O61" t="s">
         <v>138</v>
       </c>
+      <c r="P61">
+        <v>7204.82</v>
+      </c>
       <c r="Q61" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R61" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="S61" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="T61" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U61" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V61" s="1">
         <v>46107</v>
@@ -3860,7 +4043,7 @@
     </row>
     <row r="62" spans="1:22">
       <c r="A62">
-        <v>23080</v>
+        <v>23100</v>
       </c>
       <c r="B62" t="s">
         <v>22</v>
@@ -3880,20 +4063,23 @@
       <c r="O62" t="s">
         <v>139</v>
       </c>
+      <c r="P62">
+        <v>4227.84</v>
+      </c>
       <c r="Q62" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="R62" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="S62" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="T62" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U62" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V62" s="1">
         <v>46107</v>
@@ -3901,7 +4087,7 @@
     </row>
     <row r="63" spans="1:22">
       <c r="A63">
-        <v>23180</v>
+        <v>23080</v>
       </c>
       <c r="B63" t="s">
         <v>22</v>
@@ -3919,22 +4105,25 @@
         <v>86</v>
       </c>
       <c r="O63" t="s">
-        <v>138</v>
+        <v>140</v>
+      </c>
+      <c r="P63">
+        <v>4064.54</v>
       </c>
       <c r="Q63" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="R63" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="S63" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="T63" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U63" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V63" s="1">
         <v>46107</v>
@@ -3942,7 +4131,7 @@
     </row>
     <row r="64" spans="1:22">
       <c r="A64">
-        <v>23140</v>
+        <v>23180</v>
       </c>
       <c r="B64" t="s">
         <v>22</v>
@@ -3960,22 +4149,25 @@
         <v>87</v>
       </c>
       <c r="O64" t="s">
-        <v>140</v>
+        <v>139</v>
+      </c>
+      <c r="P64">
+        <v>3662.66</v>
       </c>
       <c r="Q64" t="s">
         <v>159</v>
       </c>
       <c r="R64" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="S64" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="T64" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U64" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V64" s="1">
         <v>46107</v>
@@ -3983,7 +4175,7 @@
     </row>
     <row r="65" spans="1:22">
       <c r="A65">
-        <v>23640</v>
+        <v>23140</v>
       </c>
       <c r="B65" t="s">
         <v>22</v>
@@ -3998,33 +4190,36 @@
         <v>30</v>
       </c>
       <c r="N65" t="s">
-        <v>73</v>
+        <v>88</v>
       </c>
       <c r="O65" t="s">
         <v>141</v>
       </c>
+      <c r="P65">
+        <v>1163.64</v>
+      </c>
       <c r="Q65" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="R65" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="S65" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="T65" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U65" t="s">
-        <v>29</v>
+        <v>174</v>
       </c>
       <c r="V65" s="1">
-        <v>46168</v>
+        <v>46107</v>
       </c>
     </row>
     <row r="66" spans="1:22">
       <c r="A66">
-        <v>23740</v>
+        <v>23640</v>
       </c>
       <c r="B66" t="s">
         <v>22</v>
@@ -4033,20 +4228,20 @@
         <v>22</v>
       </c>
       <c r="D66" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E66" t="s">
-        <v>29</v>
-      </c>
-      <c r="F66" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N66" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="O66" t="s">
         <v>142</v>
       </c>
+      <c r="P66">
+        <v>120000</v>
+      </c>
       <c r="Q66" t="s">
         <v>159</v>
       </c>
@@ -4054,21 +4249,21 @@
         <v>162</v>
       </c>
       <c r="S66" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T66" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U66" t="s">
         <v>29</v>
       </c>
       <c r="V66" s="1">
-        <v>46291</v>
+        <v>46168</v>
       </c>
     </row>
     <row r="67" spans="1:22">
       <c r="A67">
-        <v>24180</v>
+        <v>23740</v>
       </c>
       <c r="B67" t="s">
         <v>22</v>
@@ -4086,33 +4281,36 @@
         <v>31</v>
       </c>
       <c r="N67" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="O67" t="s">
         <v>143</v>
       </c>
+      <c r="P67">
+        <v>400000</v>
+      </c>
       <c r="Q67" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="R67" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S67" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T67" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U67" t="s">
-        <v>173</v>
+        <v>29</v>
       </c>
       <c r="V67" s="1">
-        <v>46229</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="68" spans="1:22">
       <c r="A68">
-        <v>24380</v>
+        <v>24180</v>
       </c>
       <c r="B68" t="s">
         <v>22</v>
@@ -4121,39 +4319,45 @@
         <v>22</v>
       </c>
       <c r="D68" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E68" t="s">
-        <v>30</v>
+        <v>29</v>
+      </c>
+      <c r="F68" t="s">
+        <v>31</v>
       </c>
       <c r="N68" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="O68" t="s">
         <v>144</v>
       </c>
+      <c r="P68">
+        <v>100000</v>
+      </c>
       <c r="Q68" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="R68" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="S68" t="s">
         <v>166</v>
       </c>
       <c r="T68" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U68" t="s">
-        <v>29</v>
+        <v>174</v>
       </c>
       <c r="V68" s="1">
-        <v>46260</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="69" spans="1:22">
       <c r="A69">
-        <v>24660</v>
+        <v>24380</v>
       </c>
       <c r="B69" t="s">
         <v>22</v>
@@ -4168,33 +4372,36 @@
         <v>30</v>
       </c>
       <c r="N69" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="O69" t="s">
         <v>145</v>
       </c>
+      <c r="P69">
+        <v>80000</v>
+      </c>
       <c r="Q69" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R69" t="s">
         <v>162</v>
       </c>
       <c r="S69" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="T69" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U69" t="s">
-        <v>173</v>
+        <v>29</v>
       </c>
       <c r="V69" s="1">
-        <v>46291</v>
+        <v>46260</v>
       </c>
     </row>
     <row r="70" spans="1:22">
       <c r="A70">
-        <v>24661</v>
+        <v>24660</v>
       </c>
       <c r="B70" t="s">
         <v>22</v>
@@ -4209,33 +4416,36 @@
         <v>30</v>
       </c>
       <c r="N70" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="O70" t="s">
-        <v>145</v>
+        <v>146</v>
+      </c>
+      <c r="P70">
+        <v>835000</v>
       </c>
       <c r="Q70" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R70" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S70" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="T70" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U70" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V70" s="1">
-        <v>46168</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="71" spans="1:22">
       <c r="A71">
-        <v>24680</v>
+        <v>24661</v>
       </c>
       <c r="B71" t="s">
         <v>22</v>
@@ -4250,33 +4460,36 @@
         <v>30</v>
       </c>
       <c r="N71" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="O71" t="s">
         <v>146</v>
       </c>
+      <c r="P71">
+        <v>165000</v>
+      </c>
       <c r="Q71" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R71" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S71" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="T71" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U71" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V71" s="1">
-        <v>46291</v>
+        <v>46168</v>
       </c>
     </row>
     <row r="72" spans="1:22">
       <c r="A72">
-        <v>24700</v>
+        <v>24680</v>
       </c>
       <c r="B72" t="s">
         <v>22</v>
@@ -4291,25 +4504,28 @@
         <v>30</v>
       </c>
       <c r="N72" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="O72" t="s">
         <v>147</v>
       </c>
+      <c r="P72">
+        <v>1000000</v>
+      </c>
       <c r="Q72" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R72" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S72" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="T72" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U72" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V72" s="1">
         <v>46291</v>
@@ -4317,7 +4533,7 @@
     </row>
     <row r="73" spans="1:22">
       <c r="A73">
-        <v>24720</v>
+        <v>24700</v>
       </c>
       <c r="B73" t="s">
         <v>22</v>
@@ -4332,25 +4548,28 @@
         <v>30</v>
       </c>
       <c r="N73" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="O73" t="s">
         <v>148</v>
       </c>
+      <c r="P73">
+        <v>1000000</v>
+      </c>
       <c r="Q73" t="s">
         <v>159</v>
       </c>
       <c r="R73" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S73" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="T73" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U73" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V73" s="1">
         <v>46291</v>
@@ -4358,7 +4577,7 @@
     </row>
     <row r="74" spans="1:22">
       <c r="A74">
-        <v>25180</v>
+        <v>24720</v>
       </c>
       <c r="B74" t="s">
         <v>22</v>
@@ -4367,42 +4586,42 @@
         <v>22</v>
       </c>
       <c r="D74" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E74" t="s">
-        <v>29</v>
-      </c>
-      <c r="F74" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N74" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="O74" t="s">
         <v>149</v>
       </c>
+      <c r="P74">
+        <v>100000</v>
+      </c>
       <c r="Q74" t="s">
         <v>160</v>
       </c>
       <c r="R74" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S74" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T74" t="s">
         <v>170</v>
       </c>
       <c r="U74" t="s">
-        <v>29</v>
+        <v>174</v>
       </c>
       <c r="V74" s="1">
-        <v>46321</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="75" spans="1:22">
       <c r="A75">
-        <v>25900</v>
+        <v>25180</v>
       </c>
       <c r="B75" t="s">
         <v>22</v>
@@ -4411,45 +4630,45 @@
         <v>22</v>
       </c>
       <c r="D75" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="E75" t="s">
         <v>29</v>
       </c>
       <c r="F75" t="s">
-        <v>41</v>
-      </c>
-      <c r="G75" t="s">
-        <v>45</v>
+        <v>31</v>
       </c>
       <c r="N75" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="O75" t="s">
         <v>150</v>
       </c>
+      <c r="P75">
+        <v>1000000</v>
+      </c>
       <c r="Q75" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R75" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="S75" t="s">
-        <v>41</v>
+        <v>166</v>
       </c>
       <c r="T75" t="s">
         <v>171</v>
       </c>
       <c r="U75" t="s">
-        <v>173</v>
+        <v>29</v>
       </c>
       <c r="V75" s="1">
-        <v>46381</v>
+        <v>46321</v>
       </c>
     </row>
     <row r="76" spans="1:22">
       <c r="A76">
-        <v>25920</v>
+        <v>25900</v>
       </c>
       <c r="B76" t="s">
         <v>22</v>
@@ -4470,25 +4689,28 @@
         <v>45</v>
       </c>
       <c r="N76" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="O76" t="s">
         <v>151</v>
       </c>
+      <c r="P76">
+        <v>1704503</v>
+      </c>
       <c r="Q76" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R76" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S76" t="s">
         <v>41</v>
       </c>
       <c r="T76" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U76" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="V76" s="1">
         <v>46381</v>
@@ -4496,7 +4718,7 @@
     </row>
     <row r="77" spans="1:22">
       <c r="A77">
-        <v>25940</v>
+        <v>25920</v>
       </c>
       <c r="B77" t="s">
         <v>22</v>
@@ -4517,25 +4739,28 @@
         <v>45</v>
       </c>
       <c r="N77" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="O77" t="s">
         <v>152</v>
       </c>
+      <c r="P77">
+        <v>1638125.5</v>
+      </c>
       <c r="Q77" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R77" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S77" t="s">
         <v>41</v>
       </c>
       <c r="T77" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="U77" t="s">
-        <v>29</v>
+        <v>174</v>
       </c>
       <c r="V77" s="1">
         <v>46381</v>
@@ -4543,7 +4768,7 @@
     </row>
     <row r="78" spans="1:22">
       <c r="A78">
-        <v>25960</v>
+        <v>25940</v>
       </c>
       <c r="B78" t="s">
         <v>22</v>
@@ -4564,22 +4789,25 @@
         <v>45</v>
       </c>
       <c r="N78" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="O78" t="s">
         <v>153</v>
       </c>
+      <c r="P78">
+        <v>3800000</v>
+      </c>
       <c r="Q78" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R78" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S78" t="s">
         <v>41</v>
       </c>
       <c r="T78" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U78" t="s">
         <v>29</v>
@@ -4590,7 +4818,7 @@
     </row>
     <row r="79" spans="1:22">
       <c r="A79">
-        <v>63120</v>
+        <v>25960</v>
       </c>
       <c r="B79" t="s">
         <v>22</v>
@@ -4599,39 +4827,48 @@
         <v>22</v>
       </c>
       <c r="D79" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E79" t="s">
-        <v>30</v>
+        <v>29</v>
+      </c>
+      <c r="F79" t="s">
+        <v>41</v>
+      </c>
+      <c r="G79" t="s">
+        <v>45</v>
       </c>
       <c r="N79" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="O79" t="s">
         <v>154</v>
       </c>
+      <c r="P79">
+        <v>3800000</v>
+      </c>
       <c r="Q79" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R79" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S79" t="s">
-        <v>166</v>
+        <v>41</v>
       </c>
       <c r="T79" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U79" t="s">
         <v>29</v>
       </c>
       <c r="V79" s="1">
-        <v>46382</v>
+        <v>46381</v>
       </c>
     </row>
     <row r="80" spans="1:22">
       <c r="A80">
-        <v>63140</v>
+        <v>63120</v>
       </c>
       <c r="B80" t="s">
         <v>22</v>
@@ -4640,28 +4877,31 @@
         <v>22</v>
       </c>
       <c r="D80" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E80" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N80" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="O80" t="s">
-        <v>89</v>
+        <v>155</v>
+      </c>
+      <c r="P80">
+        <v>3800000</v>
       </c>
       <c r="Q80" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="R80" t="s">
         <v>162</v>
       </c>
       <c r="S80" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="T80" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U80" t="s">
         <v>29</v>
@@ -4672,7 +4912,7 @@
     </row>
     <row r="81" spans="1:22">
       <c r="A81">
-        <v>63940</v>
+        <v>63140</v>
       </c>
       <c r="B81" t="s">
         <v>22</v>
@@ -4686,29 +4926,29 @@
       <c r="E81" t="s">
         <v>29</v>
       </c>
-      <c r="F81" t="s">
-        <v>31</v>
-      </c>
       <c r="N81" t="s">
-        <v>77</v>
+        <v>89</v>
       </c>
       <c r="O81" t="s">
-        <v>155</v>
+        <v>90</v>
+      </c>
+      <c r="P81">
+        <v>4394700</v>
       </c>
       <c r="Q81" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="R81" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="S81" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T81" t="s">
         <v>171</v>
       </c>
       <c r="U81" t="s">
-        <v>173</v>
+        <v>29</v>
       </c>
       <c r="V81" s="1">
         <v>46382</v>
@@ -4716,7 +4956,7 @@
     </row>
     <row r="82" spans="1:22">
       <c r="A82">
-        <v>63960</v>
+        <v>63940</v>
       </c>
       <c r="B82" t="s">
         <v>22</v>
@@ -4725,39 +4965,45 @@
         <v>22</v>
       </c>
       <c r="D82" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E82" t="s">
-        <v>30</v>
+        <v>29</v>
+      </c>
+      <c r="F82" t="s">
+        <v>31</v>
       </c>
       <c r="N82" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O82" t="s">
         <v>156</v>
       </c>
+      <c r="P82">
+        <v>528395.9300000001</v>
+      </c>
       <c r="Q82" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R82" t="s">
         <v>162</v>
       </c>
       <c r="S82" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="T82" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="U82" t="s">
-        <v>29</v>
+        <v>174</v>
       </c>
       <c r="V82" s="1">
-        <v>46321</v>
+        <v>46382</v>
       </c>
     </row>
     <row r="83" spans="1:22">
       <c r="A83">
-        <v>64340</v>
+        <v>63960</v>
       </c>
       <c r="B83" t="s">
         <v>22</v>
@@ -4766,39 +5012,42 @@
         <v>22</v>
       </c>
       <c r="D83" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E83" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N83" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="O83" t="s">
-        <v>89</v>
+        <v>157</v>
+      </c>
+      <c r="P83">
+        <v>1000000</v>
       </c>
       <c r="Q83" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="R83" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S83" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="T83" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U83" t="s">
         <v>29</v>
       </c>
       <c r="V83" s="1">
-        <v>46382</v>
+        <v>46321</v>
       </c>
     </row>
     <row r="84" spans="1:22">
       <c r="A84">
-        <v>64760</v>
+        <v>64340</v>
       </c>
       <c r="B84" t="s">
         <v>22</v>
@@ -4807,42 +5056,42 @@
         <v>22</v>
       </c>
       <c r="D84" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="E84" t="s">
         <v>29</v>
-      </c>
-      <c r="F84" t="s">
-        <v>41</v>
-      </c>
-      <c r="G84" t="s">
-        <v>45</v>
       </c>
       <c r="N84" t="s">
         <v>89</v>
       </c>
       <c r="O84" t="s">
-        <v>89</v>
+        <v>90</v>
+      </c>
+      <c r="P84">
+        <v>4394700</v>
       </c>
       <c r="Q84" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R84" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S84" t="s">
-        <v>41</v>
+        <v>167</v>
       </c>
       <c r="T84" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U84" t="s">
         <v>29</v>
+      </c>
+      <c r="V84" s="1">
+        <v>46382</v>
       </c>
     </row>
     <row r="85" spans="1:22">
       <c r="A85">
-        <v>64780</v>
+        <v>64760</v>
       </c>
       <c r="B85" t="s">
         <v>22</v>
@@ -4863,22 +5112,25 @@
         <v>45</v>
       </c>
       <c r="N85" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="O85" t="s">
-        <v>89</v>
+        <v>90</v>
+      </c>
+      <c r="P85">
+        <v>3306000</v>
       </c>
       <c r="Q85" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R85" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S85" t="s">
         <v>41</v>
       </c>
       <c r="T85" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="U85" t="s">
         <v>29</v>
@@ -4886,45 +5138,95 @@
     </row>
     <row r="86" spans="1:22">
       <c r="A86">
-        <v>64800</v>
+        <v>64780</v>
       </c>
       <c r="B86" t="s">
         <v>22</v>
       </c>
       <c r="C86" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D86" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="E86" t="s">
         <v>29</v>
       </c>
       <c r="F86" t="s">
-        <v>31</v>
+        <v>41</v>
+      </c>
+      <c r="G86" t="s">
+        <v>45</v>
       </c>
       <c r="N86" t="s">
         <v>90</v>
       </c>
       <c r="O86" t="s">
-        <v>157</v>
+        <v>90</v>
+      </c>
+      <c r="P86">
+        <v>3306000</v>
       </c>
       <c r="Q86" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="R86" t="s">
+        <v>163</v>
+      </c>
+      <c r="S86" t="s">
+        <v>41</v>
+      </c>
+      <c r="T86" t="s">
+        <v>171</v>
+      </c>
+      <c r="U86" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="87" spans="1:22">
+      <c r="A87">
+        <v>64800</v>
+      </c>
+      <c r="B87" t="s">
+        <v>22</v>
+      </c>
+      <c r="C87" t="s">
+        <v>24</v>
+      </c>
+      <c r="D87" t="s">
+        <v>25</v>
+      </c>
+      <c r="E87" t="s">
+        <v>29</v>
+      </c>
+      <c r="F87" t="s">
+        <v>31</v>
+      </c>
+      <c r="N87" t="s">
+        <v>91</v>
+      </c>
+      <c r="O87" t="s">
+        <v>158</v>
+      </c>
+      <c r="P87">
+        <v>212577</v>
+      </c>
+      <c r="Q87" t="s">
         <v>161</v>
       </c>
-      <c r="S86" t="s">
-        <v>165</v>
-      </c>
-      <c r="T86" t="s">
-        <v>172</v>
-      </c>
-      <c r="U86" t="s">
+      <c r="R87" t="s">
+        <v>162</v>
+      </c>
+      <c r="S87" t="s">
+        <v>166</v>
+      </c>
+      <c r="T87" t="s">
+        <v>173</v>
+      </c>
+      <c r="U87" t="s">
         <v>30</v>
       </c>
-      <c r="V86" s="1">
+      <c r="V87" s="1">
         <v>46260</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (18/08/2026 08:33)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1116" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1116" uniqueCount="174">
   <si>
     <t>linha</t>
   </si>
@@ -506,9 +506,6 @@
   </si>
   <si>
     <t>339030</t>
-  </si>
-  <si>
-    <t>409052</t>
   </si>
   <si>
     <t>449052</t>
@@ -983,13 +980,13 @@
         <v>162</v>
       </c>
       <c r="S2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U2" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V2" s="1">
         <v>46229</v>
@@ -1030,10 +1027,10 @@
         <v>163</v>
       </c>
       <c r="S3" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U3" t="s">
         <v>29</v>
@@ -1077,10 +1074,10 @@
         <v>162</v>
       </c>
       <c r="S4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T4" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U4" t="s">
         <v>29</v>
@@ -1124,10 +1121,10 @@
         <v>162</v>
       </c>
       <c r="S5" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T5" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U5" t="s">
         <v>29</v>
@@ -1174,10 +1171,10 @@
         <v>162</v>
       </c>
       <c r="S6" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T6" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U6" t="s">
         <v>29</v>
@@ -1230,10 +1227,10 @@
         <v>162</v>
       </c>
       <c r="S7" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T7" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U7" t="s">
         <v>29</v>
@@ -1277,10 +1274,10 @@
         <v>162</v>
       </c>
       <c r="S8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T8" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U8" t="s">
         <v>29</v>
@@ -1324,10 +1321,10 @@
         <v>162</v>
       </c>
       <c r="S9" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T9" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U9" t="s">
         <v>29</v>
@@ -1371,10 +1368,10 @@
         <v>162</v>
       </c>
       <c r="S10" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T10" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U10" t="s">
         <v>29</v>
@@ -1418,10 +1415,10 @@
         <v>162</v>
       </c>
       <c r="S11" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T11" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U11" t="s">
         <v>29</v>
@@ -1477,13 +1474,13 @@
         <v>163</v>
       </c>
       <c r="S12" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T12" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U12" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V12" s="1">
         <v>46079</v>
@@ -1524,13 +1521,13 @@
         <v>163</v>
       </c>
       <c r="S13" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T13" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U13" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V13" s="1">
         <v>46352</v>
@@ -1571,13 +1568,13 @@
         <v>163</v>
       </c>
       <c r="S14" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T14" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U14" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V14" s="1">
         <v>46352</v>
@@ -1618,13 +1615,13 @@
         <v>163</v>
       </c>
       <c r="S15" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T15" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U15" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V15" s="1">
         <v>46352</v>
@@ -1665,13 +1662,13 @@
         <v>163</v>
       </c>
       <c r="S16" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T16" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U16" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V16" s="1">
         <v>46229</v>
@@ -1724,13 +1721,13 @@
         <v>162</v>
       </c>
       <c r="S17" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T17" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="U17" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V17" s="1">
         <v>46107</v>
@@ -1780,10 +1777,10 @@
         <v>163</v>
       </c>
       <c r="S18" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T18" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U18" t="s">
         <v>29</v>
@@ -1836,10 +1833,10 @@
         <v>163</v>
       </c>
       <c r="S19" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T19" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U19" t="s">
         <v>29</v>
@@ -1883,10 +1880,10 @@
         <v>163</v>
       </c>
       <c r="S20" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T20" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U20" t="s">
         <v>29</v>
@@ -1930,10 +1927,10 @@
         <v>163</v>
       </c>
       <c r="S21" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T21" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U21" t="s">
         <v>29</v>
@@ -1977,10 +1974,10 @@
         <v>162</v>
       </c>
       <c r="S22" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T22" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U22" t="s">
         <v>29</v>
@@ -2024,10 +2021,10 @@
         <v>162</v>
       </c>
       <c r="S23" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T23" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U23" t="s">
         <v>29</v>
@@ -2083,13 +2080,13 @@
         <v>162</v>
       </c>
       <c r="S24" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T24" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="U24" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V24" s="1">
         <v>46138</v>
@@ -2139,10 +2136,10 @@
         <v>162</v>
       </c>
       <c r="S25" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T25" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U25" t="s">
         <v>29</v>
@@ -2195,10 +2192,10 @@
         <v>163</v>
       </c>
       <c r="S26" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T26" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U26" t="s">
         <v>29</v>
@@ -2242,13 +2239,13 @@
         <v>163</v>
       </c>
       <c r="S27" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T27" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U27" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V27" s="1">
         <v>46291</v>
@@ -2301,13 +2298,13 @@
         <v>162</v>
       </c>
       <c r="S28" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T28" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U28" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V28" s="1">
         <v>46199</v>
@@ -2360,13 +2357,13 @@
         <v>162</v>
       </c>
       <c r="S29" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T29" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U29" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V29" s="1">
         <v>46199</v>
@@ -2419,13 +2416,13 @@
         <v>162</v>
       </c>
       <c r="S30" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T30" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U30" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V30" s="1">
         <v>46199</v>
@@ -2478,13 +2475,13 @@
         <v>162</v>
       </c>
       <c r="S31" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T31" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U31" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V31" s="1">
         <v>46199</v>
@@ -2525,13 +2522,13 @@
         <v>162</v>
       </c>
       <c r="S32" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T32" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U32" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V32" s="1">
         <v>46291</v>
@@ -2584,13 +2581,13 @@
         <v>162</v>
       </c>
       <c r="S33" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T33" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="U33" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V33" s="1">
         <v>46199</v>
@@ -2640,13 +2637,13 @@
         <v>162</v>
       </c>
       <c r="S34" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T34" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="U34" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V34" s="1">
         <v>46138</v>
@@ -2696,10 +2693,10 @@
         <v>163</v>
       </c>
       <c r="S35" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T35" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U35" t="s">
         <v>29</v>
@@ -2752,10 +2749,10 @@
         <v>162</v>
       </c>
       <c r="S36" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T36" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U36" t="s">
         <v>29</v>
@@ -2808,10 +2805,10 @@
         <v>163</v>
       </c>
       <c r="S37" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T37" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U37" t="s">
         <v>29</v>
@@ -2864,10 +2861,10 @@
         <v>163</v>
       </c>
       <c r="S38" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T38" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U38" t="s">
         <v>29</v>
@@ -2920,10 +2917,10 @@
         <v>163</v>
       </c>
       <c r="S39" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T39" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U39" t="s">
         <v>29</v>
@@ -2976,10 +2973,10 @@
         <v>163</v>
       </c>
       <c r="S40" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T40" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U40" t="s">
         <v>29</v>
@@ -3032,10 +3029,10 @@
         <v>163</v>
       </c>
       <c r="S41" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T41" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U41" t="s">
         <v>29</v>
@@ -3076,10 +3073,10 @@
         <v>163</v>
       </c>
       <c r="S42" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="T42" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U42" t="s">
         <v>29</v>
@@ -3132,10 +3129,10 @@
         <v>163</v>
       </c>
       <c r="S43" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T43" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U43" t="s">
         <v>29</v>
@@ -3188,10 +3185,10 @@
         <v>163</v>
       </c>
       <c r="S44" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T44" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U44" t="s">
         <v>29</v>
@@ -3247,13 +3244,13 @@
         <v>162</v>
       </c>
       <c r="S45" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T45" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="U45" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V45" s="1">
         <v>46229</v>
@@ -3303,13 +3300,13 @@
         <v>162</v>
       </c>
       <c r="S46" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T46" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="U46" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V46" s="1">
         <v>46229</v>
@@ -3350,10 +3347,10 @@
         <v>163</v>
       </c>
       <c r="S47" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T47" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U47" t="s">
         <v>29</v>
@@ -3397,13 +3394,13 @@
         <v>163</v>
       </c>
       <c r="S48" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T48" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U48" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V48" s="1">
         <v>46291</v>
@@ -3456,13 +3453,13 @@
         <v>164</v>
       </c>
       <c r="S49" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T49" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U49" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V49" s="1">
         <v>46199</v>
@@ -3509,13 +3506,13 @@
         <v>162</v>
       </c>
       <c r="S50" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T50" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="U50" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V50" s="1">
         <v>46260</v>
@@ -3562,13 +3559,13 @@
         <v>162</v>
       </c>
       <c r="S51" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T51" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="U51" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V51" s="1">
         <v>46291</v>
@@ -3612,13 +3609,13 @@
         <v>162</v>
       </c>
       <c r="S52" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T52" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="U52" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V52" s="1">
         <v>46321</v>
@@ -3668,13 +3665,13 @@
         <v>162</v>
       </c>
       <c r="S53" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T53" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="U53" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V53" s="1">
         <v>46229</v>
@@ -3715,13 +3712,13 @@
         <v>162</v>
       </c>
       <c r="S54" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T54" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="U54" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V54" s="1">
         <v>46352</v>
@@ -3765,13 +3762,13 @@
         <v>162</v>
       </c>
       <c r="S55" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="T55" t="s">
+        <v>172</v>
+      </c>
+      <c r="U55" t="s">
         <v>173</v>
-      </c>
-      <c r="U55" t="s">
-        <v>174</v>
       </c>
       <c r="V55" s="1">
         <v>46321</v>
@@ -3815,13 +3812,13 @@
         <v>162</v>
       </c>
       <c r="S56" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="T56" t="s">
+        <v>172</v>
+      </c>
+      <c r="U56" t="s">
         <v>173</v>
-      </c>
-      <c r="U56" t="s">
-        <v>174</v>
       </c>
       <c r="V56" s="1">
         <v>46321</v>
@@ -3859,13 +3856,13 @@
         <v>162</v>
       </c>
       <c r="S57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="T57" t="s">
+        <v>172</v>
+      </c>
+      <c r="U57" t="s">
         <v>173</v>
-      </c>
-      <c r="U57" t="s">
-        <v>174</v>
       </c>
       <c r="V57" s="1">
         <v>46049</v>
@@ -3903,13 +3900,13 @@
         <v>162</v>
       </c>
       <c r="S58" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="T58" t="s">
+        <v>172</v>
+      </c>
+      <c r="U58" t="s">
         <v>173</v>
-      </c>
-      <c r="U58" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="59" spans="1:22">
@@ -3944,13 +3941,13 @@
         <v>162</v>
       </c>
       <c r="S59" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="T59" t="s">
+        <v>172</v>
+      </c>
+      <c r="U59" t="s">
         <v>173</v>
-      </c>
-      <c r="U59" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="60" spans="1:22">
@@ -3982,16 +3979,16 @@
         <v>159</v>
       </c>
       <c r="R60" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="S60" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="T60" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U60" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V60" s="1">
         <v>46107</v>
@@ -4026,16 +4023,16 @@
         <v>159</v>
       </c>
       <c r="R61" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="S61" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="T61" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U61" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V61" s="1">
         <v>46107</v>
@@ -4070,16 +4067,16 @@
         <v>159</v>
       </c>
       <c r="R62" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="S62" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="T62" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U62" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V62" s="1">
         <v>46107</v>
@@ -4114,16 +4111,16 @@
         <v>161</v>
       </c>
       <c r="R63" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="S63" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="T63" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U63" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V63" s="1">
         <v>46107</v>
@@ -4158,16 +4155,16 @@
         <v>159</v>
       </c>
       <c r="R64" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="S64" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="T64" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U64" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V64" s="1">
         <v>46107</v>
@@ -4202,16 +4199,16 @@
         <v>160</v>
       </c>
       <c r="R65" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="S65" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="T65" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U65" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V65" s="1">
         <v>46107</v>
@@ -4249,10 +4246,10 @@
         <v>162</v>
       </c>
       <c r="S66" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="T66" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U66" t="s">
         <v>29</v>
@@ -4296,10 +4293,10 @@
         <v>163</v>
       </c>
       <c r="S67" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T67" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U67" t="s">
         <v>29</v>
@@ -4343,13 +4340,13 @@
         <v>163</v>
       </c>
       <c r="S68" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T68" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U68" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V68" s="1">
         <v>46229</v>
@@ -4387,10 +4384,10 @@
         <v>162</v>
       </c>
       <c r="S69" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="T69" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U69" t="s">
         <v>29</v>
@@ -4431,13 +4428,13 @@
         <v>163</v>
       </c>
       <c r="S70" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="T70" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U70" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V70" s="1">
         <v>46291</v>
@@ -4475,13 +4472,13 @@
         <v>163</v>
       </c>
       <c r="S71" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="T71" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U71" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V71" s="1">
         <v>46168</v>
@@ -4519,13 +4516,13 @@
         <v>163</v>
       </c>
       <c r="S72" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="T72" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U72" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V72" s="1">
         <v>46291</v>
@@ -4563,13 +4560,13 @@
         <v>163</v>
       </c>
       <c r="S73" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="T73" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U73" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V73" s="1">
         <v>46291</v>
@@ -4607,13 +4604,13 @@
         <v>163</v>
       </c>
       <c r="S74" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="T74" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U74" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V74" s="1">
         <v>46291</v>
@@ -4654,10 +4651,10 @@
         <v>163</v>
       </c>
       <c r="S75" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T75" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U75" t="s">
         <v>29</v>
@@ -4707,10 +4704,10 @@
         <v>41</v>
       </c>
       <c r="T76" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="U76" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V76" s="1">
         <v>46381</v>
@@ -4757,10 +4754,10 @@
         <v>41</v>
       </c>
       <c r="T77" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="U77" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V77" s="1">
         <v>46381</v>
@@ -4807,7 +4804,7 @@
         <v>41</v>
       </c>
       <c r="T78" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U78" t="s">
         <v>29</v>
@@ -4857,7 +4854,7 @@
         <v>41</v>
       </c>
       <c r="T79" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U79" t="s">
         <v>29</v>
@@ -4898,10 +4895,10 @@
         <v>162</v>
       </c>
       <c r="S80" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="T80" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U80" t="s">
         <v>29</v>
@@ -4942,10 +4939,10 @@
         <v>163</v>
       </c>
       <c r="S81" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="T81" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U81" t="s">
         <v>29</v>
@@ -4989,13 +4986,13 @@
         <v>162</v>
       </c>
       <c r="S82" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T82" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="U82" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="V82" s="1">
         <v>46382</v>
@@ -5033,10 +5030,10 @@
         <v>163</v>
       </c>
       <c r="S83" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="T83" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U83" t="s">
         <v>29</v>
@@ -5077,10 +5074,10 @@
         <v>163</v>
       </c>
       <c r="S84" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="T84" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U84" t="s">
         <v>29</v>
@@ -5130,7 +5127,7 @@
         <v>41</v>
       </c>
       <c r="T85" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U85" t="s">
         <v>29</v>
@@ -5177,7 +5174,7 @@
         <v>41</v>
       </c>
       <c r="T86" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U86" t="s">
         <v>29</v>
@@ -5218,10 +5215,10 @@
         <v>162</v>
       </c>
       <c r="S87" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T87" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="U87" t="s">
         <v>30</v>

</xml_diff>

<commit_message>
Atualização automática: mta (18/08/2026 12:32)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -545,8 +545,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -562,7 +570,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -570,12 +578,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -875,70 +901,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -988,7 +1014,7 @@
       <c r="U2" t="s">
         <v>173</v>
       </c>
-      <c r="V2" s="1">
+      <c r="V2" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -1035,7 +1061,7 @@
       <c r="U3" t="s">
         <v>29</v>
       </c>
-      <c r="V3" s="1">
+      <c r="V3" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1082,7 +1108,7 @@
       <c r="U4" t="s">
         <v>29</v>
       </c>
-      <c r="V4" s="1">
+      <c r="V4" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1129,7 +1155,7 @@
       <c r="U5" t="s">
         <v>29</v>
       </c>
-      <c r="V5" s="1">
+      <c r="V5" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1179,7 +1205,7 @@
       <c r="U6" t="s">
         <v>29</v>
       </c>
-      <c r="V6" s="1">
+      <c r="V6" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1205,7 +1231,7 @@
       <c r="G7" t="s">
         <v>42</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1235,7 +1261,7 @@
       <c r="U7" t="s">
         <v>29</v>
       </c>
-      <c r="V7" s="1">
+      <c r="V7" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -1282,7 +1308,7 @@
       <c r="U8" t="s">
         <v>29</v>
       </c>
-      <c r="V8" s="1">
+      <c r="V8" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1329,7 +1355,7 @@
       <c r="U9" t="s">
         <v>29</v>
       </c>
-      <c r="V9" s="1">
+      <c r="V9" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1376,7 +1402,7 @@
       <c r="U10" t="s">
         <v>29</v>
       </c>
-      <c r="V10" s="1">
+      <c r="V10" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1423,7 +1449,7 @@
       <c r="U11" t="s">
         <v>29</v>
       </c>
-      <c r="V11" s="1">
+      <c r="V11" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1449,7 +1475,7 @@
       <c r="G12" t="s">
         <v>42</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46079</v>
       </c>
       <c r="I12" t="s">
@@ -1482,7 +1508,7 @@
       <c r="U12" t="s">
         <v>173</v>
       </c>
-      <c r="V12" s="1">
+      <c r="V12" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1529,7 +1555,7 @@
       <c r="U13" t="s">
         <v>173</v>
       </c>
-      <c r="V13" s="1">
+      <c r="V13" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1576,7 +1602,7 @@
       <c r="U14" t="s">
         <v>173</v>
       </c>
-      <c r="V14" s="1">
+      <c r="V14" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1623,7 +1649,7 @@
       <c r="U15" t="s">
         <v>173</v>
       </c>
-      <c r="V15" s="1">
+      <c r="V15" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1670,7 +1696,7 @@
       <c r="U16" t="s">
         <v>173</v>
       </c>
-      <c r="V16" s="1">
+      <c r="V16" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -1696,7 +1722,7 @@
       <c r="G17" t="s">
         <v>42</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46098</v>
       </c>
       <c r="I17" t="s">
@@ -1729,7 +1755,7 @@
       <c r="U17" t="s">
         <v>173</v>
       </c>
-      <c r="V17" s="1">
+      <c r="V17" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -1755,7 +1781,7 @@
       <c r="G18" t="s">
         <v>42</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46076</v>
       </c>
       <c r="I18" t="s">
@@ -1785,7 +1811,7 @@
       <c r="U18" t="s">
         <v>29</v>
       </c>
-      <c r="V18" s="1">
+      <c r="V18" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1811,7 +1837,7 @@
       <c r="G19" t="s">
         <v>42</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1841,7 +1867,7 @@
       <c r="U19" t="s">
         <v>29</v>
       </c>
-      <c r="V19" s="1">
+      <c r="V19" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1888,7 +1914,7 @@
       <c r="U20" t="s">
         <v>29</v>
       </c>
-      <c r="V20" s="1">
+      <c r="V20" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1935,7 +1961,7 @@
       <c r="U21" t="s">
         <v>29</v>
       </c>
-      <c r="V21" s="1">
+      <c r="V21" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1982,7 +2008,7 @@
       <c r="U22" t="s">
         <v>29</v>
       </c>
-      <c r="V22" s="1">
+      <c r="V22" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2029,7 +2055,7 @@
       <c r="U23" t="s">
         <v>29</v>
       </c>
-      <c r="V23" s="1">
+      <c r="V23" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2055,7 +2081,7 @@
       <c r="G24" t="s">
         <v>42</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>46119</v>
       </c>
       <c r="I24" t="s">
@@ -2088,7 +2114,7 @@
       <c r="U24" t="s">
         <v>173</v>
       </c>
-      <c r="V24" s="1">
+      <c r="V24" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2114,7 +2140,7 @@
       <c r="G25" t="s">
         <v>42</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>46121</v>
       </c>
       <c r="I25" t="s">
@@ -2144,7 +2170,7 @@
       <c r="U25" t="s">
         <v>29</v>
       </c>
-      <c r="V25" s="1">
+      <c r="V25" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2170,7 +2196,7 @@
       <c r="G26" t="s">
         <v>42</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>46076</v>
       </c>
       <c r="I26" t="s">
@@ -2200,7 +2226,7 @@
       <c r="U26" t="s">
         <v>29</v>
       </c>
-      <c r="V26" s="1">
+      <c r="V26" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -2247,7 +2273,7 @@
       <c r="U27" t="s">
         <v>173</v>
       </c>
-      <c r="V27" s="1">
+      <c r="V27" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -2273,7 +2299,7 @@
       <c r="G28" t="s">
         <v>42</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>46199</v>
       </c>
       <c r="I28" t="s">
@@ -2306,7 +2332,7 @@
       <c r="U28" t="s">
         <v>173</v>
       </c>
-      <c r="V28" s="1">
+      <c r="V28" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2332,7 +2358,7 @@
       <c r="G29" t="s">
         <v>42</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2365,7 +2391,7 @@
       <c r="U29" t="s">
         <v>173</v>
       </c>
-      <c r="V29" s="1">
+      <c r="V29" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2391,7 +2417,7 @@
       <c r="G30" t="s">
         <v>42</v>
       </c>
-      <c r="H30" s="1">
+      <c r="H30" s="2">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2424,7 +2450,7 @@
       <c r="U30" t="s">
         <v>173</v>
       </c>
-      <c r="V30" s="1">
+      <c r="V30" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2450,7 +2476,7 @@
       <c r="G31" t="s">
         <v>42</v>
       </c>
-      <c r="H31" s="1">
+      <c r="H31" s="2">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2483,7 +2509,7 @@
       <c r="U31" t="s">
         <v>173</v>
       </c>
-      <c r="V31" s="1">
+      <c r="V31" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2530,7 +2556,7 @@
       <c r="U32" t="s">
         <v>173</v>
       </c>
-      <c r="V32" s="1">
+      <c r="V32" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -2556,7 +2582,7 @@
       <c r="G33" t="s">
         <v>42</v>
       </c>
-      <c r="H33" s="1">
+      <c r="H33" s="2">
         <v>46191</v>
       </c>
       <c r="I33" t="s">
@@ -2589,7 +2615,7 @@
       <c r="U33" t="s">
         <v>173</v>
       </c>
-      <c r="V33" s="1">
+      <c r="V33" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2615,7 +2641,7 @@
       <c r="G34" t="s">
         <v>42</v>
       </c>
-      <c r="H34" s="1">
+      <c r="H34" s="2">
         <v>46119</v>
       </c>
       <c r="I34" t="s">
@@ -2645,7 +2671,7 @@
       <c r="U34" t="s">
         <v>173</v>
       </c>
-      <c r="V34" s="1">
+      <c r="V34" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2671,7 +2697,7 @@
       <c r="G35" t="s">
         <v>42</v>
       </c>
-      <c r="H35" s="1">
+      <c r="H35" s="2">
         <v>46213</v>
       </c>
       <c r="I35" t="s">
@@ -2701,7 +2727,7 @@
       <c r="U35" t="s">
         <v>29</v>
       </c>
-      <c r="V35" s="1">
+      <c r="V35" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -2727,7 +2753,7 @@
       <c r="G36" t="s">
         <v>42</v>
       </c>
-      <c r="H36" s="1">
+      <c r="H36" s="2">
         <v>46175</v>
       </c>
       <c r="I36" t="s">
@@ -2757,7 +2783,7 @@
       <c r="U36" t="s">
         <v>29</v>
       </c>
-      <c r="V36" s="1">
+      <c r="V36" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2783,7 +2809,7 @@
       <c r="G37" t="s">
         <v>42</v>
       </c>
-      <c r="H37" s="1">
+      <c r="H37" s="2">
         <v>46213</v>
       </c>
       <c r="I37" t="s">
@@ -2813,7 +2839,7 @@
       <c r="U37" t="s">
         <v>29</v>
       </c>
-      <c r="V37" s="1">
+      <c r="V37" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -2839,7 +2865,7 @@
       <c r="G38" t="s">
         <v>42</v>
       </c>
-      <c r="H38" s="1">
+      <c r="H38" s="2">
         <v>46199</v>
       </c>
       <c r="I38" t="s">
@@ -2869,7 +2895,7 @@
       <c r="U38" t="s">
         <v>29</v>
       </c>
-      <c r="V38" s="1">
+      <c r="V38" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2895,7 +2921,7 @@
       <c r="G39" t="s">
         <v>42</v>
       </c>
-      <c r="H39" s="1">
+      <c r="H39" s="2">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -2925,7 +2951,7 @@
       <c r="U39" t="s">
         <v>29</v>
       </c>
-      <c r="V39" s="1">
+      <c r="V39" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2951,7 +2977,7 @@
       <c r="G40" t="s">
         <v>42</v>
       </c>
-      <c r="H40" s="1">
+      <c r="H40" s="2">
         <v>46204</v>
       </c>
       <c r="I40" t="s">
@@ -2981,7 +3007,7 @@
       <c r="U40" t="s">
         <v>29</v>
       </c>
-      <c r="V40" s="1">
+      <c r="V40" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3007,7 +3033,7 @@
       <c r="G41" t="s">
         <v>42</v>
       </c>
-      <c r="H41" s="1">
+      <c r="H41" s="2">
         <v>46244</v>
       </c>
       <c r="I41" t="s">
@@ -3037,7 +3063,7 @@
       <c r="U41" t="s">
         <v>29</v>
       </c>
-      <c r="V41" s="1">
+      <c r="V41" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3081,7 +3107,7 @@
       <c r="U42" t="s">
         <v>29</v>
       </c>
-      <c r="V42" s="1">
+      <c r="V42" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3107,7 +3133,7 @@
       <c r="G43" t="s">
         <v>42</v>
       </c>
-      <c r="H43" s="1">
+      <c r="H43" s="2">
         <v>46191</v>
       </c>
       <c r="I43" t="s">
@@ -3137,7 +3163,7 @@
       <c r="U43" t="s">
         <v>29</v>
       </c>
-      <c r="V43" s="1">
+      <c r="V43" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3163,7 +3189,7 @@
       <c r="G44" t="s">
         <v>42</v>
       </c>
-      <c r="H44" s="1">
+      <c r="H44" s="2">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
@@ -3193,7 +3219,7 @@
       <c r="U44" t="s">
         <v>29</v>
       </c>
-      <c r="V44" s="1">
+      <c r="V44" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3219,7 +3245,7 @@
       <c r="G45" t="s">
         <v>42</v>
       </c>
-      <c r="H45" s="1">
+      <c r="H45" s="2">
         <v>46213</v>
       </c>
       <c r="I45" t="s">
@@ -3252,7 +3278,7 @@
       <c r="U45" t="s">
         <v>173</v>
       </c>
-      <c r="V45" s="1">
+      <c r="V45" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3278,7 +3304,7 @@
       <c r="G46" t="s">
         <v>42</v>
       </c>
-      <c r="H46" s="1">
+      <c r="H46" s="2">
         <v>46210</v>
       </c>
       <c r="I46" t="s">
@@ -3308,7 +3334,7 @@
       <c r="U46" t="s">
         <v>173</v>
       </c>
-      <c r="V46" s="1">
+      <c r="V46" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3355,7 +3381,7 @@
       <c r="U47" t="s">
         <v>29</v>
       </c>
-      <c r="V47" s="1">
+      <c r="V47" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3402,7 +3428,7 @@
       <c r="U48" t="s">
         <v>173</v>
       </c>
-      <c r="V48" s="1">
+      <c r="V48" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3428,7 +3454,7 @@
       <c r="G49" t="s">
         <v>42</v>
       </c>
-      <c r="H49" s="1">
+      <c r="H49" s="2">
         <v>46176</v>
       </c>
       <c r="I49" t="s">
@@ -3461,7 +3487,7 @@
       <c r="U49" t="s">
         <v>173</v>
       </c>
-      <c r="V49" s="1">
+      <c r="V49" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3514,7 +3540,7 @@
       <c r="U50" t="s">
         <v>173</v>
       </c>
-      <c r="V50" s="1">
+      <c r="V50" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3567,7 +3593,7 @@
       <c r="U51" t="s">
         <v>173</v>
       </c>
-      <c r="V51" s="1">
+      <c r="V51" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3617,7 +3643,7 @@
       <c r="U52" t="s">
         <v>173</v>
       </c>
-      <c r="V52" s="1">
+      <c r="V52" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3643,7 +3669,7 @@
       <c r="G53" t="s">
         <v>42</v>
       </c>
-      <c r="H53" s="1">
+      <c r="H53" s="2">
         <v>46227</v>
       </c>
       <c r="I53" t="s">
@@ -3673,7 +3699,7 @@
       <c r="U53" t="s">
         <v>173</v>
       </c>
-      <c r="V53" s="1">
+      <c r="V53" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3720,7 +3746,7 @@
       <c r="U54" t="s">
         <v>173</v>
       </c>
-      <c r="V54" s="1">
+      <c r="V54" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -3770,7 +3796,7 @@
       <c r="U55" t="s">
         <v>173</v>
       </c>
-      <c r="V55" s="1">
+      <c r="V55" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3820,7 +3846,7 @@
       <c r="U56" t="s">
         <v>173</v>
       </c>
-      <c r="V56" s="1">
+      <c r="V56" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3864,7 +3890,7 @@
       <c r="U57" t="s">
         <v>173</v>
       </c>
-      <c r="V57" s="1">
+      <c r="V57" s="2">
         <v>46049</v>
       </c>
     </row>
@@ -3990,7 +4016,7 @@
       <c r="U60" t="s">
         <v>173</v>
       </c>
-      <c r="V60" s="1">
+      <c r="V60" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4034,7 +4060,7 @@
       <c r="U61" t="s">
         <v>173</v>
       </c>
-      <c r="V61" s="1">
+      <c r="V61" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4078,7 +4104,7 @@
       <c r="U62" t="s">
         <v>173</v>
       </c>
-      <c r="V62" s="1">
+      <c r="V62" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4122,7 +4148,7 @@
       <c r="U63" t="s">
         <v>173</v>
       </c>
-      <c r="V63" s="1">
+      <c r="V63" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4166,7 +4192,7 @@
       <c r="U64" t="s">
         <v>173</v>
       </c>
-      <c r="V64" s="1">
+      <c r="V64" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4210,7 +4236,7 @@
       <c r="U65" t="s">
         <v>173</v>
       </c>
-      <c r="V65" s="1">
+      <c r="V65" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4254,7 +4280,7 @@
       <c r="U66" t="s">
         <v>29</v>
       </c>
-      <c r="V66" s="1">
+      <c r="V66" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4301,7 +4327,7 @@
       <c r="U67" t="s">
         <v>29</v>
       </c>
-      <c r="V67" s="1">
+      <c r="V67" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4348,7 +4374,7 @@
       <c r="U68" t="s">
         <v>173</v>
       </c>
-      <c r="V68" s="1">
+      <c r="V68" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -4392,7 +4418,7 @@
       <c r="U69" t="s">
         <v>29</v>
       </c>
-      <c r="V69" s="1">
+      <c r="V69" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -4436,7 +4462,7 @@
       <c r="U70" t="s">
         <v>173</v>
       </c>
-      <c r="V70" s="1">
+      <c r="V70" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4480,7 +4506,7 @@
       <c r="U71" t="s">
         <v>173</v>
       </c>
-      <c r="V71" s="1">
+      <c r="V71" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4524,7 +4550,7 @@
       <c r="U72" t="s">
         <v>173</v>
       </c>
-      <c r="V72" s="1">
+      <c r="V72" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4568,7 +4594,7 @@
       <c r="U73" t="s">
         <v>173</v>
       </c>
-      <c r="V73" s="1">
+      <c r="V73" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4612,7 +4638,7 @@
       <c r="U74" t="s">
         <v>173</v>
       </c>
-      <c r="V74" s="1">
+      <c r="V74" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4659,7 +4685,7 @@
       <c r="U75" t="s">
         <v>29</v>
       </c>
-      <c r="V75" s="1">
+      <c r="V75" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -4709,7 +4735,7 @@
       <c r="U76" t="s">
         <v>173</v>
       </c>
-      <c r="V76" s="1">
+      <c r="V76" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4759,7 +4785,7 @@
       <c r="U77" t="s">
         <v>173</v>
       </c>
-      <c r="V77" s="1">
+      <c r="V77" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4809,7 +4835,7 @@
       <c r="U78" t="s">
         <v>29</v>
       </c>
-      <c r="V78" s="1">
+      <c r="V78" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4859,7 +4885,7 @@
       <c r="U79" t="s">
         <v>29</v>
       </c>
-      <c r="V79" s="1">
+      <c r="V79" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4903,7 +4929,7 @@
       <c r="U80" t="s">
         <v>29</v>
       </c>
-      <c r="V80" s="1">
+      <c r="V80" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -4947,7 +4973,7 @@
       <c r="U81" t="s">
         <v>29</v>
       </c>
-      <c r="V81" s="1">
+      <c r="V81" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -4994,7 +5020,7 @@
       <c r="U82" t="s">
         <v>173</v>
       </c>
-      <c r="V82" s="1">
+      <c r="V82" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5038,7 +5064,7 @@
       <c r="U83" t="s">
         <v>29</v>
       </c>
-      <c r="V83" s="1">
+      <c r="V83" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -5082,7 +5108,7 @@
       <c r="U84" t="s">
         <v>29</v>
       </c>
-      <c r="V84" s="1">
+      <c r="V84" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5223,7 +5249,7 @@
       <c r="U87" t="s">
         <v>30</v>
       </c>
-      <c r="V87" s="1">
+      <c r="V87" s="2">
         <v>46260</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (18/08/2026 12:40)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -545,16 +545,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -570,7 +562,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -578,30 +570,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -901,70 +875,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1014,7 +988,7 @@
       <c r="U2" t="s">
         <v>173</v>
       </c>
-      <c r="V2" s="2">
+      <c r="V2" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1061,7 +1035,7 @@
       <c r="U3" t="s">
         <v>29</v>
       </c>
-      <c r="V3" s="2">
+      <c r="V3" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1108,7 +1082,7 @@
       <c r="U4" t="s">
         <v>29</v>
       </c>
-      <c r="V4" s="2">
+      <c r="V4" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1155,7 +1129,7 @@
       <c r="U5" t="s">
         <v>29</v>
       </c>
-      <c r="V5" s="2">
+      <c r="V5" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1205,7 +1179,7 @@
       <c r="U6" t="s">
         <v>29</v>
       </c>
-      <c r="V6" s="2">
+      <c r="V6" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1231,7 +1205,7 @@
       <c r="G7" t="s">
         <v>42</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1261,7 +1235,7 @@
       <c r="U7" t="s">
         <v>29</v>
       </c>
-      <c r="V7" s="2">
+      <c r="V7" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -1308,7 +1282,7 @@
       <c r="U8" t="s">
         <v>29</v>
       </c>
-      <c r="V8" s="2">
+      <c r="V8" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1355,7 +1329,7 @@
       <c r="U9" t="s">
         <v>29</v>
       </c>
-      <c r="V9" s="2">
+      <c r="V9" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1402,7 +1376,7 @@
       <c r="U10" t="s">
         <v>29</v>
       </c>
-      <c r="V10" s="2">
+      <c r="V10" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1449,7 +1423,7 @@
       <c r="U11" t="s">
         <v>29</v>
       </c>
-      <c r="V11" s="2">
+      <c r="V11" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1475,7 +1449,7 @@
       <c r="G12" t="s">
         <v>42</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46079</v>
       </c>
       <c r="I12" t="s">
@@ -1508,7 +1482,7 @@
       <c r="U12" t="s">
         <v>173</v>
       </c>
-      <c r="V12" s="2">
+      <c r="V12" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1555,7 +1529,7 @@
       <c r="U13" t="s">
         <v>173</v>
       </c>
-      <c r="V13" s="2">
+      <c r="V13" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1602,7 +1576,7 @@
       <c r="U14" t="s">
         <v>173</v>
       </c>
-      <c r="V14" s="2">
+      <c r="V14" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1649,7 +1623,7 @@
       <c r="U15" t="s">
         <v>173</v>
       </c>
-      <c r="V15" s="2">
+      <c r="V15" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1696,7 +1670,7 @@
       <c r="U16" t="s">
         <v>173</v>
       </c>
-      <c r="V16" s="2">
+      <c r="V16" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1722,7 +1696,7 @@
       <c r="G17" t="s">
         <v>42</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46098</v>
       </c>
       <c r="I17" t="s">
@@ -1755,7 +1729,7 @@
       <c r="U17" t="s">
         <v>173</v>
       </c>
-      <c r="V17" s="2">
+      <c r="V17" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -1781,7 +1755,7 @@
       <c r="G18" t="s">
         <v>42</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46076</v>
       </c>
       <c r="I18" t="s">
@@ -1811,7 +1785,7 @@
       <c r="U18" t="s">
         <v>29</v>
       </c>
-      <c r="V18" s="2">
+      <c r="V18" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1837,7 +1811,7 @@
       <c r="G19" t="s">
         <v>42</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1867,7 +1841,7 @@
       <c r="U19" t="s">
         <v>29</v>
       </c>
-      <c r="V19" s="2">
+      <c r="V19" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1914,7 +1888,7 @@
       <c r="U20" t="s">
         <v>29</v>
       </c>
-      <c r="V20" s="2">
+      <c r="V20" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1961,7 +1935,7 @@
       <c r="U21" t="s">
         <v>29</v>
       </c>
-      <c r="V21" s="2">
+      <c r="V21" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2008,7 +1982,7 @@
       <c r="U22" t="s">
         <v>29</v>
       </c>
-      <c r="V22" s="2">
+      <c r="V22" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2055,7 +2029,7 @@
       <c r="U23" t="s">
         <v>29</v>
       </c>
-      <c r="V23" s="2">
+      <c r="V23" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2081,7 +2055,7 @@
       <c r="G24" t="s">
         <v>42</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>46119</v>
       </c>
       <c r="I24" t="s">
@@ -2114,7 +2088,7 @@
       <c r="U24" t="s">
         <v>173</v>
       </c>
-      <c r="V24" s="2">
+      <c r="V24" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2140,7 +2114,7 @@
       <c r="G25" t="s">
         <v>42</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>46121</v>
       </c>
       <c r="I25" t="s">
@@ -2170,7 +2144,7 @@
       <c r="U25" t="s">
         <v>29</v>
       </c>
-      <c r="V25" s="2">
+      <c r="V25" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2196,7 +2170,7 @@
       <c r="G26" t="s">
         <v>42</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>46076</v>
       </c>
       <c r="I26" t="s">
@@ -2226,7 +2200,7 @@
       <c r="U26" t="s">
         <v>29</v>
       </c>
-      <c r="V26" s="2">
+      <c r="V26" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -2273,7 +2247,7 @@
       <c r="U27" t="s">
         <v>173</v>
       </c>
-      <c r="V27" s="2">
+      <c r="V27" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2299,7 +2273,7 @@
       <c r="G28" t="s">
         <v>42</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>46199</v>
       </c>
       <c r="I28" t="s">
@@ -2332,7 +2306,7 @@
       <c r="U28" t="s">
         <v>173</v>
       </c>
-      <c r="V28" s="2">
+      <c r="V28" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2358,7 +2332,7 @@
       <c r="G29" t="s">
         <v>42</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2391,7 +2365,7 @@
       <c r="U29" t="s">
         <v>173</v>
       </c>
-      <c r="V29" s="2">
+      <c r="V29" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2417,7 +2391,7 @@
       <c r="G30" t="s">
         <v>42</v>
       </c>
-      <c r="H30" s="2">
+      <c r="H30" s="1">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2450,7 +2424,7 @@
       <c r="U30" t="s">
         <v>173</v>
       </c>
-      <c r="V30" s="2">
+      <c r="V30" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2476,7 +2450,7 @@
       <c r="G31" t="s">
         <v>42</v>
       </c>
-      <c r="H31" s="2">
+      <c r="H31" s="1">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2509,7 +2483,7 @@
       <c r="U31" t="s">
         <v>173</v>
       </c>
-      <c r="V31" s="2">
+      <c r="V31" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2556,7 +2530,7 @@
       <c r="U32" t="s">
         <v>173</v>
       </c>
-      <c r="V32" s="2">
+      <c r="V32" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2582,7 +2556,7 @@
       <c r="G33" t="s">
         <v>42</v>
       </c>
-      <c r="H33" s="2">
+      <c r="H33" s="1">
         <v>46191</v>
       </c>
       <c r="I33" t="s">
@@ -2615,7 +2589,7 @@
       <c r="U33" t="s">
         <v>173</v>
       </c>
-      <c r="V33" s="2">
+      <c r="V33" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2641,7 +2615,7 @@
       <c r="G34" t="s">
         <v>42</v>
       </c>
-      <c r="H34" s="2">
+      <c r="H34" s="1">
         <v>46119</v>
       </c>
       <c r="I34" t="s">
@@ -2671,7 +2645,7 @@
       <c r="U34" t="s">
         <v>173</v>
       </c>
-      <c r="V34" s="2">
+      <c r="V34" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2697,7 +2671,7 @@
       <c r="G35" t="s">
         <v>42</v>
       </c>
-      <c r="H35" s="2">
+      <c r="H35" s="1">
         <v>46213</v>
       </c>
       <c r="I35" t="s">
@@ -2727,7 +2701,7 @@
       <c r="U35" t="s">
         <v>29</v>
       </c>
-      <c r="V35" s="2">
+      <c r="V35" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -2753,7 +2727,7 @@
       <c r="G36" t="s">
         <v>42</v>
       </c>
-      <c r="H36" s="2">
+      <c r="H36" s="1">
         <v>46175</v>
       </c>
       <c r="I36" t="s">
@@ -2783,7 +2757,7 @@
       <c r="U36" t="s">
         <v>29</v>
       </c>
-      <c r="V36" s="2">
+      <c r="V36" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2809,7 +2783,7 @@
       <c r="G37" t="s">
         <v>42</v>
       </c>
-      <c r="H37" s="2">
+      <c r="H37" s="1">
         <v>46213</v>
       </c>
       <c r="I37" t="s">
@@ -2839,7 +2813,7 @@
       <c r="U37" t="s">
         <v>29</v>
       </c>
-      <c r="V37" s="2">
+      <c r="V37" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -2865,7 +2839,7 @@
       <c r="G38" t="s">
         <v>42</v>
       </c>
-      <c r="H38" s="2">
+      <c r="H38" s="1">
         <v>46199</v>
       </c>
       <c r="I38" t="s">
@@ -2895,7 +2869,7 @@
       <c r="U38" t="s">
         <v>29</v>
       </c>
-      <c r="V38" s="2">
+      <c r="V38" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2921,7 +2895,7 @@
       <c r="G39" t="s">
         <v>42</v>
       </c>
-      <c r="H39" s="2">
+      <c r="H39" s="1">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -2951,7 +2925,7 @@
       <c r="U39" t="s">
         <v>29</v>
       </c>
-      <c r="V39" s="2">
+      <c r="V39" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2977,7 +2951,7 @@
       <c r="G40" t="s">
         <v>42</v>
       </c>
-      <c r="H40" s="2">
+      <c r="H40" s="1">
         <v>46204</v>
       </c>
       <c r="I40" t="s">
@@ -3007,7 +2981,7 @@
       <c r="U40" t="s">
         <v>29</v>
       </c>
-      <c r="V40" s="2">
+      <c r="V40" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3033,7 +3007,7 @@
       <c r="G41" t="s">
         <v>42</v>
       </c>
-      <c r="H41" s="2">
+      <c r="H41" s="1">
         <v>46244</v>
       </c>
       <c r="I41" t="s">
@@ -3063,7 +3037,7 @@
       <c r="U41" t="s">
         <v>29</v>
       </c>
-      <c r="V41" s="2">
+      <c r="V41" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3107,7 +3081,7 @@
       <c r="U42" t="s">
         <v>29</v>
       </c>
-      <c r="V42" s="2">
+      <c r="V42" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3133,7 +3107,7 @@
       <c r="G43" t="s">
         <v>42</v>
       </c>
-      <c r="H43" s="2">
+      <c r="H43" s="1">
         <v>46191</v>
       </c>
       <c r="I43" t="s">
@@ -3163,7 +3137,7 @@
       <c r="U43" t="s">
         <v>29</v>
       </c>
-      <c r="V43" s="2">
+      <c r="V43" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3189,7 +3163,7 @@
       <c r="G44" t="s">
         <v>42</v>
       </c>
-      <c r="H44" s="2">
+      <c r="H44" s="1">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
@@ -3219,7 +3193,7 @@
       <c r="U44" t="s">
         <v>29</v>
       </c>
-      <c r="V44" s="2">
+      <c r="V44" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3245,7 +3219,7 @@
       <c r="G45" t="s">
         <v>42</v>
       </c>
-      <c r="H45" s="2">
+      <c r="H45" s="1">
         <v>46213</v>
       </c>
       <c r="I45" t="s">
@@ -3278,7 +3252,7 @@
       <c r="U45" t="s">
         <v>173</v>
       </c>
-      <c r="V45" s="2">
+      <c r="V45" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3304,7 +3278,7 @@
       <c r="G46" t="s">
         <v>42</v>
       </c>
-      <c r="H46" s="2">
+      <c r="H46" s="1">
         <v>46210</v>
       </c>
       <c r="I46" t="s">
@@ -3334,7 +3308,7 @@
       <c r="U46" t="s">
         <v>173</v>
       </c>
-      <c r="V46" s="2">
+      <c r="V46" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3381,7 +3355,7 @@
       <c r="U47" t="s">
         <v>29</v>
       </c>
-      <c r="V47" s="2">
+      <c r="V47" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3428,7 +3402,7 @@
       <c r="U48" t="s">
         <v>173</v>
       </c>
-      <c r="V48" s="2">
+      <c r="V48" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3454,7 +3428,7 @@
       <c r="G49" t="s">
         <v>42</v>
       </c>
-      <c r="H49" s="2">
+      <c r="H49" s="1">
         <v>46176</v>
       </c>
       <c r="I49" t="s">
@@ -3487,7 +3461,7 @@
       <c r="U49" t="s">
         <v>173</v>
       </c>
-      <c r="V49" s="2">
+      <c r="V49" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3540,7 +3514,7 @@
       <c r="U50" t="s">
         <v>173</v>
       </c>
-      <c r="V50" s="2">
+      <c r="V50" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3593,7 +3567,7 @@
       <c r="U51" t="s">
         <v>173</v>
       </c>
-      <c r="V51" s="2">
+      <c r="V51" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3643,7 +3617,7 @@
       <c r="U52" t="s">
         <v>173</v>
       </c>
-      <c r="V52" s="2">
+      <c r="V52" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3669,7 +3643,7 @@
       <c r="G53" t="s">
         <v>42</v>
       </c>
-      <c r="H53" s="2">
+      <c r="H53" s="1">
         <v>46227</v>
       </c>
       <c r="I53" t="s">
@@ -3699,7 +3673,7 @@
       <c r="U53" t="s">
         <v>173</v>
       </c>
-      <c r="V53" s="2">
+      <c r="V53" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3746,7 +3720,7 @@
       <c r="U54" t="s">
         <v>173</v>
       </c>
-      <c r="V54" s="2">
+      <c r="V54" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -3796,7 +3770,7 @@
       <c r="U55" t="s">
         <v>173</v>
       </c>
-      <c r="V55" s="2">
+      <c r="V55" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3846,7 +3820,7 @@
       <c r="U56" t="s">
         <v>173</v>
       </c>
-      <c r="V56" s="2">
+      <c r="V56" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3890,7 +3864,7 @@
       <c r="U57" t="s">
         <v>173</v>
       </c>
-      <c r="V57" s="2">
+      <c r="V57" s="1">
         <v>46049</v>
       </c>
     </row>
@@ -4016,7 +3990,7 @@
       <c r="U60" t="s">
         <v>173</v>
       </c>
-      <c r="V60" s="2">
+      <c r="V60" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4060,7 +4034,7 @@
       <c r="U61" t="s">
         <v>173</v>
       </c>
-      <c r="V61" s="2">
+      <c r="V61" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4104,7 +4078,7 @@
       <c r="U62" t="s">
         <v>173</v>
       </c>
-      <c r="V62" s="2">
+      <c r="V62" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4148,7 +4122,7 @@
       <c r="U63" t="s">
         <v>173</v>
       </c>
-      <c r="V63" s="2">
+      <c r="V63" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4192,7 +4166,7 @@
       <c r="U64" t="s">
         <v>173</v>
       </c>
-      <c r="V64" s="2">
+      <c r="V64" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4236,7 +4210,7 @@
       <c r="U65" t="s">
         <v>173</v>
       </c>
-      <c r="V65" s="2">
+      <c r="V65" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4280,7 +4254,7 @@
       <c r="U66" t="s">
         <v>29</v>
       </c>
-      <c r="V66" s="2">
+      <c r="V66" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4327,7 +4301,7 @@
       <c r="U67" t="s">
         <v>29</v>
       </c>
-      <c r="V67" s="2">
+      <c r="V67" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4374,7 +4348,7 @@
       <c r="U68" t="s">
         <v>173</v>
       </c>
-      <c r="V68" s="2">
+      <c r="V68" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -4418,7 +4392,7 @@
       <c r="U69" t="s">
         <v>29</v>
       </c>
-      <c r="V69" s="2">
+      <c r="V69" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -4462,7 +4436,7 @@
       <c r="U70" t="s">
         <v>173</v>
       </c>
-      <c r="V70" s="2">
+      <c r="V70" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4506,7 +4480,7 @@
       <c r="U71" t="s">
         <v>173</v>
       </c>
-      <c r="V71" s="2">
+      <c r="V71" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4550,7 +4524,7 @@
       <c r="U72" t="s">
         <v>173</v>
       </c>
-      <c r="V72" s="2">
+      <c r="V72" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4594,7 +4568,7 @@
       <c r="U73" t="s">
         <v>173</v>
       </c>
-      <c r="V73" s="2">
+      <c r="V73" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4638,7 +4612,7 @@
       <c r="U74" t="s">
         <v>173</v>
       </c>
-      <c r="V74" s="2">
+      <c r="V74" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4685,7 +4659,7 @@
       <c r="U75" t="s">
         <v>29</v>
       </c>
-      <c r="V75" s="2">
+      <c r="V75" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -4735,7 +4709,7 @@
       <c r="U76" t="s">
         <v>173</v>
       </c>
-      <c r="V76" s="2">
+      <c r="V76" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4785,7 +4759,7 @@
       <c r="U77" t="s">
         <v>173</v>
       </c>
-      <c r="V77" s="2">
+      <c r="V77" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4835,7 +4809,7 @@
       <c r="U78" t="s">
         <v>29</v>
       </c>
-      <c r="V78" s="2">
+      <c r="V78" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4885,7 +4859,7 @@
       <c r="U79" t="s">
         <v>29</v>
       </c>
-      <c r="V79" s="2">
+      <c r="V79" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4929,7 +4903,7 @@
       <c r="U80" t="s">
         <v>29</v>
       </c>
-      <c r="V80" s="2">
+      <c r="V80" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -4973,7 +4947,7 @@
       <c r="U81" t="s">
         <v>29</v>
       </c>
-      <c r="V81" s="2">
+      <c r="V81" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5020,7 +4994,7 @@
       <c r="U82" t="s">
         <v>173</v>
       </c>
-      <c r="V82" s="2">
+      <c r="V82" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5064,7 +5038,7 @@
       <c r="U83" t="s">
         <v>29</v>
       </c>
-      <c r="V83" s="2">
+      <c r="V83" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -5108,7 +5082,7 @@
       <c r="U84" t="s">
         <v>29</v>
       </c>
-      <c r="V84" s="2">
+      <c r="V84" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5249,7 +5223,7 @@
       <c r="U87" t="s">
         <v>30</v>
       </c>
-      <c r="V87" s="2">
+      <c r="V87" s="1">
         <v>46260</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (18/08/2026 14:35)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1116" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1118" uniqueCount="176">
   <si>
     <t>linha</t>
   </si>
@@ -223,6 +223,9 @@
     <t>email do dia 24/04</t>
   </si>
   <si>
+    <t>e-mail 12/08</t>
+  </si>
+  <si>
     <t>Atender AGO</t>
   </si>
   <si>
@@ -230,6 +233,9 @@
   </si>
   <si>
     <t>Atender OUT</t>
+  </si>
+  <si>
+    <t>ATENDER com 20XV</t>
   </si>
   <si>
     <t>LIVRE</t>
@@ -962,31 +968,31 @@
         <v>31</v>
       </c>
       <c r="L2" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="N2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="O2" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="P2">
         <v>135000</v>
       </c>
       <c r="Q2" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="R2" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="S2" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T2" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="U2" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="V2" s="1">
         <v>46229</v>
@@ -1012,25 +1018,25 @@
         <v>31</v>
       </c>
       <c r="N3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="O3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="P3">
         <v>400000</v>
       </c>
       <c r="Q3" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="R3" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="S3" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T3" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="U3" t="s">
         <v>29</v>
@@ -1059,25 +1065,25 @@
         <v>31</v>
       </c>
       <c r="N4" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="O4" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="P4">
         <v>430000</v>
       </c>
       <c r="Q4" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="R4" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="S4" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T4" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="U4" t="s">
         <v>29</v>
@@ -1106,25 +1112,25 @@
         <v>31</v>
       </c>
       <c r="N5" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="O5" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="P5">
         <v>425000</v>
       </c>
       <c r="Q5" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="R5" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="S5" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T5" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="U5" t="s">
         <v>29</v>
@@ -1153,28 +1159,28 @@
         <v>31</v>
       </c>
       <c r="L6" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="N6" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="O6" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="P6">
         <v>563000</v>
       </c>
       <c r="Q6" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="R6" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="S6" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T6" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="U6" t="s">
         <v>29</v>
@@ -1212,25 +1218,25 @@
         <v>46</v>
       </c>
       <c r="N7" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="O7" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="P7">
         <v>3799999.6</v>
       </c>
       <c r="Q7" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R7" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="S7" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T7" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="U7" t="s">
         <v>29</v>
@@ -1259,25 +1265,25 @@
         <v>31</v>
       </c>
       <c r="N8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="O8" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="P8">
         <v>430000</v>
       </c>
       <c r="Q8" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="R8" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="S8" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T8" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="U8" t="s">
         <v>29</v>
@@ -1306,25 +1312,25 @@
         <v>31</v>
       </c>
       <c r="N9" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="O9" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="P9">
         <v>60000</v>
       </c>
       <c r="Q9" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="R9" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="S9" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T9" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="U9" t="s">
         <v>29</v>
@@ -1353,25 +1359,25 @@
         <v>31</v>
       </c>
       <c r="N10" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="O10" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="P10">
         <v>200000</v>
       </c>
       <c r="Q10" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="R10" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="S10" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T10" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="U10" t="s">
         <v>29</v>
@@ -1400,25 +1406,25 @@
         <v>31</v>
       </c>
       <c r="N11" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="O11" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="P11">
         <v>320000</v>
       </c>
       <c r="Q11" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="R11" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="S11" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T11" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="U11" t="s">
         <v>29</v>
@@ -1459,28 +1465,28 @@
         <v>63</v>
       </c>
       <c r="N12" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="O12" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="P12">
         <v>1187433.02</v>
       </c>
       <c r="Q12" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="R12" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="S12" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T12" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="U12" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="V12" s="1">
         <v>46079</v>
@@ -1506,28 +1512,28 @@
         <v>31</v>
       </c>
       <c r="N13" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="O13" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="P13">
         <v>1000000</v>
       </c>
       <c r="Q13" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="R13" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="S13" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T13" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="U13" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="V13" s="1">
         <v>46352</v>
@@ -1553,28 +1559,28 @@
         <v>31</v>
       </c>
       <c r="N14" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="O14" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="P14">
         <v>1000000</v>
       </c>
       <c r="Q14" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="R14" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="S14" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T14" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="U14" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="V14" s="1">
         <v>46352</v>
@@ -1600,28 +1606,28 @@
         <v>31</v>
       </c>
       <c r="N15" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="O15" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="P15">
         <v>1000000</v>
       </c>
       <c r="Q15" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="R15" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="S15" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T15" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="U15" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="V15" s="1">
         <v>46352</v>
@@ -1647,28 +1653,28 @@
         <v>31</v>
       </c>
       <c r="N16" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="O16" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="P16">
         <v>100000</v>
       </c>
       <c r="Q16" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="R16" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="S16" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T16" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="U16" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="V16" s="1">
         <v>46229</v>
@@ -1706,28 +1712,28 @@
         <v>63</v>
       </c>
       <c r="N17" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="O17" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="P17">
         <v>1770880.5</v>
       </c>
       <c r="Q17" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R17" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="S17" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T17" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="U17" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="V17" s="1">
         <v>46107</v>
@@ -1762,25 +1768,25 @@
         <v>49</v>
       </c>
       <c r="N18" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="O18" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="P18">
         <v>350000</v>
       </c>
       <c r="Q18" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R18" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="S18" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T18" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="U18" t="s">
         <v>29</v>
@@ -1818,25 +1824,25 @@
         <v>49</v>
       </c>
       <c r="N19" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="O19" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="P19">
         <v>350000</v>
       </c>
       <c r="Q19" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R19" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="S19" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T19" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="U19" t="s">
         <v>29</v>
@@ -1865,25 +1871,25 @@
         <v>31</v>
       </c>
       <c r="N20" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="O20" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="P20">
         <v>1000000</v>
       </c>
       <c r="Q20" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R20" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="S20" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T20" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="U20" t="s">
         <v>29</v>
@@ -1912,25 +1918,25 @@
         <v>31</v>
       </c>
       <c r="N21" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="O21" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="P21">
         <v>400000</v>
       </c>
       <c r="Q21" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="R21" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="S21" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T21" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="U21" t="s">
         <v>29</v>
@@ -1959,25 +1965,25 @@
         <v>31</v>
       </c>
       <c r="N22" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="O22" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="P22">
         <v>120000</v>
       </c>
       <c r="Q22" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="R22" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="S22" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T22" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="U22" t="s">
         <v>29</v>
@@ -2006,25 +2012,25 @@
         <v>31</v>
       </c>
       <c r="N23" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="O23" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="P23">
         <v>80000</v>
       </c>
       <c r="Q23" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="R23" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="S23" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T23" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="U23" t="s">
         <v>29</v>
@@ -2065,28 +2071,28 @@
         <v>64</v>
       </c>
       <c r="N24" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="O24" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="P24">
         <v>1704503</v>
       </c>
       <c r="Q24" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R24" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="S24" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T24" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="U24" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="V24" s="1">
         <v>46138</v>
@@ -2121,25 +2127,25 @@
         <v>51</v>
       </c>
       <c r="N25" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="O25" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="P25">
         <v>3799000</v>
       </c>
       <c r="Q25" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R25" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="S25" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T25" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="U25" t="s">
         <v>29</v>
@@ -2177,25 +2183,25 @@
         <v>52</v>
       </c>
       <c r="N26" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="O26" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="P26">
         <v>1000</v>
       </c>
       <c r="Q26" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R26" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="S26" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T26" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="U26" t="s">
         <v>29</v>
@@ -2224,28 +2230,28 @@
         <v>31</v>
       </c>
       <c r="N27" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="O27" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="P27">
         <v>100000</v>
       </c>
       <c r="Q27" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="R27" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="S27" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T27" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="U27" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="V27" s="1">
         <v>46291</v>
@@ -2283,28 +2289,28 @@
         <v>65</v>
       </c>
       <c r="N28" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="O28" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="P28">
         <v>150000</v>
       </c>
       <c r="Q28" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R28" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="S28" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T28" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="U28" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="V28" s="1">
         <v>46199</v>
@@ -2342,28 +2348,28 @@
         <v>65</v>
       </c>
       <c r="N29" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="O29" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="P29">
         <v>150000</v>
       </c>
       <c r="Q29" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R29" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="S29" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T29" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="U29" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="V29" s="1">
         <v>46199</v>
@@ -2401,28 +2407,28 @@
         <v>65</v>
       </c>
       <c r="N30" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="O30" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="P30">
         <v>18462.36</v>
       </c>
       <c r="Q30" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R30" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="S30" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T30" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="U30" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="V30" s="1">
         <v>46199</v>
@@ -2460,28 +2466,28 @@
         <v>65</v>
       </c>
       <c r="N31" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="O31" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="P31">
         <v>324166.14</v>
       </c>
       <c r="Q31" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R31" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="S31" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T31" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="U31" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="V31" s="1">
         <v>46199</v>
@@ -2507,28 +2513,28 @@
         <v>31</v>
       </c>
       <c r="N32" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="O32" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="P32">
         <v>30000</v>
       </c>
       <c r="Q32" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R32" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="S32" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T32" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="U32" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="V32" s="1">
         <v>46291</v>
@@ -2566,28 +2572,28 @@
         <v>66</v>
       </c>
       <c r="N33" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="O33" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="P33">
         <v>1496713.48</v>
       </c>
       <c r="Q33" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R33" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="S33" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T33" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="U33" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="V33" s="1">
         <v>46199</v>
@@ -2622,28 +2628,28 @@
         <v>50</v>
       </c>
       <c r="N34" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="O34" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="P34">
         <v>207789.52</v>
       </c>
       <c r="Q34" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R34" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="S34" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T34" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="U34" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="V34" s="1">
         <v>46138</v>
@@ -2678,25 +2684,25 @@
         <v>56</v>
       </c>
       <c r="N35" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="O35" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="P35">
         <v>962290.8</v>
       </c>
       <c r="Q35" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R35" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="S35" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T35" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="U35" t="s">
         <v>29</v>
@@ -2734,25 +2740,25 @@
         <v>57</v>
       </c>
       <c r="N36" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="O36" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="P36">
         <v>798776.97</v>
       </c>
       <c r="Q36" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R36" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="S36" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T36" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="U36" t="s">
         <v>29</v>
@@ -2790,25 +2796,25 @@
         <v>56</v>
       </c>
       <c r="N37" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="O37" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="P37">
         <v>1530656.62</v>
       </c>
       <c r="Q37" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R37" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="S37" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T37" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="U37" t="s">
         <v>29</v>
@@ -2846,25 +2852,25 @@
         <v>58</v>
       </c>
       <c r="N38" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="O38" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="P38">
         <v>72958.08</v>
       </c>
       <c r="Q38" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R38" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="S38" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T38" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="U38" t="s">
         <v>29</v>
@@ -2902,25 +2908,25 @@
         <v>58</v>
       </c>
       <c r="N39" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="O39" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="P39">
         <v>8916</v>
       </c>
       <c r="Q39" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R39" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="S39" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T39" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="U39" t="s">
         <v>29</v>
@@ -2958,25 +2964,25 @@
         <v>58</v>
       </c>
       <c r="N40" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="O40" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="P40">
         <v>425178.5</v>
       </c>
       <c r="Q40" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R40" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="S40" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T40" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="U40" t="s">
         <v>29</v>
@@ -3014,25 +3020,25 @@
         <v>59</v>
       </c>
       <c r="N41" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="O41" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="P41">
         <v>1223.03</v>
       </c>
       <c r="Q41" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R41" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="S41" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T41" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="U41" t="s">
         <v>29</v>
@@ -3061,22 +3067,22 @@
         <v>43</v>
       </c>
       <c r="N42" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="O42" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="Q42" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R42" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="S42" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="T42" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="U42" t="s">
         <v>29</v>
@@ -3114,25 +3120,25 @@
         <v>60</v>
       </c>
       <c r="N43" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="O43" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="P43">
         <v>400000</v>
       </c>
       <c r="Q43" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R43" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="S43" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T43" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="U43" t="s">
         <v>29</v>
@@ -3170,25 +3176,25 @@
         <v>60</v>
       </c>
       <c r="N44" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="O44" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="P44">
         <v>400000</v>
       </c>
       <c r="Q44" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R44" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="S44" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T44" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="U44" t="s">
         <v>29</v>
@@ -3229,28 +3235,28 @@
         <v>67</v>
       </c>
       <c r="N45" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="O45" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="P45">
         <v>173846.38</v>
       </c>
       <c r="Q45" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R45" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="S45" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T45" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="U45" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="V45" s="1">
         <v>46229</v>
@@ -3285,28 +3291,28 @@
         <v>54</v>
       </c>
       <c r="N46" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="O46" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="P46">
         <v>1530656.62</v>
       </c>
       <c r="Q46" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R46" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="S46" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T46" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="U46" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="V46" s="1">
         <v>46229</v>
@@ -3332,25 +3338,25 @@
         <v>31</v>
       </c>
       <c r="N47" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="O47" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="P47">
         <v>1000000</v>
       </c>
       <c r="Q47" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R47" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="S47" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T47" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="U47" t="s">
         <v>29</v>
@@ -3379,28 +3385,28 @@
         <v>31</v>
       </c>
       <c r="N48" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="O48" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="P48">
         <v>958040</v>
       </c>
       <c r="Q48" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="R48" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="S48" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T48" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="U48" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="V48" s="1">
         <v>46291</v>
@@ -3438,28 +3444,28 @@
         <v>68</v>
       </c>
       <c r="N49" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="O49" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="P49">
         <v>41730.64</v>
       </c>
       <c r="Q49" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="R49" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="S49" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T49" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="U49" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="V49" s="1">
         <v>46199</v>
@@ -3488,31 +3494,31 @@
         <v>67</v>
       </c>
       <c r="K50" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="N50" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="O50" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="P50">
         <v>1468159.32</v>
       </c>
       <c r="Q50" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R50" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="S50" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T50" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="U50" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="V50" s="1">
         <v>46260</v>
@@ -3541,31 +3547,31 @@
         <v>67</v>
       </c>
       <c r="K51" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="N51" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="O51" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="P51">
         <v>1704503</v>
       </c>
       <c r="Q51" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R51" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="S51" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T51" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="U51" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="V51" s="1">
         <v>46291</v>
@@ -3591,31 +3597,31 @@
         <v>31</v>
       </c>
       <c r="K52" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="N52" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="O52" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="P52">
         <v>1704503</v>
       </c>
       <c r="Q52" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R52" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="S52" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T52" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="U52" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="V52" s="1">
         <v>46321</v>
@@ -3650,28 +3656,28 @@
         <v>62</v>
       </c>
       <c r="N53" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="O53" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="P53">
         <v>236343.68</v>
       </c>
       <c r="Q53" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R53" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="S53" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T53" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="U53" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="V53" s="1">
         <v>46229</v>
@@ -3697,28 +3703,28 @@
         <v>31</v>
       </c>
       <c r="N54" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="O54" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="P54">
         <v>1295422.28</v>
       </c>
       <c r="Q54" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R54" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="S54" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T54" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="U54" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="V54" s="1">
         <v>46352</v>
@@ -3744,31 +3750,31 @@
         <v>40</v>
       </c>
       <c r="K55" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="N55" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O55" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="P55">
         <v>500000</v>
       </c>
       <c r="Q55" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R55" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="S55" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T55" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="U55" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="V55" s="1">
         <v>46321</v>
@@ -3797,28 +3803,28 @@
         <v>44</v>
       </c>
       <c r="N56" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O56" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="P56">
         <v>5000000</v>
       </c>
       <c r="Q56" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R56" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="S56" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T56" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="U56" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="V56" s="1">
         <v>46321</v>
@@ -3844,25 +3850,25 @@
         <v>43</v>
       </c>
       <c r="N57" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O57" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="Q57" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R57" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="S57" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T57" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="U57" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="V57" s="1">
         <v>46049</v>
@@ -3888,25 +3894,25 @@
         <v>43</v>
       </c>
       <c r="N58" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O58" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="Q58" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R58" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="S58" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T58" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="U58" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="59" spans="1:22">
@@ -3929,25 +3935,25 @@
         <v>43</v>
       </c>
       <c r="N59" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O59" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="Q59" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R59" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="S59" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T59" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="U59" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="60" spans="1:22">
@@ -3967,28 +3973,28 @@
         <v>30</v>
       </c>
       <c r="N60" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="O60" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="P60">
         <v>9389.959999999999</v>
       </c>
       <c r="Q60" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="R60" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="S60" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="T60" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="U60" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="V60" s="1">
         <v>46107</v>
@@ -4011,28 +4017,28 @@
         <v>30</v>
       </c>
       <c r="N61" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="O61" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="P61">
         <v>7204.82</v>
       </c>
       <c r="Q61" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="R61" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="S61" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="T61" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="U61" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="V61" s="1">
         <v>46107</v>
@@ -4055,28 +4061,28 @@
         <v>30</v>
       </c>
       <c r="N62" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="O62" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="P62">
         <v>4227.84</v>
       </c>
       <c r="Q62" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="R62" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="S62" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="T62" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="U62" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="V62" s="1">
         <v>46107</v>
@@ -4099,28 +4105,28 @@
         <v>30</v>
       </c>
       <c r="N63" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="O63" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="P63">
         <v>4064.54</v>
       </c>
       <c r="Q63" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R63" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="S63" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="T63" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="U63" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="V63" s="1">
         <v>46107</v>
@@ -4143,28 +4149,28 @@
         <v>30</v>
       </c>
       <c r="N64" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="O64" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="P64">
         <v>3662.66</v>
       </c>
       <c r="Q64" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="R64" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="S64" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="T64" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="U64" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="V64" s="1">
         <v>46107</v>
@@ -4187,28 +4193,28 @@
         <v>30</v>
       </c>
       <c r="N65" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="O65" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="P65">
         <v>1163.64</v>
       </c>
       <c r="Q65" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="R65" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="S65" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="T65" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="U65" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="V65" s="1">
         <v>46107</v>
@@ -4231,25 +4237,25 @@
         <v>30</v>
       </c>
       <c r="N66" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="O66" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="P66">
         <v>120000</v>
       </c>
       <c r="Q66" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="R66" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="S66" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="T66" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="U66" t="s">
         <v>29</v>
@@ -4278,25 +4284,25 @@
         <v>31</v>
       </c>
       <c r="N67" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="O67" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="P67">
         <v>400000</v>
       </c>
       <c r="Q67" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="R67" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="S67" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T67" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="U67" t="s">
         <v>29</v>
@@ -4325,28 +4331,28 @@
         <v>31</v>
       </c>
       <c r="N68" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="O68" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="P68">
         <v>100000</v>
       </c>
       <c r="Q68" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="R68" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="S68" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T68" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="U68" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="V68" s="1">
         <v>46229</v>
@@ -4369,25 +4375,25 @@
         <v>30</v>
       </c>
       <c r="N69" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="O69" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="P69">
         <v>80000</v>
       </c>
       <c r="Q69" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="R69" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="S69" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="T69" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="U69" t="s">
         <v>29</v>
@@ -4413,28 +4419,28 @@
         <v>30</v>
       </c>
       <c r="N70" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="O70" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="P70">
         <v>835000</v>
       </c>
       <c r="Q70" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="R70" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="S70" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="T70" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="U70" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="V70" s="1">
         <v>46291</v>
@@ -4457,28 +4463,28 @@
         <v>30</v>
       </c>
       <c r="N71" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="O71" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="P71">
         <v>165000</v>
       </c>
       <c r="Q71" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="R71" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="S71" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="T71" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="U71" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="V71" s="1">
         <v>46168</v>
@@ -4501,28 +4507,28 @@
         <v>30</v>
       </c>
       <c r="N72" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="O72" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="P72">
         <v>1000000</v>
       </c>
       <c r="Q72" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="R72" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="S72" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="T72" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="U72" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="V72" s="1">
         <v>46291</v>
@@ -4545,28 +4551,28 @@
         <v>30</v>
       </c>
       <c r="N73" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="O73" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="P73">
         <v>1000000</v>
       </c>
       <c r="Q73" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="R73" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="S73" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="T73" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="U73" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="V73" s="1">
         <v>46291</v>
@@ -4589,28 +4595,28 @@
         <v>30</v>
       </c>
       <c r="N74" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="O74" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="P74">
         <v>100000</v>
       </c>
       <c r="Q74" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="R74" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="S74" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="T74" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="U74" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="V74" s="1">
         <v>46291</v>
@@ -4636,25 +4642,25 @@
         <v>31</v>
       </c>
       <c r="N75" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="O75" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="P75">
         <v>1000000</v>
       </c>
       <c r="Q75" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R75" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="S75" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T75" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="U75" t="s">
         <v>29</v>
@@ -4686,28 +4692,28 @@
         <v>45</v>
       </c>
       <c r="N76" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="O76" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="P76">
         <v>1704503</v>
       </c>
       <c r="Q76" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R76" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="S76" t="s">
         <v>41</v>
       </c>
       <c r="T76" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="U76" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="V76" s="1">
         <v>46381</v>
@@ -4736,28 +4742,28 @@
         <v>45</v>
       </c>
       <c r="N77" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="O77" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="P77">
         <v>1638125.5</v>
       </c>
       <c r="Q77" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R77" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="S77" t="s">
         <v>41</v>
       </c>
       <c r="T77" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="U77" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="V77" s="1">
         <v>46381</v>
@@ -4786,25 +4792,25 @@
         <v>45</v>
       </c>
       <c r="N78" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="O78" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="P78">
         <v>3800000</v>
       </c>
       <c r="Q78" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R78" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="S78" t="s">
         <v>41</v>
       </c>
       <c r="T78" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="U78" t="s">
         <v>29</v>
@@ -4836,25 +4842,25 @@
         <v>45</v>
       </c>
       <c r="N79" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="O79" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="P79">
         <v>3800000</v>
       </c>
       <c r="Q79" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R79" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="S79" t="s">
         <v>41</v>
       </c>
       <c r="T79" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="U79" t="s">
         <v>29</v>
@@ -4879,26 +4885,32 @@
       <c r="E80" t="s">
         <v>30</v>
       </c>
+      <c r="J80" t="s">
+        <v>69</v>
+      </c>
+      <c r="K80" t="s">
+        <v>73</v>
+      </c>
       <c r="N80" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="O80" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="P80">
         <v>3800000</v>
       </c>
       <c r="Q80" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R80" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="S80" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="T80" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="U80" t="s">
         <v>29</v>
@@ -4924,25 +4936,25 @@
         <v>29</v>
       </c>
       <c r="N81" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="O81" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="P81">
         <v>4394700</v>
       </c>
       <c r="Q81" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="R81" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="S81" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="T81" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="U81" t="s">
         <v>29</v>
@@ -4971,28 +4983,28 @@
         <v>31</v>
       </c>
       <c r="N82" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="O82" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="P82">
         <v>528395.9300000001</v>
       </c>
       <c r="Q82" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R82" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="S82" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T82" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="U82" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="V82" s="1">
         <v>46382</v>
@@ -5015,25 +5027,25 @@
         <v>30</v>
       </c>
       <c r="N83" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="O83" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="P83">
         <v>1000000</v>
       </c>
       <c r="Q83" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R83" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="S83" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="T83" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="U83" t="s">
         <v>29</v>
@@ -5059,25 +5071,25 @@
         <v>29</v>
       </c>
       <c r="N84" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="O84" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="P84">
         <v>4394700</v>
       </c>
       <c r="Q84" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="R84" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="S84" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="T84" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="U84" t="s">
         <v>29</v>
@@ -5109,25 +5121,25 @@
         <v>45</v>
       </c>
       <c r="N85" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="O85" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="P85">
         <v>3306000</v>
       </c>
       <c r="Q85" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="R85" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="S85" t="s">
         <v>41</v>
       </c>
       <c r="T85" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="U85" t="s">
         <v>29</v>
@@ -5156,25 +5168,25 @@
         <v>45</v>
       </c>
       <c r="N86" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="O86" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="P86">
         <v>3306000</v>
       </c>
       <c r="Q86" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="R86" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="S86" t="s">
         <v>41</v>
       </c>
       <c r="T86" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="U86" t="s">
         <v>29</v>
@@ -5200,25 +5212,25 @@
         <v>31</v>
       </c>
       <c r="N87" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="O87" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="P87">
         <v>212577</v>
       </c>
       <c r="Q87" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R87" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="S87" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="T87" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="U87" t="s">
         <v>30</v>

</xml_diff>

<commit_message>
Atualização automática: mta (19/08/2026 13:07)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -551,8 +551,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -568,7 +576,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -576,12 +584,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -881,70 +907,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -994,7 +1020,7 @@
       <c r="U2" t="s">
         <v>175</v>
       </c>
-      <c r="V2" s="1">
+      <c r="V2" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -1041,7 +1067,7 @@
       <c r="U3" t="s">
         <v>29</v>
       </c>
-      <c r="V3" s="1">
+      <c r="V3" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1088,7 +1114,7 @@
       <c r="U4" t="s">
         <v>29</v>
       </c>
-      <c r="V4" s="1">
+      <c r="V4" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1135,7 +1161,7 @@
       <c r="U5" t="s">
         <v>29</v>
       </c>
-      <c r="V5" s="1">
+      <c r="V5" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1185,7 +1211,7 @@
       <c r="U6" t="s">
         <v>29</v>
       </c>
-      <c r="V6" s="1">
+      <c r="V6" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1211,7 +1237,7 @@
       <c r="G7" t="s">
         <v>42</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1241,7 +1267,7 @@
       <c r="U7" t="s">
         <v>29</v>
       </c>
-      <c r="V7" s="1">
+      <c r="V7" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -1288,7 +1314,7 @@
       <c r="U8" t="s">
         <v>29</v>
       </c>
-      <c r="V8" s="1">
+      <c r="V8" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1335,7 +1361,7 @@
       <c r="U9" t="s">
         <v>29</v>
       </c>
-      <c r="V9" s="1">
+      <c r="V9" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1382,7 +1408,7 @@
       <c r="U10" t="s">
         <v>29</v>
       </c>
-      <c r="V10" s="1">
+      <c r="V10" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1429,7 +1455,7 @@
       <c r="U11" t="s">
         <v>29</v>
       </c>
-      <c r="V11" s="1">
+      <c r="V11" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1455,7 +1481,7 @@
       <c r="G12" t="s">
         <v>42</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46079</v>
       </c>
       <c r="I12" t="s">
@@ -1488,7 +1514,7 @@
       <c r="U12" t="s">
         <v>175</v>
       </c>
-      <c r="V12" s="1">
+      <c r="V12" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1535,7 +1561,7 @@
       <c r="U13" t="s">
         <v>175</v>
       </c>
-      <c r="V13" s="1">
+      <c r="V13" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1582,7 +1608,7 @@
       <c r="U14" t="s">
         <v>175</v>
       </c>
-      <c r="V14" s="1">
+      <c r="V14" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1629,7 +1655,7 @@
       <c r="U15" t="s">
         <v>175</v>
       </c>
-      <c r="V15" s="1">
+      <c r="V15" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1676,7 +1702,7 @@
       <c r="U16" t="s">
         <v>175</v>
       </c>
-      <c r="V16" s="1">
+      <c r="V16" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -1702,7 +1728,7 @@
       <c r="G17" t="s">
         <v>42</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46098</v>
       </c>
       <c r="I17" t="s">
@@ -1735,7 +1761,7 @@
       <c r="U17" t="s">
         <v>175</v>
       </c>
-      <c r="V17" s="1">
+      <c r="V17" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -1761,7 +1787,7 @@
       <c r="G18" t="s">
         <v>42</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46076</v>
       </c>
       <c r="I18" t="s">
@@ -1791,7 +1817,7 @@
       <c r="U18" t="s">
         <v>29</v>
       </c>
-      <c r="V18" s="1">
+      <c r="V18" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1817,7 +1843,7 @@
       <c r="G19" t="s">
         <v>42</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1847,7 +1873,7 @@
       <c r="U19" t="s">
         <v>29</v>
       </c>
-      <c r="V19" s="1">
+      <c r="V19" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1894,7 +1920,7 @@
       <c r="U20" t="s">
         <v>29</v>
       </c>
-      <c r="V20" s="1">
+      <c r="V20" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1941,7 +1967,7 @@
       <c r="U21" t="s">
         <v>29</v>
       </c>
-      <c r="V21" s="1">
+      <c r="V21" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1988,7 +2014,7 @@
       <c r="U22" t="s">
         <v>29</v>
       </c>
-      <c r="V22" s="1">
+      <c r="V22" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2035,7 +2061,7 @@
       <c r="U23" t="s">
         <v>29</v>
       </c>
-      <c r="V23" s="1">
+      <c r="V23" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2061,7 +2087,7 @@
       <c r="G24" t="s">
         <v>42</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>46119</v>
       </c>
       <c r="I24" t="s">
@@ -2094,7 +2120,7 @@
       <c r="U24" t="s">
         <v>175</v>
       </c>
-      <c r="V24" s="1">
+      <c r="V24" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2120,7 +2146,7 @@
       <c r="G25" t="s">
         <v>42</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>46121</v>
       </c>
       <c r="I25" t="s">
@@ -2150,7 +2176,7 @@
       <c r="U25" t="s">
         <v>29</v>
       </c>
-      <c r="V25" s="1">
+      <c r="V25" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2176,7 +2202,7 @@
       <c r="G26" t="s">
         <v>42</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>46076</v>
       </c>
       <c r="I26" t="s">
@@ -2206,7 +2232,7 @@
       <c r="U26" t="s">
         <v>29</v>
       </c>
-      <c r="V26" s="1">
+      <c r="V26" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -2253,7 +2279,7 @@
       <c r="U27" t="s">
         <v>175</v>
       </c>
-      <c r="V27" s="1">
+      <c r="V27" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -2279,7 +2305,7 @@
       <c r="G28" t="s">
         <v>42</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>46199</v>
       </c>
       <c r="I28" t="s">
@@ -2312,7 +2338,7 @@
       <c r="U28" t="s">
         <v>175</v>
       </c>
-      <c r="V28" s="1">
+      <c r="V28" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2338,7 +2364,7 @@
       <c r="G29" t="s">
         <v>42</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2371,7 +2397,7 @@
       <c r="U29" t="s">
         <v>175</v>
       </c>
-      <c r="V29" s="1">
+      <c r="V29" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2397,7 +2423,7 @@
       <c r="G30" t="s">
         <v>42</v>
       </c>
-      <c r="H30" s="1">
+      <c r="H30" s="2">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2430,7 +2456,7 @@
       <c r="U30" t="s">
         <v>175</v>
       </c>
-      <c r="V30" s="1">
+      <c r="V30" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2456,7 +2482,7 @@
       <c r="G31" t="s">
         <v>42</v>
       </c>
-      <c r="H31" s="1">
+      <c r="H31" s="2">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2489,7 +2515,7 @@
       <c r="U31" t="s">
         <v>175</v>
       </c>
-      <c r="V31" s="1">
+      <c r="V31" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2536,7 +2562,7 @@
       <c r="U32" t="s">
         <v>175</v>
       </c>
-      <c r="V32" s="1">
+      <c r="V32" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -2562,7 +2588,7 @@
       <c r="G33" t="s">
         <v>42</v>
       </c>
-      <c r="H33" s="1">
+      <c r="H33" s="2">
         <v>46191</v>
       </c>
       <c r="I33" t="s">
@@ -2595,7 +2621,7 @@
       <c r="U33" t="s">
         <v>175</v>
       </c>
-      <c r="V33" s="1">
+      <c r="V33" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2621,7 +2647,7 @@
       <c r="G34" t="s">
         <v>42</v>
       </c>
-      <c r="H34" s="1">
+      <c r="H34" s="2">
         <v>46119</v>
       </c>
       <c r="I34" t="s">
@@ -2651,7 +2677,7 @@
       <c r="U34" t="s">
         <v>175</v>
       </c>
-      <c r="V34" s="1">
+      <c r="V34" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2677,7 +2703,7 @@
       <c r="G35" t="s">
         <v>42</v>
       </c>
-      <c r="H35" s="1">
+      <c r="H35" s="2">
         <v>46213</v>
       </c>
       <c r="I35" t="s">
@@ -2707,7 +2733,7 @@
       <c r="U35" t="s">
         <v>29</v>
       </c>
-      <c r="V35" s="1">
+      <c r="V35" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -2733,7 +2759,7 @@
       <c r="G36" t="s">
         <v>42</v>
       </c>
-      <c r="H36" s="1">
+      <c r="H36" s="2">
         <v>46175</v>
       </c>
       <c r="I36" t="s">
@@ -2763,7 +2789,7 @@
       <c r="U36" t="s">
         <v>29</v>
       </c>
-      <c r="V36" s="1">
+      <c r="V36" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2789,7 +2815,7 @@
       <c r="G37" t="s">
         <v>42</v>
       </c>
-      <c r="H37" s="1">
+      <c r="H37" s="2">
         <v>46213</v>
       </c>
       <c r="I37" t="s">
@@ -2819,7 +2845,7 @@
       <c r="U37" t="s">
         <v>29</v>
       </c>
-      <c r="V37" s="1">
+      <c r="V37" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -2845,7 +2871,7 @@
       <c r="G38" t="s">
         <v>42</v>
       </c>
-      <c r="H38" s="1">
+      <c r="H38" s="2">
         <v>46199</v>
       </c>
       <c r="I38" t="s">
@@ -2875,7 +2901,7 @@
       <c r="U38" t="s">
         <v>29</v>
       </c>
-      <c r="V38" s="1">
+      <c r="V38" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2901,7 +2927,7 @@
       <c r="G39" t="s">
         <v>42</v>
       </c>
-      <c r="H39" s="1">
+      <c r="H39" s="2">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -2931,7 +2957,7 @@
       <c r="U39" t="s">
         <v>29</v>
       </c>
-      <c r="V39" s="1">
+      <c r="V39" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2957,7 +2983,7 @@
       <c r="G40" t="s">
         <v>42</v>
       </c>
-      <c r="H40" s="1">
+      <c r="H40" s="2">
         <v>46204</v>
       </c>
       <c r="I40" t="s">
@@ -2987,7 +3013,7 @@
       <c r="U40" t="s">
         <v>29</v>
       </c>
-      <c r="V40" s="1">
+      <c r="V40" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3013,7 +3039,7 @@
       <c r="G41" t="s">
         <v>42</v>
       </c>
-      <c r="H41" s="1">
+      <c r="H41" s="2">
         <v>46244</v>
       </c>
       <c r="I41" t="s">
@@ -3043,7 +3069,7 @@
       <c r="U41" t="s">
         <v>29</v>
       </c>
-      <c r="V41" s="1">
+      <c r="V41" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3087,7 +3113,7 @@
       <c r="U42" t="s">
         <v>29</v>
       </c>
-      <c r="V42" s="1">
+      <c r="V42" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3113,7 +3139,7 @@
       <c r="G43" t="s">
         <v>42</v>
       </c>
-      <c r="H43" s="1">
+      <c r="H43" s="2">
         <v>46191</v>
       </c>
       <c r="I43" t="s">
@@ -3143,7 +3169,7 @@
       <c r="U43" t="s">
         <v>29</v>
       </c>
-      <c r="V43" s="1">
+      <c r="V43" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3169,7 +3195,7 @@
       <c r="G44" t="s">
         <v>42</v>
       </c>
-      <c r="H44" s="1">
+      <c r="H44" s="2">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
@@ -3199,7 +3225,7 @@
       <c r="U44" t="s">
         <v>29</v>
       </c>
-      <c r="V44" s="1">
+      <c r="V44" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3225,7 +3251,7 @@
       <c r="G45" t="s">
         <v>42</v>
       </c>
-      <c r="H45" s="1">
+      <c r="H45" s="2">
         <v>46213</v>
       </c>
       <c r="I45" t="s">
@@ -3258,7 +3284,7 @@
       <c r="U45" t="s">
         <v>175</v>
       </c>
-      <c r="V45" s="1">
+      <c r="V45" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3284,7 +3310,7 @@
       <c r="G46" t="s">
         <v>42</v>
       </c>
-      <c r="H46" s="1">
+      <c r="H46" s="2">
         <v>46210</v>
       </c>
       <c r="I46" t="s">
@@ -3314,7 +3340,7 @@
       <c r="U46" t="s">
         <v>175</v>
       </c>
-      <c r="V46" s="1">
+      <c r="V46" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3361,7 +3387,7 @@
       <c r="U47" t="s">
         <v>29</v>
       </c>
-      <c r="V47" s="1">
+      <c r="V47" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3408,7 +3434,7 @@
       <c r="U48" t="s">
         <v>175</v>
       </c>
-      <c r="V48" s="1">
+      <c r="V48" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3434,7 +3460,7 @@
       <c r="G49" t="s">
         <v>42</v>
       </c>
-      <c r="H49" s="1">
+      <c r="H49" s="2">
         <v>46176</v>
       </c>
       <c r="I49" t="s">
@@ -3467,7 +3493,7 @@
       <c r="U49" t="s">
         <v>175</v>
       </c>
-      <c r="V49" s="1">
+      <c r="V49" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3520,7 +3546,7 @@
       <c r="U50" t="s">
         <v>175</v>
       </c>
-      <c r="V50" s="1">
+      <c r="V50" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3573,7 +3599,7 @@
       <c r="U51" t="s">
         <v>175</v>
       </c>
-      <c r="V51" s="1">
+      <c r="V51" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3623,7 +3649,7 @@
       <c r="U52" t="s">
         <v>175</v>
       </c>
-      <c r="V52" s="1">
+      <c r="V52" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3649,7 +3675,7 @@
       <c r="G53" t="s">
         <v>42</v>
       </c>
-      <c r="H53" s="1">
+      <c r="H53" s="2">
         <v>46227</v>
       </c>
       <c r="I53" t="s">
@@ -3679,7 +3705,7 @@
       <c r="U53" t="s">
         <v>175</v>
       </c>
-      <c r="V53" s="1">
+      <c r="V53" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3726,7 +3752,7 @@
       <c r="U54" t="s">
         <v>175</v>
       </c>
-      <c r="V54" s="1">
+      <c r="V54" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -3776,7 +3802,7 @@
       <c r="U55" t="s">
         <v>175</v>
       </c>
-      <c r="V55" s="1">
+      <c r="V55" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3826,7 +3852,7 @@
       <c r="U56" t="s">
         <v>175</v>
       </c>
-      <c r="V56" s="1">
+      <c r="V56" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3870,7 +3896,7 @@
       <c r="U57" t="s">
         <v>175</v>
       </c>
-      <c r="V57" s="1">
+      <c r="V57" s="2">
         <v>46049</v>
       </c>
     </row>
@@ -3996,7 +4022,7 @@
       <c r="U60" t="s">
         <v>175</v>
       </c>
-      <c r="V60" s="1">
+      <c r="V60" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4040,7 +4066,7 @@
       <c r="U61" t="s">
         <v>175</v>
       </c>
-      <c r="V61" s="1">
+      <c r="V61" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4084,7 +4110,7 @@
       <c r="U62" t="s">
         <v>175</v>
       </c>
-      <c r="V62" s="1">
+      <c r="V62" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4128,7 +4154,7 @@
       <c r="U63" t="s">
         <v>175</v>
       </c>
-      <c r="V63" s="1">
+      <c r="V63" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4172,7 +4198,7 @@
       <c r="U64" t="s">
         <v>175</v>
       </c>
-      <c r="V64" s="1">
+      <c r="V64" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4216,7 +4242,7 @@
       <c r="U65" t="s">
         <v>175</v>
       </c>
-      <c r="V65" s="1">
+      <c r="V65" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4260,7 +4286,7 @@
       <c r="U66" t="s">
         <v>29</v>
       </c>
-      <c r="V66" s="1">
+      <c r="V66" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4307,7 +4333,7 @@
       <c r="U67" t="s">
         <v>29</v>
       </c>
-      <c r="V67" s="1">
+      <c r="V67" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4354,7 +4380,7 @@
       <c r="U68" t="s">
         <v>175</v>
       </c>
-      <c r="V68" s="1">
+      <c r="V68" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -4398,7 +4424,7 @@
       <c r="U69" t="s">
         <v>29</v>
       </c>
-      <c r="V69" s="1">
+      <c r="V69" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -4442,7 +4468,7 @@
       <c r="U70" t="s">
         <v>175</v>
       </c>
-      <c r="V70" s="1">
+      <c r="V70" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4486,7 +4512,7 @@
       <c r="U71" t="s">
         <v>175</v>
       </c>
-      <c r="V71" s="1">
+      <c r="V71" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4530,7 +4556,7 @@
       <c r="U72" t="s">
         <v>175</v>
       </c>
-      <c r="V72" s="1">
+      <c r="V72" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4574,7 +4600,7 @@
       <c r="U73" t="s">
         <v>175</v>
       </c>
-      <c r="V73" s="1">
+      <c r="V73" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4618,7 +4644,7 @@
       <c r="U74" t="s">
         <v>175</v>
       </c>
-      <c r="V74" s="1">
+      <c r="V74" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4665,7 +4691,7 @@
       <c r="U75" t="s">
         <v>29</v>
       </c>
-      <c r="V75" s="1">
+      <c r="V75" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -4715,7 +4741,7 @@
       <c r="U76" t="s">
         <v>175</v>
       </c>
-      <c r="V76" s="1">
+      <c r="V76" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4765,7 +4791,7 @@
       <c r="U77" t="s">
         <v>175</v>
       </c>
-      <c r="V77" s="1">
+      <c r="V77" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4815,7 +4841,7 @@
       <c r="U78" t="s">
         <v>29</v>
       </c>
-      <c r="V78" s="1">
+      <c r="V78" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4865,7 +4891,7 @@
       <c r="U79" t="s">
         <v>29</v>
       </c>
-      <c r="V79" s="1">
+      <c r="V79" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4915,7 +4941,7 @@
       <c r="U80" t="s">
         <v>29</v>
       </c>
-      <c r="V80" s="1">
+      <c r="V80" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -4959,7 +4985,7 @@
       <c r="U81" t="s">
         <v>29</v>
       </c>
-      <c r="V81" s="1">
+      <c r="V81" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5006,7 +5032,7 @@
       <c r="U82" t="s">
         <v>175</v>
       </c>
-      <c r="V82" s="1">
+      <c r="V82" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5050,7 +5076,7 @@
       <c r="U83" t="s">
         <v>29</v>
       </c>
-      <c r="V83" s="1">
+      <c r="V83" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -5094,7 +5120,7 @@
       <c r="U84" t="s">
         <v>29</v>
       </c>
-      <c r="V84" s="1">
+      <c r="V84" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5235,7 +5261,7 @@
       <c r="U87" t="s">
         <v>30</v>
       </c>
-      <c r="V87" s="1">
+      <c r="V87" s="2">
         <v>46260</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (19/08/2026 14:34)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1118" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1121" uniqueCount="179">
   <si>
     <t>linha</t>
   </si>
@@ -226,6 +226,9 @@
     <t>e-mail 12/08</t>
   </si>
   <si>
+    <t>REMANEJAR</t>
+  </si>
+  <si>
     <t>Atender AGO</t>
   </si>
   <si>
@@ -235,7 +238,13 @@
     <t>Atender OUT</t>
   </si>
   <si>
+    <t>Atender NOV</t>
+  </si>
+  <si>
     <t>ATENDER com 20XV</t>
+  </si>
+  <si>
+    <t>Atender DEZ</t>
   </si>
   <si>
     <t>LIVRE</t>
@@ -551,16 +560,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -576,7 +577,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -584,30 +585,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -907,70 +890,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -994,33 +977,33 @@
         <v>31</v>
       </c>
       <c r="L2" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="N2" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="O2" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="P2">
         <v>135000</v>
       </c>
       <c r="Q2" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="R2" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="S2" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T2" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="U2" t="s">
-        <v>175</v>
-      </c>
-      <c r="V2" s="2">
+        <v>178</v>
+      </c>
+      <c r="V2" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1044,30 +1027,30 @@
         <v>31</v>
       </c>
       <c r="N3" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="O3" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="P3">
         <v>400000</v>
       </c>
       <c r="Q3" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="R3" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="S3" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T3" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="U3" t="s">
         <v>29</v>
       </c>
-      <c r="V3" s="2">
+      <c r="V3" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1091,30 +1074,30 @@
         <v>31</v>
       </c>
       <c r="N4" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="O4" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="P4">
         <v>430000</v>
       </c>
       <c r="Q4" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="R4" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="S4" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T4" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="U4" t="s">
         <v>29</v>
       </c>
-      <c r="V4" s="2">
+      <c r="V4" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1138,30 +1121,30 @@
         <v>31</v>
       </c>
       <c r="N5" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="O5" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="P5">
         <v>425000</v>
       </c>
       <c r="Q5" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="R5" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="S5" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T5" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="U5" t="s">
         <v>29</v>
       </c>
-      <c r="V5" s="2">
+      <c r="V5" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1185,33 +1168,33 @@
         <v>31</v>
       </c>
       <c r="L6" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="N6" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="O6" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="P6">
         <v>563000</v>
       </c>
       <c r="Q6" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="R6" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="S6" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T6" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="U6" t="s">
         <v>29</v>
       </c>
-      <c r="V6" s="2">
+      <c r="V6" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1237,37 +1220,37 @@
       <c r="G7" t="s">
         <v>42</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
         <v>46</v>
       </c>
       <c r="N7" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="O7" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="P7">
         <v>3799999.6</v>
       </c>
       <c r="Q7" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R7" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="S7" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T7" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="U7" t="s">
         <v>29</v>
       </c>
-      <c r="V7" s="2">
+      <c r="V7" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -1291,30 +1274,30 @@
         <v>31</v>
       </c>
       <c r="N8" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="O8" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="P8">
         <v>430000</v>
       </c>
       <c r="Q8" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="R8" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="S8" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T8" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="U8" t="s">
         <v>29</v>
       </c>
-      <c r="V8" s="2">
+      <c r="V8" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1338,30 +1321,30 @@
         <v>31</v>
       </c>
       <c r="N9" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="O9" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="P9">
         <v>60000</v>
       </c>
       <c r="Q9" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="R9" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="S9" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T9" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="U9" t="s">
         <v>29</v>
       </c>
-      <c r="V9" s="2">
+      <c r="V9" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1385,30 +1368,30 @@
         <v>31</v>
       </c>
       <c r="N10" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="O10" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="P10">
         <v>200000</v>
       </c>
       <c r="Q10" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="R10" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="S10" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T10" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="U10" t="s">
         <v>29</v>
       </c>
-      <c r="V10" s="2">
+      <c r="V10" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1432,30 +1415,30 @@
         <v>31</v>
       </c>
       <c r="N11" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="O11" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="P11">
         <v>320000</v>
       </c>
       <c r="Q11" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="R11" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="S11" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T11" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="U11" t="s">
         <v>29</v>
       </c>
-      <c r="V11" s="2">
+      <c r="V11" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1481,7 +1464,7 @@
       <c r="G12" t="s">
         <v>42</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46079</v>
       </c>
       <c r="I12" t="s">
@@ -1491,30 +1474,30 @@
         <v>63</v>
       </c>
       <c r="N12" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="O12" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="P12">
         <v>1187433.02</v>
       </c>
       <c r="Q12" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="R12" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="S12" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T12" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="U12" t="s">
-        <v>175</v>
-      </c>
-      <c r="V12" s="2">
+        <v>178</v>
+      </c>
+      <c r="V12" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1538,30 +1521,30 @@
         <v>31</v>
       </c>
       <c r="N13" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="O13" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="P13">
         <v>1000000</v>
       </c>
       <c r="Q13" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="R13" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="S13" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T13" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="U13" t="s">
-        <v>175</v>
-      </c>
-      <c r="V13" s="2">
+        <v>178</v>
+      </c>
+      <c r="V13" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1585,30 +1568,30 @@
         <v>31</v>
       </c>
       <c r="N14" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="O14" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="P14">
         <v>1000000</v>
       </c>
       <c r="Q14" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="R14" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="S14" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T14" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="U14" t="s">
-        <v>175</v>
-      </c>
-      <c r="V14" s="2">
+        <v>178</v>
+      </c>
+      <c r="V14" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1632,30 +1615,30 @@
         <v>31</v>
       </c>
       <c r="N15" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="O15" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="P15">
         <v>1000000</v>
       </c>
       <c r="Q15" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="R15" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="S15" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T15" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="U15" t="s">
-        <v>175</v>
-      </c>
-      <c r="V15" s="2">
+        <v>178</v>
+      </c>
+      <c r="V15" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1679,30 +1662,30 @@
         <v>31</v>
       </c>
       <c r="N16" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="O16" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="P16">
         <v>100000</v>
       </c>
       <c r="Q16" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="R16" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="S16" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T16" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="U16" t="s">
-        <v>175</v>
-      </c>
-      <c r="V16" s="2">
+        <v>178</v>
+      </c>
+      <c r="V16" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1728,7 +1711,7 @@
       <c r="G17" t="s">
         <v>42</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46098</v>
       </c>
       <c r="I17" t="s">
@@ -1738,30 +1721,30 @@
         <v>63</v>
       </c>
       <c r="N17" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="O17" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="P17">
         <v>1770880.5</v>
       </c>
       <c r="Q17" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R17" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="S17" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T17" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U17" t="s">
-        <v>175</v>
-      </c>
-      <c r="V17" s="2">
+        <v>178</v>
+      </c>
+      <c r="V17" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -1787,37 +1770,37 @@
       <c r="G18" t="s">
         <v>42</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46076</v>
       </c>
       <c r="I18" t="s">
         <v>49</v>
       </c>
       <c r="N18" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="O18" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="P18">
         <v>350000</v>
       </c>
       <c r="Q18" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R18" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="S18" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T18" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="U18" t="s">
         <v>29</v>
       </c>
-      <c r="V18" s="2">
+      <c r="V18" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1843,37 +1826,37 @@
       <c r="G19" t="s">
         <v>42</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
         <v>49</v>
       </c>
       <c r="N19" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="O19" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="P19">
         <v>350000</v>
       </c>
       <c r="Q19" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R19" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="S19" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T19" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="U19" t="s">
         <v>29</v>
       </c>
-      <c r="V19" s="2">
+      <c r="V19" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1897,30 +1880,30 @@
         <v>31</v>
       </c>
       <c r="N20" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="O20" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="P20">
         <v>1000000</v>
       </c>
       <c r="Q20" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R20" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="S20" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T20" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="U20" t="s">
         <v>29</v>
       </c>
-      <c r="V20" s="2">
+      <c r="V20" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1944,30 +1927,30 @@
         <v>31</v>
       </c>
       <c r="N21" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="O21" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="P21">
         <v>400000</v>
       </c>
       <c r="Q21" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="R21" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="S21" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T21" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="U21" t="s">
         <v>29</v>
       </c>
-      <c r="V21" s="2">
+      <c r="V21" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1991,30 +1974,30 @@
         <v>31</v>
       </c>
       <c r="N22" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="O22" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="P22">
         <v>120000</v>
       </c>
       <c r="Q22" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="R22" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="S22" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T22" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="U22" t="s">
         <v>29</v>
       </c>
-      <c r="V22" s="2">
+      <c r="V22" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2038,30 +2021,30 @@
         <v>31</v>
       </c>
       <c r="N23" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="O23" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="P23">
         <v>80000</v>
       </c>
       <c r="Q23" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="R23" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="S23" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T23" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="U23" t="s">
         <v>29</v>
       </c>
-      <c r="V23" s="2">
+      <c r="V23" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2087,7 +2070,7 @@
       <c r="G24" t="s">
         <v>42</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>46119</v>
       </c>
       <c r="I24" t="s">
@@ -2097,30 +2080,30 @@
         <v>64</v>
       </c>
       <c r="N24" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="O24" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="P24">
         <v>1704503</v>
       </c>
       <c r="Q24" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R24" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="S24" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T24" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U24" t="s">
-        <v>175</v>
-      </c>
-      <c r="V24" s="2">
+        <v>178</v>
+      </c>
+      <c r="V24" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2146,37 +2129,37 @@
       <c r="G25" t="s">
         <v>42</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>46121</v>
       </c>
       <c r="I25" t="s">
         <v>51</v>
       </c>
       <c r="N25" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="O25" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="P25">
         <v>3799000</v>
       </c>
       <c r="Q25" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R25" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="S25" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T25" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="U25" t="s">
         <v>29</v>
       </c>
-      <c r="V25" s="2">
+      <c r="V25" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2202,37 +2185,37 @@
       <c r="G26" t="s">
         <v>42</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>46076</v>
       </c>
       <c r="I26" t="s">
         <v>52</v>
       </c>
       <c r="N26" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="O26" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="P26">
         <v>1000</v>
       </c>
       <c r="Q26" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R26" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="S26" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T26" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="U26" t="s">
         <v>29</v>
       </c>
-      <c r="V26" s="2">
+      <c r="V26" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -2256,30 +2239,30 @@
         <v>31</v>
       </c>
       <c r="N27" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="O27" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="P27">
         <v>100000</v>
       </c>
       <c r="Q27" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="R27" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="S27" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T27" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="U27" t="s">
-        <v>175</v>
-      </c>
-      <c r="V27" s="2">
+        <v>178</v>
+      </c>
+      <c r="V27" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2305,7 +2288,7 @@
       <c r="G28" t="s">
         <v>42</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>46199</v>
       </c>
       <c r="I28" t="s">
@@ -2315,30 +2298,30 @@
         <v>65</v>
       </c>
       <c r="N28" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="O28" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="P28">
         <v>150000</v>
       </c>
       <c r="Q28" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R28" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="S28" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T28" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="U28" t="s">
-        <v>175</v>
-      </c>
-      <c r="V28" s="2">
+        <v>178</v>
+      </c>
+      <c r="V28" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2364,7 +2347,7 @@
       <c r="G29" t="s">
         <v>42</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2374,30 +2357,30 @@
         <v>65</v>
       </c>
       <c r="N29" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="O29" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="P29">
         <v>150000</v>
       </c>
       <c r="Q29" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R29" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="S29" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T29" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="U29" t="s">
-        <v>175</v>
-      </c>
-      <c r="V29" s="2">
+        <v>178</v>
+      </c>
+      <c r="V29" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2423,7 +2406,7 @@
       <c r="G30" t="s">
         <v>42</v>
       </c>
-      <c r="H30" s="2">
+      <c r="H30" s="1">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2433,30 +2416,30 @@
         <v>65</v>
       </c>
       <c r="N30" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="O30" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="P30">
         <v>18462.36</v>
       </c>
       <c r="Q30" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R30" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="S30" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T30" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="U30" t="s">
-        <v>175</v>
-      </c>
-      <c r="V30" s="2">
+        <v>178</v>
+      </c>
+      <c r="V30" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2482,7 +2465,7 @@
       <c r="G31" t="s">
         <v>42</v>
       </c>
-      <c r="H31" s="2">
+      <c r="H31" s="1">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2492,30 +2475,30 @@
         <v>65</v>
       </c>
       <c r="N31" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="O31" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="P31">
         <v>324166.14</v>
       </c>
       <c r="Q31" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R31" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="S31" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T31" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="U31" t="s">
-        <v>175</v>
-      </c>
-      <c r="V31" s="2">
+        <v>178</v>
+      </c>
+      <c r="V31" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2538,31 +2521,34 @@
       <c r="F32" t="s">
         <v>31</v>
       </c>
+      <c r="K32" t="s">
+        <v>70</v>
+      </c>
       <c r="N32" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="O32" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="P32">
         <v>30000</v>
       </c>
       <c r="Q32" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R32" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="S32" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T32" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="U32" t="s">
-        <v>175</v>
-      </c>
-      <c r="V32" s="2">
+        <v>178</v>
+      </c>
+      <c r="V32" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2588,7 +2574,7 @@
       <c r="G33" t="s">
         <v>42</v>
       </c>
-      <c r="H33" s="2">
+      <c r="H33" s="1">
         <v>46191</v>
       </c>
       <c r="I33" t="s">
@@ -2598,30 +2584,30 @@
         <v>66</v>
       </c>
       <c r="N33" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="O33" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="P33">
         <v>1496713.48</v>
       </c>
       <c r="Q33" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R33" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="S33" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T33" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U33" t="s">
-        <v>175</v>
-      </c>
-      <c r="V33" s="2">
+        <v>178</v>
+      </c>
+      <c r="V33" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2647,37 +2633,37 @@
       <c r="G34" t="s">
         <v>42</v>
       </c>
-      <c r="H34" s="2">
+      <c r="H34" s="1">
         <v>46119</v>
       </c>
       <c r="I34" t="s">
         <v>50</v>
       </c>
       <c r="N34" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="O34" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="P34">
         <v>207789.52</v>
       </c>
       <c r="Q34" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R34" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="S34" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T34" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U34" t="s">
-        <v>175</v>
-      </c>
-      <c r="V34" s="2">
+        <v>178</v>
+      </c>
+      <c r="V34" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2703,37 +2689,37 @@
       <c r="G35" t="s">
         <v>42</v>
       </c>
-      <c r="H35" s="2">
+      <c r="H35" s="1">
         <v>46213</v>
       </c>
       <c r="I35" t="s">
         <v>56</v>
       </c>
       <c r="N35" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="O35" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="P35">
         <v>962290.8</v>
       </c>
       <c r="Q35" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R35" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="S35" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T35" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="U35" t="s">
         <v>29</v>
       </c>
-      <c r="V35" s="2">
+      <c r="V35" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -2759,37 +2745,37 @@
       <c r="G36" t="s">
         <v>42</v>
       </c>
-      <c r="H36" s="2">
+      <c r="H36" s="1">
         <v>46175</v>
       </c>
       <c r="I36" t="s">
         <v>57</v>
       </c>
       <c r="N36" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="O36" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="P36">
         <v>798776.97</v>
       </c>
       <c r="Q36" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R36" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="S36" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T36" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="U36" t="s">
         <v>29</v>
       </c>
-      <c r="V36" s="2">
+      <c r="V36" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2815,37 +2801,37 @@
       <c r="G37" t="s">
         <v>42</v>
       </c>
-      <c r="H37" s="2">
+      <c r="H37" s="1">
         <v>46213</v>
       </c>
       <c r="I37" t="s">
         <v>56</v>
       </c>
       <c r="N37" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="O37" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="P37">
         <v>1530656.62</v>
       </c>
       <c r="Q37" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R37" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="S37" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T37" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="U37" t="s">
         <v>29</v>
       </c>
-      <c r="V37" s="2">
+      <c r="V37" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -2871,37 +2857,37 @@
       <c r="G38" t="s">
         <v>42</v>
       </c>
-      <c r="H38" s="2">
+      <c r="H38" s="1">
         <v>46199</v>
       </c>
       <c r="I38" t="s">
         <v>58</v>
       </c>
       <c r="N38" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="O38" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="P38">
         <v>72958.08</v>
       </c>
       <c r="Q38" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R38" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="S38" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T38" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="U38" t="s">
         <v>29</v>
       </c>
-      <c r="V38" s="2">
+      <c r="V38" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2927,37 +2913,37 @@
       <c r="G39" t="s">
         <v>42</v>
       </c>
-      <c r="H39" s="2">
+      <c r="H39" s="1">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
         <v>58</v>
       </c>
       <c r="N39" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="O39" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="P39">
         <v>8916</v>
       </c>
       <c r="Q39" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R39" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="S39" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T39" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="U39" t="s">
         <v>29</v>
       </c>
-      <c r="V39" s="2">
+      <c r="V39" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2983,37 +2969,37 @@
       <c r="G40" t="s">
         <v>42</v>
       </c>
-      <c r="H40" s="2">
+      <c r="H40" s="1">
         <v>46204</v>
       </c>
       <c r="I40" t="s">
         <v>58</v>
       </c>
       <c r="N40" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="O40" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="P40">
         <v>425178.5</v>
       </c>
       <c r="Q40" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R40" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="S40" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T40" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="U40" t="s">
         <v>29</v>
       </c>
-      <c r="V40" s="2">
+      <c r="V40" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3039,37 +3025,37 @@
       <c r="G41" t="s">
         <v>42</v>
       </c>
-      <c r="H41" s="2">
+      <c r="H41" s="1">
         <v>46244</v>
       </c>
       <c r="I41" t="s">
         <v>59</v>
       </c>
       <c r="N41" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="O41" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="P41">
         <v>1223.03</v>
       </c>
       <c r="Q41" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R41" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="S41" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T41" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="U41" t="s">
         <v>29</v>
       </c>
-      <c r="V41" s="2">
+      <c r="V41" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3093,27 +3079,27 @@
         <v>43</v>
       </c>
       <c r="N42" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="O42" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="Q42" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R42" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="S42" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="T42" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="U42" t="s">
         <v>29</v>
       </c>
-      <c r="V42" s="2">
+      <c r="V42" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3139,37 +3125,37 @@
       <c r="G43" t="s">
         <v>42</v>
       </c>
-      <c r="H43" s="2">
+      <c r="H43" s="1">
         <v>46191</v>
       </c>
       <c r="I43" t="s">
         <v>60</v>
       </c>
       <c r="N43" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="O43" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="P43">
         <v>400000</v>
       </c>
       <c r="Q43" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R43" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="S43" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T43" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="U43" t="s">
         <v>29</v>
       </c>
-      <c r="V43" s="2">
+      <c r="V43" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3195,37 +3181,37 @@
       <c r="G44" t="s">
         <v>42</v>
       </c>
-      <c r="H44" s="2">
+      <c r="H44" s="1">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
         <v>60</v>
       </c>
       <c r="N44" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="O44" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="P44">
         <v>400000</v>
       </c>
       <c r="Q44" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R44" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="S44" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T44" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="U44" t="s">
         <v>29</v>
       </c>
-      <c r="V44" s="2">
+      <c r="V44" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3251,7 +3237,7 @@
       <c r="G45" t="s">
         <v>42</v>
       </c>
-      <c r="H45" s="2">
+      <c r="H45" s="1">
         <v>46213</v>
       </c>
       <c r="I45" t="s">
@@ -3261,30 +3247,30 @@
         <v>67</v>
       </c>
       <c r="N45" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="O45" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="P45">
         <v>173846.38</v>
       </c>
       <c r="Q45" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R45" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="S45" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T45" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U45" t="s">
-        <v>175</v>
-      </c>
-      <c r="V45" s="2">
+        <v>178</v>
+      </c>
+      <c r="V45" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3310,37 +3296,37 @@
       <c r="G46" t="s">
         <v>42</v>
       </c>
-      <c r="H46" s="2">
+      <c r="H46" s="1">
         <v>46210</v>
       </c>
       <c r="I46" t="s">
         <v>54</v>
       </c>
       <c r="N46" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="O46" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="P46">
         <v>1530656.62</v>
       </c>
       <c r="Q46" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R46" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="S46" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T46" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U46" t="s">
-        <v>175</v>
-      </c>
-      <c r="V46" s="2">
+        <v>178</v>
+      </c>
+      <c r="V46" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3364,30 +3350,30 @@
         <v>31</v>
       </c>
       <c r="N47" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="O47" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="P47">
         <v>1000000</v>
       </c>
       <c r="Q47" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R47" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="S47" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T47" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="U47" t="s">
         <v>29</v>
       </c>
-      <c r="V47" s="2">
+      <c r="V47" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3411,30 +3397,30 @@
         <v>31</v>
       </c>
       <c r="N48" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="O48" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="P48">
         <v>958040</v>
       </c>
       <c r="Q48" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="R48" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="S48" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T48" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="U48" t="s">
-        <v>175</v>
-      </c>
-      <c r="V48" s="2">
+        <v>178</v>
+      </c>
+      <c r="V48" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3460,7 +3446,7 @@
       <c r="G49" t="s">
         <v>42</v>
       </c>
-      <c r="H49" s="2">
+      <c r="H49" s="1">
         <v>46176</v>
       </c>
       <c r="I49" t="s">
@@ -3470,30 +3456,30 @@
         <v>68</v>
       </c>
       <c r="N49" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="O49" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="P49">
         <v>41730.64</v>
       </c>
       <c r="Q49" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="R49" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="S49" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T49" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="U49" t="s">
-        <v>175</v>
-      </c>
-      <c r="V49" s="2">
+        <v>178</v>
+      </c>
+      <c r="V49" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3520,33 +3506,33 @@
         <v>67</v>
       </c>
       <c r="K50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="N50" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="O50" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="P50">
         <v>1468159.32</v>
       </c>
       <c r="Q50" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R50" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="S50" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T50" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U50" t="s">
-        <v>175</v>
-      </c>
-      <c r="V50" s="2">
+        <v>178</v>
+      </c>
+      <c r="V50" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3573,33 +3559,33 @@
         <v>67</v>
       </c>
       <c r="K51" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="N51" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="O51" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="P51">
         <v>1704503</v>
       </c>
       <c r="Q51" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R51" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="S51" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T51" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U51" t="s">
-        <v>175</v>
-      </c>
-      <c r="V51" s="2">
+        <v>178</v>
+      </c>
+      <c r="V51" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3623,33 +3609,33 @@
         <v>31</v>
       </c>
       <c r="K52" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="N52" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="O52" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="P52">
         <v>1704503</v>
       </c>
       <c r="Q52" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R52" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="S52" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T52" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U52" t="s">
-        <v>175</v>
-      </c>
-      <c r="V52" s="2">
+        <v>178</v>
+      </c>
+      <c r="V52" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3675,37 +3661,37 @@
       <c r="G53" t="s">
         <v>42</v>
       </c>
-      <c r="H53" s="2">
+      <c r="H53" s="1">
         <v>46227</v>
       </c>
       <c r="I53" t="s">
         <v>62</v>
       </c>
       <c r="N53" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="O53" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="P53">
         <v>236343.68</v>
       </c>
       <c r="Q53" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R53" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="S53" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T53" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U53" t="s">
-        <v>175</v>
-      </c>
-      <c r="V53" s="2">
+        <v>178</v>
+      </c>
+      <c r="V53" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3728,31 +3714,34 @@
       <c r="F54" t="s">
         <v>31</v>
       </c>
+      <c r="K54" t="s">
+        <v>74</v>
+      </c>
       <c r="N54" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="O54" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="P54">
         <v>1295422.28</v>
       </c>
       <c r="Q54" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R54" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="S54" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T54" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U54" t="s">
-        <v>175</v>
-      </c>
-      <c r="V54" s="2">
+        <v>178</v>
+      </c>
+      <c r="V54" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -3776,33 +3765,33 @@
         <v>40</v>
       </c>
       <c r="K55" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="N55" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="O55" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="P55">
         <v>500000</v>
       </c>
       <c r="Q55" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R55" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="S55" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T55" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="U55" t="s">
-        <v>175</v>
-      </c>
-      <c r="V55" s="2">
+        <v>178</v>
+      </c>
+      <c r="V55" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3829,30 +3818,30 @@
         <v>44</v>
       </c>
       <c r="N56" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="O56" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="P56">
         <v>5000000</v>
       </c>
       <c r="Q56" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R56" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="S56" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T56" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="U56" t="s">
-        <v>175</v>
-      </c>
-      <c r="V56" s="2">
+        <v>178</v>
+      </c>
+      <c r="V56" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3876,27 +3865,27 @@
         <v>43</v>
       </c>
       <c r="N57" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="O57" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="Q57" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R57" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="S57" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T57" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="U57" t="s">
-        <v>175</v>
-      </c>
-      <c r="V57" s="2">
+        <v>178</v>
+      </c>
+      <c r="V57" s="1">
         <v>46049</v>
       </c>
     </row>
@@ -3920,25 +3909,25 @@
         <v>43</v>
       </c>
       <c r="N58" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="O58" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="Q58" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R58" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="S58" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T58" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="U58" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
     </row>
     <row r="59" spans="1:22">
@@ -3961,25 +3950,25 @@
         <v>43</v>
       </c>
       <c r="N59" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="O59" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="Q59" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R59" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="S59" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T59" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="U59" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
     </row>
     <row r="60" spans="1:22">
@@ -3999,30 +3988,30 @@
         <v>30</v>
       </c>
       <c r="N60" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="O60" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="P60">
         <v>9389.959999999999</v>
       </c>
       <c r="Q60" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="R60" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="S60" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="T60" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="U60" t="s">
-        <v>175</v>
-      </c>
-      <c r="V60" s="2">
+        <v>178</v>
+      </c>
+      <c r="V60" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4043,30 +4032,30 @@
         <v>30</v>
       </c>
       <c r="N61" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="O61" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="P61">
         <v>7204.82</v>
       </c>
       <c r="Q61" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="R61" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="S61" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="T61" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="U61" t="s">
-        <v>175</v>
-      </c>
-      <c r="V61" s="2">
+        <v>178</v>
+      </c>
+      <c r="V61" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4087,30 +4076,30 @@
         <v>30</v>
       </c>
       <c r="N62" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="O62" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="P62">
         <v>4227.84</v>
       </c>
       <c r="Q62" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="R62" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="S62" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="T62" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="U62" t="s">
-        <v>175</v>
-      </c>
-      <c r="V62" s="2">
+        <v>178</v>
+      </c>
+      <c r="V62" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4131,30 +4120,30 @@
         <v>30</v>
       </c>
       <c r="N63" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="O63" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="P63">
         <v>4064.54</v>
       </c>
       <c r="Q63" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R63" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="S63" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="T63" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="U63" t="s">
-        <v>175</v>
-      </c>
-      <c r="V63" s="2">
+        <v>178</v>
+      </c>
+      <c r="V63" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4175,30 +4164,30 @@
         <v>30</v>
       </c>
       <c r="N64" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="O64" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="P64">
         <v>3662.66</v>
       </c>
       <c r="Q64" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="R64" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="S64" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="T64" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="U64" t="s">
-        <v>175</v>
-      </c>
-      <c r="V64" s="2">
+        <v>178</v>
+      </c>
+      <c r="V64" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4219,30 +4208,30 @@
         <v>30</v>
       </c>
       <c r="N65" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="O65" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="P65">
         <v>1163.64</v>
       </c>
       <c r="Q65" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="R65" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="S65" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="T65" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="U65" t="s">
-        <v>175</v>
-      </c>
-      <c r="V65" s="2">
+        <v>178</v>
+      </c>
+      <c r="V65" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4263,30 +4252,30 @@
         <v>30</v>
       </c>
       <c r="N66" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="O66" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="P66">
         <v>120000</v>
       </c>
       <c r="Q66" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="R66" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="S66" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="T66" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="U66" t="s">
         <v>29</v>
       </c>
-      <c r="V66" s="2">
+      <c r="V66" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4310,30 +4299,30 @@
         <v>31</v>
       </c>
       <c r="N67" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="O67" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="P67">
         <v>400000</v>
       </c>
       <c r="Q67" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="R67" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="S67" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T67" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="U67" t="s">
         <v>29</v>
       </c>
-      <c r="V67" s="2">
+      <c r="V67" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4357,30 +4346,30 @@
         <v>31</v>
       </c>
       <c r="N68" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="O68" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="P68">
         <v>100000</v>
       </c>
       <c r="Q68" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="R68" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="S68" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T68" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="U68" t="s">
-        <v>175</v>
-      </c>
-      <c r="V68" s="2">
+        <v>178</v>
+      </c>
+      <c r="V68" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -4401,30 +4390,30 @@
         <v>30</v>
       </c>
       <c r="N69" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="O69" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="P69">
         <v>80000</v>
       </c>
       <c r="Q69" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="R69" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="S69" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="T69" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="U69" t="s">
         <v>29</v>
       </c>
-      <c r="V69" s="2">
+      <c r="V69" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -4445,30 +4434,30 @@
         <v>30</v>
       </c>
       <c r="N70" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="O70" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="P70">
         <v>835000</v>
       </c>
       <c r="Q70" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="R70" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="S70" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="T70" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="U70" t="s">
-        <v>175</v>
-      </c>
-      <c r="V70" s="2">
+        <v>178</v>
+      </c>
+      <c r="V70" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4489,30 +4478,30 @@
         <v>30</v>
       </c>
       <c r="N71" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="O71" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="P71">
         <v>165000</v>
       </c>
       <c r="Q71" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="R71" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="S71" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="T71" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="U71" t="s">
-        <v>175</v>
-      </c>
-      <c r="V71" s="2">
+        <v>178</v>
+      </c>
+      <c r="V71" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4533,30 +4522,30 @@
         <v>30</v>
       </c>
       <c r="N72" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="O72" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="P72">
         <v>1000000</v>
       </c>
       <c r="Q72" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="R72" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="S72" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="T72" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="U72" t="s">
-        <v>175</v>
-      </c>
-      <c r="V72" s="2">
+        <v>178</v>
+      </c>
+      <c r="V72" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4577,30 +4566,30 @@
         <v>30</v>
       </c>
       <c r="N73" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="O73" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="P73">
         <v>1000000</v>
       </c>
       <c r="Q73" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="R73" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="S73" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="T73" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="U73" t="s">
-        <v>175</v>
-      </c>
-      <c r="V73" s="2">
+        <v>178</v>
+      </c>
+      <c r="V73" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4621,30 +4610,30 @@
         <v>30</v>
       </c>
       <c r="N74" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="O74" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="P74">
         <v>100000</v>
       </c>
       <c r="Q74" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="R74" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="S74" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="T74" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="U74" t="s">
-        <v>175</v>
-      </c>
-      <c r="V74" s="2">
+        <v>178</v>
+      </c>
+      <c r="V74" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4668,30 +4657,30 @@
         <v>31</v>
       </c>
       <c r="N75" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="O75" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="P75">
         <v>1000000</v>
       </c>
       <c r="Q75" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R75" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="S75" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T75" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="U75" t="s">
         <v>29</v>
       </c>
-      <c r="V75" s="2">
+      <c r="V75" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -4718,30 +4707,30 @@
         <v>45</v>
       </c>
       <c r="N76" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="O76" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="P76">
         <v>1704503</v>
       </c>
       <c r="Q76" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R76" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="S76" t="s">
         <v>41</v>
       </c>
       <c r="T76" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U76" t="s">
-        <v>175</v>
-      </c>
-      <c r="V76" s="2">
+        <v>178</v>
+      </c>
+      <c r="V76" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4768,30 +4757,30 @@
         <v>45</v>
       </c>
       <c r="N77" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="O77" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="P77">
         <v>1638125.5</v>
       </c>
       <c r="Q77" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R77" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="S77" t="s">
         <v>41</v>
       </c>
       <c r="T77" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U77" t="s">
-        <v>175</v>
-      </c>
-      <c r="V77" s="2">
+        <v>178</v>
+      </c>
+      <c r="V77" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4818,30 +4807,30 @@
         <v>45</v>
       </c>
       <c r="N78" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="O78" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="P78">
         <v>3800000</v>
       </c>
       <c r="Q78" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R78" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="S78" t="s">
         <v>41</v>
       </c>
       <c r="T78" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="U78" t="s">
         <v>29</v>
       </c>
-      <c r="V78" s="2">
+      <c r="V78" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4868,30 +4857,30 @@
         <v>45</v>
       </c>
       <c r="N79" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="O79" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="P79">
         <v>3800000</v>
       </c>
       <c r="Q79" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R79" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="S79" t="s">
         <v>41</v>
       </c>
       <c r="T79" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="U79" t="s">
         <v>29</v>
       </c>
-      <c r="V79" s="2">
+      <c r="V79" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4915,33 +4904,33 @@
         <v>69</v>
       </c>
       <c r="K80" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="N80" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="O80" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="P80">
         <v>3800000</v>
       </c>
       <c r="Q80" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R80" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="S80" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="T80" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="U80" t="s">
         <v>29</v>
       </c>
-      <c r="V80" s="2">
+      <c r="V80" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -4962,30 +4951,30 @@
         <v>29</v>
       </c>
       <c r="N81" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="O81" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="P81">
         <v>4394700</v>
       </c>
       <c r="Q81" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="R81" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="S81" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="T81" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="U81" t="s">
         <v>29</v>
       </c>
-      <c r="V81" s="2">
+      <c r="V81" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5008,31 +4997,34 @@
       <c r="F82" t="s">
         <v>31</v>
       </c>
+      <c r="K82" t="s">
+        <v>76</v>
+      </c>
       <c r="N82" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="O82" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="P82">
         <v>528395.9300000001</v>
       </c>
       <c r="Q82" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R82" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="S82" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T82" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U82" t="s">
-        <v>175</v>
-      </c>
-      <c r="V82" s="2">
+        <v>178</v>
+      </c>
+      <c r="V82" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5053,30 +5045,30 @@
         <v>30</v>
       </c>
       <c r="N83" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="O83" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="P83">
         <v>1000000</v>
       </c>
       <c r="Q83" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R83" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="S83" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="T83" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="U83" t="s">
         <v>29</v>
       </c>
-      <c r="V83" s="2">
+      <c r="V83" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -5097,30 +5089,30 @@
         <v>29</v>
       </c>
       <c r="N84" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="O84" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="P84">
         <v>4394700</v>
       </c>
       <c r="Q84" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="R84" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="S84" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="T84" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="U84" t="s">
         <v>29</v>
       </c>
-      <c r="V84" s="2">
+      <c r="V84" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5147,25 +5139,25 @@
         <v>45</v>
       </c>
       <c r="N85" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="O85" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="P85">
         <v>3306000</v>
       </c>
       <c r="Q85" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="R85" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="S85" t="s">
         <v>41</v>
       </c>
       <c r="T85" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="U85" t="s">
         <v>29</v>
@@ -5194,25 +5186,25 @@
         <v>45</v>
       </c>
       <c r="N86" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="O86" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="P86">
         <v>3306000</v>
       </c>
       <c r="Q86" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="R86" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="S86" t="s">
         <v>41</v>
       </c>
       <c r="T86" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="U86" t="s">
         <v>29</v>
@@ -5238,30 +5230,30 @@
         <v>31</v>
       </c>
       <c r="N87" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="O87" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="P87">
         <v>212577</v>
       </c>
       <c r="Q87" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R87" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="S87" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="T87" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="U87" t="s">
         <v>30</v>
       </c>
-      <c r="V87" s="2">
+      <c r="V87" s="1">
         <v>46260</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (21/08/2026 10:52)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -517,10 +517,13 @@
     <t>CELOG</t>
   </si>
   <si>
-    <t>DÓLAR</t>
-  </si>
-  <si>
-    <t>REAL</t>
+    <t>339039</t>
+  </si>
+  <si>
+    <t>339030</t>
+  </si>
+  <si>
+    <t>449052</t>
   </si>
   <si>
     <t>A</t>
@@ -535,12 +538,6 @@
     <t>B</t>
   </si>
   <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
     <t>REQUISIÇÃO</t>
   </si>
   <si>
@@ -551,6 +548,9 @@
   </si>
   <si>
     <t>PARCELA FIXA</t>
+  </si>
+  <si>
+    <t>Não</t>
   </si>
 </sst>
 </file>
@@ -560,16 +560,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -585,7 +577,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -593,30 +585,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -916,70 +890,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1012,7 +986,7 @@
         <v>97</v>
       </c>
       <c r="P2">
-        <v>46229</v>
+        <v>135000</v>
       </c>
       <c r="Q2" t="s">
         <v>164</v>
@@ -1021,16 +995,16 @@
         <v>167</v>
       </c>
       <c r="S2" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T2" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="U2" t="s">
-        <v>175</v>
-      </c>
-      <c r="V2" s="2">
-        <v>46291</v>
+        <v>178</v>
+      </c>
+      <c r="V2" s="1">
+        <v>46229</v>
       </c>
     </row>
     <row r="3" spans="1:22">
@@ -1059,25 +1033,25 @@
         <v>98</v>
       </c>
       <c r="P3">
-        <v>46291</v>
+        <v>400000</v>
       </c>
       <c r="Q3" t="s">
         <v>165</v>
       </c>
       <c r="R3" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S3" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T3" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="U3" t="s">
-        <v>175</v>
-      </c>
-      <c r="V3" s="2">
-        <v>46382</v>
+        <v>29</v>
+      </c>
+      <c r="V3" s="1">
+        <v>46291</v>
       </c>
     </row>
     <row r="4" spans="1:22">
@@ -1106,7 +1080,7 @@
         <v>99</v>
       </c>
       <c r="P4">
-        <v>46321</v>
+        <v>430000</v>
       </c>
       <c r="Q4" t="s">
         <v>164</v>
@@ -1115,16 +1089,16 @@
         <v>167</v>
       </c>
       <c r="S4" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T4" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="U4" t="s">
-        <v>175</v>
-      </c>
-      <c r="V4" s="2">
-        <v>46169</v>
+        <v>29</v>
+      </c>
+      <c r="V4" s="1">
+        <v>46321</v>
       </c>
     </row>
     <row r="5" spans="1:22">
@@ -1153,7 +1127,7 @@
         <v>100</v>
       </c>
       <c r="P5">
-        <v>46321</v>
+        <v>425000</v>
       </c>
       <c r="Q5" t="s">
         <v>164</v>
@@ -1162,16 +1136,16 @@
         <v>167</v>
       </c>
       <c r="S5" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T5" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="U5" t="s">
-        <v>175</v>
-      </c>
-      <c r="V5" s="2">
-        <v>46169</v>
+        <v>29</v>
+      </c>
+      <c r="V5" s="1">
+        <v>46321</v>
       </c>
     </row>
     <row r="6" spans="1:22">
@@ -1203,7 +1177,7 @@
         <v>101</v>
       </c>
       <c r="P6">
-        <v>46291</v>
+        <v>563000</v>
       </c>
       <c r="Q6" t="s">
         <v>164</v>
@@ -1212,16 +1186,16 @@
         <v>167</v>
       </c>
       <c r="S6" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T6" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="U6" t="s">
-        <v>175</v>
-      </c>
-      <c r="V6" s="2">
-        <v>46352</v>
+        <v>29</v>
+      </c>
+      <c r="V6" s="1">
+        <v>46291</v>
       </c>
     </row>
     <row r="7" spans="1:22">
@@ -1246,7 +1220,7 @@
       <c r="G7" t="s">
         <v>42</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1259,24 +1233,24 @@
         <v>102</v>
       </c>
       <c r="P7">
-        <v>46138</v>
+        <v>3799999.6</v>
       </c>
       <c r="Q7" t="s">
         <v>166</v>
       </c>
       <c r="R7" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="S7" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T7" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="U7" t="s">
-        <v>176</v>
-      </c>
-      <c r="V7" s="2">
+        <v>29</v>
+      </c>
+      <c r="V7" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -1306,7 +1280,7 @@
         <v>103</v>
       </c>
       <c r="P8">
-        <v>46291</v>
+        <v>430000</v>
       </c>
       <c r="Q8" t="s">
         <v>164</v>
@@ -1315,16 +1289,16 @@
         <v>167</v>
       </c>
       <c r="S8" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T8" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="U8" t="s">
-        <v>175</v>
-      </c>
-      <c r="V8" s="2">
-        <v>46200</v>
+        <v>29</v>
+      </c>
+      <c r="V8" s="1">
+        <v>46291</v>
       </c>
     </row>
     <row r="9" spans="1:22">
@@ -1353,7 +1327,7 @@
         <v>104</v>
       </c>
       <c r="P9">
-        <v>46291</v>
+        <v>60000</v>
       </c>
       <c r="Q9" t="s">
         <v>164</v>
@@ -1362,16 +1336,16 @@
         <v>167</v>
       </c>
       <c r="S9" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T9" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="U9" t="s">
-        <v>175</v>
-      </c>
-      <c r="V9" s="2">
-        <v>46200</v>
+        <v>29</v>
+      </c>
+      <c r="V9" s="1">
+        <v>46291</v>
       </c>
     </row>
     <row r="10" spans="1:22">
@@ -1400,7 +1374,7 @@
         <v>105</v>
       </c>
       <c r="P10">
-        <v>46291</v>
+        <v>200000</v>
       </c>
       <c r="Q10" t="s">
         <v>164</v>
@@ -1409,16 +1383,16 @@
         <v>167</v>
       </c>
       <c r="S10" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T10" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="U10" t="s">
-        <v>175</v>
-      </c>
-      <c r="V10" s="2">
-        <v>46352</v>
+        <v>29</v>
+      </c>
+      <c r="V10" s="1">
+        <v>46291</v>
       </c>
     </row>
     <row r="11" spans="1:22">
@@ -1447,7 +1421,7 @@
         <v>106</v>
       </c>
       <c r="P11">
-        <v>46291</v>
+        <v>320000</v>
       </c>
       <c r="Q11" t="s">
         <v>164</v>
@@ -1456,16 +1430,16 @@
         <v>167</v>
       </c>
       <c r="S11" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T11" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="U11" t="s">
-        <v>175</v>
-      </c>
-      <c r="V11" s="2">
-        <v>46352</v>
+        <v>29</v>
+      </c>
+      <c r="V11" s="1">
+        <v>46291</v>
       </c>
     </row>
     <row r="12" spans="1:22">
@@ -1490,7 +1464,7 @@
       <c r="G12" t="s">
         <v>42</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46079</v>
       </c>
       <c r="I12" t="s">
@@ -1506,25 +1480,25 @@
         <v>107</v>
       </c>
       <c r="P12">
-        <v>46079</v>
+        <v>1187433.02</v>
       </c>
       <c r="Q12" t="s">
         <v>164</v>
       </c>
       <c r="R12" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S12" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T12" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="U12" t="s">
-        <v>175</v>
-      </c>
-      <c r="V12" s="2">
-        <v>46168</v>
+        <v>178</v>
+      </c>
+      <c r="V12" s="1">
+        <v>46079</v>
       </c>
     </row>
     <row r="13" spans="1:22">
@@ -1553,25 +1527,25 @@
         <v>108</v>
       </c>
       <c r="P13">
-        <v>46352</v>
+        <v>1000000</v>
       </c>
       <c r="Q13" t="s">
         <v>164</v>
       </c>
       <c r="R13" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S13" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T13" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="U13" t="s">
-        <v>175</v>
-      </c>
-      <c r="V13" s="2">
-        <v>46049</v>
+        <v>178</v>
+      </c>
+      <c r="V13" s="1">
+        <v>46352</v>
       </c>
     </row>
     <row r="14" spans="1:22">
@@ -1600,25 +1574,25 @@
         <v>109</v>
       </c>
       <c r="P14">
-        <v>46352</v>
+        <v>1000000</v>
       </c>
       <c r="Q14" t="s">
         <v>164</v>
       </c>
       <c r="R14" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S14" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T14" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="U14" t="s">
-        <v>175</v>
-      </c>
-      <c r="V14" s="2">
-        <v>46049</v>
+        <v>178</v>
+      </c>
+      <c r="V14" s="1">
+        <v>46352</v>
       </c>
     </row>
     <row r="15" spans="1:22">
@@ -1647,25 +1621,25 @@
         <v>110</v>
       </c>
       <c r="P15">
-        <v>46352</v>
+        <v>1000000</v>
       </c>
       <c r="Q15" t="s">
         <v>164</v>
       </c>
       <c r="R15" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S15" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T15" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="U15" t="s">
-        <v>175</v>
-      </c>
-      <c r="V15" s="2">
-        <v>46049</v>
+        <v>178</v>
+      </c>
+      <c r="V15" s="1">
+        <v>46352</v>
       </c>
     </row>
     <row r="16" spans="1:22">
@@ -1694,25 +1668,25 @@
         <v>111</v>
       </c>
       <c r="P16">
-        <v>46229</v>
+        <v>100000</v>
       </c>
       <c r="Q16" t="s">
         <v>165</v>
       </c>
       <c r="R16" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S16" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T16" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="U16" t="s">
-        <v>175</v>
-      </c>
-      <c r="V16" s="2">
-        <v>46291</v>
+        <v>178</v>
+      </c>
+      <c r="V16" s="1">
+        <v>46229</v>
       </c>
     </row>
     <row r="17" spans="1:22">
@@ -1737,7 +1711,7 @@
       <c r="G17" t="s">
         <v>42</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46098</v>
       </c>
       <c r="I17" t="s">
@@ -1753,25 +1727,25 @@
         <v>112</v>
       </c>
       <c r="P17">
-        <v>46107</v>
+        <v>1770880.5</v>
       </c>
       <c r="Q17" t="s">
         <v>166</v>
       </c>
       <c r="R17" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="S17" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T17" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U17" t="s">
-        <v>177</v>
-      </c>
-      <c r="V17" s="2">
-        <v>46168</v>
+        <v>178</v>
+      </c>
+      <c r="V17" s="1">
+        <v>46107</v>
       </c>
     </row>
     <row r="18" spans="1:22">
@@ -1796,7 +1770,7 @@
       <c r="G18" t="s">
         <v>42</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46076</v>
       </c>
       <c r="I18" t="s">
@@ -1809,7 +1783,7 @@
         <v>113</v>
       </c>
       <c r="P18">
-        <v>46079</v>
+        <v>350000</v>
       </c>
       <c r="Q18" t="s">
         <v>166</v>
@@ -1818,16 +1792,16 @@
         <v>168</v>
       </c>
       <c r="S18" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T18" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="U18" t="s">
-        <v>176</v>
-      </c>
-      <c r="V18" s="2">
-        <v>46260</v>
+        <v>29</v>
+      </c>
+      <c r="V18" s="1">
+        <v>46079</v>
       </c>
     </row>
     <row r="19" spans="1:22">
@@ -1852,7 +1826,7 @@
       <c r="G19" t="s">
         <v>42</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1865,7 +1839,7 @@
         <v>114</v>
       </c>
       <c r="P19">
-        <v>46079</v>
+        <v>350000</v>
       </c>
       <c r="Q19" t="s">
         <v>166</v>
@@ -1874,16 +1848,16 @@
         <v>168</v>
       </c>
       <c r="S19" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T19" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="U19" t="s">
-        <v>176</v>
-      </c>
-      <c r="V19" s="2">
-        <v>46260</v>
+        <v>29</v>
+      </c>
+      <c r="V19" s="1">
+        <v>46079</v>
       </c>
     </row>
     <row r="20" spans="1:22">
@@ -1912,7 +1886,7 @@
         <v>115</v>
       </c>
       <c r="P20">
-        <v>46321</v>
+        <v>1000000</v>
       </c>
       <c r="Q20" t="s">
         <v>166</v>
@@ -1921,16 +1895,16 @@
         <v>168</v>
       </c>
       <c r="S20" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T20" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="U20" t="s">
-        <v>176</v>
-      </c>
-      <c r="V20" s="2">
-        <v>46382</v>
+        <v>29</v>
+      </c>
+      <c r="V20" s="1">
+        <v>46321</v>
       </c>
     </row>
     <row r="21" spans="1:22">
@@ -1959,25 +1933,25 @@
         <v>116</v>
       </c>
       <c r="P21">
-        <v>46321</v>
+        <v>400000</v>
       </c>
       <c r="Q21" t="s">
         <v>165</v>
       </c>
       <c r="R21" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S21" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T21" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="U21" t="s">
-        <v>175</v>
-      </c>
-      <c r="V21" s="2">
-        <v>46382</v>
+        <v>29</v>
+      </c>
+      <c r="V21" s="1">
+        <v>46321</v>
       </c>
     </row>
     <row r="22" spans="1:22">
@@ -2006,7 +1980,7 @@
         <v>117</v>
       </c>
       <c r="P22">
-        <v>46321</v>
+        <v>120000</v>
       </c>
       <c r="Q22" t="s">
         <v>164</v>
@@ -2015,16 +1989,16 @@
         <v>167</v>
       </c>
       <c r="S22" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T22" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="U22" t="s">
-        <v>175</v>
-      </c>
-      <c r="V22" s="2">
-        <v>46230</v>
+        <v>29</v>
+      </c>
+      <c r="V22" s="1">
+        <v>46321</v>
       </c>
     </row>
     <row r="23" spans="1:22">
@@ -2053,7 +2027,7 @@
         <v>118</v>
       </c>
       <c r="P23">
-        <v>46321</v>
+        <v>80000</v>
       </c>
       <c r="Q23" t="s">
         <v>164</v>
@@ -2062,16 +2036,16 @@
         <v>167</v>
       </c>
       <c r="S23" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T23" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="U23" t="s">
-        <v>175</v>
-      </c>
-      <c r="V23" s="2">
-        <v>46230</v>
+        <v>29</v>
+      </c>
+      <c r="V23" s="1">
+        <v>46321</v>
       </c>
     </row>
     <row r="24" spans="1:22">
@@ -2096,7 +2070,7 @@
       <c r="G24" t="s">
         <v>42</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>46119</v>
       </c>
       <c r="I24" t="s">
@@ -2112,25 +2086,25 @@
         <v>119</v>
       </c>
       <c r="P24">
-        <v>46138</v>
+        <v>1704503</v>
       </c>
       <c r="Q24" t="s">
         <v>166</v>
       </c>
       <c r="R24" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="S24" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T24" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U24" t="s">
-        <v>177</v>
-      </c>
-      <c r="V24" s="2">
-        <v>46199</v>
+        <v>178</v>
+      </c>
+      <c r="V24" s="1">
+        <v>46138</v>
       </c>
     </row>
     <row r="25" spans="1:22">
@@ -2155,7 +2129,7 @@
       <c r="G25" t="s">
         <v>42</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>46121</v>
       </c>
       <c r="I25" t="s">
@@ -2168,25 +2142,25 @@
         <v>120</v>
       </c>
       <c r="P25">
-        <v>46138</v>
+        <v>3799000</v>
       </c>
       <c r="Q25" t="s">
         <v>166</v>
       </c>
       <c r="R25" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="S25" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T25" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="U25" t="s">
-        <v>176</v>
-      </c>
-      <c r="V25" s="2">
-        <v>46199</v>
+        <v>29</v>
+      </c>
+      <c r="V25" s="1">
+        <v>46138</v>
       </c>
     </row>
     <row r="26" spans="1:22">
@@ -2211,7 +2185,7 @@
       <c r="G26" t="s">
         <v>42</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>46076</v>
       </c>
       <c r="I26" t="s">
@@ -2224,7 +2198,7 @@
         <v>120</v>
       </c>
       <c r="P26">
-        <v>46079</v>
+        <v>1000</v>
       </c>
       <c r="Q26" t="s">
         <v>166</v>
@@ -2233,16 +2207,16 @@
         <v>168</v>
       </c>
       <c r="S26" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T26" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="U26" t="s">
-        <v>176</v>
-      </c>
-      <c r="V26" s="2">
-        <v>46352</v>
+        <v>29</v>
+      </c>
+      <c r="V26" s="1">
+        <v>46079</v>
       </c>
     </row>
     <row r="27" spans="1:22">
@@ -2271,25 +2245,25 @@
         <v>121</v>
       </c>
       <c r="P27">
-        <v>46291</v>
+        <v>100000</v>
       </c>
       <c r="Q27" t="s">
         <v>165</v>
       </c>
       <c r="R27" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S27" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T27" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="U27" t="s">
-        <v>175</v>
-      </c>
-      <c r="V27" s="2">
-        <v>46352</v>
+        <v>178</v>
+      </c>
+      <c r="V27" s="1">
+        <v>46291</v>
       </c>
     </row>
     <row r="28" spans="1:22">
@@ -2314,7 +2288,7 @@
       <c r="G28" t="s">
         <v>42</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>46199</v>
       </c>
       <c r="I28" t="s">
@@ -2330,25 +2304,25 @@
         <v>122</v>
       </c>
       <c r="P28">
-        <v>46199</v>
+        <v>150000</v>
       </c>
       <c r="Q28" t="s">
         <v>166</v>
       </c>
       <c r="R28" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="S28" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T28" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="U28" t="s">
-        <v>176</v>
-      </c>
-      <c r="V28" s="2">
-        <v>46260</v>
+        <v>178</v>
+      </c>
+      <c r="V28" s="1">
+        <v>46199</v>
       </c>
     </row>
     <row r="29" spans="1:22">
@@ -2373,7 +2347,7 @@
       <c r="G29" t="s">
         <v>42</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2389,25 +2363,25 @@
         <v>123</v>
       </c>
       <c r="P29">
-        <v>46199</v>
+        <v>150000</v>
       </c>
       <c r="Q29" t="s">
         <v>166</v>
       </c>
       <c r="R29" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="S29" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T29" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="U29" t="s">
-        <v>176</v>
-      </c>
-      <c r="V29" s="2">
-        <v>46260</v>
+        <v>178</v>
+      </c>
+      <c r="V29" s="1">
+        <v>46199</v>
       </c>
     </row>
     <row r="30" spans="1:22">
@@ -2432,7 +2406,7 @@
       <c r="G30" t="s">
         <v>42</v>
       </c>
-      <c r="H30" s="2">
+      <c r="H30" s="1">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2448,25 +2422,25 @@
         <v>124</v>
       </c>
       <c r="P30">
-        <v>46199</v>
+        <v>18462.36</v>
       </c>
       <c r="Q30" t="s">
         <v>166</v>
       </c>
       <c r="R30" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="S30" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T30" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="U30" t="s">
-        <v>176</v>
-      </c>
-      <c r="V30" s="2">
-        <v>46260</v>
+        <v>178</v>
+      </c>
+      <c r="V30" s="1">
+        <v>46199</v>
       </c>
     </row>
     <row r="31" spans="1:22">
@@ -2491,7 +2465,7 @@
       <c r="G31" t="s">
         <v>42</v>
       </c>
-      <c r="H31" s="2">
+      <c r="H31" s="1">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2507,25 +2481,25 @@
         <v>124</v>
       </c>
       <c r="P31">
-        <v>46199</v>
+        <v>324166.14</v>
       </c>
       <c r="Q31" t="s">
         <v>166</v>
       </c>
       <c r="R31" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="S31" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T31" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="U31" t="s">
-        <v>176</v>
-      </c>
-      <c r="V31" s="2">
-        <v>46260</v>
+        <v>178</v>
+      </c>
+      <c r="V31" s="1">
+        <v>46199</v>
       </c>
     </row>
     <row r="32" spans="1:22">
@@ -2557,25 +2531,25 @@
         <v>125</v>
       </c>
       <c r="P32">
-        <v>46291</v>
+        <v>30000</v>
       </c>
       <c r="Q32" t="s">
         <v>166</v>
       </c>
       <c r="R32" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="S32" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T32" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="U32" t="s">
-        <v>176</v>
-      </c>
-      <c r="V32" s="2">
-        <v>46352</v>
+        <v>178</v>
+      </c>
+      <c r="V32" s="1">
+        <v>46291</v>
       </c>
     </row>
     <row r="33" spans="1:22">
@@ -2600,7 +2574,7 @@
       <c r="G33" t="s">
         <v>42</v>
       </c>
-      <c r="H33" s="2">
+      <c r="H33" s="1">
         <v>46191</v>
       </c>
       <c r="I33" t="s">
@@ -2616,25 +2590,25 @@
         <v>126</v>
       </c>
       <c r="P33">
-        <v>46199</v>
+        <v>1496713.48</v>
       </c>
       <c r="Q33" t="s">
         <v>166</v>
       </c>
       <c r="R33" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="S33" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T33" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U33" t="s">
-        <v>177</v>
-      </c>
-      <c r="V33" s="2">
-        <v>46260</v>
+        <v>178</v>
+      </c>
+      <c r="V33" s="1">
+        <v>46199</v>
       </c>
     </row>
     <row r="34" spans="1:22">
@@ -2659,7 +2633,7 @@
       <c r="G34" t="s">
         <v>42</v>
       </c>
-      <c r="H34" s="2">
+      <c r="H34" s="1">
         <v>46119</v>
       </c>
       <c r="I34" t="s">
@@ -2672,25 +2646,25 @@
         <v>126</v>
       </c>
       <c r="P34">
-        <v>46138</v>
+        <v>207789.52</v>
       </c>
       <c r="Q34" t="s">
         <v>166</v>
       </c>
       <c r="R34" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="S34" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T34" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U34" t="s">
-        <v>177</v>
-      </c>
-      <c r="V34" s="2">
-        <v>46260</v>
+        <v>178</v>
+      </c>
+      <c r="V34" s="1">
+        <v>46138</v>
       </c>
     </row>
     <row r="35" spans="1:22">
@@ -2715,7 +2689,7 @@
       <c r="G35" t="s">
         <v>42</v>
       </c>
-      <c r="H35" s="2">
+      <c r="H35" s="1">
         <v>46213</v>
       </c>
       <c r="I35" t="s">
@@ -2728,7 +2702,7 @@
         <v>127</v>
       </c>
       <c r="P35">
-        <v>46229</v>
+        <v>962290.8</v>
       </c>
       <c r="Q35" t="s">
         <v>166</v>
@@ -2737,16 +2711,16 @@
         <v>168</v>
       </c>
       <c r="S35" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T35" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="U35" t="s">
-        <v>176</v>
-      </c>
-      <c r="V35" s="2">
-        <v>46352</v>
+        <v>29</v>
+      </c>
+      <c r="V35" s="1">
+        <v>46229</v>
       </c>
     </row>
     <row r="36" spans="1:22">
@@ -2771,7 +2745,7 @@
       <c r="G36" t="s">
         <v>42</v>
       </c>
-      <c r="H36" s="2">
+      <c r="H36" s="1">
         <v>46175</v>
       </c>
       <c r="I36" t="s">
@@ -2784,25 +2758,25 @@
         <v>127</v>
       </c>
       <c r="P36">
-        <v>46199</v>
+        <v>798776.97</v>
       </c>
       <c r="Q36" t="s">
         <v>166</v>
       </c>
       <c r="R36" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="S36" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T36" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="U36" t="s">
-        <v>176</v>
-      </c>
-      <c r="V36" s="2">
-        <v>46260</v>
+        <v>29</v>
+      </c>
+      <c r="V36" s="1">
+        <v>46199</v>
       </c>
     </row>
     <row r="37" spans="1:22">
@@ -2827,7 +2801,7 @@
       <c r="G37" t="s">
         <v>42</v>
       </c>
-      <c r="H37" s="2">
+      <c r="H37" s="1">
         <v>46213</v>
       </c>
       <c r="I37" t="s">
@@ -2840,7 +2814,7 @@
         <v>127</v>
       </c>
       <c r="P37">
-        <v>46229</v>
+        <v>1530656.62</v>
       </c>
       <c r="Q37" t="s">
         <v>166</v>
@@ -2849,16 +2823,16 @@
         <v>168</v>
       </c>
       <c r="S37" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T37" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="U37" t="s">
-        <v>176</v>
-      </c>
-      <c r="V37" s="2">
-        <v>46352</v>
+        <v>29</v>
+      </c>
+      <c r="V37" s="1">
+        <v>46229</v>
       </c>
     </row>
     <row r="38" spans="1:22">
@@ -2883,7 +2857,7 @@
       <c r="G38" t="s">
         <v>42</v>
       </c>
-      <c r="H38" s="2">
+      <c r="H38" s="1">
         <v>46199</v>
       </c>
       <c r="I38" t="s">
@@ -2896,7 +2870,7 @@
         <v>127</v>
       </c>
       <c r="P38">
-        <v>46199</v>
+        <v>72958.08</v>
       </c>
       <c r="Q38" t="s">
         <v>166</v>
@@ -2905,16 +2879,16 @@
         <v>168</v>
       </c>
       <c r="S38" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T38" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="U38" t="s">
-        <v>176</v>
-      </c>
-      <c r="V38" s="2">
-        <v>46229</v>
+        <v>29</v>
+      </c>
+      <c r="V38" s="1">
+        <v>46199</v>
       </c>
     </row>
     <row r="39" spans="1:22">
@@ -2939,7 +2913,7 @@
       <c r="G39" t="s">
         <v>42</v>
       </c>
-      <c r="H39" s="2">
+      <c r="H39" s="1">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -2952,7 +2926,7 @@
         <v>127</v>
       </c>
       <c r="P39">
-        <v>46199</v>
+        <v>8916</v>
       </c>
       <c r="Q39" t="s">
         <v>166</v>
@@ -2961,16 +2935,16 @@
         <v>168</v>
       </c>
       <c r="S39" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T39" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="U39" t="s">
-        <v>176</v>
-      </c>
-      <c r="V39" s="2">
-        <v>46229</v>
+        <v>29</v>
+      </c>
+      <c r="V39" s="1">
+        <v>46199</v>
       </c>
     </row>
     <row r="40" spans="1:22">
@@ -2995,7 +2969,7 @@
       <c r="G40" t="s">
         <v>42</v>
       </c>
-      <c r="H40" s="2">
+      <c r="H40" s="1">
         <v>46204</v>
       </c>
       <c r="I40" t="s">
@@ -3008,7 +2982,7 @@
         <v>127</v>
       </c>
       <c r="P40">
-        <v>46229</v>
+        <v>425178.5</v>
       </c>
       <c r="Q40" t="s">
         <v>166</v>
@@ -3017,15 +2991,15 @@
         <v>168</v>
       </c>
       <c r="S40" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T40" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="U40" t="s">
-        <v>176</v>
-      </c>
-      <c r="V40" s="2">
+        <v>29</v>
+      </c>
+      <c r="V40" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3051,7 +3025,7 @@
       <c r="G41" t="s">
         <v>42</v>
       </c>
-      <c r="H41" s="2">
+      <c r="H41" s="1">
         <v>46244</v>
       </c>
       <c r="I41" t="s">
@@ -3064,7 +3038,7 @@
         <v>127</v>
       </c>
       <c r="P41">
-        <v>46199</v>
+        <v>1223.03</v>
       </c>
       <c r="Q41" t="s">
         <v>166</v>
@@ -3073,16 +3047,16 @@
         <v>168</v>
       </c>
       <c r="S41" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T41" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="U41" t="s">
-        <v>176</v>
-      </c>
-      <c r="V41" s="2">
-        <v>46260</v>
+        <v>29</v>
+      </c>
+      <c r="V41" s="1">
+        <v>46199</v>
       </c>
     </row>
     <row r="42" spans="1:22">
@@ -3110,9 +3084,6 @@
       <c r="O42" t="s">
         <v>128</v>
       </c>
-      <c r="P42">
-        <v>46260</v>
-      </c>
       <c r="Q42" t="s">
         <v>166</v>
       </c>
@@ -3120,16 +3091,16 @@
         <v>168</v>
       </c>
       <c r="S42" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T42" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="U42" t="s">
-        <v>176</v>
-      </c>
-      <c r="V42" s="2">
-        <v>46352</v>
+        <v>29</v>
+      </c>
+      <c r="V42" s="1">
+        <v>46260</v>
       </c>
     </row>
     <row r="43" spans="1:22">
@@ -3154,7 +3125,7 @@
       <c r="G43" t="s">
         <v>42</v>
       </c>
-      <c r="H43" s="2">
+      <c r="H43" s="1">
         <v>46191</v>
       </c>
       <c r="I43" t="s">
@@ -3167,7 +3138,7 @@
         <v>129</v>
       </c>
       <c r="P43">
-        <v>46199</v>
+        <v>400000</v>
       </c>
       <c r="Q43" t="s">
         <v>166</v>
@@ -3176,16 +3147,16 @@
         <v>168</v>
       </c>
       <c r="S43" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T43" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="U43" t="s">
-        <v>176</v>
-      </c>
-      <c r="V43" s="2">
-        <v>46229</v>
+        <v>29</v>
+      </c>
+      <c r="V43" s="1">
+        <v>46199</v>
       </c>
     </row>
     <row r="44" spans="1:22">
@@ -3210,7 +3181,7 @@
       <c r="G44" t="s">
         <v>42</v>
       </c>
-      <c r="H44" s="2">
+      <c r="H44" s="1">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
@@ -3223,7 +3194,7 @@
         <v>130</v>
       </c>
       <c r="P44">
-        <v>46199</v>
+        <v>400000</v>
       </c>
       <c r="Q44" t="s">
         <v>166</v>
@@ -3232,16 +3203,16 @@
         <v>168</v>
       </c>
       <c r="S44" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T44" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="U44" t="s">
-        <v>176</v>
-      </c>
-      <c r="V44" s="2">
-        <v>46229</v>
+        <v>29</v>
+      </c>
+      <c r="V44" s="1">
+        <v>46199</v>
       </c>
     </row>
     <row r="45" spans="1:22">
@@ -3266,7 +3237,7 @@
       <c r="G45" t="s">
         <v>42</v>
       </c>
-      <c r="H45" s="2">
+      <c r="H45" s="1">
         <v>46213</v>
       </c>
       <c r="I45" t="s">
@@ -3282,25 +3253,25 @@
         <v>131</v>
       </c>
       <c r="P45">
-        <v>46229</v>
+        <v>173846.38</v>
       </c>
       <c r="Q45" t="s">
         <v>166</v>
       </c>
       <c r="R45" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="S45" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T45" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U45" t="s">
-        <v>177</v>
-      </c>
-      <c r="V45" s="2">
-        <v>46291</v>
+        <v>178</v>
+      </c>
+      <c r="V45" s="1">
+        <v>46229</v>
       </c>
     </row>
     <row r="46" spans="1:22">
@@ -3325,7 +3296,7 @@
       <c r="G46" t="s">
         <v>42</v>
       </c>
-      <c r="H46" s="2">
+      <c r="H46" s="1">
         <v>46210</v>
       </c>
       <c r="I46" t="s">
@@ -3338,25 +3309,25 @@
         <v>131</v>
       </c>
       <c r="P46">
-        <v>46229</v>
+        <v>1530656.62</v>
       </c>
       <c r="Q46" t="s">
         <v>166</v>
       </c>
       <c r="R46" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="S46" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T46" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U46" t="s">
-        <v>177</v>
-      </c>
-      <c r="V46" s="2">
-        <v>46291</v>
+        <v>178</v>
+      </c>
+      <c r="V46" s="1">
+        <v>46229</v>
       </c>
     </row>
     <row r="47" spans="1:22">
@@ -3385,7 +3356,7 @@
         <v>132</v>
       </c>
       <c r="P47">
-        <v>46321</v>
+        <v>1000000</v>
       </c>
       <c r="Q47" t="s">
         <v>166</v>
@@ -3394,15 +3365,15 @@
         <v>168</v>
       </c>
       <c r="S47" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T47" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="U47" t="s">
-        <v>176</v>
-      </c>
-      <c r="V47" s="2">
+        <v>29</v>
+      </c>
+      <c r="V47" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3432,25 +3403,25 @@
         <v>133</v>
       </c>
       <c r="P48">
-        <v>46291</v>
+        <v>958040</v>
       </c>
       <c r="Q48" t="s">
         <v>164</v>
       </c>
       <c r="R48" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S48" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T48" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="U48" t="s">
-        <v>175</v>
-      </c>
-      <c r="V48" s="2">
-        <v>46352</v>
+        <v>178</v>
+      </c>
+      <c r="V48" s="1">
+        <v>46291</v>
       </c>
     </row>
     <row r="49" spans="1:22">
@@ -3475,7 +3446,7 @@
       <c r="G49" t="s">
         <v>42</v>
       </c>
-      <c r="H49" s="2">
+      <c r="H49" s="1">
         <v>46176</v>
       </c>
       <c r="I49" t="s">
@@ -3491,25 +3462,25 @@
         <v>133</v>
       </c>
       <c r="P49">
-        <v>46199</v>
+        <v>41730.64</v>
       </c>
       <c r="Q49" t="s">
         <v>164</v>
       </c>
       <c r="R49" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="S49" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T49" t="s">
         <v>174</v>
       </c>
       <c r="U49" t="s">
-        <v>175</v>
-      </c>
-      <c r="V49" s="2">
-        <v>46352</v>
+        <v>178</v>
+      </c>
+      <c r="V49" s="1">
+        <v>46199</v>
       </c>
     </row>
     <row r="50" spans="1:22">
@@ -3544,25 +3515,25 @@
         <v>134</v>
       </c>
       <c r="P50">
-        <v>46260</v>
+        <v>1468159.32</v>
       </c>
       <c r="Q50" t="s">
         <v>166</v>
       </c>
       <c r="R50" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="S50" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T50" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U50" t="s">
-        <v>177</v>
-      </c>
-      <c r="V50" s="2">
-        <v>46321</v>
+        <v>178</v>
+      </c>
+      <c r="V50" s="1">
+        <v>46260</v>
       </c>
     </row>
     <row r="51" spans="1:22">
@@ -3597,25 +3568,25 @@
         <v>135</v>
       </c>
       <c r="P51">
-        <v>46291</v>
+        <v>1704503</v>
       </c>
       <c r="Q51" t="s">
         <v>166</v>
       </c>
       <c r="R51" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="S51" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T51" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U51" t="s">
-        <v>177</v>
-      </c>
-      <c r="V51" s="2">
-        <v>46352</v>
+        <v>178</v>
+      </c>
+      <c r="V51" s="1">
+        <v>46291</v>
       </c>
     </row>
     <row r="52" spans="1:22">
@@ -3647,25 +3618,25 @@
         <v>136</v>
       </c>
       <c r="P52">
-        <v>46321</v>
+        <v>1704503</v>
       </c>
       <c r="Q52" t="s">
         <v>166</v>
       </c>
       <c r="R52" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="S52" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T52" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U52" t="s">
-        <v>177</v>
-      </c>
-      <c r="V52" s="2">
-        <v>46382</v>
+        <v>178</v>
+      </c>
+      <c r="V52" s="1">
+        <v>46321</v>
       </c>
     </row>
     <row r="53" spans="1:22">
@@ -3690,7 +3661,7 @@
       <c r="G53" t="s">
         <v>42</v>
       </c>
-      <c r="H53" s="2">
+      <c r="H53" s="1">
         <v>46227</v>
       </c>
       <c r="I53" t="s">
@@ -3703,25 +3674,25 @@
         <v>134</v>
       </c>
       <c r="P53">
-        <v>46229</v>
+        <v>236343.68</v>
       </c>
       <c r="Q53" t="s">
         <v>166</v>
       </c>
       <c r="R53" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="S53" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T53" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U53" t="s">
-        <v>177</v>
-      </c>
-      <c r="V53" s="2">
-        <v>46321</v>
+        <v>178</v>
+      </c>
+      <c r="V53" s="1">
+        <v>46229</v>
       </c>
     </row>
     <row r="54" spans="1:22">
@@ -3753,25 +3724,25 @@
         <v>137</v>
       </c>
       <c r="P54">
-        <v>46352</v>
+        <v>1295422.28</v>
       </c>
       <c r="Q54" t="s">
         <v>166</v>
       </c>
       <c r="R54" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="S54" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T54" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U54" t="s">
-        <v>177</v>
-      </c>
-      <c r="V54" s="2">
-        <v>46049</v>
+        <v>178</v>
+      </c>
+      <c r="V54" s="1">
+        <v>46352</v>
       </c>
     </row>
     <row r="55" spans="1:22">
@@ -3803,25 +3774,25 @@
         <v>138</v>
       </c>
       <c r="P55">
-        <v>46321</v>
+        <v>500000</v>
       </c>
       <c r="Q55" t="s">
         <v>166</v>
       </c>
       <c r="R55" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="S55" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T55" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="U55" t="s">
         <v>178</v>
       </c>
-      <c r="V55" s="2">
-        <v>46049</v>
+      <c r="V55" s="1">
+        <v>46321</v>
       </c>
     </row>
     <row r="56" spans="1:22">
@@ -3853,25 +3824,25 @@
         <v>138</v>
       </c>
       <c r="P56">
-        <v>46321</v>
+        <v>5000000</v>
       </c>
       <c r="Q56" t="s">
         <v>166</v>
       </c>
       <c r="R56" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="S56" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T56" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="U56" t="s">
         <v>178</v>
       </c>
-      <c r="V56" s="2">
-        <v>46049</v>
+      <c r="V56" s="1">
+        <v>46321</v>
       </c>
     </row>
     <row r="57" spans="1:22">
@@ -3899,26 +3870,23 @@
       <c r="O57" t="s">
         <v>139</v>
       </c>
-      <c r="P57">
-        <v>46049</v>
-      </c>
       <c r="Q57" t="s">
         <v>166</v>
       </c>
       <c r="R57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="S57" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T57" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="U57" t="s">
         <v>178</v>
       </c>
-      <c r="V57" s="2">
-        <v>46139</v>
+      <c r="V57" s="1">
+        <v>46049</v>
       </c>
     </row>
     <row r="58" spans="1:22">
@@ -3950,13 +3918,13 @@
         <v>166</v>
       </c>
       <c r="R58" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="S58" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T58" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="U58" t="s">
         <v>178</v>
@@ -3991,13 +3959,13 @@
         <v>166</v>
       </c>
       <c r="R59" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="S59" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T59" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="U59" t="s">
         <v>178</v>
@@ -4026,25 +3994,25 @@
         <v>142</v>
       </c>
       <c r="P60">
-        <v>46107</v>
+        <v>9389.959999999999</v>
       </c>
       <c r="Q60" t="s">
         <v>164</v>
       </c>
       <c r="R60" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="S60" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T60" t="s">
         <v>174</v>
       </c>
       <c r="U60" t="s">
-        <v>175</v>
-      </c>
-      <c r="V60" s="2">
-        <v>46168</v>
+        <v>178</v>
+      </c>
+      <c r="V60" s="1">
+        <v>46107</v>
       </c>
     </row>
     <row r="61" spans="1:22">
@@ -4070,25 +4038,25 @@
         <v>143</v>
       </c>
       <c r="P61">
-        <v>46107</v>
+        <v>7204.82</v>
       </c>
       <c r="Q61" t="s">
         <v>164</v>
       </c>
       <c r="R61" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="S61" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T61" t="s">
         <v>174</v>
       </c>
       <c r="U61" t="s">
-        <v>175</v>
-      </c>
-      <c r="V61" s="2">
-        <v>46168</v>
+        <v>178</v>
+      </c>
+      <c r="V61" s="1">
+        <v>46107</v>
       </c>
     </row>
     <row r="62" spans="1:22">
@@ -4114,25 +4082,25 @@
         <v>144</v>
       </c>
       <c r="P62">
-        <v>46107</v>
+        <v>4227.84</v>
       </c>
       <c r="Q62" t="s">
         <v>164</v>
       </c>
       <c r="R62" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="S62" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T62" t="s">
         <v>174</v>
       </c>
       <c r="U62" t="s">
-        <v>175</v>
-      </c>
-      <c r="V62" s="2">
-        <v>46168</v>
+        <v>178</v>
+      </c>
+      <c r="V62" s="1">
+        <v>46107</v>
       </c>
     </row>
     <row r="63" spans="1:22">
@@ -4158,25 +4126,25 @@
         <v>145</v>
       </c>
       <c r="P63">
-        <v>46107</v>
+        <v>4064.54</v>
       </c>
       <c r="Q63" t="s">
         <v>166</v>
       </c>
       <c r="R63" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="S63" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T63" t="s">
         <v>174</v>
       </c>
       <c r="U63" t="s">
-        <v>175</v>
-      </c>
-      <c r="V63" s="2">
-        <v>46168</v>
+        <v>178</v>
+      </c>
+      <c r="V63" s="1">
+        <v>46107</v>
       </c>
     </row>
     <row r="64" spans="1:22">
@@ -4202,25 +4170,25 @@
         <v>144</v>
       </c>
       <c r="P64">
-        <v>46107</v>
+        <v>3662.66</v>
       </c>
       <c r="Q64" t="s">
         <v>164</v>
       </c>
       <c r="R64" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="S64" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T64" t="s">
         <v>174</v>
       </c>
       <c r="U64" t="s">
-        <v>175</v>
-      </c>
-      <c r="V64" s="2">
-        <v>46168</v>
+        <v>178</v>
+      </c>
+      <c r="V64" s="1">
+        <v>46107</v>
       </c>
     </row>
     <row r="65" spans="1:22">
@@ -4246,25 +4214,25 @@
         <v>146</v>
       </c>
       <c r="P65">
-        <v>46107</v>
+        <v>1163.64</v>
       </c>
       <c r="Q65" t="s">
         <v>165</v>
       </c>
       <c r="R65" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="S65" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T65" t="s">
         <v>174</v>
       </c>
       <c r="U65" t="s">
-        <v>175</v>
-      </c>
-      <c r="V65" s="2">
-        <v>46168</v>
+        <v>178</v>
+      </c>
+      <c r="V65" s="1">
+        <v>46107</v>
       </c>
     </row>
     <row r="66" spans="1:22">
@@ -4290,7 +4258,7 @@
         <v>147</v>
       </c>
       <c r="P66">
-        <v>46168</v>
+        <v>120000</v>
       </c>
       <c r="Q66" t="s">
         <v>164</v>
@@ -4299,15 +4267,15 @@
         <v>167</v>
       </c>
       <c r="S66" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T66" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="U66" t="s">
-        <v>175</v>
-      </c>
-      <c r="V66" s="2">
+        <v>29</v>
+      </c>
+      <c r="V66" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4337,25 +4305,25 @@
         <v>148</v>
       </c>
       <c r="P67">
-        <v>46291</v>
+        <v>400000</v>
       </c>
       <c r="Q67" t="s">
         <v>165</v>
       </c>
       <c r="R67" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S67" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T67" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="U67" t="s">
-        <v>175</v>
-      </c>
-      <c r="V67" s="2">
-        <v>46382</v>
+        <v>29</v>
+      </c>
+      <c r="V67" s="1">
+        <v>46291</v>
       </c>
     </row>
     <row r="68" spans="1:22">
@@ -4384,25 +4352,25 @@
         <v>149</v>
       </c>
       <c r="P68">
-        <v>46229</v>
+        <v>100000</v>
       </c>
       <c r="Q68" t="s">
         <v>165</v>
       </c>
       <c r="R68" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S68" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T68" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="U68" t="s">
-        <v>175</v>
-      </c>
-      <c r="V68" s="2">
-        <v>46291</v>
+        <v>178</v>
+      </c>
+      <c r="V68" s="1">
+        <v>46229</v>
       </c>
     </row>
     <row r="69" spans="1:22">
@@ -4428,7 +4396,7 @@
         <v>150</v>
       </c>
       <c r="P69">
-        <v>46260</v>
+        <v>80000</v>
       </c>
       <c r="Q69" t="s">
         <v>164</v>
@@ -4437,15 +4405,15 @@
         <v>167</v>
       </c>
       <c r="S69" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T69" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="U69" t="s">
-        <v>175</v>
-      </c>
-      <c r="V69" s="2">
+        <v>29</v>
+      </c>
+      <c r="V69" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -4472,25 +4440,25 @@
         <v>151</v>
       </c>
       <c r="P70">
-        <v>46291</v>
+        <v>835000</v>
       </c>
       <c r="Q70" t="s">
         <v>164</v>
       </c>
       <c r="R70" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S70" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T70" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="U70" t="s">
-        <v>175</v>
-      </c>
-      <c r="V70" s="2">
-        <v>46352</v>
+        <v>178</v>
+      </c>
+      <c r="V70" s="1">
+        <v>46291</v>
       </c>
     </row>
     <row r="71" spans="1:22">
@@ -4516,25 +4484,25 @@
         <v>151</v>
       </c>
       <c r="P71">
-        <v>46168</v>
+        <v>165000</v>
       </c>
       <c r="Q71" t="s">
         <v>164</v>
       </c>
       <c r="R71" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S71" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T71" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="U71" t="s">
-        <v>175</v>
-      </c>
-      <c r="V71" s="2">
-        <v>46229</v>
+        <v>178</v>
+      </c>
+      <c r="V71" s="1">
+        <v>46168</v>
       </c>
     </row>
     <row r="72" spans="1:22">
@@ -4560,25 +4528,25 @@
         <v>152</v>
       </c>
       <c r="P72">
-        <v>46291</v>
+        <v>1000000</v>
       </c>
       <c r="Q72" t="s">
         <v>164</v>
       </c>
       <c r="R72" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S72" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T72" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="U72" t="s">
-        <v>175</v>
-      </c>
-      <c r="V72" s="2">
-        <v>46352</v>
+        <v>178</v>
+      </c>
+      <c r="V72" s="1">
+        <v>46291</v>
       </c>
     </row>
     <row r="73" spans="1:22">
@@ -4604,25 +4572,25 @@
         <v>153</v>
       </c>
       <c r="P73">
-        <v>46291</v>
+        <v>1000000</v>
       </c>
       <c r="Q73" t="s">
         <v>164</v>
       </c>
       <c r="R73" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S73" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T73" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="U73" t="s">
-        <v>175</v>
-      </c>
-      <c r="V73" s="2">
-        <v>46352</v>
+        <v>178</v>
+      </c>
+      <c r="V73" s="1">
+        <v>46291</v>
       </c>
     </row>
     <row r="74" spans="1:22">
@@ -4648,25 +4616,25 @@
         <v>154</v>
       </c>
       <c r="P74">
-        <v>46291</v>
+        <v>100000</v>
       </c>
       <c r="Q74" t="s">
         <v>165</v>
       </c>
       <c r="R74" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S74" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T74" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="U74" t="s">
-        <v>175</v>
-      </c>
-      <c r="V74" s="2">
-        <v>46352</v>
+        <v>178</v>
+      </c>
+      <c r="V74" s="1">
+        <v>46291</v>
       </c>
     </row>
     <row r="75" spans="1:22">
@@ -4695,7 +4663,7 @@
         <v>155</v>
       </c>
       <c r="P75">
-        <v>46321</v>
+        <v>1000000</v>
       </c>
       <c r="Q75" t="s">
         <v>166</v>
@@ -4704,16 +4672,16 @@
         <v>168</v>
       </c>
       <c r="S75" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T75" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="U75" t="s">
-        <v>176</v>
-      </c>
-      <c r="V75" s="2">
-        <v>46382</v>
+        <v>29</v>
+      </c>
+      <c r="V75" s="1">
+        <v>46321</v>
       </c>
     </row>
     <row r="76" spans="1:22">
@@ -4745,25 +4713,25 @@
         <v>156</v>
       </c>
       <c r="P76">
-        <v>46381</v>
+        <v>1704503</v>
       </c>
       <c r="Q76" t="s">
         <v>166</v>
       </c>
       <c r="R76" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="S76" t="s">
         <v>41</v>
       </c>
       <c r="T76" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U76" t="s">
-        <v>177</v>
-      </c>
-      <c r="V76" s="2">
-        <v>46107</v>
+        <v>178</v>
+      </c>
+      <c r="V76" s="1">
+        <v>46381</v>
       </c>
     </row>
     <row r="77" spans="1:22">
@@ -4795,25 +4763,25 @@
         <v>157</v>
       </c>
       <c r="P77">
-        <v>46381</v>
+        <v>1638125.5</v>
       </c>
       <c r="Q77" t="s">
         <v>166</v>
       </c>
       <c r="R77" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="S77" t="s">
         <v>41</v>
       </c>
       <c r="T77" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U77" t="s">
-        <v>177</v>
-      </c>
-      <c r="V77" s="2">
-        <v>46138</v>
+        <v>178</v>
+      </c>
+      <c r="V77" s="1">
+        <v>46381</v>
       </c>
     </row>
     <row r="78" spans="1:22">
@@ -4845,25 +4813,25 @@
         <v>158</v>
       </c>
       <c r="P78">
-        <v>46381</v>
+        <v>3800000</v>
       </c>
       <c r="Q78" t="s">
         <v>166</v>
       </c>
       <c r="R78" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="S78" t="s">
         <v>41</v>
       </c>
       <c r="T78" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="U78" t="s">
-        <v>176</v>
-      </c>
-      <c r="V78" s="2">
-        <v>46260</v>
+        <v>29</v>
+      </c>
+      <c r="V78" s="1">
+        <v>46381</v>
       </c>
     </row>
     <row r="79" spans="1:22">
@@ -4895,25 +4863,25 @@
         <v>159</v>
       </c>
       <c r="P79">
-        <v>46381</v>
+        <v>3800000</v>
       </c>
       <c r="Q79" t="s">
         <v>166</v>
       </c>
       <c r="R79" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="S79" t="s">
         <v>41</v>
       </c>
       <c r="T79" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="U79" t="s">
-        <v>176</v>
-      </c>
-      <c r="V79" s="2">
-        <v>46260</v>
+        <v>29</v>
+      </c>
+      <c r="V79" s="1">
+        <v>46381</v>
       </c>
     </row>
     <row r="80" spans="1:22">
@@ -4945,25 +4913,25 @@
         <v>160</v>
       </c>
       <c r="P80">
-        <v>46382</v>
+        <v>3800000</v>
       </c>
       <c r="Q80" t="s">
         <v>166</v>
       </c>
       <c r="R80" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="S80" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T80" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="U80" t="s">
-        <v>176</v>
-      </c>
-      <c r="V80" s="2">
-        <v>46108</v>
+        <v>29</v>
+      </c>
+      <c r="V80" s="1">
+        <v>46382</v>
       </c>
     </row>
     <row r="81" spans="1:22">
@@ -4989,25 +4957,25 @@
         <v>95</v>
       </c>
       <c r="P81">
-        <v>46382</v>
+        <v>4394700</v>
       </c>
       <c r="Q81" t="s">
         <v>164</v>
       </c>
       <c r="R81" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S81" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T81" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="U81" t="s">
-        <v>176</v>
-      </c>
-      <c r="V81" s="2">
-        <v>46108</v>
+        <v>29</v>
+      </c>
+      <c r="V81" s="1">
+        <v>46382</v>
       </c>
     </row>
     <row r="82" spans="1:22">
@@ -5039,25 +5007,25 @@
         <v>161</v>
       </c>
       <c r="P82">
-        <v>46382</v>
+        <v>528395.9300000001</v>
       </c>
       <c r="Q82" t="s">
         <v>166</v>
       </c>
       <c r="R82" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="S82" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T82" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U82" t="s">
-        <v>177</v>
-      </c>
-      <c r="V82" s="2">
-        <v>46080</v>
+        <v>178</v>
+      </c>
+      <c r="V82" s="1">
+        <v>46382</v>
       </c>
     </row>
     <row r="83" spans="1:22">
@@ -5083,7 +5051,7 @@
         <v>162</v>
       </c>
       <c r="P83">
-        <v>46321</v>
+        <v>1000000</v>
       </c>
       <c r="Q83" t="s">
         <v>166</v>
@@ -5092,16 +5060,16 @@
         <v>168</v>
       </c>
       <c r="S83" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T83" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="U83" t="s">
-        <v>176</v>
-      </c>
-      <c r="V83" s="2">
-        <v>46382</v>
+        <v>29</v>
+      </c>
+      <c r="V83" s="1">
+        <v>46321</v>
       </c>
     </row>
     <row r="84" spans="1:22">
@@ -5127,25 +5095,25 @@
         <v>95</v>
       </c>
       <c r="P84">
-        <v>46382</v>
+        <v>4394700</v>
       </c>
       <c r="Q84" t="s">
         <v>164</v>
       </c>
       <c r="R84" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S84" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T84" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="U84" t="s">
-        <v>176</v>
-      </c>
-      <c r="V84" s="2">
-        <v>46108</v>
+        <v>29</v>
+      </c>
+      <c r="V84" s="1">
+        <v>46382</v>
       </c>
     </row>
     <row r="85" spans="1:22">
@@ -5176,20 +5144,23 @@
       <c r="O85" t="s">
         <v>95</v>
       </c>
+      <c r="P85">
+        <v>3306000</v>
+      </c>
       <c r="Q85" t="s">
         <v>164</v>
       </c>
       <c r="R85" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S85" t="s">
         <v>41</v>
       </c>
       <c r="T85" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="U85" t="s">
-        <v>176</v>
+        <v>29</v>
       </c>
     </row>
     <row r="86" spans="1:22">
@@ -5220,20 +5191,23 @@
       <c r="O86" t="s">
         <v>95</v>
       </c>
+      <c r="P86">
+        <v>3306000</v>
+      </c>
       <c r="Q86" t="s">
         <v>164</v>
       </c>
       <c r="R86" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S86" t="s">
         <v>41</v>
       </c>
       <c r="T86" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="U86" t="s">
-        <v>176</v>
+        <v>29</v>
       </c>
     </row>
     <row r="87" spans="1:22">
@@ -5262,25 +5236,25 @@
         <v>163</v>
       </c>
       <c r="P87">
-        <v>46260</v>
+        <v>212577</v>
       </c>
       <c r="Q87" t="s">
         <v>166</v>
       </c>
       <c r="R87" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="S87" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="T87" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="U87" t="s">
-        <v>178</v>
-      </c>
-      <c r="V87" s="2">
-        <v>46382</v>
+        <v>30</v>
+      </c>
+      <c r="V87" s="1">
+        <v>46260</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: mta (25/08/2026 08:31)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -560,8 +560,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -577,7 +585,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -585,12 +593,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -890,70 +916,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1003,7 +1029,7 @@
       <c r="U2" t="s">
         <v>178</v>
       </c>
-      <c r="V2" s="1">
+      <c r="V2" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -1050,7 +1076,7 @@
       <c r="U3" t="s">
         <v>29</v>
       </c>
-      <c r="V3" s="1">
+      <c r="V3" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1097,7 +1123,7 @@
       <c r="U4" t="s">
         <v>29</v>
       </c>
-      <c r="V4" s="1">
+      <c r="V4" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1144,7 +1170,7 @@
       <c r="U5" t="s">
         <v>29</v>
       </c>
-      <c r="V5" s="1">
+      <c r="V5" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1194,7 +1220,7 @@
       <c r="U6" t="s">
         <v>29</v>
       </c>
-      <c r="V6" s="1">
+      <c r="V6" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1220,7 +1246,7 @@
       <c r="G7" t="s">
         <v>42</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1250,7 +1276,7 @@
       <c r="U7" t="s">
         <v>29</v>
       </c>
-      <c r="V7" s="1">
+      <c r="V7" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -1297,7 +1323,7 @@
       <c r="U8" t="s">
         <v>29</v>
       </c>
-      <c r="V8" s="1">
+      <c r="V8" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1344,7 +1370,7 @@
       <c r="U9" t="s">
         <v>29</v>
       </c>
-      <c r="V9" s="1">
+      <c r="V9" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1391,7 +1417,7 @@
       <c r="U10" t="s">
         <v>29</v>
       </c>
-      <c r="V10" s="1">
+      <c r="V10" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1438,7 +1464,7 @@
       <c r="U11" t="s">
         <v>29</v>
       </c>
-      <c r="V11" s="1">
+      <c r="V11" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1464,7 +1490,7 @@
       <c r="G12" t="s">
         <v>42</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46079</v>
       </c>
       <c r="I12" t="s">
@@ -1497,7 +1523,7 @@
       <c r="U12" t="s">
         <v>178</v>
       </c>
-      <c r="V12" s="1">
+      <c r="V12" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1544,7 +1570,7 @@
       <c r="U13" t="s">
         <v>178</v>
       </c>
-      <c r="V13" s="1">
+      <c r="V13" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1591,7 +1617,7 @@
       <c r="U14" t="s">
         <v>178</v>
       </c>
-      <c r="V14" s="1">
+      <c r="V14" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1638,7 +1664,7 @@
       <c r="U15" t="s">
         <v>178</v>
       </c>
-      <c r="V15" s="1">
+      <c r="V15" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1685,7 +1711,7 @@
       <c r="U16" t="s">
         <v>178</v>
       </c>
-      <c r="V16" s="1">
+      <c r="V16" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -1711,7 +1737,7 @@
       <c r="G17" t="s">
         <v>42</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46098</v>
       </c>
       <c r="I17" t="s">
@@ -1744,7 +1770,7 @@
       <c r="U17" t="s">
         <v>178</v>
       </c>
-      <c r="V17" s="1">
+      <c r="V17" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -1770,7 +1796,7 @@
       <c r="G18" t="s">
         <v>42</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46076</v>
       </c>
       <c r="I18" t="s">
@@ -1800,7 +1826,7 @@
       <c r="U18" t="s">
         <v>29</v>
       </c>
-      <c r="V18" s="1">
+      <c r="V18" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1826,7 +1852,7 @@
       <c r="G19" t="s">
         <v>42</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1856,7 +1882,7 @@
       <c r="U19" t="s">
         <v>29</v>
       </c>
-      <c r="V19" s="1">
+      <c r="V19" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1903,7 +1929,7 @@
       <c r="U20" t="s">
         <v>29</v>
       </c>
-      <c r="V20" s="1">
+      <c r="V20" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1950,7 +1976,7 @@
       <c r="U21" t="s">
         <v>29</v>
       </c>
-      <c r="V21" s="1">
+      <c r="V21" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1997,7 +2023,7 @@
       <c r="U22" t="s">
         <v>29</v>
       </c>
-      <c r="V22" s="1">
+      <c r="V22" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2044,7 +2070,7 @@
       <c r="U23" t="s">
         <v>29</v>
       </c>
-      <c r="V23" s="1">
+      <c r="V23" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2070,7 +2096,7 @@
       <c r="G24" t="s">
         <v>42</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>46119</v>
       </c>
       <c r="I24" t="s">
@@ -2103,7 +2129,7 @@
       <c r="U24" t="s">
         <v>178</v>
       </c>
-      <c r="V24" s="1">
+      <c r="V24" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2129,7 +2155,7 @@
       <c r="G25" t="s">
         <v>42</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>46121</v>
       </c>
       <c r="I25" t="s">
@@ -2159,7 +2185,7 @@
       <c r="U25" t="s">
         <v>29</v>
       </c>
-      <c r="V25" s="1">
+      <c r="V25" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2185,7 +2211,7 @@
       <c r="G26" t="s">
         <v>42</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>46076</v>
       </c>
       <c r="I26" t="s">
@@ -2215,7 +2241,7 @@
       <c r="U26" t="s">
         <v>29</v>
       </c>
-      <c r="V26" s="1">
+      <c r="V26" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -2262,7 +2288,7 @@
       <c r="U27" t="s">
         <v>178</v>
       </c>
-      <c r="V27" s="1">
+      <c r="V27" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -2288,7 +2314,7 @@
       <c r="G28" t="s">
         <v>42</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>46199</v>
       </c>
       <c r="I28" t="s">
@@ -2321,7 +2347,7 @@
       <c r="U28" t="s">
         <v>178</v>
       </c>
-      <c r="V28" s="1">
+      <c r="V28" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2347,7 +2373,7 @@
       <c r="G29" t="s">
         <v>42</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2380,7 +2406,7 @@
       <c r="U29" t="s">
         <v>178</v>
       </c>
-      <c r="V29" s="1">
+      <c r="V29" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2406,7 +2432,7 @@
       <c r="G30" t="s">
         <v>42</v>
       </c>
-      <c r="H30" s="1">
+      <c r="H30" s="2">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2439,7 +2465,7 @@
       <c r="U30" t="s">
         <v>178</v>
       </c>
-      <c r="V30" s="1">
+      <c r="V30" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2465,7 +2491,7 @@
       <c r="G31" t="s">
         <v>42</v>
       </c>
-      <c r="H31" s="1">
+      <c r="H31" s="2">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2498,7 +2524,7 @@
       <c r="U31" t="s">
         <v>178</v>
       </c>
-      <c r="V31" s="1">
+      <c r="V31" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2548,7 +2574,7 @@
       <c r="U32" t="s">
         <v>178</v>
       </c>
-      <c r="V32" s="1">
+      <c r="V32" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -2574,7 +2600,7 @@
       <c r="G33" t="s">
         <v>42</v>
       </c>
-      <c r="H33" s="1">
+      <c r="H33" s="2">
         <v>46191</v>
       </c>
       <c r="I33" t="s">
@@ -2607,7 +2633,7 @@
       <c r="U33" t="s">
         <v>178</v>
       </c>
-      <c r="V33" s="1">
+      <c r="V33" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2633,7 +2659,7 @@
       <c r="G34" t="s">
         <v>42</v>
       </c>
-      <c r="H34" s="1">
+      <c r="H34" s="2">
         <v>46119</v>
       </c>
       <c r="I34" t="s">
@@ -2663,7 +2689,7 @@
       <c r="U34" t="s">
         <v>178</v>
       </c>
-      <c r="V34" s="1">
+      <c r="V34" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2689,7 +2715,7 @@
       <c r="G35" t="s">
         <v>42</v>
       </c>
-      <c r="H35" s="1">
+      <c r="H35" s="2">
         <v>46213</v>
       </c>
       <c r="I35" t="s">
@@ -2719,7 +2745,7 @@
       <c r="U35" t="s">
         <v>29</v>
       </c>
-      <c r="V35" s="1">
+      <c r="V35" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -2745,7 +2771,7 @@
       <c r="G36" t="s">
         <v>42</v>
       </c>
-      <c r="H36" s="1">
+      <c r="H36" s="2">
         <v>46175</v>
       </c>
       <c r="I36" t="s">
@@ -2775,7 +2801,7 @@
       <c r="U36" t="s">
         <v>29</v>
       </c>
-      <c r="V36" s="1">
+      <c r="V36" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2801,7 +2827,7 @@
       <c r="G37" t="s">
         <v>42</v>
       </c>
-      <c r="H37" s="1">
+      <c r="H37" s="2">
         <v>46213</v>
       </c>
       <c r="I37" t="s">
@@ -2831,7 +2857,7 @@
       <c r="U37" t="s">
         <v>29</v>
       </c>
-      <c r="V37" s="1">
+      <c r="V37" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -2857,7 +2883,7 @@
       <c r="G38" t="s">
         <v>42</v>
       </c>
-      <c r="H38" s="1">
+      <c r="H38" s="2">
         <v>46199</v>
       </c>
       <c r="I38" t="s">
@@ -2887,7 +2913,7 @@
       <c r="U38" t="s">
         <v>29</v>
       </c>
-      <c r="V38" s="1">
+      <c r="V38" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2913,7 +2939,7 @@
       <c r="G39" t="s">
         <v>42</v>
       </c>
-      <c r="H39" s="1">
+      <c r="H39" s="2">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -2943,7 +2969,7 @@
       <c r="U39" t="s">
         <v>29</v>
       </c>
-      <c r="V39" s="1">
+      <c r="V39" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2969,7 +2995,7 @@
       <c r="G40" t="s">
         <v>42</v>
       </c>
-      <c r="H40" s="1">
+      <c r="H40" s="2">
         <v>46204</v>
       </c>
       <c r="I40" t="s">
@@ -2999,7 +3025,7 @@
       <c r="U40" t="s">
         <v>29</v>
       </c>
-      <c r="V40" s="1">
+      <c r="V40" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3025,7 +3051,7 @@
       <c r="G41" t="s">
         <v>42</v>
       </c>
-      <c r="H41" s="1">
+      <c r="H41" s="2">
         <v>46244</v>
       </c>
       <c r="I41" t="s">
@@ -3055,7 +3081,7 @@
       <c r="U41" t="s">
         <v>29</v>
       </c>
-      <c r="V41" s="1">
+      <c r="V41" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3099,7 +3125,7 @@
       <c r="U42" t="s">
         <v>29</v>
       </c>
-      <c r="V42" s="1">
+      <c r="V42" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3125,7 +3151,7 @@
       <c r="G43" t="s">
         <v>42</v>
       </c>
-      <c r="H43" s="1">
+      <c r="H43" s="2">
         <v>46191</v>
       </c>
       <c r="I43" t="s">
@@ -3155,7 +3181,7 @@
       <c r="U43" t="s">
         <v>29</v>
       </c>
-      <c r="V43" s="1">
+      <c r="V43" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3181,7 +3207,7 @@
       <c r="G44" t="s">
         <v>42</v>
       </c>
-      <c r="H44" s="1">
+      <c r="H44" s="2">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
@@ -3211,7 +3237,7 @@
       <c r="U44" t="s">
         <v>29</v>
       </c>
-      <c r="V44" s="1">
+      <c r="V44" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3237,7 +3263,7 @@
       <c r="G45" t="s">
         <v>42</v>
       </c>
-      <c r="H45" s="1">
+      <c r="H45" s="2">
         <v>46213</v>
       </c>
       <c r="I45" t="s">
@@ -3270,7 +3296,7 @@
       <c r="U45" t="s">
         <v>178</v>
       </c>
-      <c r="V45" s="1">
+      <c r="V45" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3296,7 +3322,7 @@
       <c r="G46" t="s">
         <v>42</v>
       </c>
-      <c r="H46" s="1">
+      <c r="H46" s="2">
         <v>46210</v>
       </c>
       <c r="I46" t="s">
@@ -3326,7 +3352,7 @@
       <c r="U46" t="s">
         <v>178</v>
       </c>
-      <c r="V46" s="1">
+      <c r="V46" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3373,7 +3399,7 @@
       <c r="U47" t="s">
         <v>29</v>
       </c>
-      <c r="V47" s="1">
+      <c r="V47" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3420,7 +3446,7 @@
       <c r="U48" t="s">
         <v>178</v>
       </c>
-      <c r="V48" s="1">
+      <c r="V48" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3446,7 +3472,7 @@
       <c r="G49" t="s">
         <v>42</v>
       </c>
-      <c r="H49" s="1">
+      <c r="H49" s="2">
         <v>46176</v>
       </c>
       <c r="I49" t="s">
@@ -3479,7 +3505,7 @@
       <c r="U49" t="s">
         <v>178</v>
       </c>
-      <c r="V49" s="1">
+      <c r="V49" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3532,7 +3558,7 @@
       <c r="U50" t="s">
         <v>178</v>
       </c>
-      <c r="V50" s="1">
+      <c r="V50" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3585,7 +3611,7 @@
       <c r="U51" t="s">
         <v>178</v>
       </c>
-      <c r="V51" s="1">
+      <c r="V51" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3635,7 +3661,7 @@
       <c r="U52" t="s">
         <v>178</v>
       </c>
-      <c r="V52" s="1">
+      <c r="V52" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3661,7 +3687,7 @@
       <c r="G53" t="s">
         <v>42</v>
       </c>
-      <c r="H53" s="1">
+      <c r="H53" s="2">
         <v>46227</v>
       </c>
       <c r="I53" t="s">
@@ -3691,7 +3717,7 @@
       <c r="U53" t="s">
         <v>178</v>
       </c>
-      <c r="V53" s="1">
+      <c r="V53" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3741,7 +3767,7 @@
       <c r="U54" t="s">
         <v>178</v>
       </c>
-      <c r="V54" s="1">
+      <c r="V54" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -3791,7 +3817,7 @@
       <c r="U55" t="s">
         <v>178</v>
       </c>
-      <c r="V55" s="1">
+      <c r="V55" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3841,7 +3867,7 @@
       <c r="U56" t="s">
         <v>178</v>
       </c>
-      <c r="V56" s="1">
+      <c r="V56" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3885,7 +3911,7 @@
       <c r="U57" t="s">
         <v>178</v>
       </c>
-      <c r="V57" s="1">
+      <c r="V57" s="2">
         <v>46049</v>
       </c>
     </row>
@@ -4011,7 +4037,7 @@
       <c r="U60" t="s">
         <v>178</v>
       </c>
-      <c r="V60" s="1">
+      <c r="V60" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4055,7 +4081,7 @@
       <c r="U61" t="s">
         <v>178</v>
       </c>
-      <c r="V61" s="1">
+      <c r="V61" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4099,7 +4125,7 @@
       <c r="U62" t="s">
         <v>178</v>
       </c>
-      <c r="V62" s="1">
+      <c r="V62" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4143,7 +4169,7 @@
       <c r="U63" t="s">
         <v>178</v>
       </c>
-      <c r="V63" s="1">
+      <c r="V63" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4187,7 +4213,7 @@
       <c r="U64" t="s">
         <v>178</v>
       </c>
-      <c r="V64" s="1">
+      <c r="V64" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4231,7 +4257,7 @@
       <c r="U65" t="s">
         <v>178</v>
       </c>
-      <c r="V65" s="1">
+      <c r="V65" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4275,7 +4301,7 @@
       <c r="U66" t="s">
         <v>29</v>
       </c>
-      <c r="V66" s="1">
+      <c r="V66" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4322,7 +4348,7 @@
       <c r="U67" t="s">
         <v>29</v>
       </c>
-      <c r="V67" s="1">
+      <c r="V67" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4369,7 +4395,7 @@
       <c r="U68" t="s">
         <v>178</v>
       </c>
-      <c r="V68" s="1">
+      <c r="V68" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -4413,7 +4439,7 @@
       <c r="U69" t="s">
         <v>29</v>
       </c>
-      <c r="V69" s="1">
+      <c r="V69" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -4457,7 +4483,7 @@
       <c r="U70" t="s">
         <v>178</v>
       </c>
-      <c r="V70" s="1">
+      <c r="V70" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4501,7 +4527,7 @@
       <c r="U71" t="s">
         <v>178</v>
       </c>
-      <c r="V71" s="1">
+      <c r="V71" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4545,7 +4571,7 @@
       <c r="U72" t="s">
         <v>178</v>
       </c>
-      <c r="V72" s="1">
+      <c r="V72" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4589,7 +4615,7 @@
       <c r="U73" t="s">
         <v>178</v>
       </c>
-      <c r="V73" s="1">
+      <c r="V73" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4633,7 +4659,7 @@
       <c r="U74" t="s">
         <v>178</v>
       </c>
-      <c r="V74" s="1">
+      <c r="V74" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4680,7 +4706,7 @@
       <c r="U75" t="s">
         <v>29</v>
       </c>
-      <c r="V75" s="1">
+      <c r="V75" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -4730,7 +4756,7 @@
       <c r="U76" t="s">
         <v>178</v>
       </c>
-      <c r="V76" s="1">
+      <c r="V76" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4780,7 +4806,7 @@
       <c r="U77" t="s">
         <v>178</v>
       </c>
-      <c r="V77" s="1">
+      <c r="V77" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4830,7 +4856,7 @@
       <c r="U78" t="s">
         <v>29</v>
       </c>
-      <c r="V78" s="1">
+      <c r="V78" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4880,7 +4906,7 @@
       <c r="U79" t="s">
         <v>29</v>
       </c>
-      <c r="V79" s="1">
+      <c r="V79" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4930,7 +4956,7 @@
       <c r="U80" t="s">
         <v>29</v>
       </c>
-      <c r="V80" s="1">
+      <c r="V80" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -4974,7 +5000,7 @@
       <c r="U81" t="s">
         <v>29</v>
       </c>
-      <c r="V81" s="1">
+      <c r="V81" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5024,7 +5050,7 @@
       <c r="U82" t="s">
         <v>178</v>
       </c>
-      <c r="V82" s="1">
+      <c r="V82" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5068,7 +5094,7 @@
       <c r="U83" t="s">
         <v>29</v>
       </c>
-      <c r="V83" s="1">
+      <c r="V83" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -5112,7 +5138,7 @@
       <c r="U84" t="s">
         <v>29</v>
       </c>
-      <c r="V84" s="1">
+      <c r="V84" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5253,7 +5279,7 @@
       <c r="U87" t="s">
         <v>30</v>
       </c>
-      <c r="V87" s="1">
+      <c r="V87" s="2">
         <v>46260</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (25/08/2026 08:36)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -560,16 +560,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -585,7 +577,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -593,30 +585,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -916,70 +890,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1029,7 +1003,7 @@
       <c r="U2" t="s">
         <v>178</v>
       </c>
-      <c r="V2" s="2">
+      <c r="V2" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1076,7 +1050,7 @@
       <c r="U3" t="s">
         <v>29</v>
       </c>
-      <c r="V3" s="2">
+      <c r="V3" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1123,7 +1097,7 @@
       <c r="U4" t="s">
         <v>29</v>
       </c>
-      <c r="V4" s="2">
+      <c r="V4" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1170,7 +1144,7 @@
       <c r="U5" t="s">
         <v>29</v>
       </c>
-      <c r="V5" s="2">
+      <c r="V5" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1220,7 +1194,7 @@
       <c r="U6" t="s">
         <v>29</v>
       </c>
-      <c r="V6" s="2">
+      <c r="V6" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1246,7 +1220,7 @@
       <c r="G7" t="s">
         <v>42</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1276,7 +1250,7 @@
       <c r="U7" t="s">
         <v>29</v>
       </c>
-      <c r="V7" s="2">
+      <c r="V7" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -1323,7 +1297,7 @@
       <c r="U8" t="s">
         <v>29</v>
       </c>
-      <c r="V8" s="2">
+      <c r="V8" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1370,7 +1344,7 @@
       <c r="U9" t="s">
         <v>29</v>
       </c>
-      <c r="V9" s="2">
+      <c r="V9" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1417,7 +1391,7 @@
       <c r="U10" t="s">
         <v>29</v>
       </c>
-      <c r="V10" s="2">
+      <c r="V10" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1464,7 +1438,7 @@
       <c r="U11" t="s">
         <v>29</v>
       </c>
-      <c r="V11" s="2">
+      <c r="V11" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1490,7 +1464,7 @@
       <c r="G12" t="s">
         <v>42</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46079</v>
       </c>
       <c r="I12" t="s">
@@ -1523,7 +1497,7 @@
       <c r="U12" t="s">
         <v>178</v>
       </c>
-      <c r="V12" s="2">
+      <c r="V12" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1570,7 +1544,7 @@
       <c r="U13" t="s">
         <v>178</v>
       </c>
-      <c r="V13" s="2">
+      <c r="V13" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1617,7 +1591,7 @@
       <c r="U14" t="s">
         <v>178</v>
       </c>
-      <c r="V14" s="2">
+      <c r="V14" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1664,7 +1638,7 @@
       <c r="U15" t="s">
         <v>178</v>
       </c>
-      <c r="V15" s="2">
+      <c r="V15" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1711,7 +1685,7 @@
       <c r="U16" t="s">
         <v>178</v>
       </c>
-      <c r="V16" s="2">
+      <c r="V16" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1737,7 +1711,7 @@
       <c r="G17" t="s">
         <v>42</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46098</v>
       </c>
       <c r="I17" t="s">
@@ -1770,7 +1744,7 @@
       <c r="U17" t="s">
         <v>178</v>
       </c>
-      <c r="V17" s="2">
+      <c r="V17" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -1796,7 +1770,7 @@
       <c r="G18" t="s">
         <v>42</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46076</v>
       </c>
       <c r="I18" t="s">
@@ -1826,7 +1800,7 @@
       <c r="U18" t="s">
         <v>29</v>
       </c>
-      <c r="V18" s="2">
+      <c r="V18" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1852,7 +1826,7 @@
       <c r="G19" t="s">
         <v>42</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1882,7 +1856,7 @@
       <c r="U19" t="s">
         <v>29</v>
       </c>
-      <c r="V19" s="2">
+      <c r="V19" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1929,7 +1903,7 @@
       <c r="U20" t="s">
         <v>29</v>
       </c>
-      <c r="V20" s="2">
+      <c r="V20" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1976,7 +1950,7 @@
       <c r="U21" t="s">
         <v>29</v>
       </c>
-      <c r="V21" s="2">
+      <c r="V21" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2023,7 +1997,7 @@
       <c r="U22" t="s">
         <v>29</v>
       </c>
-      <c r="V22" s="2">
+      <c r="V22" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2070,7 +2044,7 @@
       <c r="U23" t="s">
         <v>29</v>
       </c>
-      <c r="V23" s="2">
+      <c r="V23" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2096,7 +2070,7 @@
       <c r="G24" t="s">
         <v>42</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>46119</v>
       </c>
       <c r="I24" t="s">
@@ -2129,7 +2103,7 @@
       <c r="U24" t="s">
         <v>178</v>
       </c>
-      <c r="V24" s="2">
+      <c r="V24" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2155,7 +2129,7 @@
       <c r="G25" t="s">
         <v>42</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>46121</v>
       </c>
       <c r="I25" t="s">
@@ -2185,7 +2159,7 @@
       <c r="U25" t="s">
         <v>29</v>
       </c>
-      <c r="V25" s="2">
+      <c r="V25" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2211,7 +2185,7 @@
       <c r="G26" t="s">
         <v>42</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>46076</v>
       </c>
       <c r="I26" t="s">
@@ -2241,7 +2215,7 @@
       <c r="U26" t="s">
         <v>29</v>
       </c>
-      <c r="V26" s="2">
+      <c r="V26" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -2288,7 +2262,7 @@
       <c r="U27" t="s">
         <v>178</v>
       </c>
-      <c r="V27" s="2">
+      <c r="V27" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2314,7 +2288,7 @@
       <c r="G28" t="s">
         <v>42</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>46199</v>
       </c>
       <c r="I28" t="s">
@@ -2347,7 +2321,7 @@
       <c r="U28" t="s">
         <v>178</v>
       </c>
-      <c r="V28" s="2">
+      <c r="V28" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2373,7 +2347,7 @@
       <c r="G29" t="s">
         <v>42</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2406,7 +2380,7 @@
       <c r="U29" t="s">
         <v>178</v>
       </c>
-      <c r="V29" s="2">
+      <c r="V29" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2432,7 +2406,7 @@
       <c r="G30" t="s">
         <v>42</v>
       </c>
-      <c r="H30" s="2">
+      <c r="H30" s="1">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2465,7 +2439,7 @@
       <c r="U30" t="s">
         <v>178</v>
       </c>
-      <c r="V30" s="2">
+      <c r="V30" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2491,7 +2465,7 @@
       <c r="G31" t="s">
         <v>42</v>
       </c>
-      <c r="H31" s="2">
+      <c r="H31" s="1">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2524,7 +2498,7 @@
       <c r="U31" t="s">
         <v>178</v>
       </c>
-      <c r="V31" s="2">
+      <c r="V31" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2574,7 +2548,7 @@
       <c r="U32" t="s">
         <v>178</v>
       </c>
-      <c r="V32" s="2">
+      <c r="V32" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2600,7 +2574,7 @@
       <c r="G33" t="s">
         <v>42</v>
       </c>
-      <c r="H33" s="2">
+      <c r="H33" s="1">
         <v>46191</v>
       </c>
       <c r="I33" t="s">
@@ -2633,7 +2607,7 @@
       <c r="U33" t="s">
         <v>178</v>
       </c>
-      <c r="V33" s="2">
+      <c r="V33" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2659,7 +2633,7 @@
       <c r="G34" t="s">
         <v>42</v>
       </c>
-      <c r="H34" s="2">
+      <c r="H34" s="1">
         <v>46119</v>
       </c>
       <c r="I34" t="s">
@@ -2689,7 +2663,7 @@
       <c r="U34" t="s">
         <v>178</v>
       </c>
-      <c r="V34" s="2">
+      <c r="V34" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2715,7 +2689,7 @@
       <c r="G35" t="s">
         <v>42</v>
       </c>
-      <c r="H35" s="2">
+      <c r="H35" s="1">
         <v>46213</v>
       </c>
       <c r="I35" t="s">
@@ -2745,7 +2719,7 @@
       <c r="U35" t="s">
         <v>29</v>
       </c>
-      <c r="V35" s="2">
+      <c r="V35" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -2771,7 +2745,7 @@
       <c r="G36" t="s">
         <v>42</v>
       </c>
-      <c r="H36" s="2">
+      <c r="H36" s="1">
         <v>46175</v>
       </c>
       <c r="I36" t="s">
@@ -2801,7 +2775,7 @@
       <c r="U36" t="s">
         <v>29</v>
       </c>
-      <c r="V36" s="2">
+      <c r="V36" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2827,7 +2801,7 @@
       <c r="G37" t="s">
         <v>42</v>
       </c>
-      <c r="H37" s="2">
+      <c r="H37" s="1">
         <v>46213</v>
       </c>
       <c r="I37" t="s">
@@ -2857,7 +2831,7 @@
       <c r="U37" t="s">
         <v>29</v>
       </c>
-      <c r="V37" s="2">
+      <c r="V37" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -2883,7 +2857,7 @@
       <c r="G38" t="s">
         <v>42</v>
       </c>
-      <c r="H38" s="2">
+      <c r="H38" s="1">
         <v>46199</v>
       </c>
       <c r="I38" t="s">
@@ -2913,7 +2887,7 @@
       <c r="U38" t="s">
         <v>29</v>
       </c>
-      <c r="V38" s="2">
+      <c r="V38" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2939,7 +2913,7 @@
       <c r="G39" t="s">
         <v>42</v>
       </c>
-      <c r="H39" s="2">
+      <c r="H39" s="1">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -2969,7 +2943,7 @@
       <c r="U39" t="s">
         <v>29</v>
       </c>
-      <c r="V39" s="2">
+      <c r="V39" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2995,7 +2969,7 @@
       <c r="G40" t="s">
         <v>42</v>
       </c>
-      <c r="H40" s="2">
+      <c r="H40" s="1">
         <v>46204</v>
       </c>
       <c r="I40" t="s">
@@ -3025,7 +2999,7 @@
       <c r="U40" t="s">
         <v>29</v>
       </c>
-      <c r="V40" s="2">
+      <c r="V40" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3051,7 +3025,7 @@
       <c r="G41" t="s">
         <v>42</v>
       </c>
-      <c r="H41" s="2">
+      <c r="H41" s="1">
         <v>46244</v>
       </c>
       <c r="I41" t="s">
@@ -3081,7 +3055,7 @@
       <c r="U41" t="s">
         <v>29</v>
       </c>
-      <c r="V41" s="2">
+      <c r="V41" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3125,7 +3099,7 @@
       <c r="U42" t="s">
         <v>29</v>
       </c>
-      <c r="V42" s="2">
+      <c r="V42" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3151,7 +3125,7 @@
       <c r="G43" t="s">
         <v>42</v>
       </c>
-      <c r="H43" s="2">
+      <c r="H43" s="1">
         <v>46191</v>
       </c>
       <c r="I43" t="s">
@@ -3181,7 +3155,7 @@
       <c r="U43" t="s">
         <v>29</v>
       </c>
-      <c r="V43" s="2">
+      <c r="V43" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3207,7 +3181,7 @@
       <c r="G44" t="s">
         <v>42</v>
       </c>
-      <c r="H44" s="2">
+      <c r="H44" s="1">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
@@ -3237,7 +3211,7 @@
       <c r="U44" t="s">
         <v>29</v>
       </c>
-      <c r="V44" s="2">
+      <c r="V44" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3263,7 +3237,7 @@
       <c r="G45" t="s">
         <v>42</v>
       </c>
-      <c r="H45" s="2">
+      <c r="H45" s="1">
         <v>46213</v>
       </c>
       <c r="I45" t="s">
@@ -3296,7 +3270,7 @@
       <c r="U45" t="s">
         <v>178</v>
       </c>
-      <c r="V45" s="2">
+      <c r="V45" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3322,7 +3296,7 @@
       <c r="G46" t="s">
         <v>42</v>
       </c>
-      <c r="H46" s="2">
+      <c r="H46" s="1">
         <v>46210</v>
       </c>
       <c r="I46" t="s">
@@ -3352,7 +3326,7 @@
       <c r="U46" t="s">
         <v>178</v>
       </c>
-      <c r="V46" s="2">
+      <c r="V46" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3399,7 +3373,7 @@
       <c r="U47" t="s">
         <v>29</v>
       </c>
-      <c r="V47" s="2">
+      <c r="V47" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3446,7 +3420,7 @@
       <c r="U48" t="s">
         <v>178</v>
       </c>
-      <c r="V48" s="2">
+      <c r="V48" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3472,7 +3446,7 @@
       <c r="G49" t="s">
         <v>42</v>
       </c>
-      <c r="H49" s="2">
+      <c r="H49" s="1">
         <v>46176</v>
       </c>
       <c r="I49" t="s">
@@ -3505,7 +3479,7 @@
       <c r="U49" t="s">
         <v>178</v>
       </c>
-      <c r="V49" s="2">
+      <c r="V49" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3558,7 +3532,7 @@
       <c r="U50" t="s">
         <v>178</v>
       </c>
-      <c r="V50" s="2">
+      <c r="V50" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3611,7 +3585,7 @@
       <c r="U51" t="s">
         <v>178</v>
       </c>
-      <c r="V51" s="2">
+      <c r="V51" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3661,7 +3635,7 @@
       <c r="U52" t="s">
         <v>178</v>
       </c>
-      <c r="V52" s="2">
+      <c r="V52" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3687,7 +3661,7 @@
       <c r="G53" t="s">
         <v>42</v>
       </c>
-      <c r="H53" s="2">
+      <c r="H53" s="1">
         <v>46227</v>
       </c>
       <c r="I53" t="s">
@@ -3717,7 +3691,7 @@
       <c r="U53" t="s">
         <v>178</v>
       </c>
-      <c r="V53" s="2">
+      <c r="V53" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3767,7 +3741,7 @@
       <c r="U54" t="s">
         <v>178</v>
       </c>
-      <c r="V54" s="2">
+      <c r="V54" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -3817,7 +3791,7 @@
       <c r="U55" t="s">
         <v>178</v>
       </c>
-      <c r="V55" s="2">
+      <c r="V55" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3867,7 +3841,7 @@
       <c r="U56" t="s">
         <v>178</v>
       </c>
-      <c r="V56" s="2">
+      <c r="V56" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3911,7 +3885,7 @@
       <c r="U57" t="s">
         <v>178</v>
       </c>
-      <c r="V57" s="2">
+      <c r="V57" s="1">
         <v>46049</v>
       </c>
     </row>
@@ -4037,7 +4011,7 @@
       <c r="U60" t="s">
         <v>178</v>
       </c>
-      <c r="V60" s="2">
+      <c r="V60" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4081,7 +4055,7 @@
       <c r="U61" t="s">
         <v>178</v>
       </c>
-      <c r="V61" s="2">
+      <c r="V61" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4125,7 +4099,7 @@
       <c r="U62" t="s">
         <v>178</v>
       </c>
-      <c r="V62" s="2">
+      <c r="V62" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4169,7 +4143,7 @@
       <c r="U63" t="s">
         <v>178</v>
       </c>
-      <c r="V63" s="2">
+      <c r="V63" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4213,7 +4187,7 @@
       <c r="U64" t="s">
         <v>178</v>
       </c>
-      <c r="V64" s="2">
+      <c r="V64" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4257,7 +4231,7 @@
       <c r="U65" t="s">
         <v>178</v>
       </c>
-      <c r="V65" s="2">
+      <c r="V65" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4301,7 +4275,7 @@
       <c r="U66" t="s">
         <v>29</v>
       </c>
-      <c r="V66" s="2">
+      <c r="V66" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4348,7 +4322,7 @@
       <c r="U67" t="s">
         <v>29</v>
       </c>
-      <c r="V67" s="2">
+      <c r="V67" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4395,7 +4369,7 @@
       <c r="U68" t="s">
         <v>178</v>
       </c>
-      <c r="V68" s="2">
+      <c r="V68" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -4439,7 +4413,7 @@
       <c r="U69" t="s">
         <v>29</v>
       </c>
-      <c r="V69" s="2">
+      <c r="V69" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -4483,7 +4457,7 @@
       <c r="U70" t="s">
         <v>178</v>
       </c>
-      <c r="V70" s="2">
+      <c r="V70" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4527,7 +4501,7 @@
       <c r="U71" t="s">
         <v>178</v>
       </c>
-      <c r="V71" s="2">
+      <c r="V71" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4571,7 +4545,7 @@
       <c r="U72" t="s">
         <v>178</v>
       </c>
-      <c r="V72" s="2">
+      <c r="V72" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4615,7 +4589,7 @@
       <c r="U73" t="s">
         <v>178</v>
       </c>
-      <c r="V73" s="2">
+      <c r="V73" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4659,7 +4633,7 @@
       <c r="U74" t="s">
         <v>178</v>
       </c>
-      <c r="V74" s="2">
+      <c r="V74" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4706,7 +4680,7 @@
       <c r="U75" t="s">
         <v>29</v>
       </c>
-      <c r="V75" s="2">
+      <c r="V75" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -4756,7 +4730,7 @@
       <c r="U76" t="s">
         <v>178</v>
       </c>
-      <c r="V76" s="2">
+      <c r="V76" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4806,7 +4780,7 @@
       <c r="U77" t="s">
         <v>178</v>
       </c>
-      <c r="V77" s="2">
+      <c r="V77" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4856,7 +4830,7 @@
       <c r="U78" t="s">
         <v>29</v>
       </c>
-      <c r="V78" s="2">
+      <c r="V78" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4906,7 +4880,7 @@
       <c r="U79" t="s">
         <v>29</v>
       </c>
-      <c r="V79" s="2">
+      <c r="V79" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4956,7 +4930,7 @@
       <c r="U80" t="s">
         <v>29</v>
       </c>
-      <c r="V80" s="2">
+      <c r="V80" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5000,7 +4974,7 @@
       <c r="U81" t="s">
         <v>29</v>
       </c>
-      <c r="V81" s="2">
+      <c r="V81" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5050,7 +5024,7 @@
       <c r="U82" t="s">
         <v>178</v>
       </c>
-      <c r="V82" s="2">
+      <c r="V82" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5094,7 +5068,7 @@
       <c r="U83" t="s">
         <v>29</v>
       </c>
-      <c r="V83" s="2">
+      <c r="V83" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -5138,7 +5112,7 @@
       <c r="U84" t="s">
         <v>29</v>
       </c>
-      <c r="V84" s="2">
+      <c r="V84" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5279,7 +5253,7 @@
       <c r="U87" t="s">
         <v>30</v>
       </c>
-      <c r="V87" s="2">
+      <c r="V87" s="1">
         <v>46260</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (26/08/2026 10:59)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1121" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1110" uniqueCount="176">
   <si>
     <t>linha</t>
   </si>
@@ -88,9 +88,6 @@
     <t>MOD C-98</t>
   </si>
   <si>
-    <t>T-27</t>
-  </si>
-  <si>
     <t>Aprovado, aguardando atendimento</t>
   </si>
   <si>
@@ -304,9 +301,6 @@
     <t>Exchange PT6A-114A</t>
   </si>
   <si>
-    <t>CNT 018/CELOG-PAMASP/2026 - SERVIÇO - TOFI</t>
-  </si>
-  <si>
     <t>Atualização de GPS</t>
   </si>
   <si>
@@ -503,9 +497,6 @@
   </si>
   <si>
     <t>Material reparo PT6A-114A (4/4)</t>
-  </si>
-  <si>
-    <t>Reparo de estatores dos geradores DO C95/T/27 - TOEG</t>
   </si>
   <si>
     <t>CABW</t>
@@ -886,7 +877,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V87"/>
+  <dimension ref="A1:V86"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
@@ -968,40 +959,43 @@
         <v>22</v>
       </c>
       <c r="D2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F2" t="s">
-        <v>31</v>
+        <v>30</v>
+      </c>
+      <c r="K2" t="s">
+        <v>69</v>
       </c>
       <c r="L2" t="s">
+        <v>76</v>
+      </c>
+      <c r="N2" t="s">
         <v>77</v>
       </c>
-      <c r="N2" t="s">
-        <v>78</v>
-      </c>
       <c r="O2" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="P2">
         <v>135000</v>
       </c>
       <c r="Q2" t="s">
+        <v>161</v>
+      </c>
+      <c r="R2" t="s">
         <v>164</v>
       </c>
-      <c r="R2" t="s">
-        <v>167</v>
-      </c>
       <c r="S2" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T2" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="U2" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="V2" s="1">
         <v>46229</v>
@@ -1018,37 +1012,37 @@
         <v>22</v>
       </c>
       <c r="D3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="O3" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="P3">
         <v>400000</v>
       </c>
       <c r="Q3" t="s">
+        <v>162</v>
+      </c>
+      <c r="R3" t="s">
         <v>165</v>
       </c>
-      <c r="R3" t="s">
-        <v>168</v>
-      </c>
       <c r="S3" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T3" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="U3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V3" s="1">
         <v>46291</v>
@@ -1065,37 +1059,37 @@
         <v>22</v>
       </c>
       <c r="D4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O4" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="P4">
         <v>430000</v>
       </c>
       <c r="Q4" t="s">
+        <v>161</v>
+      </c>
+      <c r="R4" t="s">
         <v>164</v>
       </c>
-      <c r="R4" t="s">
-        <v>167</v>
-      </c>
       <c r="S4" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T4" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="U4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V4" s="1">
         <v>46321</v>
@@ -1112,37 +1106,37 @@
         <v>22</v>
       </c>
       <c r="D5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O5" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="P5">
         <v>425000</v>
       </c>
       <c r="Q5" t="s">
+        <v>161</v>
+      </c>
+      <c r="R5" t="s">
         <v>164</v>
       </c>
-      <c r="R5" t="s">
-        <v>167</v>
-      </c>
       <c r="S5" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T5" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="U5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V5" s="1">
         <v>46321</v>
@@ -1159,40 +1153,40 @@
         <v>22</v>
       </c>
       <c r="D6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="L6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="N6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="O6" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="P6">
         <v>563000</v>
       </c>
       <c r="Q6" t="s">
+        <v>161</v>
+      </c>
+      <c r="R6" t="s">
         <v>164</v>
       </c>
-      <c r="R6" t="s">
-        <v>167</v>
-      </c>
       <c r="S6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T6" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="U6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V6" s="1">
         <v>46291</v>
@@ -1209,46 +1203,46 @@
         <v>22</v>
       </c>
       <c r="D7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H7" s="1">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="N7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O7" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="P7">
         <v>3799999.6</v>
       </c>
       <c r="Q7" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="R7" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="S7" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T7" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="U7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V7" s="1">
         <v>46138</v>
@@ -1265,37 +1259,37 @@
         <v>22</v>
       </c>
       <c r="D8" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E8" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N8" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O8" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="P8">
         <v>430000</v>
       </c>
       <c r="Q8" t="s">
+        <v>161</v>
+      </c>
+      <c r="R8" t="s">
         <v>164</v>
       </c>
-      <c r="R8" t="s">
-        <v>167</v>
-      </c>
       <c r="S8" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T8" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="U8" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V8" s="1">
         <v>46291</v>
@@ -1312,37 +1306,37 @@
         <v>22</v>
       </c>
       <c r="D9" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O9" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="P9">
         <v>60000</v>
       </c>
       <c r="Q9" t="s">
+        <v>161</v>
+      </c>
+      <c r="R9" t="s">
         <v>164</v>
       </c>
-      <c r="R9" t="s">
-        <v>167</v>
-      </c>
       <c r="S9" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="U9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V9" s="1">
         <v>46291</v>
@@ -1359,37 +1353,37 @@
         <v>22</v>
       </c>
       <c r="D10" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="O10" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="P10">
         <v>200000</v>
       </c>
       <c r="Q10" t="s">
+        <v>161</v>
+      </c>
+      <c r="R10" t="s">
         <v>164</v>
       </c>
-      <c r="R10" t="s">
-        <v>167</v>
-      </c>
       <c r="S10" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T10" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="U10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V10" s="1">
         <v>46291</v>
@@ -1406,37 +1400,37 @@
         <v>22</v>
       </c>
       <c r="D11" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E11" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N11" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="O11" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="P11">
         <v>320000</v>
       </c>
       <c r="Q11" t="s">
+        <v>161</v>
+      </c>
+      <c r="R11" t="s">
         <v>164</v>
       </c>
-      <c r="R11" t="s">
-        <v>167</v>
-      </c>
       <c r="S11" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T11" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="U11" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V11" s="1">
         <v>46291</v>
@@ -1453,49 +1447,49 @@
         <v>22</v>
       </c>
       <c r="D12" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F12" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G12" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H12" s="1">
         <v>46079</v>
       </c>
       <c r="I12" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="J12" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="N12" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="O12" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="P12">
         <v>1187433.02</v>
       </c>
       <c r="Q12" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="R12" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="S12" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T12" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="U12" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="V12" s="1">
         <v>46079</v>
@@ -1512,37 +1506,37 @@
         <v>22</v>
       </c>
       <c r="D13" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E13" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F13" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N13" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="O13" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="P13">
         <v>1000000</v>
       </c>
       <c r="Q13" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="R13" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="S13" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T13" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="U13" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="V13" s="1">
         <v>46352</v>
@@ -1559,37 +1553,37 @@
         <v>22</v>
       </c>
       <c r="D14" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E14" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F14" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="O14" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="P14">
         <v>1000000</v>
       </c>
       <c r="Q14" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="R14" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="S14" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T14" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="U14" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="V14" s="1">
         <v>46352</v>
@@ -1606,37 +1600,37 @@
         <v>22</v>
       </c>
       <c r="D15" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E15" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F15" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N15" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="O15" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="P15">
         <v>1000000</v>
       </c>
       <c r="Q15" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="R15" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="S15" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T15" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="U15" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="V15" s="1">
         <v>46352</v>
@@ -1653,37 +1647,37 @@
         <v>22</v>
       </c>
       <c r="D16" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E16" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F16" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N16" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O16" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="P16">
         <v>100000</v>
       </c>
       <c r="Q16" t="s">
+        <v>162</v>
+      </c>
+      <c r="R16" t="s">
         <v>165</v>
       </c>
-      <c r="R16" t="s">
-        <v>168</v>
-      </c>
       <c r="S16" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T16" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="U16" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="V16" s="1">
         <v>46229</v>
@@ -1700,49 +1694,49 @@
         <v>22</v>
       </c>
       <c r="D17" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E17" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F17" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G17" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H17" s="1">
         <v>46098</v>
       </c>
       <c r="I17" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J17" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="N17" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="O17" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="P17">
         <v>1770880.5</v>
       </c>
       <c r="Q17" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="R17" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="S17" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T17" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="U17" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="V17" s="1">
         <v>46107</v>
@@ -1759,46 +1753,46 @@
         <v>22</v>
       </c>
       <c r="D18" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E18" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F18" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G18" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H18" s="1">
         <v>46076</v>
       </c>
       <c r="I18" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="N18" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O18" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="P18">
         <v>350000</v>
       </c>
       <c r="Q18" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="R18" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="S18" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T18" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="U18" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V18" s="1">
         <v>46079</v>
@@ -1815,46 +1809,46 @@
         <v>22</v>
       </c>
       <c r="D19" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E19" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F19" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G19" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H19" s="1">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="N19" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O19" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="P19">
         <v>350000</v>
       </c>
       <c r="Q19" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="R19" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="S19" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T19" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="U19" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V19" s="1">
         <v>46079</v>
@@ -1871,37 +1865,37 @@
         <v>22</v>
       </c>
       <c r="D20" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E20" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F20" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N20" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="O20" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="P20">
         <v>1000000</v>
       </c>
       <c r="Q20" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="R20" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="S20" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T20" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="U20" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V20" s="1">
         <v>46321</v>
@@ -1918,37 +1912,37 @@
         <v>22</v>
       </c>
       <c r="D21" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E21" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F21" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N21" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="O21" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="P21">
         <v>400000</v>
       </c>
       <c r="Q21" t="s">
+        <v>162</v>
+      </c>
+      <c r="R21" t="s">
         <v>165</v>
       </c>
-      <c r="R21" t="s">
-        <v>168</v>
-      </c>
       <c r="S21" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T21" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="U21" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V21" s="1">
         <v>46321</v>
@@ -1965,37 +1959,37 @@
         <v>22</v>
       </c>
       <c r="D22" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E22" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F22" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N22" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O22" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="P22">
         <v>120000</v>
       </c>
       <c r="Q22" t="s">
+        <v>161</v>
+      </c>
+      <c r="R22" t="s">
         <v>164</v>
       </c>
-      <c r="R22" t="s">
-        <v>167</v>
-      </c>
       <c r="S22" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T22" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="U22" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V22" s="1">
         <v>46321</v>
@@ -2012,37 +2006,37 @@
         <v>22</v>
       </c>
       <c r="D23" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E23" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F23" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N23" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O23" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="P23">
         <v>80000</v>
       </c>
       <c r="Q23" t="s">
+        <v>161</v>
+      </c>
+      <c r="R23" t="s">
         <v>164</v>
       </c>
-      <c r="R23" t="s">
-        <v>167</v>
-      </c>
       <c r="S23" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T23" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="U23" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V23" s="1">
         <v>46321</v>
@@ -2059,49 +2053,49 @@
         <v>22</v>
       </c>
       <c r="D24" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E24" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F24" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G24" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H24" s="1">
         <v>46119</v>
       </c>
       <c r="I24" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="J24" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="N24" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="O24" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="P24">
         <v>1704503</v>
       </c>
       <c r="Q24" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="R24" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="S24" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T24" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="U24" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="V24" s="1">
         <v>46138</v>
@@ -2118,46 +2112,46 @@
         <v>22</v>
       </c>
       <c r="D25" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E25" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F25" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G25" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H25" s="1">
         <v>46121</v>
       </c>
       <c r="I25" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="N25" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="O25" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="P25">
         <v>3799000</v>
       </c>
       <c r="Q25" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="R25" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="S25" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T25" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="U25" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V25" s="1">
         <v>46138</v>
@@ -2174,46 +2168,46 @@
         <v>22</v>
       </c>
       <c r="D26" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E26" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F26" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G26" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H26" s="1">
         <v>46076</v>
       </c>
       <c r="I26" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="N26" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="O26" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="P26">
         <v>1000</v>
       </c>
       <c r="Q26" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="R26" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="S26" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T26" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="U26" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V26" s="1">
         <v>46079</v>
@@ -2230,37 +2224,37 @@
         <v>22</v>
       </c>
       <c r="D27" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E27" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F27" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N27" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O27" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="P27">
         <v>100000</v>
       </c>
       <c r="Q27" t="s">
+        <v>162</v>
+      </c>
+      <c r="R27" t="s">
         <v>165</v>
       </c>
-      <c r="R27" t="s">
-        <v>168</v>
-      </c>
       <c r="S27" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T27" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="U27" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="V27" s="1">
         <v>46291</v>
@@ -2277,49 +2271,49 @@
         <v>22</v>
       </c>
       <c r="D28" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E28" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F28" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G28" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H28" s="1">
         <v>46199</v>
       </c>
       <c r="I28" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J28" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="N28" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="O28" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="P28">
         <v>150000</v>
       </c>
       <c r="Q28" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="R28" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="S28" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T28" t="s">
+        <v>172</v>
+      </c>
+      <c r="U28" t="s">
         <v>175</v>
-      </c>
-      <c r="U28" t="s">
-        <v>178</v>
       </c>
       <c r="V28" s="1">
         <v>46199</v>
@@ -2336,49 +2330,49 @@
         <v>22</v>
       </c>
       <c r="D29" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E29" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F29" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G29" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H29" s="1">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J29" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="N29" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="O29" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="P29">
         <v>150000</v>
       </c>
       <c r="Q29" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="R29" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="S29" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T29" t="s">
+        <v>172</v>
+      </c>
+      <c r="U29" t="s">
         <v>175</v>
-      </c>
-      <c r="U29" t="s">
-        <v>178</v>
       </c>
       <c r="V29" s="1">
         <v>46199</v>
@@ -2395,49 +2389,49 @@
         <v>22</v>
       </c>
       <c r="D30" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E30" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F30" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G30" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H30" s="1">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="J30" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="N30" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="O30" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="P30">
         <v>18462.36</v>
       </c>
       <c r="Q30" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="R30" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="S30" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T30" t="s">
+        <v>172</v>
+      </c>
+      <c r="U30" t="s">
         <v>175</v>
-      </c>
-      <c r="U30" t="s">
-        <v>178</v>
       </c>
       <c r="V30" s="1">
         <v>46199</v>
@@ -2454,49 +2448,49 @@
         <v>22</v>
       </c>
       <c r="D31" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E31" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F31" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G31" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H31" s="1">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J31" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="N31" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="O31" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="P31">
         <v>324166.14</v>
       </c>
       <c r="Q31" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="R31" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="S31" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T31" t="s">
+        <v>172</v>
+      </c>
+      <c r="U31" t="s">
         <v>175</v>
-      </c>
-      <c r="U31" t="s">
-        <v>178</v>
       </c>
       <c r="V31" s="1">
         <v>46199</v>
@@ -2513,40 +2507,40 @@
         <v>22</v>
       </c>
       <c r="D32" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E32" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F32" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="K32" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="N32" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="O32" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="P32">
         <v>30000</v>
       </c>
       <c r="Q32" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="R32" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="S32" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T32" t="s">
+        <v>172</v>
+      </c>
+      <c r="U32" t="s">
         <v>175</v>
-      </c>
-      <c r="U32" t="s">
-        <v>178</v>
       </c>
       <c r="V32" s="1">
         <v>46291</v>
@@ -2563,49 +2557,49 @@
         <v>22</v>
       </c>
       <c r="D33" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E33" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F33" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G33" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H33" s="1">
         <v>46191</v>
       </c>
       <c r="I33" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="J33" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="N33" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="O33" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="P33">
         <v>1496713.48</v>
       </c>
       <c r="Q33" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="R33" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="S33" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T33" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="U33" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="V33" s="1">
         <v>46199</v>
@@ -2622,46 +2616,46 @@
         <v>22</v>
       </c>
       <c r="D34" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E34" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F34" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G34" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H34" s="1">
         <v>46119</v>
       </c>
       <c r="I34" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="N34" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="O34" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="P34">
         <v>207789.52</v>
       </c>
       <c r="Q34" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="R34" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="S34" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T34" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="U34" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="V34" s="1">
         <v>46138</v>
@@ -2678,46 +2672,46 @@
         <v>22</v>
       </c>
       <c r="D35" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E35" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F35" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G35" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H35" s="1">
         <v>46213</v>
       </c>
       <c r="I35" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="N35" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="O35" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="P35">
         <v>962290.8</v>
       </c>
       <c r="Q35" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="R35" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="S35" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T35" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="U35" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V35" s="1">
         <v>46229</v>
@@ -2734,46 +2728,46 @@
         <v>22</v>
       </c>
       <c r="D36" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E36" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F36" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G36" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H36" s="1">
         <v>46175</v>
       </c>
       <c r="I36" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="N36" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="O36" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="P36">
         <v>798776.97</v>
       </c>
       <c r="Q36" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="R36" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="S36" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T36" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="U36" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V36" s="1">
         <v>46199</v>
@@ -2790,46 +2784,46 @@
         <v>22</v>
       </c>
       <c r="D37" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E37" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F37" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G37" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H37" s="1">
         <v>46213</v>
       </c>
       <c r="I37" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="N37" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="O37" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="P37">
         <v>1530656.62</v>
       </c>
       <c r="Q37" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="R37" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="S37" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T37" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="U37" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V37" s="1">
         <v>46229</v>
@@ -2846,46 +2840,46 @@
         <v>22</v>
       </c>
       <c r="D38" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E38" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F38" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G38" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H38" s="1">
         <v>46199</v>
       </c>
       <c r="I38" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="N38" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="O38" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="P38">
         <v>72958.08</v>
       </c>
       <c r="Q38" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="R38" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="S38" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T38" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="U38" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V38" s="1">
         <v>46199</v>
@@ -2902,46 +2896,46 @@
         <v>22</v>
       </c>
       <c r="D39" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E39" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F39" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G39" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H39" s="1">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="N39" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="O39" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="P39">
         <v>8916</v>
       </c>
       <c r="Q39" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="R39" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="S39" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T39" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="U39" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V39" s="1">
         <v>46199</v>
@@ -2958,46 +2952,46 @@
         <v>22</v>
       </c>
       <c r="D40" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E40" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F40" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G40" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H40" s="1">
         <v>46204</v>
       </c>
       <c r="I40" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="N40" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="O40" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="P40">
         <v>425178.5</v>
       </c>
       <c r="Q40" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="R40" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="S40" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T40" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="U40" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V40" s="1">
         <v>46229</v>
@@ -3014,46 +3008,46 @@
         <v>22</v>
       </c>
       <c r="D41" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E41" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F41" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G41" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H41" s="1">
         <v>46244</v>
       </c>
       <c r="I41" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="N41" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="O41" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="P41">
         <v>1223.03</v>
       </c>
       <c r="Q41" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="R41" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="S41" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T41" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="U41" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V41" s="1">
         <v>46199</v>
@@ -3070,34 +3064,34 @@
         <v>22</v>
       </c>
       <c r="D42" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E42" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G42" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="N42" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="O42" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="Q42" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="R42" t="s">
+        <v>165</v>
+      </c>
+      <c r="S42" t="s">
         <v>168</v>
       </c>
-      <c r="S42" t="s">
-        <v>171</v>
-      </c>
       <c r="T42" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="U42" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V42" s="1">
         <v>46260</v>
@@ -3114,46 +3108,46 @@
         <v>22</v>
       </c>
       <c r="D43" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E43" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F43" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G43" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H43" s="1">
         <v>46191</v>
       </c>
       <c r="I43" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="N43" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O43" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="P43">
         <v>400000</v>
       </c>
       <c r="Q43" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="R43" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="S43" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T43" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="U43" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V43" s="1">
         <v>46199</v>
@@ -3170,46 +3164,46 @@
         <v>22</v>
       </c>
       <c r="D44" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E44" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F44" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G44" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H44" s="1">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="N44" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O44" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="P44">
         <v>400000</v>
       </c>
       <c r="Q44" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="R44" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="S44" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T44" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="U44" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V44" s="1">
         <v>46199</v>
@@ -3226,49 +3220,49 @@
         <v>22</v>
       </c>
       <c r="D45" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E45" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F45" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G45" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H45" s="1">
         <v>46213</v>
       </c>
       <c r="I45" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="J45" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="N45" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="O45" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="P45">
         <v>173846.38</v>
       </c>
       <c r="Q45" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="R45" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="S45" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T45" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="U45" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="V45" s="1">
         <v>46229</v>
@@ -3285,46 +3279,46 @@
         <v>22</v>
       </c>
       <c r="D46" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E46" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F46" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G46" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H46" s="1">
         <v>46210</v>
       </c>
       <c r="I46" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="N46" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="O46" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="P46">
         <v>1530656.62</v>
       </c>
       <c r="Q46" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="R46" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="S46" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T46" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="U46" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="V46" s="1">
         <v>46229</v>
@@ -3341,37 +3335,37 @@
         <v>22</v>
       </c>
       <c r="D47" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E47" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F47" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N47" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="O47" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="P47">
         <v>1000000</v>
       </c>
       <c r="Q47" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="R47" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="S47" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T47" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="U47" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V47" s="1">
         <v>46321</v>
@@ -3388,37 +3382,37 @@
         <v>22</v>
       </c>
       <c r="D48" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E48" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F48" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N48" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="O48" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="P48">
         <v>958040</v>
       </c>
       <c r="Q48" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="R48" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="S48" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T48" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="U48" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="V48" s="1">
         <v>46291</v>
@@ -3435,49 +3429,49 @@
         <v>22</v>
       </c>
       <c r="D49" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E49" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F49" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G49" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H49" s="1">
         <v>46176</v>
       </c>
       <c r="I49" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J49" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="N49" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="O49" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="P49">
         <v>41730.64</v>
       </c>
       <c r="Q49" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="R49" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="S49" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T49" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="U49" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="V49" s="1">
         <v>46199</v>
@@ -3494,43 +3488,43 @@
         <v>22</v>
       </c>
       <c r="D50" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E50" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F50" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="J50" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="K50" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="N50" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="O50" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="P50">
         <v>1468159.32</v>
       </c>
       <c r="Q50" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="R50" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="S50" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T50" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="U50" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="V50" s="1">
         <v>46260</v>
@@ -3547,43 +3541,43 @@
         <v>22</v>
       </c>
       <c r="D51" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E51" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F51" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="J51" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="K51" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="N51" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="O51" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="P51">
         <v>1704503</v>
       </c>
       <c r="Q51" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="R51" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="S51" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T51" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="U51" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="V51" s="1">
         <v>46291</v>
@@ -3600,40 +3594,40 @@
         <v>22</v>
       </c>
       <c r="D52" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E52" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F52" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="K52" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="N52" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="O52" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="P52">
         <v>1704503</v>
       </c>
       <c r="Q52" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="R52" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="S52" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T52" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="U52" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="V52" s="1">
         <v>46321</v>
@@ -3650,46 +3644,46 @@
         <v>22</v>
       </c>
       <c r="D53" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E53" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F53" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G53" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H53" s="1">
         <v>46227</v>
       </c>
       <c r="I53" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="N53" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="O53" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="P53">
         <v>236343.68</v>
       </c>
       <c r="Q53" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="R53" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="S53" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T53" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="U53" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="V53" s="1">
         <v>46229</v>
@@ -3706,40 +3700,40 @@
         <v>22</v>
       </c>
       <c r="D54" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E54" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F54" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="K54" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="N54" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="O54" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="P54">
         <v>1295422.28</v>
       </c>
       <c r="Q54" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="R54" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="S54" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T54" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="U54" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="V54" s="1">
         <v>46352</v>
@@ -3756,40 +3750,40 @@
         <v>22</v>
       </c>
       <c r="D55" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E55" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F55" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="K55" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="N55" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O55" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="P55">
         <v>500000</v>
       </c>
       <c r="Q55" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="R55" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="S55" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="T55" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="U55" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="V55" s="1">
         <v>46321</v>
@@ -3806,40 +3800,40 @@
         <v>22</v>
       </c>
       <c r="D56" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E56" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F56" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G56" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="N56" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O56" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="P56">
         <v>5000000</v>
       </c>
       <c r="Q56" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="R56" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="S56" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="T56" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="U56" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="V56" s="1">
         <v>46321</v>
@@ -3856,34 +3850,34 @@
         <v>22</v>
       </c>
       <c r="D57" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E57" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G57" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="N57" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O57" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="Q57" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="R57" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="S57" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="T57" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="U57" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="V57" s="1">
         <v>46049</v>
@@ -3900,34 +3894,34 @@
         <v>22</v>
       </c>
       <c r="D58" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E58" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G58" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="N58" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O58" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="Q58" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="R58" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="S58" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="T58" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="U58" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="59" spans="1:22">
@@ -3941,34 +3935,34 @@
         <v>22</v>
       </c>
       <c r="D59" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E59" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G59" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="N59" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O59" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="Q59" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="R59" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="S59" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="T59" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="U59" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="60" spans="1:22">
@@ -3982,34 +3976,34 @@
         <v>22</v>
       </c>
       <c r="D60" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E60" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N60" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="O60" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="P60">
         <v>9389.959999999999</v>
       </c>
       <c r="Q60" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="R60" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="S60" t="s">
+        <v>168</v>
+      </c>
+      <c r="T60" t="s">
         <v>171</v>
       </c>
-      <c r="T60" t="s">
-        <v>174</v>
-      </c>
       <c r="U60" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="V60" s="1">
         <v>46107</v>
@@ -4026,34 +4020,34 @@
         <v>22</v>
       </c>
       <c r="D61" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E61" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N61" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="O61" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="P61">
         <v>7204.82</v>
       </c>
       <c r="Q61" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="R61" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="S61" t="s">
+        <v>168</v>
+      </c>
+      <c r="T61" t="s">
         <v>171</v>
       </c>
-      <c r="T61" t="s">
-        <v>174</v>
-      </c>
       <c r="U61" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="V61" s="1">
         <v>46107</v>
@@ -4070,34 +4064,34 @@
         <v>22</v>
       </c>
       <c r="D62" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E62" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N62" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="O62" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="P62">
         <v>4227.84</v>
       </c>
       <c r="Q62" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="R62" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="S62" t="s">
+        <v>168</v>
+      </c>
+      <c r="T62" t="s">
         <v>171</v>
       </c>
-      <c r="T62" t="s">
-        <v>174</v>
-      </c>
       <c r="U62" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="V62" s="1">
         <v>46107</v>
@@ -4114,34 +4108,34 @@
         <v>22</v>
       </c>
       <c r="D63" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E63" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N63" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="O63" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="P63">
         <v>4064.54</v>
       </c>
       <c r="Q63" t="s">
+        <v>163</v>
+      </c>
+      <c r="R63" t="s">
         <v>166</v>
       </c>
-      <c r="R63" t="s">
-        <v>169</v>
-      </c>
       <c r="S63" t="s">
+        <v>168</v>
+      </c>
+      <c r="T63" t="s">
         <v>171</v>
       </c>
-      <c r="T63" t="s">
-        <v>174</v>
-      </c>
       <c r="U63" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="V63" s="1">
         <v>46107</v>
@@ -4158,34 +4152,34 @@
         <v>22</v>
       </c>
       <c r="D64" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E64" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N64" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="O64" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="P64">
         <v>3662.66</v>
       </c>
       <c r="Q64" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="R64" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="S64" t="s">
+        <v>168</v>
+      </c>
+      <c r="T64" t="s">
         <v>171</v>
       </c>
-      <c r="T64" t="s">
-        <v>174</v>
-      </c>
       <c r="U64" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="V64" s="1">
         <v>46107</v>
@@ -4202,34 +4196,34 @@
         <v>22</v>
       </c>
       <c r="D65" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E65" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N65" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="O65" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="P65">
         <v>1163.64</v>
       </c>
       <c r="Q65" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="R65" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="S65" t="s">
+        <v>168</v>
+      </c>
+      <c r="T65" t="s">
         <v>171</v>
       </c>
-      <c r="T65" t="s">
-        <v>174</v>
-      </c>
       <c r="U65" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="V65" s="1">
         <v>46107</v>
@@ -4246,34 +4240,34 @@
         <v>22</v>
       </c>
       <c r="D66" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E66" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N66" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O66" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="P66">
         <v>120000</v>
       </c>
       <c r="Q66" t="s">
+        <v>161</v>
+      </c>
+      <c r="R66" t="s">
         <v>164</v>
       </c>
-      <c r="R66" t="s">
-        <v>167</v>
-      </c>
       <c r="S66" t="s">
+        <v>168</v>
+      </c>
+      <c r="T66" t="s">
         <v>171</v>
       </c>
-      <c r="T66" t="s">
-        <v>174</v>
-      </c>
       <c r="U66" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V66" s="1">
         <v>46168</v>
@@ -4290,37 +4284,37 @@
         <v>22</v>
       </c>
       <c r="D67" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E67" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F67" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N67" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="O67" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="P67">
         <v>400000</v>
       </c>
       <c r="Q67" t="s">
+        <v>162</v>
+      </c>
+      <c r="R67" t="s">
         <v>165</v>
       </c>
-      <c r="R67" t="s">
-        <v>168</v>
-      </c>
       <c r="S67" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T67" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="U67" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V67" s="1">
         <v>46291</v>
@@ -4337,37 +4331,37 @@
         <v>22</v>
       </c>
       <c r="D68" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E68" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F68" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N68" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O68" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="P68">
         <v>100000</v>
       </c>
       <c r="Q68" t="s">
+        <v>162</v>
+      </c>
+      <c r="R68" t="s">
         <v>165</v>
       </c>
-      <c r="R68" t="s">
-        <v>168</v>
-      </c>
       <c r="S68" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T68" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="U68" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="V68" s="1">
         <v>46229</v>
@@ -4384,34 +4378,34 @@
         <v>22</v>
       </c>
       <c r="D69" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E69" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N69" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O69" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="P69">
         <v>80000</v>
       </c>
       <c r="Q69" t="s">
+        <v>161</v>
+      </c>
+      <c r="R69" t="s">
         <v>164</v>
       </c>
-      <c r="R69" t="s">
-        <v>167</v>
-      </c>
       <c r="S69" t="s">
+        <v>168</v>
+      </c>
+      <c r="T69" t="s">
         <v>171</v>
       </c>
-      <c r="T69" t="s">
-        <v>174</v>
-      </c>
       <c r="U69" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V69" s="1">
         <v>46260</v>
@@ -4428,34 +4422,34 @@
         <v>22</v>
       </c>
       <c r="D70" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E70" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N70" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="O70" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="P70">
         <v>835000</v>
       </c>
       <c r="Q70" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="R70" t="s">
+        <v>165</v>
+      </c>
+      <c r="S70" t="s">
         <v>168</v>
       </c>
-      <c r="S70" t="s">
+      <c r="T70" t="s">
         <v>171</v>
       </c>
-      <c r="T70" t="s">
-        <v>174</v>
-      </c>
       <c r="U70" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="V70" s="1">
         <v>46291</v>
@@ -4472,34 +4466,34 @@
         <v>22</v>
       </c>
       <c r="D71" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E71" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N71" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="O71" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="P71">
         <v>165000</v>
       </c>
       <c r="Q71" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="R71" t="s">
+        <v>165</v>
+      </c>
+      <c r="S71" t="s">
         <v>168</v>
       </c>
-      <c r="S71" t="s">
+      <c r="T71" t="s">
         <v>171</v>
       </c>
-      <c r="T71" t="s">
-        <v>174</v>
-      </c>
       <c r="U71" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="V71" s="1">
         <v>46168</v>
@@ -4516,34 +4510,34 @@
         <v>22</v>
       </c>
       <c r="D72" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E72" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N72" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="O72" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="P72">
         <v>1000000</v>
       </c>
       <c r="Q72" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="R72" t="s">
+        <v>165</v>
+      </c>
+      <c r="S72" t="s">
         <v>168</v>
       </c>
-      <c r="S72" t="s">
+      <c r="T72" t="s">
         <v>171</v>
       </c>
-      <c r="T72" t="s">
-        <v>174</v>
-      </c>
       <c r="U72" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="V72" s="1">
         <v>46291</v>
@@ -4560,34 +4554,34 @@
         <v>22</v>
       </c>
       <c r="D73" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E73" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N73" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="O73" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="P73">
         <v>1000000</v>
       </c>
       <c r="Q73" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="R73" t="s">
+        <v>165</v>
+      </c>
+      <c r="S73" t="s">
         <v>168</v>
       </c>
-      <c r="S73" t="s">
+      <c r="T73" t="s">
         <v>171</v>
       </c>
-      <c r="T73" t="s">
-        <v>174</v>
-      </c>
       <c r="U73" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="V73" s="1">
         <v>46291</v>
@@ -4604,34 +4598,34 @@
         <v>22</v>
       </c>
       <c r="D74" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E74" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N74" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O74" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="P74">
         <v>100000</v>
       </c>
       <c r="Q74" t="s">
+        <v>162</v>
+      </c>
+      <c r="R74" t="s">
         <v>165</v>
       </c>
-      <c r="R74" t="s">
+      <c r="S74" t="s">
         <v>168</v>
       </c>
-      <c r="S74" t="s">
+      <c r="T74" t="s">
         <v>171</v>
       </c>
-      <c r="T74" t="s">
-        <v>174</v>
-      </c>
       <c r="U74" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="V74" s="1">
         <v>46291</v>
@@ -4648,37 +4642,37 @@
         <v>22</v>
       </c>
       <c r="D75" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E75" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F75" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N75" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="O75" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="P75">
         <v>1000000</v>
       </c>
       <c r="Q75" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="R75" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="S75" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T75" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="U75" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V75" s="1">
         <v>46321</v>
@@ -4695,40 +4689,40 @@
         <v>22</v>
       </c>
       <c r="D76" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E76" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F76" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G76" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="N76" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="O76" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="P76">
         <v>1704503</v>
       </c>
       <c r="Q76" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="R76" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="S76" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="T76" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="U76" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="V76" s="1">
         <v>46381</v>
@@ -4745,40 +4739,40 @@
         <v>22</v>
       </c>
       <c r="D77" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E77" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F77" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G77" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="N77" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="O77" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="P77">
         <v>1638125.5</v>
       </c>
       <c r="Q77" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="R77" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="S77" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="T77" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="U77" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="V77" s="1">
         <v>46381</v>
@@ -4795,40 +4789,40 @@
         <v>22</v>
       </c>
       <c r="D78" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E78" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F78" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G78" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="N78" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O78" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="P78">
         <v>3800000</v>
       </c>
       <c r="Q78" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="R78" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="S78" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="T78" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="U78" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V78" s="1">
         <v>46381</v>
@@ -4845,40 +4839,40 @@
         <v>22</v>
       </c>
       <c r="D79" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E79" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F79" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G79" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="N79" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O79" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="P79">
         <v>3800000</v>
       </c>
       <c r="Q79" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="R79" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="S79" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="T79" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="U79" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V79" s="1">
         <v>46381</v>
@@ -4895,40 +4889,40 @@
         <v>22</v>
       </c>
       <c r="D80" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E80" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="J80" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K80" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="N80" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="O80" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="P80">
         <v>3800000</v>
       </c>
       <c r="Q80" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="R80" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="S80" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="T80" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="U80" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V80" s="1">
         <v>46382</v>
@@ -4945,34 +4939,34 @@
         <v>22</v>
       </c>
       <c r="D81" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E81" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N81" t="s">
+        <v>93</v>
+      </c>
+      <c r="O81" t="s">
         <v>94</v>
-      </c>
-      <c r="O81" t="s">
-        <v>95</v>
       </c>
       <c r="P81">
         <v>4394700</v>
       </c>
       <c r="Q81" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="R81" t="s">
+        <v>165</v>
+      </c>
+      <c r="S81" t="s">
         <v>168</v>
       </c>
-      <c r="S81" t="s">
-        <v>171</v>
-      </c>
       <c r="T81" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="U81" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V81" s="1">
         <v>46382</v>
@@ -4989,40 +4983,40 @@
         <v>22</v>
       </c>
       <c r="D82" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E82" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F82" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="K82" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="N82" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="O82" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="P82">
         <v>528395.9300000001</v>
       </c>
       <c r="Q82" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="R82" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="S82" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T82" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="U82" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="V82" s="1">
         <v>46382</v>
@@ -5039,34 +5033,34 @@
         <v>22</v>
       </c>
       <c r="D83" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E83" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N83" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="O83" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="P83">
         <v>1000000</v>
       </c>
       <c r="Q83" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="R83" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="S83" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="T83" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="U83" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V83" s="1">
         <v>46321</v>
@@ -5083,34 +5077,34 @@
         <v>22</v>
       </c>
       <c r="D84" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E84" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N84" t="s">
+        <v>93</v>
+      </c>
+      <c r="O84" t="s">
         <v>94</v>
-      </c>
-      <c r="O84" t="s">
-        <v>95</v>
       </c>
       <c r="P84">
         <v>4394700</v>
       </c>
       <c r="Q84" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="R84" t="s">
+        <v>165</v>
+      </c>
+      <c r="S84" t="s">
         <v>168</v>
       </c>
-      <c r="S84" t="s">
-        <v>171</v>
-      </c>
       <c r="T84" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="U84" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V84" s="1">
         <v>46382</v>
@@ -5127,40 +5121,40 @@
         <v>22</v>
       </c>
       <c r="D85" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E85" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F85" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G85" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="N85" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="O85" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="P85">
         <v>3306000</v>
       </c>
       <c r="Q85" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="R85" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="S85" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="T85" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="U85" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="86" spans="1:22">
@@ -5174,87 +5168,40 @@
         <v>22</v>
       </c>
       <c r="D86" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E86" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F86" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G86" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="N86" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="O86" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="P86">
         <v>3306000</v>
       </c>
       <c r="Q86" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="R86" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="S86" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="T86" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="U86" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="87" spans="1:22">
-      <c r="A87">
-        <v>64800</v>
-      </c>
-      <c r="B87" t="s">
-        <v>22</v>
-      </c>
-      <c r="C87" t="s">
-        <v>24</v>
-      </c>
-      <c r="D87" t="s">
-        <v>25</v>
-      </c>
-      <c r="E87" t="s">
-        <v>29</v>
-      </c>
-      <c r="F87" t="s">
-        <v>31</v>
-      </c>
-      <c r="N87" t="s">
-        <v>96</v>
-      </c>
-      <c r="O87" t="s">
-        <v>163</v>
-      </c>
-      <c r="P87">
-        <v>212577</v>
-      </c>
-      <c r="Q87" t="s">
-        <v>166</v>
-      </c>
-      <c r="R87" t="s">
-        <v>167</v>
-      </c>
-      <c r="S87" t="s">
-        <v>170</v>
-      </c>
-      <c r="T87" t="s">
-        <v>177</v>
-      </c>
-      <c r="U87" t="s">
-        <v>30</v>
-      </c>
-      <c r="V87" s="1">
-        <v>46260</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: mta (27/08/2026 17:59)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1110" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1117" uniqueCount="178">
   <si>
     <t>linha</t>
   </si>
@@ -224,6 +224,12 @@
   </si>
   <si>
     <t>REMANEJAR</t>
+  </si>
+  <si>
+    <t>ATENDER R$ 621.454,453</t>
+  </si>
+  <si>
+    <t>ATENDER</t>
   </si>
   <si>
     <t>Atender AGO</t>
@@ -971,31 +977,31 @@
         <v>69</v>
       </c>
       <c r="L2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="N2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="O2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="P2">
         <v>135000</v>
       </c>
       <c r="Q2" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R2" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="S2" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T2" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="U2" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="V2" s="1">
         <v>46229</v>
@@ -1021,25 +1027,25 @@
         <v>30</v>
       </c>
       <c r="N3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="O3" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="P3">
         <v>400000</v>
       </c>
       <c r="Q3" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="R3" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="S3" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T3" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="U3" t="s">
         <v>28</v>
@@ -1068,25 +1074,25 @@
         <v>30</v>
       </c>
       <c r="N4" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="O4" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="P4">
         <v>430000</v>
       </c>
       <c r="Q4" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R4" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="S4" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T4" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="U4" t="s">
         <v>28</v>
@@ -1115,25 +1121,25 @@
         <v>30</v>
       </c>
       <c r="N5" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="O5" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="P5">
         <v>425000</v>
       </c>
       <c r="Q5" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R5" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="S5" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T5" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="U5" t="s">
         <v>28</v>
@@ -1162,28 +1168,28 @@
         <v>30</v>
       </c>
       <c r="L6" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="N6" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="O6" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="P6">
         <v>563000</v>
       </c>
       <c r="Q6" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R6" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="S6" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T6" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="U6" t="s">
         <v>28</v>
@@ -1221,25 +1227,25 @@
         <v>45</v>
       </c>
       <c r="N7" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="O7" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="P7">
         <v>3799999.6</v>
       </c>
       <c r="Q7" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="R7" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="S7" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T7" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="U7" t="s">
         <v>28</v>
@@ -1268,25 +1274,25 @@
         <v>30</v>
       </c>
       <c r="N8" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="O8" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="P8">
         <v>430000</v>
       </c>
       <c r="Q8" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R8" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="S8" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T8" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="U8" t="s">
         <v>28</v>
@@ -1315,25 +1321,25 @@
         <v>30</v>
       </c>
       <c r="N9" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="O9" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="P9">
         <v>60000</v>
       </c>
       <c r="Q9" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R9" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="S9" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T9" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="U9" t="s">
         <v>28</v>
@@ -1362,25 +1368,25 @@
         <v>30</v>
       </c>
       <c r="N10" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="O10" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="P10">
         <v>200000</v>
       </c>
       <c r="Q10" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R10" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="S10" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T10" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="U10" t="s">
         <v>28</v>
@@ -1409,25 +1415,25 @@
         <v>30</v>
       </c>
       <c r="N11" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="O11" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="P11">
         <v>320000</v>
       </c>
       <c r="Q11" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R11" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="S11" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T11" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="U11" t="s">
         <v>28</v>
@@ -1468,28 +1474,28 @@
         <v>62</v>
       </c>
       <c r="N12" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="O12" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="P12">
         <v>1187433.02</v>
       </c>
       <c r="Q12" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R12" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="S12" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T12" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="U12" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="V12" s="1">
         <v>46079</v>
@@ -1514,29 +1520,32 @@
       <c r="F13" t="s">
         <v>30</v>
       </c>
+      <c r="K13" t="s">
+        <v>70</v>
+      </c>
       <c r="N13" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="O13" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="P13">
         <v>1000000</v>
       </c>
       <c r="Q13" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R13" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="S13" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T13" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="U13" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="V13" s="1">
         <v>46352</v>
@@ -1561,29 +1570,32 @@
       <c r="F14" t="s">
         <v>30</v>
       </c>
+      <c r="K14" t="s">
+        <v>71</v>
+      </c>
       <c r="N14" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="O14" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="P14">
         <v>1000000</v>
       </c>
       <c r="Q14" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R14" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="S14" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T14" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="U14" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="V14" s="1">
         <v>46352</v>
@@ -1608,29 +1620,32 @@
       <c r="F15" t="s">
         <v>30</v>
       </c>
+      <c r="K15" t="s">
+        <v>71</v>
+      </c>
       <c r="N15" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="O15" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="P15">
         <v>1000000</v>
       </c>
       <c r="Q15" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R15" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="S15" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T15" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="U15" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="V15" s="1">
         <v>46352</v>
@@ -1655,29 +1670,32 @@
       <c r="F16" t="s">
         <v>30</v>
       </c>
+      <c r="K16" t="s">
+        <v>71</v>
+      </c>
       <c r="N16" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="O16" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="P16">
         <v>100000</v>
       </c>
       <c r="Q16" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="R16" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="S16" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T16" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="U16" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="V16" s="1">
         <v>46229</v>
@@ -1715,28 +1733,28 @@
         <v>62</v>
       </c>
       <c r="N17" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O17" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="P17">
         <v>1770880.5</v>
       </c>
       <c r="Q17" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="R17" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="S17" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T17" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="U17" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="V17" s="1">
         <v>46107</v>
@@ -1771,25 +1789,25 @@
         <v>48</v>
       </c>
       <c r="N18" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="O18" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="P18">
         <v>350000</v>
       </c>
       <c r="Q18" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="R18" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="S18" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T18" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="U18" t="s">
         <v>28</v>
@@ -1827,25 +1845,25 @@
         <v>48</v>
       </c>
       <c r="N19" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="O19" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="P19">
         <v>350000</v>
       </c>
       <c r="Q19" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="R19" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="S19" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T19" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="U19" t="s">
         <v>28</v>
@@ -1874,25 +1892,25 @@
         <v>30</v>
       </c>
       <c r="N20" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="O20" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="P20">
         <v>1000000</v>
       </c>
       <c r="Q20" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="R20" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="S20" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T20" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="U20" t="s">
         <v>28</v>
@@ -1921,25 +1939,25 @@
         <v>30</v>
       </c>
       <c r="N21" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="O21" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="P21">
         <v>400000</v>
       </c>
       <c r="Q21" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="R21" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="S21" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T21" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="U21" t="s">
         <v>28</v>
@@ -1968,25 +1986,25 @@
         <v>30</v>
       </c>
       <c r="N22" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="O22" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="P22">
         <v>120000</v>
       </c>
       <c r="Q22" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R22" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="S22" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T22" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="U22" t="s">
         <v>28</v>
@@ -2015,25 +2033,25 @@
         <v>30</v>
       </c>
       <c r="N23" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="O23" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="P23">
         <v>80000</v>
       </c>
       <c r="Q23" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R23" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="S23" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T23" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="U23" t="s">
         <v>28</v>
@@ -2074,28 +2092,28 @@
         <v>63</v>
       </c>
       <c r="N24" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O24" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="P24">
         <v>1704503</v>
       </c>
       <c r="Q24" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="R24" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="S24" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T24" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="U24" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="V24" s="1">
         <v>46138</v>
@@ -2130,25 +2148,25 @@
         <v>50</v>
       </c>
       <c r="N25" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="O25" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="P25">
         <v>3799000</v>
       </c>
       <c r="Q25" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="R25" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="S25" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T25" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="U25" t="s">
         <v>28</v>
@@ -2186,25 +2204,25 @@
         <v>51</v>
       </c>
       <c r="N26" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="O26" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="P26">
         <v>1000</v>
       </c>
       <c r="Q26" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="R26" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="S26" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T26" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="U26" t="s">
         <v>28</v>
@@ -2232,29 +2250,32 @@
       <c r="F27" t="s">
         <v>30</v>
       </c>
+      <c r="K27" t="s">
+        <v>71</v>
+      </c>
       <c r="N27" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="O27" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="P27">
         <v>100000</v>
       </c>
       <c r="Q27" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="R27" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="S27" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T27" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="U27" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="V27" s="1">
         <v>46291</v>
@@ -2292,28 +2313,28 @@
         <v>64</v>
       </c>
       <c r="N28" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O28" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="P28">
         <v>150000</v>
       </c>
       <c r="Q28" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="R28" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="S28" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T28" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="U28" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="V28" s="1">
         <v>46199</v>
@@ -2351,28 +2372,28 @@
         <v>64</v>
       </c>
       <c r="N29" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O29" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="P29">
         <v>150000</v>
       </c>
       <c r="Q29" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="R29" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="S29" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T29" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="U29" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="V29" s="1">
         <v>46199</v>
@@ -2410,28 +2431,28 @@
         <v>64</v>
       </c>
       <c r="N30" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O30" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="P30">
         <v>18462.36</v>
       </c>
       <c r="Q30" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="R30" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="S30" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T30" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="U30" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="V30" s="1">
         <v>46199</v>
@@ -2469,28 +2490,28 @@
         <v>64</v>
       </c>
       <c r="N31" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O31" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="P31">
         <v>324166.14</v>
       </c>
       <c r="Q31" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="R31" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="S31" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T31" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="U31" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="V31" s="1">
         <v>46199</v>
@@ -2519,28 +2540,28 @@
         <v>69</v>
       </c>
       <c r="N32" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O32" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="P32">
         <v>30000</v>
       </c>
       <c r="Q32" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="R32" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="S32" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T32" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="U32" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="V32" s="1">
         <v>46291</v>
@@ -2578,28 +2599,28 @@
         <v>65</v>
       </c>
       <c r="N33" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O33" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="P33">
         <v>1496713.48</v>
       </c>
       <c r="Q33" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="R33" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="S33" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T33" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="U33" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="V33" s="1">
         <v>46199</v>
@@ -2634,28 +2655,28 @@
         <v>49</v>
       </c>
       <c r="N34" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O34" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="P34">
         <v>207789.52</v>
       </c>
       <c r="Q34" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="R34" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="S34" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T34" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="U34" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="V34" s="1">
         <v>46138</v>
@@ -2690,25 +2711,25 @@
         <v>55</v>
       </c>
       <c r="N35" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="O35" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="P35">
         <v>962290.8</v>
       </c>
       <c r="Q35" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="R35" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="S35" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T35" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="U35" t="s">
         <v>28</v>
@@ -2746,25 +2767,25 @@
         <v>56</v>
       </c>
       <c r="N36" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="O36" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="P36">
         <v>798776.97</v>
       </c>
       <c r="Q36" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="R36" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="S36" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T36" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="U36" t="s">
         <v>28</v>
@@ -2802,25 +2823,25 @@
         <v>55</v>
       </c>
       <c r="N37" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="O37" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="P37">
         <v>1530656.62</v>
       </c>
       <c r="Q37" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="R37" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="S37" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T37" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="U37" t="s">
         <v>28</v>
@@ -2858,25 +2879,25 @@
         <v>57</v>
       </c>
       <c r="N38" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="O38" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="P38">
         <v>72958.08</v>
       </c>
       <c r="Q38" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="R38" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="S38" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T38" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="U38" t="s">
         <v>28</v>
@@ -2914,25 +2935,25 @@
         <v>57</v>
       </c>
       <c r="N39" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="O39" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="P39">
         <v>8916</v>
       </c>
       <c r="Q39" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="R39" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="S39" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T39" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="U39" t="s">
         <v>28</v>
@@ -2970,25 +2991,25 @@
         <v>57</v>
       </c>
       <c r="N40" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="O40" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="P40">
         <v>425178.5</v>
       </c>
       <c r="Q40" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="R40" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="S40" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T40" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="U40" t="s">
         <v>28</v>
@@ -3026,25 +3047,25 @@
         <v>58</v>
       </c>
       <c r="N41" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="O41" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="P41">
         <v>1223.03</v>
       </c>
       <c r="Q41" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="R41" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="S41" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T41" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="U41" t="s">
         <v>28</v>
@@ -3073,22 +3094,22 @@
         <v>42</v>
       </c>
       <c r="N42" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="O42" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="Q42" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="R42" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="S42" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="T42" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="U42" t="s">
         <v>28</v>
@@ -3126,25 +3147,25 @@
         <v>59</v>
       </c>
       <c r="N43" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="O43" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="P43">
         <v>400000</v>
       </c>
       <c r="Q43" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="R43" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="S43" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T43" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="U43" t="s">
         <v>28</v>
@@ -3182,25 +3203,25 @@
         <v>59</v>
       </c>
       <c r="N44" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="O44" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="P44">
         <v>400000</v>
       </c>
       <c r="Q44" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="R44" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="S44" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T44" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="U44" t="s">
         <v>28</v>
@@ -3241,28 +3262,28 @@
         <v>66</v>
       </c>
       <c r="N45" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O45" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="P45">
         <v>173846.38</v>
       </c>
       <c r="Q45" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="R45" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="S45" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T45" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="U45" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="V45" s="1">
         <v>46229</v>
@@ -3297,28 +3318,28 @@
         <v>53</v>
       </c>
       <c r="N46" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O46" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="P46">
         <v>1530656.62</v>
       </c>
       <c r="Q46" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="R46" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="S46" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T46" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="U46" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="V46" s="1">
         <v>46229</v>
@@ -3344,25 +3365,25 @@
         <v>30</v>
       </c>
       <c r="N47" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="O47" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="P47">
         <v>1000000</v>
       </c>
       <c r="Q47" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="R47" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="S47" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T47" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="U47" t="s">
         <v>28</v>
@@ -3390,29 +3411,32 @@
       <c r="F48" t="s">
         <v>30</v>
       </c>
+      <c r="K48" t="s">
+        <v>71</v>
+      </c>
       <c r="N48" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="O48" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="P48">
         <v>958040</v>
       </c>
       <c r="Q48" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R48" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="S48" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T48" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="U48" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="V48" s="1">
         <v>46291</v>
@@ -3450,28 +3474,28 @@
         <v>67</v>
       </c>
       <c r="N49" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="O49" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="P49">
         <v>41730.64</v>
       </c>
       <c r="Q49" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R49" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="S49" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T49" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="U49" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="V49" s="1">
         <v>46199</v>
@@ -3500,31 +3524,31 @@
         <v>66</v>
       </c>
       <c r="K50" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="N50" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O50" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="P50">
         <v>1468159.32</v>
       </c>
       <c r="Q50" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="R50" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="S50" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T50" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="U50" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="V50" s="1">
         <v>46260</v>
@@ -3553,31 +3577,31 @@
         <v>66</v>
       </c>
       <c r="K51" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="N51" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O51" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="P51">
         <v>1704503</v>
       </c>
       <c r="Q51" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="R51" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="S51" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T51" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="U51" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="V51" s="1">
         <v>46291</v>
@@ -3603,31 +3627,31 @@
         <v>30</v>
       </c>
       <c r="K52" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="N52" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O52" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="P52">
         <v>1704503</v>
       </c>
       <c r="Q52" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="R52" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="S52" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T52" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="U52" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="V52" s="1">
         <v>46321</v>
@@ -3662,28 +3686,28 @@
         <v>61</v>
       </c>
       <c r="N53" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O53" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="P53">
         <v>236343.68</v>
       </c>
       <c r="Q53" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="R53" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="S53" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T53" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="U53" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="V53" s="1">
         <v>46229</v>
@@ -3709,31 +3733,31 @@
         <v>30</v>
       </c>
       <c r="K54" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="N54" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O54" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="P54">
         <v>1295422.28</v>
       </c>
       <c r="Q54" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="R54" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="S54" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T54" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="U54" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="V54" s="1">
         <v>46352</v>
@@ -3759,31 +3783,31 @@
         <v>39</v>
       </c>
       <c r="K55" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="N55" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="O55" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="P55">
         <v>500000</v>
       </c>
       <c r="Q55" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="R55" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="S55" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="T55" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="U55" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="V55" s="1">
         <v>46321</v>
@@ -3812,28 +3836,28 @@
         <v>43</v>
       </c>
       <c r="N56" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="O56" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="P56">
         <v>5000000</v>
       </c>
       <c r="Q56" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="R56" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="S56" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="T56" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="U56" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="V56" s="1">
         <v>46321</v>
@@ -3859,25 +3883,25 @@
         <v>42</v>
       </c>
       <c r="N57" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="O57" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="Q57" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="R57" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="S57" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="T57" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="U57" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="V57" s="1">
         <v>46049</v>
@@ -3903,25 +3927,25 @@
         <v>42</v>
       </c>
       <c r="N58" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="O58" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="Q58" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="R58" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="S58" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="T58" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="U58" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
     </row>
     <row r="59" spans="1:22">
@@ -3944,25 +3968,25 @@
         <v>42</v>
       </c>
       <c r="N59" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="O59" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="Q59" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="R59" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="S59" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="T59" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="U59" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
     </row>
     <row r="60" spans="1:22">
@@ -3982,28 +4006,28 @@
         <v>29</v>
       </c>
       <c r="N60" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="O60" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="P60">
         <v>9389.959999999999</v>
       </c>
       <c r="Q60" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R60" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="S60" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="T60" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="U60" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="V60" s="1">
         <v>46107</v>
@@ -4026,28 +4050,28 @@
         <v>29</v>
       </c>
       <c r="N61" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="O61" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="P61">
         <v>7204.82</v>
       </c>
       <c r="Q61" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R61" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="S61" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="T61" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="U61" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="V61" s="1">
         <v>46107</v>
@@ -4070,28 +4094,28 @@
         <v>29</v>
       </c>
       <c r="N62" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="O62" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="P62">
         <v>4227.84</v>
       </c>
       <c r="Q62" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R62" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="S62" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="T62" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="U62" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="V62" s="1">
         <v>46107</v>
@@ -4114,28 +4138,28 @@
         <v>29</v>
       </c>
       <c r="N63" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="O63" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="P63">
         <v>4064.54</v>
       </c>
       <c r="Q63" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="R63" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="S63" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="T63" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="U63" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="V63" s="1">
         <v>46107</v>
@@ -4158,28 +4182,28 @@
         <v>29</v>
       </c>
       <c r="N64" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="O64" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="P64">
         <v>3662.66</v>
       </c>
       <c r="Q64" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R64" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="S64" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="T64" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="U64" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="V64" s="1">
         <v>46107</v>
@@ -4202,28 +4226,28 @@
         <v>29</v>
       </c>
       <c r="N65" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="O65" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="P65">
         <v>1163.64</v>
       </c>
       <c r="Q65" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="R65" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="S65" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="T65" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="U65" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="V65" s="1">
         <v>46107</v>
@@ -4246,25 +4270,25 @@
         <v>29</v>
       </c>
       <c r="N66" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="O66" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="P66">
         <v>120000</v>
       </c>
       <c r="Q66" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R66" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="S66" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="T66" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="U66" t="s">
         <v>28</v>
@@ -4293,25 +4317,25 @@
         <v>30</v>
       </c>
       <c r="N67" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="O67" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="P67">
         <v>400000</v>
       </c>
       <c r="Q67" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="R67" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="S67" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T67" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="U67" t="s">
         <v>28</v>
@@ -4339,29 +4363,32 @@
       <c r="F68" t="s">
         <v>30</v>
       </c>
+      <c r="K68" t="s">
+        <v>71</v>
+      </c>
       <c r="N68" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="O68" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="P68">
         <v>100000</v>
       </c>
       <c r="Q68" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="R68" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="S68" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T68" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="U68" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="V68" s="1">
         <v>46229</v>
@@ -4384,25 +4411,25 @@
         <v>29</v>
       </c>
       <c r="N69" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="O69" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="P69">
         <v>80000</v>
       </c>
       <c r="Q69" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R69" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="S69" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="T69" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="U69" t="s">
         <v>28</v>
@@ -4428,28 +4455,28 @@
         <v>29</v>
       </c>
       <c r="N70" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="O70" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="P70">
         <v>835000</v>
       </c>
       <c r="Q70" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R70" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="S70" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="T70" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="U70" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="V70" s="1">
         <v>46291</v>
@@ -4472,28 +4499,28 @@
         <v>29</v>
       </c>
       <c r="N71" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="O71" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="P71">
         <v>165000</v>
       </c>
       <c r="Q71" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R71" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="S71" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="T71" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="U71" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="V71" s="1">
         <v>46168</v>
@@ -4516,28 +4543,28 @@
         <v>29</v>
       </c>
       <c r="N72" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="O72" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="P72">
         <v>1000000</v>
       </c>
       <c r="Q72" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R72" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="S72" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="T72" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="U72" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="V72" s="1">
         <v>46291</v>
@@ -4560,28 +4587,28 @@
         <v>29</v>
       </c>
       <c r="N73" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="O73" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="P73">
         <v>1000000</v>
       </c>
       <c r="Q73" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R73" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="S73" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="T73" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="U73" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="V73" s="1">
         <v>46291</v>
@@ -4604,28 +4631,28 @@
         <v>29</v>
       </c>
       <c r="N74" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="O74" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="P74">
         <v>100000</v>
       </c>
       <c r="Q74" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="R74" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="S74" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="T74" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="U74" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="V74" s="1">
         <v>46291</v>
@@ -4651,25 +4678,25 @@
         <v>30</v>
       </c>
       <c r="N75" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="O75" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="P75">
         <v>1000000</v>
       </c>
       <c r="Q75" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="R75" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="S75" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T75" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="U75" t="s">
         <v>28</v>
@@ -4701,28 +4728,28 @@
         <v>44</v>
       </c>
       <c r="N76" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O76" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="P76">
         <v>1704503</v>
       </c>
       <c r="Q76" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="R76" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="S76" t="s">
         <v>40</v>
       </c>
       <c r="T76" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="U76" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="V76" s="1">
         <v>46381</v>
@@ -4751,28 +4778,28 @@
         <v>44</v>
       </c>
       <c r="N77" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O77" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="P77">
         <v>1638125.5</v>
       </c>
       <c r="Q77" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="R77" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="S77" t="s">
         <v>40</v>
       </c>
       <c r="T77" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="U77" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="V77" s="1">
         <v>46381</v>
@@ -4801,25 +4828,25 @@
         <v>44</v>
       </c>
       <c r="N78" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="O78" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="P78">
         <v>3800000</v>
       </c>
       <c r="Q78" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="R78" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="S78" t="s">
         <v>40</v>
       </c>
       <c r="T78" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="U78" t="s">
         <v>28</v>
@@ -4851,25 +4878,25 @@
         <v>44</v>
       </c>
       <c r="N79" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="O79" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="P79">
         <v>3800000</v>
       </c>
       <c r="Q79" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="R79" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="S79" t="s">
         <v>40</v>
       </c>
       <c r="T79" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="U79" t="s">
         <v>28</v>
@@ -4898,28 +4925,28 @@
         <v>68</v>
       </c>
       <c r="K80" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="N80" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="O80" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="P80">
         <v>3800000</v>
       </c>
       <c r="Q80" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="R80" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="S80" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="T80" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="U80" t="s">
         <v>28</v>
@@ -4945,25 +4972,25 @@
         <v>28</v>
       </c>
       <c r="N81" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="O81" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="P81">
         <v>4394700</v>
       </c>
       <c r="Q81" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R81" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="S81" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="T81" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="U81" t="s">
         <v>28</v>
@@ -4992,31 +5019,31 @@
         <v>30</v>
       </c>
       <c r="K82" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="N82" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O82" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="P82">
         <v>528395.9300000001</v>
       </c>
       <c r="Q82" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="R82" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="S82" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="T82" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="U82" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="V82" s="1">
         <v>46382</v>
@@ -5039,25 +5066,25 @@
         <v>29</v>
       </c>
       <c r="N83" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="O83" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="P83">
         <v>1000000</v>
       </c>
       <c r="Q83" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="R83" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="S83" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="T83" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="U83" t="s">
         <v>28</v>
@@ -5083,25 +5110,25 @@
         <v>28</v>
       </c>
       <c r="N84" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="O84" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="P84">
         <v>4394700</v>
       </c>
       <c r="Q84" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R84" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="S84" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="T84" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="U84" t="s">
         <v>28</v>
@@ -5133,25 +5160,25 @@
         <v>44</v>
       </c>
       <c r="N85" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="O85" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="P85">
         <v>3306000</v>
       </c>
       <c r="Q85" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R85" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="S85" t="s">
         <v>40</v>
       </c>
       <c r="T85" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="U85" t="s">
         <v>28</v>
@@ -5180,25 +5207,25 @@
         <v>44</v>
       </c>
       <c r="N86" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="O86" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="P86">
         <v>3306000</v>
       </c>
       <c r="Q86" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R86" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="S86" t="s">
         <v>40</v>
       </c>
       <c r="T86" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="U86" t="s">
         <v>28</v>

</xml_diff>

<commit_message>
Atualização automática: mta (28/08/2026 18:22)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1117" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1130" uniqueCount="182">
   <si>
     <t>linha</t>
   </si>
@@ -88,18 +88,21 @@
     <t>MOD C-98</t>
   </si>
   <si>
+    <t>T-27</t>
+  </si>
+  <si>
     <t>Aprovado, aguardando atendimento</t>
   </si>
   <si>
+    <t>Sem informação</t>
+  </si>
+  <si>
     <t>Atendido</t>
   </si>
   <si>
     <t>Não aprovado</t>
   </si>
   <si>
-    <t>Sem informação</t>
-  </si>
-  <si>
     <t>SIM</t>
   </si>
   <si>
@@ -139,12 +142,12 @@
     <t>RAP</t>
   </si>
   <si>
+    <t>CANCELADO</t>
+  </si>
+  <si>
     <t>ATENDIDO</t>
   </si>
   <si>
-    <t>CANCELADO</t>
-  </si>
-  <si>
     <t>BLOQUEIO</t>
   </si>
   <si>
@@ -307,6 +310,9 @@
     <t>Exchange PT6A-114A</t>
   </si>
   <si>
+    <t>CNT 001/CABW-PAMASP/2025 - EXCHANGE - FLORIDA SUPPLY</t>
+  </si>
+  <si>
     <t>Atualização de GPS</t>
   </si>
   <si>
@@ -505,6 +511,9 @@
     <t>Material reparo PT6A-114A (4/4)</t>
   </si>
   <si>
+    <t>Pagar avaliação dos cores</t>
+  </si>
+  <si>
     <t>CABW</t>
   </si>
   <si>
@@ -545,6 +554,9 @@
   </si>
   <si>
     <t>PARCELA FIXA</t>
+  </si>
+  <si>
+    <t>CONTRATO</t>
   </si>
   <si>
     <t>Não</t>
@@ -883,7 +895,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V86"/>
+  <dimension ref="A1:V87"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
@@ -965,43 +977,43 @@
         <v>22</v>
       </c>
       <c r="D2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="K2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="L2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="N2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O2" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="P2">
         <v>135000</v>
       </c>
       <c r="Q2" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R2" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="S2" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T2" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U2" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="V2" s="1">
         <v>46229</v>
@@ -1018,37 +1030,37 @@
         <v>22</v>
       </c>
       <c r="D3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O3" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="P3">
         <v>400000</v>
       </c>
       <c r="Q3" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="R3" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="S3" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T3" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V3" s="1">
         <v>46291</v>
@@ -1065,37 +1077,37 @@
         <v>22</v>
       </c>
       <c r="D4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F4" t="s">
-        <v>30</v>
+        <v>31</v>
+      </c>
+      <c r="G4" t="s">
+        <v>42</v>
       </c>
       <c r="N4" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="O4" t="s">
-        <v>99</v>
-      </c>
-      <c r="P4">
-        <v>430000</v>
+        <v>101</v>
       </c>
       <c r="Q4" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R4" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="S4" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T4" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V4" s="1">
         <v>46321</v>
@@ -1112,37 +1124,37 @@
         <v>22</v>
       </c>
       <c r="D5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="O5" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="P5">
-        <v>425000</v>
+        <v>384180</v>
       </c>
       <c r="Q5" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R5" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="S5" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T5" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V5" s="1">
         <v>46321</v>
@@ -1159,40 +1171,40 @@
         <v>22</v>
       </c>
       <c r="D6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="L6" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="N6" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="O6" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="P6">
         <v>563000</v>
       </c>
       <c r="Q6" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R6" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="S6" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T6" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V6" s="1">
         <v>46291</v>
@@ -1209,46 +1221,46 @@
         <v>22</v>
       </c>
       <c r="D7" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G7" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H7" s="1">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="N7" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="O7" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="P7">
         <v>3799999.6</v>
       </c>
       <c r="Q7" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="R7" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="S7" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T7" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="U7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V7" s="1">
         <v>46138</v>
@@ -1265,37 +1277,37 @@
         <v>22</v>
       </c>
       <c r="D8" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E8" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N8" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="O8" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="P8">
         <v>430000</v>
       </c>
       <c r="Q8" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R8" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="S8" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T8" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U8" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V8" s="1">
         <v>46291</v>
@@ -1312,37 +1324,37 @@
         <v>22</v>
       </c>
       <c r="D9" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E9" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F9" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N9" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="O9" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="P9">
         <v>60000</v>
       </c>
       <c r="Q9" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R9" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="S9" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T9" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U9" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V9" s="1">
         <v>46291</v>
@@ -1359,37 +1371,37 @@
         <v>22</v>
       </c>
       <c r="D10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E10" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F10" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N10" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="O10" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="P10">
         <v>200000</v>
       </c>
       <c r="Q10" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R10" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="S10" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T10" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U10" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V10" s="1">
         <v>46291</v>
@@ -1406,37 +1418,37 @@
         <v>22</v>
       </c>
       <c r="D11" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E11" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F11" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N11" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="O11" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="P11">
         <v>320000</v>
       </c>
       <c r="Q11" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R11" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="S11" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T11" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U11" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V11" s="1">
         <v>46291</v>
@@ -1453,49 +1465,49 @@
         <v>22</v>
       </c>
       <c r="D12" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E12" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F12" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G12" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H12" s="1">
         <v>46079</v>
       </c>
       <c r="I12" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J12" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="N12" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O12" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="P12">
         <v>1187433.02</v>
       </c>
       <c r="Q12" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R12" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="S12" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T12" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U12" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="V12" s="1">
         <v>46079</v>
@@ -1512,40 +1524,40 @@
         <v>22</v>
       </c>
       <c r="D13" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E13" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F13" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="K13" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="N13" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O13" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="P13">
         <v>1000000</v>
       </c>
       <c r="Q13" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R13" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="S13" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T13" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U13" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="V13" s="1">
         <v>46352</v>
@@ -1562,40 +1574,40 @@
         <v>22</v>
       </c>
       <c r="D14" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E14" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F14" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="K14" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="N14" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O14" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="P14">
         <v>1000000</v>
       </c>
       <c r="Q14" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R14" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="S14" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T14" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U14" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="V14" s="1">
         <v>46352</v>
@@ -1612,40 +1624,40 @@
         <v>22</v>
       </c>
       <c r="D15" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E15" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F15" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="K15" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="N15" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O15" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="P15">
         <v>1000000</v>
       </c>
       <c r="Q15" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R15" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="S15" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T15" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U15" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="V15" s="1">
         <v>46352</v>
@@ -1662,40 +1674,40 @@
         <v>22</v>
       </c>
       <c r="D16" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E16" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F16" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="K16" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="N16" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="O16" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="P16">
         <v>100000</v>
       </c>
       <c r="Q16" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="R16" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="S16" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T16" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U16" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="V16" s="1">
         <v>46229</v>
@@ -1712,49 +1724,49 @@
         <v>22</v>
       </c>
       <c r="D17" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E17" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F17" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G17" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H17" s="1">
         <v>46098</v>
       </c>
       <c r="I17" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J17" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="N17" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="O17" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="P17">
         <v>1770880.5</v>
       </c>
       <c r="Q17" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="R17" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="S17" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T17" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="U17" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="V17" s="1">
         <v>46107</v>
@@ -1771,46 +1783,46 @@
         <v>22</v>
       </c>
       <c r="D18" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E18" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F18" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G18" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H18" s="1">
         <v>46076</v>
       </c>
       <c r="I18" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="N18" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="O18" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="P18">
         <v>350000</v>
       </c>
       <c r="Q18" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="R18" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="S18" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T18" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="U18" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V18" s="1">
         <v>46079</v>
@@ -1827,46 +1839,46 @@
         <v>22</v>
       </c>
       <c r="D19" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E19" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F19" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G19" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H19" s="1">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="N19" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="O19" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="P19">
         <v>350000</v>
       </c>
       <c r="Q19" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="R19" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="S19" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T19" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="U19" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V19" s="1">
         <v>46079</v>
@@ -1883,37 +1895,37 @@
         <v>22</v>
       </c>
       <c r="D20" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E20" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F20" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N20" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="O20" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="P20">
         <v>1000000</v>
       </c>
       <c r="Q20" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="R20" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="S20" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T20" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="U20" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V20" s="1">
         <v>46321</v>
@@ -1930,37 +1942,37 @@
         <v>22</v>
       </c>
       <c r="D21" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E21" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F21" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N21" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O21" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="P21">
         <v>400000</v>
       </c>
       <c r="Q21" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="R21" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="S21" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T21" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U21" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V21" s="1">
         <v>46321</v>
@@ -1977,37 +1989,37 @@
         <v>22</v>
       </c>
       <c r="D22" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E22" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F22" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N22" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="O22" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="P22">
         <v>120000</v>
       </c>
       <c r="Q22" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R22" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="S22" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T22" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U22" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V22" s="1">
         <v>46321</v>
@@ -2024,37 +2036,37 @@
         <v>22</v>
       </c>
       <c r="D23" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E23" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F23" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N23" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="O23" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="P23">
         <v>80000</v>
       </c>
       <c r="Q23" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R23" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="S23" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T23" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U23" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V23" s="1">
         <v>46321</v>
@@ -2071,49 +2083,49 @@
         <v>22</v>
       </c>
       <c r="D24" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E24" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F24" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G24" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H24" s="1">
         <v>46119</v>
       </c>
       <c r="I24" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J24" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="N24" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="O24" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="P24">
         <v>1704503</v>
       </c>
       <c r="Q24" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="R24" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="S24" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T24" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="U24" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="V24" s="1">
         <v>46138</v>
@@ -2130,46 +2142,46 @@
         <v>22</v>
       </c>
       <c r="D25" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E25" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F25" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G25" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H25" s="1">
         <v>46121</v>
       </c>
       <c r="I25" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="N25" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="O25" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="P25">
         <v>3799000</v>
       </c>
       <c r="Q25" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="R25" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="S25" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T25" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="U25" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V25" s="1">
         <v>46138</v>
@@ -2186,46 +2198,46 @@
         <v>22</v>
       </c>
       <c r="D26" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E26" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F26" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G26" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H26" s="1">
         <v>46076</v>
       </c>
       <c r="I26" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="N26" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="O26" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="P26">
         <v>1000</v>
       </c>
       <c r="Q26" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="R26" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="S26" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T26" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="U26" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V26" s="1">
         <v>46079</v>
@@ -2242,40 +2254,40 @@
         <v>22</v>
       </c>
       <c r="D27" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E27" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F27" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="K27" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="N27" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="O27" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="P27">
         <v>100000</v>
       </c>
       <c r="Q27" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="R27" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="S27" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T27" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U27" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="V27" s="1">
         <v>46291</v>
@@ -2292,49 +2304,49 @@
         <v>22</v>
       </c>
       <c r="D28" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E28" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F28" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G28" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H28" s="1">
         <v>46199</v>
       </c>
       <c r="I28" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J28" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="N28" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="O28" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="P28">
         <v>150000</v>
       </c>
       <c r="Q28" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="R28" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="S28" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T28" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="U28" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="V28" s="1">
         <v>46199</v>
@@ -2351,49 +2363,49 @@
         <v>22</v>
       </c>
       <c r="D29" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E29" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F29" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G29" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H29" s="1">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J29" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="N29" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="O29" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="P29">
         <v>150000</v>
       </c>
       <c r="Q29" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="R29" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="S29" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T29" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="U29" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="V29" s="1">
         <v>46199</v>
@@ -2410,49 +2422,49 @@
         <v>22</v>
       </c>
       <c r="D30" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E30" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F30" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G30" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H30" s="1">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="J30" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="N30" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="O30" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="P30">
         <v>18462.36</v>
       </c>
       <c r="Q30" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="R30" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="S30" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T30" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="U30" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="V30" s="1">
         <v>46199</v>
@@ -2469,49 +2481,49 @@
         <v>22</v>
       </c>
       <c r="D31" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E31" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F31" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G31" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H31" s="1">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J31" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="N31" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="O31" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="P31">
         <v>324166.14</v>
       </c>
       <c r="Q31" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="R31" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="S31" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T31" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="U31" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="V31" s="1">
         <v>46199</v>
@@ -2528,40 +2540,40 @@
         <v>22</v>
       </c>
       <c r="D32" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E32" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F32" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="K32" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="N32" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="O32" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="P32">
         <v>30000</v>
       </c>
       <c r="Q32" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="R32" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="S32" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T32" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="U32" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="V32" s="1">
         <v>46291</v>
@@ -2578,49 +2590,49 @@
         <v>22</v>
       </c>
       <c r="D33" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E33" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F33" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G33" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H33" s="1">
         <v>46191</v>
       </c>
       <c r="I33" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J33" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="N33" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="O33" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="P33">
         <v>1496713.48</v>
       </c>
       <c r="Q33" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="R33" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="S33" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T33" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="U33" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="V33" s="1">
         <v>46199</v>
@@ -2637,46 +2649,46 @@
         <v>22</v>
       </c>
       <c r="D34" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E34" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F34" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G34" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H34" s="1">
         <v>46119</v>
       </c>
       <c r="I34" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="N34" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="O34" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="P34">
         <v>207789.52</v>
       </c>
       <c r="Q34" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="R34" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="S34" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T34" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="U34" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="V34" s="1">
         <v>46138</v>
@@ -2693,46 +2705,46 @@
         <v>22</v>
       </c>
       <c r="D35" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E35" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F35" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G35" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H35" s="1">
         <v>46213</v>
       </c>
       <c r="I35" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="N35" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="O35" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="P35">
         <v>962290.8</v>
       </c>
       <c r="Q35" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="R35" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="S35" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T35" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="U35" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V35" s="1">
         <v>46229</v>
@@ -2749,46 +2761,46 @@
         <v>22</v>
       </c>
       <c r="D36" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E36" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F36" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G36" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H36" s="1">
         <v>46175</v>
       </c>
       <c r="I36" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="N36" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="O36" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="P36">
         <v>798776.97</v>
       </c>
       <c r="Q36" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="R36" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="S36" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T36" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="U36" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V36" s="1">
         <v>46199</v>
@@ -2805,46 +2817,46 @@
         <v>22</v>
       </c>
       <c r="D37" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E37" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F37" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G37" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H37" s="1">
         <v>46213</v>
       </c>
       <c r="I37" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="N37" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="O37" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="P37">
         <v>1530656.62</v>
       </c>
       <c r="Q37" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="R37" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="S37" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T37" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="U37" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V37" s="1">
         <v>46229</v>
@@ -2861,46 +2873,46 @@
         <v>22</v>
       </c>
       <c r="D38" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E38" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F38" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G38" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H38" s="1">
         <v>46199</v>
       </c>
       <c r="I38" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="N38" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="O38" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="P38">
         <v>72958.08</v>
       </c>
       <c r="Q38" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="R38" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="S38" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T38" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="U38" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V38" s="1">
         <v>46199</v>
@@ -2917,46 +2929,46 @@
         <v>22</v>
       </c>
       <c r="D39" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E39" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F39" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G39" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H39" s="1">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="N39" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="O39" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="P39">
         <v>8916</v>
       </c>
       <c r="Q39" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="R39" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="S39" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T39" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="U39" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V39" s="1">
         <v>46199</v>
@@ -2973,46 +2985,46 @@
         <v>22</v>
       </c>
       <c r="D40" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E40" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F40" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G40" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H40" s="1">
         <v>46204</v>
       </c>
       <c r="I40" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="N40" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="O40" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="P40">
         <v>425178.5</v>
       </c>
       <c r="Q40" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="R40" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="S40" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T40" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="U40" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V40" s="1">
         <v>46229</v>
@@ -3029,46 +3041,46 @@
         <v>22</v>
       </c>
       <c r="D41" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E41" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F41" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G41" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H41" s="1">
         <v>46244</v>
       </c>
       <c r="I41" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="N41" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="O41" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="P41">
         <v>1223.03</v>
       </c>
       <c r="Q41" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="R41" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="S41" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T41" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="U41" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V41" s="1">
         <v>46199</v>
@@ -3085,34 +3097,34 @@
         <v>22</v>
       </c>
       <c r="D42" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E42" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G42" t="s">
         <v>42</v>
       </c>
       <c r="N42" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="O42" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="Q42" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="R42" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="S42" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="T42" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="U42" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V42" s="1">
         <v>46260</v>
@@ -3129,46 +3141,46 @@
         <v>22</v>
       </c>
       <c r="D43" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E43" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F43" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G43" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H43" s="1">
         <v>46191</v>
       </c>
       <c r="I43" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="N43" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="O43" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="P43">
         <v>400000</v>
       </c>
       <c r="Q43" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="R43" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="S43" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T43" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="U43" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V43" s="1">
         <v>46199</v>
@@ -3185,46 +3197,46 @@
         <v>22</v>
       </c>
       <c r="D44" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E44" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F44" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G44" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H44" s="1">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="N44" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="O44" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="P44">
         <v>400000</v>
       </c>
       <c r="Q44" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="R44" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="S44" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T44" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="U44" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V44" s="1">
         <v>46199</v>
@@ -3241,49 +3253,49 @@
         <v>22</v>
       </c>
       <c r="D45" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E45" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F45" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G45" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H45" s="1">
         <v>46213</v>
       </c>
       <c r="I45" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J45" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="N45" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="O45" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="P45">
         <v>173846.38</v>
       </c>
       <c r="Q45" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="R45" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="S45" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T45" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="U45" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="V45" s="1">
         <v>46229</v>
@@ -3300,46 +3312,46 @@
         <v>22</v>
       </c>
       <c r="D46" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E46" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F46" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G46" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H46" s="1">
         <v>46210</v>
       </c>
       <c r="I46" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="N46" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="O46" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="P46">
         <v>1530656.62</v>
       </c>
       <c r="Q46" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="R46" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="S46" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T46" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="U46" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="V46" s="1">
         <v>46229</v>
@@ -3356,37 +3368,37 @@
         <v>22</v>
       </c>
       <c r="D47" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E47" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F47" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N47" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="O47" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="P47">
         <v>1000000</v>
       </c>
       <c r="Q47" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="R47" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="S47" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T47" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="U47" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V47" s="1">
         <v>46321</v>
@@ -3403,40 +3415,40 @@
         <v>22</v>
       </c>
       <c r="D48" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E48" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F48" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="K48" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="N48" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O48" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="P48">
         <v>958040</v>
       </c>
       <c r="Q48" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R48" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="S48" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T48" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U48" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="V48" s="1">
         <v>46291</v>
@@ -3453,49 +3465,49 @@
         <v>22</v>
       </c>
       <c r="D49" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E49" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F49" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G49" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H49" s="1">
         <v>46176</v>
       </c>
       <c r="I49" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="J49" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="N49" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O49" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="P49">
         <v>41730.64</v>
       </c>
       <c r="Q49" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R49" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="S49" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T49" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U49" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="V49" s="1">
         <v>46199</v>
@@ -3512,43 +3524,43 @@
         <v>22</v>
       </c>
       <c r="D50" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E50" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F50" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="J50" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="K50" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="N50" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="O50" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="P50">
         <v>1468159.32</v>
       </c>
       <c r="Q50" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="R50" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="S50" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T50" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="U50" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="V50" s="1">
         <v>46260</v>
@@ -3565,43 +3577,43 @@
         <v>22</v>
       </c>
       <c r="D51" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E51" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F51" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="J51" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="K51" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="N51" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="O51" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="P51">
         <v>1704503</v>
       </c>
       <c r="Q51" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="R51" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="S51" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T51" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="U51" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="V51" s="1">
         <v>46291</v>
@@ -3618,40 +3630,40 @@
         <v>22</v>
       </c>
       <c r="D52" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E52" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F52" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="K52" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="N52" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="O52" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="P52">
         <v>1704503</v>
       </c>
       <c r="Q52" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="R52" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="S52" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T52" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="U52" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="V52" s="1">
         <v>46321</v>
@@ -3668,46 +3680,46 @@
         <v>22</v>
       </c>
       <c r="D53" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E53" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F53" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G53" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H53" s="1">
         <v>46227</v>
       </c>
       <c r="I53" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="N53" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="O53" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="P53">
         <v>236343.68</v>
       </c>
       <c r="Q53" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="R53" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="S53" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T53" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="U53" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="V53" s="1">
         <v>46229</v>
@@ -3724,40 +3736,40 @@
         <v>22</v>
       </c>
       <c r="D54" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E54" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F54" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="K54" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="N54" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="O54" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="P54">
         <v>1295422.28</v>
       </c>
       <c r="Q54" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="R54" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="S54" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T54" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="U54" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="V54" s="1">
         <v>46352</v>
@@ -3774,40 +3786,40 @@
         <v>22</v>
       </c>
       <c r="D55" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E55" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F55" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="K55" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="N55" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="O55" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="P55">
         <v>500000</v>
       </c>
       <c r="Q55" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="R55" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="S55" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="T55" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="U55" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="V55" s="1">
         <v>46321</v>
@@ -3824,40 +3836,40 @@
         <v>22</v>
       </c>
       <c r="D56" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E56" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F56" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G56" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="N56" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="O56" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="P56">
         <v>5000000</v>
       </c>
       <c r="Q56" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="R56" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="S56" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="T56" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="U56" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="V56" s="1">
         <v>46321</v>
@@ -3874,34 +3886,34 @@
         <v>22</v>
       </c>
       <c r="D57" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E57" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G57" t="s">
         <v>42</v>
       </c>
       <c r="N57" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="O57" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="Q57" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="R57" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="S57" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="T57" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="U57" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="V57" s="1">
         <v>46049</v>
@@ -3918,34 +3930,34 @@
         <v>22</v>
       </c>
       <c r="D58" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E58" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G58" t="s">
         <v>42</v>
       </c>
       <c r="N58" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="O58" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="Q58" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="R58" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="S58" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="T58" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="U58" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
     </row>
     <row r="59" spans="1:22">
@@ -3959,34 +3971,34 @@
         <v>22</v>
       </c>
       <c r="D59" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E59" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G59" t="s">
         <v>42</v>
       </c>
       <c r="N59" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="O59" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="Q59" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="R59" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="S59" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="T59" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="U59" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
     </row>
     <row r="60" spans="1:22">
@@ -4000,34 +4012,34 @@
         <v>22</v>
       </c>
       <c r="D60" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E60" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N60" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="O60" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="P60">
         <v>9389.959999999999</v>
       </c>
       <c r="Q60" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R60" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="S60" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="T60" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U60" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="V60" s="1">
         <v>46107</v>
@@ -4044,34 +4056,34 @@
         <v>22</v>
       </c>
       <c r="D61" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E61" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N61" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="O61" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="P61">
         <v>7204.82</v>
       </c>
       <c r="Q61" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R61" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="S61" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="T61" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U61" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="V61" s="1">
         <v>46107</v>
@@ -4088,34 +4100,34 @@
         <v>22</v>
       </c>
       <c r="D62" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E62" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N62" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="O62" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="P62">
         <v>4227.84</v>
       </c>
       <c r="Q62" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R62" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="S62" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="T62" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U62" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="V62" s="1">
         <v>46107</v>
@@ -4132,34 +4144,34 @@
         <v>22</v>
       </c>
       <c r="D63" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E63" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N63" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="O63" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="P63">
         <v>4064.54</v>
       </c>
       <c r="Q63" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="R63" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="S63" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="T63" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U63" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="V63" s="1">
         <v>46107</v>
@@ -4176,34 +4188,34 @@
         <v>22</v>
       </c>
       <c r="D64" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E64" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N64" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="O64" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="P64">
         <v>3662.66</v>
       </c>
       <c r="Q64" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R64" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="S64" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="T64" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U64" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="V64" s="1">
         <v>46107</v>
@@ -4220,34 +4232,34 @@
         <v>22</v>
       </c>
       <c r="D65" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E65" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N65" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="O65" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="P65">
         <v>1163.64</v>
       </c>
       <c r="Q65" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="R65" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="S65" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="T65" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U65" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="V65" s="1">
         <v>46107</v>
@@ -4264,34 +4276,34 @@
         <v>22</v>
       </c>
       <c r="D66" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E66" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N66" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="O66" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="P66">
         <v>120000</v>
       </c>
       <c r="Q66" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R66" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="S66" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="T66" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U66" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V66" s="1">
         <v>46168</v>
@@ -4308,37 +4320,37 @@
         <v>22</v>
       </c>
       <c r="D67" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E67" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F67" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N67" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O67" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="P67">
         <v>400000</v>
       </c>
       <c r="Q67" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="R67" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="S67" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T67" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U67" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V67" s="1">
         <v>46291</v>
@@ -4355,40 +4367,40 @@
         <v>22</v>
       </c>
       <c r="D68" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E68" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F68" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="K68" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="N68" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="O68" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="P68">
         <v>100000</v>
       </c>
       <c r="Q68" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="R68" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="S68" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T68" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U68" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="V68" s="1">
         <v>46229</v>
@@ -4405,34 +4417,34 @@
         <v>22</v>
       </c>
       <c r="D69" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E69" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N69" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="O69" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="P69">
         <v>80000</v>
       </c>
       <c r="Q69" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R69" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="S69" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="T69" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U69" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V69" s="1">
         <v>46260</v>
@@ -4449,34 +4461,34 @@
         <v>22</v>
       </c>
       <c r="D70" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E70" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N70" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O70" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="P70">
         <v>835000</v>
       </c>
       <c r="Q70" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R70" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="S70" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="T70" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U70" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="V70" s="1">
         <v>46291</v>
@@ -4493,34 +4505,34 @@
         <v>22</v>
       </c>
       <c r="D71" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E71" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N71" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O71" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="P71">
         <v>165000</v>
       </c>
       <c r="Q71" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R71" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="S71" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="T71" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U71" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="V71" s="1">
         <v>46168</v>
@@ -4537,34 +4549,34 @@
         <v>22</v>
       </c>
       <c r="D72" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E72" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N72" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O72" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="P72">
         <v>1000000</v>
       </c>
       <c r="Q72" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R72" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="S72" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="T72" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U72" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="V72" s="1">
         <v>46291</v>
@@ -4581,34 +4593,34 @@
         <v>22</v>
       </c>
       <c r="D73" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E73" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N73" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O73" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="P73">
         <v>1000000</v>
       </c>
       <c r="Q73" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R73" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="S73" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="T73" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U73" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="V73" s="1">
         <v>46291</v>
@@ -4625,34 +4637,34 @@
         <v>22</v>
       </c>
       <c r="D74" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E74" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N74" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="O74" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="P74">
         <v>100000</v>
       </c>
       <c r="Q74" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="R74" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="S74" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="T74" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U74" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="V74" s="1">
         <v>46291</v>
@@ -4669,37 +4681,37 @@
         <v>22</v>
       </c>
       <c r="D75" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E75" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F75" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N75" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="O75" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="P75">
         <v>1000000</v>
       </c>
       <c r="Q75" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="R75" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="S75" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T75" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="U75" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V75" s="1">
         <v>46321</v>
@@ -4716,40 +4728,40 @@
         <v>22</v>
       </c>
       <c r="D76" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E76" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F76" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G76" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="N76" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="O76" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="P76">
         <v>1704503</v>
       </c>
       <c r="Q76" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="R76" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="S76" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="T76" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="U76" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="V76" s="1">
         <v>46381</v>
@@ -4766,40 +4778,40 @@
         <v>22</v>
       </c>
       <c r="D77" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E77" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F77" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G77" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="N77" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="O77" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="P77">
         <v>1638125.5</v>
       </c>
       <c r="Q77" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="R77" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="S77" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="T77" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="U77" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="V77" s="1">
         <v>46381</v>
@@ -4816,40 +4828,40 @@
         <v>22</v>
       </c>
       <c r="D78" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E78" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F78" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G78" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="N78" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="O78" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="P78">
         <v>3800000</v>
       </c>
       <c r="Q78" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="R78" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="S78" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="T78" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="U78" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V78" s="1">
         <v>46381</v>
@@ -4866,40 +4878,40 @@
         <v>22</v>
       </c>
       <c r="D79" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E79" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F79" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G79" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="N79" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="O79" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="P79">
         <v>3800000</v>
       </c>
       <c r="Q79" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="R79" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="S79" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="T79" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="U79" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V79" s="1">
         <v>46381</v>
@@ -4916,40 +4928,40 @@
         <v>22</v>
       </c>
       <c r="D80" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E80" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="J80" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="K80" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="N80" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="O80" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="P80">
         <v>3800000</v>
       </c>
       <c r="Q80" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="R80" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="S80" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="T80" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="U80" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V80" s="1">
         <v>46382</v>
@@ -4966,34 +4978,34 @@
         <v>22</v>
       </c>
       <c r="D81" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E81" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N81" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="O81" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="P81">
         <v>4394700</v>
       </c>
       <c r="Q81" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R81" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="S81" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="T81" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="U81" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V81" s="1">
         <v>46382</v>
@@ -5010,40 +5022,40 @@
         <v>22</v>
       </c>
       <c r="D82" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E82" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F82" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="K82" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="N82" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="O82" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="P82">
         <v>528395.9300000001</v>
       </c>
       <c r="Q82" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="R82" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="S82" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="T82" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="U82" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="V82" s="1">
         <v>46382</v>
@@ -5060,34 +5072,34 @@
         <v>22</v>
       </c>
       <c r="D83" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E83" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N83" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="O83" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="P83">
         <v>1000000</v>
       </c>
       <c r="Q83" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="R83" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="S83" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="T83" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="U83" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V83" s="1">
         <v>46321</v>
@@ -5104,34 +5116,34 @@
         <v>22</v>
       </c>
       <c r="D84" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E84" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N84" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="O84" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="P84">
         <v>4394700</v>
       </c>
       <c r="Q84" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R84" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="S84" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="T84" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="U84" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V84" s="1">
         <v>46382</v>
@@ -5148,40 +5160,40 @@
         <v>22</v>
       </c>
       <c r="D85" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E85" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F85" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G85" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="N85" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="O85" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="P85">
         <v>3306000</v>
       </c>
       <c r="Q85" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R85" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="S85" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="T85" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="U85" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="86" spans="1:22">
@@ -5195,40 +5207,87 @@
         <v>22</v>
       </c>
       <c r="D86" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E86" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F86" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G86" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="N86" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="O86" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="P86">
         <v>3306000</v>
       </c>
       <c r="Q86" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="R86" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="S86" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="T86" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="U86" t="s">
-        <v>28</v>
+        <v>29</v>
+      </c>
+    </row>
+    <row r="87" spans="1:22">
+      <c r="A87">
+        <v>64840</v>
+      </c>
+      <c r="B87" t="s">
+        <v>24</v>
+      </c>
+      <c r="C87" t="s">
+        <v>22</v>
+      </c>
+      <c r="D87" t="s">
+        <v>25</v>
+      </c>
+      <c r="E87" t="s">
+        <v>29</v>
+      </c>
+      <c r="F87" t="s">
+        <v>31</v>
+      </c>
+      <c r="N87" t="s">
+        <v>98</v>
+      </c>
+      <c r="O87" t="s">
+        <v>165</v>
+      </c>
+      <c r="P87">
+        <v>470820</v>
+      </c>
+      <c r="Q87" t="s">
+        <v>166</v>
+      </c>
+      <c r="R87" t="s">
+        <v>170</v>
+      </c>
+      <c r="S87" t="s">
+        <v>172</v>
+      </c>
+      <c r="T87" t="s">
+        <v>180</v>
+      </c>
+      <c r="U87" t="s">
+        <v>29</v>
+      </c>
+      <c r="V87" s="1">
+        <v>46291</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: mta (01/09/2026 11:15)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -569,8 +569,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -586,7 +594,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -594,12 +602,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -899,70 +925,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1015,7 +1041,7 @@
       <c r="U2" t="s">
         <v>181</v>
       </c>
-      <c r="V2" s="1">
+      <c r="V2" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -1062,7 +1088,7 @@
       <c r="U3" t="s">
         <v>29</v>
       </c>
-      <c r="V3" s="1">
+      <c r="V3" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1109,7 +1135,7 @@
       <c r="U4" t="s">
         <v>29</v>
       </c>
-      <c r="V4" s="1">
+      <c r="V4" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1156,7 +1182,7 @@
       <c r="U5" t="s">
         <v>29</v>
       </c>
-      <c r="V5" s="1">
+      <c r="V5" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1206,7 +1232,7 @@
       <c r="U6" t="s">
         <v>29</v>
       </c>
-      <c r="V6" s="1">
+      <c r="V6" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1232,7 +1258,7 @@
       <c r="G7" t="s">
         <v>43</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1262,7 +1288,7 @@
       <c r="U7" t="s">
         <v>29</v>
       </c>
-      <c r="V7" s="1">
+      <c r="V7" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -1309,7 +1335,7 @@
       <c r="U8" t="s">
         <v>29</v>
       </c>
-      <c r="V8" s="1">
+      <c r="V8" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1356,7 +1382,7 @@
       <c r="U9" t="s">
         <v>29</v>
       </c>
-      <c r="V9" s="1">
+      <c r="V9" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1403,7 +1429,7 @@
       <c r="U10" t="s">
         <v>29</v>
       </c>
-      <c r="V10" s="1">
+      <c r="V10" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1450,7 +1476,7 @@
       <c r="U11" t="s">
         <v>29</v>
       </c>
-      <c r="V11" s="1">
+      <c r="V11" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1476,7 +1502,7 @@
       <c r="G12" t="s">
         <v>43</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46079</v>
       </c>
       <c r="I12" t="s">
@@ -1509,7 +1535,7 @@
       <c r="U12" t="s">
         <v>181</v>
       </c>
-      <c r="V12" s="1">
+      <c r="V12" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1559,7 +1585,7 @@
       <c r="U13" t="s">
         <v>181</v>
       </c>
-      <c r="V13" s="1">
+      <c r="V13" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1609,7 +1635,7 @@
       <c r="U14" t="s">
         <v>181</v>
       </c>
-      <c r="V14" s="1">
+      <c r="V14" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1659,7 +1685,7 @@
       <c r="U15" t="s">
         <v>181</v>
       </c>
-      <c r="V15" s="1">
+      <c r="V15" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1709,7 +1735,7 @@
       <c r="U16" t="s">
         <v>181</v>
       </c>
-      <c r="V16" s="1">
+      <c r="V16" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -1735,7 +1761,7 @@
       <c r="G17" t="s">
         <v>43</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46098</v>
       </c>
       <c r="I17" t="s">
@@ -1768,7 +1794,7 @@
       <c r="U17" t="s">
         <v>181</v>
       </c>
-      <c r="V17" s="1">
+      <c r="V17" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -1794,7 +1820,7 @@
       <c r="G18" t="s">
         <v>43</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46076</v>
       </c>
       <c r="I18" t="s">
@@ -1824,7 +1850,7 @@
       <c r="U18" t="s">
         <v>29</v>
       </c>
-      <c r="V18" s="1">
+      <c r="V18" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1850,7 +1876,7 @@
       <c r="G19" t="s">
         <v>43</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1880,7 +1906,7 @@
       <c r="U19" t="s">
         <v>29</v>
       </c>
-      <c r="V19" s="1">
+      <c r="V19" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1927,7 +1953,7 @@
       <c r="U20" t="s">
         <v>29</v>
       </c>
-      <c r="V20" s="1">
+      <c r="V20" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1974,7 +2000,7 @@
       <c r="U21" t="s">
         <v>29</v>
       </c>
-      <c r="V21" s="1">
+      <c r="V21" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2021,7 +2047,7 @@
       <c r="U22" t="s">
         <v>29</v>
       </c>
-      <c r="V22" s="1">
+      <c r="V22" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2068,7 +2094,7 @@
       <c r="U23" t="s">
         <v>29</v>
       </c>
-      <c r="V23" s="1">
+      <c r="V23" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2094,7 +2120,7 @@
       <c r="G24" t="s">
         <v>43</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>46119</v>
       </c>
       <c r="I24" t="s">
@@ -2127,7 +2153,7 @@
       <c r="U24" t="s">
         <v>181</v>
       </c>
-      <c r="V24" s="1">
+      <c r="V24" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2153,7 +2179,7 @@
       <c r="G25" t="s">
         <v>43</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>46121</v>
       </c>
       <c r="I25" t="s">
@@ -2183,7 +2209,7 @@
       <c r="U25" t="s">
         <v>29</v>
       </c>
-      <c r="V25" s="1">
+      <c r="V25" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2209,7 +2235,7 @@
       <c r="G26" t="s">
         <v>43</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>46076</v>
       </c>
       <c r="I26" t="s">
@@ -2239,7 +2265,7 @@
       <c r="U26" t="s">
         <v>29</v>
       </c>
-      <c r="V26" s="1">
+      <c r="V26" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -2289,7 +2315,7 @@
       <c r="U27" t="s">
         <v>181</v>
       </c>
-      <c r="V27" s="1">
+      <c r="V27" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -2315,7 +2341,7 @@
       <c r="G28" t="s">
         <v>43</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>46199</v>
       </c>
       <c r="I28" t="s">
@@ -2348,7 +2374,7 @@
       <c r="U28" t="s">
         <v>181</v>
       </c>
-      <c r="V28" s="1">
+      <c r="V28" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2374,7 +2400,7 @@
       <c r="G29" t="s">
         <v>43</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2407,7 +2433,7 @@
       <c r="U29" t="s">
         <v>181</v>
       </c>
-      <c r="V29" s="1">
+      <c r="V29" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2433,7 +2459,7 @@
       <c r="G30" t="s">
         <v>43</v>
       </c>
-      <c r="H30" s="1">
+      <c r="H30" s="2">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2466,7 +2492,7 @@
       <c r="U30" t="s">
         <v>181</v>
       </c>
-      <c r="V30" s="1">
+      <c r="V30" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2492,7 +2518,7 @@
       <c r="G31" t="s">
         <v>43</v>
       </c>
-      <c r="H31" s="1">
+      <c r="H31" s="2">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2525,7 +2551,7 @@
       <c r="U31" t="s">
         <v>181</v>
       </c>
-      <c r="V31" s="1">
+      <c r="V31" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2575,7 +2601,7 @@
       <c r="U32" t="s">
         <v>181</v>
       </c>
-      <c r="V32" s="1">
+      <c r="V32" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -2601,7 +2627,7 @@
       <c r="G33" t="s">
         <v>43</v>
       </c>
-      <c r="H33" s="1">
+      <c r="H33" s="2">
         <v>46191</v>
       </c>
       <c r="I33" t="s">
@@ -2634,7 +2660,7 @@
       <c r="U33" t="s">
         <v>181</v>
       </c>
-      <c r="V33" s="1">
+      <c r="V33" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2660,7 +2686,7 @@
       <c r="G34" t="s">
         <v>43</v>
       </c>
-      <c r="H34" s="1">
+      <c r="H34" s="2">
         <v>46119</v>
       </c>
       <c r="I34" t="s">
@@ -2690,7 +2716,7 @@
       <c r="U34" t="s">
         <v>181</v>
       </c>
-      <c r="V34" s="1">
+      <c r="V34" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2716,7 +2742,7 @@
       <c r="G35" t="s">
         <v>43</v>
       </c>
-      <c r="H35" s="1">
+      <c r="H35" s="2">
         <v>46213</v>
       </c>
       <c r="I35" t="s">
@@ -2746,7 +2772,7 @@
       <c r="U35" t="s">
         <v>29</v>
       </c>
-      <c r="V35" s="1">
+      <c r="V35" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -2772,7 +2798,7 @@
       <c r="G36" t="s">
         <v>43</v>
       </c>
-      <c r="H36" s="1">
+      <c r="H36" s="2">
         <v>46175</v>
       </c>
       <c r="I36" t="s">
@@ -2802,7 +2828,7 @@
       <c r="U36" t="s">
         <v>29</v>
       </c>
-      <c r="V36" s="1">
+      <c r="V36" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2828,7 +2854,7 @@
       <c r="G37" t="s">
         <v>43</v>
       </c>
-      <c r="H37" s="1">
+      <c r="H37" s="2">
         <v>46213</v>
       </c>
       <c r="I37" t="s">
@@ -2858,7 +2884,7 @@
       <c r="U37" t="s">
         <v>29</v>
       </c>
-      <c r="V37" s="1">
+      <c r="V37" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -2884,7 +2910,7 @@
       <c r="G38" t="s">
         <v>43</v>
       </c>
-      <c r="H38" s="1">
+      <c r="H38" s="2">
         <v>46199</v>
       </c>
       <c r="I38" t="s">
@@ -2914,7 +2940,7 @@
       <c r="U38" t="s">
         <v>29</v>
       </c>
-      <c r="V38" s="1">
+      <c r="V38" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2940,7 +2966,7 @@
       <c r="G39" t="s">
         <v>43</v>
       </c>
-      <c r="H39" s="1">
+      <c r="H39" s="2">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -2970,7 +2996,7 @@
       <c r="U39" t="s">
         <v>29</v>
       </c>
-      <c r="V39" s="1">
+      <c r="V39" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2996,7 +3022,7 @@
       <c r="G40" t="s">
         <v>43</v>
       </c>
-      <c r="H40" s="1">
+      <c r="H40" s="2">
         <v>46204</v>
       </c>
       <c r="I40" t="s">
@@ -3026,7 +3052,7 @@
       <c r="U40" t="s">
         <v>29</v>
       </c>
-      <c r="V40" s="1">
+      <c r="V40" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3052,7 +3078,7 @@
       <c r="G41" t="s">
         <v>43</v>
       </c>
-      <c r="H41" s="1">
+      <c r="H41" s="2">
         <v>46244</v>
       </c>
       <c r="I41" t="s">
@@ -3082,7 +3108,7 @@
       <c r="U41" t="s">
         <v>29</v>
       </c>
-      <c r="V41" s="1">
+      <c r="V41" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3126,7 +3152,7 @@
       <c r="U42" t="s">
         <v>29</v>
       </c>
-      <c r="V42" s="1">
+      <c r="V42" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3152,7 +3178,7 @@
       <c r="G43" t="s">
         <v>43</v>
       </c>
-      <c r="H43" s="1">
+      <c r="H43" s="2">
         <v>46191</v>
       </c>
       <c r="I43" t="s">
@@ -3182,7 +3208,7 @@
       <c r="U43" t="s">
         <v>29</v>
       </c>
-      <c r="V43" s="1">
+      <c r="V43" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3208,7 +3234,7 @@
       <c r="G44" t="s">
         <v>43</v>
       </c>
-      <c r="H44" s="1">
+      <c r="H44" s="2">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
@@ -3238,7 +3264,7 @@
       <c r="U44" t="s">
         <v>29</v>
       </c>
-      <c r="V44" s="1">
+      <c r="V44" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3264,7 +3290,7 @@
       <c r="G45" t="s">
         <v>43</v>
       </c>
-      <c r="H45" s="1">
+      <c r="H45" s="2">
         <v>46213</v>
       </c>
       <c r="I45" t="s">
@@ -3297,7 +3323,7 @@
       <c r="U45" t="s">
         <v>181</v>
       </c>
-      <c r="V45" s="1">
+      <c r="V45" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3323,7 +3349,7 @@
       <c r="G46" t="s">
         <v>43</v>
       </c>
-      <c r="H46" s="1">
+      <c r="H46" s="2">
         <v>46210</v>
       </c>
       <c r="I46" t="s">
@@ -3353,7 +3379,7 @@
       <c r="U46" t="s">
         <v>181</v>
       </c>
-      <c r="V46" s="1">
+      <c r="V46" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3400,7 +3426,7 @@
       <c r="U47" t="s">
         <v>29</v>
       </c>
-      <c r="V47" s="1">
+      <c r="V47" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3450,7 +3476,7 @@
       <c r="U48" t="s">
         <v>181</v>
       </c>
-      <c r="V48" s="1">
+      <c r="V48" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3476,7 +3502,7 @@
       <c r="G49" t="s">
         <v>43</v>
       </c>
-      <c r="H49" s="1">
+      <c r="H49" s="2">
         <v>46176</v>
       </c>
       <c r="I49" t="s">
@@ -3509,7 +3535,7 @@
       <c r="U49" t="s">
         <v>181</v>
       </c>
-      <c r="V49" s="1">
+      <c r="V49" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3562,7 +3588,7 @@
       <c r="U50" t="s">
         <v>181</v>
       </c>
-      <c r="V50" s="1">
+      <c r="V50" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3615,7 +3641,7 @@
       <c r="U51" t="s">
         <v>181</v>
       </c>
-      <c r="V51" s="1">
+      <c r="V51" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3665,7 +3691,7 @@
       <c r="U52" t="s">
         <v>181</v>
       </c>
-      <c r="V52" s="1">
+      <c r="V52" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3691,7 +3717,7 @@
       <c r="G53" t="s">
         <v>43</v>
       </c>
-      <c r="H53" s="1">
+      <c r="H53" s="2">
         <v>46227</v>
       </c>
       <c r="I53" t="s">
@@ -3721,7 +3747,7 @@
       <c r="U53" t="s">
         <v>181</v>
       </c>
-      <c r="V53" s="1">
+      <c r="V53" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3771,7 +3797,7 @@
       <c r="U54" t="s">
         <v>181</v>
       </c>
-      <c r="V54" s="1">
+      <c r="V54" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -3821,7 +3847,7 @@
       <c r="U55" t="s">
         <v>181</v>
       </c>
-      <c r="V55" s="1">
+      <c r="V55" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3871,7 +3897,7 @@
       <c r="U56" t="s">
         <v>181</v>
       </c>
-      <c r="V56" s="1">
+      <c r="V56" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3915,7 +3941,7 @@
       <c r="U57" t="s">
         <v>181</v>
       </c>
-      <c r="V57" s="1">
+      <c r="V57" s="2">
         <v>46049</v>
       </c>
     </row>
@@ -4041,7 +4067,7 @@
       <c r="U60" t="s">
         <v>181</v>
       </c>
-      <c r="V60" s="1">
+      <c r="V60" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4085,7 +4111,7 @@
       <c r="U61" t="s">
         <v>181</v>
       </c>
-      <c r="V61" s="1">
+      <c r="V61" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4129,7 +4155,7 @@
       <c r="U62" t="s">
         <v>181</v>
       </c>
-      <c r="V62" s="1">
+      <c r="V62" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4173,7 +4199,7 @@
       <c r="U63" t="s">
         <v>181</v>
       </c>
-      <c r="V63" s="1">
+      <c r="V63" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4217,7 +4243,7 @@
       <c r="U64" t="s">
         <v>181</v>
       </c>
-      <c r="V64" s="1">
+      <c r="V64" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4261,7 +4287,7 @@
       <c r="U65" t="s">
         <v>181</v>
       </c>
-      <c r="V65" s="1">
+      <c r="V65" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4305,7 +4331,7 @@
       <c r="U66" t="s">
         <v>29</v>
       </c>
-      <c r="V66" s="1">
+      <c r="V66" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4352,7 +4378,7 @@
       <c r="U67" t="s">
         <v>29</v>
       </c>
-      <c r="V67" s="1">
+      <c r="V67" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4402,7 +4428,7 @@
       <c r="U68" t="s">
         <v>181</v>
       </c>
-      <c r="V68" s="1">
+      <c r="V68" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -4446,7 +4472,7 @@
       <c r="U69" t="s">
         <v>29</v>
       </c>
-      <c r="V69" s="1">
+      <c r="V69" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -4490,7 +4516,7 @@
       <c r="U70" t="s">
         <v>181</v>
       </c>
-      <c r="V70" s="1">
+      <c r="V70" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4534,7 +4560,7 @@
       <c r="U71" t="s">
         <v>181</v>
       </c>
-      <c r="V71" s="1">
+      <c r="V71" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4578,7 +4604,7 @@
       <c r="U72" t="s">
         <v>181</v>
       </c>
-      <c r="V72" s="1">
+      <c r="V72" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4622,7 +4648,7 @@
       <c r="U73" t="s">
         <v>181</v>
       </c>
-      <c r="V73" s="1">
+      <c r="V73" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4666,7 +4692,7 @@
       <c r="U74" t="s">
         <v>181</v>
       </c>
-      <c r="V74" s="1">
+      <c r="V74" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4713,7 +4739,7 @@
       <c r="U75" t="s">
         <v>29</v>
       </c>
-      <c r="V75" s="1">
+      <c r="V75" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -4763,7 +4789,7 @@
       <c r="U76" t="s">
         <v>181</v>
       </c>
-      <c r="V76" s="1">
+      <c r="V76" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4813,7 +4839,7 @@
       <c r="U77" t="s">
         <v>181</v>
       </c>
-      <c r="V77" s="1">
+      <c r="V77" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4863,7 +4889,7 @@
       <c r="U78" t="s">
         <v>29</v>
       </c>
-      <c r="V78" s="1">
+      <c r="V78" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4913,7 +4939,7 @@
       <c r="U79" t="s">
         <v>29</v>
       </c>
-      <c r="V79" s="1">
+      <c r="V79" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4963,7 +4989,7 @@
       <c r="U80" t="s">
         <v>29</v>
       </c>
-      <c r="V80" s="1">
+      <c r="V80" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5007,7 +5033,7 @@
       <c r="U81" t="s">
         <v>29</v>
       </c>
-      <c r="V81" s="1">
+      <c r="V81" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5057,7 +5083,7 @@
       <c r="U82" t="s">
         <v>181</v>
       </c>
-      <c r="V82" s="1">
+      <c r="V82" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5101,7 +5127,7 @@
       <c r="U83" t="s">
         <v>29</v>
       </c>
-      <c r="V83" s="1">
+      <c r="V83" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -5145,7 +5171,7 @@
       <c r="U84" t="s">
         <v>29</v>
       </c>
-      <c r="V84" s="1">
+      <c r="V84" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5286,7 +5312,7 @@
       <c r="U87" t="s">
         <v>29</v>
       </c>
-      <c r="V87" s="1">
+      <c r="V87" s="2">
         <v>46291</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (01/09/2026 12:28)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -569,16 +569,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -594,7 +586,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -602,30 +594,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -925,70 +899,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1041,7 +1015,7 @@
       <c r="U2" t="s">
         <v>181</v>
       </c>
-      <c r="V2" s="2">
+      <c r="V2" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1088,7 +1062,7 @@
       <c r="U3" t="s">
         <v>29</v>
       </c>
-      <c r="V3" s="2">
+      <c r="V3" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1135,7 +1109,7 @@
       <c r="U4" t="s">
         <v>29</v>
       </c>
-      <c r="V4" s="2">
+      <c r="V4" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1182,7 +1156,7 @@
       <c r="U5" t="s">
         <v>29</v>
       </c>
-      <c r="V5" s="2">
+      <c r="V5" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1232,7 +1206,7 @@
       <c r="U6" t="s">
         <v>29</v>
       </c>
-      <c r="V6" s="2">
+      <c r="V6" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1258,7 +1232,7 @@
       <c r="G7" t="s">
         <v>43</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1288,7 +1262,7 @@
       <c r="U7" t="s">
         <v>29</v>
       </c>
-      <c r="V7" s="2">
+      <c r="V7" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -1335,7 +1309,7 @@
       <c r="U8" t="s">
         <v>29</v>
       </c>
-      <c r="V8" s="2">
+      <c r="V8" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1382,7 +1356,7 @@
       <c r="U9" t="s">
         <v>29</v>
       </c>
-      <c r="V9" s="2">
+      <c r="V9" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1429,7 +1403,7 @@
       <c r="U10" t="s">
         <v>29</v>
       </c>
-      <c r="V10" s="2">
+      <c r="V10" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1476,7 +1450,7 @@
       <c r="U11" t="s">
         <v>29</v>
       </c>
-      <c r="V11" s="2">
+      <c r="V11" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1502,7 +1476,7 @@
       <c r="G12" t="s">
         <v>43</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46079</v>
       </c>
       <c r="I12" t="s">
@@ -1535,7 +1509,7 @@
       <c r="U12" t="s">
         <v>181</v>
       </c>
-      <c r="V12" s="2">
+      <c r="V12" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1585,7 +1559,7 @@
       <c r="U13" t="s">
         <v>181</v>
       </c>
-      <c r="V13" s="2">
+      <c r="V13" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1635,7 +1609,7 @@
       <c r="U14" t="s">
         <v>181</v>
       </c>
-      <c r="V14" s="2">
+      <c r="V14" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1685,7 +1659,7 @@
       <c r="U15" t="s">
         <v>181</v>
       </c>
-      <c r="V15" s="2">
+      <c r="V15" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1735,7 +1709,7 @@
       <c r="U16" t="s">
         <v>181</v>
       </c>
-      <c r="V16" s="2">
+      <c r="V16" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1761,7 +1735,7 @@
       <c r="G17" t="s">
         <v>43</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46098</v>
       </c>
       <c r="I17" t="s">
@@ -1794,7 +1768,7 @@
       <c r="U17" t="s">
         <v>181</v>
       </c>
-      <c r="V17" s="2">
+      <c r="V17" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -1820,7 +1794,7 @@
       <c r="G18" t="s">
         <v>43</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46076</v>
       </c>
       <c r="I18" t="s">
@@ -1850,7 +1824,7 @@
       <c r="U18" t="s">
         <v>29</v>
       </c>
-      <c r="V18" s="2">
+      <c r="V18" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1876,7 +1850,7 @@
       <c r="G19" t="s">
         <v>43</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1906,7 +1880,7 @@
       <c r="U19" t="s">
         <v>29</v>
       </c>
-      <c r="V19" s="2">
+      <c r="V19" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1953,7 +1927,7 @@
       <c r="U20" t="s">
         <v>29</v>
       </c>
-      <c r="V20" s="2">
+      <c r="V20" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2000,7 +1974,7 @@
       <c r="U21" t="s">
         <v>29</v>
       </c>
-      <c r="V21" s="2">
+      <c r="V21" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2047,7 +2021,7 @@
       <c r="U22" t="s">
         <v>29</v>
       </c>
-      <c r="V22" s="2">
+      <c r="V22" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2094,7 +2068,7 @@
       <c r="U23" t="s">
         <v>29</v>
       </c>
-      <c r="V23" s="2">
+      <c r="V23" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2120,7 +2094,7 @@
       <c r="G24" t="s">
         <v>43</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>46119</v>
       </c>
       <c r="I24" t="s">
@@ -2153,7 +2127,7 @@
       <c r="U24" t="s">
         <v>181</v>
       </c>
-      <c r="V24" s="2">
+      <c r="V24" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2179,7 +2153,7 @@
       <c r="G25" t="s">
         <v>43</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>46121</v>
       </c>
       <c r="I25" t="s">
@@ -2209,7 +2183,7 @@
       <c r="U25" t="s">
         <v>29</v>
       </c>
-      <c r="V25" s="2">
+      <c r="V25" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2235,7 +2209,7 @@
       <c r="G26" t="s">
         <v>43</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>46076</v>
       </c>
       <c r="I26" t="s">
@@ -2265,7 +2239,7 @@
       <c r="U26" t="s">
         <v>29</v>
       </c>
-      <c r="V26" s="2">
+      <c r="V26" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -2315,7 +2289,7 @@
       <c r="U27" t="s">
         <v>181</v>
       </c>
-      <c r="V27" s="2">
+      <c r="V27" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2341,7 +2315,7 @@
       <c r="G28" t="s">
         <v>43</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>46199</v>
       </c>
       <c r="I28" t="s">
@@ -2374,7 +2348,7 @@
       <c r="U28" t="s">
         <v>181</v>
       </c>
-      <c r="V28" s="2">
+      <c r="V28" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2400,7 +2374,7 @@
       <c r="G29" t="s">
         <v>43</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2433,7 +2407,7 @@
       <c r="U29" t="s">
         <v>181</v>
       </c>
-      <c r="V29" s="2">
+      <c r="V29" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2459,7 +2433,7 @@
       <c r="G30" t="s">
         <v>43</v>
       </c>
-      <c r="H30" s="2">
+      <c r="H30" s="1">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2492,7 +2466,7 @@
       <c r="U30" t="s">
         <v>181</v>
       </c>
-      <c r="V30" s="2">
+      <c r="V30" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2518,7 +2492,7 @@
       <c r="G31" t="s">
         <v>43</v>
       </c>
-      <c r="H31" s="2">
+      <c r="H31" s="1">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2551,7 +2525,7 @@
       <c r="U31" t="s">
         <v>181</v>
       </c>
-      <c r="V31" s="2">
+      <c r="V31" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2601,7 +2575,7 @@
       <c r="U32" t="s">
         <v>181</v>
       </c>
-      <c r="V32" s="2">
+      <c r="V32" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2627,7 +2601,7 @@
       <c r="G33" t="s">
         <v>43</v>
       </c>
-      <c r="H33" s="2">
+      <c r="H33" s="1">
         <v>46191</v>
       </c>
       <c r="I33" t="s">
@@ -2660,7 +2634,7 @@
       <c r="U33" t="s">
         <v>181</v>
       </c>
-      <c r="V33" s="2">
+      <c r="V33" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2686,7 +2660,7 @@
       <c r="G34" t="s">
         <v>43</v>
       </c>
-      <c r="H34" s="2">
+      <c r="H34" s="1">
         <v>46119</v>
       </c>
       <c r="I34" t="s">
@@ -2716,7 +2690,7 @@
       <c r="U34" t="s">
         <v>181</v>
       </c>
-      <c r="V34" s="2">
+      <c r="V34" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2742,7 +2716,7 @@
       <c r="G35" t="s">
         <v>43</v>
       </c>
-      <c r="H35" s="2">
+      <c r="H35" s="1">
         <v>46213</v>
       </c>
       <c r="I35" t="s">
@@ -2772,7 +2746,7 @@
       <c r="U35" t="s">
         <v>29</v>
       </c>
-      <c r="V35" s="2">
+      <c r="V35" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -2798,7 +2772,7 @@
       <c r="G36" t="s">
         <v>43</v>
       </c>
-      <c r="H36" s="2">
+      <c r="H36" s="1">
         <v>46175</v>
       </c>
       <c r="I36" t="s">
@@ -2828,7 +2802,7 @@
       <c r="U36" t="s">
         <v>29</v>
       </c>
-      <c r="V36" s="2">
+      <c r="V36" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2854,7 +2828,7 @@
       <c r="G37" t="s">
         <v>43</v>
       </c>
-      <c r="H37" s="2">
+      <c r="H37" s="1">
         <v>46213</v>
       </c>
       <c r="I37" t="s">
@@ -2884,7 +2858,7 @@
       <c r="U37" t="s">
         <v>29</v>
       </c>
-      <c r="V37" s="2">
+      <c r="V37" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -2910,7 +2884,7 @@
       <c r="G38" t="s">
         <v>43</v>
       </c>
-      <c r="H38" s="2">
+      <c r="H38" s="1">
         <v>46199</v>
       </c>
       <c r="I38" t="s">
@@ -2940,7 +2914,7 @@
       <c r="U38" t="s">
         <v>29</v>
       </c>
-      <c r="V38" s="2">
+      <c r="V38" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2966,7 +2940,7 @@
       <c r="G39" t="s">
         <v>43</v>
       </c>
-      <c r="H39" s="2">
+      <c r="H39" s="1">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -2996,7 +2970,7 @@
       <c r="U39" t="s">
         <v>29</v>
       </c>
-      <c r="V39" s="2">
+      <c r="V39" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3022,7 +2996,7 @@
       <c r="G40" t="s">
         <v>43</v>
       </c>
-      <c r="H40" s="2">
+      <c r="H40" s="1">
         <v>46204</v>
       </c>
       <c r="I40" t="s">
@@ -3052,7 +3026,7 @@
       <c r="U40" t="s">
         <v>29</v>
       </c>
-      <c r="V40" s="2">
+      <c r="V40" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3078,7 +3052,7 @@
       <c r="G41" t="s">
         <v>43</v>
       </c>
-      <c r="H41" s="2">
+      <c r="H41" s="1">
         <v>46244</v>
       </c>
       <c r="I41" t="s">
@@ -3108,7 +3082,7 @@
       <c r="U41" t="s">
         <v>29</v>
       </c>
-      <c r="V41" s="2">
+      <c r="V41" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3152,7 +3126,7 @@
       <c r="U42" t="s">
         <v>29</v>
       </c>
-      <c r="V42" s="2">
+      <c r="V42" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3178,7 +3152,7 @@
       <c r="G43" t="s">
         <v>43</v>
       </c>
-      <c r="H43" s="2">
+      <c r="H43" s="1">
         <v>46191</v>
       </c>
       <c r="I43" t="s">
@@ -3208,7 +3182,7 @@
       <c r="U43" t="s">
         <v>29</v>
       </c>
-      <c r="V43" s="2">
+      <c r="V43" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3234,7 +3208,7 @@
       <c r="G44" t="s">
         <v>43</v>
       </c>
-      <c r="H44" s="2">
+      <c r="H44" s="1">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
@@ -3264,7 +3238,7 @@
       <c r="U44" t="s">
         <v>29</v>
       </c>
-      <c r="V44" s="2">
+      <c r="V44" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3290,7 +3264,7 @@
       <c r="G45" t="s">
         <v>43</v>
       </c>
-      <c r="H45" s="2">
+      <c r="H45" s="1">
         <v>46213</v>
       </c>
       <c r="I45" t="s">
@@ -3323,7 +3297,7 @@
       <c r="U45" t="s">
         <v>181</v>
       </c>
-      <c r="V45" s="2">
+      <c r="V45" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3349,7 +3323,7 @@
       <c r="G46" t="s">
         <v>43</v>
       </c>
-      <c r="H46" s="2">
+      <c r="H46" s="1">
         <v>46210</v>
       </c>
       <c r="I46" t="s">
@@ -3379,7 +3353,7 @@
       <c r="U46" t="s">
         <v>181</v>
       </c>
-      <c r="V46" s="2">
+      <c r="V46" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3426,7 +3400,7 @@
       <c r="U47" t="s">
         <v>29</v>
       </c>
-      <c r="V47" s="2">
+      <c r="V47" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3476,7 +3450,7 @@
       <c r="U48" t="s">
         <v>181</v>
       </c>
-      <c r="V48" s="2">
+      <c r="V48" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3502,7 +3476,7 @@
       <c r="G49" t="s">
         <v>43</v>
       </c>
-      <c r="H49" s="2">
+      <c r="H49" s="1">
         <v>46176</v>
       </c>
       <c r="I49" t="s">
@@ -3535,7 +3509,7 @@
       <c r="U49" t="s">
         <v>181</v>
       </c>
-      <c r="V49" s="2">
+      <c r="V49" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3588,7 +3562,7 @@
       <c r="U50" t="s">
         <v>181</v>
       </c>
-      <c r="V50" s="2">
+      <c r="V50" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3641,7 +3615,7 @@
       <c r="U51" t="s">
         <v>181</v>
       </c>
-      <c r="V51" s="2">
+      <c r="V51" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3691,7 +3665,7 @@
       <c r="U52" t="s">
         <v>181</v>
       </c>
-      <c r="V52" s="2">
+      <c r="V52" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3717,7 +3691,7 @@
       <c r="G53" t="s">
         <v>43</v>
       </c>
-      <c r="H53" s="2">
+      <c r="H53" s="1">
         <v>46227</v>
       </c>
       <c r="I53" t="s">
@@ -3747,7 +3721,7 @@
       <c r="U53" t="s">
         <v>181</v>
       </c>
-      <c r="V53" s="2">
+      <c r="V53" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3797,7 +3771,7 @@
       <c r="U54" t="s">
         <v>181</v>
       </c>
-      <c r="V54" s="2">
+      <c r="V54" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -3847,7 +3821,7 @@
       <c r="U55" t="s">
         <v>181</v>
       </c>
-      <c r="V55" s="2">
+      <c r="V55" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3897,7 +3871,7 @@
       <c r="U56" t="s">
         <v>181</v>
       </c>
-      <c r="V56" s="2">
+      <c r="V56" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3941,7 +3915,7 @@
       <c r="U57" t="s">
         <v>181</v>
       </c>
-      <c r="V57" s="2">
+      <c r="V57" s="1">
         <v>46049</v>
       </c>
     </row>
@@ -4067,7 +4041,7 @@
       <c r="U60" t="s">
         <v>181</v>
       </c>
-      <c r="V60" s="2">
+      <c r="V60" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4111,7 +4085,7 @@
       <c r="U61" t="s">
         <v>181</v>
       </c>
-      <c r="V61" s="2">
+      <c r="V61" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4155,7 +4129,7 @@
       <c r="U62" t="s">
         <v>181</v>
       </c>
-      <c r="V62" s="2">
+      <c r="V62" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4199,7 +4173,7 @@
       <c r="U63" t="s">
         <v>181</v>
       </c>
-      <c r="V63" s="2">
+      <c r="V63" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4243,7 +4217,7 @@
       <c r="U64" t="s">
         <v>181</v>
       </c>
-      <c r="V64" s="2">
+      <c r="V64" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4287,7 +4261,7 @@
       <c r="U65" t="s">
         <v>181</v>
       </c>
-      <c r="V65" s="2">
+      <c r="V65" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4331,7 +4305,7 @@
       <c r="U66" t="s">
         <v>29</v>
       </c>
-      <c r="V66" s="2">
+      <c r="V66" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4378,7 +4352,7 @@
       <c r="U67" t="s">
         <v>29</v>
       </c>
-      <c r="V67" s="2">
+      <c r="V67" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4428,7 +4402,7 @@
       <c r="U68" t="s">
         <v>181</v>
       </c>
-      <c r="V68" s="2">
+      <c r="V68" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -4472,7 +4446,7 @@
       <c r="U69" t="s">
         <v>29</v>
       </c>
-      <c r="V69" s="2">
+      <c r="V69" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -4516,7 +4490,7 @@
       <c r="U70" t="s">
         <v>181</v>
       </c>
-      <c r="V70" s="2">
+      <c r="V70" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4560,7 +4534,7 @@
       <c r="U71" t="s">
         <v>181</v>
       </c>
-      <c r="V71" s="2">
+      <c r="V71" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4604,7 +4578,7 @@
       <c r="U72" t="s">
         <v>181</v>
       </c>
-      <c r="V72" s="2">
+      <c r="V72" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4648,7 +4622,7 @@
       <c r="U73" t="s">
         <v>181</v>
       </c>
-      <c r="V73" s="2">
+      <c r="V73" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4692,7 +4666,7 @@
       <c r="U74" t="s">
         <v>181</v>
       </c>
-      <c r="V74" s="2">
+      <c r="V74" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4739,7 +4713,7 @@
       <c r="U75" t="s">
         <v>29</v>
       </c>
-      <c r="V75" s="2">
+      <c r="V75" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -4789,7 +4763,7 @@
       <c r="U76" t="s">
         <v>181</v>
       </c>
-      <c r="V76" s="2">
+      <c r="V76" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4839,7 +4813,7 @@
       <c r="U77" t="s">
         <v>181</v>
       </c>
-      <c r="V77" s="2">
+      <c r="V77" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4889,7 +4863,7 @@
       <c r="U78" t="s">
         <v>29</v>
       </c>
-      <c r="V78" s="2">
+      <c r="V78" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4939,7 +4913,7 @@
       <c r="U79" t="s">
         <v>29</v>
       </c>
-      <c r="V79" s="2">
+      <c r="V79" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4989,7 +4963,7 @@
       <c r="U80" t="s">
         <v>29</v>
       </c>
-      <c r="V80" s="2">
+      <c r="V80" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5033,7 +5007,7 @@
       <c r="U81" t="s">
         <v>29</v>
       </c>
-      <c r="V81" s="2">
+      <c r="V81" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5083,7 +5057,7 @@
       <c r="U82" t="s">
         <v>181</v>
       </c>
-      <c r="V82" s="2">
+      <c r="V82" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5127,7 +5101,7 @@
       <c r="U83" t="s">
         <v>29</v>
       </c>
-      <c r="V83" s="2">
+      <c r="V83" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -5171,7 +5145,7 @@
       <c r="U84" t="s">
         <v>29</v>
       </c>
-      <c r="V84" s="2">
+      <c r="V84" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5312,7 +5286,7 @@
       <c r="U87" t="s">
         <v>29</v>
       </c>
-      <c r="V87" s="2">
+      <c r="V87" s="1">
         <v>46291</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (02/09/2026 09:38)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -569,8 +569,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -586,7 +594,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -594,12 +602,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -899,70 +925,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1015,7 +1041,7 @@
       <c r="U2" t="s">
         <v>181</v>
       </c>
-      <c r="V2" s="1">
+      <c r="V2" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -1062,7 +1088,7 @@
       <c r="U3" t="s">
         <v>29</v>
       </c>
-      <c r="V3" s="1">
+      <c r="V3" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1109,7 +1135,7 @@
       <c r="U4" t="s">
         <v>29</v>
       </c>
-      <c r="V4" s="1">
+      <c r="V4" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1156,7 +1182,7 @@
       <c r="U5" t="s">
         <v>29</v>
       </c>
-      <c r="V5" s="1">
+      <c r="V5" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1206,7 +1232,7 @@
       <c r="U6" t="s">
         <v>29</v>
       </c>
-      <c r="V6" s="1">
+      <c r="V6" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1232,7 +1258,7 @@
       <c r="G7" t="s">
         <v>43</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1262,7 +1288,7 @@
       <c r="U7" t="s">
         <v>29</v>
       </c>
-      <c r="V7" s="1">
+      <c r="V7" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -1309,7 +1335,7 @@
       <c r="U8" t="s">
         <v>29</v>
       </c>
-      <c r="V8" s="1">
+      <c r="V8" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1356,7 +1382,7 @@
       <c r="U9" t="s">
         <v>29</v>
       </c>
-      <c r="V9" s="1">
+      <c r="V9" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1403,7 +1429,7 @@
       <c r="U10" t="s">
         <v>29</v>
       </c>
-      <c r="V10" s="1">
+      <c r="V10" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1450,7 +1476,7 @@
       <c r="U11" t="s">
         <v>29</v>
       </c>
-      <c r="V11" s="1">
+      <c r="V11" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1476,7 +1502,7 @@
       <c r="G12" t="s">
         <v>43</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46079</v>
       </c>
       <c r="I12" t="s">
@@ -1509,7 +1535,7 @@
       <c r="U12" t="s">
         <v>181</v>
       </c>
-      <c r="V12" s="1">
+      <c r="V12" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1559,7 +1585,7 @@
       <c r="U13" t="s">
         <v>181</v>
       </c>
-      <c r="V13" s="1">
+      <c r="V13" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1609,7 +1635,7 @@
       <c r="U14" t="s">
         <v>181</v>
       </c>
-      <c r="V14" s="1">
+      <c r="V14" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1659,7 +1685,7 @@
       <c r="U15" t="s">
         <v>181</v>
       </c>
-      <c r="V15" s="1">
+      <c r="V15" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1709,7 +1735,7 @@
       <c r="U16" t="s">
         <v>181</v>
       </c>
-      <c r="V16" s="1">
+      <c r="V16" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -1735,7 +1761,7 @@
       <c r="G17" t="s">
         <v>43</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46098</v>
       </c>
       <c r="I17" t="s">
@@ -1768,7 +1794,7 @@
       <c r="U17" t="s">
         <v>181</v>
       </c>
-      <c r="V17" s="1">
+      <c r="V17" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -1794,7 +1820,7 @@
       <c r="G18" t="s">
         <v>43</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46076</v>
       </c>
       <c r="I18" t="s">
@@ -1824,7 +1850,7 @@
       <c r="U18" t="s">
         <v>29</v>
       </c>
-      <c r="V18" s="1">
+      <c r="V18" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1850,7 +1876,7 @@
       <c r="G19" t="s">
         <v>43</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1880,7 +1906,7 @@
       <c r="U19" t="s">
         <v>29</v>
       </c>
-      <c r="V19" s="1">
+      <c r="V19" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1927,7 +1953,7 @@
       <c r="U20" t="s">
         <v>29</v>
       </c>
-      <c r="V20" s="1">
+      <c r="V20" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1974,7 +2000,7 @@
       <c r="U21" t="s">
         <v>29</v>
       </c>
-      <c r="V21" s="1">
+      <c r="V21" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2021,7 +2047,7 @@
       <c r="U22" t="s">
         <v>29</v>
       </c>
-      <c r="V22" s="1">
+      <c r="V22" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2068,7 +2094,7 @@
       <c r="U23" t="s">
         <v>29</v>
       </c>
-      <c r="V23" s="1">
+      <c r="V23" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2094,7 +2120,7 @@
       <c r="G24" t="s">
         <v>43</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>46119</v>
       </c>
       <c r="I24" t="s">
@@ -2127,7 +2153,7 @@
       <c r="U24" t="s">
         <v>181</v>
       </c>
-      <c r="V24" s="1">
+      <c r="V24" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2153,7 +2179,7 @@
       <c r="G25" t="s">
         <v>43</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>46121</v>
       </c>
       <c r="I25" t="s">
@@ -2183,7 +2209,7 @@
       <c r="U25" t="s">
         <v>29</v>
       </c>
-      <c r="V25" s="1">
+      <c r="V25" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2209,7 +2235,7 @@
       <c r="G26" t="s">
         <v>43</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>46076</v>
       </c>
       <c r="I26" t="s">
@@ -2239,7 +2265,7 @@
       <c r="U26" t="s">
         <v>29</v>
       </c>
-      <c r="V26" s="1">
+      <c r="V26" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -2289,7 +2315,7 @@
       <c r="U27" t="s">
         <v>181</v>
       </c>
-      <c r="V27" s="1">
+      <c r="V27" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -2315,7 +2341,7 @@
       <c r="G28" t="s">
         <v>43</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>46199</v>
       </c>
       <c r="I28" t="s">
@@ -2348,7 +2374,7 @@
       <c r="U28" t="s">
         <v>181</v>
       </c>
-      <c r="V28" s="1">
+      <c r="V28" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2374,7 +2400,7 @@
       <c r="G29" t="s">
         <v>43</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2407,7 +2433,7 @@
       <c r="U29" t="s">
         <v>181</v>
       </c>
-      <c r="V29" s="1">
+      <c r="V29" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2433,7 +2459,7 @@
       <c r="G30" t="s">
         <v>43</v>
       </c>
-      <c r="H30" s="1">
+      <c r="H30" s="2">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2466,7 +2492,7 @@
       <c r="U30" t="s">
         <v>181</v>
       </c>
-      <c r="V30" s="1">
+      <c r="V30" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2492,7 +2518,7 @@
       <c r="G31" t="s">
         <v>43</v>
       </c>
-      <c r="H31" s="1">
+      <c r="H31" s="2">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2525,7 +2551,7 @@
       <c r="U31" t="s">
         <v>181</v>
       </c>
-      <c r="V31" s="1">
+      <c r="V31" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2575,7 +2601,7 @@
       <c r="U32" t="s">
         <v>181</v>
       </c>
-      <c r="V32" s="1">
+      <c r="V32" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -2601,7 +2627,7 @@
       <c r="G33" t="s">
         <v>43</v>
       </c>
-      <c r="H33" s="1">
+      <c r="H33" s="2">
         <v>46191</v>
       </c>
       <c r="I33" t="s">
@@ -2634,7 +2660,7 @@
       <c r="U33" t="s">
         <v>181</v>
       </c>
-      <c r="V33" s="1">
+      <c r="V33" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2660,7 +2686,7 @@
       <c r="G34" t="s">
         <v>43</v>
       </c>
-      <c r="H34" s="1">
+      <c r="H34" s="2">
         <v>46119</v>
       </c>
       <c r="I34" t="s">
@@ -2690,7 +2716,7 @@
       <c r="U34" t="s">
         <v>181</v>
       </c>
-      <c r="V34" s="1">
+      <c r="V34" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2716,7 +2742,7 @@
       <c r="G35" t="s">
         <v>43</v>
       </c>
-      <c r="H35" s="1">
+      <c r="H35" s="2">
         <v>46213</v>
       </c>
       <c r="I35" t="s">
@@ -2746,7 +2772,7 @@
       <c r="U35" t="s">
         <v>29</v>
       </c>
-      <c r="V35" s="1">
+      <c r="V35" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -2772,7 +2798,7 @@
       <c r="G36" t="s">
         <v>43</v>
       </c>
-      <c r="H36" s="1">
+      <c r="H36" s="2">
         <v>46175</v>
       </c>
       <c r="I36" t="s">
@@ -2802,7 +2828,7 @@
       <c r="U36" t="s">
         <v>29</v>
       </c>
-      <c r="V36" s="1">
+      <c r="V36" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2828,7 +2854,7 @@
       <c r="G37" t="s">
         <v>43</v>
       </c>
-      <c r="H37" s="1">
+      <c r="H37" s="2">
         <v>46213</v>
       </c>
       <c r="I37" t="s">
@@ -2858,7 +2884,7 @@
       <c r="U37" t="s">
         <v>29</v>
       </c>
-      <c r="V37" s="1">
+      <c r="V37" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -2884,7 +2910,7 @@
       <c r="G38" t="s">
         <v>43</v>
       </c>
-      <c r="H38" s="1">
+      <c r="H38" s="2">
         <v>46199</v>
       </c>
       <c r="I38" t="s">
@@ -2914,7 +2940,7 @@
       <c r="U38" t="s">
         <v>29</v>
       </c>
-      <c r="V38" s="1">
+      <c r="V38" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2940,7 +2966,7 @@
       <c r="G39" t="s">
         <v>43</v>
       </c>
-      <c r="H39" s="1">
+      <c r="H39" s="2">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -2970,7 +2996,7 @@
       <c r="U39" t="s">
         <v>29</v>
       </c>
-      <c r="V39" s="1">
+      <c r="V39" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2996,7 +3022,7 @@
       <c r="G40" t="s">
         <v>43</v>
       </c>
-      <c r="H40" s="1">
+      <c r="H40" s="2">
         <v>46204</v>
       </c>
       <c r="I40" t="s">
@@ -3026,7 +3052,7 @@
       <c r="U40" t="s">
         <v>29</v>
       </c>
-      <c r="V40" s="1">
+      <c r="V40" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3052,7 +3078,7 @@
       <c r="G41" t="s">
         <v>43</v>
       </c>
-      <c r="H41" s="1">
+      <c r="H41" s="2">
         <v>46244</v>
       </c>
       <c r="I41" t="s">
@@ -3082,7 +3108,7 @@
       <c r="U41" t="s">
         <v>29</v>
       </c>
-      <c r="V41" s="1">
+      <c r="V41" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3126,7 +3152,7 @@
       <c r="U42" t="s">
         <v>29</v>
       </c>
-      <c r="V42" s="1">
+      <c r="V42" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3152,7 +3178,7 @@
       <c r="G43" t="s">
         <v>43</v>
       </c>
-      <c r="H43" s="1">
+      <c r="H43" s="2">
         <v>46191</v>
       </c>
       <c r="I43" t="s">
@@ -3182,7 +3208,7 @@
       <c r="U43" t="s">
         <v>29</v>
       </c>
-      <c r="V43" s="1">
+      <c r="V43" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3208,7 +3234,7 @@
       <c r="G44" t="s">
         <v>43</v>
       </c>
-      <c r="H44" s="1">
+      <c r="H44" s="2">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
@@ -3238,7 +3264,7 @@
       <c r="U44" t="s">
         <v>29</v>
       </c>
-      <c r="V44" s="1">
+      <c r="V44" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3264,7 +3290,7 @@
       <c r="G45" t="s">
         <v>43</v>
       </c>
-      <c r="H45" s="1">
+      <c r="H45" s="2">
         <v>46213</v>
       </c>
       <c r="I45" t="s">
@@ -3297,7 +3323,7 @@
       <c r="U45" t="s">
         <v>181</v>
       </c>
-      <c r="V45" s="1">
+      <c r="V45" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3323,7 +3349,7 @@
       <c r="G46" t="s">
         <v>43</v>
       </c>
-      <c r="H46" s="1">
+      <c r="H46" s="2">
         <v>46210</v>
       </c>
       <c r="I46" t="s">
@@ -3353,7 +3379,7 @@
       <c r="U46" t="s">
         <v>181</v>
       </c>
-      <c r="V46" s="1">
+      <c r="V46" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3400,7 +3426,7 @@
       <c r="U47" t="s">
         <v>29</v>
       </c>
-      <c r="V47" s="1">
+      <c r="V47" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3450,7 +3476,7 @@
       <c r="U48" t="s">
         <v>181</v>
       </c>
-      <c r="V48" s="1">
+      <c r="V48" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3476,7 +3502,7 @@
       <c r="G49" t="s">
         <v>43</v>
       </c>
-      <c r="H49" s="1">
+      <c r="H49" s="2">
         <v>46176</v>
       </c>
       <c r="I49" t="s">
@@ -3509,7 +3535,7 @@
       <c r="U49" t="s">
         <v>181</v>
       </c>
-      <c r="V49" s="1">
+      <c r="V49" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3562,7 +3588,7 @@
       <c r="U50" t="s">
         <v>181</v>
       </c>
-      <c r="V50" s="1">
+      <c r="V50" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3615,7 +3641,7 @@
       <c r="U51" t="s">
         <v>181</v>
       </c>
-      <c r="V51" s="1">
+      <c r="V51" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3665,7 +3691,7 @@
       <c r="U52" t="s">
         <v>181</v>
       </c>
-      <c r="V52" s="1">
+      <c r="V52" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3691,7 +3717,7 @@
       <c r="G53" t="s">
         <v>43</v>
       </c>
-      <c r="H53" s="1">
+      <c r="H53" s="2">
         <v>46227</v>
       </c>
       <c r="I53" t="s">
@@ -3721,7 +3747,7 @@
       <c r="U53" t="s">
         <v>181</v>
       </c>
-      <c r="V53" s="1">
+      <c r="V53" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3771,7 +3797,7 @@
       <c r="U54" t="s">
         <v>181</v>
       </c>
-      <c r="V54" s="1">
+      <c r="V54" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -3821,7 +3847,7 @@
       <c r="U55" t="s">
         <v>181</v>
       </c>
-      <c r="V55" s="1">
+      <c r="V55" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3871,7 +3897,7 @@
       <c r="U56" t="s">
         <v>181</v>
       </c>
-      <c r="V56" s="1">
+      <c r="V56" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3915,7 +3941,7 @@
       <c r="U57" t="s">
         <v>181</v>
       </c>
-      <c r="V57" s="1">
+      <c r="V57" s="2">
         <v>46049</v>
       </c>
     </row>
@@ -4041,7 +4067,7 @@
       <c r="U60" t="s">
         <v>181</v>
       </c>
-      <c r="V60" s="1">
+      <c r="V60" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4085,7 +4111,7 @@
       <c r="U61" t="s">
         <v>181</v>
       </c>
-      <c r="V61" s="1">
+      <c r="V61" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4129,7 +4155,7 @@
       <c r="U62" t="s">
         <v>181</v>
       </c>
-      <c r="V62" s="1">
+      <c r="V62" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4173,7 +4199,7 @@
       <c r="U63" t="s">
         <v>181</v>
       </c>
-      <c r="V63" s="1">
+      <c r="V63" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4217,7 +4243,7 @@
       <c r="U64" t="s">
         <v>181</v>
       </c>
-      <c r="V64" s="1">
+      <c r="V64" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4261,7 +4287,7 @@
       <c r="U65" t="s">
         <v>181</v>
       </c>
-      <c r="V65" s="1">
+      <c r="V65" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4305,7 +4331,7 @@
       <c r="U66" t="s">
         <v>29</v>
       </c>
-      <c r="V66" s="1">
+      <c r="V66" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4352,7 +4378,7 @@
       <c r="U67" t="s">
         <v>29</v>
       </c>
-      <c r="V67" s="1">
+      <c r="V67" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4402,7 +4428,7 @@
       <c r="U68" t="s">
         <v>181</v>
       </c>
-      <c r="V68" s="1">
+      <c r="V68" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -4446,7 +4472,7 @@
       <c r="U69" t="s">
         <v>29</v>
       </c>
-      <c r="V69" s="1">
+      <c r="V69" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -4490,7 +4516,7 @@
       <c r="U70" t="s">
         <v>181</v>
       </c>
-      <c r="V70" s="1">
+      <c r="V70" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4534,7 +4560,7 @@
       <c r="U71" t="s">
         <v>181</v>
       </c>
-      <c r="V71" s="1">
+      <c r="V71" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4578,7 +4604,7 @@
       <c r="U72" t="s">
         <v>181</v>
       </c>
-      <c r="V72" s="1">
+      <c r="V72" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4622,7 +4648,7 @@
       <c r="U73" t="s">
         <v>181</v>
       </c>
-      <c r="V73" s="1">
+      <c r="V73" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4666,7 +4692,7 @@
       <c r="U74" t="s">
         <v>181</v>
       </c>
-      <c r="V74" s="1">
+      <c r="V74" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4713,7 +4739,7 @@
       <c r="U75" t="s">
         <v>29</v>
       </c>
-      <c r="V75" s="1">
+      <c r="V75" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -4763,7 +4789,7 @@
       <c r="U76" t="s">
         <v>181</v>
       </c>
-      <c r="V76" s="1">
+      <c r="V76" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4813,7 +4839,7 @@
       <c r="U77" t="s">
         <v>181</v>
       </c>
-      <c r="V77" s="1">
+      <c r="V77" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4863,7 +4889,7 @@
       <c r="U78" t="s">
         <v>29</v>
       </c>
-      <c r="V78" s="1">
+      <c r="V78" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4913,7 +4939,7 @@
       <c r="U79" t="s">
         <v>29</v>
       </c>
-      <c r="V79" s="1">
+      <c r="V79" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4963,7 +4989,7 @@
       <c r="U80" t="s">
         <v>29</v>
       </c>
-      <c r="V80" s="1">
+      <c r="V80" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5007,7 +5033,7 @@
       <c r="U81" t="s">
         <v>29</v>
       </c>
-      <c r="V81" s="1">
+      <c r="V81" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5057,7 +5083,7 @@
       <c r="U82" t="s">
         <v>181</v>
       </c>
-      <c r="V82" s="1">
+      <c r="V82" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5101,7 +5127,7 @@
       <c r="U83" t="s">
         <v>29</v>
       </c>
-      <c r="V83" s="1">
+      <c r="V83" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -5145,7 +5171,7 @@
       <c r="U84" t="s">
         <v>29</v>
       </c>
-      <c r="V84" s="1">
+      <c r="V84" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5286,7 +5312,7 @@
       <c r="U87" t="s">
         <v>29</v>
       </c>
-      <c r="V87" s="1">
+      <c r="V87" s="2">
         <v>46291</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (02/09/2026 12:04)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -569,16 +569,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -594,7 +586,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -602,30 +594,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -925,70 +899,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1041,7 +1015,7 @@
       <c r="U2" t="s">
         <v>181</v>
       </c>
-      <c r="V2" s="2">
+      <c r="V2" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1088,7 +1062,7 @@
       <c r="U3" t="s">
         <v>29</v>
       </c>
-      <c r="V3" s="2">
+      <c r="V3" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1135,7 +1109,7 @@
       <c r="U4" t="s">
         <v>29</v>
       </c>
-      <c r="V4" s="2">
+      <c r="V4" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1182,7 +1156,7 @@
       <c r="U5" t="s">
         <v>29</v>
       </c>
-      <c r="V5" s="2">
+      <c r="V5" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1232,7 +1206,7 @@
       <c r="U6" t="s">
         <v>29</v>
       </c>
-      <c r="V6" s="2">
+      <c r="V6" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1258,7 +1232,7 @@
       <c r="G7" t="s">
         <v>43</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1288,7 +1262,7 @@
       <c r="U7" t="s">
         <v>29</v>
       </c>
-      <c r="V7" s="2">
+      <c r="V7" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -1335,7 +1309,7 @@
       <c r="U8" t="s">
         <v>29</v>
       </c>
-      <c r="V8" s="2">
+      <c r="V8" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1382,7 +1356,7 @@
       <c r="U9" t="s">
         <v>29</v>
       </c>
-      <c r="V9" s="2">
+      <c r="V9" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1429,7 +1403,7 @@
       <c r="U10" t="s">
         <v>29</v>
       </c>
-      <c r="V10" s="2">
+      <c r="V10" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1476,7 +1450,7 @@
       <c r="U11" t="s">
         <v>29</v>
       </c>
-      <c r="V11" s="2">
+      <c r="V11" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1502,7 +1476,7 @@
       <c r="G12" t="s">
         <v>43</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46079</v>
       </c>
       <c r="I12" t="s">
@@ -1535,7 +1509,7 @@
       <c r="U12" t="s">
         <v>181</v>
       </c>
-      <c r="V12" s="2">
+      <c r="V12" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1585,7 +1559,7 @@
       <c r="U13" t="s">
         <v>181</v>
       </c>
-      <c r="V13" s="2">
+      <c r="V13" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1635,7 +1609,7 @@
       <c r="U14" t="s">
         <v>181</v>
       </c>
-      <c r="V14" s="2">
+      <c r="V14" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1685,7 +1659,7 @@
       <c r="U15" t="s">
         <v>181</v>
       </c>
-      <c r="V15" s="2">
+      <c r="V15" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1735,7 +1709,7 @@
       <c r="U16" t="s">
         <v>181</v>
       </c>
-      <c r="V16" s="2">
+      <c r="V16" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1761,7 +1735,7 @@
       <c r="G17" t="s">
         <v>43</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46098</v>
       </c>
       <c r="I17" t="s">
@@ -1794,7 +1768,7 @@
       <c r="U17" t="s">
         <v>181</v>
       </c>
-      <c r="V17" s="2">
+      <c r="V17" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -1820,7 +1794,7 @@
       <c r="G18" t="s">
         <v>43</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46076</v>
       </c>
       <c r="I18" t="s">
@@ -1850,7 +1824,7 @@
       <c r="U18" t="s">
         <v>29</v>
       </c>
-      <c r="V18" s="2">
+      <c r="V18" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1876,7 +1850,7 @@
       <c r="G19" t="s">
         <v>43</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1906,7 +1880,7 @@
       <c r="U19" t="s">
         <v>29</v>
       </c>
-      <c r="V19" s="2">
+      <c r="V19" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1953,7 +1927,7 @@
       <c r="U20" t="s">
         <v>29</v>
       </c>
-      <c r="V20" s="2">
+      <c r="V20" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2000,7 +1974,7 @@
       <c r="U21" t="s">
         <v>29</v>
       </c>
-      <c r="V21" s="2">
+      <c r="V21" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2047,7 +2021,7 @@
       <c r="U22" t="s">
         <v>29</v>
       </c>
-      <c r="V22" s="2">
+      <c r="V22" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2094,7 +2068,7 @@
       <c r="U23" t="s">
         <v>29</v>
       </c>
-      <c r="V23" s="2">
+      <c r="V23" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2120,7 +2094,7 @@
       <c r="G24" t="s">
         <v>43</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>46119</v>
       </c>
       <c r="I24" t="s">
@@ -2153,7 +2127,7 @@
       <c r="U24" t="s">
         <v>181</v>
       </c>
-      <c r="V24" s="2">
+      <c r="V24" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2179,7 +2153,7 @@
       <c r="G25" t="s">
         <v>43</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>46121</v>
       </c>
       <c r="I25" t="s">
@@ -2209,7 +2183,7 @@
       <c r="U25" t="s">
         <v>29</v>
       </c>
-      <c r="V25" s="2">
+      <c r="V25" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2235,7 +2209,7 @@
       <c r="G26" t="s">
         <v>43</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>46076</v>
       </c>
       <c r="I26" t="s">
@@ -2265,7 +2239,7 @@
       <c r="U26" t="s">
         <v>29</v>
       </c>
-      <c r="V26" s="2">
+      <c r="V26" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -2315,7 +2289,7 @@
       <c r="U27" t="s">
         <v>181</v>
       </c>
-      <c r="V27" s="2">
+      <c r="V27" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2341,7 +2315,7 @@
       <c r="G28" t="s">
         <v>43</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>46199</v>
       </c>
       <c r="I28" t="s">
@@ -2374,7 +2348,7 @@
       <c r="U28" t="s">
         <v>181</v>
       </c>
-      <c r="V28" s="2">
+      <c r="V28" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2400,7 +2374,7 @@
       <c r="G29" t="s">
         <v>43</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2433,7 +2407,7 @@
       <c r="U29" t="s">
         <v>181</v>
       </c>
-      <c r="V29" s="2">
+      <c r="V29" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2459,7 +2433,7 @@
       <c r="G30" t="s">
         <v>43</v>
       </c>
-      <c r="H30" s="2">
+      <c r="H30" s="1">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2492,7 +2466,7 @@
       <c r="U30" t="s">
         <v>181</v>
       </c>
-      <c r="V30" s="2">
+      <c r="V30" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2518,7 +2492,7 @@
       <c r="G31" t="s">
         <v>43</v>
       </c>
-      <c r="H31" s="2">
+      <c r="H31" s="1">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2551,7 +2525,7 @@
       <c r="U31" t="s">
         <v>181</v>
       </c>
-      <c r="V31" s="2">
+      <c r="V31" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2601,7 +2575,7 @@
       <c r="U32" t="s">
         <v>181</v>
       </c>
-      <c r="V32" s="2">
+      <c r="V32" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2627,7 +2601,7 @@
       <c r="G33" t="s">
         <v>43</v>
       </c>
-      <c r="H33" s="2">
+      <c r="H33" s="1">
         <v>46191</v>
       </c>
       <c r="I33" t="s">
@@ -2660,7 +2634,7 @@
       <c r="U33" t="s">
         <v>181</v>
       </c>
-      <c r="V33" s="2">
+      <c r="V33" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2686,7 +2660,7 @@
       <c r="G34" t="s">
         <v>43</v>
       </c>
-      <c r="H34" s="2">
+      <c r="H34" s="1">
         <v>46119</v>
       </c>
       <c r="I34" t="s">
@@ -2716,7 +2690,7 @@
       <c r="U34" t="s">
         <v>181</v>
       </c>
-      <c r="V34" s="2">
+      <c r="V34" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2742,7 +2716,7 @@
       <c r="G35" t="s">
         <v>43</v>
       </c>
-      <c r="H35" s="2">
+      <c r="H35" s="1">
         <v>46213</v>
       </c>
       <c r="I35" t="s">
@@ -2772,7 +2746,7 @@
       <c r="U35" t="s">
         <v>29</v>
       </c>
-      <c r="V35" s="2">
+      <c r="V35" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -2798,7 +2772,7 @@
       <c r="G36" t="s">
         <v>43</v>
       </c>
-      <c r="H36" s="2">
+      <c r="H36" s="1">
         <v>46175</v>
       </c>
       <c r="I36" t="s">
@@ -2828,7 +2802,7 @@
       <c r="U36" t="s">
         <v>29</v>
       </c>
-      <c r="V36" s="2">
+      <c r="V36" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2854,7 +2828,7 @@
       <c r="G37" t="s">
         <v>43</v>
       </c>
-      <c r="H37" s="2">
+      <c r="H37" s="1">
         <v>46213</v>
       </c>
       <c r="I37" t="s">
@@ -2884,7 +2858,7 @@
       <c r="U37" t="s">
         <v>29</v>
       </c>
-      <c r="V37" s="2">
+      <c r="V37" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -2910,7 +2884,7 @@
       <c r="G38" t="s">
         <v>43</v>
       </c>
-      <c r="H38" s="2">
+      <c r="H38" s="1">
         <v>46199</v>
       </c>
       <c r="I38" t="s">
@@ -2940,7 +2914,7 @@
       <c r="U38" t="s">
         <v>29</v>
       </c>
-      <c r="V38" s="2">
+      <c r="V38" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2966,7 +2940,7 @@
       <c r="G39" t="s">
         <v>43</v>
       </c>
-      <c r="H39" s="2">
+      <c r="H39" s="1">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -2996,7 +2970,7 @@
       <c r="U39" t="s">
         <v>29</v>
       </c>
-      <c r="V39" s="2">
+      <c r="V39" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3022,7 +2996,7 @@
       <c r="G40" t="s">
         <v>43</v>
       </c>
-      <c r="H40" s="2">
+      <c r="H40" s="1">
         <v>46204</v>
       </c>
       <c r="I40" t="s">
@@ -3052,7 +3026,7 @@
       <c r="U40" t="s">
         <v>29</v>
       </c>
-      <c r="V40" s="2">
+      <c r="V40" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3078,7 +3052,7 @@
       <c r="G41" t="s">
         <v>43</v>
       </c>
-      <c r="H41" s="2">
+      <c r="H41" s="1">
         <v>46244</v>
       </c>
       <c r="I41" t="s">
@@ -3108,7 +3082,7 @@
       <c r="U41" t="s">
         <v>29</v>
       </c>
-      <c r="V41" s="2">
+      <c r="V41" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3152,7 +3126,7 @@
       <c r="U42" t="s">
         <v>29</v>
       </c>
-      <c r="V42" s="2">
+      <c r="V42" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3178,7 +3152,7 @@
       <c r="G43" t="s">
         <v>43</v>
       </c>
-      <c r="H43" s="2">
+      <c r="H43" s="1">
         <v>46191</v>
       </c>
       <c r="I43" t="s">
@@ -3208,7 +3182,7 @@
       <c r="U43" t="s">
         <v>29</v>
       </c>
-      <c r="V43" s="2">
+      <c r="V43" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3234,7 +3208,7 @@
       <c r="G44" t="s">
         <v>43</v>
       </c>
-      <c r="H44" s="2">
+      <c r="H44" s="1">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
@@ -3264,7 +3238,7 @@
       <c r="U44" t="s">
         <v>29</v>
       </c>
-      <c r="V44" s="2">
+      <c r="V44" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3290,7 +3264,7 @@
       <c r="G45" t="s">
         <v>43</v>
       </c>
-      <c r="H45" s="2">
+      <c r="H45" s="1">
         <v>46213</v>
       </c>
       <c r="I45" t="s">
@@ -3323,7 +3297,7 @@
       <c r="U45" t="s">
         <v>181</v>
       </c>
-      <c r="V45" s="2">
+      <c r="V45" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3349,7 +3323,7 @@
       <c r="G46" t="s">
         <v>43</v>
       </c>
-      <c r="H46" s="2">
+      <c r="H46" s="1">
         <v>46210</v>
       </c>
       <c r="I46" t="s">
@@ -3379,7 +3353,7 @@
       <c r="U46" t="s">
         <v>181</v>
       </c>
-      <c r="V46" s="2">
+      <c r="V46" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3426,7 +3400,7 @@
       <c r="U47" t="s">
         <v>29</v>
       </c>
-      <c r="V47" s="2">
+      <c r="V47" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3476,7 +3450,7 @@
       <c r="U48" t="s">
         <v>181</v>
       </c>
-      <c r="V48" s="2">
+      <c r="V48" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3502,7 +3476,7 @@
       <c r="G49" t="s">
         <v>43</v>
       </c>
-      <c r="H49" s="2">
+      <c r="H49" s="1">
         <v>46176</v>
       </c>
       <c r="I49" t="s">
@@ -3535,7 +3509,7 @@
       <c r="U49" t="s">
         <v>181</v>
       </c>
-      <c r="V49" s="2">
+      <c r="V49" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3588,7 +3562,7 @@
       <c r="U50" t="s">
         <v>181</v>
       </c>
-      <c r="V50" s="2">
+      <c r="V50" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3641,7 +3615,7 @@
       <c r="U51" t="s">
         <v>181</v>
       </c>
-      <c r="V51" s="2">
+      <c r="V51" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3691,7 +3665,7 @@
       <c r="U52" t="s">
         <v>181</v>
       </c>
-      <c r="V52" s="2">
+      <c r="V52" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3717,7 +3691,7 @@
       <c r="G53" t="s">
         <v>43</v>
       </c>
-      <c r="H53" s="2">
+      <c r="H53" s="1">
         <v>46227</v>
       </c>
       <c r="I53" t="s">
@@ -3747,7 +3721,7 @@
       <c r="U53" t="s">
         <v>181</v>
       </c>
-      <c r="V53" s="2">
+      <c r="V53" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3797,7 +3771,7 @@
       <c r="U54" t="s">
         <v>181</v>
       </c>
-      <c r="V54" s="2">
+      <c r="V54" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -3847,7 +3821,7 @@
       <c r="U55" t="s">
         <v>181</v>
       </c>
-      <c r="V55" s="2">
+      <c r="V55" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3897,7 +3871,7 @@
       <c r="U56" t="s">
         <v>181</v>
       </c>
-      <c r="V56" s="2">
+      <c r="V56" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3941,7 +3915,7 @@
       <c r="U57" t="s">
         <v>181</v>
       </c>
-      <c r="V57" s="2">
+      <c r="V57" s="1">
         <v>46049</v>
       </c>
     </row>
@@ -4067,7 +4041,7 @@
       <c r="U60" t="s">
         <v>181</v>
       </c>
-      <c r="V60" s="2">
+      <c r="V60" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4111,7 +4085,7 @@
       <c r="U61" t="s">
         <v>181</v>
       </c>
-      <c r="V61" s="2">
+      <c r="V61" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4155,7 +4129,7 @@
       <c r="U62" t="s">
         <v>181</v>
       </c>
-      <c r="V62" s="2">
+      <c r="V62" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4199,7 +4173,7 @@
       <c r="U63" t="s">
         <v>181</v>
       </c>
-      <c r="V63" s="2">
+      <c r="V63" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4243,7 +4217,7 @@
       <c r="U64" t="s">
         <v>181</v>
       </c>
-      <c r="V64" s="2">
+      <c r="V64" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4287,7 +4261,7 @@
       <c r="U65" t="s">
         <v>181</v>
       </c>
-      <c r="V65" s="2">
+      <c r="V65" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4331,7 +4305,7 @@
       <c r="U66" t="s">
         <v>29</v>
       </c>
-      <c r="V66" s="2">
+      <c r="V66" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4378,7 +4352,7 @@
       <c r="U67" t="s">
         <v>29</v>
       </c>
-      <c r="V67" s="2">
+      <c r="V67" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4428,7 +4402,7 @@
       <c r="U68" t="s">
         <v>181</v>
       </c>
-      <c r="V68" s="2">
+      <c r="V68" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -4472,7 +4446,7 @@
       <c r="U69" t="s">
         <v>29</v>
       </c>
-      <c r="V69" s="2">
+      <c r="V69" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -4516,7 +4490,7 @@
       <c r="U70" t="s">
         <v>181</v>
       </c>
-      <c r="V70" s="2">
+      <c r="V70" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4560,7 +4534,7 @@
       <c r="U71" t="s">
         <v>181</v>
       </c>
-      <c r="V71" s="2">
+      <c r="V71" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4604,7 +4578,7 @@
       <c r="U72" t="s">
         <v>181</v>
       </c>
-      <c r="V72" s="2">
+      <c r="V72" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4648,7 +4622,7 @@
       <c r="U73" t="s">
         <v>181</v>
       </c>
-      <c r="V73" s="2">
+      <c r="V73" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4692,7 +4666,7 @@
       <c r="U74" t="s">
         <v>181</v>
       </c>
-      <c r="V74" s="2">
+      <c r="V74" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4739,7 +4713,7 @@
       <c r="U75" t="s">
         <v>29</v>
       </c>
-      <c r="V75" s="2">
+      <c r="V75" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -4789,7 +4763,7 @@
       <c r="U76" t="s">
         <v>181</v>
       </c>
-      <c r="V76" s="2">
+      <c r="V76" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4839,7 +4813,7 @@
       <c r="U77" t="s">
         <v>181</v>
       </c>
-      <c r="V77" s="2">
+      <c r="V77" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4889,7 +4863,7 @@
       <c r="U78" t="s">
         <v>29</v>
       </c>
-      <c r="V78" s="2">
+      <c r="V78" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4939,7 +4913,7 @@
       <c r="U79" t="s">
         <v>29</v>
       </c>
-      <c r="V79" s="2">
+      <c r="V79" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4989,7 +4963,7 @@
       <c r="U80" t="s">
         <v>29</v>
       </c>
-      <c r="V80" s="2">
+      <c r="V80" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5033,7 +5007,7 @@
       <c r="U81" t="s">
         <v>29</v>
       </c>
-      <c r="V81" s="2">
+      <c r="V81" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5083,7 +5057,7 @@
       <c r="U82" t="s">
         <v>181</v>
       </c>
-      <c r="V82" s="2">
+      <c r="V82" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5127,7 +5101,7 @@
       <c r="U83" t="s">
         <v>29</v>
       </c>
-      <c r="V83" s="2">
+      <c r="V83" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -5171,7 +5145,7 @@
       <c r="U84" t="s">
         <v>29</v>
       </c>
-      <c r="V84" s="2">
+      <c r="V84" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5312,7 +5286,7 @@
       <c r="U87" t="s">
         <v>29</v>
       </c>
-      <c r="V87" s="2">
+      <c r="V87" s="1">
         <v>46291</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (03/09/2026 13:42)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -569,8 +569,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -586,7 +594,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -594,12 +602,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -899,70 +925,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1015,7 +1041,7 @@
       <c r="U2" t="s">
         <v>181</v>
       </c>
-      <c r="V2" s="1">
+      <c r="V2" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -1062,7 +1088,7 @@
       <c r="U3" t="s">
         <v>29</v>
       </c>
-      <c r="V3" s="1">
+      <c r="V3" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1109,7 +1135,7 @@
       <c r="U4" t="s">
         <v>29</v>
       </c>
-      <c r="V4" s="1">
+      <c r="V4" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1156,7 +1182,7 @@
       <c r="U5" t="s">
         <v>29</v>
       </c>
-      <c r="V5" s="1">
+      <c r="V5" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1206,7 +1232,7 @@
       <c r="U6" t="s">
         <v>29</v>
       </c>
-      <c r="V6" s="1">
+      <c r="V6" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1232,7 +1258,7 @@
       <c r="G7" t="s">
         <v>43</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1262,7 +1288,7 @@
       <c r="U7" t="s">
         <v>29</v>
       </c>
-      <c r="V7" s="1">
+      <c r="V7" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -1309,7 +1335,7 @@
       <c r="U8" t="s">
         <v>29</v>
       </c>
-      <c r="V8" s="1">
+      <c r="V8" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1356,7 +1382,7 @@
       <c r="U9" t="s">
         <v>29</v>
       </c>
-      <c r="V9" s="1">
+      <c r="V9" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1403,7 +1429,7 @@
       <c r="U10" t="s">
         <v>29</v>
       </c>
-      <c r="V10" s="1">
+      <c r="V10" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1450,7 +1476,7 @@
       <c r="U11" t="s">
         <v>29</v>
       </c>
-      <c r="V11" s="1">
+      <c r="V11" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1476,7 +1502,7 @@
       <c r="G12" t="s">
         <v>43</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46079</v>
       </c>
       <c r="I12" t="s">
@@ -1509,7 +1535,7 @@
       <c r="U12" t="s">
         <v>181</v>
       </c>
-      <c r="V12" s="1">
+      <c r="V12" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1559,7 +1585,7 @@
       <c r="U13" t="s">
         <v>181</v>
       </c>
-      <c r="V13" s="1">
+      <c r="V13" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1609,7 +1635,7 @@
       <c r="U14" t="s">
         <v>181</v>
       </c>
-      <c r="V14" s="1">
+      <c r="V14" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1659,7 +1685,7 @@
       <c r="U15" t="s">
         <v>181</v>
       </c>
-      <c r="V15" s="1">
+      <c r="V15" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1709,7 +1735,7 @@
       <c r="U16" t="s">
         <v>181</v>
       </c>
-      <c r="V16" s="1">
+      <c r="V16" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -1735,7 +1761,7 @@
       <c r="G17" t="s">
         <v>43</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46098</v>
       </c>
       <c r="I17" t="s">
@@ -1768,7 +1794,7 @@
       <c r="U17" t="s">
         <v>181</v>
       </c>
-      <c r="V17" s="1">
+      <c r="V17" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -1794,7 +1820,7 @@
       <c r="G18" t="s">
         <v>43</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46076</v>
       </c>
       <c r="I18" t="s">
@@ -1824,7 +1850,7 @@
       <c r="U18" t="s">
         <v>29</v>
       </c>
-      <c r="V18" s="1">
+      <c r="V18" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1850,7 +1876,7 @@
       <c r="G19" t="s">
         <v>43</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1880,7 +1906,7 @@
       <c r="U19" t="s">
         <v>29</v>
       </c>
-      <c r="V19" s="1">
+      <c r="V19" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1927,7 +1953,7 @@
       <c r="U20" t="s">
         <v>29</v>
       </c>
-      <c r="V20" s="1">
+      <c r="V20" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1974,7 +2000,7 @@
       <c r="U21" t="s">
         <v>29</v>
       </c>
-      <c r="V21" s="1">
+      <c r="V21" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2021,7 +2047,7 @@
       <c r="U22" t="s">
         <v>29</v>
       </c>
-      <c r="V22" s="1">
+      <c r="V22" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2068,7 +2094,7 @@
       <c r="U23" t="s">
         <v>29</v>
       </c>
-      <c r="V23" s="1">
+      <c r="V23" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2094,7 +2120,7 @@
       <c r="G24" t="s">
         <v>43</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>46119</v>
       </c>
       <c r="I24" t="s">
@@ -2127,7 +2153,7 @@
       <c r="U24" t="s">
         <v>181</v>
       </c>
-      <c r="V24" s="1">
+      <c r="V24" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2153,7 +2179,7 @@
       <c r="G25" t="s">
         <v>43</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>46121</v>
       </c>
       <c r="I25" t="s">
@@ -2183,7 +2209,7 @@
       <c r="U25" t="s">
         <v>29</v>
       </c>
-      <c r="V25" s="1">
+      <c r="V25" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2209,7 +2235,7 @@
       <c r="G26" t="s">
         <v>43</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>46076</v>
       </c>
       <c r="I26" t="s">
@@ -2239,7 +2265,7 @@
       <c r="U26" t="s">
         <v>29</v>
       </c>
-      <c r="V26" s="1">
+      <c r="V26" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -2289,7 +2315,7 @@
       <c r="U27" t="s">
         <v>181</v>
       </c>
-      <c r="V27" s="1">
+      <c r="V27" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -2315,7 +2341,7 @@
       <c r="G28" t="s">
         <v>43</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>46199</v>
       </c>
       <c r="I28" t="s">
@@ -2348,7 +2374,7 @@
       <c r="U28" t="s">
         <v>181</v>
       </c>
-      <c r="V28" s="1">
+      <c r="V28" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2374,7 +2400,7 @@
       <c r="G29" t="s">
         <v>43</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2407,7 +2433,7 @@
       <c r="U29" t="s">
         <v>181</v>
       </c>
-      <c r="V29" s="1">
+      <c r="V29" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2433,7 +2459,7 @@
       <c r="G30" t="s">
         <v>43</v>
       </c>
-      <c r="H30" s="1">
+      <c r="H30" s="2">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2466,7 +2492,7 @@
       <c r="U30" t="s">
         <v>181</v>
       </c>
-      <c r="V30" s="1">
+      <c r="V30" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2492,7 +2518,7 @@
       <c r="G31" t="s">
         <v>43</v>
       </c>
-      <c r="H31" s="1">
+      <c r="H31" s="2">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2525,7 +2551,7 @@
       <c r="U31" t="s">
         <v>181</v>
       </c>
-      <c r="V31" s="1">
+      <c r="V31" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2575,7 +2601,7 @@
       <c r="U32" t="s">
         <v>181</v>
       </c>
-      <c r="V32" s="1">
+      <c r="V32" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -2601,7 +2627,7 @@
       <c r="G33" t="s">
         <v>43</v>
       </c>
-      <c r="H33" s="1">
+      <c r="H33" s="2">
         <v>46191</v>
       </c>
       <c r="I33" t="s">
@@ -2634,7 +2660,7 @@
       <c r="U33" t="s">
         <v>181</v>
       </c>
-      <c r="V33" s="1">
+      <c r="V33" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2660,7 +2686,7 @@
       <c r="G34" t="s">
         <v>43</v>
       </c>
-      <c r="H34" s="1">
+      <c r="H34" s="2">
         <v>46119</v>
       </c>
       <c r="I34" t="s">
@@ -2690,7 +2716,7 @@
       <c r="U34" t="s">
         <v>181</v>
       </c>
-      <c r="V34" s="1">
+      <c r="V34" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2716,7 +2742,7 @@
       <c r="G35" t="s">
         <v>43</v>
       </c>
-      <c r="H35" s="1">
+      <c r="H35" s="2">
         <v>46213</v>
       </c>
       <c r="I35" t="s">
@@ -2746,7 +2772,7 @@
       <c r="U35" t="s">
         <v>29</v>
       </c>
-      <c r="V35" s="1">
+      <c r="V35" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -2772,7 +2798,7 @@
       <c r="G36" t="s">
         <v>43</v>
       </c>
-      <c r="H36" s="1">
+      <c r="H36" s="2">
         <v>46175</v>
       </c>
       <c r="I36" t="s">
@@ -2802,7 +2828,7 @@
       <c r="U36" t="s">
         <v>29</v>
       </c>
-      <c r="V36" s="1">
+      <c r="V36" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2828,7 +2854,7 @@
       <c r="G37" t="s">
         <v>43</v>
       </c>
-      <c r="H37" s="1">
+      <c r="H37" s="2">
         <v>46213</v>
       </c>
       <c r="I37" t="s">
@@ -2858,7 +2884,7 @@
       <c r="U37" t="s">
         <v>29</v>
       </c>
-      <c r="V37" s="1">
+      <c r="V37" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -2884,7 +2910,7 @@
       <c r="G38" t="s">
         <v>43</v>
       </c>
-      <c r="H38" s="1">
+      <c r="H38" s="2">
         <v>46199</v>
       </c>
       <c r="I38" t="s">
@@ -2914,7 +2940,7 @@
       <c r="U38" t="s">
         <v>29</v>
       </c>
-      <c r="V38" s="1">
+      <c r="V38" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2940,7 +2966,7 @@
       <c r="G39" t="s">
         <v>43</v>
       </c>
-      <c r="H39" s="1">
+      <c r="H39" s="2">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -2970,7 +2996,7 @@
       <c r="U39" t="s">
         <v>29</v>
       </c>
-      <c r="V39" s="1">
+      <c r="V39" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2996,7 +3022,7 @@
       <c r="G40" t="s">
         <v>43</v>
       </c>
-      <c r="H40" s="1">
+      <c r="H40" s="2">
         <v>46204</v>
       </c>
       <c r="I40" t="s">
@@ -3026,7 +3052,7 @@
       <c r="U40" t="s">
         <v>29</v>
       </c>
-      <c r="V40" s="1">
+      <c r="V40" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3052,7 +3078,7 @@
       <c r="G41" t="s">
         <v>43</v>
       </c>
-      <c r="H41" s="1">
+      <c r="H41" s="2">
         <v>46244</v>
       </c>
       <c r="I41" t="s">
@@ -3082,7 +3108,7 @@
       <c r="U41" t="s">
         <v>29</v>
       </c>
-      <c r="V41" s="1">
+      <c r="V41" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3126,7 +3152,7 @@
       <c r="U42" t="s">
         <v>29</v>
       </c>
-      <c r="V42" s="1">
+      <c r="V42" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3152,7 +3178,7 @@
       <c r="G43" t="s">
         <v>43</v>
       </c>
-      <c r="H43" s="1">
+      <c r="H43" s="2">
         <v>46191</v>
       </c>
       <c r="I43" t="s">
@@ -3182,7 +3208,7 @@
       <c r="U43" t="s">
         <v>29</v>
       </c>
-      <c r="V43" s="1">
+      <c r="V43" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3208,7 +3234,7 @@
       <c r="G44" t="s">
         <v>43</v>
       </c>
-      <c r="H44" s="1">
+      <c r="H44" s="2">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
@@ -3238,7 +3264,7 @@
       <c r="U44" t="s">
         <v>29</v>
       </c>
-      <c r="V44" s="1">
+      <c r="V44" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3264,7 +3290,7 @@
       <c r="G45" t="s">
         <v>43</v>
       </c>
-      <c r="H45" s="1">
+      <c r="H45" s="2">
         <v>46213</v>
       </c>
       <c r="I45" t="s">
@@ -3297,7 +3323,7 @@
       <c r="U45" t="s">
         <v>181</v>
       </c>
-      <c r="V45" s="1">
+      <c r="V45" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3323,7 +3349,7 @@
       <c r="G46" t="s">
         <v>43</v>
       </c>
-      <c r="H46" s="1">
+      <c r="H46" s="2">
         <v>46210</v>
       </c>
       <c r="I46" t="s">
@@ -3353,7 +3379,7 @@
       <c r="U46" t="s">
         <v>181</v>
       </c>
-      <c r="V46" s="1">
+      <c r="V46" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3400,7 +3426,7 @@
       <c r="U47" t="s">
         <v>29</v>
       </c>
-      <c r="V47" s="1">
+      <c r="V47" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3450,7 +3476,7 @@
       <c r="U48" t="s">
         <v>181</v>
       </c>
-      <c r="V48" s="1">
+      <c r="V48" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3476,7 +3502,7 @@
       <c r="G49" t="s">
         <v>43</v>
       </c>
-      <c r="H49" s="1">
+      <c r="H49" s="2">
         <v>46176</v>
       </c>
       <c r="I49" t="s">
@@ -3509,7 +3535,7 @@
       <c r="U49" t="s">
         <v>181</v>
       </c>
-      <c r="V49" s="1">
+      <c r="V49" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3562,7 +3588,7 @@
       <c r="U50" t="s">
         <v>181</v>
       </c>
-      <c r="V50" s="1">
+      <c r="V50" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3615,7 +3641,7 @@
       <c r="U51" t="s">
         <v>181</v>
       </c>
-      <c r="V51" s="1">
+      <c r="V51" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3665,7 +3691,7 @@
       <c r="U52" t="s">
         <v>181</v>
       </c>
-      <c r="V52" s="1">
+      <c r="V52" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3691,7 +3717,7 @@
       <c r="G53" t="s">
         <v>43</v>
       </c>
-      <c r="H53" s="1">
+      <c r="H53" s="2">
         <v>46227</v>
       </c>
       <c r="I53" t="s">
@@ -3721,7 +3747,7 @@
       <c r="U53" t="s">
         <v>181</v>
       </c>
-      <c r="V53" s="1">
+      <c r="V53" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3771,7 +3797,7 @@
       <c r="U54" t="s">
         <v>181</v>
       </c>
-      <c r="V54" s="1">
+      <c r="V54" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -3821,7 +3847,7 @@
       <c r="U55" t="s">
         <v>181</v>
       </c>
-      <c r="V55" s="1">
+      <c r="V55" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3871,7 +3897,7 @@
       <c r="U56" t="s">
         <v>181</v>
       </c>
-      <c r="V56" s="1">
+      <c r="V56" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3915,7 +3941,7 @@
       <c r="U57" t="s">
         <v>181</v>
       </c>
-      <c r="V57" s="1">
+      <c r="V57" s="2">
         <v>46049</v>
       </c>
     </row>
@@ -4041,7 +4067,7 @@
       <c r="U60" t="s">
         <v>181</v>
       </c>
-      <c r="V60" s="1">
+      <c r="V60" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4085,7 +4111,7 @@
       <c r="U61" t="s">
         <v>181</v>
       </c>
-      <c r="V61" s="1">
+      <c r="V61" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4129,7 +4155,7 @@
       <c r="U62" t="s">
         <v>181</v>
       </c>
-      <c r="V62" s="1">
+      <c r="V62" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4173,7 +4199,7 @@
       <c r="U63" t="s">
         <v>181</v>
       </c>
-      <c r="V63" s="1">
+      <c r="V63" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4217,7 +4243,7 @@
       <c r="U64" t="s">
         <v>181</v>
       </c>
-      <c r="V64" s="1">
+      <c r="V64" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4261,7 +4287,7 @@
       <c r="U65" t="s">
         <v>181</v>
       </c>
-      <c r="V65" s="1">
+      <c r="V65" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4305,7 +4331,7 @@
       <c r="U66" t="s">
         <v>29</v>
       </c>
-      <c r="V66" s="1">
+      <c r="V66" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4352,7 +4378,7 @@
       <c r="U67" t="s">
         <v>29</v>
       </c>
-      <c r="V67" s="1">
+      <c r="V67" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4402,7 +4428,7 @@
       <c r="U68" t="s">
         <v>181</v>
       </c>
-      <c r="V68" s="1">
+      <c r="V68" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -4446,7 +4472,7 @@
       <c r="U69" t="s">
         <v>29</v>
       </c>
-      <c r="V69" s="1">
+      <c r="V69" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -4490,7 +4516,7 @@
       <c r="U70" t="s">
         <v>181</v>
       </c>
-      <c r="V70" s="1">
+      <c r="V70" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4534,7 +4560,7 @@
       <c r="U71" t="s">
         <v>181</v>
       </c>
-      <c r="V71" s="1">
+      <c r="V71" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4578,7 +4604,7 @@
       <c r="U72" t="s">
         <v>181</v>
       </c>
-      <c r="V72" s="1">
+      <c r="V72" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4622,7 +4648,7 @@
       <c r="U73" t="s">
         <v>181</v>
       </c>
-      <c r="V73" s="1">
+      <c r="V73" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4666,7 +4692,7 @@
       <c r="U74" t="s">
         <v>181</v>
       </c>
-      <c r="V74" s="1">
+      <c r="V74" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4713,7 +4739,7 @@
       <c r="U75" t="s">
         <v>29</v>
       </c>
-      <c r="V75" s="1">
+      <c r="V75" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -4763,7 +4789,7 @@
       <c r="U76" t="s">
         <v>181</v>
       </c>
-      <c r="V76" s="1">
+      <c r="V76" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4813,7 +4839,7 @@
       <c r="U77" t="s">
         <v>181</v>
       </c>
-      <c r="V77" s="1">
+      <c r="V77" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4863,7 +4889,7 @@
       <c r="U78" t="s">
         <v>29</v>
       </c>
-      <c r="V78" s="1">
+      <c r="V78" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4913,7 +4939,7 @@
       <c r="U79" t="s">
         <v>29</v>
       </c>
-      <c r="V79" s="1">
+      <c r="V79" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4963,7 +4989,7 @@
       <c r="U80" t="s">
         <v>29</v>
       </c>
-      <c r="V80" s="1">
+      <c r="V80" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5007,7 +5033,7 @@
       <c r="U81" t="s">
         <v>29</v>
       </c>
-      <c r="V81" s="1">
+      <c r="V81" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5057,7 +5083,7 @@
       <c r="U82" t="s">
         <v>181</v>
       </c>
-      <c r="V82" s="1">
+      <c r="V82" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5101,7 +5127,7 @@
       <c r="U83" t="s">
         <v>29</v>
       </c>
-      <c r="V83" s="1">
+      <c r="V83" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -5145,7 +5171,7 @@
       <c r="U84" t="s">
         <v>29</v>
       </c>
-      <c r="V84" s="1">
+      <c r="V84" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5286,7 +5312,7 @@
       <c r="U87" t="s">
         <v>29</v>
       </c>
-      <c r="V87" s="1">
+      <c r="V87" s="2">
         <v>46291</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (08/09/2026 08:22)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -566,8 +566,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -583,7 +591,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -591,12 +599,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -896,70 +922,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1012,7 +1038,7 @@
       <c r="U2" t="s">
         <v>180</v>
       </c>
-      <c r="V2" s="1">
+      <c r="V2" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -1059,7 +1085,7 @@
       <c r="U3" t="s">
         <v>28</v>
       </c>
-      <c r="V3" s="1">
+      <c r="V3" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1106,7 +1132,7 @@
       <c r="U4" t="s">
         <v>28</v>
       </c>
-      <c r="V4" s="1">
+      <c r="V4" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1153,7 +1179,7 @@
       <c r="U5" t="s">
         <v>28</v>
       </c>
-      <c r="V5" s="1">
+      <c r="V5" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1203,7 +1229,7 @@
       <c r="U6" t="s">
         <v>28</v>
       </c>
-      <c r="V6" s="1">
+      <c r="V6" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1229,7 +1255,7 @@
       <c r="G7" t="s">
         <v>42</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1259,7 +1285,7 @@
       <c r="U7" t="s">
         <v>28</v>
       </c>
-      <c r="V7" s="1">
+      <c r="V7" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -1306,7 +1332,7 @@
       <c r="U8" t="s">
         <v>28</v>
       </c>
-      <c r="V8" s="1">
+      <c r="V8" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1353,7 +1379,7 @@
       <c r="U9" t="s">
         <v>28</v>
       </c>
-      <c r="V9" s="1">
+      <c r="V9" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1400,7 +1426,7 @@
       <c r="U10" t="s">
         <v>28</v>
       </c>
-      <c r="V10" s="1">
+      <c r="V10" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1447,7 +1473,7 @@
       <c r="U11" t="s">
         <v>28</v>
       </c>
-      <c r="V11" s="1">
+      <c r="V11" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1473,7 +1499,7 @@
       <c r="G12" t="s">
         <v>42</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46079</v>
       </c>
       <c r="I12" t="s">
@@ -1506,7 +1532,7 @@
       <c r="U12" t="s">
         <v>180</v>
       </c>
-      <c r="V12" s="1">
+      <c r="V12" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1556,7 +1582,7 @@
       <c r="U13" t="s">
         <v>180</v>
       </c>
-      <c r="V13" s="1">
+      <c r="V13" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1606,7 +1632,7 @@
       <c r="U14" t="s">
         <v>180</v>
       </c>
-      <c r="V14" s="1">
+      <c r="V14" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1656,7 +1682,7 @@
       <c r="U15" t="s">
         <v>180</v>
       </c>
-      <c r="V15" s="1">
+      <c r="V15" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1706,7 +1732,7 @@
       <c r="U16" t="s">
         <v>180</v>
       </c>
-      <c r="V16" s="1">
+      <c r="V16" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -1732,7 +1758,7 @@
       <c r="G17" t="s">
         <v>42</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46098</v>
       </c>
       <c r="I17" t="s">
@@ -1765,7 +1791,7 @@
       <c r="U17" t="s">
         <v>180</v>
       </c>
-      <c r="V17" s="1">
+      <c r="V17" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -1791,7 +1817,7 @@
       <c r="G18" t="s">
         <v>42</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46076</v>
       </c>
       <c r="I18" t="s">
@@ -1821,7 +1847,7 @@
       <c r="U18" t="s">
         <v>28</v>
       </c>
-      <c r="V18" s="1">
+      <c r="V18" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1847,7 +1873,7 @@
       <c r="G19" t="s">
         <v>42</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1877,7 +1903,7 @@
       <c r="U19" t="s">
         <v>28</v>
       </c>
-      <c r="V19" s="1">
+      <c r="V19" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1924,7 +1950,7 @@
       <c r="U20" t="s">
         <v>28</v>
       </c>
-      <c r="V20" s="1">
+      <c r="V20" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1971,7 +1997,7 @@
       <c r="U21" t="s">
         <v>28</v>
       </c>
-      <c r="V21" s="1">
+      <c r="V21" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2018,7 +2044,7 @@
       <c r="U22" t="s">
         <v>28</v>
       </c>
-      <c r="V22" s="1">
+      <c r="V22" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2065,7 +2091,7 @@
       <c r="U23" t="s">
         <v>28</v>
       </c>
-      <c r="V23" s="1">
+      <c r="V23" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2091,7 +2117,7 @@
       <c r="G24" t="s">
         <v>42</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>46119</v>
       </c>
       <c r="I24" t="s">
@@ -2124,7 +2150,7 @@
       <c r="U24" t="s">
         <v>180</v>
       </c>
-      <c r="V24" s="1">
+      <c r="V24" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2150,7 +2176,7 @@
       <c r="G25" t="s">
         <v>42</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>46121</v>
       </c>
       <c r="I25" t="s">
@@ -2180,7 +2206,7 @@
       <c r="U25" t="s">
         <v>28</v>
       </c>
-      <c r="V25" s="1">
+      <c r="V25" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2206,7 +2232,7 @@
       <c r="G26" t="s">
         <v>42</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>46076</v>
       </c>
       <c r="I26" t="s">
@@ -2236,7 +2262,7 @@
       <c r="U26" t="s">
         <v>28</v>
       </c>
-      <c r="V26" s="1">
+      <c r="V26" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -2286,7 +2312,7 @@
       <c r="U27" t="s">
         <v>180</v>
       </c>
-      <c r="V27" s="1">
+      <c r="V27" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -2312,7 +2338,7 @@
       <c r="G28" t="s">
         <v>42</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>46199</v>
       </c>
       <c r="I28" t="s">
@@ -2345,7 +2371,7 @@
       <c r="U28" t="s">
         <v>180</v>
       </c>
-      <c r="V28" s="1">
+      <c r="V28" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2371,7 +2397,7 @@
       <c r="G29" t="s">
         <v>42</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2404,7 +2430,7 @@
       <c r="U29" t="s">
         <v>180</v>
       </c>
-      <c r="V29" s="1">
+      <c r="V29" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2430,7 +2456,7 @@
       <c r="G30" t="s">
         <v>42</v>
       </c>
-      <c r="H30" s="1">
+      <c r="H30" s="2">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2463,7 +2489,7 @@
       <c r="U30" t="s">
         <v>180</v>
       </c>
-      <c r="V30" s="1">
+      <c r="V30" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2489,7 +2515,7 @@
       <c r="G31" t="s">
         <v>42</v>
       </c>
-      <c r="H31" s="1">
+      <c r="H31" s="2">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2522,7 +2548,7 @@
       <c r="U31" t="s">
         <v>180</v>
       </c>
-      <c r="V31" s="1">
+      <c r="V31" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2572,7 +2598,7 @@
       <c r="U32" t="s">
         <v>180</v>
       </c>
-      <c r="V32" s="1">
+      <c r="V32" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -2598,7 +2624,7 @@
       <c r="G33" t="s">
         <v>42</v>
       </c>
-      <c r="H33" s="1">
+      <c r="H33" s="2">
         <v>46191</v>
       </c>
       <c r="I33" t="s">
@@ -2631,7 +2657,7 @@
       <c r="U33" t="s">
         <v>180</v>
       </c>
-      <c r="V33" s="1">
+      <c r="V33" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2657,7 +2683,7 @@
       <c r="G34" t="s">
         <v>42</v>
       </c>
-      <c r="H34" s="1">
+      <c r="H34" s="2">
         <v>46119</v>
       </c>
       <c r="I34" t="s">
@@ -2687,7 +2713,7 @@
       <c r="U34" t="s">
         <v>180</v>
       </c>
-      <c r="V34" s="1">
+      <c r="V34" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2713,7 +2739,7 @@
       <c r="G35" t="s">
         <v>42</v>
       </c>
-      <c r="H35" s="1">
+      <c r="H35" s="2">
         <v>46213</v>
       </c>
       <c r="I35" t="s">
@@ -2743,7 +2769,7 @@
       <c r="U35" t="s">
         <v>28</v>
       </c>
-      <c r="V35" s="1">
+      <c r="V35" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -2769,7 +2795,7 @@
       <c r="G36" t="s">
         <v>42</v>
       </c>
-      <c r="H36" s="1">
+      <c r="H36" s="2">
         <v>46175</v>
       </c>
       <c r="I36" t="s">
@@ -2799,7 +2825,7 @@
       <c r="U36" t="s">
         <v>28</v>
       </c>
-      <c r="V36" s="1">
+      <c r="V36" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2825,7 +2851,7 @@
       <c r="G37" t="s">
         <v>42</v>
       </c>
-      <c r="H37" s="1">
+      <c r="H37" s="2">
         <v>46213</v>
       </c>
       <c r="I37" t="s">
@@ -2855,7 +2881,7 @@
       <c r="U37" t="s">
         <v>28</v>
       </c>
-      <c r="V37" s="1">
+      <c r="V37" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -2881,7 +2907,7 @@
       <c r="G38" t="s">
         <v>42</v>
       </c>
-      <c r="H38" s="1">
+      <c r="H38" s="2">
         <v>46199</v>
       </c>
       <c r="I38" t="s">
@@ -2911,7 +2937,7 @@
       <c r="U38" t="s">
         <v>28</v>
       </c>
-      <c r="V38" s="1">
+      <c r="V38" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2937,7 +2963,7 @@
       <c r="G39" t="s">
         <v>42</v>
       </c>
-      <c r="H39" s="1">
+      <c r="H39" s="2">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -2967,7 +2993,7 @@
       <c r="U39" t="s">
         <v>28</v>
       </c>
-      <c r="V39" s="1">
+      <c r="V39" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2993,7 +3019,7 @@
       <c r="G40" t="s">
         <v>42</v>
       </c>
-      <c r="H40" s="1">
+      <c r="H40" s="2">
         <v>46204</v>
       </c>
       <c r="I40" t="s">
@@ -3023,7 +3049,7 @@
       <c r="U40" t="s">
         <v>28</v>
       </c>
-      <c r="V40" s="1">
+      <c r="V40" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3049,7 +3075,7 @@
       <c r="G41" t="s">
         <v>42</v>
       </c>
-      <c r="H41" s="1">
+      <c r="H41" s="2">
         <v>46244</v>
       </c>
       <c r="I41" t="s">
@@ -3079,7 +3105,7 @@
       <c r="U41" t="s">
         <v>28</v>
       </c>
-      <c r="V41" s="1">
+      <c r="V41" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3123,7 +3149,7 @@
       <c r="U42" t="s">
         <v>28</v>
       </c>
-      <c r="V42" s="1">
+      <c r="V42" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3149,7 +3175,7 @@
       <c r="G43" t="s">
         <v>42</v>
       </c>
-      <c r="H43" s="1">
+      <c r="H43" s="2">
         <v>46191</v>
       </c>
       <c r="I43" t="s">
@@ -3179,7 +3205,7 @@
       <c r="U43" t="s">
         <v>28</v>
       </c>
-      <c r="V43" s="1">
+      <c r="V43" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3205,7 +3231,7 @@
       <c r="G44" t="s">
         <v>42</v>
       </c>
-      <c r="H44" s="1">
+      <c r="H44" s="2">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
@@ -3235,7 +3261,7 @@
       <c r="U44" t="s">
         <v>28</v>
       </c>
-      <c r="V44" s="1">
+      <c r="V44" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3261,7 +3287,7 @@
       <c r="G45" t="s">
         <v>42</v>
       </c>
-      <c r="H45" s="1">
+      <c r="H45" s="2">
         <v>46213</v>
       </c>
       <c r="I45" t="s">
@@ -3294,7 +3320,7 @@
       <c r="U45" t="s">
         <v>180</v>
       </c>
-      <c r="V45" s="1">
+      <c r="V45" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3320,7 +3346,7 @@
       <c r="G46" t="s">
         <v>42</v>
       </c>
-      <c r="H46" s="1">
+      <c r="H46" s="2">
         <v>46210</v>
       </c>
       <c r="I46" t="s">
@@ -3350,7 +3376,7 @@
       <c r="U46" t="s">
         <v>180</v>
       </c>
-      <c r="V46" s="1">
+      <c r="V46" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3397,7 +3423,7 @@
       <c r="U47" t="s">
         <v>28</v>
       </c>
-      <c r="V47" s="1">
+      <c r="V47" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3447,7 +3473,7 @@
       <c r="U48" t="s">
         <v>180</v>
       </c>
-      <c r="V48" s="1">
+      <c r="V48" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3473,7 +3499,7 @@
       <c r="G49" t="s">
         <v>42</v>
       </c>
-      <c r="H49" s="1">
+      <c r="H49" s="2">
         <v>46176</v>
       </c>
       <c r="I49" t="s">
@@ -3506,7 +3532,7 @@
       <c r="U49" t="s">
         <v>180</v>
       </c>
-      <c r="V49" s="1">
+      <c r="V49" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3559,7 +3585,7 @@
       <c r="U50" t="s">
         <v>180</v>
       </c>
-      <c r="V50" s="1">
+      <c r="V50" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3612,7 +3638,7 @@
       <c r="U51" t="s">
         <v>180</v>
       </c>
-      <c r="V51" s="1">
+      <c r="V51" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3662,7 +3688,7 @@
       <c r="U52" t="s">
         <v>180</v>
       </c>
-      <c r="V52" s="1">
+      <c r="V52" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3688,7 +3714,7 @@
       <c r="G53" t="s">
         <v>42</v>
       </c>
-      <c r="H53" s="1">
+      <c r="H53" s="2">
         <v>46227</v>
       </c>
       <c r="I53" t="s">
@@ -3718,7 +3744,7 @@
       <c r="U53" t="s">
         <v>180</v>
       </c>
-      <c r="V53" s="1">
+      <c r="V53" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3768,7 +3794,7 @@
       <c r="U54" t="s">
         <v>180</v>
       </c>
-      <c r="V54" s="1">
+      <c r="V54" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -3818,7 +3844,7 @@
       <c r="U55" t="s">
         <v>180</v>
       </c>
-      <c r="V55" s="1">
+      <c r="V55" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3868,7 +3894,7 @@
       <c r="U56" t="s">
         <v>180</v>
       </c>
-      <c r="V56" s="1">
+      <c r="V56" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3912,7 +3938,7 @@
       <c r="U57" t="s">
         <v>180</v>
       </c>
-      <c r="V57" s="1">
+      <c r="V57" s="2">
         <v>46049</v>
       </c>
     </row>
@@ -4038,7 +4064,7 @@
       <c r="U60" t="s">
         <v>180</v>
       </c>
-      <c r="V60" s="1">
+      <c r="V60" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4082,7 +4108,7 @@
       <c r="U61" t="s">
         <v>180</v>
       </c>
-      <c r="V61" s="1">
+      <c r="V61" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4126,7 +4152,7 @@
       <c r="U62" t="s">
         <v>180</v>
       </c>
-      <c r="V62" s="1">
+      <c r="V62" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4170,7 +4196,7 @@
       <c r="U63" t="s">
         <v>180</v>
       </c>
-      <c r="V63" s="1">
+      <c r="V63" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4214,7 +4240,7 @@
       <c r="U64" t="s">
         <v>180</v>
       </c>
-      <c r="V64" s="1">
+      <c r="V64" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4258,7 +4284,7 @@
       <c r="U65" t="s">
         <v>180</v>
       </c>
-      <c r="V65" s="1">
+      <c r="V65" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4302,7 +4328,7 @@
       <c r="U66" t="s">
         <v>28</v>
       </c>
-      <c r="V66" s="1">
+      <c r="V66" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4349,7 +4375,7 @@
       <c r="U67" t="s">
         <v>28</v>
       </c>
-      <c r="V67" s="1">
+      <c r="V67" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4399,7 +4425,7 @@
       <c r="U68" t="s">
         <v>180</v>
       </c>
-      <c r="V68" s="1">
+      <c r="V68" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -4443,7 +4469,7 @@
       <c r="U69" t="s">
         <v>28</v>
       </c>
-      <c r="V69" s="1">
+      <c r="V69" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -4487,7 +4513,7 @@
       <c r="U70" t="s">
         <v>180</v>
       </c>
-      <c r="V70" s="1">
+      <c r="V70" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4531,7 +4557,7 @@
       <c r="U71" t="s">
         <v>180</v>
       </c>
-      <c r="V71" s="1">
+      <c r="V71" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4575,7 +4601,7 @@
       <c r="U72" t="s">
         <v>180</v>
       </c>
-      <c r="V72" s="1">
+      <c r="V72" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4619,7 +4645,7 @@
       <c r="U73" t="s">
         <v>180</v>
       </c>
-      <c r="V73" s="1">
+      <c r="V73" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4663,7 +4689,7 @@
       <c r="U74" t="s">
         <v>180</v>
       </c>
-      <c r="V74" s="1">
+      <c r="V74" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4710,7 +4736,7 @@
       <c r="U75" t="s">
         <v>28</v>
       </c>
-      <c r="V75" s="1">
+      <c r="V75" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -4760,7 +4786,7 @@
       <c r="U76" t="s">
         <v>180</v>
       </c>
-      <c r="V76" s="1">
+      <c r="V76" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4810,7 +4836,7 @@
       <c r="U77" t="s">
         <v>180</v>
       </c>
-      <c r="V77" s="1">
+      <c r="V77" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4860,7 +4886,7 @@
       <c r="U78" t="s">
         <v>28</v>
       </c>
-      <c r="V78" s="1">
+      <c r="V78" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4910,7 +4936,7 @@
       <c r="U79" t="s">
         <v>28</v>
       </c>
-      <c r="V79" s="1">
+      <c r="V79" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4960,7 +4986,7 @@
       <c r="U80" t="s">
         <v>28</v>
       </c>
-      <c r="V80" s="1">
+      <c r="V80" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5004,7 +5030,7 @@
       <c r="U81" t="s">
         <v>28</v>
       </c>
-      <c r="V81" s="1">
+      <c r="V81" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5054,7 +5080,7 @@
       <c r="U82" t="s">
         <v>180</v>
       </c>
-      <c r="V82" s="1">
+      <c r="V82" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5098,7 +5124,7 @@
       <c r="U83" t="s">
         <v>28</v>
       </c>
-      <c r="V83" s="1">
+      <c r="V83" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -5142,7 +5168,7 @@
       <c r="U84" t="s">
         <v>28</v>
       </c>
-      <c r="V84" s="1">
+      <c r="V84" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5283,7 +5309,7 @@
       <c r="U87" t="s">
         <v>28</v>
       </c>
-      <c r="V87" s="1">
+      <c r="V87" s="2">
         <v>46291</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (08/09/2026 12:04)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -566,16 +566,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -591,7 +583,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -599,30 +591,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -922,70 +896,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1038,7 +1012,7 @@
       <c r="U2" t="s">
         <v>180</v>
       </c>
-      <c r="V2" s="2">
+      <c r="V2" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1085,7 +1059,7 @@
       <c r="U3" t="s">
         <v>28</v>
       </c>
-      <c r="V3" s="2">
+      <c r="V3" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1132,7 +1106,7 @@
       <c r="U4" t="s">
         <v>28</v>
       </c>
-      <c r="V4" s="2">
+      <c r="V4" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1179,7 +1153,7 @@
       <c r="U5" t="s">
         <v>28</v>
       </c>
-      <c r="V5" s="2">
+      <c r="V5" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1229,7 +1203,7 @@
       <c r="U6" t="s">
         <v>28</v>
       </c>
-      <c r="V6" s="2">
+      <c r="V6" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1255,7 +1229,7 @@
       <c r="G7" t="s">
         <v>42</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1285,7 +1259,7 @@
       <c r="U7" t="s">
         <v>28</v>
       </c>
-      <c r="V7" s="2">
+      <c r="V7" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -1332,7 +1306,7 @@
       <c r="U8" t="s">
         <v>28</v>
       </c>
-      <c r="V8" s="2">
+      <c r="V8" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1379,7 +1353,7 @@
       <c r="U9" t="s">
         <v>28</v>
       </c>
-      <c r="V9" s="2">
+      <c r="V9" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1426,7 +1400,7 @@
       <c r="U10" t="s">
         <v>28</v>
       </c>
-      <c r="V10" s="2">
+      <c r="V10" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1473,7 +1447,7 @@
       <c r="U11" t="s">
         <v>28</v>
       </c>
-      <c r="V11" s="2">
+      <c r="V11" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1499,7 +1473,7 @@
       <c r="G12" t="s">
         <v>42</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46079</v>
       </c>
       <c r="I12" t="s">
@@ -1532,7 +1506,7 @@
       <c r="U12" t="s">
         <v>180</v>
       </c>
-      <c r="V12" s="2">
+      <c r="V12" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1582,7 +1556,7 @@
       <c r="U13" t="s">
         <v>180</v>
       </c>
-      <c r="V13" s="2">
+      <c r="V13" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1632,7 +1606,7 @@
       <c r="U14" t="s">
         <v>180</v>
       </c>
-      <c r="V14" s="2">
+      <c r="V14" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1682,7 +1656,7 @@
       <c r="U15" t="s">
         <v>180</v>
       </c>
-      <c r="V15" s="2">
+      <c r="V15" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1732,7 +1706,7 @@
       <c r="U16" t="s">
         <v>180</v>
       </c>
-      <c r="V16" s="2">
+      <c r="V16" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1758,7 +1732,7 @@
       <c r="G17" t="s">
         <v>42</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46098</v>
       </c>
       <c r="I17" t="s">
@@ -1791,7 +1765,7 @@
       <c r="U17" t="s">
         <v>180</v>
       </c>
-      <c r="V17" s="2">
+      <c r="V17" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -1817,7 +1791,7 @@
       <c r="G18" t="s">
         <v>42</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46076</v>
       </c>
       <c r="I18" t="s">
@@ -1847,7 +1821,7 @@
       <c r="U18" t="s">
         <v>28</v>
       </c>
-      <c r="V18" s="2">
+      <c r="V18" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1873,7 +1847,7 @@
       <c r="G19" t="s">
         <v>42</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1903,7 +1877,7 @@
       <c r="U19" t="s">
         <v>28</v>
       </c>
-      <c r="V19" s="2">
+      <c r="V19" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1950,7 +1924,7 @@
       <c r="U20" t="s">
         <v>28</v>
       </c>
-      <c r="V20" s="2">
+      <c r="V20" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1997,7 +1971,7 @@
       <c r="U21" t="s">
         <v>28</v>
       </c>
-      <c r="V21" s="2">
+      <c r="V21" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2044,7 +2018,7 @@
       <c r="U22" t="s">
         <v>28</v>
       </c>
-      <c r="V22" s="2">
+      <c r="V22" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2091,7 +2065,7 @@
       <c r="U23" t="s">
         <v>28</v>
       </c>
-      <c r="V23" s="2">
+      <c r="V23" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2117,7 +2091,7 @@
       <c r="G24" t="s">
         <v>42</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>46119</v>
       </c>
       <c r="I24" t="s">
@@ -2150,7 +2124,7 @@
       <c r="U24" t="s">
         <v>180</v>
       </c>
-      <c r="V24" s="2">
+      <c r="V24" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2176,7 +2150,7 @@
       <c r="G25" t="s">
         <v>42</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>46121</v>
       </c>
       <c r="I25" t="s">
@@ -2206,7 +2180,7 @@
       <c r="U25" t="s">
         <v>28</v>
       </c>
-      <c r="V25" s="2">
+      <c r="V25" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2232,7 +2206,7 @@
       <c r="G26" t="s">
         <v>42</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>46076</v>
       </c>
       <c r="I26" t="s">
@@ -2262,7 +2236,7 @@
       <c r="U26" t="s">
         <v>28</v>
       </c>
-      <c r="V26" s="2">
+      <c r="V26" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -2312,7 +2286,7 @@
       <c r="U27" t="s">
         <v>180</v>
       </c>
-      <c r="V27" s="2">
+      <c r="V27" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2338,7 +2312,7 @@
       <c r="G28" t="s">
         <v>42</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>46199</v>
       </c>
       <c r="I28" t="s">
@@ -2371,7 +2345,7 @@
       <c r="U28" t="s">
         <v>180</v>
       </c>
-      <c r="V28" s="2">
+      <c r="V28" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2397,7 +2371,7 @@
       <c r="G29" t="s">
         <v>42</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2430,7 +2404,7 @@
       <c r="U29" t="s">
         <v>180</v>
       </c>
-      <c r="V29" s="2">
+      <c r="V29" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2456,7 +2430,7 @@
       <c r="G30" t="s">
         <v>42</v>
       </c>
-      <c r="H30" s="2">
+      <c r="H30" s="1">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2489,7 +2463,7 @@
       <c r="U30" t="s">
         <v>180</v>
       </c>
-      <c r="V30" s="2">
+      <c r="V30" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2515,7 +2489,7 @@
       <c r="G31" t="s">
         <v>42</v>
       </c>
-      <c r="H31" s="2">
+      <c r="H31" s="1">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2548,7 +2522,7 @@
       <c r="U31" t="s">
         <v>180</v>
       </c>
-      <c r="V31" s="2">
+      <c r="V31" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2598,7 +2572,7 @@
       <c r="U32" t="s">
         <v>180</v>
       </c>
-      <c r="V32" s="2">
+      <c r="V32" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2624,7 +2598,7 @@
       <c r="G33" t="s">
         <v>42</v>
       </c>
-      <c r="H33" s="2">
+      <c r="H33" s="1">
         <v>46191</v>
       </c>
       <c r="I33" t="s">
@@ -2657,7 +2631,7 @@
       <c r="U33" t="s">
         <v>180</v>
       </c>
-      <c r="V33" s="2">
+      <c r="V33" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2683,7 +2657,7 @@
       <c r="G34" t="s">
         <v>42</v>
       </c>
-      <c r="H34" s="2">
+      <c r="H34" s="1">
         <v>46119</v>
       </c>
       <c r="I34" t="s">
@@ -2713,7 +2687,7 @@
       <c r="U34" t="s">
         <v>180</v>
       </c>
-      <c r="V34" s="2">
+      <c r="V34" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2739,7 +2713,7 @@
       <c r="G35" t="s">
         <v>42</v>
       </c>
-      <c r="H35" s="2">
+      <c r="H35" s="1">
         <v>46213</v>
       </c>
       <c r="I35" t="s">
@@ -2769,7 +2743,7 @@
       <c r="U35" t="s">
         <v>28</v>
       </c>
-      <c r="V35" s="2">
+      <c r="V35" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -2795,7 +2769,7 @@
       <c r="G36" t="s">
         <v>42</v>
       </c>
-      <c r="H36" s="2">
+      <c r="H36" s="1">
         <v>46175</v>
       </c>
       <c r="I36" t="s">
@@ -2825,7 +2799,7 @@
       <c r="U36" t="s">
         <v>28</v>
       </c>
-      <c r="V36" s="2">
+      <c r="V36" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2851,7 +2825,7 @@
       <c r="G37" t="s">
         <v>42</v>
       </c>
-      <c r="H37" s="2">
+      <c r="H37" s="1">
         <v>46213</v>
       </c>
       <c r="I37" t="s">
@@ -2881,7 +2855,7 @@
       <c r="U37" t="s">
         <v>28</v>
       </c>
-      <c r="V37" s="2">
+      <c r="V37" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -2907,7 +2881,7 @@
       <c r="G38" t="s">
         <v>42</v>
       </c>
-      <c r="H38" s="2">
+      <c r="H38" s="1">
         <v>46199</v>
       </c>
       <c r="I38" t="s">
@@ -2937,7 +2911,7 @@
       <c r="U38" t="s">
         <v>28</v>
       </c>
-      <c r="V38" s="2">
+      <c r="V38" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2963,7 +2937,7 @@
       <c r="G39" t="s">
         <v>42</v>
       </c>
-      <c r="H39" s="2">
+      <c r="H39" s="1">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -2993,7 +2967,7 @@
       <c r="U39" t="s">
         <v>28</v>
       </c>
-      <c r="V39" s="2">
+      <c r="V39" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3019,7 +2993,7 @@
       <c r="G40" t="s">
         <v>42</v>
       </c>
-      <c r="H40" s="2">
+      <c r="H40" s="1">
         <v>46204</v>
       </c>
       <c r="I40" t="s">
@@ -3049,7 +3023,7 @@
       <c r="U40" t="s">
         <v>28</v>
       </c>
-      <c r="V40" s="2">
+      <c r="V40" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3075,7 +3049,7 @@
       <c r="G41" t="s">
         <v>42</v>
       </c>
-      <c r="H41" s="2">
+      <c r="H41" s="1">
         <v>46244</v>
       </c>
       <c r="I41" t="s">
@@ -3105,7 +3079,7 @@
       <c r="U41" t="s">
         <v>28</v>
       </c>
-      <c r="V41" s="2">
+      <c r="V41" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3149,7 +3123,7 @@
       <c r="U42" t="s">
         <v>28</v>
       </c>
-      <c r="V42" s="2">
+      <c r="V42" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3175,7 +3149,7 @@
       <c r="G43" t="s">
         <v>42</v>
       </c>
-      <c r="H43" s="2">
+      <c r="H43" s="1">
         <v>46191</v>
       </c>
       <c r="I43" t="s">
@@ -3205,7 +3179,7 @@
       <c r="U43" t="s">
         <v>28</v>
       </c>
-      <c r="V43" s="2">
+      <c r="V43" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3231,7 +3205,7 @@
       <c r="G44" t="s">
         <v>42</v>
       </c>
-      <c r="H44" s="2">
+      <c r="H44" s="1">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
@@ -3261,7 +3235,7 @@
       <c r="U44" t="s">
         <v>28</v>
       </c>
-      <c r="V44" s="2">
+      <c r="V44" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3287,7 +3261,7 @@
       <c r="G45" t="s">
         <v>42</v>
       </c>
-      <c r="H45" s="2">
+      <c r="H45" s="1">
         <v>46213</v>
       </c>
       <c r="I45" t="s">
@@ -3320,7 +3294,7 @@
       <c r="U45" t="s">
         <v>180</v>
       </c>
-      <c r="V45" s="2">
+      <c r="V45" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3346,7 +3320,7 @@
       <c r="G46" t="s">
         <v>42</v>
       </c>
-      <c r="H46" s="2">
+      <c r="H46" s="1">
         <v>46210</v>
       </c>
       <c r="I46" t="s">
@@ -3376,7 +3350,7 @@
       <c r="U46" t="s">
         <v>180</v>
       </c>
-      <c r="V46" s="2">
+      <c r="V46" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3423,7 +3397,7 @@
       <c r="U47" t="s">
         <v>28</v>
       </c>
-      <c r="V47" s="2">
+      <c r="V47" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3473,7 +3447,7 @@
       <c r="U48" t="s">
         <v>180</v>
       </c>
-      <c r="V48" s="2">
+      <c r="V48" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3499,7 +3473,7 @@
       <c r="G49" t="s">
         <v>42</v>
       </c>
-      <c r="H49" s="2">
+      <c r="H49" s="1">
         <v>46176</v>
       </c>
       <c r="I49" t="s">
@@ -3532,7 +3506,7 @@
       <c r="U49" t="s">
         <v>180</v>
       </c>
-      <c r="V49" s="2">
+      <c r="V49" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3585,7 +3559,7 @@
       <c r="U50" t="s">
         <v>180</v>
       </c>
-      <c r="V50" s="2">
+      <c r="V50" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3638,7 +3612,7 @@
       <c r="U51" t="s">
         <v>180</v>
       </c>
-      <c r="V51" s="2">
+      <c r="V51" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3688,7 +3662,7 @@
       <c r="U52" t="s">
         <v>180</v>
       </c>
-      <c r="V52" s="2">
+      <c r="V52" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3714,7 +3688,7 @@
       <c r="G53" t="s">
         <v>42</v>
       </c>
-      <c r="H53" s="2">
+      <c r="H53" s="1">
         <v>46227</v>
       </c>
       <c r="I53" t="s">
@@ -3744,7 +3718,7 @@
       <c r="U53" t="s">
         <v>180</v>
       </c>
-      <c r="V53" s="2">
+      <c r="V53" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3794,7 +3768,7 @@
       <c r="U54" t="s">
         <v>180</v>
       </c>
-      <c r="V54" s="2">
+      <c r="V54" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -3844,7 +3818,7 @@
       <c r="U55" t="s">
         <v>180</v>
       </c>
-      <c r="V55" s="2">
+      <c r="V55" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3894,7 +3868,7 @@
       <c r="U56" t="s">
         <v>180</v>
       </c>
-      <c r="V56" s="2">
+      <c r="V56" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3938,7 +3912,7 @@
       <c r="U57" t="s">
         <v>180</v>
       </c>
-      <c r="V57" s="2">
+      <c r="V57" s="1">
         <v>46049</v>
       </c>
     </row>
@@ -4064,7 +4038,7 @@
       <c r="U60" t="s">
         <v>180</v>
       </c>
-      <c r="V60" s="2">
+      <c r="V60" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4108,7 +4082,7 @@
       <c r="U61" t="s">
         <v>180</v>
       </c>
-      <c r="V61" s="2">
+      <c r="V61" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4152,7 +4126,7 @@
       <c r="U62" t="s">
         <v>180</v>
       </c>
-      <c r="V62" s="2">
+      <c r="V62" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4196,7 +4170,7 @@
       <c r="U63" t="s">
         <v>180</v>
       </c>
-      <c r="V63" s="2">
+      <c r="V63" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4240,7 +4214,7 @@
       <c r="U64" t="s">
         <v>180</v>
       </c>
-      <c r="V64" s="2">
+      <c r="V64" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4284,7 +4258,7 @@
       <c r="U65" t="s">
         <v>180</v>
       </c>
-      <c r="V65" s="2">
+      <c r="V65" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4328,7 +4302,7 @@
       <c r="U66" t="s">
         <v>28</v>
       </c>
-      <c r="V66" s="2">
+      <c r="V66" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4375,7 +4349,7 @@
       <c r="U67" t="s">
         <v>28</v>
       </c>
-      <c r="V67" s="2">
+      <c r="V67" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4425,7 +4399,7 @@
       <c r="U68" t="s">
         <v>180</v>
       </c>
-      <c r="V68" s="2">
+      <c r="V68" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -4469,7 +4443,7 @@
       <c r="U69" t="s">
         <v>28</v>
       </c>
-      <c r="V69" s="2">
+      <c r="V69" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -4513,7 +4487,7 @@
       <c r="U70" t="s">
         <v>180</v>
       </c>
-      <c r="V70" s="2">
+      <c r="V70" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4557,7 +4531,7 @@
       <c r="U71" t="s">
         <v>180</v>
       </c>
-      <c r="V71" s="2">
+      <c r="V71" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4601,7 +4575,7 @@
       <c r="U72" t="s">
         <v>180</v>
       </c>
-      <c r="V72" s="2">
+      <c r="V72" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4645,7 +4619,7 @@
       <c r="U73" t="s">
         <v>180</v>
       </c>
-      <c r="V73" s="2">
+      <c r="V73" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4689,7 +4663,7 @@
       <c r="U74" t="s">
         <v>180</v>
       </c>
-      <c r="V74" s="2">
+      <c r="V74" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4736,7 +4710,7 @@
       <c r="U75" t="s">
         <v>28</v>
       </c>
-      <c r="V75" s="2">
+      <c r="V75" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -4786,7 +4760,7 @@
       <c r="U76" t="s">
         <v>180</v>
       </c>
-      <c r="V76" s="2">
+      <c r="V76" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4836,7 +4810,7 @@
       <c r="U77" t="s">
         <v>180</v>
       </c>
-      <c r="V77" s="2">
+      <c r="V77" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4886,7 +4860,7 @@
       <c r="U78" t="s">
         <v>28</v>
       </c>
-      <c r="V78" s="2">
+      <c r="V78" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4936,7 +4910,7 @@
       <c r="U79" t="s">
         <v>28</v>
       </c>
-      <c r="V79" s="2">
+      <c r="V79" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4986,7 +4960,7 @@
       <c r="U80" t="s">
         <v>28</v>
       </c>
-      <c r="V80" s="2">
+      <c r="V80" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5030,7 +5004,7 @@
       <c r="U81" t="s">
         <v>28</v>
       </c>
-      <c r="V81" s="2">
+      <c r="V81" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5080,7 +5054,7 @@
       <c r="U82" t="s">
         <v>180</v>
       </c>
-      <c r="V82" s="2">
+      <c r="V82" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5124,7 +5098,7 @@
       <c r="U83" t="s">
         <v>28</v>
       </c>
-      <c r="V83" s="2">
+      <c r="V83" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -5168,7 +5142,7 @@
       <c r="U84" t="s">
         <v>28</v>
       </c>
-      <c r="V84" s="2">
+      <c r="V84" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5309,7 +5283,7 @@
       <c r="U87" t="s">
         <v>28</v>
       </c>
-      <c r="V87" s="2">
+      <c r="V87" s="1">
         <v>46291</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (08/09/2026 13:59)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -232,7 +232,7 @@
     <t>ATENDER</t>
   </si>
   <si>
-    <t>Atender AGO</t>
+    <t>Remanejar</t>
   </si>
   <si>
     <t>Atender SET</t>
@@ -247,7 +247,7 @@
     <t>ATENDER com 20XV</t>
   </si>
   <si>
-    <t>Atender DEZ</t>
+    <t>Remanejar tarefa módulo extra</t>
   </si>
   <si>
     <t>LIVRE</t>
@@ -566,8 +566,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -583,7 +591,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -591,12 +599,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -896,70 +922,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1012,7 +1038,7 @@
       <c r="U2" t="s">
         <v>180</v>
       </c>
-      <c r="V2" s="1">
+      <c r="V2" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -1059,7 +1085,7 @@
       <c r="U3" t="s">
         <v>28</v>
       </c>
-      <c r="V3" s="1">
+      <c r="V3" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1106,7 +1132,7 @@
       <c r="U4" t="s">
         <v>28</v>
       </c>
-      <c r="V4" s="1">
+      <c r="V4" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1153,7 +1179,7 @@
       <c r="U5" t="s">
         <v>28</v>
       </c>
-      <c r="V5" s="1">
+      <c r="V5" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1203,7 +1229,7 @@
       <c r="U6" t="s">
         <v>28</v>
       </c>
-      <c r="V6" s="1">
+      <c r="V6" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1229,7 +1255,7 @@
       <c r="G7" t="s">
         <v>42</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1259,7 +1285,7 @@
       <c r="U7" t="s">
         <v>28</v>
       </c>
-      <c r="V7" s="1">
+      <c r="V7" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -1306,7 +1332,7 @@
       <c r="U8" t="s">
         <v>28</v>
       </c>
-      <c r="V8" s="1">
+      <c r="V8" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1353,7 +1379,7 @@
       <c r="U9" t="s">
         <v>28</v>
       </c>
-      <c r="V9" s="1">
+      <c r="V9" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1400,7 +1426,7 @@
       <c r="U10" t="s">
         <v>28</v>
       </c>
-      <c r="V10" s="1">
+      <c r="V10" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1447,7 +1473,7 @@
       <c r="U11" t="s">
         <v>28</v>
       </c>
-      <c r="V11" s="1">
+      <c r="V11" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -1473,7 +1499,7 @@
       <c r="G12" t="s">
         <v>42</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46079</v>
       </c>
       <c r="I12" t="s">
@@ -1506,7 +1532,7 @@
       <c r="U12" t="s">
         <v>180</v>
       </c>
-      <c r="V12" s="1">
+      <c r="V12" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1556,7 +1582,7 @@
       <c r="U13" t="s">
         <v>180</v>
       </c>
-      <c r="V13" s="1">
+      <c r="V13" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1606,7 +1632,7 @@
       <c r="U14" t="s">
         <v>180</v>
       </c>
-      <c r="V14" s="1">
+      <c r="V14" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1656,7 +1682,7 @@
       <c r="U15" t="s">
         <v>180</v>
       </c>
-      <c r="V15" s="1">
+      <c r="V15" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -1706,7 +1732,7 @@
       <c r="U16" t="s">
         <v>180</v>
       </c>
-      <c r="V16" s="1">
+      <c r="V16" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -1732,7 +1758,7 @@
       <c r="G17" t="s">
         <v>42</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46098</v>
       </c>
       <c r="I17" t="s">
@@ -1765,7 +1791,7 @@
       <c r="U17" t="s">
         <v>180</v>
       </c>
-      <c r="V17" s="1">
+      <c r="V17" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -1791,7 +1817,7 @@
       <c r="G18" t="s">
         <v>42</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46076</v>
       </c>
       <c r="I18" t="s">
@@ -1821,7 +1847,7 @@
       <c r="U18" t="s">
         <v>28</v>
       </c>
-      <c r="V18" s="1">
+      <c r="V18" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1847,7 +1873,7 @@
       <c r="G19" t="s">
         <v>42</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1877,7 +1903,7 @@
       <c r="U19" t="s">
         <v>28</v>
       </c>
-      <c r="V19" s="1">
+      <c r="V19" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -1924,7 +1950,7 @@
       <c r="U20" t="s">
         <v>28</v>
       </c>
-      <c r="V20" s="1">
+      <c r="V20" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -1971,7 +1997,7 @@
       <c r="U21" t="s">
         <v>28</v>
       </c>
-      <c r="V21" s="1">
+      <c r="V21" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2018,7 +2044,7 @@
       <c r="U22" t="s">
         <v>28</v>
       </c>
-      <c r="V22" s="1">
+      <c r="V22" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2065,7 +2091,7 @@
       <c r="U23" t="s">
         <v>28</v>
       </c>
-      <c r="V23" s="1">
+      <c r="V23" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -2091,7 +2117,7 @@
       <c r="G24" t="s">
         <v>42</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>46119</v>
       </c>
       <c r="I24" t="s">
@@ -2124,7 +2150,7 @@
       <c r="U24" t="s">
         <v>180</v>
       </c>
-      <c r="V24" s="1">
+      <c r="V24" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2150,7 +2176,7 @@
       <c r="G25" t="s">
         <v>42</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>46121</v>
       </c>
       <c r="I25" t="s">
@@ -2180,7 +2206,7 @@
       <c r="U25" t="s">
         <v>28</v>
       </c>
-      <c r="V25" s="1">
+      <c r="V25" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2206,7 +2232,7 @@
       <c r="G26" t="s">
         <v>42</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>46076</v>
       </c>
       <c r="I26" t="s">
@@ -2236,7 +2262,7 @@
       <c r="U26" t="s">
         <v>28</v>
       </c>
-      <c r="V26" s="1">
+      <c r="V26" s="2">
         <v>46079</v>
       </c>
     </row>
@@ -2286,7 +2312,7 @@
       <c r="U27" t="s">
         <v>180</v>
       </c>
-      <c r="V27" s="1">
+      <c r="V27" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -2312,7 +2338,7 @@
       <c r="G28" t="s">
         <v>42</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>46199</v>
       </c>
       <c r="I28" t="s">
@@ -2345,7 +2371,7 @@
       <c r="U28" t="s">
         <v>180</v>
       </c>
-      <c r="V28" s="1">
+      <c r="V28" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2371,7 +2397,7 @@
       <c r="G29" t="s">
         <v>42</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2404,7 +2430,7 @@
       <c r="U29" t="s">
         <v>180</v>
       </c>
-      <c r="V29" s="1">
+      <c r="V29" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2430,7 +2456,7 @@
       <c r="G30" t="s">
         <v>42</v>
       </c>
-      <c r="H30" s="1">
+      <c r="H30" s="2">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2463,7 +2489,7 @@
       <c r="U30" t="s">
         <v>180</v>
       </c>
-      <c r="V30" s="1">
+      <c r="V30" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2489,7 +2515,7 @@
       <c r="G31" t="s">
         <v>42</v>
       </c>
-      <c r="H31" s="1">
+      <c r="H31" s="2">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2522,7 +2548,7 @@
       <c r="U31" t="s">
         <v>180</v>
       </c>
-      <c r="V31" s="1">
+      <c r="V31" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2546,7 +2572,7 @@
         <v>30</v>
       </c>
       <c r="K32" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="N32" t="s">
         <v>84</v>
@@ -2572,7 +2598,7 @@
       <c r="U32" t="s">
         <v>180</v>
       </c>
-      <c r="V32" s="1">
+      <c r="V32" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -2598,7 +2624,7 @@
       <c r="G33" t="s">
         <v>42</v>
       </c>
-      <c r="H33" s="1">
+      <c r="H33" s="2">
         <v>46191</v>
       </c>
       <c r="I33" t="s">
@@ -2631,7 +2657,7 @@
       <c r="U33" t="s">
         <v>180</v>
       </c>
-      <c r="V33" s="1">
+      <c r="V33" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2657,7 +2683,7 @@
       <c r="G34" t="s">
         <v>42</v>
       </c>
-      <c r="H34" s="1">
+      <c r="H34" s="2">
         <v>46119</v>
       </c>
       <c r="I34" t="s">
@@ -2687,7 +2713,7 @@
       <c r="U34" t="s">
         <v>180</v>
       </c>
-      <c r="V34" s="1">
+      <c r="V34" s="2">
         <v>46138</v>
       </c>
     </row>
@@ -2713,7 +2739,7 @@
       <c r="G35" t="s">
         <v>42</v>
       </c>
-      <c r="H35" s="1">
+      <c r="H35" s="2">
         <v>46213</v>
       </c>
       <c r="I35" t="s">
@@ -2743,7 +2769,7 @@
       <c r="U35" t="s">
         <v>28</v>
       </c>
-      <c r="V35" s="1">
+      <c r="V35" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -2769,7 +2795,7 @@
       <c r="G36" t="s">
         <v>42</v>
       </c>
-      <c r="H36" s="1">
+      <c r="H36" s="2">
         <v>46175</v>
       </c>
       <c r="I36" t="s">
@@ -2799,7 +2825,7 @@
       <c r="U36" t="s">
         <v>28</v>
       </c>
-      <c r="V36" s="1">
+      <c r="V36" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2825,7 +2851,7 @@
       <c r="G37" t="s">
         <v>42</v>
       </c>
-      <c r="H37" s="1">
+      <c r="H37" s="2">
         <v>46213</v>
       </c>
       <c r="I37" t="s">
@@ -2855,7 +2881,7 @@
       <c r="U37" t="s">
         <v>28</v>
       </c>
-      <c r="V37" s="1">
+      <c r="V37" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -2881,7 +2907,7 @@
       <c r="G38" t="s">
         <v>42</v>
       </c>
-      <c r="H38" s="1">
+      <c r="H38" s="2">
         <v>46199</v>
       </c>
       <c r="I38" t="s">
@@ -2911,7 +2937,7 @@
       <c r="U38" t="s">
         <v>28</v>
       </c>
-      <c r="V38" s="1">
+      <c r="V38" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2937,7 +2963,7 @@
       <c r="G39" t="s">
         <v>42</v>
       </c>
-      <c r="H39" s="1">
+      <c r="H39" s="2">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -2967,7 +2993,7 @@
       <c r="U39" t="s">
         <v>28</v>
       </c>
-      <c r="V39" s="1">
+      <c r="V39" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -2993,7 +3019,7 @@
       <c r="G40" t="s">
         <v>42</v>
       </c>
-      <c r="H40" s="1">
+      <c r="H40" s="2">
         <v>46204</v>
       </c>
       <c r="I40" t="s">
@@ -3023,7 +3049,7 @@
       <c r="U40" t="s">
         <v>28</v>
       </c>
-      <c r="V40" s="1">
+      <c r="V40" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3049,7 +3075,7 @@
       <c r="G41" t="s">
         <v>42</v>
       </c>
-      <c r="H41" s="1">
+      <c r="H41" s="2">
         <v>46244</v>
       </c>
       <c r="I41" t="s">
@@ -3079,7 +3105,7 @@
       <c r="U41" t="s">
         <v>28</v>
       </c>
-      <c r="V41" s="1">
+      <c r="V41" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3123,7 +3149,7 @@
       <c r="U42" t="s">
         <v>28</v>
       </c>
-      <c r="V42" s="1">
+      <c r="V42" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3149,7 +3175,7 @@
       <c r="G43" t="s">
         <v>42</v>
       </c>
-      <c r="H43" s="1">
+      <c r="H43" s="2">
         <v>46191</v>
       </c>
       <c r="I43" t="s">
@@ -3179,7 +3205,7 @@
       <c r="U43" t="s">
         <v>28</v>
       </c>
-      <c r="V43" s="1">
+      <c r="V43" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3205,7 +3231,7 @@
       <c r="G44" t="s">
         <v>42</v>
       </c>
-      <c r="H44" s="1">
+      <c r="H44" s="2">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
@@ -3235,7 +3261,7 @@
       <c r="U44" t="s">
         <v>28</v>
       </c>
-      <c r="V44" s="1">
+      <c r="V44" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3261,7 +3287,7 @@
       <c r="G45" t="s">
         <v>42</v>
       </c>
-      <c r="H45" s="1">
+      <c r="H45" s="2">
         <v>46213</v>
       </c>
       <c r="I45" t="s">
@@ -3294,7 +3320,7 @@
       <c r="U45" t="s">
         <v>180</v>
       </c>
-      <c r="V45" s="1">
+      <c r="V45" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3320,7 +3346,7 @@
       <c r="G46" t="s">
         <v>42</v>
       </c>
-      <c r="H46" s="1">
+      <c r="H46" s="2">
         <v>46210</v>
       </c>
       <c r="I46" t="s">
@@ -3350,7 +3376,7 @@
       <c r="U46" t="s">
         <v>180</v>
       </c>
-      <c r="V46" s="1">
+      <c r="V46" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3397,7 +3423,7 @@
       <c r="U47" t="s">
         <v>28</v>
       </c>
-      <c r="V47" s="1">
+      <c r="V47" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3447,7 +3473,7 @@
       <c r="U48" t="s">
         <v>180</v>
       </c>
-      <c r="V48" s="1">
+      <c r="V48" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3473,7 +3499,7 @@
       <c r="G49" t="s">
         <v>42</v>
       </c>
-      <c r="H49" s="1">
+      <c r="H49" s="2">
         <v>46176</v>
       </c>
       <c r="I49" t="s">
@@ -3506,7 +3532,7 @@
       <c r="U49" t="s">
         <v>180</v>
       </c>
-      <c r="V49" s="1">
+      <c r="V49" s="2">
         <v>46199</v>
       </c>
     </row>
@@ -3533,7 +3559,7 @@
         <v>66</v>
       </c>
       <c r="K50" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="N50" t="s">
         <v>84</v>
@@ -3559,7 +3585,7 @@
       <c r="U50" t="s">
         <v>180</v>
       </c>
-      <c r="V50" s="1">
+      <c r="V50" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -3586,7 +3612,7 @@
         <v>66</v>
       </c>
       <c r="K51" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="N51" t="s">
         <v>84</v>
@@ -3612,7 +3638,7 @@
       <c r="U51" t="s">
         <v>180</v>
       </c>
-      <c r="V51" s="1">
+      <c r="V51" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -3662,7 +3688,7 @@
       <c r="U52" t="s">
         <v>180</v>
       </c>
-      <c r="V52" s="1">
+      <c r="V52" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3688,7 +3714,7 @@
       <c r="G53" t="s">
         <v>42</v>
       </c>
-      <c r="H53" s="1">
+      <c r="H53" s="2">
         <v>46227</v>
       </c>
       <c r="I53" t="s">
@@ -3718,7 +3744,7 @@
       <c r="U53" t="s">
         <v>180</v>
       </c>
-      <c r="V53" s="1">
+      <c r="V53" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -3768,7 +3794,7 @@
       <c r="U54" t="s">
         <v>180</v>
       </c>
-      <c r="V54" s="1">
+      <c r="V54" s="2">
         <v>46352</v>
       </c>
     </row>
@@ -3818,7 +3844,7 @@
       <c r="U55" t="s">
         <v>180</v>
       </c>
-      <c r="V55" s="1">
+      <c r="V55" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3868,7 +3894,7 @@
       <c r="U56" t="s">
         <v>180</v>
       </c>
-      <c r="V56" s="1">
+      <c r="V56" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -3912,7 +3938,7 @@
       <c r="U57" t="s">
         <v>180</v>
       </c>
-      <c r="V57" s="1">
+      <c r="V57" s="2">
         <v>46049</v>
       </c>
     </row>
@@ -4038,7 +4064,7 @@
       <c r="U60" t="s">
         <v>180</v>
       </c>
-      <c r="V60" s="1">
+      <c r="V60" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4082,7 +4108,7 @@
       <c r="U61" t="s">
         <v>180</v>
       </c>
-      <c r="V61" s="1">
+      <c r="V61" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4126,7 +4152,7 @@
       <c r="U62" t="s">
         <v>180</v>
       </c>
-      <c r="V62" s="1">
+      <c r="V62" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4170,7 +4196,7 @@
       <c r="U63" t="s">
         <v>180</v>
       </c>
-      <c r="V63" s="1">
+      <c r="V63" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4214,7 +4240,7 @@
       <c r="U64" t="s">
         <v>180</v>
       </c>
-      <c r="V64" s="1">
+      <c r="V64" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4258,7 +4284,7 @@
       <c r="U65" t="s">
         <v>180</v>
       </c>
-      <c r="V65" s="1">
+      <c r="V65" s="2">
         <v>46107</v>
       </c>
     </row>
@@ -4302,7 +4328,7 @@
       <c r="U66" t="s">
         <v>28</v>
       </c>
-      <c r="V66" s="1">
+      <c r="V66" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4349,7 +4375,7 @@
       <c r="U67" t="s">
         <v>28</v>
       </c>
-      <c r="V67" s="1">
+      <c r="V67" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4399,7 +4425,7 @@
       <c r="U68" t="s">
         <v>180</v>
       </c>
-      <c r="V68" s="1">
+      <c r="V68" s="2">
         <v>46229</v>
       </c>
     </row>
@@ -4443,7 +4469,7 @@
       <c r="U69" t="s">
         <v>28</v>
       </c>
-      <c r="V69" s="1">
+      <c r="V69" s="2">
         <v>46260</v>
       </c>
     </row>
@@ -4487,7 +4513,7 @@
       <c r="U70" t="s">
         <v>180</v>
       </c>
-      <c r="V70" s="1">
+      <c r="V70" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4531,7 +4557,7 @@
       <c r="U71" t="s">
         <v>180</v>
       </c>
-      <c r="V71" s="1">
+      <c r="V71" s="2">
         <v>46168</v>
       </c>
     </row>
@@ -4575,7 +4601,7 @@
       <c r="U72" t="s">
         <v>180</v>
       </c>
-      <c r="V72" s="1">
+      <c r="V72" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4619,7 +4645,7 @@
       <c r="U73" t="s">
         <v>180</v>
       </c>
-      <c r="V73" s="1">
+      <c r="V73" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4663,7 +4689,7 @@
       <c r="U74" t="s">
         <v>180</v>
       </c>
-      <c r="V74" s="1">
+      <c r="V74" s="2">
         <v>46291</v>
       </c>
     </row>
@@ -4710,7 +4736,7 @@
       <c r="U75" t="s">
         <v>28</v>
       </c>
-      <c r="V75" s="1">
+      <c r="V75" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -4760,7 +4786,7 @@
       <c r="U76" t="s">
         <v>180</v>
       </c>
-      <c r="V76" s="1">
+      <c r="V76" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4810,7 +4836,7 @@
       <c r="U77" t="s">
         <v>180</v>
       </c>
-      <c r="V77" s="1">
+      <c r="V77" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4860,7 +4886,7 @@
       <c r="U78" t="s">
         <v>28</v>
       </c>
-      <c r="V78" s="1">
+      <c r="V78" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4910,7 +4936,7 @@
       <c r="U79" t="s">
         <v>28</v>
       </c>
-      <c r="V79" s="1">
+      <c r="V79" s="2">
         <v>46381</v>
       </c>
     </row>
@@ -4960,7 +4986,7 @@
       <c r="U80" t="s">
         <v>28</v>
       </c>
-      <c r="V80" s="1">
+      <c r="V80" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5004,7 +5030,7 @@
       <c r="U81" t="s">
         <v>28</v>
       </c>
-      <c r="V81" s="1">
+      <c r="V81" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5054,7 +5080,7 @@
       <c r="U82" t="s">
         <v>180</v>
       </c>
-      <c r="V82" s="1">
+      <c r="V82" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5098,7 +5124,7 @@
       <c r="U83" t="s">
         <v>28</v>
       </c>
-      <c r="V83" s="1">
+      <c r="V83" s="2">
         <v>46321</v>
       </c>
     </row>
@@ -5142,7 +5168,7 @@
       <c r="U84" t="s">
         <v>28</v>
       </c>
-      <c r="V84" s="1">
+      <c r="V84" s="2">
         <v>46382</v>
       </c>
     </row>
@@ -5283,7 +5309,7 @@
       <c r="U87" t="s">
         <v>28</v>
       </c>
-      <c r="V87" s="1">
+      <c r="V87" s="2">
         <v>46291</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (08/09/2026 15:18)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1130" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1130" uniqueCount="180">
   <si>
     <t>linha</t>
   </si>
@@ -223,10 +223,7 @@
     <t>e-mail 12/08</t>
   </si>
   <si>
-    <t>REMANEJAR</t>
-  </si>
-  <si>
-    <t>ATENDER R$ 621.454,453</t>
+    <t>REMANEJAR P/ CABW 30</t>
   </si>
   <si>
     <t>ATENDER</t>
@@ -1012,31 +1009,31 @@
         <v>69</v>
       </c>
       <c r="L2" t="s">
+        <v>77</v>
+      </c>
+      <c r="N2" t="s">
         <v>78</v>
       </c>
-      <c r="N2" t="s">
-        <v>79</v>
-      </c>
       <c r="O2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="P2">
         <v>135000</v>
       </c>
       <c r="Q2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="R2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="S2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="U2" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="V2" s="2">
         <v>46229</v>
@@ -1062,25 +1059,25 @@
         <v>30</v>
       </c>
       <c r="N3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="P3">
         <v>400000</v>
       </c>
       <c r="Q3" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="R3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="S3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="U3" t="s">
         <v>28</v>
@@ -1112,22 +1109,22 @@
         <v>41</v>
       </c>
       <c r="N4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="O4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="Q4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="R4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="S4" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T4" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="U4" t="s">
         <v>28</v>
@@ -1156,25 +1153,25 @@
         <v>30</v>
       </c>
       <c r="N5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="O5" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="P5">
         <v>384180</v>
       </c>
       <c r="Q5" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="R5" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="S5" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T5" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="U5" t="s">
         <v>28</v>
@@ -1203,28 +1200,28 @@
         <v>30</v>
       </c>
       <c r="L6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="N6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="P6">
         <v>563000</v>
       </c>
       <c r="Q6" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="R6" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="S6" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T6" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="U6" t="s">
         <v>28</v>
@@ -1262,25 +1259,25 @@
         <v>45</v>
       </c>
       <c r="N7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="P7">
         <v>3799999.6</v>
       </c>
       <c r="Q7" t="s">
+        <v>166</v>
+      </c>
+      <c r="R7" t="s">
         <v>167</v>
       </c>
-      <c r="R7" t="s">
-        <v>168</v>
-      </c>
       <c r="S7" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T7" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="U7" t="s">
         <v>28</v>
@@ -1309,25 +1306,25 @@
         <v>30</v>
       </c>
       <c r="N8" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="O8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="P8">
         <v>430000</v>
       </c>
       <c r="Q8" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="R8" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="S8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T8" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="U8" t="s">
         <v>28</v>
@@ -1356,25 +1353,25 @@
         <v>30</v>
       </c>
       <c r="N9" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="O9" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="P9">
         <v>60000</v>
       </c>
       <c r="Q9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="R9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="S9" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T9" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="U9" t="s">
         <v>28</v>
@@ -1403,25 +1400,25 @@
         <v>30</v>
       </c>
       <c r="N10" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O10" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="P10">
         <v>200000</v>
       </c>
       <c r="Q10" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="R10" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="S10" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T10" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="U10" t="s">
         <v>28</v>
@@ -1450,25 +1447,25 @@
         <v>30</v>
       </c>
       <c r="N11" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O11" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="P11">
         <v>320000</v>
       </c>
       <c r="Q11" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="R11" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="S11" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T11" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="U11" t="s">
         <v>28</v>
@@ -1509,28 +1506,28 @@
         <v>62</v>
       </c>
       <c r="N12" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O12" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="P12">
         <v>1187433.02</v>
       </c>
       <c r="Q12" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="R12" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="S12" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T12" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="U12" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="V12" s="2">
         <v>46079</v>
@@ -1559,28 +1556,28 @@
         <v>70</v>
       </c>
       <c r="N13" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O13" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="P13">
         <v>1000000</v>
       </c>
       <c r="Q13" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="R13" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="S13" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T13" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="U13" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="V13" s="2">
         <v>46352</v>
@@ -1606,31 +1603,31 @@
         <v>30</v>
       </c>
       <c r="K14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="N14" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O14" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="P14">
         <v>1000000</v>
       </c>
       <c r="Q14" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="R14" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="S14" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T14" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="U14" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="V14" s="2">
         <v>46352</v>
@@ -1656,31 +1653,31 @@
         <v>30</v>
       </c>
       <c r="K15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="N15" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O15" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="P15">
         <v>1000000</v>
       </c>
       <c r="Q15" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="R15" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="S15" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T15" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="U15" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="V15" s="2">
         <v>46352</v>
@@ -1706,31 +1703,31 @@
         <v>30</v>
       </c>
       <c r="K16" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="N16" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="O16" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="P16">
         <v>100000</v>
       </c>
       <c r="Q16" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="R16" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="S16" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T16" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="U16" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="V16" s="2">
         <v>46229</v>
@@ -1768,28 +1765,28 @@
         <v>62</v>
       </c>
       <c r="N17" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O17" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="P17">
         <v>1770880.5</v>
       </c>
       <c r="Q17" t="s">
+        <v>166</v>
+      </c>
+      <c r="R17" t="s">
         <v>167</v>
       </c>
-      <c r="R17" t="s">
-        <v>168</v>
-      </c>
       <c r="S17" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T17" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="U17" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="V17" s="2">
         <v>46107</v>
@@ -1824,25 +1821,25 @@
         <v>48</v>
       </c>
       <c r="N18" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="O18" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="P18">
         <v>350000</v>
       </c>
       <c r="Q18" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="R18" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="S18" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T18" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="U18" t="s">
         <v>28</v>
@@ -1880,25 +1877,25 @@
         <v>48</v>
       </c>
       <c r="N19" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="O19" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="P19">
         <v>350000</v>
       </c>
       <c r="Q19" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="R19" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="S19" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T19" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="U19" t="s">
         <v>28</v>
@@ -1927,25 +1924,25 @@
         <v>30</v>
       </c>
       <c r="N20" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="O20" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="P20">
         <v>1000000</v>
       </c>
       <c r="Q20" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="R20" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="S20" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T20" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="U20" t="s">
         <v>28</v>
@@ -1974,25 +1971,25 @@
         <v>30</v>
       </c>
       <c r="N21" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O21" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="P21">
         <v>400000</v>
       </c>
       <c r="Q21" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="R21" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="S21" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T21" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="U21" t="s">
         <v>28</v>
@@ -2021,25 +2018,25 @@
         <v>30</v>
       </c>
       <c r="N22" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="O22" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="P22">
         <v>120000</v>
       </c>
       <c r="Q22" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="R22" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="S22" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T22" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="U22" t="s">
         <v>28</v>
@@ -2068,25 +2065,25 @@
         <v>30</v>
       </c>
       <c r="N23" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="O23" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="P23">
         <v>80000</v>
       </c>
       <c r="Q23" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="R23" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="S23" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T23" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="U23" t="s">
         <v>28</v>
@@ -2127,28 +2124,28 @@
         <v>63</v>
       </c>
       <c r="N24" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O24" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="P24">
         <v>1704503</v>
       </c>
       <c r="Q24" t="s">
+        <v>166</v>
+      </c>
+      <c r="R24" t="s">
         <v>167</v>
       </c>
-      <c r="R24" t="s">
-        <v>168</v>
-      </c>
       <c r="S24" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T24" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="U24" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="V24" s="2">
         <v>46138</v>
@@ -2183,25 +2180,25 @@
         <v>50</v>
       </c>
       <c r="N25" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O25" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="P25">
         <v>3799000</v>
       </c>
       <c r="Q25" t="s">
+        <v>166</v>
+      </c>
+      <c r="R25" t="s">
         <v>167</v>
       </c>
-      <c r="R25" t="s">
-        <v>168</v>
-      </c>
       <c r="S25" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T25" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="U25" t="s">
         <v>28</v>
@@ -2239,25 +2236,25 @@
         <v>51</v>
       </c>
       <c r="N26" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O26" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="P26">
         <v>1000</v>
       </c>
       <c r="Q26" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="R26" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="S26" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T26" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="U26" t="s">
         <v>28</v>
@@ -2286,31 +2283,31 @@
         <v>30</v>
       </c>
       <c r="K27" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="N27" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="O27" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="P27">
         <v>100000</v>
       </c>
       <c r="Q27" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="R27" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="S27" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T27" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="U27" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="V27" s="2">
         <v>46291</v>
@@ -2348,28 +2345,28 @@
         <v>64</v>
       </c>
       <c r="N28" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O28" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="P28">
         <v>150000</v>
       </c>
       <c r="Q28" t="s">
+        <v>166</v>
+      </c>
+      <c r="R28" t="s">
         <v>167</v>
       </c>
-      <c r="R28" t="s">
-        <v>168</v>
-      </c>
       <c r="S28" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T28" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="U28" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="V28" s="2">
         <v>46199</v>
@@ -2407,28 +2404,28 @@
         <v>64</v>
       </c>
       <c r="N29" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O29" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="P29">
         <v>150000</v>
       </c>
       <c r="Q29" t="s">
+        <v>166</v>
+      </c>
+      <c r="R29" t="s">
         <v>167</v>
       </c>
-      <c r="R29" t="s">
-        <v>168</v>
-      </c>
       <c r="S29" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T29" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="U29" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="V29" s="2">
         <v>46199</v>
@@ -2466,28 +2463,28 @@
         <v>64</v>
       </c>
       <c r="N30" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O30" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="P30">
         <v>18462.36</v>
       </c>
       <c r="Q30" t="s">
+        <v>166</v>
+      </c>
+      <c r="R30" t="s">
         <v>167</v>
       </c>
-      <c r="R30" t="s">
-        <v>168</v>
-      </c>
       <c r="S30" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T30" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="U30" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="V30" s="2">
         <v>46199</v>
@@ -2525,28 +2522,28 @@
         <v>64</v>
       </c>
       <c r="N31" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O31" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="P31">
         <v>324166.14</v>
       </c>
       <c r="Q31" t="s">
+        <v>166</v>
+      </c>
+      <c r="R31" t="s">
         <v>167</v>
       </c>
-      <c r="R31" t="s">
-        <v>168</v>
-      </c>
       <c r="S31" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T31" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="U31" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="V31" s="2">
         <v>46199</v>
@@ -2572,31 +2569,31 @@
         <v>30</v>
       </c>
       <c r="K32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="N32" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O32" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="P32">
         <v>30000</v>
       </c>
       <c r="Q32" t="s">
+        <v>166</v>
+      </c>
+      <c r="R32" t="s">
         <v>167</v>
       </c>
-      <c r="R32" t="s">
-        <v>168</v>
-      </c>
       <c r="S32" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T32" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="U32" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="V32" s="2">
         <v>46291</v>
@@ -2634,28 +2631,28 @@
         <v>65</v>
       </c>
       <c r="N33" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O33" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="P33">
         <v>1496713.48</v>
       </c>
       <c r="Q33" t="s">
+        <v>166</v>
+      </c>
+      <c r="R33" t="s">
         <v>167</v>
       </c>
-      <c r="R33" t="s">
-        <v>168</v>
-      </c>
       <c r="S33" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T33" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="U33" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="V33" s="2">
         <v>46199</v>
@@ -2690,28 +2687,28 @@
         <v>49</v>
       </c>
       <c r="N34" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O34" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="P34">
         <v>207789.52</v>
       </c>
       <c r="Q34" t="s">
+        <v>166</v>
+      </c>
+      <c r="R34" t="s">
         <v>167</v>
       </c>
-      <c r="R34" t="s">
-        <v>168</v>
-      </c>
       <c r="S34" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T34" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="U34" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="V34" s="2">
         <v>46138</v>
@@ -2746,25 +2743,25 @@
         <v>55</v>
       </c>
       <c r="N35" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O35" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="P35">
         <v>962290.8</v>
       </c>
       <c r="Q35" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="R35" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="S35" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T35" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="U35" t="s">
         <v>28</v>
@@ -2802,25 +2799,25 @@
         <v>56</v>
       </c>
       <c r="N36" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O36" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="P36">
         <v>798776.97</v>
       </c>
       <c r="Q36" t="s">
+        <v>166</v>
+      </c>
+      <c r="R36" t="s">
         <v>167</v>
       </c>
-      <c r="R36" t="s">
-        <v>168</v>
-      </c>
       <c r="S36" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T36" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="U36" t="s">
         <v>28</v>
@@ -2858,25 +2855,25 @@
         <v>55</v>
       </c>
       <c r="N37" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O37" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="P37">
         <v>1530656.62</v>
       </c>
       <c r="Q37" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="R37" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="S37" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T37" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="U37" t="s">
         <v>28</v>
@@ -2914,25 +2911,25 @@
         <v>57</v>
       </c>
       <c r="N38" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O38" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="P38">
         <v>72958.08</v>
       </c>
       <c r="Q38" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="R38" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="S38" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T38" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="U38" t="s">
         <v>28</v>
@@ -2970,25 +2967,25 @@
         <v>57</v>
       </c>
       <c r="N39" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O39" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="P39">
         <v>8916</v>
       </c>
       <c r="Q39" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="R39" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="S39" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T39" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="U39" t="s">
         <v>28</v>
@@ -3026,25 +3023,25 @@
         <v>57</v>
       </c>
       <c r="N40" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O40" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="P40">
         <v>425178.5</v>
       </c>
       <c r="Q40" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="R40" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="S40" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T40" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="U40" t="s">
         <v>28</v>
@@ -3082,25 +3079,25 @@
         <v>58</v>
       </c>
       <c r="N41" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O41" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="P41">
         <v>1223.03</v>
       </c>
       <c r="Q41" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="R41" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="S41" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T41" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="U41" t="s">
         <v>28</v>
@@ -3129,22 +3126,22 @@
         <v>41</v>
       </c>
       <c r="N42" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O42" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q42" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="R42" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="S42" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="T42" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="U42" t="s">
         <v>28</v>
@@ -3182,25 +3179,25 @@
         <v>59</v>
       </c>
       <c r="N43" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="O43" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="P43">
         <v>400000</v>
       </c>
       <c r="Q43" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="R43" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="S43" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T43" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="U43" t="s">
         <v>28</v>
@@ -3238,25 +3235,25 @@
         <v>59</v>
       </c>
       <c r="N44" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="O44" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="P44">
         <v>400000</v>
       </c>
       <c r="Q44" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="R44" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="S44" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T44" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="U44" t="s">
         <v>28</v>
@@ -3297,28 +3294,28 @@
         <v>66</v>
       </c>
       <c r="N45" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O45" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="P45">
         <v>173846.38</v>
       </c>
       <c r="Q45" t="s">
+        <v>166</v>
+      </c>
+      <c r="R45" t="s">
         <v>167</v>
       </c>
-      <c r="R45" t="s">
-        <v>168</v>
-      </c>
       <c r="S45" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T45" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="U45" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="V45" s="2">
         <v>46229</v>
@@ -3353,28 +3350,28 @@
         <v>53</v>
       </c>
       <c r="N46" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O46" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="P46">
         <v>1530656.62</v>
       </c>
       <c r="Q46" t="s">
+        <v>166</v>
+      </c>
+      <c r="R46" t="s">
         <v>167</v>
       </c>
-      <c r="R46" t="s">
-        <v>168</v>
-      </c>
       <c r="S46" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T46" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="U46" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="V46" s="2">
         <v>46229</v>
@@ -3400,25 +3397,25 @@
         <v>30</v>
       </c>
       <c r="N47" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="O47" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="P47">
         <v>1000000</v>
       </c>
       <c r="Q47" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="R47" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="S47" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T47" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="U47" t="s">
         <v>28</v>
@@ -3447,31 +3444,31 @@
         <v>30</v>
       </c>
       <c r="K48" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="N48" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O48" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="P48">
         <v>958040</v>
       </c>
       <c r="Q48" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="R48" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="S48" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T48" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="U48" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="V48" s="2">
         <v>46291</v>
@@ -3509,28 +3506,28 @@
         <v>67</v>
       </c>
       <c r="N49" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O49" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="P49">
         <v>41730.64</v>
       </c>
       <c r="Q49" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="R49" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="S49" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T49" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="U49" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="V49" s="2">
         <v>46199</v>
@@ -3559,31 +3556,31 @@
         <v>66</v>
       </c>
       <c r="K50" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="N50" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O50" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="P50">
         <v>1468159.32</v>
       </c>
       <c r="Q50" t="s">
+        <v>166</v>
+      </c>
+      <c r="R50" t="s">
         <v>167</v>
       </c>
-      <c r="R50" t="s">
-        <v>168</v>
-      </c>
       <c r="S50" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T50" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="U50" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="V50" s="2">
         <v>46260</v>
@@ -3612,31 +3609,31 @@
         <v>66</v>
       </c>
       <c r="K51" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="N51" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O51" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="P51">
         <v>1704503</v>
       </c>
       <c r="Q51" t="s">
+        <v>166</v>
+      </c>
+      <c r="R51" t="s">
         <v>167</v>
       </c>
-      <c r="R51" t="s">
-        <v>168</v>
-      </c>
       <c r="S51" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T51" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="U51" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="V51" s="2">
         <v>46291</v>
@@ -3662,31 +3659,31 @@
         <v>30</v>
       </c>
       <c r="K52" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="N52" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O52" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="P52">
         <v>1704503</v>
       </c>
       <c r="Q52" t="s">
+        <v>166</v>
+      </c>
+      <c r="R52" t="s">
         <v>167</v>
       </c>
-      <c r="R52" t="s">
-        <v>168</v>
-      </c>
       <c r="S52" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T52" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="U52" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="V52" s="2">
         <v>46321</v>
@@ -3721,28 +3718,28 @@
         <v>61</v>
       </c>
       <c r="N53" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O53" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="P53">
         <v>236343.68</v>
       </c>
       <c r="Q53" t="s">
+        <v>166</v>
+      </c>
+      <c r="R53" t="s">
         <v>167</v>
       </c>
-      <c r="R53" t="s">
-        <v>168</v>
-      </c>
       <c r="S53" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T53" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="U53" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="V53" s="2">
         <v>46229</v>
@@ -3768,31 +3765,31 @@
         <v>30</v>
       </c>
       <c r="K54" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="N54" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O54" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="P54">
         <v>1295422.28</v>
       </c>
       <c r="Q54" t="s">
+        <v>166</v>
+      </c>
+      <c r="R54" t="s">
         <v>167</v>
       </c>
-      <c r="R54" t="s">
-        <v>168</v>
-      </c>
       <c r="S54" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T54" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="U54" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="V54" s="2">
         <v>46352</v>
@@ -3818,31 +3815,31 @@
         <v>39</v>
       </c>
       <c r="K55" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="N55" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="O55" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="P55">
         <v>500000</v>
       </c>
       <c r="Q55" t="s">
+        <v>166</v>
+      </c>
+      <c r="R55" t="s">
         <v>167</v>
       </c>
-      <c r="R55" t="s">
-        <v>168</v>
-      </c>
       <c r="S55" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="T55" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="U55" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="V55" s="2">
         <v>46321</v>
@@ -3871,28 +3868,28 @@
         <v>43</v>
       </c>
       <c r="N56" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="O56" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="P56">
         <v>5000000</v>
       </c>
       <c r="Q56" t="s">
+        <v>166</v>
+      </c>
+      <c r="R56" t="s">
         <v>167</v>
       </c>
-      <c r="R56" t="s">
-        <v>168</v>
-      </c>
       <c r="S56" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="T56" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="U56" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="V56" s="2">
         <v>46321</v>
@@ -3918,25 +3915,25 @@
         <v>41</v>
       </c>
       <c r="N57" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="O57" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="Q57" t="s">
+        <v>166</v>
+      </c>
+      <c r="R57" t="s">
         <v>167</v>
       </c>
-      <c r="R57" t="s">
-        <v>168</v>
-      </c>
       <c r="S57" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="T57" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="U57" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="V57" s="2">
         <v>46049</v>
@@ -3962,25 +3959,25 @@
         <v>41</v>
       </c>
       <c r="N58" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="O58" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="Q58" t="s">
+        <v>166</v>
+      </c>
+      <c r="R58" t="s">
         <v>167</v>
       </c>
-      <c r="R58" t="s">
-        <v>168</v>
-      </c>
       <c r="S58" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="T58" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="U58" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="59" spans="1:22">
@@ -4003,25 +4000,25 @@
         <v>41</v>
       </c>
       <c r="N59" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="O59" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="Q59" t="s">
+        <v>166</v>
+      </c>
+      <c r="R59" t="s">
         <v>167</v>
       </c>
-      <c r="R59" t="s">
-        <v>168</v>
-      </c>
       <c r="S59" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="T59" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="U59" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="60" spans="1:22">
@@ -4041,28 +4038,28 @@
         <v>29</v>
       </c>
       <c r="N60" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="O60" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="P60">
         <v>9389.959999999999</v>
       </c>
       <c r="Q60" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="R60" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="S60" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="T60" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="U60" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="V60" s="2">
         <v>46107</v>
@@ -4085,28 +4082,28 @@
         <v>29</v>
       </c>
       <c r="N61" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="O61" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="P61">
         <v>7204.82</v>
       </c>
       <c r="Q61" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="R61" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="S61" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="T61" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="U61" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="V61" s="2">
         <v>46107</v>
@@ -4129,28 +4126,28 @@
         <v>29</v>
       </c>
       <c r="N62" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="O62" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="P62">
         <v>4227.84</v>
       </c>
       <c r="Q62" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="R62" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="S62" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="T62" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="U62" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="V62" s="2">
         <v>46107</v>
@@ -4173,28 +4170,28 @@
         <v>29</v>
       </c>
       <c r="N63" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="O63" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="P63">
         <v>4064.54</v>
       </c>
       <c r="Q63" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="R63" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="S63" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="T63" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="U63" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="V63" s="2">
         <v>46107</v>
@@ -4217,28 +4214,28 @@
         <v>29</v>
       </c>
       <c r="N64" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="O64" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="P64">
         <v>3662.66</v>
       </c>
       <c r="Q64" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="R64" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="S64" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="T64" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="U64" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="V64" s="2">
         <v>46107</v>
@@ -4261,28 +4258,28 @@
         <v>29</v>
       </c>
       <c r="N65" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="O65" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="P65">
         <v>1163.64</v>
       </c>
       <c r="Q65" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="R65" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="S65" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="T65" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="U65" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="V65" s="2">
         <v>46107</v>
@@ -4305,25 +4302,25 @@
         <v>29</v>
       </c>
       <c r="N66" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="O66" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="P66">
         <v>120000</v>
       </c>
       <c r="Q66" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="R66" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="S66" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="T66" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="U66" t="s">
         <v>28</v>
@@ -4352,25 +4349,25 @@
         <v>30</v>
       </c>
       <c r="N67" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O67" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="P67">
         <v>400000</v>
       </c>
       <c r="Q67" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="R67" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="S67" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T67" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="U67" t="s">
         <v>28</v>
@@ -4399,31 +4396,31 @@
         <v>30</v>
       </c>
       <c r="K68" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="N68" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="O68" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="P68">
         <v>100000</v>
       </c>
       <c r="Q68" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="R68" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="S68" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T68" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="U68" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="V68" s="2">
         <v>46229</v>
@@ -4446,25 +4443,25 @@
         <v>29</v>
       </c>
       <c r="N69" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="O69" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="P69">
         <v>80000</v>
       </c>
       <c r="Q69" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="R69" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="S69" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="T69" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="U69" t="s">
         <v>28</v>
@@ -4490,28 +4487,28 @@
         <v>29</v>
       </c>
       <c r="N70" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O70" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="P70">
         <v>835000</v>
       </c>
       <c r="Q70" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="R70" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="S70" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="T70" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="U70" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="V70" s="2">
         <v>46291</v>
@@ -4534,28 +4531,28 @@
         <v>29</v>
       </c>
       <c r="N71" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O71" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="P71">
         <v>165000</v>
       </c>
       <c r="Q71" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="R71" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="S71" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="T71" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="U71" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="V71" s="2">
         <v>46168</v>
@@ -4578,28 +4575,28 @@
         <v>29</v>
       </c>
       <c r="N72" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O72" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="P72">
         <v>1000000</v>
       </c>
       <c r="Q72" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="R72" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="S72" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="T72" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="U72" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="V72" s="2">
         <v>46291</v>
@@ -4622,28 +4619,28 @@
         <v>29</v>
       </c>
       <c r="N73" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O73" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="P73">
         <v>1000000</v>
       </c>
       <c r="Q73" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="R73" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="S73" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="T73" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="U73" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="V73" s="2">
         <v>46291</v>
@@ -4666,28 +4663,28 @@
         <v>29</v>
       </c>
       <c r="N74" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="O74" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="P74">
         <v>100000</v>
       </c>
       <c r="Q74" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="R74" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="S74" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="T74" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="U74" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="V74" s="2">
         <v>46291</v>
@@ -4713,25 +4710,25 @@
         <v>30</v>
       </c>
       <c r="N75" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="O75" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="P75">
         <v>1000000</v>
       </c>
       <c r="Q75" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="R75" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="S75" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T75" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="U75" t="s">
         <v>28</v>
@@ -4763,28 +4760,28 @@
         <v>44</v>
       </c>
       <c r="N76" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O76" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="P76">
         <v>1704503</v>
       </c>
       <c r="Q76" t="s">
+        <v>166</v>
+      </c>
+      <c r="R76" t="s">
         <v>167</v>
-      </c>
-      <c r="R76" t="s">
-        <v>168</v>
       </c>
       <c r="S76" t="s">
         <v>40</v>
       </c>
       <c r="T76" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="U76" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="V76" s="2">
         <v>46381</v>
@@ -4813,28 +4810,28 @@
         <v>44</v>
       </c>
       <c r="N77" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O77" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="P77">
         <v>1638125.5</v>
       </c>
       <c r="Q77" t="s">
+        <v>166</v>
+      </c>
+      <c r="R77" t="s">
         <v>167</v>
-      </c>
-      <c r="R77" t="s">
-        <v>168</v>
       </c>
       <c r="S77" t="s">
         <v>40</v>
       </c>
       <c r="T77" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="U77" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="V77" s="2">
         <v>46381</v>
@@ -4863,25 +4860,25 @@
         <v>44</v>
       </c>
       <c r="N78" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O78" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="P78">
         <v>3800000</v>
       </c>
       <c r="Q78" t="s">
+        <v>166</v>
+      </c>
+      <c r="R78" t="s">
         <v>167</v>
-      </c>
-      <c r="R78" t="s">
-        <v>168</v>
       </c>
       <c r="S78" t="s">
         <v>40</v>
       </c>
       <c r="T78" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="U78" t="s">
         <v>28</v>
@@ -4913,25 +4910,25 @@
         <v>44</v>
       </c>
       <c r="N79" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O79" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="P79">
         <v>3800000</v>
       </c>
       <c r="Q79" t="s">
+        <v>166</v>
+      </c>
+      <c r="R79" t="s">
         <v>167</v>
-      </c>
-      <c r="R79" t="s">
-        <v>168</v>
       </c>
       <c r="S79" t="s">
         <v>40</v>
       </c>
       <c r="T79" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="U79" t="s">
         <v>28</v>
@@ -4960,28 +4957,28 @@
         <v>68</v>
       </c>
       <c r="K80" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="N80" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O80" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="P80">
         <v>3800000</v>
       </c>
       <c r="Q80" t="s">
+        <v>166</v>
+      </c>
+      <c r="R80" t="s">
         <v>167</v>
       </c>
-      <c r="R80" t="s">
-        <v>168</v>
-      </c>
       <c r="S80" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="T80" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="U80" t="s">
         <v>28</v>
@@ -5007,25 +5004,25 @@
         <v>28</v>
       </c>
       <c r="N81" t="s">
+        <v>94</v>
+      </c>
+      <c r="O81" t="s">
         <v>95</v>
-      </c>
-      <c r="O81" t="s">
-        <v>96</v>
       </c>
       <c r="P81">
         <v>4394700</v>
       </c>
       <c r="Q81" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="R81" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="S81" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="T81" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="U81" t="s">
         <v>28</v>
@@ -5054,31 +5051,31 @@
         <v>30</v>
       </c>
       <c r="K82" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="N82" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O82" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="P82">
         <v>528395.9300000001</v>
       </c>
       <c r="Q82" t="s">
+        <v>166</v>
+      </c>
+      <c r="R82" t="s">
         <v>167</v>
       </c>
-      <c r="R82" t="s">
-        <v>168</v>
-      </c>
       <c r="S82" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T82" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="U82" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="V82" s="2">
         <v>46382</v>
@@ -5101,25 +5098,25 @@
         <v>29</v>
       </c>
       <c r="N83" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="O83" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="P83">
         <v>1000000</v>
       </c>
       <c r="Q83" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="R83" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="S83" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="T83" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="U83" t="s">
         <v>28</v>
@@ -5145,25 +5142,25 @@
         <v>28</v>
       </c>
       <c r="N84" t="s">
+        <v>94</v>
+      </c>
+      <c r="O84" t="s">
         <v>95</v>
-      </c>
-      <c r="O84" t="s">
-        <v>96</v>
       </c>
       <c r="P84">
         <v>4394700</v>
       </c>
       <c r="Q84" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="R84" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="S84" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="T84" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="U84" t="s">
         <v>28</v>
@@ -5195,25 +5192,25 @@
         <v>44</v>
       </c>
       <c r="N85" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="O85" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="P85">
         <v>3306000</v>
       </c>
       <c r="Q85" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="R85" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="S85" t="s">
         <v>40</v>
       </c>
       <c r="T85" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="U85" t="s">
         <v>28</v>
@@ -5242,25 +5239,25 @@
         <v>44</v>
       </c>
       <c r="N86" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="O86" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="P86">
         <v>3306000</v>
       </c>
       <c r="Q86" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="R86" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="S86" t="s">
         <v>40</v>
       </c>
       <c r="T86" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="U86" t="s">
         <v>28</v>
@@ -5286,25 +5283,25 @@
         <v>30</v>
       </c>
       <c r="N87" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="O87" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="P87">
         <v>470820</v>
       </c>
       <c r="Q87" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="R87" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="S87" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T87" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="U87" t="s">
         <v>28</v>

</xml_diff>

<commit_message>
Atualização automática: mta (09/09/2026 12:06)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -244,7 +244,7 @@
     <t>ATENDER com 20XV</t>
   </si>
   <si>
-    <t>Remanejar tarefa módulo extra</t>
+    <t>Remanejar tarefa módulo extra ctt 005</t>
   </si>
   <si>
     <t>LIVRE</t>
@@ -563,16 +563,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -588,7 +580,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -596,30 +588,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -919,70 +893,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1035,7 +1009,7 @@
       <c r="U2" t="s">
         <v>179</v>
       </c>
-      <c r="V2" s="2">
+      <c r="V2" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1082,7 +1056,7 @@
       <c r="U3" t="s">
         <v>28</v>
       </c>
-      <c r="V3" s="2">
+      <c r="V3" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1129,7 +1103,7 @@
       <c r="U4" t="s">
         <v>28</v>
       </c>
-      <c r="V4" s="2">
+      <c r="V4" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1176,7 +1150,7 @@
       <c r="U5" t="s">
         <v>28</v>
       </c>
-      <c r="V5" s="2">
+      <c r="V5" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1226,7 +1200,7 @@
       <c r="U6" t="s">
         <v>28</v>
       </c>
-      <c r="V6" s="2">
+      <c r="V6" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1252,7 +1226,7 @@
       <c r="G7" t="s">
         <v>42</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>46121</v>
       </c>
       <c r="I7" t="s">
@@ -1282,7 +1256,7 @@
       <c r="U7" t="s">
         <v>28</v>
       </c>
-      <c r="V7" s="2">
+      <c r="V7" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -1329,7 +1303,7 @@
       <c r="U8" t="s">
         <v>28</v>
       </c>
-      <c r="V8" s="2">
+      <c r="V8" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1376,7 +1350,7 @@
       <c r="U9" t="s">
         <v>28</v>
       </c>
-      <c r="V9" s="2">
+      <c r="V9" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1423,7 +1397,7 @@
       <c r="U10" t="s">
         <v>28</v>
       </c>
-      <c r="V10" s="2">
+      <c r="V10" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1470,7 +1444,7 @@
       <c r="U11" t="s">
         <v>28</v>
       </c>
-      <c r="V11" s="2">
+      <c r="V11" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -1496,7 +1470,7 @@
       <c r="G12" t="s">
         <v>42</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46079</v>
       </c>
       <c r="I12" t="s">
@@ -1529,7 +1503,7 @@
       <c r="U12" t="s">
         <v>179</v>
       </c>
-      <c r="V12" s="2">
+      <c r="V12" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1579,7 +1553,7 @@
       <c r="U13" t="s">
         <v>179</v>
       </c>
-      <c r="V13" s="2">
+      <c r="V13" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1629,7 +1603,7 @@
       <c r="U14" t="s">
         <v>179</v>
       </c>
-      <c r="V14" s="2">
+      <c r="V14" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1679,7 +1653,7 @@
       <c r="U15" t="s">
         <v>179</v>
       </c>
-      <c r="V15" s="2">
+      <c r="V15" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -1729,7 +1703,7 @@
       <c r="U16" t="s">
         <v>179</v>
       </c>
-      <c r="V16" s="2">
+      <c r="V16" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -1755,7 +1729,7 @@
       <c r="G17" t="s">
         <v>42</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46098</v>
       </c>
       <c r="I17" t="s">
@@ -1788,7 +1762,7 @@
       <c r="U17" t="s">
         <v>179</v>
       </c>
-      <c r="V17" s="2">
+      <c r="V17" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -1814,7 +1788,7 @@
       <c r="G18" t="s">
         <v>42</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46076</v>
       </c>
       <c r="I18" t="s">
@@ -1844,7 +1818,7 @@
       <c r="U18" t="s">
         <v>28</v>
       </c>
-      <c r="V18" s="2">
+      <c r="V18" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1870,7 +1844,7 @@
       <c r="G19" t="s">
         <v>42</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46076</v>
       </c>
       <c r="I19" t="s">
@@ -1900,7 +1874,7 @@
       <c r="U19" t="s">
         <v>28</v>
       </c>
-      <c r="V19" s="2">
+      <c r="V19" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -1947,7 +1921,7 @@
       <c r="U20" t="s">
         <v>28</v>
       </c>
-      <c r="V20" s="2">
+      <c r="V20" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -1994,7 +1968,7 @@
       <c r="U21" t="s">
         <v>28</v>
       </c>
-      <c r="V21" s="2">
+      <c r="V21" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2041,7 +2015,7 @@
       <c r="U22" t="s">
         <v>28</v>
       </c>
-      <c r="V22" s="2">
+      <c r="V22" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2088,7 +2062,7 @@
       <c r="U23" t="s">
         <v>28</v>
       </c>
-      <c r="V23" s="2">
+      <c r="V23" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -2114,7 +2088,7 @@
       <c r="G24" t="s">
         <v>42</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>46119</v>
       </c>
       <c r="I24" t="s">
@@ -2147,7 +2121,7 @@
       <c r="U24" t="s">
         <v>179</v>
       </c>
-      <c r="V24" s="2">
+      <c r="V24" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2173,7 +2147,7 @@
       <c r="G25" t="s">
         <v>42</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>46121</v>
       </c>
       <c r="I25" t="s">
@@ -2203,7 +2177,7 @@
       <c r="U25" t="s">
         <v>28</v>
       </c>
-      <c r="V25" s="2">
+      <c r="V25" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2229,7 +2203,7 @@
       <c r="G26" t="s">
         <v>42</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>46076</v>
       </c>
       <c r="I26" t="s">
@@ -2259,7 +2233,7 @@
       <c r="U26" t="s">
         <v>28</v>
       </c>
-      <c r="V26" s="2">
+      <c r="V26" s="1">
         <v>46079</v>
       </c>
     </row>
@@ -2309,7 +2283,7 @@
       <c r="U27" t="s">
         <v>179</v>
       </c>
-      <c r="V27" s="2">
+      <c r="V27" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2335,7 +2309,7 @@
       <c r="G28" t="s">
         <v>42</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>46199</v>
       </c>
       <c r="I28" t="s">
@@ -2368,7 +2342,7 @@
       <c r="U28" t="s">
         <v>179</v>
       </c>
-      <c r="V28" s="2">
+      <c r="V28" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2394,7 +2368,7 @@
       <c r="G29" t="s">
         <v>42</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>46199</v>
       </c>
       <c r="I29" t="s">
@@ -2427,7 +2401,7 @@
       <c r="U29" t="s">
         <v>179</v>
       </c>
-      <c r="V29" s="2">
+      <c r="V29" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2453,7 +2427,7 @@
       <c r="G30" t="s">
         <v>42</v>
       </c>
-      <c r="H30" s="2">
+      <c r="H30" s="1">
         <v>46199</v>
       </c>
       <c r="I30" t="s">
@@ -2486,7 +2460,7 @@
       <c r="U30" t="s">
         <v>179</v>
       </c>
-      <c r="V30" s="2">
+      <c r="V30" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2512,7 +2486,7 @@
       <c r="G31" t="s">
         <v>42</v>
       </c>
-      <c r="H31" s="2">
+      <c r="H31" s="1">
         <v>46199</v>
       </c>
       <c r="I31" t="s">
@@ -2545,7 +2519,7 @@
       <c r="U31" t="s">
         <v>179</v>
       </c>
-      <c r="V31" s="2">
+      <c r="V31" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2595,7 +2569,7 @@
       <c r="U32" t="s">
         <v>179</v>
       </c>
-      <c r="V32" s="2">
+      <c r="V32" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -2621,7 +2595,7 @@
       <c r="G33" t="s">
         <v>42</v>
       </c>
-      <c r="H33" s="2">
+      <c r="H33" s="1">
         <v>46191</v>
       </c>
       <c r="I33" t="s">
@@ -2654,7 +2628,7 @@
       <c r="U33" t="s">
         <v>179</v>
       </c>
-      <c r="V33" s="2">
+      <c r="V33" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2680,7 +2654,7 @@
       <c r="G34" t="s">
         <v>42</v>
       </c>
-      <c r="H34" s="2">
+      <c r="H34" s="1">
         <v>46119</v>
       </c>
       <c r="I34" t="s">
@@ -2710,7 +2684,7 @@
       <c r="U34" t="s">
         <v>179</v>
       </c>
-      <c r="V34" s="2">
+      <c r="V34" s="1">
         <v>46138</v>
       </c>
     </row>
@@ -2736,7 +2710,7 @@
       <c r="G35" t="s">
         <v>42</v>
       </c>
-      <c r="H35" s="2">
+      <c r="H35" s="1">
         <v>46213</v>
       </c>
       <c r="I35" t="s">
@@ -2766,7 +2740,7 @@
       <c r="U35" t="s">
         <v>28</v>
       </c>
-      <c r="V35" s="2">
+      <c r="V35" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -2792,7 +2766,7 @@
       <c r="G36" t="s">
         <v>42</v>
       </c>
-      <c r="H36" s="2">
+      <c r="H36" s="1">
         <v>46175</v>
       </c>
       <c r="I36" t="s">
@@ -2822,7 +2796,7 @@
       <c r="U36" t="s">
         <v>28</v>
       </c>
-      <c r="V36" s="2">
+      <c r="V36" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2848,7 +2822,7 @@
       <c r="G37" t="s">
         <v>42</v>
       </c>
-      <c r="H37" s="2">
+      <c r="H37" s="1">
         <v>46213</v>
       </c>
       <c r="I37" t="s">
@@ -2878,7 +2852,7 @@
       <c r="U37" t="s">
         <v>28</v>
       </c>
-      <c r="V37" s="2">
+      <c r="V37" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -2904,7 +2878,7 @@
       <c r="G38" t="s">
         <v>42</v>
       </c>
-      <c r="H38" s="2">
+      <c r="H38" s="1">
         <v>46199</v>
       </c>
       <c r="I38" t="s">
@@ -2934,7 +2908,7 @@
       <c r="U38" t="s">
         <v>28</v>
       </c>
-      <c r="V38" s="2">
+      <c r="V38" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -2960,7 +2934,7 @@
       <c r="G39" t="s">
         <v>42</v>
       </c>
-      <c r="H39" s="2">
+      <c r="H39" s="1">
         <v>46199</v>
       </c>
       <c r="I39" t="s">
@@ -2990,7 +2964,7 @@
       <c r="U39" t="s">
         <v>28</v>
       </c>
-      <c r="V39" s="2">
+      <c r="V39" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3016,7 +2990,7 @@
       <c r="G40" t="s">
         <v>42</v>
       </c>
-      <c r="H40" s="2">
+      <c r="H40" s="1">
         <v>46204</v>
       </c>
       <c r="I40" t="s">
@@ -3046,7 +3020,7 @@
       <c r="U40" t="s">
         <v>28</v>
       </c>
-      <c r="V40" s="2">
+      <c r="V40" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3072,7 +3046,7 @@
       <c r="G41" t="s">
         <v>42</v>
       </c>
-      <c r="H41" s="2">
+      <c r="H41" s="1">
         <v>46244</v>
       </c>
       <c r="I41" t="s">
@@ -3102,7 +3076,7 @@
       <c r="U41" t="s">
         <v>28</v>
       </c>
-      <c r="V41" s="2">
+      <c r="V41" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3146,7 +3120,7 @@
       <c r="U42" t="s">
         <v>28</v>
       </c>
-      <c r="V42" s="2">
+      <c r="V42" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3172,7 +3146,7 @@
       <c r="G43" t="s">
         <v>42</v>
       </c>
-      <c r="H43" s="2">
+      <c r="H43" s="1">
         <v>46191</v>
       </c>
       <c r="I43" t="s">
@@ -3202,7 +3176,7 @@
       <c r="U43" t="s">
         <v>28</v>
       </c>
-      <c r="V43" s="2">
+      <c r="V43" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3228,7 +3202,7 @@
       <c r="G44" t="s">
         <v>42</v>
       </c>
-      <c r="H44" s="2">
+      <c r="H44" s="1">
         <v>46191</v>
       </c>
       <c r="I44" t="s">
@@ -3258,7 +3232,7 @@
       <c r="U44" t="s">
         <v>28</v>
       </c>
-      <c r="V44" s="2">
+      <c r="V44" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3284,7 +3258,7 @@
       <c r="G45" t="s">
         <v>42</v>
       </c>
-      <c r="H45" s="2">
+      <c r="H45" s="1">
         <v>46213</v>
       </c>
       <c r="I45" t="s">
@@ -3317,7 +3291,7 @@
       <c r="U45" t="s">
         <v>179</v>
       </c>
-      <c r="V45" s="2">
+      <c r="V45" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3343,7 +3317,7 @@
       <c r="G46" t="s">
         <v>42</v>
       </c>
-      <c r="H46" s="2">
+      <c r="H46" s="1">
         <v>46210</v>
       </c>
       <c r="I46" t="s">
@@ -3373,7 +3347,7 @@
       <c r="U46" t="s">
         <v>179</v>
       </c>
-      <c r="V46" s="2">
+      <c r="V46" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3420,7 +3394,7 @@
       <c r="U47" t="s">
         <v>28</v>
       </c>
-      <c r="V47" s="2">
+      <c r="V47" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3470,7 +3444,7 @@
       <c r="U48" t="s">
         <v>179</v>
       </c>
-      <c r="V48" s="2">
+      <c r="V48" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3496,7 +3470,7 @@
       <c r="G49" t="s">
         <v>42</v>
       </c>
-      <c r="H49" s="2">
+      <c r="H49" s="1">
         <v>46176</v>
       </c>
       <c r="I49" t="s">
@@ -3529,7 +3503,7 @@
       <c r="U49" t="s">
         <v>179</v>
       </c>
-      <c r="V49" s="2">
+      <c r="V49" s="1">
         <v>46199</v>
       </c>
     </row>
@@ -3582,7 +3556,7 @@
       <c r="U50" t="s">
         <v>179</v>
       </c>
-      <c r="V50" s="2">
+      <c r="V50" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -3635,7 +3609,7 @@
       <c r="U51" t="s">
         <v>179</v>
       </c>
-      <c r="V51" s="2">
+      <c r="V51" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -3685,7 +3659,7 @@
       <c r="U52" t="s">
         <v>179</v>
       </c>
-      <c r="V52" s="2">
+      <c r="V52" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3711,7 +3685,7 @@
       <c r="G53" t="s">
         <v>42</v>
       </c>
-      <c r="H53" s="2">
+      <c r="H53" s="1">
         <v>46227</v>
       </c>
       <c r="I53" t="s">
@@ -3741,7 +3715,7 @@
       <c r="U53" t="s">
         <v>179</v>
       </c>
-      <c r="V53" s="2">
+      <c r="V53" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -3791,7 +3765,7 @@
       <c r="U54" t="s">
         <v>179</v>
       </c>
-      <c r="V54" s="2">
+      <c r="V54" s="1">
         <v>46352</v>
       </c>
     </row>
@@ -3841,7 +3815,7 @@
       <c r="U55" t="s">
         <v>179</v>
       </c>
-      <c r="V55" s="2">
+      <c r="V55" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3891,7 +3865,7 @@
       <c r="U56" t="s">
         <v>179</v>
       </c>
-      <c r="V56" s="2">
+      <c r="V56" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -3935,7 +3909,7 @@
       <c r="U57" t="s">
         <v>179</v>
       </c>
-      <c r="V57" s="2">
+      <c r="V57" s="1">
         <v>46049</v>
       </c>
     </row>
@@ -4061,7 +4035,7 @@
       <c r="U60" t="s">
         <v>179</v>
       </c>
-      <c r="V60" s="2">
+      <c r="V60" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4105,7 +4079,7 @@
       <c r="U61" t="s">
         <v>179</v>
       </c>
-      <c r="V61" s="2">
+      <c r="V61" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4149,7 +4123,7 @@
       <c r="U62" t="s">
         <v>179</v>
       </c>
-      <c r="V62" s="2">
+      <c r="V62" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4193,7 +4167,7 @@
       <c r="U63" t="s">
         <v>179</v>
       </c>
-      <c r="V63" s="2">
+      <c r="V63" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4237,7 +4211,7 @@
       <c r="U64" t="s">
         <v>179</v>
       </c>
-      <c r="V64" s="2">
+      <c r="V64" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4281,7 +4255,7 @@
       <c r="U65" t="s">
         <v>179</v>
       </c>
-      <c r="V65" s="2">
+      <c r="V65" s="1">
         <v>46107</v>
       </c>
     </row>
@@ -4325,7 +4299,7 @@
       <c r="U66" t="s">
         <v>28</v>
       </c>
-      <c r="V66" s="2">
+      <c r="V66" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4372,7 +4346,7 @@
       <c r="U67" t="s">
         <v>28</v>
       </c>
-      <c r="V67" s="2">
+      <c r="V67" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4422,7 +4396,7 @@
       <c r="U68" t="s">
         <v>179</v>
       </c>
-      <c r="V68" s="2">
+      <c r="V68" s="1">
         <v>46229</v>
       </c>
     </row>
@@ -4466,7 +4440,7 @@
       <c r="U69" t="s">
         <v>28</v>
       </c>
-      <c r="V69" s="2">
+      <c r="V69" s="1">
         <v>46260</v>
       </c>
     </row>
@@ -4510,7 +4484,7 @@
       <c r="U70" t="s">
         <v>179</v>
       </c>
-      <c r="V70" s="2">
+      <c r="V70" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4554,7 +4528,7 @@
       <c r="U71" t="s">
         <v>179</v>
       </c>
-      <c r="V71" s="2">
+      <c r="V71" s="1">
         <v>46168</v>
       </c>
     </row>
@@ -4598,7 +4572,7 @@
       <c r="U72" t="s">
         <v>179</v>
       </c>
-      <c r="V72" s="2">
+      <c r="V72" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4642,7 +4616,7 @@
       <c r="U73" t="s">
         <v>179</v>
       </c>
-      <c r="V73" s="2">
+      <c r="V73" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4686,7 +4660,7 @@
       <c r="U74" t="s">
         <v>179</v>
       </c>
-      <c r="V74" s="2">
+      <c r="V74" s="1">
         <v>46291</v>
       </c>
     </row>
@@ -4733,7 +4707,7 @@
       <c r="U75" t="s">
         <v>28</v>
       </c>
-      <c r="V75" s="2">
+      <c r="V75" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -4783,7 +4757,7 @@
       <c r="U76" t="s">
         <v>179</v>
       </c>
-      <c r="V76" s="2">
+      <c r="V76" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4833,7 +4807,7 @@
       <c r="U77" t="s">
         <v>179</v>
       </c>
-      <c r="V77" s="2">
+      <c r="V77" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4883,7 +4857,7 @@
       <c r="U78" t="s">
         <v>28</v>
       </c>
-      <c r="V78" s="2">
+      <c r="V78" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4933,7 +4907,7 @@
       <c r="U79" t="s">
         <v>28</v>
       </c>
-      <c r="V79" s="2">
+      <c r="V79" s="1">
         <v>46381</v>
       </c>
     </row>
@@ -4983,7 +4957,7 @@
       <c r="U80" t="s">
         <v>28</v>
       </c>
-      <c r="V80" s="2">
+      <c r="V80" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5027,7 +5001,7 @@
       <c r="U81" t="s">
         <v>28</v>
       </c>
-      <c r="V81" s="2">
+      <c r="V81" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5077,7 +5051,7 @@
       <c r="U82" t="s">
         <v>179</v>
       </c>
-      <c r="V82" s="2">
+      <c r="V82" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5121,7 +5095,7 @@
       <c r="U83" t="s">
         <v>28</v>
       </c>
-      <c r="V83" s="2">
+      <c r="V83" s="1">
         <v>46321</v>
       </c>
     </row>
@@ -5165,7 +5139,7 @@
       <c r="U84" t="s">
         <v>28</v>
       </c>
-      <c r="V84" s="2">
+      <c r="V84" s="1">
         <v>46382</v>
       </c>
     </row>
@@ -5306,7 +5280,7 @@
       <c r="U87" t="s">
         <v>28</v>
       </c>
-      <c r="V87" s="2">
+      <c r="V87" s="1">
         <v>46291</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: mta (10/09/2026 11:58)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_mta_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1130" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1131" uniqueCount="181">
   <si>
     <t>linha</t>
   </si>
@@ -220,16 +220,19 @@
     <t>email do dia 24/04</t>
   </si>
   <si>
+    <t>2026-09-09 00:00:00</t>
+  </si>
+  <si>
     <t>e-mail 12/08</t>
   </si>
   <si>
-    <t>REMANEJAR P/ CABW 30</t>
+    <t>ATENDER E REMANEJAR P/ CABW 30</t>
   </si>
   <si>
     <t>ATENDER</t>
   </si>
   <si>
-    <t>Remanejar</t>
+    <t>REMANEJAR</t>
   </si>
   <si>
     <t>Atender SET</t>
@@ -244,7 +247,7 @@
     <t>ATENDER com 20XV</t>
   </si>
   <si>
-    <t>Remanejar tarefa módulo extra ctt 005</t>
+    <t>Remanejar tarefa módulo extra ctt 005 e Atender</t>
   </si>
   <si>
     <t>LIVRE</t>
@@ -980,34 +983,34 @@
         <v>30</v>
       </c>
       <c r="K2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="L2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="N2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="O2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="P2">
         <v>135000</v>
       </c>
       <c r="Q2" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R2" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S2" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T2" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U2" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="V2" s="1">
         <v>46229</v>
@@ -1033,25 +1036,25 @@
         <v>30</v>
       </c>
       <c r="N3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="O3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="P3">
         <v>400000</v>
       </c>
       <c r="Q3" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="R3" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="S3" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T3" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U3" t="s">
         <v>28</v>
@@ -1083,22 +1086,22 @@
         <v>41</v>
       </c>
       <c r="N4" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O4" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="Q4" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R4" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S4" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T4" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U4" t="s">
         <v>28</v>
@@ -1127,25 +1130,25 @@
         <v>30</v>
       </c>
       <c r="N5" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="P5">
         <v>384180</v>
       </c>
       <c r="Q5" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R5" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S5" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T5" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U5" t="s">
         <v>28</v>
@@ -1174,28 +1177,28 @@
         <v>30</v>
       </c>
       <c r="L6" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="N6" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="O6" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="P6">
         <v>563000</v>
       </c>
       <c r="Q6" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R6" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U6" t="s">
         <v>28</v>
@@ -1233,25 +1236,25 @@
         <v>45</v>
       </c>
       <c r="N7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="O7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="P7">
         <v>3799999.6</v>
       </c>
       <c r="Q7" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="R7" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S7" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T7" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U7" t="s">
         <v>28</v>
@@ -1280,25 +1283,25 @@
         <v>30</v>
       </c>
       <c r="N8" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O8" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="P8">
         <v>430000</v>
       </c>
       <c r="Q8" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R8" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S8" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T8" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U8" t="s">
         <v>28</v>
@@ -1327,25 +1330,25 @@
         <v>30</v>
       </c>
       <c r="N9" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O9" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="P9">
         <v>60000</v>
       </c>
       <c r="Q9" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R9" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T9" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U9" t="s">
         <v>28</v>
@@ -1374,25 +1377,25 @@
         <v>30</v>
       </c>
       <c r="N10" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="O10" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="P10">
         <v>200000</v>
       </c>
       <c r="Q10" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R10" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S10" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T10" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U10" t="s">
         <v>28</v>
@@ -1421,25 +1424,25 @@
         <v>30</v>
       </c>
       <c r="N11" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="O11" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="P11">
         <v>320000</v>
       </c>
       <c r="Q11" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R11" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S11" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T11" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U11" t="s">
         <v>28</v>
@@ -1480,28 +1483,28 @@
         <v>62</v>
       </c>
       <c r="N12" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="O12" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="P12">
         <v>1187433.02</v>
       </c>
       <c r="Q12" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R12" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="S12" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T12" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U12" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="V12" s="1">
         <v>46079</v>
@@ -1527,31 +1530,31 @@
         <v>30</v>
       </c>
       <c r="K13" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="N13" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="O13" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="P13">
         <v>1000000</v>
       </c>
       <c r="Q13" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R13" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="S13" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T13" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U13" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="V13" s="1">
         <v>46352</v>
@@ -1577,31 +1580,31 @@
         <v>30</v>
       </c>
       <c r="K14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="N14" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="O14" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="P14">
         <v>1000000</v>
       </c>
       <c r="Q14" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R14" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="S14" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T14" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U14" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="V14" s="1">
         <v>46352</v>
@@ -1627,31 +1630,31 @@
         <v>30</v>
       </c>
       <c r="K15" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="N15" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="O15" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="P15">
         <v>1000000</v>
       </c>
       <c r="Q15" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R15" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="S15" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T15" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U15" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="V15" s="1">
         <v>46352</v>
@@ -1677,31 +1680,31 @@
         <v>30</v>
       </c>
       <c r="K16" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="N16" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="O16" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="P16">
         <v>100000</v>
       </c>
       <c r="Q16" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="R16" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="S16" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T16" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U16" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="V16" s="1">
         <v>46229</v>
@@ -1739,28 +1742,28 @@
         <v>62</v>
       </c>
       <c r="N17" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="O17" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="P17">
         <v>1770880.5</v>
       </c>
       <c r="Q17" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="R17" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S17" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T17" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U17" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="V17" s="1">
         <v>46107</v>
@@ -1795,25 +1798,25 @@
         <v>48</v>
       </c>
       <c r="N18" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="O18" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="P18">
         <v>350000</v>
       </c>
       <c r="Q18" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="R18" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="S18" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T18" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U18" t="s">
         <v>28</v>
@@ -1851,25 +1854,25 @@
         <v>48</v>
       </c>
       <c r="N19" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="O19" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="P19">
         <v>350000</v>
       </c>
       <c r="Q19" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="R19" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="S19" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T19" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U19" t="s">
         <v>28</v>
@@ -1898,25 +1901,25 @@
         <v>30</v>
       </c>
       <c r="N20" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="O20" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="P20">
         <v>1000000</v>
       </c>
       <c r="Q20" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="R20" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="S20" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T20" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U20" t="s">
         <v>28</v>
@@ -1945,25 +1948,25 @@
         <v>30</v>
       </c>
       <c r="N21" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="O21" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="P21">
         <v>400000</v>
       </c>
       <c r="Q21" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="R21" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="S21" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T21" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U21" t="s">
         <v>28</v>
@@ -1992,25 +1995,25 @@
         <v>30</v>
       </c>
       <c r="N22" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O22" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="P22">
         <v>120000</v>
       </c>
       <c r="Q22" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R22" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S22" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T22" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U22" t="s">
         <v>28</v>
@@ -2039,25 +2042,25 @@
         <v>30</v>
       </c>
       <c r="N23" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O23" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="P23">
         <v>80000</v>
       </c>
       <c r="Q23" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R23" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S23" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T23" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U23" t="s">
         <v>28</v>
@@ -2098,28 +2101,28 @@
         <v>63</v>
       </c>
       <c r="N24" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="O24" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="P24">
         <v>1704503</v>
       </c>
       <c r="Q24" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="R24" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S24" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T24" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U24" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="V24" s="1">
         <v>46138</v>
@@ -2154,25 +2157,25 @@
         <v>50</v>
       </c>
       <c r="N25" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="O25" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="P25">
         <v>3799000</v>
       </c>
       <c r="Q25" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="R25" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S25" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T25" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U25" t="s">
         <v>28</v>
@@ -2210,25 +2213,25 @@
         <v>51</v>
       </c>
       <c r="N26" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="O26" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="P26">
         <v>1000</v>
       </c>
       <c r="Q26" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="R26" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="S26" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T26" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U26" t="s">
         <v>28</v>
@@ -2257,31 +2260,31 @@
         <v>30</v>
       </c>
       <c r="K27" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="N27" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="O27" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="P27">
         <v>100000</v>
       </c>
       <c r="Q27" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="R27" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="S27" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T27" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U27" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="V27" s="1">
         <v>46291</v>
@@ -2319,28 +2322,28 @@
         <v>64</v>
       </c>
       <c r="N28" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="O28" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="P28">
         <v>150000</v>
       </c>
       <c r="Q28" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="R28" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S28" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T28" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U28" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="V28" s="1">
         <v>46199</v>
@@ -2378,28 +2381,28 @@
         <v>64</v>
       </c>
       <c r="N29" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="O29" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="P29">
         <v>150000</v>
       </c>
       <c r="Q29" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="R29" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S29" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T29" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U29" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="V29" s="1">
         <v>46199</v>
@@ -2437,28 +2440,28 @@
         <v>64</v>
       </c>
       <c r="N30" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="O30" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="P30">
         <v>18462.36</v>
       </c>
       <c r="Q30" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="R30" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S30" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T30" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U30" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="V30" s="1">
         <v>46199</v>
@@ -2496,28 +2499,28 @@
         <v>64</v>
       </c>
       <c r="N31" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="O31" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="P31">
         <v>324166.14</v>
       </c>
       <c r="Q31" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="R31" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S31" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T31" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U31" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="V31" s="1">
         <v>46199</v>
@@ -2543,31 +2546,31 @@
         <v>30</v>
       </c>
       <c r="K32" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="N32" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="O32" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="P32">
         <v>30000</v>
       </c>
       <c r="Q32" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="R32" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S32" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T32" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U32" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="V32" s="1">
         <v>46291</v>
@@ -2605,28 +2608,28 @@
         <v>65</v>
       </c>
       <c r="N33" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="O33" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="P33">
         <v>1496713.48</v>
       </c>
       <c r="Q33" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="R33" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S33" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T33" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U33" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="V33" s="1">
         <v>46199</v>
@@ -2661,28 +2664,28 @@
         <v>49</v>
       </c>
       <c r="N34" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="O34" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="P34">
         <v>207789.52</v>
       </c>
       <c r="Q34" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="R34" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S34" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T34" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U34" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="V34" s="1">
         <v>46138</v>
@@ -2717,25 +2720,25 @@
         <v>55</v>
       </c>
       <c r="N35" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="O35" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="P35">
         <v>962290.8</v>
       </c>
       <c r="Q35" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="R35" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="S35" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T35" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U35" t="s">
         <v>28</v>
@@ -2773,25 +2776,25 @@
         <v>56</v>
       </c>
       <c r="N36" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="O36" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="P36">
         <v>798776.97</v>
       </c>
       <c r="Q36" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="R36" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S36" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T36" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U36" t="s">
         <v>28</v>
@@ -2829,25 +2832,25 @@
         <v>55</v>
       </c>
       <c r="N37" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="O37" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="P37">
         <v>1530656.62</v>
       </c>
       <c r="Q37" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="R37" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="S37" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T37" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U37" t="s">
         <v>28</v>
@@ -2885,25 +2888,25 @@
         <v>57</v>
       </c>
       <c r="N38" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="O38" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="P38">
         <v>72958.08</v>
       </c>
       <c r="Q38" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="R38" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="S38" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T38" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U38" t="s">
         <v>28</v>
@@ -2941,25 +2944,25 @@
         <v>57</v>
       </c>
       <c r="N39" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="O39" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="P39">
         <v>8916</v>
       </c>
       <c r="Q39" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="R39" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="S39" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T39" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U39" t="s">
         <v>28</v>
@@ -2997,25 +3000,25 @@
         <v>57</v>
       </c>
       <c r="N40" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="O40" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="P40">
         <v>425178.5</v>
       </c>
       <c r="Q40" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="R40" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="S40" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T40" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U40" t="s">
         <v>28</v>
@@ -3053,25 +3056,25 @@
         <v>58</v>
       </c>
       <c r="N41" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="O41" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="P41">
         <v>1223.03</v>
       </c>
       <c r="Q41" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="R41" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="S41" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T41" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U41" t="s">
         <v>28</v>
@@ -3100,22 +3103,22 @@
         <v>41</v>
       </c>
       <c r="N42" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="O42" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="Q42" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="R42" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="S42" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T42" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U42" t="s">
         <v>28</v>
@@ -3153,25 +3156,25 @@
         <v>59</v>
       </c>
       <c r="N43" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="O43" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="P43">
         <v>400000</v>
       </c>
       <c r="Q43" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="R43" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="S43" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T43" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U43" t="s">
         <v>28</v>
@@ -3209,25 +3212,25 @@
         <v>59</v>
       </c>
       <c r="N44" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="O44" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="P44">
         <v>400000</v>
       </c>
       <c r="Q44" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="R44" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="S44" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T44" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U44" t="s">
         <v>28</v>
@@ -3268,28 +3271,28 @@
         <v>66</v>
       </c>
       <c r="N45" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="O45" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="P45">
         <v>173846.38</v>
       </c>
       <c r="Q45" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="R45" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S45" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T45" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U45" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="V45" s="1">
         <v>46229</v>
@@ -3324,28 +3327,28 @@
         <v>53</v>
       </c>
       <c r="N46" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="O46" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="P46">
         <v>1530656.62</v>
       </c>
       <c r="Q46" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="R46" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S46" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T46" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U46" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="V46" s="1">
         <v>46229</v>
@@ -3371,25 +3374,25 @@
         <v>30</v>
       </c>
       <c r="N47" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="O47" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="P47">
         <v>1000000</v>
       </c>
       <c r="Q47" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="R47" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="S47" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T47" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U47" t="s">
         <v>28</v>
@@ -3418,31 +3421,31 @@
         <v>30</v>
       </c>
       <c r="K48" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="N48" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="O48" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="P48">
         <v>958040</v>
       </c>
       <c r="Q48" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R48" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="S48" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T48" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U48" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="V48" s="1">
         <v>46291</v>
@@ -3480,28 +3483,28 @@
         <v>67</v>
       </c>
       <c r="N49" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="O49" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="P49">
         <v>41730.64</v>
       </c>
       <c r="Q49" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R49" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="S49" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T49" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U49" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="V49" s="1">
         <v>46199</v>
@@ -3530,31 +3533,31 @@
         <v>66</v>
       </c>
       <c r="K50" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="N50" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="O50" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="P50">
         <v>1468159.32</v>
       </c>
       <c r="Q50" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="R50" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S50" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T50" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U50" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="V50" s="1">
         <v>46260</v>
@@ -3583,31 +3586,31 @@
         <v>66</v>
       </c>
       <c r="K51" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="N51" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="O51" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="P51">
         <v>1704503</v>
       </c>
       <c r="Q51" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="R51" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S51" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T51" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U51" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="V51" s="1">
         <v>46291</v>
@@ -3633,31 +3636,31 @@
         <v>30</v>
       </c>
       <c r="K52" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="N52" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="O52" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="P52">
         <v>1704503</v>
       </c>
       <c r="Q52" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="R52" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S52" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T52" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U52" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="V52" s="1">
         <v>46321</v>
@@ -3692,28 +3695,28 @@
         <v>61</v>
       </c>
       <c r="N53" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="O53" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="P53">
         <v>236343.68</v>
       </c>
       <c r="Q53" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="R53" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S53" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T53" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U53" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="V53" s="1">
         <v>46229</v>
@@ -3739,31 +3742,31 @@
         <v>30</v>
       </c>
       <c r="K54" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="N54" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="O54" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="P54">
         <v>1295422.28</v>
       </c>
       <c r="Q54" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="R54" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S54" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T54" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U54" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="V54" s="1">
         <v>46352</v>
@@ -3788,32 +3791,35 @@
       <c r="F55" t="s">
         <v>39</v>
       </c>
+      <c r="J55" t="s">
+        <v>68</v>
+      </c>
       <c r="K55" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="N55" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="O55" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="P55">
         <v>500000</v>
       </c>
       <c r="Q55" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="R55" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S55" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T55" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="U55" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="V55" s="1">
         <v>46321</v>
@@ -3842,28 +3848,28 @@
         <v>43</v>
       </c>
       <c r="N56" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="O56" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="P56">
         <v>5000000</v>
       </c>
       <c r="Q56" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="R56" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S56" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T56" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="U56" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="V56" s="1">
         <v>46321</v>
@@ -3889,25 +3895,25 @@
         <v>41</v>
       </c>
       <c r="N57" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="O57" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="Q57" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="R57" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S57" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T57" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="U57" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="V57" s="1">
         <v>46049</v>
@@ -3933,25 +3939,25 @@
         <v>41</v>
       </c>
       <c r="N58" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="O58" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="Q58" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="R58" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S58" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T58" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="U58" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="59" spans="1:22">
@@ -3974,25 +3980,25 @@
         <v>41</v>
       </c>
       <c r="N59" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="O59" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="Q59" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="R59" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S59" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T59" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="U59" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="60" spans="1:22">
@@ -4012,28 +4018,28 @@
         <v>29</v>
       </c>
       <c r="N60" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="O60" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="P60">
         <v>9389.959999999999</v>
       </c>
       <c r="Q60" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R60" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="S60" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T60" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U60" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="V60" s="1">
         <v>46107</v>
@@ -4056,28 +4062,28 @@
         <v>29</v>
       </c>
       <c r="N61" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="O61" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="P61">
         <v>7204.82</v>
       </c>
       <c r="Q61" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R61" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="S61" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T61" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U61" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="V61" s="1">
         <v>46107</v>
@@ -4100,28 +4106,28 @@
         <v>29</v>
       </c>
       <c r="N62" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="O62" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="P62">
         <v>4227.84</v>
       </c>
       <c r="Q62" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R62" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="S62" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T62" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U62" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="V62" s="1">
         <v>46107</v>
@@ -4144,28 +4150,28 @@
         <v>29</v>
       </c>
       <c r="N63" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="O63" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="P63">
         <v>4064.54</v>
       </c>
       <c r="Q63" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="R63" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="S63" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T63" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U63" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="V63" s="1">
         <v>46107</v>
@@ -4188,28 +4194,28 @@
         <v>29</v>
       </c>
       <c r="N64" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="O64" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="P64">
         <v>3662.66</v>
       </c>
       <c r="Q64" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R64" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="S64" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T64" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U64" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="V64" s="1">
         <v>46107</v>
@@ -4232,28 +4238,28 @@
         <v>29</v>
       </c>
       <c r="N65" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="O65" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="P65">
         <v>1163.64</v>
       </c>
       <c r="Q65" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="R65" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="S65" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T65" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U65" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="V65" s="1">
         <v>46107</v>
@@ -4276,25 +4282,25 @@
         <v>29</v>
       </c>
       <c r="N66" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O66" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="P66">
         <v>120000</v>
       </c>
       <c r="Q66" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R66" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S66" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T66" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U66" t="s">
         <v>28</v>
@@ -4323,25 +4329,25 @@
         <v>30</v>
       </c>
       <c r="N67" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="O67" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="P67">
         <v>400000</v>
       </c>
       <c r="Q67" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="R67" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="S67" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T67" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U67" t="s">
         <v>28</v>
@@ -4370,31 +4376,31 @@
         <v>30</v>
       </c>
       <c r="K68" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="N68" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="O68" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="P68">
         <v>100000</v>
       </c>
       <c r="Q68" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="R68" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="S68" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T68" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U68" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="V68" s="1">
         <v>46229</v>
@@ -4417,25 +4423,25 @@
         <v>29</v>
       </c>
       <c r="N69" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O69" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="P69">
         <v>80000</v>
       </c>
       <c r="Q69" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R69" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S69" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T69" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U69" t="s">
         <v>28</v>
@@ -4461,28 +4467,28 @@
         <v>29</v>
       </c>
       <c r="N70" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="O70" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="P70">
         <v>835000</v>
       </c>
       <c r="Q70" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R70" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="S70" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T70" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U70" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="V70" s="1">
         <v>46291</v>
@@ -4505,28 +4511,28 @@
         <v>29</v>
       </c>
       <c r="N71" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="O71" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="P71">
         <v>165000</v>
       </c>
       <c r="Q71" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R71" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="S71" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T71" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U71" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="V71" s="1">
         <v>46168</v>
@@ -4549,28 +4555,28 @@
         <v>29</v>
       </c>
       <c r="N72" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="O72" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="P72">
         <v>1000000</v>
       </c>
       <c r="Q72" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R72" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="S72" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T72" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U72" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="V72" s="1">
         <v>46291</v>
@@ -4593,28 +4599,28 @@
         <v>29</v>
       </c>
       <c r="N73" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="O73" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="P73">
         <v>1000000</v>
       </c>
       <c r="Q73" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R73" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="S73" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T73" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U73" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="V73" s="1">
         <v>46291</v>
@@ -4637,28 +4643,28 @@
         <v>29</v>
       </c>
       <c r="N74" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="O74" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="P74">
         <v>100000</v>
       </c>
       <c r="Q74" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="R74" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="S74" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T74" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U74" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="V74" s="1">
         <v>46291</v>
@@ -4684,25 +4690,25 @@
         <v>30</v>
       </c>
       <c r="N75" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="O75" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="P75">
         <v>1000000</v>
       </c>
       <c r="Q75" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="R75" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="S75" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T75" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U75" t="s">
         <v>28</v>
@@ -4734,28 +4740,28 @@
         <v>44</v>
       </c>
       <c r="N76" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="O76" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="P76">
         <v>1704503</v>
       </c>
       <c r="Q76" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="R76" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S76" t="s">
         <v>40</v>
       </c>
       <c r="T76" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U76" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="V76" s="1">
         <v>46381</v>
@@ -4784,28 +4790,28 @@
         <v>44</v>
       </c>
       <c r="N77" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="O77" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="P77">
         <v>1638125.5</v>
       </c>
       <c r="Q77" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="R77" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S77" t="s">
         <v>40</v>
       </c>
       <c r="T77" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U77" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="V77" s="1">
         <v>46381</v>
@@ -4834,25 +4840,25 @@
         <v>44</v>
       </c>
       <c r="N78" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="O78" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="P78">
         <v>3800000</v>
       </c>
       <c r="Q78" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="R78" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S78" t="s">
         <v>40</v>
       </c>
       <c r="T78" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U78" t="s">
         <v>28</v>
@@ -4884,25 +4890,25 @@
         <v>44</v>
       </c>
       <c r="N79" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="O79" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="P79">
         <v>3800000</v>
       </c>
       <c r="Q79" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="R79" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S79" t="s">
         <v>40</v>
       </c>
       <c r="T79" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U79" t="s">
         <v>28</v>
@@ -4928,31 +4934,31 @@
         <v>29</v>
       </c>
       <c r="J80" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="K80" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="N80" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="O80" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="P80">
         <v>3800000</v>
       </c>
       <c r="Q80" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="R80" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S80" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T80" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U80" t="s">
         <v>28</v>
@@ -4978,25 +4984,25 @@
         <v>28</v>
       </c>
       <c r="N81" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="O81" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="P81">
         <v>4394700</v>
       </c>
       <c r="Q81" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R81" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="S81" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T81" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U81" t="s">
         <v>28</v>
@@ -5025,31 +5031,31 @@
         <v>30</v>
       </c>
       <c r="K82" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="N82" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="O82" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="P82">
         <v>528395.9300000001</v>
       </c>
       <c r="Q82" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="R82" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="S82" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T82" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="U82" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="V82" s="1">
         <v>46382</v>
@@ -5072,25 +5078,25 @@
         <v>29</v>
       </c>
       <c r="N83" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="O83" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="P83">
         <v>1000000</v>
       </c>
       <c r="Q83" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="R83" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="S83" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="T83" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U83" t="s">
         <v>28</v>
@@ -5116,25 +5122,25 @@
         <v>28</v>
       </c>
       <c r="N84" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="O84" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="P84">
         <v>4394700</v>
       </c>
       <c r="Q84" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R84" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="S84" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="T84" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U84" t="s">
         <v>28</v>
@@ -5166,25 +5172,25 @@
         <v>44</v>
       </c>
       <c r="N85" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="O85" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="P85">
         <v>3306000</v>
       </c>
       <c r="Q85" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R85" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="S85" t="s">
         <v>40</v>
       </c>
       <c r="T85" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U85" t="s">
         <v>28</v>
@@ -5213,25 +5219,25 @@
         <v>44</v>
       </c>
       <c r="N86" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="O86" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="P86">
         <v>3306000</v>
       </c>
       <c r="Q86" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R86" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="S86" t="s">
         <v>40</v>
       </c>
       <c r="T86" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U86" t="s">
         <v>28</v>
@@ -5257,25 +5263,25 @@
         <v>30</v>
       </c>
       <c r="N87" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="O87" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="P87">
         <v>470820</v>
       </c>
       <c r="Q87" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R87" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="S87" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="T87" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="U87" t="s">
         <v>28</v>

</xml_diff>